<commit_message>
NL-wortel: wapen-hero ingesteld zodat startscherm zichtbaar is
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR65"/>
+  <dimension ref="A2:AR65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -923,9 +923,9 @@
           <t>0</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="C3" s="33" t="inlineStr"/>
+      <c r="D3" s="33" t="inlineStr"/>
+      <c r="E3" s="33" t="inlineStr">
         <is>
           <t>talenring</t>
         </is>
@@ -941,35 +941,35 @@
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="I3" s="33" t="inlineStr"/>
+      <c r="J3" s="33" t="inlineStr">
         <is>
           <t>../assets/wat-opkomt/wapen_nova_democratia.png</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="33" t="inlineStr">
         <is>
           <t>center</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="L3" s="33" t="inlineStr">
         <is>
           <t>geen</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="M3" s="33" t="inlineStr">
         <is>
           <t>bottom</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="N3" s="33" t="inlineStr">
         <is>
           <t>licht</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr"/>
-      <c r="P3" s="3" t="inlineStr"/>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="O3" s="33" t="inlineStr"/>
+      <c r="P3" s="33" t="inlineStr"/>
+      <c r="Q3" s="33" t="inlineStr">
         <is>
           <t>self</t>
         </is>
@@ -979,15 +979,15 @@
           <t>live</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr"/>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="S3" s="33" t="inlineStr"/>
+      <c r="T3" s="33" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="U3" s="3" t="inlineStr"/>
-      <c r="V3" s="3" t="inlineStr"/>
-      <c r="W3" s="3" t="inlineStr"/>
+      <c r="U3" s="33" t="inlineStr"/>
+      <c r="V3" s="33" t="inlineStr"/>
+      <c r="W3" s="33" t="inlineStr"/>
       <c r="X3" s="4" t="inlineStr">
         <is>
           <t>De talenring is het startscherm: kies een taal voor je verkennen</t>
@@ -1037,10 +1037,14 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
+          <t>Nederlands</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
           <t>Het Open Vizier</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr"/>
       <c r="H4" s="8" t="inlineStr"/>
       <c r="I4" s="7" t="inlineStr"/>
       <c r="J4" s="7" t="inlineStr">
@@ -1055,7 +1059,7 @@
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
-          <t>standaard</t>
+          <t>geen</t>
         </is>
       </c>
       <c r="M4" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Excel: volledig gevuld met metadata uit artikelen (beschrijving, datum, tags, gerelateerd, talen, auteur)
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -650,8 +650,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR65"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:AR65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -1045,7 +1045,11 @@
           <t>Het Open Vizier</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr"/>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Nederlandse uitgave van Het Open Vizier — onderzoeksjournalistiek over governance, energie en economie.</t>
+        </is>
+      </c>
       <c r="I4" s="7" t="inlineStr"/>
       <c r="J4" s="7" t="inlineStr">
         <is>
@@ -1108,11 +1112,27 @@
       <c r="AF4" s="33" t="n"/>
       <c r="AG4" s="33" t="n"/>
       <c r="AH4" s="33" t="n"/>
-      <c r="AI4" s="33" t="n"/>
+      <c r="AI4" s="33" t="inlineStr">
+        <is>
+          <t>talen, nederlands</t>
+        </is>
+      </c>
       <c r="AJ4" s="33" t="n"/>
-      <c r="AK4" s="33" t="n"/>
-      <c r="AL4" s="33" t="n"/>
-      <c r="AM4" s="33" t="n"/>
+      <c r="AK4" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL4" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM4" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN4" s="33" t="n"/>
       <c r="AO4" s="33" t="n"/>
       <c r="AP4" s="33" t="n"/>
@@ -1150,7 +1170,11 @@
           <t>wat is er nieuw</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr"/>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>De gewone bladlezer: laatste artikelen, voorpagina, en alle edities op één plek.</t>
+        </is>
+      </c>
       <c r="I5" s="10" t="inlineStr"/>
       <c r="J5" s="10" t="inlineStr">
         <is>
@@ -1169,7 +1193,7 @@
       </c>
       <c r="M5" s="10" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>top</t>
         </is>
       </c>
       <c r="N5" s="10" t="inlineStr">
@@ -1215,9 +1239,21 @@
       <c r="AH5" s="33" t="n"/>
       <c r="AI5" s="33" t="n"/>
       <c r="AJ5" s="33" t="n"/>
-      <c r="AK5" s="33" t="n"/>
-      <c r="AL5" s="33" t="n"/>
-      <c r="AM5" s="33" t="n"/>
+      <c r="AK5" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL5" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM5" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN5" s="33" t="n"/>
       <c r="AO5" s="33" t="n"/>
       <c r="AP5" s="33" t="n"/>
@@ -1324,9 +1360,21 @@
       <c r="AH6" s="33" t="n"/>
       <c r="AI6" s="33" t="n"/>
       <c r="AJ6" s="33" t="n"/>
-      <c r="AK6" s="33" t="n"/>
-      <c r="AL6" s="33" t="n"/>
-      <c r="AM6" s="33" t="n"/>
+      <c r="AK6" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL6" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM6" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN6" s="33" t="n"/>
       <c r="AO6" s="33" t="n"/>
       <c r="AP6" s="33" t="n"/>
@@ -1433,9 +1481,21 @@
       <c r="AH7" s="33" t="n"/>
       <c r="AI7" s="33" t="n"/>
       <c r="AJ7" s="33" t="n"/>
-      <c r="AK7" s="33" t="n"/>
-      <c r="AL7" s="33" t="n"/>
-      <c r="AM7" s="33" t="n"/>
+      <c r="AK7" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL7" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM7" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN7" s="33" t="n"/>
       <c r="AO7" s="33" t="n"/>
       <c r="AP7" s="33" t="n"/>
@@ -1538,9 +1598,21 @@
       <c r="AH8" s="33" t="n"/>
       <c r="AI8" s="33" t="n"/>
       <c r="AJ8" s="33" t="n"/>
-      <c r="AK8" s="33" t="n"/>
-      <c r="AL8" s="33" t="n"/>
-      <c r="AM8" s="33" t="n"/>
+      <c r="AK8" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL8" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM8" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN8" s="33" t="n"/>
       <c r="AO8" s="33" t="n"/>
       <c r="AP8" s="33" t="n"/>
@@ -1574,7 +1646,11 @@
         </is>
       </c>
       <c r="G9" s="17" t="inlineStr"/>
-      <c r="H9" s="17" t="inlineStr"/>
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>Wat Brussel, Den Haag, Berlijn en Malta cumulatief doen met de huishoudens van het continent — gespiegeld in wat Trump-II tegenover ze zet. Zeven stukken d</t>
+        </is>
+      </c>
       <c r="I9" s="16" t="inlineStr">
         <is>
           <t>editie-0/</t>
@@ -1645,11 +1721,31 @@
       <c r="AF9" s="33" t="n"/>
       <c r="AG9" s="33" t="n"/>
       <c r="AH9" s="33" t="n"/>
-      <c r="AI9" s="33" t="n"/>
-      <c r="AJ9" s="33" t="n"/>
-      <c r="AK9" s="33" t="n"/>
-      <c r="AL9" s="33" t="n"/>
-      <c r="AM9" s="33" t="n"/>
+      <c r="AI9" s="33" t="inlineStr">
+        <is>
+          <t>bladeren, edities</t>
+        </is>
+      </c>
+      <c r="AJ9" s="33" t="inlineStr">
+        <is>
+          <t>1.1.3.2, 1.1.3.3, 1.1.3.4, 1.1.3.5</t>
+        </is>
+      </c>
+      <c r="AK9" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL9" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM9" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN9" s="33" t="n"/>
       <c r="AO9" s="33" t="n"/>
       <c r="AP9" s="33" t="n"/>
@@ -1754,11 +1850,31 @@
       <c r="AF10" s="33" t="n"/>
       <c r="AG10" s="33" t="n"/>
       <c r="AH10" s="33" t="n"/>
-      <c r="AI10" s="33" t="n"/>
-      <c r="AJ10" s="33" t="n"/>
-      <c r="AK10" s="33" t="n"/>
-      <c r="AL10" s="33" t="n"/>
-      <c r="AM10" s="33" t="n"/>
+      <c r="AI10" s="33" t="inlineStr">
+        <is>
+          <t>bladeren, edities</t>
+        </is>
+      </c>
+      <c r="AJ10" s="33" t="inlineStr">
+        <is>
+          <t>1.1.3.1, 1.1.3.3, 1.1.3.4, 1.1.3.5</t>
+        </is>
+      </c>
+      <c r="AK10" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="AL10" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM10" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN10" s="33" t="n"/>
       <c r="AO10" s="33" t="n"/>
       <c r="AP10" s="33" t="n"/>
@@ -1792,7 +1908,11 @@
         </is>
       </c>
       <c r="G11" s="17" t="inlineStr"/>
-      <c r="H11" s="17" t="inlineStr"/>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>Editie 2 — Negen stukken over de Nederlandse systeemcrisis, het grondvest voor herstel en concrete beleidsadviezen — inclusief een onderwijs-trilogie en een data-bijblad.</t>
+        </is>
+      </c>
       <c r="I11" s="16" t="inlineStr">
         <is>
           <t>editie-2/</t>
@@ -1863,11 +1983,31 @@
       <c r="AF11" s="33" t="n"/>
       <c r="AG11" s="33" t="n"/>
       <c r="AH11" s="33" t="n"/>
-      <c r="AI11" s="33" t="n"/>
-      <c r="AJ11" s="33" t="n"/>
-      <c r="AK11" s="33" t="n"/>
-      <c r="AL11" s="33" t="n"/>
-      <c r="AM11" s="33" t="n"/>
+      <c r="AI11" s="33" t="inlineStr">
+        <is>
+          <t>bladeren, edities</t>
+        </is>
+      </c>
+      <c r="AJ11" s="33" t="inlineStr">
+        <is>
+          <t>1.1.3.1, 1.1.3.2, 1.1.3.4, 1.1.3.5</t>
+        </is>
+      </c>
+      <c r="AK11" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="AL11" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM11" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN11" s="33" t="n"/>
       <c r="AO11" s="33" t="n"/>
       <c r="AP11" s="33" t="n"/>
@@ -1901,7 +2041,11 @@
         </is>
       </c>
       <c r="G12" s="17" t="inlineStr"/>
-      <c r="H12" s="17" t="inlineStr"/>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t>Een gedachtegoed over het oergevoel, het driedubbele brein, en de mens die wij niet meer opleiden.</t>
+        </is>
+      </c>
       <c r="I12" s="16" t="inlineStr">
         <is>
           <t>editie-3/</t>
@@ -1972,11 +2116,31 @@
       <c r="AF12" s="33" t="n"/>
       <c r="AG12" s="33" t="n"/>
       <c r="AH12" s="33" t="n"/>
-      <c r="AI12" s="33" t="n"/>
-      <c r="AJ12" s="33" t="n"/>
-      <c r="AK12" s="33" t="n"/>
-      <c r="AL12" s="33" t="n"/>
-      <c r="AM12" s="33" t="n"/>
+      <c r="AI12" s="33" t="inlineStr">
+        <is>
+          <t>bladeren, edities</t>
+        </is>
+      </c>
+      <c r="AJ12" s="33" t="inlineStr">
+        <is>
+          <t>1.1.3.1, 1.1.3.2, 1.1.3.3, 1.1.3.5</t>
+        </is>
+      </c>
+      <c r="AK12" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL12" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM12" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN12" s="33" t="n"/>
       <c r="AO12" s="33" t="n"/>
       <c r="AP12" s="33" t="n"/>
@@ -2010,7 +2174,11 @@
         </is>
       </c>
       <c r="G13" s="17" t="inlineStr"/>
-      <c r="H13" s="17" t="inlineStr"/>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>Een editie over hoe regels, verzekeringen, financiering en toezicht het oergevoel uit de beroepspraktijk hebben gewrongen — en wat dat met ons heeft gedaan.</t>
+        </is>
+      </c>
       <c r="I13" s="16" t="inlineStr">
         <is>
           <t>editie-4/</t>
@@ -2081,11 +2249,31 @@
       <c r="AF13" s="33" t="n"/>
       <c r="AG13" s="33" t="n"/>
       <c r="AH13" s="33" t="n"/>
-      <c r="AI13" s="33" t="n"/>
-      <c r="AJ13" s="33" t="n"/>
-      <c r="AK13" s="33" t="n"/>
-      <c r="AL13" s="33" t="n"/>
-      <c r="AM13" s="33" t="n"/>
+      <c r="AI13" s="33" t="inlineStr">
+        <is>
+          <t>bladeren, edities</t>
+        </is>
+      </c>
+      <c r="AJ13" s="33" t="inlineStr">
+        <is>
+          <t>1.1.3.1, 1.1.3.2, 1.1.3.3, 1.1.3.4</t>
+        </is>
+      </c>
+      <c r="AK13" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL13" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM13" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN13" s="33" t="n"/>
       <c r="AO13" s="33" t="n"/>
       <c r="AP13" s="33" t="n"/>
@@ -2119,7 +2307,11 @@
         </is>
       </c>
       <c r="G14" s="17" t="inlineStr"/>
-      <c r="H14" s="17" t="inlineStr"/>
+      <c r="H14" s="17" t="inlineStr">
+        <is>
+          <t>Wat zwaar weegt, en wat de pers ervan maakt. Een diagnostische editie in vier delen.</t>
+        </is>
+      </c>
       <c r="I14" s="16" t="inlineStr">
         <is>
           <t>editie-5/</t>
@@ -2190,11 +2382,31 @@
       <c r="AF14" s="33" t="n"/>
       <c r="AG14" s="33" t="n"/>
       <c r="AH14" s="33" t="n"/>
-      <c r="AI14" s="33" t="n"/>
-      <c r="AJ14" s="33" t="n"/>
-      <c r="AK14" s="33" t="n"/>
-      <c r="AL14" s="33" t="n"/>
-      <c r="AM14" s="33" t="n"/>
+      <c r="AI14" s="33" t="inlineStr">
+        <is>
+          <t>bladeren, edities</t>
+        </is>
+      </c>
+      <c r="AJ14" s="33" t="inlineStr">
+        <is>
+          <t>1.1.3.1, 1.1.3.2, 1.1.3.3, 1.1.3.4</t>
+        </is>
+      </c>
+      <c r="AK14" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="AL14" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM14" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN14" s="33" t="n"/>
       <c r="AO14" s="33" t="n"/>
       <c r="AP14" s="33" t="n"/>
@@ -2228,7 +2440,11 @@
         </is>
       </c>
       <c r="G15" s="17" t="inlineStr"/>
-      <c r="H15" s="17" t="inlineStr"/>
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>Een editie over de fysica van de Nederlandse hervorming — Pareto, ordes, het ontwerp dat werkt, en de kennislaag die de behoudende kracht draagt. Veertien stukken.</t>
+        </is>
+      </c>
       <c r="I15" s="16" t="inlineStr">
         <is>
           <t>editie-6/</t>
@@ -2299,11 +2515,31 @@
       <c r="AF15" s="33" t="n"/>
       <c r="AG15" s="33" t="n"/>
       <c r="AH15" s="33" t="n"/>
-      <c r="AI15" s="33" t="n"/>
-      <c r="AJ15" s="33" t="n"/>
-      <c r="AK15" s="33" t="n"/>
-      <c r="AL15" s="33" t="n"/>
-      <c r="AM15" s="33" t="n"/>
+      <c r="AI15" s="33" t="inlineStr">
+        <is>
+          <t>bladeren, edities</t>
+        </is>
+      </c>
+      <c r="AJ15" s="33" t="inlineStr">
+        <is>
+          <t>1.1.3.1, 1.1.3.2, 1.1.3.3, 1.1.3.4</t>
+        </is>
+      </c>
+      <c r="AK15" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL15" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM15" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN15" s="33" t="n"/>
       <c r="AO15" s="33" t="n"/>
       <c r="AP15" s="33" t="n"/>
@@ -2341,7 +2577,11 @@
           <t>de analyses</t>
         </is>
       </c>
-      <c r="H16" s="11" t="inlineStr"/>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>Voor wie de analyses zoekt — Gevolgenkaarten, BiCRS, politiek en de Nederlandse context.</t>
+        </is>
+      </c>
       <c r="I16" s="10" t="inlineStr"/>
       <c r="J16" s="10" t="inlineStr">
         <is>
@@ -2360,7 +2600,7 @@
       </c>
       <c r="M16" s="10" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>top</t>
         </is>
       </c>
       <c r="N16" s="10" t="inlineStr">
@@ -2406,9 +2646,21 @@
       <c r="AH16" s="33" t="n"/>
       <c r="AI16" s="33" t="n"/>
       <c r="AJ16" s="33" t="n"/>
-      <c r="AK16" s="33" t="n"/>
-      <c r="AL16" s="33" t="n"/>
-      <c r="AM16" s="33" t="n"/>
+      <c r="AK16" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL16" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM16" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN16" s="33" t="n"/>
       <c r="AO16" s="33" t="n"/>
       <c r="AP16" s="33" t="n"/>
@@ -2465,7 +2717,7 @@
       </c>
       <c r="M17" s="19" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>top</t>
         </is>
       </c>
       <c r="N17" s="19" t="inlineStr">
@@ -2511,9 +2763,21 @@
       <c r="AH17" s="33" t="n"/>
       <c r="AI17" s="33" t="n"/>
       <c r="AJ17" s="33" t="n"/>
-      <c r="AK17" s="33" t="n"/>
-      <c r="AL17" s="33" t="n"/>
-      <c r="AM17" s="33" t="n"/>
+      <c r="AK17" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL17" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM17" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN17" s="33" t="n"/>
       <c r="AO17" s="33" t="n"/>
       <c r="AP17" s="33" t="n"/>
@@ -2616,9 +2880,21 @@
       <c r="AH18" s="33" t="n"/>
       <c r="AI18" s="33" t="n"/>
       <c r="AJ18" s="33" t="n"/>
-      <c r="AK18" s="33" t="n"/>
-      <c r="AL18" s="33" t="n"/>
-      <c r="AM18" s="33" t="n"/>
+      <c r="AK18" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL18" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM18" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN18" s="33" t="n"/>
       <c r="AO18" s="33" t="n"/>
       <c r="AP18" s="33" t="n"/>
@@ -2727,11 +3003,31 @@
       <c r="AF19" s="33" t="n"/>
       <c r="AG19" s="33" t="n"/>
       <c r="AH19" s="33" t="n"/>
-      <c r="AI19" s="33" t="n"/>
-      <c r="AJ19" s="33" t="n"/>
-      <c r="AK19" s="33" t="n"/>
-      <c r="AL19" s="33" t="n"/>
-      <c r="AM19" s="33" t="n"/>
+      <c r="AI19" s="33" t="inlineStr">
+        <is>
+          <t>fundament, gevolgenkaarten, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ19" s="33" t="inlineStr">
+        <is>
+          <t>1.2.1.1.2</t>
+        </is>
+      </c>
+      <c r="AK19" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL19" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM19" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN19" s="33" t="n"/>
       <c r="AO19" s="33" t="n"/>
       <c r="AP19" s="33" t="n"/>
@@ -2840,11 +3136,31 @@
       <c r="AF20" s="33" t="n"/>
       <c r="AG20" s="33" t="n"/>
       <c r="AH20" s="33" t="n"/>
-      <c r="AI20" s="33" t="n"/>
-      <c r="AJ20" s="33" t="n"/>
-      <c r="AK20" s="33" t="n"/>
-      <c r="AL20" s="33" t="n"/>
-      <c r="AM20" s="33" t="n"/>
+      <c r="AI20" s="33" t="inlineStr">
+        <is>
+          <t>fundament, gevolgenkaarten, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ20" s="33" t="inlineStr">
+        <is>
+          <t>1.2.1.1.1</t>
+        </is>
+      </c>
+      <c r="AK20" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL20" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM20" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN20" s="33" t="n"/>
       <c r="AO20" s="33" t="n"/>
       <c r="AP20" s="33" t="n"/>
@@ -2947,9 +3263,21 @@
       <c r="AH21" s="33" t="n"/>
       <c r="AI21" s="33" t="n"/>
       <c r="AJ21" s="33" t="n"/>
-      <c r="AK21" s="33" t="n"/>
-      <c r="AL21" s="33" t="n"/>
-      <c r="AM21" s="33" t="n"/>
+      <c r="AK21" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL21" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM21" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN21" s="33" t="n"/>
       <c r="AO21" s="33" t="n"/>
       <c r="AP21" s="33" t="n"/>
@@ -3058,11 +3386,31 @@
       <c r="AF22" s="33" t="n"/>
       <c r="AG22" s="33" t="n"/>
       <c r="AH22" s="33" t="n"/>
-      <c r="AI22" s="33" t="n"/>
-      <c r="AJ22" s="33" t="n"/>
-      <c r="AK22" s="33" t="n"/>
-      <c r="AL22" s="33" t="n"/>
-      <c r="AM22" s="33" t="n"/>
+      <c r="AI22" s="33" t="inlineStr">
+        <is>
+          <t>europese-&amp;-globale-kaarten, gevolgenkaarten, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ22" s="33" t="inlineStr">
+        <is>
+          <t>1.2.1.2.2, 1.2.1.2.3, 1.2.1.2.4</t>
+        </is>
+      </c>
+      <c r="AK22" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL22" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM22" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN22" s="33" t="n"/>
       <c r="AO22" s="33" t="n"/>
       <c r="AP22" s="33" t="n"/>
@@ -3171,11 +3519,31 @@
       <c r="AF23" s="33" t="n"/>
       <c r="AG23" s="33" t="n"/>
       <c r="AH23" s="33" t="n"/>
-      <c r="AI23" s="33" t="n"/>
-      <c r="AJ23" s="33" t="n"/>
-      <c r="AK23" s="33" t="n"/>
-      <c r="AL23" s="33" t="n"/>
-      <c r="AM23" s="33" t="n"/>
+      <c r="AI23" s="33" t="inlineStr">
+        <is>
+          <t>europese-&amp;-globale-kaarten, gevolgenkaarten, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ23" s="33" t="inlineStr">
+        <is>
+          <t>1.2.1.2.1, 1.2.1.2.3, 1.2.1.2.4</t>
+        </is>
+      </c>
+      <c r="AK23" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL23" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM23" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN23" s="33" t="n"/>
       <c r="AO23" s="33" t="n"/>
       <c r="AP23" s="33" t="n"/>
@@ -3284,11 +3652,31 @@
       <c r="AF24" s="33" t="n"/>
       <c r="AG24" s="33" t="n"/>
       <c r="AH24" s="33" t="n"/>
-      <c r="AI24" s="33" t="n"/>
-      <c r="AJ24" s="33" t="n"/>
-      <c r="AK24" s="33" t="n"/>
-      <c r="AL24" s="33" t="n"/>
-      <c r="AM24" s="33" t="n"/>
+      <c r="AI24" s="33" t="inlineStr">
+        <is>
+          <t>europese-&amp;-globale-kaarten, gevolgenkaarten, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ24" s="33" t="inlineStr">
+        <is>
+          <t>1.2.1.2.1, 1.2.1.2.2, 1.2.1.2.4</t>
+        </is>
+      </c>
+      <c r="AK24" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL24" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM24" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN24" s="33" t="n"/>
       <c r="AO24" s="33" t="n"/>
       <c r="AP24" s="33" t="n"/>
@@ -3397,11 +3785,31 @@
       <c r="AF25" s="33" t="n"/>
       <c r="AG25" s="33" t="n"/>
       <c r="AH25" s="33" t="n"/>
-      <c r="AI25" s="33" t="n"/>
-      <c r="AJ25" s="33" t="n"/>
-      <c r="AK25" s="33" t="n"/>
-      <c r="AL25" s="33" t="n"/>
-      <c r="AM25" s="33" t="n"/>
+      <c r="AI25" s="33" t="inlineStr">
+        <is>
+          <t>europese-&amp;-globale-kaarten, gevolgenkaarten, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ25" s="33" t="inlineStr">
+        <is>
+          <t>1.2.1.2.1, 1.2.1.2.2, 1.2.1.2.3</t>
+        </is>
+      </c>
+      <c r="AK25" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL25" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM25" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN25" s="33" t="n"/>
       <c r="AO25" s="33" t="n"/>
       <c r="AP25" s="33" t="n"/>
@@ -3504,9 +3912,21 @@
       <c r="AH26" s="33" t="n"/>
       <c r="AI26" s="33" t="n"/>
       <c r="AJ26" s="33" t="n"/>
-      <c r="AK26" s="33" t="n"/>
-      <c r="AL26" s="33" t="n"/>
-      <c r="AM26" s="33" t="n"/>
+      <c r="AK26" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL26" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM26" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN26" s="33" t="n"/>
       <c r="AO26" s="33" t="n"/>
       <c r="AP26" s="33" t="n"/>
@@ -3615,11 +4035,31 @@
       <c r="AF27" s="33" t="n"/>
       <c r="AG27" s="33" t="n"/>
       <c r="AH27" s="33" t="n"/>
-      <c r="AI27" s="33" t="n"/>
-      <c r="AJ27" s="33" t="n"/>
-      <c r="AK27" s="33" t="n"/>
-      <c r="AL27" s="33" t="n"/>
-      <c r="AM27" s="33" t="n"/>
+      <c r="AI27" s="33" t="inlineStr">
+        <is>
+          <t>gevolgenkaarten, internationale-spiegels, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ27" s="33" t="inlineStr">
+        <is>
+          <t>1.2.1.3.2, 1.2.1.3.3</t>
+        </is>
+      </c>
+      <c r="AK27" s="33" t="inlineStr">
+        <is>
+          <t>2025-02-01</t>
+        </is>
+      </c>
+      <c r="AL27" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM27" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN27" s="33" t="n"/>
       <c r="AO27" s="33" t="n"/>
       <c r="AP27" s="33" t="n"/>
@@ -3728,11 +4168,31 @@
       <c r="AF28" s="33" t="n"/>
       <c r="AG28" s="33" t="n"/>
       <c r="AH28" s="33" t="n"/>
-      <c r="AI28" s="33" t="n"/>
-      <c r="AJ28" s="33" t="n"/>
-      <c r="AK28" s="33" t="n"/>
-      <c r="AL28" s="33" t="n"/>
-      <c r="AM28" s="33" t="n"/>
+      <c r="AI28" s="33" t="inlineStr">
+        <is>
+          <t>gevolgenkaarten, internationale-spiegels, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ28" s="33" t="inlineStr">
+        <is>
+          <t>1.2.1.3.1, 1.2.1.3.3</t>
+        </is>
+      </c>
+      <c r="AK28" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL28" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM28" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN28" s="33" t="n"/>
       <c r="AO28" s="33" t="n"/>
       <c r="AP28" s="33" t="n"/>
@@ -3841,11 +4301,31 @@
       <c r="AF29" s="33" t="n"/>
       <c r="AG29" s="33" t="n"/>
       <c r="AH29" s="33" t="n"/>
-      <c r="AI29" s="33" t="n"/>
-      <c r="AJ29" s="33" t="n"/>
-      <c r="AK29" s="33" t="n"/>
-      <c r="AL29" s="33" t="n"/>
-      <c r="AM29" s="33" t="n"/>
+      <c r="AI29" s="33" t="inlineStr">
+        <is>
+          <t>gevolgenkaarten, internationale-spiegels, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ29" s="33" t="inlineStr">
+        <is>
+          <t>1.2.1.3.1, 1.2.1.3.2</t>
+        </is>
+      </c>
+      <c r="AK29" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL29" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM29" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN29" s="33" t="n"/>
       <c r="AO29" s="33" t="n"/>
       <c r="AP29" s="33" t="n"/>
@@ -3902,7 +4382,7 @@
       </c>
       <c r="M30" s="19" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>top</t>
         </is>
       </c>
       <c r="N30" s="19" t="inlineStr">
@@ -3948,9 +4428,21 @@
       <c r="AH30" s="33" t="n"/>
       <c r="AI30" s="33" t="n"/>
       <c r="AJ30" s="33" t="n"/>
-      <c r="AK30" s="33" t="n"/>
-      <c r="AL30" s="33" t="n"/>
-      <c r="AM30" s="33" t="n"/>
+      <c r="AK30" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL30" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM30" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN30" s="33" t="n"/>
       <c r="AO30" s="33" t="n"/>
       <c r="AP30" s="33" t="n"/>
@@ -4059,11 +4551,31 @@
       <c r="AF31" s="33" t="n"/>
       <c r="AG31" s="33" t="n"/>
       <c r="AH31" s="33" t="n"/>
-      <c r="AI31" s="33" t="n"/>
-      <c r="AJ31" s="33" t="n"/>
-      <c r="AK31" s="33" t="n"/>
-      <c r="AL31" s="33" t="n"/>
-      <c r="AM31" s="33" t="n"/>
+      <c r="AI31" s="33" t="inlineStr">
+        <is>
+          <t>bicrs-energie, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ31" s="33" t="inlineStr">
+        <is>
+          <t>1.2.2.2, 1.2.2.3, 1.2.2.4, 1.2.2.5</t>
+        </is>
+      </c>
+      <c r="AK31" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL31" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM31" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN31" s="33" t="n"/>
       <c r="AO31" s="33" t="n"/>
       <c r="AP31" s="33" t="n"/>
@@ -4172,11 +4684,31 @@
       <c r="AF32" s="33" t="n"/>
       <c r="AG32" s="33" t="n"/>
       <c r="AH32" s="33" t="n"/>
-      <c r="AI32" s="33" t="n"/>
-      <c r="AJ32" s="33" t="n"/>
-      <c r="AK32" s="33" t="n"/>
-      <c r="AL32" s="33" t="n"/>
-      <c r="AM32" s="33" t="n"/>
+      <c r="AI32" s="33" t="inlineStr">
+        <is>
+          <t>bicrs-energie, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ32" s="33" t="inlineStr">
+        <is>
+          <t>1.2.2.1, 1.2.2.3, 1.2.2.4, 1.2.2.5</t>
+        </is>
+      </c>
+      <c r="AK32" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL32" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM32" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN32" s="33" t="n"/>
       <c r="AO32" s="33" t="n"/>
       <c r="AP32" s="33" t="n"/>
@@ -4285,11 +4817,31 @@
       <c r="AF33" s="33" t="n"/>
       <c r="AG33" s="33" t="n"/>
       <c r="AH33" s="33" t="n"/>
-      <c r="AI33" s="33" t="n"/>
-      <c r="AJ33" s="33" t="n"/>
-      <c r="AK33" s="33" t="n"/>
-      <c r="AL33" s="33" t="n"/>
-      <c r="AM33" s="33" t="n"/>
+      <c r="AI33" s="33" t="inlineStr">
+        <is>
+          <t>bicrs-energie, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ33" s="33" t="inlineStr">
+        <is>
+          <t>1.2.2.1, 1.2.2.2, 1.2.2.4, 1.2.2.5</t>
+        </is>
+      </c>
+      <c r="AK33" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL33" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM33" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN33" s="33" t="n"/>
       <c r="AO33" s="33" t="n"/>
       <c r="AP33" s="33" t="n"/>
@@ -4398,11 +4950,27 @@
       <c r="AF34" s="33" t="n"/>
       <c r="AG34" s="33" t="n"/>
       <c r="AH34" s="33" t="n"/>
-      <c r="AI34" s="33" t="n"/>
-      <c r="AJ34" s="33" t="n"/>
+      <c r="AI34" s="33" t="inlineStr">
+        <is>
+          <t>bicrs-energie, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ34" s="33" t="inlineStr">
+        <is>
+          <t>1.2.2.1, 1.2.2.2, 1.2.2.3, 1.2.2.5</t>
+        </is>
+      </c>
       <c r="AK34" s="33" t="n"/>
-      <c r="AL34" s="33" t="n"/>
-      <c r="AM34" s="33" t="n"/>
+      <c r="AL34" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM34" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN34" s="33" t="n"/>
       <c r="AO34" s="33" t="n"/>
       <c r="AP34" s="33" t="n"/>
@@ -4511,11 +5079,27 @@
       <c r="AF35" s="33" t="n"/>
       <c r="AG35" s="33" t="n"/>
       <c r="AH35" s="33" t="n"/>
-      <c r="AI35" s="33" t="n"/>
-      <c r="AJ35" s="33" t="n"/>
+      <c r="AI35" s="33" t="inlineStr">
+        <is>
+          <t>bicrs-energie, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ35" s="33" t="inlineStr">
+        <is>
+          <t>1.2.2.1, 1.2.2.2, 1.2.2.3, 1.2.2.4</t>
+        </is>
+      </c>
       <c r="AK35" s="33" t="n"/>
-      <c r="AL35" s="33" t="n"/>
-      <c r="AM35" s="33" t="n"/>
+      <c r="AL35" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM35" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN35" s="33" t="n"/>
       <c r="AO35" s="33" t="n"/>
       <c r="AP35" s="33" t="n"/>
@@ -4624,11 +5208,27 @@
       <c r="AF36" s="33" t="n"/>
       <c r="AG36" s="33" t="n"/>
       <c r="AH36" s="33" t="n"/>
-      <c r="AI36" s="33" t="n"/>
-      <c r="AJ36" s="33" t="n"/>
+      <c r="AI36" s="33" t="inlineStr">
+        <is>
+          <t>bicrs-energie, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ36" s="33" t="inlineStr">
+        <is>
+          <t>1.2.2.1, 1.2.2.2, 1.2.2.3, 1.2.2.4</t>
+        </is>
+      </c>
       <c r="AK36" s="33" t="n"/>
-      <c r="AL36" s="33" t="n"/>
-      <c r="AM36" s="33" t="n"/>
+      <c r="AL36" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM36" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN36" s="33" t="n"/>
       <c r="AO36" s="33" t="n"/>
       <c r="AP36" s="33" t="n"/>
@@ -4737,11 +5337,27 @@
       <c r="AF37" s="33" t="n"/>
       <c r="AG37" s="33" t="n"/>
       <c r="AH37" s="33" t="n"/>
-      <c r="AI37" s="33" t="n"/>
-      <c r="AJ37" s="33" t="n"/>
+      <c r="AI37" s="33" t="inlineStr">
+        <is>
+          <t>bicrs-energie, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ37" s="33" t="inlineStr">
+        <is>
+          <t>1.2.2.1, 1.2.2.2, 1.2.2.3, 1.2.2.4</t>
+        </is>
+      </c>
       <c r="AK37" s="33" t="n"/>
-      <c r="AL37" s="33" t="n"/>
-      <c r="AM37" s="33" t="n"/>
+      <c r="AL37" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM37" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN37" s="33" t="n"/>
       <c r="AO37" s="33" t="n"/>
       <c r="AP37" s="33" t="n"/>
@@ -4850,11 +5466,27 @@
       <c r="AF38" s="33" t="n"/>
       <c r="AG38" s="33" t="n"/>
       <c r="AH38" s="33" t="n"/>
-      <c r="AI38" s="33" t="n"/>
-      <c r="AJ38" s="33" t="n"/>
+      <c r="AI38" s="33" t="inlineStr">
+        <is>
+          <t>bicrs-energie, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ38" s="33" t="inlineStr">
+        <is>
+          <t>1.2.2.1, 1.2.2.2, 1.2.2.3, 1.2.2.4</t>
+        </is>
+      </c>
       <c r="AK38" s="33" t="n"/>
-      <c r="AL38" s="33" t="n"/>
-      <c r="AM38" s="33" t="n"/>
+      <c r="AL38" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM38" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN38" s="33" t="n"/>
       <c r="AO38" s="33" t="n"/>
       <c r="AP38" s="33" t="n"/>
@@ -4911,7 +5543,7 @@
       </c>
       <c r="M39" s="19" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>bottom</t>
         </is>
       </c>
       <c r="N39" s="19" t="inlineStr">
@@ -4957,9 +5589,21 @@
       <c r="AH39" s="33" t="n"/>
       <c r="AI39" s="33" t="n"/>
       <c r="AJ39" s="33" t="n"/>
-      <c r="AK39" s="33" t="n"/>
-      <c r="AL39" s="33" t="n"/>
-      <c r="AM39" s="33" t="n"/>
+      <c r="AK39" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL39" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM39" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN39" s="33" t="n"/>
       <c r="AO39" s="33" t="n"/>
       <c r="AP39" s="33" t="n"/>
@@ -5060,7 +5704,11 @@
         </is>
       </c>
       <c r="Z40" s="33" t="n"/>
-      <c r="AA40" s="33" t="n"/>
+      <c r="AA40" s="33" t="inlineStr">
+        <is>
+          <t>../assets/audio/de/ausgabe-2/nova-democratia.mp3</t>
+        </is>
+      </c>
       <c r="AB40" s="33" t="n"/>
       <c r="AC40" s="33" t="n"/>
       <c r="AD40" s="33" t="n"/>
@@ -5068,11 +5716,31 @@
       <c r="AF40" s="33" t="n"/>
       <c r="AG40" s="33" t="n"/>
       <c r="AH40" s="33" t="n"/>
-      <c r="AI40" s="33" t="n"/>
-      <c r="AJ40" s="33" t="n"/>
-      <c r="AK40" s="33" t="n"/>
-      <c r="AL40" s="33" t="n"/>
-      <c r="AM40" s="33" t="n"/>
+      <c r="AI40" s="33" t="inlineStr">
+        <is>
+          <t>politiek-hervorming, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ40" s="33" t="inlineStr">
+        <is>
+          <t>1.2.3.2, 1.2.3.4</t>
+        </is>
+      </c>
+      <c r="AK40" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL40" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM40" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN40" s="33" t="n"/>
       <c r="AO40" s="33" t="n"/>
       <c r="AP40" s="33" t="n"/>
@@ -5181,11 +5849,31 @@
       <c r="AF41" s="33" t="n"/>
       <c r="AG41" s="33" t="n"/>
       <c r="AH41" s="33" t="n"/>
-      <c r="AI41" s="33" t="n"/>
-      <c r="AJ41" s="33" t="n"/>
-      <c r="AK41" s="33" t="n"/>
-      <c r="AL41" s="33" t="n"/>
-      <c r="AM41" s="33" t="n"/>
+      <c r="AI41" s="33" t="inlineStr">
+        <is>
+          <t>politiek-hervorming, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ41" s="33" t="inlineStr">
+        <is>
+          <t>1.2.3.1, 1.2.3.4</t>
+        </is>
+      </c>
+      <c r="AK41" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL41" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM41" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN41" s="33" t="n"/>
       <c r="AO41" s="33" t="n"/>
       <c r="AP41" s="33" t="n"/>
@@ -5292,9 +5980,21 @@
       <c r="AH42" s="33" t="n"/>
       <c r="AI42" s="33" t="n"/>
       <c r="AJ42" s="33" t="n"/>
-      <c r="AK42" s="33" t="n"/>
-      <c r="AL42" s="33" t="n"/>
-      <c r="AM42" s="33" t="n"/>
+      <c r="AK42" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL42" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM42" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN42" s="33" t="n"/>
       <c r="AO42" s="33" t="n"/>
       <c r="AP42" s="33" t="n"/>
@@ -5328,7 +6028,11 @@
         </is>
       </c>
       <c r="G43" s="17" t="inlineStr"/>
-      <c r="H43" s="17" t="inlineStr"/>
+      <c r="H43" s="17" t="inlineStr">
+        <is>
+          <t>De cirkel van onrecht waarin Europa zichzelf vernietigt</t>
+        </is>
+      </c>
       <c r="I43" s="16" t="inlineStr">
         <is>
           <t>wat-opkomt/plundering-0-eerst-plukken-dan-oordelen.html</t>
@@ -5399,11 +6103,31 @@
       <c r="AF43" s="33" t="n"/>
       <c r="AG43" s="33" t="n"/>
       <c r="AH43" s="33" t="n"/>
-      <c r="AI43" s="33" t="n"/>
-      <c r="AJ43" s="33" t="n"/>
-      <c r="AK43" s="33" t="n"/>
-      <c r="AL43" s="33" t="n"/>
-      <c r="AM43" s="33" t="n"/>
+      <c r="AI43" s="33" t="inlineStr">
+        <is>
+          <t>de-grote-plundering, politiek-hervorming, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ43" s="33" t="inlineStr">
+        <is>
+          <t>1.2.3.3.2, 1.2.3.3.3, 1.2.3.3.4, 1.2.3.3.5</t>
+        </is>
+      </c>
+      <c r="AK43" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL43" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM43" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN43" s="33" t="n"/>
       <c r="AO43" s="33" t="n"/>
       <c r="AP43" s="33" t="n"/>
@@ -5437,7 +6161,11 @@
         </is>
       </c>
       <c r="G44" s="17" t="inlineStr"/>
-      <c r="H44" s="17" t="inlineStr"/>
+      <c r="H44" s="17" t="inlineStr">
+        <is>
+          <t>Wij plukken wie ons voedt</t>
+        </is>
+      </c>
       <c r="I44" s="16" t="inlineStr">
         <is>
           <t>wat-opkomt/plundering-1-diagnose.html</t>
@@ -5508,11 +6236,31 @@
       <c r="AF44" s="33" t="n"/>
       <c r="AG44" s="33" t="n"/>
       <c r="AH44" s="33" t="n"/>
-      <c r="AI44" s="33" t="n"/>
-      <c r="AJ44" s="33" t="n"/>
-      <c r="AK44" s="33" t="n"/>
-      <c r="AL44" s="33" t="n"/>
-      <c r="AM44" s="33" t="n"/>
+      <c r="AI44" s="33" t="inlineStr">
+        <is>
+          <t>de-grote-plundering, politiek-hervorming, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ44" s="33" t="inlineStr">
+        <is>
+          <t>1.2.3.3.1, 1.2.3.3.3, 1.2.3.3.4, 1.2.3.3.5</t>
+        </is>
+      </c>
+      <c r="AK44" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL44" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM44" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN44" s="33" t="n"/>
       <c r="AO44" s="33" t="n"/>
       <c r="AP44" s="33" t="n"/>
@@ -5546,7 +6294,11 @@
         </is>
       </c>
       <c r="G45" s="17" t="inlineStr"/>
-      <c r="H45" s="17" t="inlineStr"/>
+      <c r="H45" s="17" t="inlineStr">
+        <is>
+          <t>De muren die wij hebben gemetseld om onze bouwers op te sluiten</t>
+        </is>
+      </c>
       <c r="I45" s="16" t="inlineStr">
         <is>
           <t>wat-opkomt/plundering-2-mechaniek.html</t>
@@ -5617,11 +6369,31 @@
       <c r="AF45" s="33" t="n"/>
       <c r="AG45" s="33" t="n"/>
       <c r="AH45" s="33" t="n"/>
-      <c r="AI45" s="33" t="n"/>
-      <c r="AJ45" s="33" t="n"/>
-      <c r="AK45" s="33" t="n"/>
-      <c r="AL45" s="33" t="n"/>
-      <c r="AM45" s="33" t="n"/>
+      <c r="AI45" s="33" t="inlineStr">
+        <is>
+          <t>de-grote-plundering, politiek-hervorming, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ45" s="33" t="inlineStr">
+        <is>
+          <t>1.2.3.3.1, 1.2.3.3.2, 1.2.3.3.4, 1.2.3.3.5</t>
+        </is>
+      </c>
+      <c r="AK45" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL45" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM45" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN45" s="33" t="n"/>
       <c r="AO45" s="33" t="n"/>
       <c r="AP45" s="33" t="n"/>
@@ -5655,7 +6427,11 @@
         </is>
       </c>
       <c r="G46" s="17" t="inlineStr"/>
-      <c r="H46" s="17" t="inlineStr"/>
+      <c r="H46" s="17" t="inlineStr">
+        <is>
+          <t>Waarom de plunderaars zwaarder zullen lijden dan de geplunderden</t>
+        </is>
+      </c>
       <c r="I46" s="16" t="inlineStr">
         <is>
           <t>wat-opkomt/plundering-3-afloop.html</t>
@@ -5726,11 +6502,31 @@
       <c r="AF46" s="33" t="n"/>
       <c r="AG46" s="33" t="n"/>
       <c r="AH46" s="33" t="n"/>
-      <c r="AI46" s="33" t="n"/>
-      <c r="AJ46" s="33" t="n"/>
-      <c r="AK46" s="33" t="n"/>
-      <c r="AL46" s="33" t="n"/>
-      <c r="AM46" s="33" t="n"/>
+      <c r="AI46" s="33" t="inlineStr">
+        <is>
+          <t>de-grote-plundering, politiek-hervorming, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ46" s="33" t="inlineStr">
+        <is>
+          <t>1.2.3.3.1, 1.2.3.3.2, 1.2.3.3.3, 1.2.3.3.5</t>
+        </is>
+      </c>
+      <c r="AK46" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL46" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM46" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN46" s="33" t="n"/>
       <c r="AO46" s="33" t="n"/>
       <c r="AP46" s="33" t="n"/>
@@ -5764,7 +6560,11 @@
         </is>
       </c>
       <c r="G47" s="17" t="inlineStr"/>
-      <c r="H47" s="17" t="inlineStr"/>
+      <c r="H47" s="17" t="inlineStr">
+        <is>
+          <t>Wie wil wat, en waarom Brussel niet weet hoe verder</t>
+        </is>
+      </c>
       <c r="I47" s="16" t="inlineStr">
         <is>
           <t>wat-opkomt/plundering-4-politieke-landschap.html</t>
@@ -5835,11 +6635,31 @@
       <c r="AF47" s="33" t="n"/>
       <c r="AG47" s="33" t="n"/>
       <c r="AH47" s="33" t="n"/>
-      <c r="AI47" s="33" t="n"/>
-      <c r="AJ47" s="33" t="n"/>
-      <c r="AK47" s="33" t="n"/>
-      <c r="AL47" s="33" t="n"/>
-      <c r="AM47" s="33" t="n"/>
+      <c r="AI47" s="33" t="inlineStr">
+        <is>
+          <t>de-grote-plundering, politiek-hervorming, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ47" s="33" t="inlineStr">
+        <is>
+          <t>1.2.3.3.1, 1.2.3.3.2, 1.2.3.3.3, 1.2.3.3.4</t>
+        </is>
+      </c>
+      <c r="AK47" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL47" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM47" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN47" s="33" t="n"/>
       <c r="AO47" s="33" t="n"/>
       <c r="AP47" s="33" t="n"/>
@@ -5948,11 +6768,31 @@
       <c r="AF48" s="33" t="n"/>
       <c r="AG48" s="33" t="n"/>
       <c r="AH48" s="33" t="n"/>
-      <c r="AI48" s="33" t="n"/>
-      <c r="AJ48" s="33" t="n"/>
-      <c r="AK48" s="33" t="n"/>
-      <c r="AL48" s="33" t="n"/>
-      <c r="AM48" s="33" t="n"/>
+      <c r="AI48" s="33" t="inlineStr">
+        <is>
+          <t>politiek-hervorming, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ48" s="33" t="inlineStr">
+        <is>
+          <t>1.2.3.1, 1.2.3.2</t>
+        </is>
+      </c>
+      <c r="AK48" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL48" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM48" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN48" s="33" t="n"/>
       <c r="AO48" s="33" t="n"/>
       <c r="AP48" s="33" t="n"/>
@@ -6009,7 +6849,7 @@
       </c>
       <c r="M49" s="19" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>bottom</t>
         </is>
       </c>
       <c r="N49" s="19" t="inlineStr">
@@ -6055,9 +6895,21 @@
       <c r="AH49" s="33" t="n"/>
       <c r="AI49" s="33" t="n"/>
       <c r="AJ49" s="33" t="n"/>
-      <c r="AK49" s="33" t="n"/>
-      <c r="AL49" s="33" t="n"/>
-      <c r="AM49" s="33" t="n"/>
+      <c r="AK49" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL49" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM49" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN49" s="33" t="n"/>
       <c r="AO49" s="33" t="n"/>
       <c r="AP49" s="33" t="n"/>
@@ -6166,11 +7018,31 @@
       <c r="AF50" s="33" t="n"/>
       <c r="AG50" s="33" t="n"/>
       <c r="AH50" s="33" t="n"/>
-      <c r="AI50" s="33" t="n"/>
-      <c r="AJ50" s="33" t="n"/>
-      <c r="AK50" s="33" t="n"/>
-      <c r="AL50" s="33" t="n"/>
-      <c r="AM50" s="33" t="n"/>
+      <c r="AI50" s="33" t="inlineStr">
+        <is>
+          <t>nederland-&amp;-wereld, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ50" s="33" t="inlineStr">
+        <is>
+          <t>1.2.4.2, 1.2.4.3</t>
+        </is>
+      </c>
+      <c r="AK50" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL50" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM50" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN50" s="33" t="n"/>
       <c r="AO50" s="33" t="n"/>
       <c r="AP50" s="33" t="n"/>
@@ -6279,11 +7151,31 @@
       <c r="AF51" s="33" t="n"/>
       <c r="AG51" s="33" t="n"/>
       <c r="AH51" s="33" t="n"/>
-      <c r="AI51" s="33" t="n"/>
-      <c r="AJ51" s="33" t="n"/>
-      <c r="AK51" s="33" t="n"/>
-      <c r="AL51" s="33" t="n"/>
-      <c r="AM51" s="33" t="n"/>
+      <c r="AI51" s="33" t="inlineStr">
+        <is>
+          <t>nederland-&amp;-wereld, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ51" s="33" t="inlineStr">
+        <is>
+          <t>1.2.4.1, 1.2.4.3</t>
+        </is>
+      </c>
+      <c r="AK51" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL51" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM51" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN51" s="33" t="n"/>
       <c r="AO51" s="33" t="n"/>
       <c r="AP51" s="33" t="n"/>
@@ -6392,11 +7284,31 @@
       <c r="AF52" s="33" t="n"/>
       <c r="AG52" s="33" t="n"/>
       <c r="AH52" s="33" t="n"/>
-      <c r="AI52" s="33" t="n"/>
-      <c r="AJ52" s="33" t="n"/>
-      <c r="AK52" s="33" t="n"/>
-      <c r="AL52" s="33" t="n"/>
-      <c r="AM52" s="33" t="n"/>
+      <c r="AI52" s="33" t="inlineStr">
+        <is>
+          <t>nederland-&amp;-wereld, verdiepen</t>
+        </is>
+      </c>
+      <c r="AJ52" s="33" t="inlineStr">
+        <is>
+          <t>1.2.4.1, 1.2.4.2</t>
+        </is>
+      </c>
+      <c r="AK52" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL52" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM52" s="33" t="inlineStr">
+        <is>
+          <t>nl,de,en,es,fr,it,pt,ru</t>
+        </is>
+      </c>
       <c r="AN52" s="33" t="n"/>
       <c r="AO52" s="33" t="n"/>
       <c r="AP52" s="33" t="n"/>
@@ -6434,7 +7346,11 @@
           <t>dossiers en bronnen</t>
         </is>
       </c>
-      <c r="H53" s="11" t="inlineStr"/>
+      <c r="H53" s="11" t="inlineStr">
+        <is>
+          <t>Voor dossiers, primaire bronnen, het volledige archief, en wie er achter Het Open Vizier staat.</t>
+        </is>
+      </c>
       <c r="I53" s="10" t="inlineStr"/>
       <c r="J53" s="10" t="inlineStr">
         <is>
@@ -6453,7 +7369,7 @@
       </c>
       <c r="M53" s="10" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>bottom</t>
         </is>
       </c>
       <c r="N53" s="10" t="inlineStr">
@@ -6499,9 +7415,21 @@
       <c r="AH53" s="33" t="n"/>
       <c r="AI53" s="33" t="n"/>
       <c r="AJ53" s="33" t="n"/>
-      <c r="AK53" s="33" t="n"/>
-      <c r="AL53" s="33" t="n"/>
-      <c r="AM53" s="33" t="n"/>
+      <c r="AK53" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL53" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM53" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN53" s="33" t="n"/>
       <c r="AO53" s="33" t="n"/>
       <c r="AP53" s="33" t="n"/>
@@ -6608,9 +7536,21 @@
       <c r="AH54" s="33" t="n"/>
       <c r="AI54" s="33" t="n"/>
       <c r="AJ54" s="33" t="n"/>
-      <c r="AK54" s="33" t="n"/>
-      <c r="AL54" s="33" t="n"/>
-      <c r="AM54" s="33" t="n"/>
+      <c r="AK54" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL54" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM54" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN54" s="33" t="n"/>
       <c r="AO54" s="33" t="n"/>
       <c r="AP54" s="33" t="n"/>
@@ -6717,9 +7657,21 @@
       <c r="AH55" s="33" t="n"/>
       <c r="AI55" s="33" t="n"/>
       <c r="AJ55" s="33" t="n"/>
-      <c r="AK55" s="33" t="n"/>
-      <c r="AL55" s="33" t="n"/>
-      <c r="AM55" s="33" t="n"/>
+      <c r="AK55" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL55" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM55" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN55" s="33" t="n"/>
       <c r="AO55" s="33" t="n"/>
       <c r="AP55" s="33" t="n"/>
@@ -6826,9 +7778,21 @@
       <c r="AH56" s="33" t="n"/>
       <c r="AI56" s="33" t="n"/>
       <c r="AJ56" s="33" t="n"/>
-      <c r="AK56" s="33" t="n"/>
-      <c r="AL56" s="33" t="n"/>
-      <c r="AM56" s="33" t="n"/>
+      <c r="AK56" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL56" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM56" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN56" s="33" t="n"/>
       <c r="AO56" s="33" t="n"/>
       <c r="AP56" s="33" t="n"/>
@@ -6935,9 +7899,21 @@
       <c r="AH57" s="33" t="n"/>
       <c r="AI57" s="33" t="n"/>
       <c r="AJ57" s="33" t="n"/>
-      <c r="AK57" s="33" t="n"/>
-      <c r="AL57" s="33" t="n"/>
-      <c r="AM57" s="33" t="n"/>
+      <c r="AK57" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL57" s="33" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM57" s="33" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
       <c r="AN57" s="33" t="n"/>
       <c r="AO57" s="33" t="n"/>
       <c r="AP57" s="33" t="n"/>
@@ -6971,7 +7947,11 @@
         </is>
       </c>
       <c r="G58" s="8" t="inlineStr"/>
-      <c r="H58" s="8" t="inlineStr"/>
+      <c r="H58" s="8" t="inlineStr">
+        <is>
+          <t>Vertaling van Het Open Vizier in Deutsch — nog niet gevuld.</t>
+        </is>
+      </c>
       <c r="I58" s="7" t="inlineStr"/>
       <c r="J58" s="7" t="inlineStr"/>
       <c r="K58" s="7" t="inlineStr"/>
@@ -6997,7 +7977,7 @@
       <c r="W58" s="7" t="inlineStr"/>
       <c r="X58" s="8" t="inlineStr">
         <is>
-          <t>Nog niet gevuld</t>
+          <t>Activeer door 'actief' op TRUE en 'status' op 'live' te zetten. Voeg dan rijen toe met deze code als prefix.</t>
         </is>
       </c>
       <c r="Y58" s="33" t="n"/>
@@ -7012,7 +7992,11 @@
       <c r="AH58" s="33" t="n"/>
       <c r="AI58" s="33" t="n"/>
       <c r="AJ58" s="33" t="n"/>
-      <c r="AK58" s="33" t="n"/>
+      <c r="AK58" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="AL58" s="33" t="n"/>
       <c r="AM58" s="33" t="n"/>
       <c r="AN58" s="33" t="n"/>
@@ -7048,7 +8032,11 @@
         </is>
       </c>
       <c r="G59" s="8" t="inlineStr"/>
-      <c r="H59" s="8" t="inlineStr"/>
+      <c r="H59" s="8" t="inlineStr">
+        <is>
+          <t>Vertaling van Het Open Vizier in English — nog niet gevuld.</t>
+        </is>
+      </c>
       <c r="I59" s="7" t="inlineStr"/>
       <c r="J59" s="7" t="inlineStr"/>
       <c r="K59" s="7" t="inlineStr"/>
@@ -7074,7 +8062,7 @@
       <c r="W59" s="7" t="inlineStr"/>
       <c r="X59" s="8" t="inlineStr">
         <is>
-          <t>Nog niet gevuld</t>
+          <t>Activeer door 'actief' op TRUE en 'status' op 'live' te zetten. Voeg dan rijen toe met deze code als prefix.</t>
         </is>
       </c>
       <c r="Y59" s="33" t="n"/>
@@ -7089,7 +8077,11 @@
       <c r="AH59" s="33" t="n"/>
       <c r="AI59" s="33" t="n"/>
       <c r="AJ59" s="33" t="n"/>
-      <c r="AK59" s="33" t="n"/>
+      <c r="AK59" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="AL59" s="33" t="n"/>
       <c r="AM59" s="33" t="n"/>
       <c r="AN59" s="33" t="n"/>
@@ -7125,7 +8117,11 @@
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr"/>
-      <c r="H60" s="8" t="inlineStr"/>
+      <c r="H60" s="8" t="inlineStr">
+        <is>
+          <t>Vertaling van Het Open Vizier in Русский — nog niet gevuld.</t>
+        </is>
+      </c>
       <c r="I60" s="7" t="inlineStr"/>
       <c r="J60" s="7" t="inlineStr"/>
       <c r="K60" s="7" t="inlineStr"/>
@@ -7151,7 +8147,7 @@
       <c r="W60" s="7" t="inlineStr"/>
       <c r="X60" s="8" t="inlineStr">
         <is>
-          <t>Nog niet gevuld</t>
+          <t>Activeer door 'actief' op TRUE en 'status' op 'live' te zetten. Voeg dan rijen toe met deze code als prefix.</t>
         </is>
       </c>
       <c r="Y60" s="33" t="n"/>
@@ -7166,7 +8162,11 @@
       <c r="AH60" s="33" t="n"/>
       <c r="AI60" s="33" t="n"/>
       <c r="AJ60" s="33" t="n"/>
-      <c r="AK60" s="33" t="n"/>
+      <c r="AK60" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="AL60" s="33" t="n"/>
       <c r="AM60" s="33" t="n"/>
       <c r="AN60" s="33" t="n"/>
@@ -7202,7 +8202,11 @@
         </is>
       </c>
       <c r="G61" s="8" t="inlineStr"/>
-      <c r="H61" s="8" t="inlineStr"/>
+      <c r="H61" s="8" t="inlineStr">
+        <is>
+          <t>Vertaling van Het Open Vizier in Français — nog niet gevuld.</t>
+        </is>
+      </c>
       <c r="I61" s="7" t="inlineStr"/>
       <c r="J61" s="7" t="inlineStr"/>
       <c r="K61" s="7" t="inlineStr"/>
@@ -7228,7 +8232,7 @@
       <c r="W61" s="7" t="inlineStr"/>
       <c r="X61" s="8" t="inlineStr">
         <is>
-          <t>Nog niet gevuld</t>
+          <t>Activeer door 'actief' op TRUE en 'status' op 'live' te zetten. Voeg dan rijen toe met deze code als prefix.</t>
         </is>
       </c>
       <c r="Y61" s="33" t="n"/>
@@ -7243,7 +8247,11 @@
       <c r="AH61" s="33" t="n"/>
       <c r="AI61" s="33" t="n"/>
       <c r="AJ61" s="33" t="n"/>
-      <c r="AK61" s="33" t="n"/>
+      <c r="AK61" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="AL61" s="33" t="n"/>
       <c r="AM61" s="33" t="n"/>
       <c r="AN61" s="33" t="n"/>
@@ -7279,7 +8287,11 @@
         </is>
       </c>
       <c r="G62" s="8" t="inlineStr"/>
-      <c r="H62" s="8" t="inlineStr"/>
+      <c r="H62" s="8" t="inlineStr">
+        <is>
+          <t>Vertaling van Het Open Vizier in Español — nog niet gevuld.</t>
+        </is>
+      </c>
       <c r="I62" s="7" t="inlineStr"/>
       <c r="J62" s="7" t="inlineStr"/>
       <c r="K62" s="7" t="inlineStr"/>
@@ -7305,7 +8317,7 @@
       <c r="W62" s="7" t="inlineStr"/>
       <c r="X62" s="8" t="inlineStr">
         <is>
-          <t>Nog niet gevuld</t>
+          <t>Activeer door 'actief' op TRUE en 'status' op 'live' te zetten. Voeg dan rijen toe met deze code als prefix.</t>
         </is>
       </c>
       <c r="Y62" s="33" t="n"/>
@@ -7320,7 +8332,11 @@
       <c r="AH62" s="33" t="n"/>
       <c r="AI62" s="33" t="n"/>
       <c r="AJ62" s="33" t="n"/>
-      <c r="AK62" s="33" t="n"/>
+      <c r="AK62" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="AL62" s="33" t="n"/>
       <c r="AM62" s="33" t="n"/>
       <c r="AN62" s="33" t="n"/>
@@ -7356,7 +8372,11 @@
         </is>
       </c>
       <c r="G63" s="8" t="inlineStr"/>
-      <c r="H63" s="8" t="inlineStr"/>
+      <c r="H63" s="8" t="inlineStr">
+        <is>
+          <t>Vertaling van Het Open Vizier in Italiano — nog niet gevuld.</t>
+        </is>
+      </c>
       <c r="I63" s="7" t="inlineStr"/>
       <c r="J63" s="7" t="inlineStr"/>
       <c r="K63" s="7" t="inlineStr"/>
@@ -7382,7 +8402,7 @@
       <c r="W63" s="7" t="inlineStr"/>
       <c r="X63" s="8" t="inlineStr">
         <is>
-          <t>Nog niet gevuld</t>
+          <t>Activeer door 'actief' op TRUE en 'status' op 'live' te zetten. Voeg dan rijen toe met deze code als prefix.</t>
         </is>
       </c>
       <c r="Y63" s="33" t="n"/>
@@ -7397,7 +8417,11 @@
       <c r="AH63" s="33" t="n"/>
       <c r="AI63" s="33" t="n"/>
       <c r="AJ63" s="33" t="n"/>
-      <c r="AK63" s="33" t="n"/>
+      <c r="AK63" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="AL63" s="33" t="n"/>
       <c r="AM63" s="33" t="n"/>
       <c r="AN63" s="33" t="n"/>
@@ -7433,7 +8457,11 @@
         </is>
       </c>
       <c r="G64" s="8" t="inlineStr"/>
-      <c r="H64" s="8" t="inlineStr"/>
+      <c r="H64" s="8" t="inlineStr">
+        <is>
+          <t>Vertaling van Het Open Vizier in Português — nog niet gevuld.</t>
+        </is>
+      </c>
       <c r="I64" s="7" t="inlineStr"/>
       <c r="J64" s="7" t="inlineStr"/>
       <c r="K64" s="7" t="inlineStr"/>
@@ -7459,7 +8487,7 @@
       <c r="W64" s="7" t="inlineStr"/>
       <c r="X64" s="8" t="inlineStr">
         <is>
-          <t>Nog niet gevuld</t>
+          <t>Activeer door 'actief' op TRUE en 'status' op 'live' te zetten. Voeg dan rijen toe met deze code als prefix.</t>
         </is>
       </c>
       <c r="Y64" s="33" t="n"/>
@@ -7474,7 +8502,11 @@
       <c r="AH64" s="33" t="n"/>
       <c r="AI64" s="33" t="n"/>
       <c r="AJ64" s="33" t="n"/>
-      <c r="AK64" s="33" t="n"/>
+      <c r="AK64" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="AL64" s="33" t="n"/>
       <c r="AM64" s="33" t="n"/>
       <c r="AN64" s="33" t="n"/>
@@ -7510,7 +8542,11 @@
         </is>
       </c>
       <c r="G65" s="8" t="inlineStr"/>
-      <c r="H65" s="8" t="inlineStr"/>
+      <c r="H65" s="8" t="inlineStr">
+        <is>
+          <t>Vertaling van Het Open Vizier in Malti — nog niet gevuld.</t>
+        </is>
+      </c>
       <c r="I65" s="7" t="inlineStr"/>
       <c r="J65" s="7" t="inlineStr"/>
       <c r="K65" s="7" t="inlineStr"/>
@@ -7536,7 +8572,7 @@
       <c r="W65" s="7" t="inlineStr"/>
       <c r="X65" s="8" t="inlineStr">
         <is>
-          <t>Nog niet gevuld</t>
+          <t>Activeer door 'actief' op TRUE en 'status' op 'live' te zetten. Voeg dan rijen toe met deze code als prefix.</t>
         </is>
       </c>
       <c r="Y65" s="33" t="n"/>
@@ -7551,7 +8587,11 @@
       <c r="AH65" s="33" t="n"/>
       <c r="AI65" s="33" t="n"/>
       <c r="AJ65" s="33" t="n"/>
-      <c r="AK65" s="33" t="n"/>
+      <c r="AK65" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="AL65" s="33" t="n"/>
       <c r="AM65" s="33" t="n"/>
       <c r="AN65" s="33" t="n"/>
@@ -7573,7 +8613,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:F11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -7823,7 +8863,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -8098,7 +9138,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:D45"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -8866,7 +9906,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:C22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
fix(DE-menu): 29 DE-artikelen hernoemd naar NL-slug om menu-404 op te lossen
Het menu wordt vanuit één xlsx-URL-cel per artikel gegenereerd, en de
menu-generator vertaalt alleen mapnamen (wat-opkomt→was-aufkommt), niet
bestandsnamen. Wanneer NL en DE verschillende slugs hadden (bv. 'frankrijk-
revolutionair-moment.html' vs 'frankreich-revolutionaerer-moment.html'), gaf
de DE-versie een 404 in het menu.

Aanpak: DE-bestand hernoemd naar de NL-slug zodat het menu-URL werkt.

Ook op te lossen NL-rij:
- Rij 247 (Beleidsadvies aantrekken): URL van 'wat-opkomt/…' naar 'editie-2/…'
  (het bestand stond niet in wat-opkomt maar in editie-2)

29 DE-hernoemingen (23 zeker + 6 handmatig-gecheckte ambigue matches).
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -688,7 +688,6 @@
           <t>De talenring is het startscherm: kies een taal voor je verkennen.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>center</t>
@@ -769,7 +768,6 @@
           <t>Nederlandse uitgave van Het Open Vizier — onderzoeksjournalistiek over governance, energie en economie.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>center</t>
@@ -850,7 +848,6 @@
           <t>De vaste voorpagina van Het Open Vizier.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>center</t>
@@ -931,7 +928,6 @@
           <t>Partijen, campagnes, revolutie, media — wat er nu speelt.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>center</t>
@@ -1012,7 +1008,6 @@
           <t>Dimensies, oergevoel, samenhang, films en boeken.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>center</t>
@@ -1093,7 +1088,6 @@
           <t>Klimaatdividend, BiCRS, thermostaat, wereldgordel.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>center</t>
@@ -1174,7 +1168,6 @@
           <t>Nederland, Europa, andere landen, Nova Democratia.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>center</t>
@@ -1255,7 +1248,6 @@
           <t>Kantelmechanica, vergeten orde, veerkracht.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>center</t>
@@ -1336,7 +1328,6 @@
           <t>Vermogensvlucht, plundering, stemmetjeswinning, BBP.</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>center</t>
@@ -1417,7 +1408,6 @@
           <t>Onderzoeksrapporten, dossiers, achter-de-cijfers.</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>center</t>
@@ -1498,7 +1488,6 @@
           <t>Colofon, over, archief, structuur, talenring.</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>center</t>
@@ -1579,7 +1568,6 @@
           <t>Delen, verkennen, discussie, tien seconden.</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>center</t>
@@ -1755,7 +1743,6 @@
           <t>De artikelen onder Frankrijk &amp; Europese revolutie.</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>center</t>
@@ -2227,7 +2214,6 @@
           <t>De artikelen onder Kantelmechanica &amp; mensen.</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>center</t>
@@ -2298,7 +2284,6 @@
           <t>Kantelmechanica</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>Hoe een gedachtegoed kantelt naar invloed.</t>
@@ -2399,7 +2384,6 @@
           <t>Mensen die mee bouwen</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>Tropische ethanol-steden 2040. Een visionair stuk over wie Europa's energietoekomst kan helpen bouwen — als we de moed hebben de migratiekwestie en de energietransitie samen te denken. Goede huizen, scholen, bibliotheken, internet. Niet wegsturen, niet binnenhouden — verder gaan.</t>
@@ -2488,7 +2472,6 @@
           <t>Actievoerders bouwen continenten</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Drive zoekt grond. Wat hier schuurt, kan ginds bouwen. Een open uitnodiging aan organisaties met visie en aan iedereen die zijn energie zoekt waar zij iets kan opbouwen — niet als straf, niet als afvoer, maar als kans.</t>
@@ -2577,7 +2560,6 @@
           <t>Wie zijn opbouwers wegjaagt</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>Een waarneming van Jacobus van Merksteijn. Dit stuk is geen analyse, geen onderzoek en geen advies. Het is een observatie — bedoeld om ogen te openen en de discussie te voeden.</t>
@@ -2588,7 +2570,6 @@
           <t>opbouwers-wegjagen/index.html</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>center</t>
@@ -2769,7 +2750,6 @@
           <t>De artikelen onder Partijen &amp; pareto.</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
           <t>center</t>
@@ -2840,8 +2820,6 @@
           <t>Wie blokkeert, en hoe zwaar?</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>editie-6/aflevering-02-pareto-top12.html</t>
@@ -2927,8 +2905,6 @@
           <t>Waar staat uw partij?</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>editie-6/aflevering-08-partijen-in-kaart.html</t>
@@ -3014,8 +2990,6 @@
           <t>Wie verzet zich, wie helpt mee?</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>editie-6/aflevering-09-pareto-per-actor.html</t>
@@ -3101,8 +3075,6 @@
           <t>Ordes van bezwaar</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>editie-6/aflevering-04-ordes-van-bezwaar.html</t>
@@ -3188,8 +3160,6 @@
           <t>Twintig actuele bezwaren</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>editie-6/aflevering-05-twintig-bezwaren.html</t>
@@ -3275,7 +3245,6 @@
           <t>Plundering 4: politiek</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>Wie wil wat, en waarom Brussel niet weet hoe verder</t>
@@ -3386,7 +3355,6 @@
           <t>De artikelen onder Pers &amp; media.</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
           <t>center</t>
@@ -3653,7 +3621,6 @@
           <t>Trump als spiegel</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>Wat Trump-II met Europa doet.</t>
@@ -3754,8 +3721,6 @@
           <t>Media als rekstrook</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>editie-6/aflevering-03-media-als-rekstrook.html</t>
@@ -3841,7 +3806,6 @@
           <t>De anti-immuunziekte van Brussel maakt dat we arm worden</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>CBAM, ETS, Pillar Two en vermogensbelastingen tegelijk. De BiCRS/Ethanol-route wordt genegeerd. Brussel maakt zijn eigen inwoners arm.</t>
@@ -3852,7 +3816,6 @@
           <t>wat-opkomt/de-anti-immuunziekte-van-brussel.html</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
           <t>center</t>
@@ -3926,7 +3889,6 @@
           <t>De anti-immuunziekte van onze overheid slaat toe</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>Het kabinet-Jetten presenteert eind juni 2026 zijn stikstofpakket. Een aanval op het laatste productieve weefsel. En er is een andere weg.</t>
@@ -3937,7 +3899,6 @@
           <t>wat-opkomt/de-auto-immuunziekte-slaat-toe.html</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
           <t>center</t>
@@ -4011,7 +3972,6 @@
           <t>De dertig cent die Europa omdraait</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>Bio-ethanol uit cellulose-route haalt €0,30 per liter in 2036, zonder een cent subsidie. Combineer met de nieuwste brandstofcellen en je hebt stroom voor minder dan de helft van de Spaanse netprijs. In Den Haag, Berlijn en Brussel hoort u er niets over.</t>
@@ -4110,7 +4070,6 @@
           <t>De artikelen onder Stemgedrag &amp; keuzemomenten.</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
           <t>center</t>
@@ -4181,7 +4140,6 @@
           <t>Gevolgenkaart</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>Partij × Persoon × Basislijn = Projectie</t>
@@ -4192,7 +4150,6 @@
           <t>stemgedrag.html</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
           <t>center</t>
@@ -4459,7 +4416,6 @@
           <t>Op de bok of op de bagagedrager</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>Een sturend artikel. Wie nu niet ziet en aanpakt, zit straks weer achterin. Europa heeft een keuze: zelf de teugels nemen of zich laten leiden door Tokio, Seoul en Peking. De drie blokken — bron, omzetting, eindsysteem — zonder één cent subsidie. Eén route wint. Wie hem niet pakt, verliest.</t>
@@ -4548,7 +4504,6 @@
           <t>Eerst plukken, dan oordelen</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>De cirkel van onrecht waarin Europa zichzelf vernietigt</t>
@@ -4649,7 +4604,6 @@
           <t>Kies een kant</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>Het sluitstuk van de onderwijs-trilogie: wat wij wel kunnen redden, wat wij niet meer kunnen redden, en waarom u zich nu moet uitspreken.</t>
@@ -4740,7 +4694,6 @@
           <t>Waarom deze krant?</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>Voorwoord bij de eerste editie van Het Open Vizier. Over verbanden zien, intelligentie als kruisbestuiving, en waarom een onafhankelijke krant nodig is.</t>
@@ -4939,7 +4892,6 @@
           <t>De artikelen onder Zeven Dimensies &amp; denkraam.</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
           <t>center</t>
@@ -5201,7 +5153,6 @@
           <t>Drie dimensies zijn te weinig</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>Het 7D-denkraam uitgelegd: x, y, z, t, G (schaal), W (waarde van antimaterie tot materie) en N (veelvoud van universa). In gewone taal.</t>
@@ -5292,7 +5243,6 @@
           <t>Hoe alles samenhangt</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>De synthese van de eerste editie: hoe de 7D-denkwijze politiek, onderwijs, techniek en wetenschap met elkaar verbindt.</t>
@@ -5383,7 +5333,6 @@
           <t>Alles stroomt — moeder van alle wetenschap</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>Stromingsleer als universele taal: van scheepscoatings tot economie tot democratie. Een pleidooi voor vakoverschrijdend denken.</t>
@@ -5474,7 +5423,6 @@
           <t>Zeven Dimensies</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>Hoe G, W en N het standaardmodel verruimen — van vacuümstructuur tot quantum computing en nanotechnologie</t>
@@ -5575,7 +5523,6 @@
           <t>De artikelen onder Oergevoel &amp; Kosaris.</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
           <t>center</t>
@@ -5646,7 +5593,6 @@
           <t>Het oergevoel</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>Wat de eerste laag is en hoe wij hem voelen</t>
@@ -5737,7 +5683,6 @@
           <t>De zeven dimensies</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>Het 7D-model van menselijk gevoel</t>
@@ -5828,7 +5773,6 @@
           <t>De drie hersenlagen</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>Oergevoel, zoogdierbrein, mensenbrein</t>
@@ -5919,7 +5863,6 @@
           <t>Communicatie tussen oergevoelens</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>Hoogfrequente gravitatie en het voorhoofdsbeen</t>
@@ -6010,7 +5953,6 @@
           <t>Wat we kinderen aandoen</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
           <t>De systematische uitknijping</t>
@@ -6101,7 +6043,6 @@
           <t>Mama ik heb honger</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>De voortdurende aanwezigheid en wat afwezigheid kost</t>
@@ -6192,7 +6133,6 @@
           <t>Het oergevoel in de beroepspraktijk</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
           <t>Verkoper, baas, consultant en bankier — vier beroepen, één instrument</t>
@@ -6283,7 +6223,6 @@
           <t>De mens onder het ijs — Het Open Vizier · Editie 3 — Juni 2026</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>Een gedachtegoed over het oergevoel, het driedubbele brein, en de mens die wij niet meer opleiden.</t>
@@ -6294,7 +6233,6 @@
           <t>editie-3/index.html</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr">
         <is>
           <t>center</t>
@@ -6365,7 +6303,6 @@
           <t>Manifest Oergevoel</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
           <t>Ruimte voor het oergevoel.</t>
@@ -6466,7 +6403,6 @@
           <t>Waarom ik ben zoals ik ben</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
           <t>Over de uitkomst aan het eind, en de mensen die alleen aan morgen denken</t>
@@ -6567,7 +6503,6 @@
           <t>De artikelen onder Films, sprookjes, leesboek.</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr">
         <is>
           <t>center</t>
@@ -6638,7 +6573,6 @@
           <t>De 7-Dim Film</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>De Zeven Dimensies — een filmisch essay van tien minuten over de zeven fundamentele assen van de werkelijkheid: x, y, z, t, G, W en N. Door Jacobus van Merksteijn.</t>
@@ -6649,7 +6583,6 @@
           <t>7-dim-film/index.html</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr">
         <is>
           <t>center</t>
@@ -6720,7 +6653,6 @@
           <t>De Kosaris — De Film</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
           <t>De Kosaris — een filmisch essay van elf minuten over de vier zuilen die dragen: Chronesis, Philotimos, Aletheris en Timaris. Twaalf hoofdstukken. Door Jacobus van Merksteijn.</t>
@@ -6731,7 +6663,6 @@
           <t>kosaris-film/index.html</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr">
         <is>
           <t>center</t>
@@ -6802,7 +6733,6 @@
           <t>De Kosaris — Leesboek</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>De Kosaris, Boek Eén: het volledige leesboek van Jacobus van Merksteijn, met de vier zuilen Chronesis, Philotimos, Aletheris en Timaris.</t>
@@ -6813,7 +6743,6 @@
           <t>leesboek/index.html</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr">
         <is>
           <t>center</t>
@@ -6884,7 +6813,6 @@
           <t>Het sprookje van Jacobus</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>Een sprookje voor kinderen om te horen, en voor volwassenen om te herkennen. Elke pagina heeft twee lezingen: het sprookje in beeld en woord, en de volwassen betekenis ernaast.</t>
@@ -6895,7 +6823,6 @@
           <t>sprookjes/index.html</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr"/>
       <c r="K73" t="inlineStr">
         <is>
           <t>center</t>
@@ -6966,7 +6893,6 @@
           <t>Filosofie</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
           <t>Wat ligt onder de keuzes die wij maken? Welke begrippen dragen onze instellingen, en welke begrippen kunnen wij nog niet missen omdat wij ze nog niet hebben uitgedacht? De Filosofie-sectie verzamelt manifesten en essays die de grondslagen ter discussie stellen — niet als debatkunst, maar als oefening in vrijer denken.</t>
@@ -6977,7 +6903,6 @@
           <t>filosofie/index.html</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr">
         <is>
           <t>center</t>
@@ -7058,7 +6983,6 @@
           <t>De artikelen onder Gevoelsconnectiesysteem.</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr"/>
       <c r="K75" t="inlineStr">
         <is>
           <t>center</t>
@@ -7129,7 +7053,6 @@
           <t>Het gevoelsconnectiesysteem</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>Een onderzoeksplan over de basale menselijke gevoelslaag, nachtelijke integratie van dagkennis, foutdetectie in opvoeding en leiderschap, en de hypothese van een fysiek kanaal voor gevoel-naar-gevoel-overdracht.</t>
@@ -7140,7 +7063,6 @@
           <t>onderzoeken/gevoelsconnectiesysteem.html</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr"/>
       <c r="K76" t="inlineStr">
         <is>
           <t>center</t>
@@ -7211,7 +7133,6 @@
           <t>Het gevoelsconnectiesysteem — volledig onderzoeksplan</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
           <t>Volledig onderzoeksplan over het basaal menselijke gevoelsconnectiesysteem, nachtelijke integratie van verstand naar gevoel, foutdetectie als sleutelvariabele, en de hypothese van menselijke gravitatiegolven als drager.</t>
@@ -7222,7 +7143,6 @@
           <t>onderzoeken/gevoelsconnectiesysteem-volledig.html</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr"/>
       <c r="K77" t="inlineStr">
         <is>
           <t>center</t>
@@ -7293,7 +7213,6 @@
           <t>Krantbriefing — gevoelsconnectiesysteem</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
           <t>Journalistieke briefingtekst over het gevoelsconnectiesysteem, nachtelijke integratie en de hypothese van menselijke gravitatiegolven — voor een collega die het onderwerp in krantstijl wil uitwerken.</t>
@@ -7304,7 +7223,6 @@
           <t>onderzoeken/krantbriefing.html</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr">
         <is>
           <t>center</t>
@@ -7375,7 +7293,6 @@
           <t>Routekaart van vervolgvragen</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
           <t>Vierentwintig vervolgvragen rond het gevoelsconnectiesysteem, in acht fasen — van begrippen naar detector. Een werkroute voor wie wil meedenken.</t>
@@ -7386,7 +7303,6 @@
           <t>onderzoeken/routekaart-vervolgvragen.html</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr">
         <is>
           <t>center</t>
@@ -7467,7 +7383,6 @@
           <t>De artikelen onder Klimaatdividend &amp; oversterfte.</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr">
         <is>
           <t>center</t>
@@ -7844,7 +7759,6 @@
           <t>De artikelen onder BiCRS &amp; Carbon-Alert.</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr">
         <is>
           <t>center</t>
@@ -7915,7 +7829,6 @@
           <t>Visie 2036 — Carbon-Alert Energie-Hub</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>Het technische ontwerp van de 100 kW Carbon-Alert energie-hub. LCOE-analyse, vijf bouwblokken, kasstroom, risico-matrix. Het bewijs onder het sturend artikel — alle cijfers zonder subsidie.</t>
@@ -8004,7 +7917,6 @@
           <t>BiCRS-versie EU</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>Volledige doorrekening Brussel met BiCRS-vervanging.</t>
@@ -8203,7 +8115,6 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
           <t>Carbon-Alert op Europese schaal: zes miljoen hectare koolzaad, twintig miljoen ton sojaschroot-import, en het volledige GLB-budget. Wat verandert er als de architectuur op een derde van het Europese koolzaadareaal wordt toegepast — en wat krijgt Brussel ervoor terug?</t>
@@ -8214,7 +8125,6 @@
           <t>editie-0/carbon-alert-europa.html</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr">
         <is>
           <t>center</t>
@@ -8285,7 +8195,6 @@
           <t>De biomimetische krachtcentrale</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
           <t>Whitepaper Carbon-Alert R&amp;D: het optimaalste systeem voor energieverwerking uit biomassa over 25, 50 en 100 jaar. Drie horizonten — 2050, 2075, 2125 — met membranen, katalysatoren, actuators en kunstmatige fotosynthese.</t>
@@ -8296,7 +8205,6 @@
           <t>editie-0/biomimetische-krachtcentrale.html</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr">
         <is>
           <t>center</t>
@@ -8367,7 +8275,6 @@
           <t>Editie Europa</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
           <t>Wat Brussel, Den Haag, Berlijn en Malta cumulatief doen met de huishoudens van het continent — gespiegeld in wat Trump-II tegenover ze zet. Zeven stukken d</t>
@@ -8378,7 +8285,6 @@
           <t>editie-0/index.html</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr">
         <is>
           <t>center</t>
@@ -8459,7 +8365,6 @@
           <t>De artikelen onder Thermostaat &amp; fysieke aarde.</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr">
         <is>
           <t>center</t>
@@ -8530,7 +8435,6 @@
           <t>Uw thermostaat is slimmer dan uw minister</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>En dat is geen grapje. Dat is wiskunde.</t>
@@ -8621,7 +8525,6 @@
           <t>NEPK-FX — Neurale Voorspelling</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>Hoe de NEPK-formule structurele wisselkoersrichting voorspelt. Met concrete handelssignalen op basis van zes-maands en twaalf-maands neurale-netwerkprojecties.</t>
@@ -8712,7 +8615,6 @@
           <t>De NEPK-Klimaatlogica</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>Waarom de Nederlandse economische implosie sneller gaat dan verwacht</t>
@@ -8803,7 +8705,6 @@
           <t>De zon staat op de evenaar</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
           <t>Een Socratische confrontatie met de Nederlandse en Europese energieroute. Vijf oogkleppen, één route die wel werkt, en Europa terug op de leiderschapstroon — niet door overheersing, maar door partnerschap met de evenaar.</t>
@@ -8902,7 +8803,6 @@
           <t>De artikelen onder Autoband, plastic, vervuiling.</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr">
         <is>
           <t>center</t>
@@ -8973,7 +8873,6 @@
           <t>Autoband-sigaret</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
           <t>Bandenslijtage als verborgen vervuilingsdrager.</t>
@@ -9074,7 +8973,6 @@
           <t>De voedingslijn</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
           <t>De durf om revolutionair te zeggen dat het niet klopt ontbreekt door gebrek aan eigenkennis — een structurele fout. Heel Europa heeft zijn omwegen dichtgemetseld. De wetten van mensen kennen de toekomst niet; de natuur kent haar wel en moet weer voorop staan.</t>
@@ -9085,7 +8983,6 @@
           <t>wat-opkomt/de-methodologie-van-de-aanpassing.html</t>
         </is>
       </c>
-      <c r="J98" t="inlineStr"/>
       <c r="K98" t="inlineStr">
         <is>
           <t>center</t>
@@ -9159,7 +9056,6 @@
           <t>Natuur-analyse</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
           <t>Nederlandse cascade onder twee biomassa-sporen.</t>
@@ -9270,7 +9166,6 @@
           <t>De artikelen onder Editie Klimaat / Stikstof / Duitsland.</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr"/>
       <c r="K100" t="inlineStr">
         <is>
           <t>center</t>
@@ -9341,7 +9236,6 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
           <t>Editie Klimaat — energie, mobiliteit, verwarming, voedsel, migratie en CO₂-verwijdering. Een brede thematische editie van Het Open Vizier rond de klimaatkeuze die Europa vandaag voor zich heeft.</t>
@@ -9352,7 +9246,6 @@
           <t>editie-klimaat/index.html</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
       <c r="K101" t="inlineStr">
         <is>
           <t>center</t>
@@ -9423,7 +9316,6 @@
           <t>Editie Stikstof</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
         <is>
           <t>Alle artikelen die met de Nederlandse stikstofcrisis te maken hebben: de oplossing-architectuur, de diagnose van het beleidsfalen, het Europese kader, en de geografie van wat verhuist.</t>
@@ -9434,7 +9326,6 @@
           <t>editie-stikstof/index.html</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr"/>
       <c r="K102" t="inlineStr">
         <is>
           <t>center</t>
@@ -9505,7 +9396,6 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
         <is>
           <t>Hoe één architectuur — vorstbestendige Juncao met koude druk-explosie en mechanische verfijning — de Nederlandse stikstofcrisis, het methaan-probleem en de soja-afhankelijkheid tegelijk oplost. Met een vierde, vergeten winnaar: de boer in het transitiegebied.</t>
@@ -9516,7 +9406,6 @@
           <t>editie-stikstof/drie-problemen-een-antwoord.html</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr"/>
       <c r="K103" t="inlineStr">
         <is>
           <t>center</t>
@@ -9587,7 +9476,6 @@
           <t>Editie Duitsland</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
           <t>Carbon-Alert in Brandenburg en Mecklenburg-Voor-Pommeren, de Konsequenzkarte als instrument, en de spiegel van andere Europese landen. Met een doorverwijzing naar het Europese verhaal in Editie Europa.</t>
@@ -9598,7 +9486,6 @@
           <t>editie-duitsland/index.html</t>
         </is>
       </c>
-      <c r="J104" t="inlineStr"/>
       <c r="K104" t="inlineStr">
         <is>
           <t>center</t>
@@ -9669,7 +9556,6 @@
           <t>De Koolzaad-Multiplicator</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr">
         <is>
           <t>Brandenburg en Mecklenburg-Voor-Pommeren bouwen vandaag op circa 285.000 hectare winterkoolzaad. Met de Carbon-Alert-architectuur — vorstbestendige Juncao plus koude druk-explosie met mechanische verfijning — is op dezelfde hectare een veelvoud aan opbrengst te behalen, ingebed in het GLB-Strategisch Plan 2023-2027.</t>
@@ -9680,7 +9566,6 @@
           <t>editie-duitsland/raps-multiplicator-oost-duitsland.html</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr">
         <is>
           <t>center</t>
@@ -9761,7 +9646,6 @@
           <t>De artikelen onder Wat het niet ziet.</t>
         </is>
       </c>
-      <c r="J106" t="inlineStr"/>
       <c r="K106" t="inlineStr">
         <is>
           <t>center</t>
@@ -9832,7 +9716,6 @@
           <t>Actievoerders bouwen continenten</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
           <t>Drive zoekt grond. Wat hier schuurt, kan ginds bouwen. Een open uitnodiging aan organisaties met visie en aan iedereen die zijn energie zoekt waar zij iets kan opbouwen — niet als straf, niet als afvoer, maar als kans.</t>
@@ -9921,7 +9804,6 @@
           <t>De boer én de natuur beide vooruit</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
           <t>Van driehoeksdilemma naar vier scenario's — inclusief de radicale koevrije randzone die vijftien jaar CO₂ vangt, biodiversiteit herstelt en Natura 2000 laat ademen. Met kosten-baten-tabel per hectare per jaar.</t>
@@ -9932,7 +9814,6 @@
           <t>wat-opkomt/boer-en-natuur-beide-vooruit.html</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr"/>
       <c r="K108" t="inlineStr">
         <is>
           <t>center</t>
@@ -10201,7 +10082,6 @@
           <t>Zij doden hun levensader</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr">
         <is>
           <t>Brussel en Den Haag hebben een auto-immuunziekte. De patiënt heet Nederland. Diagnose, medische parallel, behandeling — in snijdende vorm.</t>
@@ -10212,7 +10092,6 @@
           <t>wat-opkomt/zij-doden-hun-levensader.html</t>
         </is>
       </c>
-      <c r="J111" t="inlineStr"/>
       <c r="K111" t="inlineStr">
         <is>
           <t>center</t>
@@ -10286,7 +10165,6 @@
           <t>Zij doden hun levensaders — Brussel</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
           <t>Brussel heeft een auto-immuunziekte. De patiënt heet Europa. Diagnose, medische parallel, behandeling — in snijdende vorm.</t>
@@ -10297,7 +10175,6 @@
           <t>wat-opkomt/zij-doden-hun-levensaders-brussel.html</t>
         </is>
       </c>
-      <c r="J112" t="inlineStr"/>
       <c r="K112" t="inlineStr">
         <is>
           <t>center</t>
@@ -10368,7 +10245,6 @@
           <t>Een fusiereactor zonder magnetische kooi</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr">
         <is>
           <t>Een alternatief reactorontwerp: de conische vortexreactor. Plasma wordt niet opgesloten met magneten maar versneld in een ronddraaiende stroming, vergelijkbaar met water in een wervel.</t>
@@ -10459,7 +10335,6 @@
           <t>Wat er nu al ligt</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr">
         <is>
           <t>Overzicht van technische projecten: SeaSkin, GuardSkin, AeroSkin, SolarSkin, TerraClean, Tyre-patenten, conische vortex-reactor.</t>
@@ -10560,7 +10435,6 @@
           <t>De artikelen onder Nederland.</t>
         </is>
       </c>
-      <c r="J115" t="inlineStr"/>
       <c r="K115" t="inlineStr">
         <is>
           <t>center</t>
@@ -10631,7 +10505,6 @@
           <t>Stille Analyse (NL)</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr">
         <is>
           <t>20 NL-posities × 11 mechanismen, met BiCRS-uitweg.</t>
@@ -10732,7 +10605,6 @@
           <t>Zelf aan de bak (NL)</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr">
         <is>
           <t>Nederland moet zijn eigen kracht terugvinden.</t>
@@ -11129,7 +11001,6 @@
           <t>De eerste gemeente</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
         <is>
           <t>Een open en eerlijk voorstel aan wie het aandurft</t>
@@ -11140,7 +11011,6 @@
           <t>de-eerste-gemeente/index.html</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr"/>
       <c r="K121" t="inlineStr">
         <is>
           <t>center</t>
@@ -11211,7 +11081,6 @@
           <t>De halve gemeente</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr">
         <is>
           <t>Wat gebeurt er met een stad als de helft van het stadhuis verdwijnt?</t>
@@ -11222,7 +11091,6 @@
           <t>de-halve-gemeente/index.html</t>
         </is>
       </c>
-      <c r="J122" t="inlineStr"/>
       <c r="K122" t="inlineStr">
         <is>
           <t>center</t>
@@ -11293,7 +11161,6 @@
           <t>Nederland · Toekomst</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr">
         <is>
           <t>Drie hervormingen voor Nederland: van fiscaal beleid via een modern selectiesysteem naar de partijen op de kaart. Wat lokaal mogelijk is op basis van het Open Vizier-gedachtegoed.</t>
@@ -11304,7 +11171,6 @@
           <t>toekomst/overheden/nederland/index.html</t>
         </is>
       </c>
-      <c r="J123" t="inlineStr"/>
       <c r="K123" t="inlineStr">
         <is>
           <t>center</t>
@@ -11375,7 +11241,6 @@
           <t>Gevolgenkaart Nederland</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -11386,7 +11251,6 @@
           <t>gevolgenkaart-nl/index.html</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr"/>
       <c r="K124" t="inlineStr">
         <is>
           <t>center</t>
@@ -11467,7 +11331,6 @@
           <t>De artikelen onder Europa.</t>
         </is>
       </c>
-      <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr">
         <is>
           <t>center</t>
@@ -11538,7 +11401,6 @@
           <t>Europa-opener</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr">
         <is>
           <t>Hoe BiCRS Green Deal en CBAM kan vervangen.</t>
@@ -11732,7 +11594,6 @@
           <t>Brusselse (EU)</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
           <t>20 EU-scenario's × 11 mechanismen.</t>
@@ -11833,7 +11694,6 @@
           <t>De anti-immuunziekte van Brussel maakt dat we arm worden</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr">
         <is>
           <t>CBAM, ETS, Pillar Two en vermogensbelastingen tegelijk. De BiCRS/Ethanol-route wordt genegeerd. Brussel maakt zijn eigen inwoners arm.</t>
@@ -11844,7 +11704,6 @@
           <t>wat-opkomt/de-anti-immuunziekte-van-brussel.html</t>
         </is>
       </c>
-      <c r="J129" t="inlineStr"/>
       <c r="K129" t="inlineStr">
         <is>
           <t>center</t>
@@ -11918,7 +11777,6 @@
           <t>De anti-immuunziekte van onze overheid slaat toe</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr">
         <is>
           <t>Het kabinet-Jetten presenteert eind juni 2026 zijn stikstofpakket. Een aanval op het laatste productieve weefsel. En er is een andere weg.</t>
@@ -11929,7 +11787,6 @@
           <t>wat-opkomt/de-auto-immuunziekte-slaat-toe.html</t>
         </is>
       </c>
-      <c r="J130" t="inlineStr"/>
       <c r="K130" t="inlineStr">
         <is>
           <t>center</t>
@@ -12003,7 +11860,6 @@
           <t>Een staat met een auto-immuunziekte</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr">
         <is>
           <t>Een zachte, beschouwende uitleg van de medische metafoor die de Brussel-campagne van Het Open Vizier draagt. Geen aanklacht, maar een beeld om mee te denken.</t>
@@ -12014,7 +11870,6 @@
           <t>wat-opkomt/de-metafoor-auto-immuunziekte.html</t>
         </is>
       </c>
-      <c r="J131" t="inlineStr"/>
       <c r="K131" t="inlineStr">
         <is>
           <t>center</t>
@@ -12088,7 +11943,6 @@
           <t>Het immuunsysteem dat gezonde cellen aanvalt</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr">
         <is>
           <t>Waarom organisaties en politieke systemen rebellen reflexmatig uitstoten — niet uit kwaad opzet, maar uit zelfbehoud. Een opinie over hoe biomass-to-ethanol als gezonde cel in Brussel als ziektekiem wordt aangevallen, en hoe we dit immuunsysteem kunnen omzeilen.</t>
@@ -12099,7 +11953,6 @@
           <t>wat-opkomt/het-immuunsysteem-van-organisaties.html</t>
         </is>
       </c>
-      <c r="J132" t="inlineStr"/>
       <c r="K132" t="inlineStr">
         <is>
           <t>center</t>
@@ -12170,7 +12023,6 @@
           <t>Open brief aan de regeringen van Europa</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr">
         <is>
           <t>Een open brief aan de Europese Commissie, lidstaatregeringen en parlementen. 350.000 banen, €9 miljard jaaromzet, energie-onafhankelijkheid — zonder één eurocent subsidie. Begin nu met Carbon-Alert.</t>
@@ -12259,7 +12111,6 @@
           <t>De dertig cent die Europa omdraait</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr">
         <is>
           <t>Bio-ethanol uit cellulose-route haalt €0,30 per liter in 2036, zonder een cent subsidie. Combineer met de nieuwste brandstofcellen en je hebt stroom voor minder dan de helft van de Spaanse netprijs. In Den Haag, Berlijn en Brussel hoort u er niets over.</t>
@@ -12544,7 +12395,6 @@
           <t>Zij doden hun levensaders — Brussel</t>
         </is>
       </c>
-      <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr">
         <is>
           <t>Brussel heeft een auto-immuunziekte. De patiënt heet Europa. Diagnose, medische parallel, behandeling — in snijdende vorm.</t>
@@ -12555,7 +12405,6 @@
           <t>wat-opkomt/zij-doden-hun-levensaders-brussel.html</t>
         </is>
       </c>
-      <c r="J137" t="inlineStr"/>
       <c r="K137" t="inlineStr">
         <is>
           <t>center</t>
@@ -12626,7 +12475,6 @@
           <t>Gevolgenkaart Europa (EU-27)</t>
         </is>
       </c>
-      <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -12637,7 +12485,6 @@
           <t>gevolgenkaart-eu/index.html</t>
         </is>
       </c>
-      <c r="J138" t="inlineStr"/>
       <c r="K138" t="inlineStr">
         <is>
           <t>center</t>
@@ -12708,7 +12555,6 @@
           <t>Europa · Toekomst</t>
         </is>
       </c>
-      <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr">
         <is>
           <t>Hoe Brussel anders kan werken — niet als regeltool maar als ontwerpper. Wat de Carbon-Alert-architectuur teruggeeft, en welke tegenmacht uit Zwitserland tegen blokkades helpt.</t>
@@ -12719,7 +12565,6 @@
           <t>toekomst/overheden/europa/index.html</t>
         </is>
       </c>
-      <c r="J139" t="inlineStr"/>
       <c r="K139" t="inlineStr">
         <is>
           <t>center</t>
@@ -12800,7 +12645,6 @@
           <t>De artikelen onder Andere landen.</t>
         </is>
       </c>
-      <c r="J140" t="inlineStr"/>
       <c r="K140" t="inlineStr">
         <is>
           <t>center</t>
@@ -12871,7 +12715,6 @@
           <t>Gevolgenkaart Brazilië</t>
         </is>
       </c>
-      <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -12882,7 +12725,6 @@
           <t>gevolgenkaart-br/index.html</t>
         </is>
       </c>
-      <c r="J141" t="inlineStr"/>
       <c r="K141" t="inlineStr">
         <is>
           <t>center</t>
@@ -12953,7 +12795,6 @@
           <t>Gevolgenkaart Zwitserland</t>
         </is>
       </c>
-      <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -12964,7 +12805,6 @@
           <t>gevolgenkaart-ch/index.html</t>
         </is>
       </c>
-      <c r="J142" t="inlineStr"/>
       <c r="K142" t="inlineStr">
         <is>
           <t>center</t>
@@ -13035,7 +12875,6 @@
           <t>Zwitserse</t>
         </is>
       </c>
-      <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr">
         <is>
           <t>15 Zwitserse scenario's × Bondsraad-beleid + BiCRS.</t>
@@ -13136,7 +12975,6 @@
           <t>Gevolgenkaart China</t>
         </is>
       </c>
-      <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13147,7 +12985,6 @@
           <t>gevolgenkaart-cn/index.html</t>
         </is>
       </c>
-      <c r="J144" t="inlineStr"/>
       <c r="K144" t="inlineStr">
         <is>
           <t>center</t>
@@ -13218,7 +13055,6 @@
           <t>Gevolgenkaart Cuba</t>
         </is>
       </c>
-      <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13229,7 +13065,6 @@
           <t>gevolgenkaart-cu/index.html</t>
         </is>
       </c>
-      <c r="J145" t="inlineStr"/>
       <c r="K145" t="inlineStr">
         <is>
           <t>center</t>
@@ -13300,7 +13135,6 @@
           <t>Gevolgenkaart Duitsland</t>
         </is>
       </c>
-      <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13311,7 +13145,6 @@
           <t>gevolgenkaart-de/index.html</t>
         </is>
       </c>
-      <c r="J146" t="inlineStr"/>
       <c r="K146" t="inlineStr">
         <is>
           <t>center</t>
@@ -13382,7 +13215,6 @@
           <t>Konsequenzkarte (DE)</t>
         </is>
       </c>
-      <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr">
         <is>
           <t>Duitse spiegel, Bundestag februari 2025.</t>
@@ -13483,7 +13315,6 @@
           <t>Gevolgenkaart Spanje</t>
         </is>
       </c>
-      <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13494,7 +13325,6 @@
           <t>gevolgenkaart-es/index.html</t>
         </is>
       </c>
-      <c r="J148" t="inlineStr"/>
       <c r="K148" t="inlineStr">
         <is>
           <t>center</t>
@@ -13565,7 +13395,6 @@
           <t>Gevolgenkaart Israël</t>
         </is>
       </c>
-      <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13576,7 +13405,6 @@
           <t>gevolgenkaart-il/index.html</t>
         </is>
       </c>
-      <c r="J149" t="inlineStr"/>
       <c r="K149" t="inlineStr">
         <is>
           <t>center</t>
@@ -13647,7 +13475,6 @@
           <t>Gevolgenkaart India</t>
         </is>
       </c>
-      <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13658,7 +13485,6 @@
           <t>gevolgenkaart-in/index.html</t>
         </is>
       </c>
-      <c r="J150" t="inlineStr"/>
       <c r="K150" t="inlineStr">
         <is>
           <t>center</t>
@@ -13729,7 +13555,6 @@
           <t>Gevolgenkaart Iran</t>
         </is>
       </c>
-      <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13740,7 +13565,6 @@
           <t>gevolgenkaart-ir/index.html</t>
         </is>
       </c>
-      <c r="J151" t="inlineStr"/>
       <c r="K151" t="inlineStr">
         <is>
           <t>center</t>
@@ -13811,7 +13635,6 @@
           <t>Gevolgenkaart Japan</t>
         </is>
       </c>
-      <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13822,7 +13645,6 @@
           <t>gevolgenkaart-jp/index.html</t>
         </is>
       </c>
-      <c r="J152" t="inlineStr"/>
       <c r="K152" t="inlineStr">
         <is>
           <t>center</t>
@@ -13893,7 +13715,6 @@
           <t>Gevolgenkaart Zuid-Korea</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13904,7 +13725,6 @@
           <t>gevolgenkaart-kr/index.html</t>
         </is>
       </c>
-      <c r="J153" t="inlineStr"/>
       <c r="K153" t="inlineStr">
         <is>
           <t>center</t>
@@ -13975,7 +13795,6 @@
           <t>Gevolgenkaart Zweden</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13986,7 +13805,6 @@
           <t>gevolgenkaart-se/index.html</t>
         </is>
       </c>
-      <c r="J154" t="inlineStr"/>
       <c r="K154" t="inlineStr">
         <is>
           <t>center</t>
@@ -14057,7 +13875,6 @@
           <t>Gevolgenkaart Suriname</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -14068,7 +13885,6 @@
           <t>gevolgenkaart-sr/index.html</t>
         </is>
       </c>
-      <c r="J155" t="inlineStr"/>
       <c r="K155" t="inlineStr">
         <is>
           <t>center</t>
@@ -14139,7 +13955,6 @@
           <t>Gevolgenkaart Taiwan</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -14150,7 +13965,6 @@
           <t>gevolgenkaart-tw/index.html</t>
         </is>
       </c>
-      <c r="J156" t="inlineStr"/>
       <c r="K156" t="inlineStr">
         <is>
           <t>center</t>
@@ -14221,7 +14035,6 @@
           <t>Gevolgenkaart Verenigd Koninkrijk</t>
         </is>
       </c>
-      <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -14232,7 +14045,6 @@
           <t>gevolgenkaart-uk/index.html</t>
         </is>
       </c>
-      <c r="J157" t="inlineStr"/>
       <c r="K157" t="inlineStr">
         <is>
           <t>center</t>
@@ -14303,7 +14115,6 @@
           <t>Gevolgenkaart de Verenigde Staten</t>
         </is>
       </c>
-      <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -14314,7 +14125,6 @@
           <t>gevolgenkaart-us/index.html</t>
         </is>
       </c>
-      <c r="J158" t="inlineStr"/>
       <c r="K158" t="inlineStr">
         <is>
           <t>center</t>
@@ -14385,7 +14195,6 @@
           <t>Gevolgenkaart Zuid-Afrika</t>
         </is>
       </c>
-      <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -14396,7 +14205,6 @@
           <t>gevolgenkaart-za/index.html</t>
         </is>
       </c>
-      <c r="J159" t="inlineStr"/>
       <c r="K159" t="inlineStr">
         <is>
           <t>center</t>
@@ -14467,7 +14275,6 @@
           <t>Mappa Malta</t>
         </is>
       </c>
-      <c r="G160" t="inlineStr"/>
       <c r="H160" t="inlineStr">
         <is>
           <t>Maltese politiek en EU-druk samen.</t>
@@ -14568,7 +14375,6 @@
           <t>Singaporese</t>
         </is>
       </c>
-      <c r="G161" t="inlineStr"/>
       <c r="H161" t="inlineStr">
         <is>
           <t>15 SG scenario's × MOF/MAS/MOM + BiCRS-uitweg.</t>
@@ -14669,7 +14475,6 @@
           <t>Trump als spiegel</t>
         </is>
       </c>
-      <c r="G162" t="inlineStr"/>
       <c r="H162" t="inlineStr">
         <is>
           <t>Wat Trump-II met Europa doet.</t>
@@ -14770,7 +14575,6 @@
           <t>Duitsland · Toekomst</t>
         </is>
       </c>
-      <c r="G163" t="inlineStr"/>
       <c r="H163" t="inlineStr">
         <is>
           <t>Een eerste artikel over Duitsland: de Koolzaad-Multiplicator als regionale uitvoering van de Carbon-Alert-architectuur in Brandenburg en Mecklenburg-Voor-Pommeren.</t>
@@ -14781,7 +14585,6 @@
           <t>toekomst/overheden/duitsland/index.html</t>
         </is>
       </c>
-      <c r="J163" t="inlineStr"/>
       <c r="K163" t="inlineStr">
         <is>
           <t>center</t>
@@ -14862,7 +14665,6 @@
           <t>De artikelen onder Nova Democratia &amp; institutioneel ontwerp.</t>
         </is>
       </c>
-      <c r="J164" t="inlineStr"/>
       <c r="K164" t="inlineStr">
         <is>
           <t>center</t>
@@ -14933,7 +14735,6 @@
           <t>Nova Democratia — Het Open Vizier · Editie 6 — Juni 2026</t>
         </is>
       </c>
-      <c r="G165" t="inlineStr"/>
       <c r="H165" t="inlineStr">
         <is>
           <t>Een editie over de fysica van de Nederlandse hervorming — Pareto, ordes, het ontwerp dat werkt, en de kennislaag die de behoudende kracht draagt. Veertien stukken.</t>
@@ -14944,7 +14745,6 @@
           <t>editie-6/index.html</t>
         </is>
       </c>
-      <c r="J165" t="inlineStr"/>
       <c r="K165" t="inlineStr">
         <is>
           <t>center</t>
@@ -15015,8 +14815,6 @@
           <t>Voorwoord — Waarom dit moet</t>
         </is>
       </c>
-      <c r="G166" t="inlineStr"/>
-      <c r="H166" t="inlineStr"/>
       <c r="I166" t="inlineStr">
         <is>
           <t>editie-6/voorwoord-waarom-dit-moet.html</t>
@@ -15102,8 +14900,6 @@
           <t>Brussel als variabele, niet als constante</t>
         </is>
       </c>
-      <c r="G167" t="inlineStr"/>
-      <c r="H167" t="inlineStr"/>
       <c r="I167" t="inlineStr">
         <is>
           <t>editie-6/aflevering-00-brussel-als-variabele.html</t>
@@ -15189,8 +14985,6 @@
           <t>De zes ordes van fasering</t>
         </is>
       </c>
-      <c r="G168" t="inlineStr"/>
-      <c r="H168" t="inlineStr"/>
       <c r="I168" t="inlineStr">
         <is>
           <t>editie-6/aflevering-01-zes-ordes-van-fasering.html</t>
@@ -15276,8 +15070,6 @@
           <t>Wie blokkeert, en hoe zwaar?</t>
         </is>
       </c>
-      <c r="G169" t="inlineStr"/>
-      <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr">
         <is>
           <t>editie-6/aflevering-02-pareto-top12.html</t>
@@ -15363,8 +15155,6 @@
           <t>Media als rekstrook</t>
         </is>
       </c>
-      <c r="G170" t="inlineStr"/>
-      <c r="H170" t="inlineStr"/>
       <c r="I170" t="inlineStr">
         <is>
           <t>editie-6/aflevering-03-media-als-rekstrook.html</t>
@@ -15450,8 +15240,6 @@
           <t>Ordes van bezwaar</t>
         </is>
       </c>
-      <c r="G171" t="inlineStr"/>
-      <c r="H171" t="inlineStr"/>
       <c r="I171" t="inlineStr">
         <is>
           <t>editie-6/aflevering-04-ordes-van-bezwaar.html</t>
@@ -15537,8 +15325,6 @@
           <t>Twintig actuele bezwaren</t>
         </is>
       </c>
-      <c r="G172" t="inlineStr"/>
-      <c r="H172" t="inlineStr"/>
       <c r="I172" t="inlineStr">
         <is>
           <t>editie-6/aflevering-05-twintig-bezwaren.html</t>
@@ -15624,8 +15410,6 @@
           <t>De Zwitserse spiegel</t>
         </is>
       </c>
-      <c r="G173" t="inlineStr"/>
-      <c r="H173" t="inlineStr"/>
       <c r="I173" t="inlineStr">
         <is>
           <t>editie-6/aflevering-06-zwitserse-spiegel.html</t>
@@ -15711,8 +15495,6 @@
           <t>De Canadese spiegel</t>
         </is>
       </c>
-      <c r="G174" t="inlineStr"/>
-      <c r="H174" t="inlineStr"/>
       <c r="I174" t="inlineStr">
         <is>
           <t>editie-6/aflevering-07-canadese-spiegel.html</t>
@@ -15798,8 +15580,6 @@
           <t>Waar staat uw partij?</t>
         </is>
       </c>
-      <c r="G175" t="inlineStr"/>
-      <c r="H175" t="inlineStr"/>
       <c r="I175" t="inlineStr">
         <is>
           <t>editie-6/aflevering-08-partijen-in-kaart.html</t>
@@ -15885,8 +15665,6 @@
           <t>Wie verzet zich, wie helpt mee?</t>
         </is>
       </c>
-      <c r="G176" t="inlineStr"/>
-      <c r="H176" t="inlineStr"/>
       <c r="I176" t="inlineStr">
         <is>
           <t>editie-6/aflevering-09-pareto-per-actor.html</t>
@@ -15972,8 +15750,6 @@
           <t>UEI — een Europese tegenmacht uit Zwitserland</t>
         </is>
       </c>
-      <c r="G177" t="inlineStr"/>
-      <c r="H177" t="inlineStr"/>
       <c r="I177" t="inlineStr">
         <is>
           <t>editie-6/aflevering-10-uei.html</t>
@@ -16059,8 +15835,6 @@
           <t>De kennislaag als bondgenoot</t>
         </is>
       </c>
-      <c r="G178" t="inlineStr"/>
-      <c r="H178" t="inlineStr"/>
       <c r="I178" t="inlineStr">
         <is>
           <t>editie-6/aflevering-11-kennislaag-als-bondgenoot.html</t>
@@ -16146,8 +15920,6 @@
           <t>De beste weg vooruit</t>
         </is>
       </c>
-      <c r="G179" t="inlineStr"/>
-      <c r="H179" t="inlineStr"/>
       <c r="I179" t="inlineStr">
         <is>
           <t>editie-6/aflevering-12-beste-weg-vooruit.html</t>
@@ -16233,7 +16005,6 @@
           <t>Wat is er mis met partijpolitiek?</t>
         </is>
       </c>
-      <c r="G180" t="inlineStr"/>
       <c r="H180" t="inlineStr">
         <is>
           <t>Partijpolitiek bundelt belangen die niets met elkaar te maken hebben. Nova Democratia stelt voor per onderwerp te beslissen, met meetbare prijs-prestatie.</t>
@@ -16324,7 +16095,6 @@
           <t>Nova Democratia</t>
         </is>
       </c>
-      <c r="G181" t="inlineStr"/>
       <c r="H181" t="inlineStr">
         <is>
           <t>Een nieuw politiek-staatkundig model — grondslagdocument</t>
@@ -16415,7 +16185,6 @@
           <t>Nova Democratia</t>
         </is>
       </c>
-      <c r="G182" t="inlineStr"/>
       <c r="H182" t="inlineStr">
         <is>
           <t>De Nova Democratia / VMP politieke vorm.</t>
@@ -16521,7 +16290,6 @@
           <t>De actor is de regel</t>
         </is>
       </c>
-      <c r="G183" t="inlineStr"/>
       <c r="H183" t="inlineStr">
         <is>
           <t>Waarom hervorming onmogelijk is en vervanging onvermijdelijk. Een revolutie-bijdrage die de tetralogie sluit: van oergevoel via scholing en eigenkennis-tekort naar auto-immuun-instituties — en de medische therapieën die ons leren hoe genezing eruitziet.</t>
@@ -16532,7 +16300,6 @@
           <t>wat-opkomt/de-actor-is-de-regel.html</t>
         </is>
       </c>
-      <c r="J183" t="inlineStr"/>
       <c r="K183" t="inlineStr">
         <is>
           <t>center</t>
@@ -16603,7 +16370,6 @@
           <t>Soevereiniteit als cyclus</t>
         </is>
       </c>
-      <c r="G184" t="inlineStr"/>
       <c r="H184" t="inlineStr">
         <is>
           <t>Een uitweg uit het oudste dilemma van de staatstheorie</t>
@@ -16614,7 +16380,6 @@
           <t>soevereiniteit-als-cyclus/index.html</t>
         </is>
       </c>
-      <c r="J184" t="inlineStr"/>
       <c r="K184" t="inlineStr">
         <is>
           <t>center</t>
@@ -16685,7 +16450,6 @@
           <t>Beslissen zonder uitzicht</t>
         </is>
       </c>
-      <c r="G185" t="inlineStr"/>
       <c r="H185" t="inlineStr">
         <is>
           <t>Het BBP telt €419 miljard aan lucht als productie. De Nederlandse schuldquote is niet 43%. Zij is 69%. Ver boven de EU-alarmgrens. En het parlement stemt met de ogen dicht.</t>
@@ -16774,7 +16538,6 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
-      <c r="G186" t="inlineStr"/>
       <c r="H186" t="inlineStr">
         <is>
           <t>Hoe blokkades worden ontgrendeld: Nova Democratia als grondslag, Pareto-analyse om te zien wie blokkeert, en spiegels uit Zwitserland en Canada om te zien wat elders al werkt. Vijftien artikelen verdeeld over drie groepen.</t>
@@ -16785,7 +16548,6 @@
           <t>toekomst/overheden/methode/index.html</t>
         </is>
       </c>
-      <c r="J186" t="inlineStr"/>
       <c r="K186" t="inlineStr">
         <is>
           <t>center</t>
@@ -16856,7 +16618,6 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
-      <c r="G187" t="inlineStr"/>
       <c r="H187" t="inlineStr">
         <is>
           <t>Drie landen, één methode. Wat lokaal mogelijk is in Nederland, Duitsland en Europa — en de instrumenten en spiegels waarmee dat lukt.</t>
@@ -16867,7 +16628,6 @@
           <t>toekomst/overheden/index.html</t>
         </is>
       </c>
-      <c r="J187" t="inlineStr"/>
       <c r="K187" t="inlineStr">
         <is>
           <t>center</t>
@@ -16948,7 +16708,6 @@
           <t>De artikelen onder Leiderschap &amp; organisaties.</t>
         </is>
       </c>
-      <c r="J188" t="inlineStr"/>
       <c r="K188" t="inlineStr">
         <is>
           <t>center</t>
@@ -17019,7 +16778,6 @@
           <t>Hoe de papier-industrie macht kreeg over het echte werk — Het Open Vizier · Editie 4 — Juni 2026</t>
         </is>
       </c>
-      <c r="G189" t="inlineStr"/>
       <c r="H189" t="inlineStr">
         <is>
           <t>Een editie over hoe regels, verzekeringen, financiering en toezicht het oergevoel uit de beroepspraktijk hebben gewrongen — en wat dat met ons heeft gedaan.</t>
@@ -17030,7 +16788,6 @@
           <t>editie-4/index.html</t>
         </is>
       </c>
-      <c r="J189" t="inlineStr"/>
       <c r="K189" t="inlineStr">
         <is>
           <t>center</t>
@@ -17101,7 +16858,6 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
-      <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr">
         <is>
           <t>Waar deze editie heen gaat en waarom</t>
@@ -17192,7 +16948,6 @@
           <t>De wet van de papier-industrie</t>
         </is>
       </c>
-      <c r="G191" t="inlineStr"/>
       <c r="H191" t="inlineStr">
         <is>
           <t>Hoe regels, verzekeringen en financiering het echte werk verdrongen</t>
@@ -17283,7 +17038,6 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
-      <c r="G192" t="inlineStr"/>
       <c r="H192" t="inlineStr">
         <is>
           <t>Wat een leidinggevende verliest als hij alleen op cijfers stuurt</t>
@@ -17374,7 +17128,6 @@
           <t>De consultant bij het bijna-failliete bedrijf</t>
         </is>
       </c>
-      <c r="G193" t="inlineStr"/>
       <c r="H193" t="inlineStr">
         <is>
           <t>Waarom een buitenstaander binnen drie dagen weet wat insiders niet kunnen zien</t>
@@ -17465,7 +17218,6 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
-      <c r="G194" t="inlineStr"/>
       <c r="H194" t="inlineStr">
         <is>
           <t>Waarom alleen wie het niet nodig heeft krediet krijgt</t>
@@ -17556,7 +17308,6 @@
           <t>De verzekeraar tegen het leven</t>
         </is>
       </c>
-      <c r="G195" t="inlineStr"/>
       <c r="H195" t="inlineStr">
         <is>
           <t>Hoe risico-mijding zelf het grootste risico werd</t>
@@ -17647,7 +17398,6 @@
           <t>De toezichthouder die niets ziet</t>
         </is>
       </c>
-      <c r="G196" t="inlineStr"/>
       <c r="H196" t="inlineStr">
         <is>
           <t>Inspectie zonder oergevoel is administratie van het verleden</t>
@@ -17738,7 +17488,6 @@
           <t>De rechter zonder kompas</t>
         </is>
       </c>
-      <c r="G197" t="inlineStr"/>
       <c r="H197" t="inlineStr">
         <is>
           <t>Recht spreken op basis van paragrafen in plaats van mensen</t>
@@ -17829,7 +17578,6 @@
           <t>De diepere vraag</t>
         </is>
       </c>
-      <c r="G198" t="inlineStr"/>
       <c r="H198" t="inlineStr">
         <is>
           <t>Waarom een hele samenleving haar oergevoel kwijtraakte</t>
@@ -17920,7 +17668,6 @@
           <t>Retrospectief</t>
         </is>
       </c>
-      <c r="G199" t="inlineStr"/>
       <c r="H199" t="inlineStr">
         <is>
           <t>Wat deze editie samen vertelt</t>
@@ -18011,7 +17758,6 @@
           <t>Editie Leiderschap</t>
         </is>
       </c>
-      <c r="G200" t="inlineStr"/>
       <c r="H200" t="inlineStr">
         <is>
           <t>Gevoelsleiden boven verstandsleiden. Het verstandsleiden dat nu domineert verlamt het organisme. Twaalf artikelen over hoe het oergevoel werkelijk leidt — bij de CEO, in het bestuur, in de politiek.</t>
@@ -18022,7 +17768,6 @@
           <t>editie-leiderschap/index.html</t>
         </is>
       </c>
-      <c r="J200" t="inlineStr"/>
       <c r="K200" t="inlineStr">
         <is>
           <t>center</t>
@@ -18103,7 +17848,6 @@
           <t>De artikelen onder Onderwijs.</t>
         </is>
       </c>
-      <c r="J201" t="inlineStr"/>
       <c r="K201" t="inlineStr">
         <is>
           <t>center</t>
@@ -18174,7 +17918,6 @@
           <t>Kies een kant</t>
         </is>
       </c>
-      <c r="G202" t="inlineStr"/>
       <c r="H202" t="inlineStr">
         <is>
           <t>Het sluitstuk van de onderwijs-trilogie: wat wij wel kunnen redden, wat wij niet meer kunnen redden, en waarom u zich nu moet uitspreken.</t>
@@ -18265,7 +18008,6 @@
           <t>Terug naar de werkbank, vooruit naar het denken</t>
         </is>
       </c>
-      <c r="G203" t="inlineStr"/>
       <c r="H203" t="inlineStr">
         <is>
           <t>Onderwijs-trilogie · Deel I — Eenvoudig herstel van kwaliteit, vakmanschap en breedte. Vóór een land dat zichzelf weg-diplomeert en zijn ambacht vergeet.</t>
@@ -18356,7 +18098,6 @@
           <t>De prijs van de bloei</t>
         </is>
       </c>
-      <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr">
         <is>
           <t>Onderwijs-trilogie · Deel II — Wat het kost om het Nederlandse onderwijs te herstellen. Over geld, gemak, en wie de rekening voelt.</t>
@@ -18447,7 +18188,6 @@
           <t>Van leerfabriek naar leerwerkplaats</t>
         </is>
       </c>
-      <c r="G205" t="inlineStr"/>
       <c r="H205" t="inlineStr">
         <is>
           <t>Voorstellen voor radicale onderwijshervorming: bekostiging op uitkomst, strengere toelating, risico terug in de kindertijd, vakmensen weer in ere.</t>
@@ -18538,7 +18278,6 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
-      <c r="G206" t="inlineStr"/>
       <c r="H206" t="inlineStr">
         <is>
           <t>Waarom alles wat we nu leren straks niet meer telt</t>
@@ -18629,7 +18368,6 @@
           <t>Editie Kind &amp;amp; Loopbaan</t>
         </is>
       </c>
-      <c r="G207" t="inlineStr"/>
       <c r="H207" t="inlineStr">
         <is>
           <t>Het kind als toekomstig mens. Oergevoel als beginsel, scholing als instrument, loopbaan als bestemming. Dertien artikelen over hoe wij de volgende generatie vormgeven en wat dat betekent voor hun werk en plaats in de wereld.</t>
@@ -18640,7 +18378,6 @@
           <t>editie-kind-loopbaan/index.html</t>
         </is>
       </c>
-      <c r="J207" t="inlineStr"/>
       <c r="K207" t="inlineStr">
         <is>
           <t>center</t>
@@ -18711,7 +18448,6 @@
           <t>Opvoeding · Toekomst</t>
         </is>
       </c>
-      <c r="G208" t="inlineStr"/>
       <c r="H208" t="inlineStr">
         <is>
           <t>Drie vragen onder één onderwerp: hoe het zich heeft ontwikkeld, hoe het zou kunnen gaan, en hoe opvoeding er werkelijk uit zou moeten zien. Vier artikelen verdeeld over die drie vragen.</t>
@@ -18722,7 +18458,6 @@
           <t>toekomst/opvoeding/index.html</t>
         </is>
       </c>
-      <c r="J208" t="inlineStr"/>
       <c r="K208" t="inlineStr">
         <is>
           <t>center</t>
@@ -18793,7 +18528,6 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
-      <c r="G209" t="inlineStr"/>
       <c r="H209" t="inlineStr">
         <is>
           <t>Drie vragen onder één onderwerp: hoe scholing zich heeft ontwikkeld, hoe de evolutie zou kunnen gaan, en hoe scholing zou moeten worden ingericht om de kennis die wij hebben werkelijk te benutten. Vijf artikelen verdeeld over die drie vragen.</t>
@@ -18804,7 +18538,6 @@
           <t>toekomst/scholing/index.html</t>
         </is>
       </c>
-      <c r="J209" t="inlineStr"/>
       <c r="K209" t="inlineStr">
         <is>
           <t>center</t>
@@ -18885,7 +18618,6 @@
           <t>De artikelen onder Industrie, energie, toekomst.</t>
         </is>
       </c>
-      <c r="J210" t="inlineStr"/>
       <c r="K210" t="inlineStr">
         <is>
           <t>center</t>
@@ -19056,7 +18788,6 @@
           <t>Wie zijn opbouwers wegjaagt</t>
         </is>
       </c>
-      <c r="G212" t="inlineStr"/>
       <c r="H212" t="inlineStr">
         <is>
           <t>Een waarneming van Jacobus van Merksteijn. Dit stuk is geen analyse, geen onderzoek en geen advies. Het is een observatie — bedoeld om ogen te openen en de discussie te voeden.</t>
@@ -19067,7 +18798,6 @@
           <t>opbouwers-wegjagen/index.html</t>
         </is>
       </c>
-      <c r="J212" t="inlineStr"/>
       <c r="K212" t="inlineStr">
         <is>
           <t>center</t>
@@ -19138,7 +18868,6 @@
           <t>Toekomst</t>
         </is>
       </c>
-      <c r="G213" t="inlineStr"/>
       <c r="H213" t="inlineStr">
         <is>
           <t>Vragen die over generaties heen spelen — opvoeding, scholing, energie, overheden, industrie. Geen losse artikelen maar een vaste plek waar het denken over de lange termijn wordt verzameld.</t>
@@ -19149,7 +18878,6 @@
           <t>toekomst/index.html</t>
         </is>
       </c>
-      <c r="J213" t="inlineStr"/>
       <c r="K213" t="inlineStr">
         <is>
           <t>center</t>
@@ -19220,7 +18948,6 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
-      <c r="G214" t="inlineStr"/>
       <c r="H214" t="inlineStr">
         <is>
           <t>Drie vragen onder één onderwerp: hoe energie wordt opgewekt en verdeeld, hoe de evolutie zou kunnen gaan, en hoe de architectuur er op Europese schaal uit zou moeten zien. Vijf artikelen verdeeld over die drie vragen.</t>
@@ -19231,7 +18958,6 @@
           <t>toekomst/energie/index.html</t>
         </is>
       </c>
-      <c r="J214" t="inlineStr"/>
       <c r="K214" t="inlineStr">
         <is>
           <t>center</t>
@@ -19302,7 +19028,6 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
-      <c r="G215" t="inlineStr"/>
       <c r="H215" t="inlineStr">
         <is>
           <t>Drie vragen onder één onderwerp: hoe maakindustrie het oergevoel verloor, welke instrumenten daadwerkelijk werken, en hoe scholing en vakmanschap terug kunnen komen. Twaalf artikelen verdeeld over die drie vragen.</t>
@@ -19313,7 +19038,6 @@
           <t>toekomst/industrie/index.html</t>
         </is>
       </c>
-      <c r="J215" t="inlineStr"/>
       <c r="K215" t="inlineStr">
         <is>
           <t>center</t>
@@ -19675,7 +19399,6 @@
           <t>Kantelmechanica</t>
         </is>
       </c>
-      <c r="G219" t="inlineStr"/>
       <c r="H219" t="inlineStr">
         <is>
           <t>Hoe een gedachtegoed kantelt naar invloed.</t>
@@ -19776,7 +19499,6 @@
           <t>Mensen die mee bouwen</t>
         </is>
       </c>
-      <c r="G220" t="inlineStr"/>
       <c r="H220" t="inlineStr">
         <is>
           <t>Tropische ethanol-steden 2040. Een visionair stuk over wie Europa's energietoekomst kan helpen bouwen — als we de moed hebben de migratiekwestie en de energietransitie samen te denken. Goede huizen, scholen, bibliotheken, internet. Niet wegsturen, niet binnenhouden — verder gaan.</t>
@@ -19865,7 +19587,6 @@
           <t>De vergeten orde — Het Open Vizier · Editie 5 — Juli 2026</t>
         </is>
       </c>
-      <c r="G221" t="inlineStr"/>
       <c r="H221" t="inlineStr">
         <is>
           <t>Wat zwaar weegt, en wat de pers ervan maakt. Een diagnostische editie in vier delen.</t>
@@ -19876,7 +19597,6 @@
           <t>editie-5/index.html</t>
         </is>
       </c>
-      <c r="J221" t="inlineStr"/>
       <c r="K221" t="inlineStr">
         <is>
           <t>center</t>
@@ -19947,7 +19667,6 @@
           <t>Brief aan de lezer</t>
         </is>
       </c>
-      <c r="G222" t="inlineStr"/>
       <c r="H222" t="inlineStr">
         <is>
           <t>Editie 5 levert geen mening af, maar een instrument.</t>
@@ -20038,7 +19757,6 @@
           <t>七つ道具 — De zeven die het verschil maakten</t>
         </is>
       </c>
-      <c r="G223" t="inlineStr"/>
       <c r="H223" t="inlineStr">
         <is>
           <t>Kaoru Ishikawa's zeven kwaliteitsinstrumenten, plus orde-analyse uit de staalbouw. Het gereedschap waarmee Japan ons inhaalde.</t>
@@ -20129,7 +19847,6 @@
           <t>De succesformule die wij verleerd hebben</t>
         </is>
       </c>
-      <c r="G224" t="inlineStr"/>
       <c r="H224" t="inlineStr">
         <is>
           <t>Japan, Korea en China zijn ons ingehaald omdat ze het instrument omarmden dat wij hebben weggegooid.</t>
@@ -20220,7 +19937,6 @@
           <t>De vergeten orde</t>
         </is>
       </c>
-      <c r="G225" t="inlineStr"/>
       <c r="H225" t="inlineStr">
         <is>
           <t>Drie tradities, één principe: wat 5× kleiner bijdraagt dan de hoofdfactor, telt niet mee.</t>
@@ -20311,7 +20027,6 @@
           <t>De methaan-misleiding</t>
         </is>
       </c>
-      <c r="G226" t="inlineStr"/>
       <c r="H226" t="inlineStr">
         <is>
           <t>Drie FD-stukken in één week, drie omkeringen van zwaarte, vier eisen aan de pers.</t>
@@ -20402,7 +20117,6 @@
           <t>De plant die verhuist</t>
         </is>
       </c>
-      <c r="G227" t="inlineStr"/>
       <c r="H227" t="inlineStr">
         <is>
           <t>Stikstof, droogte, klimaatverschuiving, fragmentatie — en het beleid dat slechts één van de vier ziet.</t>
@@ -20493,7 +20207,6 @@
           <t>De zeven van Bern</t>
         </is>
       </c>
-      <c r="G228" t="inlineStr"/>
       <c r="H228" t="inlineStr">
         <is>
           <t>Een collegiale democratie als sluitsteen — wat Zwitserland in 1848 deed wat wij hadden kunnen overnemen, en wat de NEPK-cijfers van eenentwintig landen ervan laten zien.</t>
@@ -20584,7 +20297,6 @@
           <t>De afwijkers</t>
         </is>
       </c>
-      <c r="G229" t="inlineStr"/>
       <c r="H229" t="inlineStr">
         <is>
           <t>Sandra Palmen-Schlangen, Eva González Pérez, Ad Bos — drie geverifieerde kompasdragers.</t>
@@ -20675,7 +20387,6 @@
           <t>De eis aan de lezer</t>
         </is>
       </c>
-      <c r="G230" t="inlineStr"/>
       <c r="H230" t="inlineStr">
         <is>
           <t>Wat u kunt doen met dit instrument — en waarom dát is wat de papier-industrie het minst kan dragen.</t>
@@ -20766,7 +20477,6 @@
           <t>Veerkracht en Selectie</t>
         </is>
       </c>
-      <c r="G231" t="inlineStr"/>
       <c r="H231" t="inlineStr">
         <is>
           <t>Hoe de overheid een modern selectiesysteem kan aansturen. Een radicaal herstructureringsprogramma: bescherm de productieve kern, bouw interne diensten af, met behoud van basiszekerheid.</t>
@@ -20857,14 +20567,11 @@
           <t>Editie 1</t>
         </is>
       </c>
-      <c r="G232" t="inlineStr"/>
-      <c r="H232" t="inlineStr"/>
       <c r="I232" t="inlineStr">
         <is>
           <t>editie-1/index.html</t>
         </is>
       </c>
-      <c r="J232" t="inlineStr"/>
       <c r="K232" t="inlineStr">
         <is>
           <t>center</t>
@@ -21229,7 +20936,6 @@
           <t>De Grote Plundering</t>
         </is>
       </c>
-      <c r="G236" t="inlineStr"/>
       <c r="H236" t="inlineStr">
         <is>
           <t>Vijfluik over hoe Europa zijn productieven uitkleedt.</t>
@@ -21320,7 +21026,6 @@
           <t>Eerst plukken, dan oordelen</t>
         </is>
       </c>
-      <c r="G237" t="inlineStr"/>
       <c r="H237" t="inlineStr">
         <is>
           <t>De cirkel van onrecht waarin Europa zichzelf vernietigt</t>
@@ -21421,7 +21126,6 @@
           <t>Plundering 1: diagnose</t>
         </is>
       </c>
-      <c r="G238" t="inlineStr"/>
       <c r="H238" t="inlineStr">
         <is>
           <t>Wij plukken wie ons voedt</t>
@@ -21522,7 +21226,6 @@
           <t>Plundering 2: mechaniek</t>
         </is>
       </c>
-      <c r="G239" t="inlineStr"/>
       <c r="H239" t="inlineStr">
         <is>
           <t>De muren die wij hebben gemetseld om onze bouwers op te sluiten</t>
@@ -21623,7 +21326,6 @@
           <t>Plundering 3: afloop</t>
         </is>
       </c>
-      <c r="G240" t="inlineStr"/>
       <c r="H240" t="inlineStr">
         <is>
           <t>Waarom de plunderaars zwaarder zullen lijden dan de geplunderden</t>
@@ -21724,7 +21426,6 @@
           <t>Plundering 4: politiek</t>
         </is>
       </c>
-      <c r="G241" t="inlineStr"/>
       <c r="H241" t="inlineStr">
         <is>
           <t>Wie wil wat, en waarom Brussel niet weet hoe verder</t>
@@ -22023,7 +21724,6 @@
           <t>Ferrari Junção</t>
         </is>
       </c>
-      <c r="G244" t="inlineStr"/>
       <c r="H244" t="inlineStr">
         <is>
           <t>Dagelijks idee: Ferrari Junção.</t>
@@ -22124,7 +21824,6 @@
           <t>VMB ESG</t>
         </is>
       </c>
-      <c r="G245" t="inlineStr"/>
       <c r="H245" t="inlineStr">
         <is>
           <t>Wat ik achterlaat — VMB ESG essay.</t>
@@ -22225,7 +21924,6 @@
           <t>Manifest</t>
         </is>
       </c>
-      <c r="G246" t="inlineStr"/>
       <c r="H246" t="inlineStr">
         <is>
           <t>Waarom de StemWijzer u nooit zal vertellen wat u eigenlijk stemt.</t>
@@ -22326,14 +22024,11 @@
           <t>Beleidsadvies aantrekken</t>
         </is>
       </c>
-      <c r="G247" t="inlineStr"/>
-      <c r="H247" t="inlineStr"/>
       <c r="I247" t="inlineStr">
         <is>
-          <t>wat-opkomt/beleidsadvies-aantrekken.html</t>
-        </is>
-      </c>
-      <c r="J247" t="inlineStr"/>
+          <t>editie-2/beleidsadvies-aantrekken.html</t>
+        </is>
+      </c>
       <c r="K247" t="inlineStr">
         <is>
           <t>center</t>
@@ -22502,7 +22197,6 @@
           <t>Gevolgenkaart</t>
         </is>
       </c>
-      <c r="G249" t="inlineStr"/>
       <c r="H249" t="inlineStr">
         <is>
           <t>Partij × Persoon × Basislijn = Projectie</t>
@@ -22513,7 +22207,6 @@
           <t>stemgedrag.html</t>
         </is>
       </c>
-      <c r="J249" t="inlineStr"/>
       <c r="K249" t="inlineStr">
         <is>
           <t>center</t>
@@ -22584,7 +22277,6 @@
           <t>Beslissen zonder uitzicht</t>
         </is>
       </c>
-      <c r="G250" t="inlineStr"/>
       <c r="H250" t="inlineStr">
         <is>
           <t>Het BBP telt €419 miljard aan lucht als productie. De Nederlandse schuldquote is niet 43%. Zij is 69%. Ver boven de EU-alarmgrens. En het parlement stemt met de ogen dicht.</t>
@@ -22673,7 +22365,6 @@
           <t>Dossiers</t>
         </is>
       </c>
-      <c r="G251" t="inlineStr"/>
       <c r="H251" t="inlineStr">
         <is>
           <t>Diepte-dossiers van Het Open Vizier. Businessplannen, technologie-dossiers, IP-strategieën — voor wie verder wil dan de krantenkop.</t>
@@ -22684,7 +22375,6 @@
           <t>dossiers/index.html</t>
         </is>
       </c>
-      <c r="J251" t="inlineStr"/>
       <c r="K251" t="inlineStr">
         <is>
           <t>center</t>
@@ -22755,7 +22445,6 @@
           <t>Vortex-Hair™ Adaptive Dimple Golf Ball — Dossier · Het Open Vizier</t>
         </is>
       </c>
-      <c r="G252" t="inlineStr"/>
       <c r="H252" t="inlineStr">
         <is>
           <t>Businessplan-dossier voor de Vortex-Hair™ golfbal: flexibele micro-filamenten in elke dimple voor 5–15% extra carry distance. IP-strategie, licentiemodellen en marktanalyse.</t>
@@ -22766,7 +22455,6 @@
           <t>dossiers/vortex-hair.html</t>
         </is>
       </c>
-      <c r="J252" t="inlineStr"/>
       <c r="K252" t="inlineStr">
         <is>
           <t>center</t>
@@ -22837,7 +22525,6 @@
           <t>Achter de Cijfers</t>
         </is>
       </c>
-      <c r="G253" t="inlineStr"/>
       <c r="H253" t="inlineStr">
         <is>
           <t>Onderzoek &amp;amp; technische analyses bij Het Open Vizier. Voor wie achter de cijfers wil kijken.</t>
@@ -22848,7 +22535,6 @@
           <t>onderzoek/index.html</t>
         </is>
       </c>
-      <c r="J253" t="inlineStr"/>
       <c r="K253" t="inlineStr">
         <is>
           <t>center</t>
@@ -22919,7 +22605,6 @@
           <t>EU: BBP, Reële Lonen en de Overheidsmultiplicator</t>
         </is>
       </c>
-      <c r="G254" t="inlineStr"/>
       <c r="H254" t="inlineStr">
         <is>
           <t>Bbp-loonmaat na aftrek van groei van totale overheidskosten — wat blijft over aan macro-economische ruimte?</t>
@@ -22930,7 +22615,6 @@
           <t>onderzoek/eu-multiplicator.html</t>
         </is>
       </c>
-      <c r="J254" t="inlineStr"/>
       <c r="K254" t="inlineStr">
         <is>
           <t>center</t>
@@ -23001,7 +22685,6 @@
           <t>Is Nederland op weg naar ontwikkelingslandstatus? — Het Open Vizier · Achter de Cijfers</t>
         </is>
       </c>
-      <c r="G255" t="inlineStr"/>
       <c r="H255" t="inlineStr">
         <is>
           <t>Een data-gedreven analyse van faillissementen, bedrijfsuitval, werkgelegenheid en de-industrialisatie in Nederland — 2000 tot en met 2026</t>
@@ -23012,7 +22695,6 @@
           <t>onderzoek/ontwikkelingslandstatus.html</t>
         </is>
       </c>
-      <c r="J255" t="inlineStr"/>
       <c r="K255" t="inlineStr">
         <is>
           <t>center</t>
@@ -23083,7 +22765,6 @@
           <t>Onderzoek</t>
         </is>
       </c>
-      <c r="G256" t="inlineStr"/>
       <c r="H256" t="inlineStr">
         <is>
           <t>Onderzoekslijnen die nog open staan. Plannen, hypothesen en metingen die op tafel liggen — niet als afgesloten verhaal, maar als uitnodiging om mee te denken.</t>
@@ -23094,7 +22775,6 @@
           <t>onderzoeken/index.html</t>
         </is>
       </c>
-      <c r="J256" t="inlineStr"/>
       <c r="K256" t="inlineStr">
         <is>
           <t>center</t>
@@ -23170,7 +22850,6 @@
           <t>wie maakt dit</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr"/>
       <c r="I257" t="inlineStr">
         <is>
           <t>colofon.html</t>
@@ -23256,7 +22935,6 @@
           <t>Over deze krant</t>
         </is>
       </c>
-      <c r="G258" t="inlineStr"/>
       <c r="H258" t="inlineStr">
         <is>
           <t>Wat Het Open Vizier wil, wat het niet wil, en hoe het werkt — en wie het schrijft.</t>
@@ -23267,7 +22945,6 @@
           <t>over.html</t>
         </is>
       </c>
-      <c r="J258" t="inlineStr"/>
       <c r="K258" t="inlineStr">
         <is>
           <t>center</t>
@@ -23343,7 +23020,6 @@
           <t>alles teruglezen</t>
         </is>
       </c>
-      <c r="H259" t="inlineStr"/>
       <c r="I259" t="inlineStr">
         <is>
           <t>archief.html</t>
@@ -23429,14 +23105,11 @@
           <t>Bedankt — controleer uw inbox</t>
         </is>
       </c>
-      <c r="G260" t="inlineStr"/>
-      <c r="H260" t="inlineStr"/>
       <c r="I260" t="inlineStr">
         <is>
           <t>bedankt.html</t>
         </is>
       </c>
-      <c r="J260" t="inlineStr"/>
       <c r="K260" t="inlineStr">
         <is>
           <t>center</t>
@@ -23507,7 +23180,6 @@
           <t>Op de hoogte blijven</t>
         </is>
       </c>
-      <c r="G261" t="inlineStr"/>
       <c r="H261" t="inlineStr">
         <is>
           <t>Vraag een korte melding aan wanneer een nieuw stuk verschijnt op openvizier.org. Geen mening, geen verkoop van gegevens. Uitschrijven met één klik.</t>
@@ -23518,7 +23190,6 @@
           <t>op-de-hoogte.html</t>
         </is>
       </c>
-      <c r="J261" t="inlineStr"/>
       <c r="K261" t="inlineStr">
         <is>
           <t>center</t>
@@ -23589,14 +23260,11 @@
           <t>Structuur — Beheer · Het Open Vizier</t>
         </is>
       </c>
-      <c r="G262" t="inlineStr"/>
-      <c r="H262" t="inlineStr"/>
       <c r="I262" t="inlineStr">
         <is>
           <t>structuur.html</t>
         </is>
       </c>
-      <c r="J262" t="inlineStr"/>
       <c r="K262" t="inlineStr">
         <is>
           <t>center</t>
@@ -23667,7 +23335,6 @@
           <t>Navigatie · Het Open Vizier</t>
         </is>
       </c>
-      <c r="G263" t="inlineStr"/>
       <c r="H263" t="inlineStr">
         <is>
           <t>Visuele navigatie door Het Open Vizier — vier hoofdthemes, alle artikelen in beeld.</t>
@@ -23678,7 +23345,6 @@
           <t>navigatie.html</t>
         </is>
       </c>
-      <c r="J263" t="inlineStr"/>
       <c r="K263" t="inlineStr">
         <is>
           <t>center</t>
@@ -23749,14 +23415,11 @@
           <t>Het Open Vizier — Kies een taal</t>
         </is>
       </c>
-      <c r="G264" t="inlineStr"/>
-      <c r="H264" t="inlineStr"/>
       <c r="I264" t="inlineStr">
         <is>
           <t>talenring.html</t>
         </is>
       </c>
-      <c r="J264" t="inlineStr"/>
       <c r="K264" t="inlineStr">
         <is>
           <t>center</t>
@@ -23827,14 +23490,11 @@
           <t>Het Open Vizier — Kies een taal</t>
         </is>
       </c>
-      <c r="G265" t="inlineStr"/>
-      <c r="H265" t="inlineStr"/>
       <c r="I265" t="inlineStr">
         <is>
           <t>index-talenring.html</t>
         </is>
       </c>
-      <c r="J265" t="inlineStr"/>
       <c r="K265" t="inlineStr">
         <is>
           <t>center</t>
@@ -23905,7 +23565,6 @@
           <t>Het Open Vizier — een krant over denken zonder oogkleppen</t>
         </is>
       </c>
-      <c r="G266" t="inlineStr"/>
       <c r="H266" t="inlineStr">
         <is>
           <t>Onafhankelijke maandelijkse krant van Jacobus van Merksteijn. Politiek, democratie, onderwijs, natuurkunde en techniek — in gewone taal, open voor discussie.</t>
@@ -23916,7 +23575,6 @@
           <t>index-klassiek.html</t>
         </is>
       </c>
-      <c r="J266" t="inlineStr"/>
       <c r="K266" t="inlineStr">
         <is>
           <t>center</t>
@@ -23987,7 +23645,6 @@
           <t>Delen</t>
         </is>
       </c>
-      <c r="G267" t="inlineStr"/>
       <c r="H267" t="inlineStr">
         <is>
           <t>Hoe Het Open Vizier het beste verder gedragen kan worden — naar lezers in parlementen, universiteiten, redacties en eigen netwerken.</t>
@@ -23998,7 +23655,6 @@
           <t>delen.html</t>
         </is>
       </c>
-      <c r="J267" t="inlineStr"/>
       <c r="K267" t="inlineStr">
         <is>
           <t>center</t>
@@ -24069,7 +23725,6 @@
           <t>Verkennen</t>
         </is>
       </c>
-      <c r="G268" t="inlineStr"/>
       <c r="H268" t="inlineStr">
         <is>
           <t>Visueel verkennen van de structuur van Het Open Vizier — klik door de lagen.</t>
@@ -24080,7 +23735,6 @@
           <t>verkennen.html</t>
         </is>
       </c>
-      <c r="J268" t="inlineStr"/>
       <c r="K268" t="inlineStr">
         <is>
           <t>center</t>
@@ -24151,14 +23805,11 @@
           <t>Verkennen</t>
         </is>
       </c>
-      <c r="G269" t="inlineStr"/>
-      <c r="H269" t="inlineStr"/>
       <c r="I269" t="inlineStr">
         <is>
           <t>verkennen-embed.html</t>
         </is>
       </c>
-      <c r="J269" t="inlineStr"/>
       <c r="K269" t="inlineStr">
         <is>
           <t>center</t>
@@ -24229,7 +23880,6 @@
           <t>Tien seconden</t>
         </is>
       </c>
-      <c r="G270" t="inlineStr"/>
       <c r="H270" t="inlineStr">
         <is>
           <t>Binnen tien seconden weet een kind van vier wie er echt aanwezig is. Tussen vier en twaalf leren wij het kind dat het niet mag vertrouwen op die wetenschap. Wij noemen dat opvoeding.</t>
@@ -24240,7 +23890,6 @@
           <t>idee.html</t>
         </is>
       </c>
-      <c r="J270" t="inlineStr"/>
       <c r="K270" t="inlineStr">
         <is>
           <t>center</t>
@@ -24311,7 +23960,6 @@
           <t>Hoe u meedoet aan de discussie</t>
         </is>
       </c>
-      <c r="G271" t="inlineStr"/>
       <c r="H271" t="inlineStr">
         <is>
           <t>Hoe het discussiesysteem van Het Open Vizier werkt: registratie, spelregels, AI-moderatie en wat ermee gebeurt.</t>
@@ -24402,7 +24050,6 @@
           <t>Wat er nu al ligt</t>
         </is>
       </c>
-      <c r="G272" t="inlineStr"/>
       <c r="H272" t="inlineStr">
         <is>
           <t>Overzicht van technische projecten: SeaSkin, GuardSkin, AeroSkin, SolarSkin, TerraClean, Tyre-patenten, conische vortex-reactor.</t>
@@ -24478,10 +24125,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="B2:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
@@ -24715,10 +24361,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="B2:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
@@ -24985,10 +24630,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="B2:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
@@ -25748,10 +25392,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="B2:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
@@ -25759,7 +25402,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
@@ -25772,7 +25414,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
@@ -25785,7 +25426,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
@@ -25798,7 +25438,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
@@ -25811,7 +25450,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
@@ -25824,7 +25462,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
@@ -25837,7 +25474,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
@@ -25850,7 +25486,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
@@ -25863,7 +25498,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
@@ -25876,7 +25510,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wat opkomt: 'Waar een wil is is een weg' — reactie op FD-reportage
Nieuw opinie-artikel over jonge werkenden in de WIA en de drie hersenlagen.
Aansluitend bij Editie 3 (Onder het ijs).

Bestanden:
- nl/wat-opkomt/waar-een-wil-is.html (nieuw artikel, 6 illustraties)
- assets/wat-opkomt/wil/wil_01_thuis.jpg (nieuwe hero, warme olieverf)
- assets/wat-opkomt/wil/wil_06_spreekkamer.jpg (nieuwe illustratie)
- 4 hero's hergebruikt uit Editie 3 (drie hersenlagen, wat we doen, ai-onderwijs, mama)

Matrix-inschrijvingen (via vizier.xlsx):
- 1.4.6.9  (NL Voorpagina > Wat het niet ziet) Volgorde=1, datum 2026-08-05
- 1.3.2.11 (NL Filosofie > Oergevoel & Kosaris) Terug naar 1.3.2
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR272"/>
+  <dimension ref="A2:AR274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -688,7 +688,6 @@
           <t>De talenring is het startscherm: kies een taal voor je verkennen.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>center</t>
@@ -769,7 +768,6 @@
           <t>Nederlandse uitgave van Het Open Vizier — onderzoeksjournalistiek over governance, energie en economie.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>center</t>
@@ -850,7 +848,6 @@
           <t>De vaste voorpagina van Het Open Vizier.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>center</t>
@@ -931,7 +928,6 @@
           <t>Partijen, campagnes, revolutie, media — wat er nu speelt.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>center</t>
@@ -1012,7 +1008,6 @@
           <t>Dimensies, oergevoel, samenhang, films en boeken.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>center</t>
@@ -1093,7 +1088,6 @@
           <t>Klimaatdividend, BiCRS, thermostaat, wereldgordel.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>center</t>
@@ -1174,7 +1168,6 @@
           <t>Nederland, Europa, andere landen, Nova Democratia.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>center</t>
@@ -1255,7 +1248,6 @@
           <t>Kantelmechanica, vergeten orde, veerkracht.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>center</t>
@@ -1336,7 +1328,6 @@
           <t>Vermogensvlucht, plundering, stemmetjeswinning, BBP.</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>center</t>
@@ -1417,7 +1408,6 @@
           <t>Onderzoeksrapporten, dossiers, achter-de-cijfers.</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>center</t>
@@ -1498,7 +1488,6 @@
           <t>Colofon, over, archief, structuur, talenring.</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>center</t>
@@ -1579,7 +1568,6 @@
           <t>Delen, verkennen, discussie, tien seconden.</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>center</t>
@@ -1755,7 +1743,6 @@
           <t>De artikelen onder Frankrijk &amp; Europese revolutie.</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>center</t>
@@ -2227,7 +2214,6 @@
           <t>De artikelen onder Kantelmechanica &amp; mensen.</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>center</t>
@@ -2298,7 +2284,6 @@
           <t>Kantelmechanica</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>Hoe een gedachtegoed kantelt naar invloed.</t>
@@ -2399,7 +2384,6 @@
           <t>Mensen die mee bouwen</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>Tropische ethanol-steden 2040. Een visionair stuk over wie Europa's energietoekomst kan helpen bouwen — als we de moed hebben de migratiekwestie en de energietransitie samen te denken. Goede huizen, scholen, bibliotheken, internet. Niet wegsturen, niet binnenhouden — verder gaan.</t>
@@ -2488,7 +2472,6 @@
           <t>Actievoerders bouwen continenten</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Drive zoekt grond. Wat hier schuurt, kan ginds bouwen. Een open uitnodiging aan organisaties met visie en aan iedereen die zijn energie zoekt waar zij iets kan opbouwen — niet als straf, niet als afvoer, maar als kans.</t>
@@ -2577,7 +2560,6 @@
           <t>Wie zijn opbouwers wegjaagt</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>Een waarneming van Jacobus van Merksteijn. Dit stuk is geen analyse, geen onderzoek en geen advies. Het is een observatie — bedoeld om ogen te openen en de discussie te voeden.</t>
@@ -2588,7 +2570,6 @@
           <t>opbouwers-wegjagen/index.html</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>center</t>
@@ -2769,7 +2750,6 @@
           <t>De artikelen onder Partijen &amp; pareto.</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
           <t>center</t>
@@ -2840,8 +2820,6 @@
           <t>Wie blokkeert, en hoe zwaar?</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>editie-6/aflevering-02-pareto-top12.html</t>
@@ -2927,8 +2905,6 @@
           <t>Waar staat uw partij?</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>editie-6/aflevering-08-partijen-in-kaart.html</t>
@@ -3014,8 +2990,6 @@
           <t>Wie verzet zich, wie helpt mee?</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>editie-6/aflevering-09-pareto-per-actor.html</t>
@@ -3101,8 +3075,6 @@
           <t>Ordes van bezwaar</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>editie-6/aflevering-04-ordes-van-bezwaar.html</t>
@@ -3188,8 +3160,6 @@
           <t>Twintig actuele bezwaren</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>editie-6/aflevering-05-twintig-bezwaren.html</t>
@@ -3275,7 +3245,6 @@
           <t>Plundering 4: politiek</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>Wie wil wat, en waarom Brussel niet weet hoe verder</t>
@@ -3386,7 +3355,6 @@
           <t>De artikelen onder Pers &amp; media.</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr">
         <is>
           <t>center</t>
@@ -3653,7 +3621,6 @@
           <t>Trump als spiegel</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>Wat Trump-II met Europa doet.</t>
@@ -3754,8 +3721,6 @@
           <t>Media als rekstrook</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>editie-6/aflevering-03-media-als-rekstrook.html</t>
@@ -3841,7 +3806,6 @@
           <t>De anti-immuunziekte van Brussel maakt dat we arm worden</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>CBAM, ETS, Pillar Two en vermogensbelastingen tegelijk. De BiCRS/Ethanol-route wordt genegeerd. Brussel maakt zijn eigen inwoners arm.</t>
@@ -3852,7 +3816,6 @@
           <t>wat-opkomt/de-anti-immuunziekte-van-brussel.html</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
           <t>center</t>
@@ -3926,7 +3889,6 @@
           <t>De anti-immuunziekte van onze overheid slaat toe</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>Het kabinet-Jetten presenteert eind juni 2026 zijn stikstofpakket. Een aanval op het laatste productieve weefsel. En er is een andere weg.</t>
@@ -3937,7 +3899,6 @@
           <t>wat-opkomt/de-auto-immuunziekte-slaat-toe.html</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr">
         <is>
           <t>center</t>
@@ -4011,7 +3972,6 @@
           <t>De dertig cent die Europa omdraait</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>Bio-ethanol uit cellulose-route haalt €0,30 per liter in 2036, zonder een cent subsidie. Combineer met de nieuwste brandstofcellen en je hebt stroom voor minder dan de helft van de Spaanse netprijs. In Den Haag, Berlijn en Brussel hoort u er niets over.</t>
@@ -4110,7 +4070,6 @@
           <t>De artikelen onder Stemgedrag &amp; keuzemomenten.</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
           <t>center</t>
@@ -4181,7 +4140,6 @@
           <t>Gevolgenkaart</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>Partij × Persoon × Basislijn = Projectie</t>
@@ -4192,7 +4150,6 @@
           <t>stemgedrag.html</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
           <t>center</t>
@@ -4459,7 +4416,6 @@
           <t>Op de bok of op de bagagedrager</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>Een sturend artikel. Wie nu niet ziet en aanpakt, zit straks weer achterin. Europa heeft een keuze: zelf de teugels nemen of zich laten leiden door Tokio, Seoul en Peking. De drie blokken — bron, omzetting, eindsysteem — zonder één cent subsidie. Eén route wint. Wie hem niet pakt, verliest.</t>
@@ -4548,7 +4504,6 @@
           <t>Eerst plukken, dan oordelen</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>De cirkel van onrecht waarin Europa zichzelf vernietigt</t>
@@ -4649,7 +4604,6 @@
           <t>Kies een kant</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>Het sluitstuk van de onderwijs-trilogie: wat wij wel kunnen redden, wat wij niet meer kunnen redden, en waarom u zich nu moet uitspreken.</t>
@@ -4740,7 +4694,6 @@
           <t>Waarom deze krant?</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>Voorwoord bij de eerste editie van Het Open Vizier. Over verbanden zien, intelligentie als kruisbestuiving, en waarom een onafhankelijke krant nodig is.</t>
@@ -4939,7 +4892,6 @@
           <t>De artikelen onder Zeven Dimensies &amp; denkraam.</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
           <t>center</t>
@@ -5201,7 +5153,6 @@
           <t>Drie dimensies zijn te weinig</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>Het 7D-denkraam uitgelegd: x, y, z, t, G (schaal), W (waarde van antimaterie tot materie) en N (veelvoud van universa). In gewone taal.</t>
@@ -5292,7 +5243,6 @@
           <t>Hoe alles samenhangt</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>De synthese van de eerste editie: hoe de 7D-denkwijze politiek, onderwijs, techniek en wetenschap met elkaar verbindt.</t>
@@ -5383,7 +5333,6 @@
           <t>Alles stroomt — moeder van alle wetenschap</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>Stromingsleer als universele taal: van scheepscoatings tot economie tot democratie. Een pleidooi voor vakoverschrijdend denken.</t>
@@ -5474,7 +5423,6 @@
           <t>Zeven Dimensies</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>Hoe G, W en N het standaardmodel verruimen — van vacuümstructuur tot quantum computing en nanotechnologie</t>
@@ -5575,7 +5523,6 @@
           <t>De artikelen onder Oergevoel &amp; Kosaris.</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
           <t>center</t>
@@ -5646,7 +5593,6 @@
           <t>Het oergevoel</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>Wat de eerste laag is en hoe wij hem voelen</t>
@@ -5737,7 +5683,6 @@
           <t>De zeven dimensies</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>Het 7D-model van menselijk gevoel</t>
@@ -5828,7 +5773,6 @@
           <t>De drie hersenlagen</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>Oergevoel, zoogdierbrein, mensenbrein</t>
@@ -5919,7 +5863,6 @@
           <t>Communicatie tussen oergevoelens</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>Hoogfrequente gravitatie en het voorhoofdsbeen</t>
@@ -6010,7 +5953,6 @@
           <t>Wat we kinderen aandoen</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
           <t>De systematische uitknijping</t>
@@ -6101,7 +6043,6 @@
           <t>Mama ik heb honger</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>De voortdurende aanwezigheid en wat afwezigheid kost</t>
@@ -6192,7 +6133,6 @@
           <t>Het oergevoel in de beroepspraktijk</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
           <t>Verkoper, baas, consultant en bankier — vier beroepen, één instrument</t>
@@ -6283,7 +6223,6 @@
           <t>De mens onder het ijs — Het Open Vizier · Editie 3 — Juni 2026</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>Een gedachtegoed over het oergevoel, het driedubbele brein, en de mens die wij niet meer opleiden.</t>
@@ -6294,7 +6233,6 @@
           <t>editie-3/index.html</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr">
         <is>
           <t>center</t>
@@ -6365,7 +6303,6 @@
           <t>Manifest Oergevoel</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
           <t>Ruimte voor het oergevoel.</t>
@@ -6466,7 +6403,6 @@
           <t>Waarom ik ben zoals ik ben</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
           <t>Over de uitkomst aan het eind, en de mensen die alleen aan morgen denken</t>
@@ -6567,7 +6503,6 @@
           <t>De artikelen onder Films, sprookjes, leesboek.</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr">
         <is>
           <t>center</t>
@@ -6638,7 +6573,6 @@
           <t>De 7-Dim Film</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>De Zeven Dimensies — een filmisch essay van tien minuten over de zeven fundamentele assen van de werkelijkheid: x, y, z, t, G, W en N. Door Jacobus van Merksteijn.</t>
@@ -6649,7 +6583,6 @@
           <t>7-dim-film/index.html</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr">
         <is>
           <t>center</t>
@@ -6720,7 +6653,6 @@
           <t>De Kosaris — De Film</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
           <t>De Kosaris — een filmisch essay van elf minuten over de vier zuilen die dragen: Chronesis, Philotimos, Aletheris en Timaris. Twaalf hoofdstukken. Door Jacobus van Merksteijn.</t>
@@ -6731,7 +6663,6 @@
           <t>kosaris-film/index.html</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr">
         <is>
           <t>center</t>
@@ -6802,7 +6733,6 @@
           <t>De Kosaris — Leesboek</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>De Kosaris, Boek Eén: het volledige leesboek van Jacobus van Merksteijn, met de vier zuilen Chronesis, Philotimos, Aletheris en Timaris.</t>
@@ -6813,7 +6743,6 @@
           <t>leesboek/index.html</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr">
         <is>
           <t>center</t>
@@ -6884,7 +6813,6 @@
           <t>Het sprookje van Jacobus</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>Een sprookje voor kinderen om te horen, en voor volwassenen om te herkennen. Elke pagina heeft twee lezingen: het sprookje in beeld en woord, en de volwassen betekenis ernaast.</t>
@@ -6895,7 +6823,6 @@
           <t>sprookjes/index.html</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr"/>
       <c r="K73" t="inlineStr">
         <is>
           <t>center</t>
@@ -6966,7 +6893,6 @@
           <t>Filosofie</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
           <t>Wat ligt onder de keuzes die wij maken? Welke begrippen dragen onze instellingen, en welke begrippen kunnen wij nog niet missen omdat wij ze nog niet hebben uitgedacht? De Filosofie-sectie verzamelt manifesten en essays die de grondslagen ter discussie stellen — niet als debatkunst, maar als oefening in vrijer denken.</t>
@@ -6977,7 +6903,6 @@
           <t>filosofie/index.html</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr">
         <is>
           <t>center</t>
@@ -7058,7 +6983,6 @@
           <t>De artikelen onder Gevoelsconnectiesysteem.</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr"/>
       <c r="K75" t="inlineStr">
         <is>
           <t>center</t>
@@ -7129,7 +7053,6 @@
           <t>Het gevoelsconnectiesysteem</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
           <t>Een onderzoeksplan over de basale menselijke gevoelslaag, nachtelijke integratie van dagkennis, foutdetectie in opvoeding en leiderschap, en de hypothese van een fysiek kanaal voor gevoel-naar-gevoel-overdracht.</t>
@@ -7140,7 +7063,6 @@
           <t>onderzoeken/gevoelsconnectiesysteem.html</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr"/>
       <c r="K76" t="inlineStr">
         <is>
           <t>center</t>
@@ -7211,7 +7133,6 @@
           <t>Het gevoelsconnectiesysteem — volledig onderzoeksplan</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
           <t>Volledig onderzoeksplan over het basaal menselijke gevoelsconnectiesysteem, nachtelijke integratie van verstand naar gevoel, foutdetectie als sleutelvariabele, en de hypothese van menselijke gravitatiegolven als drager.</t>
@@ -7222,7 +7143,6 @@
           <t>onderzoeken/gevoelsconnectiesysteem-volledig.html</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr"/>
       <c r="K77" t="inlineStr">
         <is>
           <t>center</t>
@@ -7293,7 +7213,6 @@
           <t>Krantbriefing — gevoelsconnectiesysteem</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
           <t>Journalistieke briefingtekst over het gevoelsconnectiesysteem, nachtelijke integratie en de hypothese van menselijke gravitatiegolven — voor een collega die het onderwerp in krantstijl wil uitwerken.</t>
@@ -7304,7 +7223,6 @@
           <t>onderzoeken/krantbriefing.html</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr">
         <is>
           <t>center</t>
@@ -7375,7 +7293,6 @@
           <t>Routekaart van vervolgvragen</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
           <t>Vierentwintig vervolgvragen rond het gevoelsconnectiesysteem, in acht fasen — van begrippen naar detector. Een werkroute voor wie wil meedenken.</t>
@@ -7386,7 +7303,6 @@
           <t>onderzoeken/routekaart-vervolgvragen.html</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr">
         <is>
           <t>center</t>
@@ -7467,7 +7383,6 @@
           <t>De artikelen onder Klimaatdividend &amp; oversterfte.</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr">
         <is>
           <t>center</t>
@@ -7844,7 +7759,6 @@
           <t>De artikelen onder BiCRS &amp; Carbon-Alert.</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr">
         <is>
           <t>center</t>
@@ -7915,7 +7829,6 @@
           <t>Visie 2036 — Carbon-Alert Energie-Hub</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>Het technische ontwerp van de 100 kW Carbon-Alert energie-hub. LCOE-analyse, vijf bouwblokken, kasstroom, risico-matrix. Het bewijs onder het sturend artikel — alle cijfers zonder subsidie.</t>
@@ -8004,7 +7917,6 @@
           <t>BiCRS-versie EU</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
           <t>Volledige doorrekening Brussel met BiCRS-vervanging.</t>
@@ -8203,7 +8115,6 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
           <t>Carbon-Alert op Europese schaal: zes miljoen hectare koolzaad, twintig miljoen ton sojaschroot-import, en het volledige GLB-budget. Wat verandert er als de architectuur op een derde van het Europese koolzaadareaal wordt toegepast — en wat krijgt Brussel ervoor terug?</t>
@@ -8214,7 +8125,6 @@
           <t>editie-0/carbon-alert-europa.html</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr">
         <is>
           <t>center</t>
@@ -8285,7 +8195,6 @@
           <t>De biomimetische krachtcentrale</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
           <t>Whitepaper Carbon-Alert R&amp;D: het optimaalste systeem voor energieverwerking uit biomassa over 25, 50 en 100 jaar. Drie horizonten — 2050, 2075, 2125 — met membranen, katalysatoren, actuators en kunstmatige fotosynthese.</t>
@@ -8296,7 +8205,6 @@
           <t>editie-0/biomimetische-krachtcentrale.html</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr">
         <is>
           <t>center</t>
@@ -8367,7 +8275,6 @@
           <t>Editie Europa</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
           <t>Wat Brussel, Den Haag, Berlijn en Malta cumulatief doen met de huishoudens van het continent — gespiegeld in wat Trump-II tegenover ze zet. Zeven stukken d</t>
@@ -8378,7 +8285,6 @@
           <t>editie-0/index.html</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr">
         <is>
           <t>center</t>
@@ -8459,7 +8365,6 @@
           <t>De artikelen onder Thermostaat &amp; fysieke aarde.</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr">
         <is>
           <t>center</t>
@@ -8530,7 +8435,6 @@
           <t>Uw thermostaat is slimmer dan uw minister</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>En dat is geen grapje. Dat is wiskunde.</t>
@@ -8621,7 +8525,6 @@
           <t>NEPK-FX — Neurale Voorspelling</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>Hoe de NEPK-formule structurele wisselkoersrichting voorspelt. Met concrete handelssignalen op basis van zes-maands en twaalf-maands neurale-netwerkprojecties.</t>
@@ -8712,7 +8615,6 @@
           <t>De NEPK-Klimaatlogica</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>Waarom de Nederlandse economische implosie sneller gaat dan verwacht</t>
@@ -8803,7 +8705,6 @@
           <t>De zon staat op de evenaar</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
           <t>Een Socratische confrontatie met de Nederlandse en Europese energieroute. Vijf oogkleppen, één route die wel werkt, en Europa terug op de leiderschapstroon — niet door overheersing, maar door partnerschap met de evenaar.</t>
@@ -8902,7 +8803,6 @@
           <t>De artikelen onder Autoband, plastic, vervuiling.</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr">
         <is>
           <t>center</t>
@@ -8973,7 +8873,6 @@
           <t>Autoband-sigaret</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
           <t>Bandenslijtage als verborgen vervuilingsdrager.</t>
@@ -9074,7 +8973,6 @@
           <t>De voedingslijn</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
           <t>De durf om revolutionair te zeggen dat het niet klopt ontbreekt door gebrek aan eigenkennis — een structurele fout. Heel Europa heeft zijn omwegen dichtgemetseld. De wetten van mensen kennen de toekomst niet; de natuur kent haar wel en moet weer voorop staan.</t>
@@ -9085,7 +8983,6 @@
           <t>wat-opkomt/de-methodologie-van-de-aanpassing.html</t>
         </is>
       </c>
-      <c r="J98" t="inlineStr"/>
       <c r="K98" t="inlineStr">
         <is>
           <t>center</t>
@@ -9159,7 +9056,6 @@
           <t>Natuur-analyse</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
           <t>Nederlandse cascade onder twee biomassa-sporen.</t>
@@ -9270,7 +9166,6 @@
           <t>De artikelen onder Editie Klimaat / Stikstof / Duitsland.</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr"/>
       <c r="K100" t="inlineStr">
         <is>
           <t>center</t>
@@ -9341,7 +9236,6 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
           <t>Editie Klimaat — energie, mobiliteit, verwarming, voedsel, migratie en CO₂-verwijdering. Een brede thematische editie van Het Open Vizier rond de klimaatkeuze die Europa vandaag voor zich heeft.</t>
@@ -9352,7 +9246,6 @@
           <t>editie-klimaat/index.html</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
       <c r="K101" t="inlineStr">
         <is>
           <t>center</t>
@@ -9423,7 +9316,6 @@
           <t>Editie Stikstof</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
         <is>
           <t>Alle artikelen die met de Nederlandse stikstofcrisis te maken hebben: de oplossing-architectuur, de diagnose van het beleidsfalen, het Europese kader, en de geografie van wat verhuist.</t>
@@ -9434,7 +9326,6 @@
           <t>editie-stikstof/index.html</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr"/>
       <c r="K102" t="inlineStr">
         <is>
           <t>center</t>
@@ -9505,7 +9396,6 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
         <is>
           <t>Hoe één architectuur — vorstbestendige Juncao met koude druk-explosie en mechanische verfijning — de Nederlandse stikstofcrisis, het methaan-probleem en de soja-afhankelijkheid tegelijk oplost. Met een vierde, vergeten winnaar: de boer in het transitiegebied.</t>
@@ -9516,7 +9406,6 @@
           <t>editie-stikstof/drie-problemen-een-antwoord.html</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr"/>
       <c r="K103" t="inlineStr">
         <is>
           <t>center</t>
@@ -9587,7 +9476,6 @@
           <t>Editie Duitsland</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
           <t>Carbon-Alert in Brandenburg en Mecklenburg-Voor-Pommeren, de Konsequenzkarte als instrument, en de spiegel van andere Europese landen. Met een doorverwijzing naar het Europese verhaal in Editie Europa.</t>
@@ -9598,7 +9486,6 @@
           <t>editie-duitsland/index.html</t>
         </is>
       </c>
-      <c r="J104" t="inlineStr"/>
       <c r="K104" t="inlineStr">
         <is>
           <t>center</t>
@@ -9669,7 +9556,6 @@
           <t>De Koolzaad-Multiplicator</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr">
         <is>
           <t>Brandenburg en Mecklenburg-Voor-Pommeren bouwen vandaag op circa 285.000 hectare winterkoolzaad. Met de Carbon-Alert-architectuur — vorstbestendige Juncao plus koude druk-explosie met mechanische verfijning — is op dezelfde hectare een veelvoud aan opbrengst te behalen, ingebed in het GLB-Strategisch Plan 2023-2027.</t>
@@ -9680,7 +9566,6 @@
           <t>editie-duitsland/raps-multiplicator-oost-duitsland.html</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr">
         <is>
           <t>center</t>
@@ -9761,7 +9646,6 @@
           <t>De artikelen onder Wat het niet ziet.</t>
         </is>
       </c>
-      <c r="J106" t="inlineStr"/>
       <c r="K106" t="inlineStr">
         <is>
           <t>center</t>
@@ -9832,7 +9716,6 @@
           <t>Actievoerders bouwen continenten</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
           <t>Drive zoekt grond. Wat hier schuurt, kan ginds bouwen. Een open uitnodiging aan organisaties met visie en aan iedereen die zijn energie zoekt waar zij iets kan opbouwen — niet als straf, niet als afvoer, maar als kans.</t>
@@ -9921,7 +9804,6 @@
           <t>De boer én de natuur beide vooruit</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
           <t>Van driehoeksdilemma naar vier scenario's — inclusief de radicale koevrije randzone die vijftien jaar CO₂ vangt, biodiversiteit herstelt en Natura 2000 laat ademen. Met kosten-baten-tabel per hectare per jaar.</t>
@@ -9932,7 +9814,6 @@
           <t>wat-opkomt/boer-en-natuur-beide-vooruit.html</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr"/>
       <c r="K108" t="inlineStr">
         <is>
           <t>center</t>
@@ -10201,7 +10082,6 @@
           <t>Zij doden hun levensader</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr">
         <is>
           <t>Brussel en Den Haag hebben een auto-immuunziekte. De patiënt heet Nederland. Diagnose, medische parallel, behandeling — in snijdende vorm.</t>
@@ -10212,7 +10092,6 @@
           <t>wat-opkomt/zij-doden-hun-levensader.html</t>
         </is>
       </c>
-      <c r="J111" t="inlineStr"/>
       <c r="K111" t="inlineStr">
         <is>
           <t>center</t>
@@ -10286,7 +10165,6 @@
           <t>Zij doden hun levensaders — Brussel</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
           <t>Brussel heeft een auto-immuunziekte. De patiënt heet Europa. Diagnose, medische parallel, behandeling — in snijdende vorm.</t>
@@ -10297,7 +10175,6 @@
           <t>wat-opkomt/zij-doden-hun-levensaders-brussel.html</t>
         </is>
       </c>
-      <c r="J112" t="inlineStr"/>
       <c r="K112" t="inlineStr">
         <is>
           <t>center</t>
@@ -10368,7 +10245,6 @@
           <t>Een fusiereactor zonder magnetische kooi</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr">
         <is>
           <t>Een alternatief reactorontwerp: de conische vortexreactor. Plasma wordt niet opgesloten met magneten maar versneld in een ronddraaiende stroming, vergelijkbaar met water in een wervel.</t>
@@ -10459,7 +10335,6 @@
           <t>Wat er nu al ligt</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr">
         <is>
           <t>Overzicht van technische projecten: SeaSkin, GuardSkin, AeroSkin, SolarSkin, TerraClean, Tyre-patenten, conische vortex-reactor.</t>
@@ -10560,7 +10435,6 @@
           <t>De artikelen onder Nederland.</t>
         </is>
       </c>
-      <c r="J115" t="inlineStr"/>
       <c r="K115" t="inlineStr">
         <is>
           <t>center</t>
@@ -10631,7 +10505,6 @@
           <t>Stille Analyse (NL)</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr"/>
       <c r="H116" t="inlineStr">
         <is>
           <t>20 NL-posities × 11 mechanismen, met BiCRS-uitweg.</t>
@@ -10732,7 +10605,6 @@
           <t>Zelf aan de bak (NL)</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr">
         <is>
           <t>Nederland moet zijn eigen kracht terugvinden.</t>
@@ -11129,7 +11001,6 @@
           <t>De eerste gemeente</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
         <is>
           <t>Een open en eerlijk voorstel aan wie het aandurft</t>
@@ -11140,7 +11011,6 @@
           <t>de-eerste-gemeente/index.html</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr"/>
       <c r="K121" t="inlineStr">
         <is>
           <t>center</t>
@@ -11211,7 +11081,6 @@
           <t>De halve gemeente</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
       <c r="H122" t="inlineStr">
         <is>
           <t>Wat gebeurt er met een stad als de helft van het stadhuis verdwijnt?</t>
@@ -11222,7 +11091,6 @@
           <t>de-halve-gemeente/index.html</t>
         </is>
       </c>
-      <c r="J122" t="inlineStr"/>
       <c r="K122" t="inlineStr">
         <is>
           <t>center</t>
@@ -11293,7 +11161,6 @@
           <t>Nederland · Toekomst</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr">
         <is>
           <t>Drie hervormingen voor Nederland: van fiscaal beleid via een modern selectiesysteem naar de partijen op de kaart. Wat lokaal mogelijk is op basis van het Open Vizier-gedachtegoed.</t>
@@ -11304,7 +11171,6 @@
           <t>toekomst/overheden/nederland/index.html</t>
         </is>
       </c>
-      <c r="J123" t="inlineStr"/>
       <c r="K123" t="inlineStr">
         <is>
           <t>center</t>
@@ -11375,7 +11241,6 @@
           <t>Gevolgenkaart Nederland</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr"/>
       <c r="H124" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -11386,7 +11251,6 @@
           <t>gevolgenkaart-nl/index.html</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr"/>
       <c r="K124" t="inlineStr">
         <is>
           <t>center</t>
@@ -11467,7 +11331,6 @@
           <t>De artikelen onder Europa.</t>
         </is>
       </c>
-      <c r="J125" t="inlineStr"/>
       <c r="K125" t="inlineStr">
         <is>
           <t>center</t>
@@ -11538,7 +11401,6 @@
           <t>Europa-opener</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr">
         <is>
           <t>Hoe BiCRS Green Deal en CBAM kan vervangen.</t>
@@ -11732,7 +11594,6 @@
           <t>Brusselse (EU)</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr"/>
       <c r="H128" t="inlineStr">
         <is>
           <t>20 EU-scenario's × 11 mechanismen.</t>
@@ -11833,7 +11694,6 @@
           <t>De anti-immuunziekte van Brussel maakt dat we arm worden</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr">
         <is>
           <t>CBAM, ETS, Pillar Two en vermogensbelastingen tegelijk. De BiCRS/Ethanol-route wordt genegeerd. Brussel maakt zijn eigen inwoners arm.</t>
@@ -11844,7 +11704,6 @@
           <t>wat-opkomt/de-anti-immuunziekte-van-brussel.html</t>
         </is>
       </c>
-      <c r="J129" t="inlineStr"/>
       <c r="K129" t="inlineStr">
         <is>
           <t>center</t>
@@ -11918,7 +11777,6 @@
           <t>De anti-immuunziekte van onze overheid slaat toe</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr"/>
       <c r="H130" t="inlineStr">
         <is>
           <t>Het kabinet-Jetten presenteert eind juni 2026 zijn stikstofpakket. Een aanval op het laatste productieve weefsel. En er is een andere weg.</t>
@@ -11929,7 +11787,6 @@
           <t>wat-opkomt/de-auto-immuunziekte-slaat-toe.html</t>
         </is>
       </c>
-      <c r="J130" t="inlineStr"/>
       <c r="K130" t="inlineStr">
         <is>
           <t>center</t>
@@ -12003,7 +11860,6 @@
           <t>Een staat met een auto-immuunziekte</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr">
         <is>
           <t>Een zachte, beschouwende uitleg van de medische metafoor die de Brussel-campagne van Het Open Vizier draagt. Geen aanklacht, maar een beeld om mee te denken.</t>
@@ -12014,7 +11870,6 @@
           <t>wat-opkomt/de-metafoor-auto-immuunziekte.html</t>
         </is>
       </c>
-      <c r="J131" t="inlineStr"/>
       <c r="K131" t="inlineStr">
         <is>
           <t>center</t>
@@ -12088,7 +11943,6 @@
           <t>Het immuunsysteem dat gezonde cellen aanvalt</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr">
         <is>
           <t>Waarom organisaties en politieke systemen rebellen reflexmatig uitstoten — niet uit kwaad opzet, maar uit zelfbehoud. Een opinie over hoe biomass-to-ethanol als gezonde cel in Brussel als ziektekiem wordt aangevallen, en hoe we dit immuunsysteem kunnen omzeilen.</t>
@@ -12099,7 +11953,6 @@
           <t>wat-opkomt/het-immuunsysteem-van-organisaties.html</t>
         </is>
       </c>
-      <c r="J132" t="inlineStr"/>
       <c r="K132" t="inlineStr">
         <is>
           <t>center</t>
@@ -12170,7 +12023,6 @@
           <t>Open brief aan de regeringen van Europa</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr">
         <is>
           <t>Een open brief aan de Europese Commissie, lidstaatregeringen en parlementen. 350.000 banen, €9 miljard jaaromzet, energie-onafhankelijkheid — zonder één eurocent subsidie. Begin nu met Carbon-Alert.</t>
@@ -12259,7 +12111,6 @@
           <t>De dertig cent die Europa omdraait</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr">
         <is>
           <t>Bio-ethanol uit cellulose-route haalt €0,30 per liter in 2036, zonder een cent subsidie. Combineer met de nieuwste brandstofcellen en je hebt stroom voor minder dan de helft van de Spaanse netprijs. In Den Haag, Berlijn en Brussel hoort u er niets over.</t>
@@ -12544,7 +12395,6 @@
           <t>Zij doden hun levensaders — Brussel</t>
         </is>
       </c>
-      <c r="G137" t="inlineStr"/>
       <c r="H137" t="inlineStr">
         <is>
           <t>Brussel heeft een auto-immuunziekte. De patiënt heet Europa. Diagnose, medische parallel, behandeling — in snijdende vorm.</t>
@@ -12555,7 +12405,6 @@
           <t>wat-opkomt/zij-doden-hun-levensaders-brussel.html</t>
         </is>
       </c>
-      <c r="J137" t="inlineStr"/>
       <c r="K137" t="inlineStr">
         <is>
           <t>center</t>
@@ -12626,7 +12475,6 @@
           <t>Gevolgenkaart Europa (EU-27)</t>
         </is>
       </c>
-      <c r="G138" t="inlineStr"/>
       <c r="H138" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -12637,7 +12485,6 @@
           <t>gevolgenkaart-eu/index.html</t>
         </is>
       </c>
-      <c r="J138" t="inlineStr"/>
       <c r="K138" t="inlineStr">
         <is>
           <t>center</t>
@@ -12708,7 +12555,6 @@
           <t>Europa · Toekomst</t>
         </is>
       </c>
-      <c r="G139" t="inlineStr"/>
       <c r="H139" t="inlineStr">
         <is>
           <t>Hoe Brussel anders kan werken — niet als regeltool maar als ontwerpper. Wat de Carbon-Alert-architectuur teruggeeft, en welke tegenmacht uit Zwitserland tegen blokkades helpt.</t>
@@ -12719,7 +12565,6 @@
           <t>toekomst/overheden/europa/index.html</t>
         </is>
       </c>
-      <c r="J139" t="inlineStr"/>
       <c r="K139" t="inlineStr">
         <is>
           <t>center</t>
@@ -12800,7 +12645,6 @@
           <t>De artikelen onder Andere landen.</t>
         </is>
       </c>
-      <c r="J140" t="inlineStr"/>
       <c r="K140" t="inlineStr">
         <is>
           <t>center</t>
@@ -12871,7 +12715,6 @@
           <t>Gevolgenkaart Brazilië</t>
         </is>
       </c>
-      <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -12882,7 +12725,6 @@
           <t>gevolgenkaart-br/index.html</t>
         </is>
       </c>
-      <c r="J141" t="inlineStr"/>
       <c r="K141" t="inlineStr">
         <is>
           <t>center</t>
@@ -12953,7 +12795,6 @@
           <t>Gevolgenkaart Zwitserland</t>
         </is>
       </c>
-      <c r="G142" t="inlineStr"/>
       <c r="H142" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -12964,7 +12805,6 @@
           <t>gevolgenkaart-ch/index.html</t>
         </is>
       </c>
-      <c r="J142" t="inlineStr"/>
       <c r="K142" t="inlineStr">
         <is>
           <t>center</t>
@@ -13035,7 +12875,6 @@
           <t>Zwitserse</t>
         </is>
       </c>
-      <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr">
         <is>
           <t>15 Zwitserse scenario's × Bondsraad-beleid + BiCRS.</t>
@@ -13136,7 +12975,6 @@
           <t>Gevolgenkaart China</t>
         </is>
       </c>
-      <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13147,7 +12985,6 @@
           <t>gevolgenkaart-cn/index.html</t>
         </is>
       </c>
-      <c r="J144" t="inlineStr"/>
       <c r="K144" t="inlineStr">
         <is>
           <t>center</t>
@@ -13218,7 +13055,6 @@
           <t>Gevolgenkaart Cuba</t>
         </is>
       </c>
-      <c r="G145" t="inlineStr"/>
       <c r="H145" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13229,7 +13065,6 @@
           <t>gevolgenkaart-cu/index.html</t>
         </is>
       </c>
-      <c r="J145" t="inlineStr"/>
       <c r="K145" t="inlineStr">
         <is>
           <t>center</t>
@@ -13300,7 +13135,6 @@
           <t>Gevolgenkaart Duitsland</t>
         </is>
       </c>
-      <c r="G146" t="inlineStr"/>
       <c r="H146" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13311,7 +13145,6 @@
           <t>gevolgenkaart-de/index.html</t>
         </is>
       </c>
-      <c r="J146" t="inlineStr"/>
       <c r="K146" t="inlineStr">
         <is>
           <t>center</t>
@@ -13382,7 +13215,6 @@
           <t>Konsequenzkarte (DE)</t>
         </is>
       </c>
-      <c r="G147" t="inlineStr"/>
       <c r="H147" t="inlineStr">
         <is>
           <t>Duitse spiegel, Bundestag februari 2025.</t>
@@ -13483,7 +13315,6 @@
           <t>Gevolgenkaart Spanje</t>
         </is>
       </c>
-      <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13494,7 +13325,6 @@
           <t>gevolgenkaart-es/index.html</t>
         </is>
       </c>
-      <c r="J148" t="inlineStr"/>
       <c r="K148" t="inlineStr">
         <is>
           <t>center</t>
@@ -13565,7 +13395,6 @@
           <t>Gevolgenkaart Israël</t>
         </is>
       </c>
-      <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13576,7 +13405,6 @@
           <t>gevolgenkaart-il/index.html</t>
         </is>
       </c>
-      <c r="J149" t="inlineStr"/>
       <c r="K149" t="inlineStr">
         <is>
           <t>center</t>
@@ -13647,7 +13475,6 @@
           <t>Gevolgenkaart India</t>
         </is>
       </c>
-      <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13658,7 +13485,6 @@
           <t>gevolgenkaart-in/index.html</t>
         </is>
       </c>
-      <c r="J150" t="inlineStr"/>
       <c r="K150" t="inlineStr">
         <is>
           <t>center</t>
@@ -13729,7 +13555,6 @@
           <t>Gevolgenkaart Iran</t>
         </is>
       </c>
-      <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13740,7 +13565,6 @@
           <t>gevolgenkaart-ir/index.html</t>
         </is>
       </c>
-      <c r="J151" t="inlineStr"/>
       <c r="K151" t="inlineStr">
         <is>
           <t>center</t>
@@ -13811,7 +13635,6 @@
           <t>Gevolgenkaart Japan</t>
         </is>
       </c>
-      <c r="G152" t="inlineStr"/>
       <c r="H152" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13822,7 +13645,6 @@
           <t>gevolgenkaart-jp/index.html</t>
         </is>
       </c>
-      <c r="J152" t="inlineStr"/>
       <c r="K152" t="inlineStr">
         <is>
           <t>center</t>
@@ -13893,7 +13715,6 @@
           <t>Gevolgenkaart Zuid-Korea</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr"/>
       <c r="H153" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13904,7 +13725,6 @@
           <t>gevolgenkaart-kr/index.html</t>
         </is>
       </c>
-      <c r="J153" t="inlineStr"/>
       <c r="K153" t="inlineStr">
         <is>
           <t>center</t>
@@ -13975,7 +13795,6 @@
           <t>Gevolgenkaart Zweden</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -13986,7 +13805,6 @@
           <t>gevolgenkaart-se/index.html</t>
         </is>
       </c>
-      <c r="J154" t="inlineStr"/>
       <c r="K154" t="inlineStr">
         <is>
           <t>center</t>
@@ -14057,7 +13875,6 @@
           <t>Gevolgenkaart Suriname</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -14068,7 +13885,6 @@
           <t>gevolgenkaart-sr/index.html</t>
         </is>
       </c>
-      <c r="J155" t="inlineStr"/>
       <c r="K155" t="inlineStr">
         <is>
           <t>center</t>
@@ -14139,7 +13955,6 @@
           <t>Gevolgenkaart Taiwan</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr"/>
       <c r="H156" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -14150,7 +13965,6 @@
           <t>gevolgenkaart-tw/index.html</t>
         </is>
       </c>
-      <c r="J156" t="inlineStr"/>
       <c r="K156" t="inlineStr">
         <is>
           <t>center</t>
@@ -14221,7 +14035,6 @@
           <t>Gevolgenkaart Verenigd Koninkrijk</t>
         </is>
       </c>
-      <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -14232,7 +14045,6 @@
           <t>gevolgenkaart-uk/index.html</t>
         </is>
       </c>
-      <c r="J157" t="inlineStr"/>
       <c r="K157" t="inlineStr">
         <is>
           <t>center</t>
@@ -14303,7 +14115,6 @@
           <t>Gevolgenkaart de Verenigde Staten</t>
         </is>
       </c>
-      <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -14314,7 +14125,6 @@
           <t>gevolgenkaart-us/index.html</t>
         </is>
       </c>
-      <c r="J158" t="inlineStr"/>
       <c r="K158" t="inlineStr">
         <is>
           <t>center</t>
@@ -14385,7 +14195,6 @@
           <t>Gevolgenkaart Zuid-Afrika</t>
         </is>
       </c>
-      <c r="G159" t="inlineStr"/>
       <c r="H159" t="inlineStr">
         <is>
           <t>Een persoonlijke politieke bijsluiter: wat betekent een stem op een partij voor uw sector? De cascade-effecten in drie ordes, jaar 1 tot jaar 10.</t>
@@ -14396,7 +14205,6 @@
           <t>gevolgenkaart-za/index.html</t>
         </is>
       </c>
-      <c r="J159" t="inlineStr"/>
       <c r="K159" t="inlineStr">
         <is>
           <t>center</t>
@@ -14467,7 +14275,6 @@
           <t>Mappa Malta</t>
         </is>
       </c>
-      <c r="G160" t="inlineStr"/>
       <c r="H160" t="inlineStr">
         <is>
           <t>Maltese politiek en EU-druk samen.</t>
@@ -14568,7 +14375,6 @@
           <t>Singaporese</t>
         </is>
       </c>
-      <c r="G161" t="inlineStr"/>
       <c r="H161" t="inlineStr">
         <is>
           <t>15 SG scenario's × MOF/MAS/MOM + BiCRS-uitweg.</t>
@@ -14669,7 +14475,6 @@
           <t>Trump als spiegel</t>
         </is>
       </c>
-      <c r="G162" t="inlineStr"/>
       <c r="H162" t="inlineStr">
         <is>
           <t>Wat Trump-II met Europa doet.</t>
@@ -14770,7 +14575,6 @@
           <t>Duitsland · Toekomst</t>
         </is>
       </c>
-      <c r="G163" t="inlineStr"/>
       <c r="H163" t="inlineStr">
         <is>
           <t>Een eerste artikel over Duitsland: de Koolzaad-Multiplicator als regionale uitvoering van de Carbon-Alert-architectuur in Brandenburg en Mecklenburg-Voor-Pommeren.</t>
@@ -14781,7 +14585,6 @@
           <t>toekomst/overheden/duitsland/index.html</t>
         </is>
       </c>
-      <c r="J163" t="inlineStr"/>
       <c r="K163" t="inlineStr">
         <is>
           <t>center</t>
@@ -14862,7 +14665,6 @@
           <t>De artikelen onder Nova Democratia &amp; institutioneel ontwerp.</t>
         </is>
       </c>
-      <c r="J164" t="inlineStr"/>
       <c r="K164" t="inlineStr">
         <is>
           <t>center</t>
@@ -14933,7 +14735,6 @@
           <t>Nova Democratia — Het Open Vizier · Editie 6 — Juni 2026</t>
         </is>
       </c>
-      <c r="G165" t="inlineStr"/>
       <c r="H165" t="inlineStr">
         <is>
           <t>Een editie over de fysica van de Nederlandse hervorming — Pareto, ordes, het ontwerp dat werkt, en de kennislaag die de behoudende kracht draagt. Veertien stukken.</t>
@@ -14944,7 +14745,6 @@
           <t>editie-6/index.html</t>
         </is>
       </c>
-      <c r="J165" t="inlineStr"/>
       <c r="K165" t="inlineStr">
         <is>
           <t>center</t>
@@ -15015,8 +14815,6 @@
           <t>Voorwoord — Waarom dit moet</t>
         </is>
       </c>
-      <c r="G166" t="inlineStr"/>
-      <c r="H166" t="inlineStr"/>
       <c r="I166" t="inlineStr">
         <is>
           <t>editie-6/voorwoord-waarom-dit-moet.html</t>
@@ -15102,8 +14900,6 @@
           <t>Brussel als variabele, niet als constante</t>
         </is>
       </c>
-      <c r="G167" t="inlineStr"/>
-      <c r="H167" t="inlineStr"/>
       <c r="I167" t="inlineStr">
         <is>
           <t>editie-6/aflevering-00-brussel-als-variabele.html</t>
@@ -15189,8 +14985,6 @@
           <t>De zes ordes van fasering</t>
         </is>
       </c>
-      <c r="G168" t="inlineStr"/>
-      <c r="H168" t="inlineStr"/>
       <c r="I168" t="inlineStr">
         <is>
           <t>editie-6/aflevering-01-zes-ordes-van-fasering.html</t>
@@ -15276,8 +15070,6 @@
           <t>Wie blokkeert, en hoe zwaar?</t>
         </is>
       </c>
-      <c r="G169" t="inlineStr"/>
-      <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr">
         <is>
           <t>editie-6/aflevering-02-pareto-top12.html</t>
@@ -15363,8 +15155,6 @@
           <t>Media als rekstrook</t>
         </is>
       </c>
-      <c r="G170" t="inlineStr"/>
-      <c r="H170" t="inlineStr"/>
       <c r="I170" t="inlineStr">
         <is>
           <t>editie-6/aflevering-03-media-als-rekstrook.html</t>
@@ -15450,8 +15240,6 @@
           <t>Ordes van bezwaar</t>
         </is>
       </c>
-      <c r="G171" t="inlineStr"/>
-      <c r="H171" t="inlineStr"/>
       <c r="I171" t="inlineStr">
         <is>
           <t>editie-6/aflevering-04-ordes-van-bezwaar.html</t>
@@ -15537,8 +15325,6 @@
           <t>Twintig actuele bezwaren</t>
         </is>
       </c>
-      <c r="G172" t="inlineStr"/>
-      <c r="H172" t="inlineStr"/>
       <c r="I172" t="inlineStr">
         <is>
           <t>editie-6/aflevering-05-twintig-bezwaren.html</t>
@@ -15624,8 +15410,6 @@
           <t>De Zwitserse spiegel</t>
         </is>
       </c>
-      <c r="G173" t="inlineStr"/>
-      <c r="H173" t="inlineStr"/>
       <c r="I173" t="inlineStr">
         <is>
           <t>editie-6/aflevering-06-zwitserse-spiegel.html</t>
@@ -15711,8 +15495,6 @@
           <t>De Canadese spiegel</t>
         </is>
       </c>
-      <c r="G174" t="inlineStr"/>
-      <c r="H174" t="inlineStr"/>
       <c r="I174" t="inlineStr">
         <is>
           <t>editie-6/aflevering-07-canadese-spiegel.html</t>
@@ -15798,8 +15580,6 @@
           <t>Waar staat uw partij?</t>
         </is>
       </c>
-      <c r="G175" t="inlineStr"/>
-      <c r="H175" t="inlineStr"/>
       <c r="I175" t="inlineStr">
         <is>
           <t>editie-6/aflevering-08-partijen-in-kaart.html</t>
@@ -15885,8 +15665,6 @@
           <t>Wie verzet zich, wie helpt mee?</t>
         </is>
       </c>
-      <c r="G176" t="inlineStr"/>
-      <c r="H176" t="inlineStr"/>
       <c r="I176" t="inlineStr">
         <is>
           <t>editie-6/aflevering-09-pareto-per-actor.html</t>
@@ -15972,8 +15750,6 @@
           <t>UEI — een Europese tegenmacht uit Zwitserland</t>
         </is>
       </c>
-      <c r="G177" t="inlineStr"/>
-      <c r="H177" t="inlineStr"/>
       <c r="I177" t="inlineStr">
         <is>
           <t>editie-6/aflevering-10-uei.html</t>
@@ -16059,8 +15835,6 @@
           <t>De kennislaag als bondgenoot</t>
         </is>
       </c>
-      <c r="G178" t="inlineStr"/>
-      <c r="H178" t="inlineStr"/>
       <c r="I178" t="inlineStr">
         <is>
           <t>editie-6/aflevering-11-kennislaag-als-bondgenoot.html</t>
@@ -16146,8 +15920,6 @@
           <t>De beste weg vooruit</t>
         </is>
       </c>
-      <c r="G179" t="inlineStr"/>
-      <c r="H179" t="inlineStr"/>
       <c r="I179" t="inlineStr">
         <is>
           <t>editie-6/aflevering-12-beste-weg-vooruit.html</t>
@@ -16233,7 +16005,6 @@
           <t>Wat is er mis met partijpolitiek?</t>
         </is>
       </c>
-      <c r="G180" t="inlineStr"/>
       <c r="H180" t="inlineStr">
         <is>
           <t>Partijpolitiek bundelt belangen die niets met elkaar te maken hebben. Nova Democratia stelt voor per onderwerp te beslissen, met meetbare prijs-prestatie.</t>
@@ -16324,7 +16095,6 @@
           <t>Nova Democratia</t>
         </is>
       </c>
-      <c r="G181" t="inlineStr"/>
       <c r="H181" t="inlineStr">
         <is>
           <t>Een nieuw politiek-staatkundig model — grondslagdocument</t>
@@ -16415,7 +16185,6 @@
           <t>Nova Democratia</t>
         </is>
       </c>
-      <c r="G182" t="inlineStr"/>
       <c r="H182" t="inlineStr">
         <is>
           <t>De Nova Democratia / VMP politieke vorm.</t>
@@ -16521,7 +16290,6 @@
           <t>De actor is de regel</t>
         </is>
       </c>
-      <c r="G183" t="inlineStr"/>
       <c r="H183" t="inlineStr">
         <is>
           <t>Waarom hervorming onmogelijk is en vervanging onvermijdelijk. Een revolutie-bijdrage die de tetralogie sluit: van oergevoel via scholing en eigenkennis-tekort naar auto-immuun-instituties — en de medische therapieën die ons leren hoe genezing eruitziet.</t>
@@ -16532,7 +16300,6 @@
           <t>wat-opkomt/de-actor-is-de-regel.html</t>
         </is>
       </c>
-      <c r="J183" t="inlineStr"/>
       <c r="K183" t="inlineStr">
         <is>
           <t>center</t>
@@ -16603,7 +16370,6 @@
           <t>Soevereiniteit als cyclus</t>
         </is>
       </c>
-      <c r="G184" t="inlineStr"/>
       <c r="H184" t="inlineStr">
         <is>
           <t>Een uitweg uit het oudste dilemma van de staatstheorie</t>
@@ -16614,7 +16380,6 @@
           <t>soevereiniteit-als-cyclus/index.html</t>
         </is>
       </c>
-      <c r="J184" t="inlineStr"/>
       <c r="K184" t="inlineStr">
         <is>
           <t>center</t>
@@ -16685,7 +16450,6 @@
           <t>Beslissen zonder uitzicht</t>
         </is>
       </c>
-      <c r="G185" t="inlineStr"/>
       <c r="H185" t="inlineStr">
         <is>
           <t>Het BBP telt €419 miljard aan lucht als productie. De Nederlandse schuldquote is niet 43%. Zij is 69%. Ver boven de EU-alarmgrens. En het parlement stemt met de ogen dicht.</t>
@@ -16774,7 +16538,6 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
-      <c r="G186" t="inlineStr"/>
       <c r="H186" t="inlineStr">
         <is>
           <t>Hoe blokkades worden ontgrendeld: Nova Democratia als grondslag, Pareto-analyse om te zien wie blokkeert, en spiegels uit Zwitserland en Canada om te zien wat elders al werkt. Vijftien artikelen verdeeld over drie groepen.</t>
@@ -16785,7 +16548,6 @@
           <t>toekomst/overheden/methode/index.html</t>
         </is>
       </c>
-      <c r="J186" t="inlineStr"/>
       <c r="K186" t="inlineStr">
         <is>
           <t>center</t>
@@ -16856,7 +16618,6 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
-      <c r="G187" t="inlineStr"/>
       <c r="H187" t="inlineStr">
         <is>
           <t>Drie landen, één methode. Wat lokaal mogelijk is in Nederland, Duitsland en Europa — en de instrumenten en spiegels waarmee dat lukt.</t>
@@ -16867,7 +16628,6 @@
           <t>toekomst/overheden/index.html</t>
         </is>
       </c>
-      <c r="J187" t="inlineStr"/>
       <c r="K187" t="inlineStr">
         <is>
           <t>center</t>
@@ -16948,7 +16708,6 @@
           <t>De artikelen onder Leiderschap &amp; organisaties.</t>
         </is>
       </c>
-      <c r="J188" t="inlineStr"/>
       <c r="K188" t="inlineStr">
         <is>
           <t>center</t>
@@ -17019,7 +16778,6 @@
           <t>Hoe de papier-industrie macht kreeg over het echte werk — Het Open Vizier · Editie 4 — Juni 2026</t>
         </is>
       </c>
-      <c r="G189" t="inlineStr"/>
       <c r="H189" t="inlineStr">
         <is>
           <t>Een editie over hoe regels, verzekeringen, financiering en toezicht het oergevoel uit de beroepspraktijk hebben gewrongen — en wat dat met ons heeft gedaan.</t>
@@ -17030,7 +16788,6 @@
           <t>editie-4/index.html</t>
         </is>
       </c>
-      <c r="J189" t="inlineStr"/>
       <c r="K189" t="inlineStr">
         <is>
           <t>center</t>
@@ -17101,7 +16858,6 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
-      <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr">
         <is>
           <t>Waar deze editie heen gaat en waarom</t>
@@ -17192,7 +16948,6 @@
           <t>De wet van de papier-industrie</t>
         </is>
       </c>
-      <c r="G191" t="inlineStr"/>
       <c r="H191" t="inlineStr">
         <is>
           <t>Hoe regels, verzekeringen en financiering het echte werk verdrongen</t>
@@ -17283,7 +17038,6 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
-      <c r="G192" t="inlineStr"/>
       <c r="H192" t="inlineStr">
         <is>
           <t>Wat een leidinggevende verliest als hij alleen op cijfers stuurt</t>
@@ -17374,7 +17128,6 @@
           <t>De consultant bij het bijna-failliete bedrijf</t>
         </is>
       </c>
-      <c r="G193" t="inlineStr"/>
       <c r="H193" t="inlineStr">
         <is>
           <t>Waarom een buitenstaander binnen drie dagen weet wat insiders niet kunnen zien</t>
@@ -17465,7 +17218,6 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
-      <c r="G194" t="inlineStr"/>
       <c r="H194" t="inlineStr">
         <is>
           <t>Waarom alleen wie het niet nodig heeft krediet krijgt</t>
@@ -17556,7 +17308,6 @@
           <t>De verzekeraar tegen het leven</t>
         </is>
       </c>
-      <c r="G195" t="inlineStr"/>
       <c r="H195" t="inlineStr">
         <is>
           <t>Hoe risico-mijding zelf het grootste risico werd</t>
@@ -17647,7 +17398,6 @@
           <t>De toezichthouder die niets ziet</t>
         </is>
       </c>
-      <c r="G196" t="inlineStr"/>
       <c r="H196" t="inlineStr">
         <is>
           <t>Inspectie zonder oergevoel is administratie van het verleden</t>
@@ -17738,7 +17488,6 @@
           <t>De rechter zonder kompas</t>
         </is>
       </c>
-      <c r="G197" t="inlineStr"/>
       <c r="H197" t="inlineStr">
         <is>
           <t>Recht spreken op basis van paragrafen in plaats van mensen</t>
@@ -17829,7 +17578,6 @@
           <t>De diepere vraag</t>
         </is>
       </c>
-      <c r="G198" t="inlineStr"/>
       <c r="H198" t="inlineStr">
         <is>
           <t>Waarom een hele samenleving haar oergevoel kwijtraakte</t>
@@ -17920,7 +17668,6 @@
           <t>Retrospectief</t>
         </is>
       </c>
-      <c r="G199" t="inlineStr"/>
       <c r="H199" t="inlineStr">
         <is>
           <t>Wat deze editie samen vertelt</t>
@@ -18011,7 +17758,6 @@
           <t>Editie Leiderschap</t>
         </is>
       </c>
-      <c r="G200" t="inlineStr"/>
       <c r="H200" t="inlineStr">
         <is>
           <t>Gevoelsleiden boven verstandsleiden. Het verstandsleiden dat nu domineert verlamt het organisme. Twaalf artikelen over hoe het oergevoel werkelijk leidt — bij de CEO, in het bestuur, in de politiek.</t>
@@ -18022,7 +17768,6 @@
           <t>editie-leiderschap/index.html</t>
         </is>
       </c>
-      <c r="J200" t="inlineStr"/>
       <c r="K200" t="inlineStr">
         <is>
           <t>center</t>
@@ -18103,7 +17848,6 @@
           <t>De artikelen onder Onderwijs.</t>
         </is>
       </c>
-      <c r="J201" t="inlineStr"/>
       <c r="K201" t="inlineStr">
         <is>
           <t>center</t>
@@ -18174,7 +17918,6 @@
           <t>Kies een kant</t>
         </is>
       </c>
-      <c r="G202" t="inlineStr"/>
       <c r="H202" t="inlineStr">
         <is>
           <t>Het sluitstuk van de onderwijs-trilogie: wat wij wel kunnen redden, wat wij niet meer kunnen redden, en waarom u zich nu moet uitspreken.</t>
@@ -18265,7 +18008,6 @@
           <t>Terug naar de werkbank, vooruit naar het denken</t>
         </is>
       </c>
-      <c r="G203" t="inlineStr"/>
       <c r="H203" t="inlineStr">
         <is>
           <t>Onderwijs-trilogie · Deel I — Eenvoudig herstel van kwaliteit, vakmanschap en breedte. Vóór een land dat zichzelf weg-diplomeert en zijn ambacht vergeet.</t>
@@ -18356,7 +18098,6 @@
           <t>De prijs van de bloei</t>
         </is>
       </c>
-      <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr">
         <is>
           <t>Onderwijs-trilogie · Deel II — Wat het kost om het Nederlandse onderwijs te herstellen. Over geld, gemak, en wie de rekening voelt.</t>
@@ -18447,7 +18188,6 @@
           <t>Van leerfabriek naar leerwerkplaats</t>
         </is>
       </c>
-      <c r="G205" t="inlineStr"/>
       <c r="H205" t="inlineStr">
         <is>
           <t>Voorstellen voor radicale onderwijshervorming: bekostiging op uitkomst, strengere toelating, risico terug in de kindertijd, vakmensen weer in ere.</t>
@@ -18538,7 +18278,6 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
-      <c r="G206" t="inlineStr"/>
       <c r="H206" t="inlineStr">
         <is>
           <t>Waarom alles wat we nu leren straks niet meer telt</t>
@@ -18629,7 +18368,6 @@
           <t>Editie Kind &amp;amp; Loopbaan</t>
         </is>
       </c>
-      <c r="G207" t="inlineStr"/>
       <c r="H207" t="inlineStr">
         <is>
           <t>Het kind als toekomstig mens. Oergevoel als beginsel, scholing als instrument, loopbaan als bestemming. Dertien artikelen over hoe wij de volgende generatie vormgeven en wat dat betekent voor hun werk en plaats in de wereld.</t>
@@ -18640,7 +18378,6 @@
           <t>editie-kind-loopbaan/index.html</t>
         </is>
       </c>
-      <c r="J207" t="inlineStr"/>
       <c r="K207" t="inlineStr">
         <is>
           <t>center</t>
@@ -18711,7 +18448,6 @@
           <t>Opvoeding · Toekomst</t>
         </is>
       </c>
-      <c r="G208" t="inlineStr"/>
       <c r="H208" t="inlineStr">
         <is>
           <t>Drie vragen onder één onderwerp: hoe het zich heeft ontwikkeld, hoe het zou kunnen gaan, en hoe opvoeding er werkelijk uit zou moeten zien. Vier artikelen verdeeld over die drie vragen.</t>
@@ -18722,7 +18458,6 @@
           <t>toekomst/opvoeding/index.html</t>
         </is>
       </c>
-      <c r="J208" t="inlineStr"/>
       <c r="K208" t="inlineStr">
         <is>
           <t>center</t>
@@ -18793,7 +18528,6 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
-      <c r="G209" t="inlineStr"/>
       <c r="H209" t="inlineStr">
         <is>
           <t>Drie vragen onder één onderwerp: hoe scholing zich heeft ontwikkeld, hoe de evolutie zou kunnen gaan, en hoe scholing zou moeten worden ingericht om de kennis die wij hebben werkelijk te benutten. Vijf artikelen verdeeld over die drie vragen.</t>
@@ -18804,7 +18538,6 @@
           <t>toekomst/scholing/index.html</t>
         </is>
       </c>
-      <c r="J209" t="inlineStr"/>
       <c r="K209" t="inlineStr">
         <is>
           <t>center</t>
@@ -18885,7 +18618,6 @@
           <t>De artikelen onder Industrie, energie, toekomst.</t>
         </is>
       </c>
-      <c r="J210" t="inlineStr"/>
       <c r="K210" t="inlineStr">
         <is>
           <t>center</t>
@@ -19056,7 +18788,6 @@
           <t>Wie zijn opbouwers wegjaagt</t>
         </is>
       </c>
-      <c r="G212" t="inlineStr"/>
       <c r="H212" t="inlineStr">
         <is>
           <t>Een waarneming van Jacobus van Merksteijn. Dit stuk is geen analyse, geen onderzoek en geen advies. Het is een observatie — bedoeld om ogen te openen en de discussie te voeden.</t>
@@ -19067,7 +18798,6 @@
           <t>opbouwers-wegjagen/index.html</t>
         </is>
       </c>
-      <c r="J212" t="inlineStr"/>
       <c r="K212" t="inlineStr">
         <is>
           <t>center</t>
@@ -19138,7 +18868,6 @@
           <t>Toekomst</t>
         </is>
       </c>
-      <c r="G213" t="inlineStr"/>
       <c r="H213" t="inlineStr">
         <is>
           <t>Vragen die over generaties heen spelen — opvoeding, scholing, energie, overheden, industrie. Geen losse artikelen maar een vaste plek waar het denken over de lange termijn wordt verzameld.</t>
@@ -19149,7 +18878,6 @@
           <t>toekomst/index.html</t>
         </is>
       </c>
-      <c r="J213" t="inlineStr"/>
       <c r="K213" t="inlineStr">
         <is>
           <t>center</t>
@@ -19220,7 +18948,6 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
-      <c r="G214" t="inlineStr"/>
       <c r="H214" t="inlineStr">
         <is>
           <t>Drie vragen onder één onderwerp: hoe energie wordt opgewekt en verdeeld, hoe de evolutie zou kunnen gaan, en hoe de architectuur er op Europese schaal uit zou moeten zien. Vijf artikelen verdeeld over die drie vragen.</t>
@@ -19231,7 +18958,6 @@
           <t>toekomst/energie/index.html</t>
         </is>
       </c>
-      <c r="J214" t="inlineStr"/>
       <c r="K214" t="inlineStr">
         <is>
           <t>center</t>
@@ -19302,7 +19028,6 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
-      <c r="G215" t="inlineStr"/>
       <c r="H215" t="inlineStr">
         <is>
           <t>Drie vragen onder één onderwerp: hoe maakindustrie het oergevoel verloor, welke instrumenten daadwerkelijk werken, en hoe scholing en vakmanschap terug kunnen komen. Twaalf artikelen verdeeld over die drie vragen.</t>
@@ -19313,7 +19038,6 @@
           <t>toekomst/industrie/index.html</t>
         </is>
       </c>
-      <c r="J215" t="inlineStr"/>
       <c r="K215" t="inlineStr">
         <is>
           <t>center</t>
@@ -19675,7 +19399,6 @@
           <t>Kantelmechanica</t>
         </is>
       </c>
-      <c r="G219" t="inlineStr"/>
       <c r="H219" t="inlineStr">
         <is>
           <t>Hoe een gedachtegoed kantelt naar invloed.</t>
@@ -19776,7 +19499,6 @@
           <t>Mensen die mee bouwen</t>
         </is>
       </c>
-      <c r="G220" t="inlineStr"/>
       <c r="H220" t="inlineStr">
         <is>
           <t>Tropische ethanol-steden 2040. Een visionair stuk over wie Europa's energietoekomst kan helpen bouwen — als we de moed hebben de migratiekwestie en de energietransitie samen te denken. Goede huizen, scholen, bibliotheken, internet. Niet wegsturen, niet binnenhouden — verder gaan.</t>
@@ -19865,7 +19587,6 @@
           <t>De vergeten orde — Het Open Vizier · Editie 5 — Juli 2026</t>
         </is>
       </c>
-      <c r="G221" t="inlineStr"/>
       <c r="H221" t="inlineStr">
         <is>
           <t>Wat zwaar weegt, en wat de pers ervan maakt. Een diagnostische editie in vier delen.</t>
@@ -19876,7 +19597,6 @@
           <t>editie-5/index.html</t>
         </is>
       </c>
-      <c r="J221" t="inlineStr"/>
       <c r="K221" t="inlineStr">
         <is>
           <t>center</t>
@@ -19947,7 +19667,6 @@
           <t>Brief aan de lezer</t>
         </is>
       </c>
-      <c r="G222" t="inlineStr"/>
       <c r="H222" t="inlineStr">
         <is>
           <t>Editie 5 levert geen mening af, maar een instrument.</t>
@@ -20038,7 +19757,6 @@
           <t>七つ道具 — De zeven die het verschil maakten</t>
         </is>
       </c>
-      <c r="G223" t="inlineStr"/>
       <c r="H223" t="inlineStr">
         <is>
           <t>Kaoru Ishikawa's zeven kwaliteitsinstrumenten, plus orde-analyse uit de staalbouw. Het gereedschap waarmee Japan ons inhaalde.</t>
@@ -20129,7 +19847,6 @@
           <t>De succesformule die wij verleerd hebben</t>
         </is>
       </c>
-      <c r="G224" t="inlineStr"/>
       <c r="H224" t="inlineStr">
         <is>
           <t>Japan, Korea en China zijn ons ingehaald omdat ze het instrument omarmden dat wij hebben weggegooid.</t>
@@ -20220,7 +19937,6 @@
           <t>De vergeten orde</t>
         </is>
       </c>
-      <c r="G225" t="inlineStr"/>
       <c r="H225" t="inlineStr">
         <is>
           <t>Drie tradities, één principe: wat 5× kleiner bijdraagt dan de hoofdfactor, telt niet mee.</t>
@@ -20311,7 +20027,6 @@
           <t>De methaan-misleiding</t>
         </is>
       </c>
-      <c r="G226" t="inlineStr"/>
       <c r="H226" t="inlineStr">
         <is>
           <t>Drie FD-stukken in één week, drie omkeringen van zwaarte, vier eisen aan de pers.</t>
@@ -20402,7 +20117,6 @@
           <t>De plant die verhuist</t>
         </is>
       </c>
-      <c r="G227" t="inlineStr"/>
       <c r="H227" t="inlineStr">
         <is>
           <t>Stikstof, droogte, klimaatverschuiving, fragmentatie — en het beleid dat slechts één van de vier ziet.</t>
@@ -20493,7 +20207,6 @@
           <t>De zeven van Bern</t>
         </is>
       </c>
-      <c r="G228" t="inlineStr"/>
       <c r="H228" t="inlineStr">
         <is>
           <t>Een collegiale democratie als sluitsteen — wat Zwitserland in 1848 deed wat wij hadden kunnen overnemen, en wat de NEPK-cijfers van eenentwintig landen ervan laten zien.</t>
@@ -20584,7 +20297,6 @@
           <t>De afwijkers</t>
         </is>
       </c>
-      <c r="G229" t="inlineStr"/>
       <c r="H229" t="inlineStr">
         <is>
           <t>Sandra Palmen-Schlangen, Eva González Pérez, Ad Bos — drie geverifieerde kompasdragers.</t>
@@ -20675,7 +20387,6 @@
           <t>De eis aan de lezer</t>
         </is>
       </c>
-      <c r="G230" t="inlineStr"/>
       <c r="H230" t="inlineStr">
         <is>
           <t>Wat u kunt doen met dit instrument — en waarom dát is wat de papier-industrie het minst kan dragen.</t>
@@ -20766,7 +20477,6 @@
           <t>Veerkracht en Selectie</t>
         </is>
       </c>
-      <c r="G231" t="inlineStr"/>
       <c r="H231" t="inlineStr">
         <is>
           <t>Hoe de overheid een modern selectiesysteem kan aansturen. Een radicaal herstructureringsprogramma: bescherm de productieve kern, bouw interne diensten af, met behoud van basiszekerheid.</t>
@@ -20857,14 +20567,11 @@
           <t>Editie 1</t>
         </is>
       </c>
-      <c r="G232" t="inlineStr"/>
-      <c r="H232" t="inlineStr"/>
       <c r="I232" t="inlineStr">
         <is>
           <t>editie-1/index.html</t>
         </is>
       </c>
-      <c r="J232" t="inlineStr"/>
       <c r="K232" t="inlineStr">
         <is>
           <t>center</t>
@@ -21229,7 +20936,6 @@
           <t>De Grote Plundering</t>
         </is>
       </c>
-      <c r="G236" t="inlineStr"/>
       <c r="H236" t="inlineStr">
         <is>
           <t>Vijfluik over hoe Europa zijn productieven uitkleedt.</t>
@@ -21320,7 +21026,6 @@
           <t>Eerst plukken, dan oordelen</t>
         </is>
       </c>
-      <c r="G237" t="inlineStr"/>
       <c r="H237" t="inlineStr">
         <is>
           <t>De cirkel van onrecht waarin Europa zichzelf vernietigt</t>
@@ -21421,7 +21126,6 @@
           <t>Plundering 1: diagnose</t>
         </is>
       </c>
-      <c r="G238" t="inlineStr"/>
       <c r="H238" t="inlineStr">
         <is>
           <t>Wij plukken wie ons voedt</t>
@@ -21522,7 +21226,6 @@
           <t>Plundering 2: mechaniek</t>
         </is>
       </c>
-      <c r="G239" t="inlineStr"/>
       <c r="H239" t="inlineStr">
         <is>
           <t>De muren die wij hebben gemetseld om onze bouwers op te sluiten</t>
@@ -21623,7 +21326,6 @@
           <t>Plundering 3: afloop</t>
         </is>
       </c>
-      <c r="G240" t="inlineStr"/>
       <c r="H240" t="inlineStr">
         <is>
           <t>Waarom de plunderaars zwaarder zullen lijden dan de geplunderden</t>
@@ -21724,7 +21426,6 @@
           <t>Plundering 4: politiek</t>
         </is>
       </c>
-      <c r="G241" t="inlineStr"/>
       <c r="H241" t="inlineStr">
         <is>
           <t>Wie wil wat, en waarom Brussel niet weet hoe verder</t>
@@ -22023,7 +21724,6 @@
           <t>Ferrari Junção</t>
         </is>
       </c>
-      <c r="G244" t="inlineStr"/>
       <c r="H244" t="inlineStr">
         <is>
           <t>Dagelijks idee: Ferrari Junção.</t>
@@ -22124,7 +21824,6 @@
           <t>VMB ESG</t>
         </is>
       </c>
-      <c r="G245" t="inlineStr"/>
       <c r="H245" t="inlineStr">
         <is>
           <t>Wat ik achterlaat — VMB ESG essay.</t>
@@ -22225,7 +21924,6 @@
           <t>Manifest</t>
         </is>
       </c>
-      <c r="G246" t="inlineStr"/>
       <c r="H246" t="inlineStr">
         <is>
           <t>Waarom de StemWijzer u nooit zal vertellen wat u eigenlijk stemt.</t>
@@ -22326,14 +22024,11 @@
           <t>Beleidsadvies aantrekken</t>
         </is>
       </c>
-      <c r="G247" t="inlineStr"/>
-      <c r="H247" t="inlineStr"/>
       <c r="I247" t="inlineStr">
         <is>
           <t>wat-opkomt/beleidsadvies-aantrekken.html</t>
         </is>
       </c>
-      <c r="J247" t="inlineStr"/>
       <c r="K247" t="inlineStr">
         <is>
           <t>center</t>
@@ -22502,7 +22197,6 @@
           <t>Gevolgenkaart</t>
         </is>
       </c>
-      <c r="G249" t="inlineStr"/>
       <c r="H249" t="inlineStr">
         <is>
           <t>Partij × Persoon × Basislijn = Projectie</t>
@@ -22513,7 +22207,6 @@
           <t>stemgedrag.html</t>
         </is>
       </c>
-      <c r="J249" t="inlineStr"/>
       <c r="K249" t="inlineStr">
         <is>
           <t>center</t>
@@ -22584,7 +22277,6 @@
           <t>Beslissen zonder uitzicht</t>
         </is>
       </c>
-      <c r="G250" t="inlineStr"/>
       <c r="H250" t="inlineStr">
         <is>
           <t>Het BBP telt €419 miljard aan lucht als productie. De Nederlandse schuldquote is niet 43%. Zij is 69%. Ver boven de EU-alarmgrens. En het parlement stemt met de ogen dicht.</t>
@@ -22673,7 +22365,6 @@
           <t>Dossiers</t>
         </is>
       </c>
-      <c r="G251" t="inlineStr"/>
       <c r="H251" t="inlineStr">
         <is>
           <t>Diepte-dossiers van Het Open Vizier. Businessplannen, technologie-dossiers, IP-strategieën — voor wie verder wil dan de krantenkop.</t>
@@ -22684,7 +22375,6 @@
           <t>dossiers/index.html</t>
         </is>
       </c>
-      <c r="J251" t="inlineStr"/>
       <c r="K251" t="inlineStr">
         <is>
           <t>center</t>
@@ -22755,7 +22445,6 @@
           <t>Vortex-Hair™ Adaptive Dimple Golf Ball — Dossier · Het Open Vizier</t>
         </is>
       </c>
-      <c r="G252" t="inlineStr"/>
       <c r="H252" t="inlineStr">
         <is>
           <t>Businessplan-dossier voor de Vortex-Hair™ golfbal: flexibele micro-filamenten in elke dimple voor 5–15% extra carry distance. IP-strategie, licentiemodellen en marktanalyse.</t>
@@ -22766,7 +22455,6 @@
           <t>dossiers/vortex-hair.html</t>
         </is>
       </c>
-      <c r="J252" t="inlineStr"/>
       <c r="K252" t="inlineStr">
         <is>
           <t>center</t>
@@ -22837,7 +22525,6 @@
           <t>Achter de Cijfers</t>
         </is>
       </c>
-      <c r="G253" t="inlineStr"/>
       <c r="H253" t="inlineStr">
         <is>
           <t>Onderzoek &amp;amp; technische analyses bij Het Open Vizier. Voor wie achter de cijfers wil kijken.</t>
@@ -22848,7 +22535,6 @@
           <t>onderzoek/index.html</t>
         </is>
       </c>
-      <c r="J253" t="inlineStr"/>
       <c r="K253" t="inlineStr">
         <is>
           <t>center</t>
@@ -22919,7 +22605,6 @@
           <t>EU: BBP, Reële Lonen en de Overheidsmultiplicator</t>
         </is>
       </c>
-      <c r="G254" t="inlineStr"/>
       <c r="H254" t="inlineStr">
         <is>
           <t>Bbp-loonmaat na aftrek van groei van totale overheidskosten — wat blijft over aan macro-economische ruimte?</t>
@@ -22930,7 +22615,6 @@
           <t>onderzoek/eu-multiplicator.html</t>
         </is>
       </c>
-      <c r="J254" t="inlineStr"/>
       <c r="K254" t="inlineStr">
         <is>
           <t>center</t>
@@ -23001,7 +22685,6 @@
           <t>Is Nederland op weg naar ontwikkelingslandstatus? — Het Open Vizier · Achter de Cijfers</t>
         </is>
       </c>
-      <c r="G255" t="inlineStr"/>
       <c r="H255" t="inlineStr">
         <is>
           <t>Een data-gedreven analyse van faillissementen, bedrijfsuitval, werkgelegenheid en de-industrialisatie in Nederland — 2000 tot en met 2026</t>
@@ -23012,7 +22695,6 @@
           <t>onderzoek/ontwikkelingslandstatus.html</t>
         </is>
       </c>
-      <c r="J255" t="inlineStr"/>
       <c r="K255" t="inlineStr">
         <is>
           <t>center</t>
@@ -23083,7 +22765,6 @@
           <t>Onderzoek</t>
         </is>
       </c>
-      <c r="G256" t="inlineStr"/>
       <c r="H256" t="inlineStr">
         <is>
           <t>Onderzoekslijnen die nog open staan. Plannen, hypothesen en metingen die op tafel liggen — niet als afgesloten verhaal, maar als uitnodiging om mee te denken.</t>
@@ -23094,7 +22775,6 @@
           <t>onderzoeken/index.html</t>
         </is>
       </c>
-      <c r="J256" t="inlineStr"/>
       <c r="K256" t="inlineStr">
         <is>
           <t>center</t>
@@ -23170,7 +22850,6 @@
           <t>wie maakt dit</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr"/>
       <c r="I257" t="inlineStr">
         <is>
           <t>colofon.html</t>
@@ -23256,7 +22935,6 @@
           <t>Over deze krant</t>
         </is>
       </c>
-      <c r="G258" t="inlineStr"/>
       <c r="H258" t="inlineStr">
         <is>
           <t>Wat Het Open Vizier wil, wat het niet wil, en hoe het werkt — en wie het schrijft.</t>
@@ -23267,7 +22945,6 @@
           <t>over.html</t>
         </is>
       </c>
-      <c r="J258" t="inlineStr"/>
       <c r="K258" t="inlineStr">
         <is>
           <t>center</t>
@@ -23343,7 +23020,6 @@
           <t>alles teruglezen</t>
         </is>
       </c>
-      <c r="H259" t="inlineStr"/>
       <c r="I259" t="inlineStr">
         <is>
           <t>archief.html</t>
@@ -23429,14 +23105,11 @@
           <t>Bedankt — controleer uw inbox</t>
         </is>
       </c>
-      <c r="G260" t="inlineStr"/>
-      <c r="H260" t="inlineStr"/>
       <c r="I260" t="inlineStr">
         <is>
           <t>bedankt.html</t>
         </is>
       </c>
-      <c r="J260" t="inlineStr"/>
       <c r="K260" t="inlineStr">
         <is>
           <t>center</t>
@@ -23507,7 +23180,6 @@
           <t>Op de hoogte blijven</t>
         </is>
       </c>
-      <c r="G261" t="inlineStr"/>
       <c r="H261" t="inlineStr">
         <is>
           <t>Vraag een korte melding aan wanneer een nieuw stuk verschijnt op openvizier.org. Geen mening, geen verkoop van gegevens. Uitschrijven met één klik.</t>
@@ -23518,7 +23190,6 @@
           <t>op-de-hoogte.html</t>
         </is>
       </c>
-      <c r="J261" t="inlineStr"/>
       <c r="K261" t="inlineStr">
         <is>
           <t>center</t>
@@ -23589,14 +23260,11 @@
           <t>Structuur — Beheer · Het Open Vizier</t>
         </is>
       </c>
-      <c r="G262" t="inlineStr"/>
-      <c r="H262" t="inlineStr"/>
       <c r="I262" t="inlineStr">
         <is>
           <t>structuur.html</t>
         </is>
       </c>
-      <c r="J262" t="inlineStr"/>
       <c r="K262" t="inlineStr">
         <is>
           <t>center</t>
@@ -23667,7 +23335,6 @@
           <t>Navigatie · Het Open Vizier</t>
         </is>
       </c>
-      <c r="G263" t="inlineStr"/>
       <c r="H263" t="inlineStr">
         <is>
           <t>Visuele navigatie door Het Open Vizier — vier hoofdthemes, alle artikelen in beeld.</t>
@@ -23678,7 +23345,6 @@
           <t>navigatie.html</t>
         </is>
       </c>
-      <c r="J263" t="inlineStr"/>
       <c r="K263" t="inlineStr">
         <is>
           <t>center</t>
@@ -23749,14 +23415,11 @@
           <t>Het Open Vizier — Kies een taal</t>
         </is>
       </c>
-      <c r="G264" t="inlineStr"/>
-      <c r="H264" t="inlineStr"/>
       <c r="I264" t="inlineStr">
         <is>
           <t>talenring.html</t>
         </is>
       </c>
-      <c r="J264" t="inlineStr"/>
       <c r="K264" t="inlineStr">
         <is>
           <t>center</t>
@@ -23827,14 +23490,11 @@
           <t>Het Open Vizier — Kies een taal</t>
         </is>
       </c>
-      <c r="G265" t="inlineStr"/>
-      <c r="H265" t="inlineStr"/>
       <c r="I265" t="inlineStr">
         <is>
           <t>index-talenring.html</t>
         </is>
       </c>
-      <c r="J265" t="inlineStr"/>
       <c r="K265" t="inlineStr">
         <is>
           <t>center</t>
@@ -23905,7 +23565,6 @@
           <t>Het Open Vizier — een krant over denken zonder oogkleppen</t>
         </is>
       </c>
-      <c r="G266" t="inlineStr"/>
       <c r="H266" t="inlineStr">
         <is>
           <t>Onafhankelijke maandelijkse krant van Jacobus van Merksteijn. Politiek, democratie, onderwijs, natuurkunde en techniek — in gewone taal, open voor discussie.</t>
@@ -23916,7 +23575,6 @@
           <t>index-klassiek.html</t>
         </is>
       </c>
-      <c r="J266" t="inlineStr"/>
       <c r="K266" t="inlineStr">
         <is>
           <t>center</t>
@@ -23987,7 +23645,6 @@
           <t>Delen</t>
         </is>
       </c>
-      <c r="G267" t="inlineStr"/>
       <c r="H267" t="inlineStr">
         <is>
           <t>Hoe Het Open Vizier het beste verder gedragen kan worden — naar lezers in parlementen, universiteiten, redacties en eigen netwerken.</t>
@@ -23998,7 +23655,6 @@
           <t>delen.html</t>
         </is>
       </c>
-      <c r="J267" t="inlineStr"/>
       <c r="K267" t="inlineStr">
         <is>
           <t>center</t>
@@ -24069,7 +23725,6 @@
           <t>Verkennen</t>
         </is>
       </c>
-      <c r="G268" t="inlineStr"/>
       <c r="H268" t="inlineStr">
         <is>
           <t>Visueel verkennen van de structuur van Het Open Vizier — klik door de lagen.</t>
@@ -24080,7 +23735,6 @@
           <t>verkennen.html</t>
         </is>
       </c>
-      <c r="J268" t="inlineStr"/>
       <c r="K268" t="inlineStr">
         <is>
           <t>center</t>
@@ -24151,14 +23805,11 @@
           <t>Verkennen</t>
         </is>
       </c>
-      <c r="G269" t="inlineStr"/>
-      <c r="H269" t="inlineStr"/>
       <c r="I269" t="inlineStr">
         <is>
           <t>verkennen-embed.html</t>
         </is>
       </c>
-      <c r="J269" t="inlineStr"/>
       <c r="K269" t="inlineStr">
         <is>
           <t>center</t>
@@ -24229,7 +23880,6 @@
           <t>Tien seconden</t>
         </is>
       </c>
-      <c r="G270" t="inlineStr"/>
       <c r="H270" t="inlineStr">
         <is>
           <t>Binnen tien seconden weet een kind van vier wie er echt aanwezig is. Tussen vier en twaalf leren wij het kind dat het niet mag vertrouwen op die wetenschap. Wij noemen dat opvoeding.</t>
@@ -24240,7 +23890,6 @@
           <t>idee.html</t>
         </is>
       </c>
-      <c r="J270" t="inlineStr"/>
       <c r="K270" t="inlineStr">
         <is>
           <t>center</t>
@@ -24311,7 +23960,6 @@
           <t>Hoe u meedoet aan de discussie</t>
         </is>
       </c>
-      <c r="G271" t="inlineStr"/>
       <c r="H271" t="inlineStr">
         <is>
           <t>Hoe het discussiesysteem van Het Open Vizier werkt: registratie, spelregels, AI-moderatie en wat ermee gebeurt.</t>
@@ -24402,7 +24050,6 @@
           <t>Wat er nu al ligt</t>
         </is>
       </c>
-      <c r="G272" t="inlineStr"/>
       <c r="H272" t="inlineStr">
         <is>
           <t>Overzicht van technische projecten: SeaSkin, GuardSkin, AeroSkin, SolarSkin, TerraClean, Tyre-patenten, conische vortex-reactor.</t>
@@ -24464,6 +24111,197 @@
       <c r="AM272" t="inlineStr">
         <is>
           <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>1.4.6.9</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>1.4.6</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Waar een wil is is een weg</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Waarom een generatie jongeren ziek thuis zit, en wat de opvoeding daarmee te maken heeft.</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>Een generatie jongeren belandt met angst, vermoeidheid en depressie in de WIA. Het FD beschrijft de symptomen. Dit stuk gaat over de andere kant: opvoeding, onderwijs, contract, en het systeem dat zijn eigen productiefouten opruimt met zijn eigen consumptiecircuit.</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>wat-opkomt/waar-een-wil-is.html</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/wil/wil_01_thuis.jpg</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N273" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="R273" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S273" t="n">
+        <v>1</v>
+      </c>
+      <c r="T273" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI273" t="inlineStr">
+        <is>
+          <t>opvoeding, oergevoel, drie hersenlagen, WIA, jongeren, medicalisering, opmaakeconomie, AI-onderwijs, Kosaris</t>
+        </is>
+      </c>
+      <c r="AK273" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="AL273" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>1.3.2.11</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>1.3.2</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Waar een wil is is een weg</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Waarom een generatie jongeren ziek thuis zit, en wat de opvoeding daarmee te maken heeft.</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>Reactie op de FD-reportage over jonge werkenden in de WIA. De drie hersenlagen, wat we kinderen aandoen, onderwijs in het AI-tijdperk, en het systeem dat symptomen bestrijdt in plaats van oorzaken.</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>wat-opkomt/waar-een-wil-is.html</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/wil/wil_01_thuis.jpg</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N274" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>1.3.2</t>
+        </is>
+      </c>
+      <c r="R274" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S274" t="n">
+        <v>11</v>
+      </c>
+      <c r="T274" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI274" t="inlineStr">
+        <is>
+          <t>opvoeding, oergevoel, drie hersenlagen, WIA, jongeren, medicalisering, opmaakeconomie, AI-onderwijs, Kosaris</t>
+        </is>
+      </c>
+      <c r="AK274" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="AL274" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
         </is>
       </c>
     </row>
@@ -24478,10 +24316,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="B2:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
@@ -24715,10 +24552,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="B2:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
@@ -24985,10 +24821,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="B2:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
@@ -25748,10 +25583,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="B2:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
@@ -25759,7 +25593,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
@@ -25772,7 +25605,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
@@ -25785,7 +25617,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
@@ -25798,7 +25629,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
@@ -25811,7 +25641,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
@@ -25824,7 +25653,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
@@ -25837,7 +25665,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
@@ -25850,7 +25677,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
@@ -25863,7 +25689,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
@@ -25876,7 +25701,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wat opkomt: 'Denk eens aan de natuur' - integraal beleidsadvies
Volledige tekst (2299 woorden bron -> 3068 woorden HTML met opmaak).
Alle tien hoofdstukken plus stap 6 IP-waarschuwing intact.

Bestanden:
- nl/wat-opkomt/denk-aan-de-natuur.html (nieuw artikel, moderne ov-nav)
- assets/wat-opkomt/denk-natuur/hero_kringloop.jpg (realistische cross-section)

Plaatsing:
- nl/index.html: dgk-top blok bovenaan de dagkrant-stapel (donker-groen)
- nl/editie-klimaat/index.html: ek-kaart--breed goud direct na de intro,
  voor het centrale triptiek

Matrix-inschrijvingen (via vizier.xlsx):
- 1.4.6.10  (NL Voorpagina > Wat het niet ziet) Volgorde=1
- 1.4.5.1.1 (NL Editie Klimaat) Terug naar 1.4.5.1
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR274"/>
+  <dimension ref="A2:AR276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -24300,6 +24300,197 @@
         </is>
       </c>
       <c r="AL274" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>1.4.6.10</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>1.4.6</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Denk eens aan de natuur, met de natuur als basis</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Een integraal klimaat-, industrie- en handelsvoorstel voor de Nederlandse regering.</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>Vier bewezen sporen — tropische co-teelt, biobased plastic, cement- en houtvervanging, superieure isolatie — vormen samen een gesloten koolstofcyclus, met permanente ondergrondse plastic-opslag als fundament. De rekensom is klaar. De technologie is bewezen. Alleen de politieke wil ontbreekt.</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>wat-opkomt/denk-aan-de-natuur.html</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/denk-natuur/hero_kringloop.jpg</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N275" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="R275" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S275" t="n">
+        <v>1</v>
+      </c>
+      <c r="T275" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI275" t="inlineStr">
+        <is>
+          <t>klimaat, biomassa, Juncao, Moringa, biobased plastic, geologische opslag, CRCF, cement, hout, aerogel, isolatie, CO2, koolstofcyclus, beleidsadvies</t>
+        </is>
+      </c>
+      <c r="AK275" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="AL275" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>1.4.5.1.1</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>1.4.5.1</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Denk eens aan de natuur, met de natuur als basis</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Integraal beleidsadvies voor de Nederlandse regering.</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Vier bewezen sporen: tropische co-teelt (Juncao + Moringa), biobased plastic, cement- en houtvervanging, polymeer-aerogel isolatie. Samen een gesloten koolstofcyclus met permanente ondergrondse plastic-opslag als fundament.</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>wat-opkomt/denk-aan-de-natuur.html</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/denk-natuur/hero_kringloop.jpg</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N276" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>1.4.5.1</t>
+        </is>
+      </c>
+      <c r="R276" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S276" t="n">
+        <v>1</v>
+      </c>
+      <c r="T276" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI276" t="inlineStr">
+        <is>
+          <t>klimaat, biomassa, Juncao, Moringa, biobased plastic, geologische opslag, CRCF, cement, hout, aerogel, isolatie, CO2, koolstofcyclus, beleidsadvies</t>
+        </is>
+      </c>
+      <c r="AK276" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="AL276" t="inlineStr">
         <is>
           <t>Jacobus van Merksteijn</t>
         </is>

</xml_diff>

<commit_message>
kosaris-boek-twee: nieuw leesboek via matrix (rij 1.3.3.6 in xlsx)
Nieuwe pagina nl/leesboek-boek-twee/index.html met de volledige inhoud
van De Kosaris — Boek Twee — Diakrisis:
- Vooraf + 12 delen + 44 verhalen + Nawoord + Colofon
- Zelfde opbouw en styling als Boek Eén
- Slotformule per verhaal: 'En niemand had gelogen.'
- Omslag hergebruikt: assets/kosaris/image2.png
- Nav-blok identiek aan boek 1 (geen menu-wijziging aan andere pagina's)

Xlsx-uitbreiding (volgens MATRIX-REGELS.md §3.2):
- Knopen-tab: nieuwe rij 1.3.3.6 onder ouder 1.3.3 'Films, sprookjes, leesboek'
- Type=artikel, Taal=nl, URL=leesboek-boek-twee/index.html
- Status=live, Actief=true
- JSONs onder nl/_data/tabellen/ lokaal geregenereerd via xlsx_naar_json.py

Verkennen/, cirkelnavigatie en structuur.html pikken deze nieuwe knoop
automatisch op zonder verdere aanpassingen.
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR276"/>
+  <dimension ref="A2:AR277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -24493,6 +24493,86 @@
       <c r="AL276" t="inlineStr">
         <is>
           <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>1.3.3.6</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>1.3.3</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>De Kosaris — Boek Twee — Diakrisis</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>De Kosaris, Boek Twee — Diakrisis: het boek van het onderscheid. Vierenveertig verhalen in twaalf delen door Jacobus van Merksteijn.</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>leesboek-boek-twee/index.html</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N277" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="Q277" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R277" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="T277" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL277" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM277" t="inlineStr">
+        <is>
+          <t>nl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "kosaris-boek-twee: nieuw leesboek via matrix (rij 1.3.3.6 in xlsx)"
This reverts commit a7654f18bea43fda176e007ca49052d996433a82.
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR277"/>
+  <dimension ref="A2:AR276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -24493,86 +24493,6 @@
       <c r="AL276" t="inlineStr">
         <is>
           <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-    </row>
-    <row r="277">
-      <c r="B277" t="inlineStr">
-        <is>
-          <t>1.3.3.6</t>
-        </is>
-      </c>
-      <c r="C277" t="inlineStr">
-        <is>
-          <t>1.3.3</t>
-        </is>
-      </c>
-      <c r="D277" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-      <c r="E277" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F277" t="inlineStr">
-        <is>
-          <t>De Kosaris — Boek Twee — Diakrisis</t>
-        </is>
-      </c>
-      <c r="H277" t="inlineStr">
-        <is>
-          <t>De Kosaris, Boek Twee — Diakrisis: het boek van het onderscheid. Vierenveertig verhalen in twaalf delen door Jacobus van Merksteijn.</t>
-        </is>
-      </c>
-      <c r="I277" t="inlineStr">
-        <is>
-          <t>leesboek-boek-twee/index.html</t>
-        </is>
-      </c>
-      <c r="K277" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L277" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M277" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N277" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="Q277" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="R277" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="T277" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL277" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-      <c r="AM277" t="inlineStr">
-        <is>
-          <t>nl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(nl): De Kosaris - Boek Twee - Diakrisis toegevoegd aan matrix (code 1.3.3.6)
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR276"/>
+  <dimension ref="B2:AR277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -24493,6 +24493,86 @@
       <c r="AL276" t="inlineStr">
         <is>
           <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>1.3.3.6</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>1.3.3</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>De Kosaris — Boek Twee — Diakrisis</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>De Kosaris, Boek Twee — Diakrisis: het boek van het onderscheid. Vierenveertig verhalen in twaalf delen door Jacobus van Merksteijn.</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>leesboek-boek-twee/index.html</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N277" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="Q277" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R277" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="T277" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL277" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM277" t="inlineStr">
+        <is>
+          <t>nl</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "Europa Slavenland" — artikel op verzoek van auteur teruggetrokken
Het gepubliceerde artikel had een linkse framing (klassenverhaal
arm-vs-rijk, vermogensbelasting als hoofdoplossing) die de auteur
achteraf niet passend vond bij het bredere Open Vizier-kader. Wordt
volledig herschreven op basis van de correcte tegenstelling
werkend-vs-niet-werkend-maar-wel-kunnend, en rendabele-vs-rendementsloze
overheidsuitgaven.

Verwijdert:
- nl/wat-opkomt/europa-slavenland.html
- assets/wat-opkomt/H_europa_slavenland.jpg
- nl/index.html: dagkrantbanner naar dit artikel

Herstelt:
- nl/_data/vizier.xlsx naar pre-publicatie versie
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -20,9 +20,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -61,13 +60,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -433,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR278"/>
+  <dimension ref="B2:AR277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -24573,112 +24571,6 @@
         </is>
       </c>
       <c r="AM277" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-    </row>
-    <row r="278">
-      <c r="B278" t="inlineStr">
-        <is>
-          <t>1.1.1.1</t>
-        </is>
-      </c>
-      <c r="C278" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
-      <c r="D278" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-      <c r="E278" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F278" t="inlineStr">
-        <is>
-          <t>Europa Slavenland</t>
-        </is>
-      </c>
-      <c r="G278" t="inlineStr">
-        <is>
-          <t>Zeven signalen wijzen op één soevereiniteitscrisis</t>
-        </is>
-      </c>
-      <c r="H278" t="inlineStr">
-        <is>
-          <t>Zeven signalen in één week wijzen op hetzelfde: onze energie komt uit Arabië, onze materialen uit China, onze tech uit Amerika. Als wij niet ingrijpen worden wij binnen tien jaar cliënt van drie machtsblokken tegelijk. Wij hebben alles wat wij nodig hebben om dat te voorkomen. Behalve tijd en politieke bereidheid.</t>
-        </is>
-      </c>
-      <c r="I278" t="inlineStr">
-        <is>
-          <t>wat-opkomt/europa-slavenland.html</t>
-        </is>
-      </c>
-      <c r="J278" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_europa_slavenland.jpg</t>
-        </is>
-      </c>
-      <c r="K278" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L278" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M278" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N278" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="P278" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="Q278" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="R278" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="S278" t="n">
-        <v>1</v>
-      </c>
-      <c r="T278" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI278" t="inlineStr">
-        <is>
-          <t>klimaat, soevereiniteit, biomassa, biochar, EU-CDR, doom loop, belasting, vermogen, NEPK, Carbon Alert, Juncao, Amazon, datacenters, tech-fossiel</t>
-        </is>
-      </c>
-      <c r="AK278" s="3" t="n">
-        <v>46244</v>
-      </c>
-      <c r="AL278" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-      <c r="AM278" t="inlineStr">
         <is>
           <t>nl</t>
         </is>

</xml_diff>

<commit_message>
De gedachte in de kluis — nieuw artikel NL/EN/DE
Wat opkomt · Filosofie · 11 augustus 2026

Ondertitel: 'Europese innovatie moet zich wel terugtrekken, ter verdediging tegen om te overleven'.

- Nieuwe artikelen NL/EN/DE onder wat-opkomt / what-surfaces / was-aufkommt
- Hero-illustratie: fotorealistische klassieke schilderstijl (kluisdeur in rotsuitloper onder oude eik, bewaarder met sleutel bij dageraad)
- Matrix (vizier.xlsx): 2 NL-rijen — code 1.7.19 onder Belasting/wat-opkomt, code 1.3.1.7 als kruisverwijzing onder Filosofie (terug_naar 1.3.1)
- Dagkrantbanner (.dgk-top) op nl/en/de index — geplaatst op live-versie zodat bestaande banners (Europa Slavenland e.a.) behouden blijven
- Eerste wo-item op wat-opkomt/index in de drie talen
- Hoofdmenu (.ov-nav) NIET gewijzigd — rollback met één git revert mogelijk
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR278"/>
+  <dimension ref="A2:AR280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -24679,6 +24679,227 @@
         </is>
       </c>
       <c r="AM278" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>1.7.19</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>De gedachte in de kluis</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Europese innovatie moet zich wel terugtrekken, ter verdediging tegen om te overleven</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Een innovatieve gedachte heeft een drager, een omgeving, middelen en tijd nodig. Europa levert die vier niet meer. Wie iets waardevols wil bewaren, bouwt buiten Europa een kluis — geen vluchtruimte, maar een werkende installatie waaruit later een nieuwe generatie kan putten. Waarom dat geen vlucht is, en waarom de overheid het als vlucht ziet.</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>wat-opkomt/gedachte-in-de-kluis.html</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/H_gedachte-in-de-kluis.jpg</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N279" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P279" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q279" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R279" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S279" t="n">
+        <v>19</v>
+      </c>
+      <c r="T279" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI279" t="inlineStr">
+        <is>
+          <t>filosofie, wat-opkomt, europese-systeemcrisis, kluis, bewaring, innovatie, jurisdictie, symptoombestrijding</t>
+        </is>
+      </c>
+      <c r="AK279" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AL279" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM279" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>1.3.1.7</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>1.3.1</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>De gedachte in de kluis</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Europese innovatie moet zich wel terugtrekken, ter verdediging tegen om te overleven</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>Een innovatieve gedachte heeft een drager, een omgeving, middelen en tijd nodig. Europa levert die vier niet meer. Wie iets waardevols wil bewaren, bouwt buiten Europa een kluis — geen vluchtruimte, maar een werkende installatie waaruit later een nieuwe generatie kan putten. Waarom dat geen vlucht is, en waarom de overheid het als vlucht ziet.</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>wat-opkomt/gedachte-in-de-kluis.html</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/H_gedachte-in-de-kluis.jpg</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N280" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>1.3.1</t>
+        </is>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R280" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S280" t="n">
+        <v>7</v>
+      </c>
+      <c r="T280" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI280" t="inlineStr">
+        <is>
+          <t>filosofie, wat-opkomt, europese-systeemcrisis, kluis, bewaring, innovatie, jurisdictie, symptoombestrijding</t>
+        </is>
+      </c>
+      <c r="AK280" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AL280" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM280" t="inlineStr">
         <is>
           <t>nl</t>
         </is>

</xml_diff>

<commit_message>
Kosaris Boek 3 Deel 1/2/3 + Boek Twee-film - 7 rijen toegevoegd in Knopen
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR280"/>
+  <dimension ref="A2:AR287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -24900,6 +24900,765 @@
         </is>
       </c>
       <c r="AM280" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>1.3.3.7</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>1.3.3</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>De Kosaris — Boek Twee — De Film</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Filmisch essay in twaalf hoofdstukken</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>De filmversie van Diakrisis. Twaalf hoofdstukken, vierenveertig verhalen, elfeneenhalve minuut Nederlandse voice-over.</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-twee-film.html</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>../assets/kosaris/boek2-film-poster.png</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N281" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P281" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q281" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R281" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="T281" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI281" t="inlineStr">
+        <is>
+          <t>Kosaris,film,Diakrisis</t>
+        </is>
+      </c>
+      <c r="AK281" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="AL281" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM281" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>1.3.3.8</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>1.3.3</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>De Kosaris — Boek Drie — De Opvoeding — Deel 1</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>De grond</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Eerste film naar Boek Drie. Van de veertien pagina's van Anthea, via de zeven dagen en zeven maanden, tot het staan van het kind en het eerste terugkijken.</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-deel-1-film.html</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>../assets/kosaris/boek3-deel1.mp4</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N282" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P282" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q282" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="T282" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI282" t="inlineStr">
+        <is>
+          <t>Kosaris,film,Opvoeding,Anthea</t>
+        </is>
+      </c>
+      <c r="AK282" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AL282" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM282" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>1.3.3.9</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>1.3.3</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>De Kosaris — Boek Drie — De Opvoeding — Deel 2</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>De vier zuilen meegemaakt</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Tweede film naar Boek Drie. Wat er in de zeven jaar in gaat, niet als les maar als geleefde vanzelfsprekendheid. Vier dingen die een kind meemaakt.</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-deel-2-film.html</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>../assets/kosaris/boek3-deel2.mp4</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N283" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P283" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q283" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R283" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="T283" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI283" t="inlineStr">
+        <is>
+          <t>Kosaris,film,Opvoeding,Anthea</t>
+        </is>
+      </c>
+      <c r="AK283" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AL283" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM283" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>1.3.3.10</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>1.3.3</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>De Kosaris — Boek Drie — De Opvoeding — Deel 3</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>De tweede lijn</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Derde film naar Boek Drie. De laatste drie richtingen, wat niet op het rooster staat, veertien en eenentwintig, en dan een lange stilte tot zevenenzeventig.</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-deel-3-film.html</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>../assets/kosaris/boek3-deel3.mp4</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N284" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R284" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="T284" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI284" t="inlineStr">
+        <is>
+          <t>Kosaris,film,Opvoeding,Anthea</t>
+        </is>
+      </c>
+      <c r="AK284" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AL284" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM284" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>1.1.1.18</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>De Kosaris — Boek Drie — De Opvoeding — Deel 1</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>De grond</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Eerste film naar Boek Drie. Van de veertien pagina's van Anthea tot het eerste terugkijken.</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-deel-1-film.html</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>../assets/kosaris/boek3-deel1.mp4</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N285" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>1.3.3</t>
+        </is>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q285" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R285" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S285" t="n">
+        <v>18</v>
+      </c>
+      <c r="T285" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI285" t="inlineStr">
+        <is>
+          <t>Kosaris,film,Opvoeding,Anthea</t>
+        </is>
+      </c>
+      <c r="AK285" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AL285" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM285" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>1.1.1.19</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>De Kosaris — Boek Drie — De Opvoeding — Deel 2</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>De vier zuilen meegemaakt</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Tweede film naar Boek Drie. Wat er in de zeven jaar in gaat.</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-deel-2-film.html</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>../assets/kosaris/boek3-deel2.mp4</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N286" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>1.3.3</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R286" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S286" t="n">
+        <v>19</v>
+      </c>
+      <c r="T286" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI286" t="inlineStr">
+        <is>
+          <t>Kosaris,film,Opvoeding,Anthea</t>
+        </is>
+      </c>
+      <c r="AK286" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AL286" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM286" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>1.1.1.20</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>De Kosaris — Boek Drie — De Opvoeding — Deel 3</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>De tweede lijn</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Derde film naar Boek Drie. De laatste drie richtingen en de lange stilte tot zevenenzeventig.</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-deel-3-film.html</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>../assets/kosaris/boek3-deel3.mp4</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N287" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>1.3.3</t>
+        </is>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R287" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S287" t="n">
+        <v>20</v>
+      </c>
+      <c r="T287" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI287" t="inlineStr">
+        <is>
+          <t>Kosaris,film,Opvoeding,Anthea</t>
+        </is>
+      </c>
+      <c r="AK287" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AL287" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM287" t="inlineStr">
         <is>
           <t>nl</t>
         </is>

</xml_diff>

<commit_message>
Fix hero-paden volgens §2.3/§3.2: H_<slug>.jpg in assets/wat-opkomt/
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -24948,7 +24948,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>../assets/kosaris/boek2-film-poster.png</t>
+          <t>../assets/wat-opkomt/H_de-kosaris-boek-twee-film.jpg</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -25053,7 +25053,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>../assets/kosaris/boek3-deel1.mp4</t>
+          <t>../assets/wat-opkomt/H_de-kosaris-boek-drie-deel-1-film.jpg</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -25158,7 +25158,7 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>../assets/kosaris/boek3-deel2.mp4</t>
+          <t>../assets/wat-opkomt/H_de-kosaris-boek-drie-deel-2-film.jpg</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -25263,7 +25263,7 @@
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>../assets/kosaris/boek3-deel3.mp4</t>
+          <t>../assets/wat-opkomt/H_de-kosaris-boek-drie-deel-3-film.jpg</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -25368,7 +25368,7 @@
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>../assets/kosaris/boek3-deel1.mp4</t>
+          <t>../assets/wat-opkomt/H_de-kosaris-boek-drie-deel-1-film.jpg</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -25481,7 +25481,7 @@
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>../assets/kosaris/boek3-deel2.mp4</t>
+          <t>../assets/wat-opkomt/H_de-kosaris-boek-drie-deel-2-film.jpg</t>
         </is>
       </c>
       <c r="K286" t="inlineStr">
@@ -25594,7 +25594,7 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>../assets/kosaris/boek3-deel3.mp4</t>
+          <t>../assets/wat-opkomt/H_de-kosaris-boek-drie-deel-3-film.jpg</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">

</xml_diff>

<commit_message>
feat(nl): De gouden kooi - publicatie volgens matrix-regels §3.1-3.7 (hero 896x1200, artikel, xlsx 2 knopen, homepage banner)
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR287"/>
+  <dimension ref="A2:AR289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -25661,6 +25661,237 @@
       <c r="AM287" t="inlineStr">
         <is>
           <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>1.7.20</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>De gouden kooi</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Nederlanders opgesloten in een kooi van 74 tot 90 procent belastingdruk, terwijl buitenlandse eigenaren er onbelast doorheen lopen</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Nederland is voor zijn eigen werkende burgers een gouden kooi. Wie hier woont, werkt en verdient, betaalt tussen de 74 en 90 procent van zijn werkelijke inkomen. Wie hier alleen eigenaar is loopt onbelast door de tralies. De statistiek verhult dit via de BBP-BNP-truc. Een oproep tot herkadering.</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-gouden-kooi.html</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/H_de-gouden-kooi.jpg</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N288" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R288" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S288" t="n">
+        <v>19</v>
+      </c>
+      <c r="T288" t="n">
+        <v>20</v>
+      </c>
+      <c r="AI288" t="inlineStr">
+        <is>
+          <t>filosofie, wat-opkomt, europese-systeemcrisis, kluis, bewaring, innovatie, jurisdictie, symptoombestrijding</t>
+        </is>
+      </c>
+      <c r="AK288" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AL288" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM288" t="inlineStr">
+        <is>
+          <t>wat-opkomt, belasting, gouden-kooi, bnp, bbp, nederland, buitenlandse-eigenaar, belastingdruk, nova-democratia</t>
+        </is>
+      </c>
+      <c r="AO288" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>1.3.1.8</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>1.3.1</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>De gouden kooi</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Nederlanders opgesloten in een kooi van 74 tot 90 procent belastingdruk, terwijl buitenlandse eigenaren er onbelast doorheen lopen</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Nederland is voor zijn eigen werkende burgers een gouden kooi. Wie hier woont, werkt en verdient, betaalt tussen de 74 en 90 procent van zijn werkelijke inkomen. Wie hier alleen eigenaar is loopt onbelast door de tralies. De statistiek verhult dit via de BBP-BNP-truc. Een oproep tot herkadering.</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-gouden-kooi.html</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/H_de-gouden-kooi.jpg</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N289" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>1.3.1</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R289" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S289" t="n">
+        <v>7</v>
+      </c>
+      <c r="T289" t="n">
+        <v>8</v>
+      </c>
+      <c r="AI289" t="inlineStr">
+        <is>
+          <t>filosofie, wat-opkomt, europese-systeemcrisis, kluis, bewaring, innovatie, jurisdictie, symptoombestrijding</t>
+        </is>
+      </c>
+      <c r="AK289" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="AL289" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM289" t="inlineStr">
+        <is>
+          <t>wat-opkomt, belasting, gouden-kooi, bnp, bbp, nederland, buitenlandse-eigenaar, belastingdruk, nova-democratia</t>
+        </is>
+      </c>
+      <c r="AO289" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vizier.xlsx: Der goldene Käfig — Duitse rij 2.1.1.63 onder Neueste Artikel
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR289"/>
+  <dimension ref="A2:AR290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -25890,6 +25890,120 @@
         </is>
       </c>
       <c r="AO289" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>2.1.1.63</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>2.1.1</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Der goldene Käfig</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Warnstufe Rot für arbeitende Deutsche — bis 2030 Warnstufe Schwarz, während ausländische Eigentümer unbelastet hindurchgehen</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Deutschland ist für seine eigenen arbeitenden Bürger ein goldener Käfig. Wer hier wohnt, arbeitet und verdient, zahlt zwischen 74 und 90 Prozent seines tatsächlichen Einkommens. Wer hier nur Eigentümer ist, geht unbelastet durch die Gitterstäbe. Die Statistik verhüllt dies über die BIP-BNP-Trick. Ein Aufruf zur Neurahmung.</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>was-aufkommt/der-goldene-kaefig.html</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/H_der-goldene-kaefig.jpg</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="O290" t="inlineStr"/>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R290" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S290" t="n">
+        <v>63</v>
+      </c>
+      <c r="T290" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI290" t="inlineStr">
+        <is>
+          <t>steuern, staatsquote, bip, bnp, deutschland, ausländische-eigentümer, verteidigung</t>
+        </is>
+      </c>
+      <c r="AK290" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="AL290" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM290" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="AO290" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>

</xml_diff>

<commit_message>
vizier.xlsx: The Golden Cage — EN row 3.1.1.63 under Latest Articles
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR290"/>
+  <dimension ref="A2:AR291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -25961,7 +25961,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O290" t="inlineStr"/>
       <c r="P290" t="inlineStr">
         <is>
           <t>auto</t>
@@ -26004,6 +26003,120 @@
         </is>
       </c>
       <c r="AO290" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>3.1.1.63</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>3.1.1</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>The Golden Cage</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Warning Level Red for working Britons — Warning Level Black by 2030, while foreign owners pass unhindered through the bars</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>The UK is a golden cage for its own working citizens. Whoever lives, works and earns here pays between 74 and 90 percent of their real income. Whoever is only an owner walks unhindered through the bars. Statistics conceal this via the GDP-GNP trick. A call for reframing.</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>what-surfaces/the-golden-cage.html</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>../assets/wat-opkomt/H_the-golden-cage.jpg</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N291" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="O291" t="inlineStr"/>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R291" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S291" t="n">
+        <v>63</v>
+      </c>
+      <c r="T291" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI291" t="inlineStr">
+        <is>
+          <t>taxation, public spending, gdp, gnp, uk, foreign-owners, defence</t>
+        </is>
+      </c>
+      <c r="AK291" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="AL291" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM291" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="AO291" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>

</xml_diff>

<commit_message>
Publicatie 2026-08-14: twee artikelen onder Politiek (1.2.6 Economie & compositie)
- Nieuw onderwerp 1.2.6 in matrix
- Artikel 1.2.6.1 'De groei die de overheid zelf uitgeeft'
- Artikel 1.2.6.2 'De prikkel die we bij een groep uitschakelen'
- Kruisverwijzingen 1.1.1.21 en 1.1.1.22 onder Laatste artikelen
- Twee dgk-top banners bovenaan nl/index.html (bestaande banners bewaard)
- Hero-assets 896x1200 volgens conventie
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -20,9 +20,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -61,13 +60,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -433,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR291"/>
+  <dimension ref="A2:AR281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -24501,12 +24499,12 @@
     <row r="277">
       <c r="B277" t="inlineStr">
         <is>
-          <t>1.3.3.6</t>
+          <t>1.2.6</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>1.3.3</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -24516,22 +24514,22 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>artikel</t>
+          <t>onderwerp</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Twee — Diakrisis</t>
+          <t>Economie &amp; compositie</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>wat de koppen wegdrukken</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>De Kosaris, Boek Twee — Diakrisis: het boek van het onderscheid. Vierenveertig verhalen in twaalf delen door Jacobus van Merksteijn.</t>
-        </is>
-      </c>
-      <c r="I277" t="inlineStr">
-        <is>
-          <t>leesboek-boek-twee/index.html</t>
+          <t>De artikelen onder Economie &amp; compositie.</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -24563,6 +24561,9 @@
         <is>
           <t>live</t>
         </is>
+      </c>
+      <c r="S277" t="n">
+        <v>6</v>
       </c>
       <c r="T277" t="b">
         <v>1</v>
@@ -24581,12 +24582,12 @@
     <row r="278">
       <c r="B278" t="inlineStr">
         <is>
-          <t>1.1.1.1</t>
+          <t>1.2.6.1</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>1.1.1</t>
+          <t>1.2.6</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -24601,27 +24602,27 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>Europa Slavenland</t>
+          <t>De groei die de overheid zelf uitgeeft</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>Zeven signalen wijzen op één soevereiniteitscrisis</t>
+          <t>Kwartaalcijfer 0,4% en de kop die de compositie wegliet</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>Zeven signalen in één week wijzen op hetzelfde: onze energie komt uit Arabië, onze materialen uit China, onze tech uit Amerika. Wij eten onze basis op via NEPK-daling. De rekening gaat niet naar werk of vermogen — naar onrendabele overheid.</t>
+          <t>CBS meldt 0,4% BBP-groei in Q2 2026 en de pers kopt dat de "rampscenario’s" uitblijven. Wat de koppen wegdrukken: overheidsconsumptie groeide 2,5% j-o-j — twee keer zo hard als huishoudconsumptie, zes keer zo hard als investeringen. De productieve kern (bouw, energie, delfstoffen, financiën, landbouw) krimpt. Tekort boven EU-norm.</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>wat-opkomt/europa-slavenland.html</t>
+          <t>wat-opkomt/de-groei-die-de-overheid-zelf-uitgeeft.html</t>
         </is>
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>../assets/wat-opkomt/H_europa_slavenland.jpg</t>
+          <t>../assets/wat-opkomt/H_groei_overheid_zelf.jpg</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
@@ -24644,11 +24645,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="P278" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
       <c r="Q278" t="inlineStr">
         <is>
           <t>self</t>
@@ -24667,11 +24663,13 @@
       </c>
       <c r="AI278" t="inlineStr">
         <is>
-          <t>klimaat, soevereiniteit, NEPK, biomassa, biochar, EU-CDR, doom loop, rendabele overheid, politie, zwartgeldbestrijding, Carbon Alert, Juncao, Amazon, datacenters, tech-fossiel</t>
-        </is>
-      </c>
-      <c r="AK278" s="3" t="n">
-        <v>46244</v>
+          <t>BBP, opmaakeconomie, overheidsconsumptie, CBS, pers, framing, begrotingstekort, EU-norm</t>
+        </is>
+      </c>
+      <c r="AK278" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
       </c>
       <c r="AL278" t="inlineStr">
         <is>
@@ -24687,12 +24685,12 @@
     <row r="279">
       <c r="B279" t="inlineStr">
         <is>
-          <t>1.7.19</t>
+          <t>1.2.6.2</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.2.6</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -24707,27 +24705,27 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>De gedachte in de kluis</t>
+          <t>De prikkel die we bij één groep uitschakelen</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>Europese innovatie moet zich wel terugtrekken, ter verdediging tegen om te overleven</t>
+          <t>Waarom bedrijven vertrekken, migranten komen, en onze eigen onderklasse blijft staan</t>
         </is>
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>Een innovatieve gedachte heeft een drager, een omgeving, middelen en tijd nodig. Europa levert die vier niet meer. Wie iets waardevols wil bewaren, bouwt buiten Europa een kluis — geen vluchtruimte, maar een werkende installatie waaruit later een nieuwe generatie kan putten. Waarom dat geen vlucht is, en waarom de overheid het als vlucht ziet.</t>
+          <t>Dezelfde drijfveer — ga naar waar arbeid of kapitaal iets kan verdienen — beweegt bedrijven het land uit en migranten Europa in. Bij de eigen onderklasse is die prikkel stelselmatig uitgeschakeld. Netto verhuist het aanpassingsvermogen naar buiten en het passieve deel naar binnen.</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>wat-opkomt/gedachte-in-de-kluis.html</t>
+          <t>wat-opkomt/de-prikkel-die-we-bij-een-groep-uitschakelen.html</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>../assets/wat-opkomt/H_gedachte-in-de-kluis.jpg</t>
+          <t>../assets/wat-opkomt/H_prikkel_uitgeschakeld.jpg</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
@@ -24750,11 +24748,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="P279" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
       <c r="Q279" t="inlineStr">
         <is>
           <t>self</t>
@@ -24766,19 +24759,19 @@
         </is>
       </c>
       <c r="S279" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="T279" t="b">
         <v>1</v>
       </c>
       <c r="AI279" t="inlineStr">
         <is>
-          <t>filosofie, wat-opkomt, europese-systeemcrisis, kluis, bewaring, innovatie, jurisdictie, symptoombestrijding</t>
+          <t>prikkel, migratie, uitkeringen, WIA, participatiewet, opmaakeconomie, aanpassingsvermogen</t>
         </is>
       </c>
       <c r="AK279" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AL279" t="inlineStr">
@@ -24795,12 +24788,12 @@
     <row r="280">
       <c r="B280" t="inlineStr">
         <is>
-          <t>1.3.1.7</t>
+          <t>1.1.1.21</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>1.3.1</t>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -24815,27 +24808,27 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>De gedachte in de kluis</t>
+          <t>De groei die de overheid zelf uitgeeft</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>Europese innovatie moet zich wel terugtrekken, ter verdediging tegen om te overleven</t>
+          <t>Kwartaalcijfer 0,4% en de kop die de compositie wegliet</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>Een innovatieve gedachte heeft een drager, een omgeving, middelen en tijd nodig. Europa levert die vier niet meer. Wie iets waardevols wil bewaren, bouwt buiten Europa een kluis — geen vluchtruimte, maar een werkende installatie waaruit later een nieuwe generatie kan putten. Waarom dat geen vlucht is, en waarom de overheid het als vlucht ziet.</t>
+          <t>CBS meldt 0,4% BBP-groei in Q2 2026 en de pers kopt dat de "rampscenario’s" uitblijven. Wat de koppen wegdrukken: overheidsconsumptie groeide 2,5% j-o-j.</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>wat-opkomt/gedachte-in-de-kluis.html</t>
+          <t>wat-opkomt/de-groei-die-de-overheid-zelf-uitgeeft.html</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>../assets/wat-opkomt/H_gedachte-in-de-kluis.jpg</t>
+          <t>../assets/wat-opkomt/H_groei_overheid_zelf.jpg</t>
         </is>
       </c>
       <c r="K280" t="inlineStr">
@@ -24860,12 +24853,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>1.3.1</t>
-        </is>
-      </c>
-      <c r="P280" t="inlineStr">
-        <is>
-          <t>auto</t>
+          <t>1.2.6</t>
         </is>
       </c>
       <c r="Q280" t="inlineStr">
@@ -24879,19 +24867,19 @@
         </is>
       </c>
       <c r="S280" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="T280" t="b">
         <v>1</v>
       </c>
       <c r="AI280" t="inlineStr">
         <is>
-          <t>filosofie, wat-opkomt, europese-systeemcrisis, kluis, bewaring, innovatie, jurisdictie, symptoombestrijding</t>
+          <t>BBP, opmaakeconomie, overheidsconsumptie, CBS, pers, framing</t>
         </is>
       </c>
       <c r="AK280" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AL280" t="inlineStr">
@@ -24908,12 +24896,12 @@
     <row r="281">
       <c r="B281" t="inlineStr">
         <is>
-          <t>1.3.3.7</t>
+          <t>1.1.1.22</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>1.3.3</t>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -24928,27 +24916,27 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Twee — De Film</t>
+          <t>De prikkel die we bij één groep uitschakelen</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>Filmisch essay in twaalf hoofdstukken</t>
+          <t>Waarom bedrijven vertrekken, migranten komen, en onze eigen onderklasse blijft staan</t>
         </is>
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>De filmversie van Diakrisis. Twaalf hoofdstukken, vierenveertig verhalen, elfeneenhalve minuut Nederlandse voice-over.</t>
+          <t>Dezelfde drijfveer beweegt bedrijven het land uit en migranten Europa in. Bij de eigen onderklasse is die prikkel uitgeschakeld.</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
         <is>
-          <t>wat-opkomt/de-kosaris-boek-twee-film.html</t>
+          <t>wat-opkomt/de-prikkel-die-we-bij-een-groep-uitschakelen.html</t>
         </is>
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>../assets/wat-opkomt/H_de-kosaris-boek-twee-film.jpg</t>
+          <t>../assets/wat-opkomt/H_prikkel_uitgeschakeld.jpg</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -24971,9 +24959,9 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="P281" t="inlineStr">
-        <is>
-          <t>auto</t>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>1.2.6</t>
         </is>
       </c>
       <c r="Q281" t="inlineStr">
@@ -24986,17 +24974,20 @@
           <t>live</t>
         </is>
       </c>
+      <c r="S281" t="n">
+        <v>22</v>
+      </c>
       <c r="T281" t="b">
         <v>1</v>
       </c>
       <c r="AI281" t="inlineStr">
         <is>
-          <t>Kosaris,film,Diakrisis</t>
+          <t>prikkel, migratie, uitkeringen, opmaakeconomie, aanpassingsvermogen</t>
         </is>
       </c>
       <c r="AK281" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="AL281" t="inlineStr">
@@ -25007,1118 +24998,6 @@
       <c r="AM281" t="inlineStr">
         <is>
           <t>nl</t>
-        </is>
-      </c>
-    </row>
-    <row r="282">
-      <c r="B282" t="inlineStr">
-        <is>
-          <t>1.3.3.8</t>
-        </is>
-      </c>
-      <c r="C282" t="inlineStr">
-        <is>
-          <t>1.3.3</t>
-        </is>
-      </c>
-      <c r="D282" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-      <c r="E282" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F282" t="inlineStr">
-        <is>
-          <t>De Kosaris — Boek Drie — De Opvoeding — Deel 1</t>
-        </is>
-      </c>
-      <c r="G282" t="inlineStr">
-        <is>
-          <t>De grond</t>
-        </is>
-      </c>
-      <c r="H282" t="inlineStr">
-        <is>
-          <t>Eerste film naar Boek Drie. Van de veertien pagina's van Anthea, via de zeven dagen en zeven maanden, tot het staan van het kind en het eerste terugkijken.</t>
-        </is>
-      </c>
-      <c r="I282" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-kosaris-boek-drie-deel-1-film.html</t>
-        </is>
-      </c>
-      <c r="J282" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_de-kosaris-boek-drie-deel-1-film.jpg</t>
-        </is>
-      </c>
-      <c r="K282" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L282" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M282" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N282" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="P282" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="Q282" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="R282" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="T282" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI282" t="inlineStr">
-        <is>
-          <t>Kosaris,film,Opvoeding,Anthea</t>
-        </is>
-      </c>
-      <c r="AK282" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="AL282" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-      <c r="AM282" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-    </row>
-    <row r="283">
-      <c r="B283" t="inlineStr">
-        <is>
-          <t>1.3.3.9</t>
-        </is>
-      </c>
-      <c r="C283" t="inlineStr">
-        <is>
-          <t>1.3.3</t>
-        </is>
-      </c>
-      <c r="D283" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-      <c r="E283" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F283" t="inlineStr">
-        <is>
-          <t>De Kosaris — Boek Drie — De Opvoeding — Deel 2</t>
-        </is>
-      </c>
-      <c r="G283" t="inlineStr">
-        <is>
-          <t>De vier zuilen meegemaakt</t>
-        </is>
-      </c>
-      <c r="H283" t="inlineStr">
-        <is>
-          <t>Tweede film naar Boek Drie. Wat er in de zeven jaar in gaat, niet als les maar als geleefde vanzelfsprekendheid. Vier dingen die een kind meemaakt.</t>
-        </is>
-      </c>
-      <c r="I283" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-kosaris-boek-drie-deel-2-film.html</t>
-        </is>
-      </c>
-      <c r="J283" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_de-kosaris-boek-drie-deel-2-film.jpg</t>
-        </is>
-      </c>
-      <c r="K283" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L283" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M283" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N283" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="P283" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="Q283" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="R283" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="T283" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI283" t="inlineStr">
-        <is>
-          <t>Kosaris,film,Opvoeding,Anthea</t>
-        </is>
-      </c>
-      <c r="AK283" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="AL283" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-      <c r="AM283" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-    </row>
-    <row r="284">
-      <c r="B284" t="inlineStr">
-        <is>
-          <t>1.3.3.10</t>
-        </is>
-      </c>
-      <c r="C284" t="inlineStr">
-        <is>
-          <t>1.3.3</t>
-        </is>
-      </c>
-      <c r="D284" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-      <c r="E284" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F284" t="inlineStr">
-        <is>
-          <t>De Kosaris — Boek Drie — De Opvoeding — Deel 3</t>
-        </is>
-      </c>
-      <c r="G284" t="inlineStr">
-        <is>
-          <t>De tweede lijn</t>
-        </is>
-      </c>
-      <c r="H284" t="inlineStr">
-        <is>
-          <t>Derde film naar Boek Drie. De laatste drie richtingen, wat niet op het rooster staat, veertien en eenentwintig, en dan een lange stilte tot zevenenzeventig.</t>
-        </is>
-      </c>
-      <c r="I284" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-kosaris-boek-drie-deel-3-film.html</t>
-        </is>
-      </c>
-      <c r="J284" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_de-kosaris-boek-drie-deel-3-film.jpg</t>
-        </is>
-      </c>
-      <c r="K284" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L284" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M284" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N284" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="P284" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="Q284" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="R284" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="T284" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI284" t="inlineStr">
-        <is>
-          <t>Kosaris,film,Opvoeding,Anthea</t>
-        </is>
-      </c>
-      <c r="AK284" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="AL284" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-      <c r="AM284" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-    </row>
-    <row r="285">
-      <c r="B285" t="inlineStr">
-        <is>
-          <t>1.1.1.18</t>
-        </is>
-      </c>
-      <c r="C285" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
-      <c r="D285" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-      <c r="E285" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F285" t="inlineStr">
-        <is>
-          <t>De Kosaris — Boek Drie — De Opvoeding — Deel 1</t>
-        </is>
-      </c>
-      <c r="G285" t="inlineStr">
-        <is>
-          <t>De grond</t>
-        </is>
-      </c>
-      <c r="H285" t="inlineStr">
-        <is>
-          <t>Eerste film naar Boek Drie. Van de veertien pagina's van Anthea tot het eerste terugkijken.</t>
-        </is>
-      </c>
-      <c r="I285" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-kosaris-boek-drie-deel-1-film.html</t>
-        </is>
-      </c>
-      <c r="J285" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_de-kosaris-boek-drie-deel-1-film.jpg</t>
-        </is>
-      </c>
-      <c r="K285" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L285" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M285" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N285" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="O285" t="inlineStr">
-        <is>
-          <t>1.3.3</t>
-        </is>
-      </c>
-      <c r="P285" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="Q285" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="R285" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="S285" t="n">
-        <v>18</v>
-      </c>
-      <c r="T285" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI285" t="inlineStr">
-        <is>
-          <t>Kosaris,film,Opvoeding,Anthea</t>
-        </is>
-      </c>
-      <c r="AK285" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="AL285" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-      <c r="AM285" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-    </row>
-    <row r="286">
-      <c r="B286" t="inlineStr">
-        <is>
-          <t>1.1.1.19</t>
-        </is>
-      </c>
-      <c r="C286" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
-      <c r="D286" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-      <c r="E286" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F286" t="inlineStr">
-        <is>
-          <t>De Kosaris — Boek Drie — De Opvoeding — Deel 2</t>
-        </is>
-      </c>
-      <c r="G286" t="inlineStr">
-        <is>
-          <t>De vier zuilen meegemaakt</t>
-        </is>
-      </c>
-      <c r="H286" t="inlineStr">
-        <is>
-          <t>Tweede film naar Boek Drie. Wat er in de zeven jaar in gaat.</t>
-        </is>
-      </c>
-      <c r="I286" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-kosaris-boek-drie-deel-2-film.html</t>
-        </is>
-      </c>
-      <c r="J286" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_de-kosaris-boek-drie-deel-2-film.jpg</t>
-        </is>
-      </c>
-      <c r="K286" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L286" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M286" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N286" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="O286" t="inlineStr">
-        <is>
-          <t>1.3.3</t>
-        </is>
-      </c>
-      <c r="P286" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="Q286" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="R286" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="S286" t="n">
-        <v>19</v>
-      </c>
-      <c r="T286" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI286" t="inlineStr">
-        <is>
-          <t>Kosaris,film,Opvoeding,Anthea</t>
-        </is>
-      </c>
-      <c r="AK286" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="AL286" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-      <c r="AM286" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-    </row>
-    <row r="287">
-      <c r="B287" t="inlineStr">
-        <is>
-          <t>1.1.1.20</t>
-        </is>
-      </c>
-      <c r="C287" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
-      <c r="D287" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-      <c r="E287" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F287" t="inlineStr">
-        <is>
-          <t>De Kosaris — Boek Drie — De Opvoeding — Deel 3</t>
-        </is>
-      </c>
-      <c r="G287" t="inlineStr">
-        <is>
-          <t>De tweede lijn</t>
-        </is>
-      </c>
-      <c r="H287" t="inlineStr">
-        <is>
-          <t>Derde film naar Boek Drie. De laatste drie richtingen en de lange stilte tot zevenenzeventig.</t>
-        </is>
-      </c>
-      <c r="I287" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-kosaris-boek-drie-deel-3-film.html</t>
-        </is>
-      </c>
-      <c r="J287" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_de-kosaris-boek-drie-deel-3-film.jpg</t>
-        </is>
-      </c>
-      <c r="K287" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L287" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M287" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N287" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="O287" t="inlineStr">
-        <is>
-          <t>1.3.3</t>
-        </is>
-      </c>
-      <c r="P287" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="Q287" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="R287" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="S287" t="n">
-        <v>20</v>
-      </c>
-      <c r="T287" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI287" t="inlineStr">
-        <is>
-          <t>Kosaris,film,Opvoeding,Anthea</t>
-        </is>
-      </c>
-      <c r="AK287" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="AL287" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-      <c r="AM287" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-    </row>
-    <row r="288">
-      <c r="B288" t="inlineStr">
-        <is>
-          <t>1.7.20</t>
-        </is>
-      </c>
-      <c r="C288" t="inlineStr">
-        <is>
-          <t>1.7</t>
-        </is>
-      </c>
-      <c r="D288" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-      <c r="E288" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F288" t="inlineStr">
-        <is>
-          <t>De gouden kooi</t>
-        </is>
-      </c>
-      <c r="G288" t="inlineStr">
-        <is>
-          <t>Nederlanders opgesloten in een kooi van 74 tot 90 procent belastingdruk, terwijl buitenlandse eigenaren er onbelast doorheen lopen</t>
-        </is>
-      </c>
-      <c r="H288" t="inlineStr">
-        <is>
-          <t>Nederland is voor zijn eigen werkende burgers een gouden kooi. Wie hier woont, werkt en verdient, betaalt tussen de 74 en 90 procent van zijn werkelijke inkomen. Wie hier alleen eigenaar is loopt onbelast door de tralies. De statistiek verhult dit via de BBP-BNP-truc. Een oproep tot herkadering.</t>
-        </is>
-      </c>
-      <c r="I288" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-gouden-kooi.html</t>
-        </is>
-      </c>
-      <c r="J288" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_de-gouden-kooi.jpg</t>
-        </is>
-      </c>
-      <c r="K288" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L288" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M288" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N288" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="P288" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="Q288" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="R288" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="S288" t="n">
-        <v>19</v>
-      </c>
-      <c r="T288" t="n">
-        <v>20</v>
-      </c>
-      <c r="AI288" t="inlineStr">
-        <is>
-          <t>filosofie, wat-opkomt, europese-systeemcrisis, kluis, bewaring, innovatie, jurisdictie, symptoombestrijding</t>
-        </is>
-      </c>
-      <c r="AK288" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="AL288" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-      <c r="AM288" t="inlineStr">
-        <is>
-          <t>wat-opkomt, belasting, gouden-kooi, bnp, bbp, nederland, buitenlandse-eigenaar, belastingdruk, nova-democratia</t>
-        </is>
-      </c>
-      <c r="AO288" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="289">
-      <c r="B289" t="inlineStr">
-        <is>
-          <t>1.3.1.8</t>
-        </is>
-      </c>
-      <c r="C289" t="inlineStr">
-        <is>
-          <t>1.3.1</t>
-        </is>
-      </c>
-      <c r="D289" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-      <c r="E289" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F289" t="inlineStr">
-        <is>
-          <t>De gouden kooi</t>
-        </is>
-      </c>
-      <c r="G289" t="inlineStr">
-        <is>
-          <t>Nederlanders opgesloten in een kooi van 74 tot 90 procent belastingdruk, terwijl buitenlandse eigenaren er onbelast doorheen lopen</t>
-        </is>
-      </c>
-      <c r="H289" t="inlineStr">
-        <is>
-          <t>Nederland is voor zijn eigen werkende burgers een gouden kooi. Wie hier woont, werkt en verdient, betaalt tussen de 74 en 90 procent van zijn werkelijke inkomen. Wie hier alleen eigenaar is loopt onbelast door de tralies. De statistiek verhult dit via de BBP-BNP-truc. Een oproep tot herkadering.</t>
-        </is>
-      </c>
-      <c r="I289" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-gouden-kooi.html</t>
-        </is>
-      </c>
-      <c r="J289" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_de-gouden-kooi.jpg</t>
-        </is>
-      </c>
-      <c r="K289" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L289" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M289" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N289" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="O289" t="inlineStr">
-        <is>
-          <t>1.3.1</t>
-        </is>
-      </c>
-      <c r="P289" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="Q289" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="R289" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="S289" t="n">
-        <v>7</v>
-      </c>
-      <c r="T289" t="n">
-        <v>8</v>
-      </c>
-      <c r="AI289" t="inlineStr">
-        <is>
-          <t>filosofie, wat-opkomt, europese-systeemcrisis, kluis, bewaring, innovatie, jurisdictie, symptoombestrijding</t>
-        </is>
-      </c>
-      <c r="AK289" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="AL289" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-      <c r="AM289" t="inlineStr">
-        <is>
-          <t>wat-opkomt, belasting, gouden-kooi, bnp, bbp, nederland, buitenlandse-eigenaar, belastingdruk, nova-democratia</t>
-        </is>
-      </c>
-      <c r="AO289" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="290">
-      <c r="B290" t="inlineStr">
-        <is>
-          <t>2.1.1.63</t>
-        </is>
-      </c>
-      <c r="C290" t="inlineStr">
-        <is>
-          <t>2.1.1</t>
-        </is>
-      </c>
-      <c r="D290" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="E290" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F290" t="inlineStr">
-        <is>
-          <t>Der goldene Käfig</t>
-        </is>
-      </c>
-      <c r="G290" t="inlineStr">
-        <is>
-          <t>Warnstufe Rot für arbeitende Deutsche — bis 2030 Warnstufe Schwarz, während ausländische Eigentümer unbelastet hindurchgehen</t>
-        </is>
-      </c>
-      <c r="H290" t="inlineStr">
-        <is>
-          <t>Deutschland ist für seine eigenen arbeitenden Bürger ein goldener Käfig. Wer hier wohnt, arbeitet und verdient, zahlt zwischen 74 und 90 Prozent seines tatsächlichen Einkommens. Wer hier nur Eigentümer ist, geht unbelastet durch die Gitterstäbe. Die Statistik verhüllt dies über die BIP-BNP-Trick. Ein Aufruf zur Neurahmung.</t>
-        </is>
-      </c>
-      <c r="I290" t="inlineStr">
-        <is>
-          <t>was-aufkommt/der-goldene-kaefig.html</t>
-        </is>
-      </c>
-      <c r="J290" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_der-goldene-kaefig.jpg</t>
-        </is>
-      </c>
-      <c r="K290" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L290" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M290" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N290" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="P290" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="Q290" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="R290" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="S290" t="n">
-        <v>63</v>
-      </c>
-      <c r="T290" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI290" t="inlineStr">
-        <is>
-          <t>steuern, staatsquote, bip, bnp, deutschland, ausländische-eigentümer, verteidigung</t>
-        </is>
-      </c>
-      <c r="AK290" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="AL290" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-      <c r="AM290" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="AO290" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="291">
-      <c r="B291" t="inlineStr">
-        <is>
-          <t>3.1.1.63</t>
-        </is>
-      </c>
-      <c r="C291" t="inlineStr">
-        <is>
-          <t>3.1.1</t>
-        </is>
-      </c>
-      <c r="D291" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="E291" t="inlineStr">
-        <is>
-          <t>artikel</t>
-        </is>
-      </c>
-      <c r="F291" t="inlineStr">
-        <is>
-          <t>The Golden Cage</t>
-        </is>
-      </c>
-      <c r="G291" t="inlineStr">
-        <is>
-          <t>Warning Level Red for working Britons — Warning Level Black by 2030, while foreign owners pass unhindered through the bars</t>
-        </is>
-      </c>
-      <c r="H291" t="inlineStr">
-        <is>
-          <t>The UK is a golden cage for its own working citizens. Whoever lives, works and earns here pays between 74 and 90 percent of their real income. Whoever is only an owner walks unhindered through the bars. Statistics conceal this via the GDP-GNP trick. A call for reframing.</t>
-        </is>
-      </c>
-      <c r="I291" t="inlineStr">
-        <is>
-          <t>what-surfaces/the-golden-cage.html</t>
-        </is>
-      </c>
-      <c r="J291" t="inlineStr">
-        <is>
-          <t>../assets/wat-opkomt/H_the-golden-cage.jpg</t>
-        </is>
-      </c>
-      <c r="K291" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L291" t="inlineStr">
-        <is>
-          <t>standaard</t>
-        </is>
-      </c>
-      <c r="M291" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N291" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="O291" t="inlineStr"/>
-      <c r="P291" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="Q291" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="R291" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="S291" t="n">
-        <v>63</v>
-      </c>
-      <c r="T291" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI291" t="inlineStr">
-        <is>
-          <t>taxation, public spending, gdp, gnp, uk, foreign-owners, defence</t>
-        </is>
-      </c>
-      <c r="AK291" t="inlineStr">
-        <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="AL291" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-      <c r="AM291" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="AO291" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nederland aug 2026 – aug 2028: het complete beeld — 28 breuk-elementen
Uitgebreide systeemanalyse Nederland peildatum 15 augustus 2026:
- 1 hoofdpagina (nederland-kompleet/index.html) met DEEL A kern-diagnose
  + DEEL C-L (fundamentele conditie, 12 cascades, 5 zwarte gaten in
  begroting, Groningen, Deltaplan, jachtwerven-cascade, kalender-tijdlijn,
  revolutie-scenario's, structurele conclusies, volledige bronnenlijst)
- 28 subpagina's per breuk-element (B.1 t/m B.28), elk met eigen grafiek
- 1 hero-illustratie (Leo Belgicus op brekend fundament, klassieke litho)
- 29 analytische grafieken (matplotlib) uit brondocument

Xlsx: rijen 282-310 toegevoegd onder ouder 1.5.1 (Nederland-submenu).
Hoofdpagina code 1.5.1.10, elementen 1.5.1.10.1 t/m 1.5.1.10.28.

Bron: Jacobus van Merksteijn, NL_kompleet.docx (Het Open Vizier).
Publicatie onder Nederland pull-down menu, niet op voorpagina.
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -20,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -60,12 +61,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR281"/>
+  <dimension ref="B2:AR310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -24996,6 +24998,2968 @@
         </is>
       </c>
       <c r="AM281" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>1.5.1</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Nederland aug 2026 – aug 2028: het complete beeld</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Systeembreuk en revolutie-kans — 28 breuk-elementen volledig uitgewerkt</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Compleet en volledig beeld van de systeembreuk en revolutie-kans Nederland aug 2026 – aug 2028. Alle 28 breuk-elementen, elk uitgewerkt met per-maand-dynamiek, brondocumentatie, kritieke datums, mechanica, uitwerking en revolutie-scenario's. Peildatum: 15 augustus 2026.</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>../assets/nederland-kompleet/H_nederland_kompleet.jpg</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N282" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P282" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q282" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S282" t="n">
+        <v>10</v>
+      </c>
+      <c r="T282" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI282" t="inlineStr">
+        <is>
+          <t>Nederland, systeembreuk, revolutie, BBP, werkloosheid, industrie, cascade, Rotterdam, Rijn, KVK, MKB, EBITDA, jachtwerven, demografie, zeespiegel, klimaat, AI, asiel, Groningen, Schiphol, kern-diagnose</t>
+        </is>
+      </c>
+      <c r="AK282" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL282" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM282" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>1.5.1.10.1</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Element 1 — Werkloosheid officieel versus reëel</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Breuk-element 1 van 28</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Breuk-element 1 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Werkloosheid officieel versus reëel.</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/werkloosheid-officieel-versus-reeel.html</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr"/>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N283" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P283" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q283" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R283" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S283" t="n">
+        <v>1</v>
+      </c>
+      <c r="T283" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI283" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 1, Werkloosheid officieel versus reëel</t>
+        </is>
+      </c>
+      <c r="AK283" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL283" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM283" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>1.5.1.10.2</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Element 2 — Duitse industrie-cascade</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>Breuk-element 2 van 28</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Breuk-element 2 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Duitse industrie-cascade.</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/duitse-industrie-cascade.html</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr"/>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N284" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R284" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S284" t="n">
+        <v>2</v>
+      </c>
+      <c r="T284" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI284" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 2, Duitse industrie-cascade</t>
+        </is>
+      </c>
+      <c r="AK284" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL284" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM284" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>1.5.1.10.3</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Element 3 — Nederlandse industrie-cascade</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Breuk-element 3 van 28</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Breuk-element 3 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Nederlandse industrie-cascade.</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/nederlandse-industrie-cascade.html</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr"/>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N285" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q285" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R285" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S285" t="n">
+        <v>3</v>
+      </c>
+      <c r="T285" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI285" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 3, Nederlandse industrie-cascade</t>
+        </is>
+      </c>
+      <c r="AK285" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL285" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM285" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>1.5.1.10.4</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Element 4 — Multiplicator-effect banen</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Breuk-element 4 van 28</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Breuk-element 4 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Multiplicator-effect banen.</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/multiplicator-effect-banen.html</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr"/>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N286" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R286" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S286" t="n">
+        <v>4</v>
+      </c>
+      <c r="T286" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI286" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 4, Multiplicator-effect banen</t>
+        </is>
+      </c>
+      <c r="AK286" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL286" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM286" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>1.5.1.10.5</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Element 5 — Rotterdam-doorvoer: permanent -30% + Rijn-laagwater</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Breuk-element 5 van 28</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Breuk-element 5 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Rotterdam-doorvoer: permanent -30% + Rijn-laagwater.</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/rotterdam-doorvoer.html</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr"/>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N287" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R287" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S287" t="n">
+        <v>5</v>
+      </c>
+      <c r="T287" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI287" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 5, Rotterdam-doorvoer: permanent -30% + Rijn-laagwater</t>
+        </is>
+      </c>
+      <c r="AK287" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL287" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM287" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>1.5.1.10.6</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Element 6 — KVK stoppers-versnelling MKB</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Breuk-element 6 van 28</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Breuk-element 6 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: KVK stoppers-versnelling MKB.</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/kvk-stoppers-versnelling.html</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr"/>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N288" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R288" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S288" t="n">
+        <v>6</v>
+      </c>
+      <c r="T288" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI288" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 6, KVK stoppers-versnelling MKB</t>
+        </is>
+      </c>
+      <c r="AK288" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL288" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM288" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>1.5.1.10.7</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Element 7 — EBITDA-multiple collaps (opschmuck-mechaniek)</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Breuk-element 7 van 28</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Breuk-element 7 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: EBITDA-multiple collaps (opschmuck-mechaniek).</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/ebitda-multiple-collaps.html</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr"/>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N289" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R289" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S289" t="n">
+        <v>7</v>
+      </c>
+      <c r="T289" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI289" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 7, EBITDA-multiple collaps (opschmuck-mechaniek)</t>
+        </is>
+      </c>
+      <c r="AK289" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL289" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM289" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>1.5.1.10.8</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Element 8 — Middenstand exit-realisatie (5 op 6 intentie)</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Breuk-element 8 van 28</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Breuk-element 8 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Middenstand exit-realisatie (5 op 6 intentie).</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/middenstand-exit-realisatie.html</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr"/>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R290" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S290" t="n">
+        <v>8</v>
+      </c>
+      <c r="T290" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI290" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 8, Middenstand exit-realisatie (5 op 6 intentie)</t>
+        </is>
+      </c>
+      <c r="AK290" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL290" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM290" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>1.5.1.10.9</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Element 9 — Jachtwerven-cascade (Lengers 28 juli 2026)</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Breuk-element 9 van 28</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Breuk-element 9 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Jachtwerven-cascade (Lengers 28 juli 2026).</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/jachtwerven-cascade.html</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr"/>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N291" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R291" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S291" t="n">
+        <v>9</v>
+      </c>
+      <c r="T291" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI291" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 9, Jachtwerven-cascade (Lengers 28 juli 2026)</t>
+        </is>
+      </c>
+      <c r="AK291" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL291" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM291" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>1.5.1.10.10</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Element 10 — Balans-fictie MKB (Lengers case + EU-schaal)</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Breuk-element 10 van 28</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>Breuk-element 10 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Balans-fictie MKB (Lengers case + EU-schaal).</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/balans-fictie-mkb.html</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr"/>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N292" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R292" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S292" t="n">
+        <v>10</v>
+      </c>
+      <c r="T292" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI292" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 10, Balans-fictie MKB (Lengers case + EU-schaal)</t>
+        </is>
+      </c>
+      <c r="AK292" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL292" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM292" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>1.5.1.10.11</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Element 11 — Consumentenvertrouwen</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Breuk-element 11 van 28</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>Breuk-element 11 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Consumentenvertrouwen.</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/consumentenvertrouwen.html</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr"/>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N293" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R293" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S293" t="n">
+        <v>11</v>
+      </c>
+      <c r="T293" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI293" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 11, Consumentenvertrouwen</t>
+        </is>
+      </c>
+      <c r="AK293" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL293" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM293" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>1.5.1.10.12</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Element 12 — Premium-auto (BPM 3-fasen)</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Breuk-element 12 van 28</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>Breuk-element 12 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Premium-auto (BPM 3-fasen).</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/premium-auto-bpm.html</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr"/>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N294" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R294" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S294" t="n">
+        <v>12</v>
+      </c>
+      <c r="T294" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI294" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 12, Premium-auto (BPM 3-fasen)</t>
+        </is>
+      </c>
+      <c r="AK294" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL294" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM294" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>1.5.1.10.13</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Element 13 — Superjachten (tweedeling)</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Breuk-element 13 van 28</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Breuk-element 13 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Superjachten (tweedeling).</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/superjachten-tweedeling.html</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr"/>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N295" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R295" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S295" t="n">
+        <v>13</v>
+      </c>
+      <c r="T295" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI295" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 13, Superjachten (tweedeling)</t>
+        </is>
+      </c>
+      <c r="AK295" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL295" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM295" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>1.5.1.10.14</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Element 14 — EU fertiliteit 1,34 (Eurostat)</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Breuk-element 14 van 28</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Breuk-element 14 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: EU fertiliteit 1,34 (Eurostat).</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/eu-fertiliteit.html</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr"/>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N296" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R296" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S296" t="n">
+        <v>14</v>
+      </c>
+      <c r="T296" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI296" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 14, EU fertiliteit 1,34 (Eurostat)</t>
+        </is>
+      </c>
+      <c r="AK296" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL296" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM296" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>1.5.1.10.15</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Element 15 — NL TFR 1,42 (arbeidsaanbod 20 jaar out)</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>Breuk-element 15 van 28</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Breuk-element 15 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: NL TFR 1,42 (arbeidsaanbod 20 jaar out).</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/nl-tfr.html</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr"/>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N297" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R297" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S297" t="n">
+        <v>15</v>
+      </c>
+      <c r="T297" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI297" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 15, NL TFR 1,42 (arbeidsaanbod 20 jaar out)</t>
+        </is>
+      </c>
+      <c r="AK297" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL297" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM297" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>1.5.1.10.16</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Element 16 — EU-populatie 2100-projectie</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>Breuk-element 16 van 28</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Breuk-element 16 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: EU-populatie 2100-projectie.</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/eu-populatie-2100.html</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr"/>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N298" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R298" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S298" t="n">
+        <v>16</v>
+      </c>
+      <c r="T298" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI298" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 16, EU-populatie 2100-projectie</t>
+        </is>
+      </c>
+      <c r="AK298" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL298" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM298" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>1.5.1.10.17</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Element 17 — Zeespiegel + Deltaplan</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>Breuk-element 17 van 28</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Breuk-element 17 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Zeespiegel + Deltaplan.</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/zeespiegel-deltaplan.html</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr"/>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N299" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R299" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S299" t="n">
+        <v>17</v>
+      </c>
+      <c r="T299" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI299" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 17, Zeespiegel + Deltaplan</t>
+        </is>
+      </c>
+      <c r="AK299" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL299" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM299" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>1.5.1.10.18</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Element 18 — RWS + ProRail achterstallig onderhoud</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>Breuk-element 18 van 28</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>Breuk-element 18 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: RWS + ProRail achterstallig onderhoud.</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/rws-prorail-onderhoud.html</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr"/>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N300" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q300" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R300" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S300" t="n">
+        <v>18</v>
+      </c>
+      <c r="T300" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI300" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 18, RWS + ProRail achterstallig onderhoud</t>
+        </is>
+      </c>
+      <c r="AK300" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL300" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM300" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>1.5.1.10.19</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Element 19 — EU bosbranden + klimaatschade</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>Breuk-element 19 van 28</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>Breuk-element 19 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: EU bosbranden + klimaatschade.</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/eu-bosbranden-klimaatschade.html</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr"/>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N301" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P301" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q301" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R301" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S301" t="n">
+        <v>19</v>
+      </c>
+      <c r="T301" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI301" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 19, EU bosbranden + klimaatschade</t>
+        </is>
+      </c>
+      <c r="AK301" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL301" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM301" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>1.5.1.10.20</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Element 20 — Rijn-waterstand (aug 2026 record)</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>Breuk-element 20 van 28</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Breuk-element 20 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Rijn-waterstand (aug 2026 record).</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/rijn-waterstand.html</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr"/>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N302" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q302" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R302" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S302" t="n">
+        <v>20</v>
+      </c>
+      <c r="T302" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI302" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 20, Rijn-waterstand (aug 2026 record)</t>
+        </is>
+      </c>
+      <c r="AK302" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL302" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM302" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>1.5.1.10.21</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Element 21 — AI-disruptie hoger opgeleiden</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>Breuk-element 21 van 28</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Breuk-element 21 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: AI-disruptie hoger opgeleiden.</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/ai-disruptie.html</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr"/>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N303" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P303" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q303" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R303" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S303" t="n">
+        <v>21</v>
+      </c>
+      <c r="T303" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI303" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 21, AI-disruptie hoger opgeleiden</t>
+        </is>
+      </c>
+      <c r="AK303" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL303" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM303" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>1.5.1.10.22</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Element 22 — Asielkosten NL</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>Breuk-element 22 van 28</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>Breuk-element 22 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Asielkosten NL.</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/asielkosten-nl.html</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr"/>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N304" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P304" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q304" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R304" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S304" t="n">
+        <v>22</v>
+      </c>
+      <c r="T304" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI304" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 22, Asielkosten NL</t>
+        </is>
+      </c>
+      <c r="AK304" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL304" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM304" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>1.5.1.10.23</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Element 23 — Kinderopvang bovenmatig gedeelte</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>Breuk-element 23 van 28</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Breuk-element 23 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Kinderopvang bovenmatig gedeelte.</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/kinderopvang-bovenmatig.html</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr"/>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N305" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P305" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q305" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R305" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S305" t="n">
+        <v>23</v>
+      </c>
+      <c r="T305" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI305" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 23, Kinderopvang bovenmatig gedeelte</t>
+        </is>
+      </c>
+      <c r="AK305" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL305" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM305" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>1.5.1.10.24</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Element 24 — Vrachtauto elektrificatie (ZE-zone deadlines)</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Breuk-element 24 van 28</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>Breuk-element 24 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Vrachtauto elektrificatie (ZE-zone deadlines).</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/vrachtauto-elektrificatie.html</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr"/>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N306" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P306" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R306" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S306" t="n">
+        <v>24</v>
+      </c>
+      <c r="T306" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI306" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 24, Vrachtauto elektrificatie (ZE-zone deadlines)</t>
+        </is>
+      </c>
+      <c r="AK306" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL306" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM306" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>1.5.1.10.25</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Element 25 — Groningen gas + Markerwaard-alternatief</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>Breuk-element 25 van 28</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>Breuk-element 25 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Groningen gas + Markerwaard-alternatief.</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/groningen-gas.html</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr"/>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N307" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P307" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R307" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S307" t="n">
+        <v>25</v>
+      </c>
+      <c r="T307" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI307" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 25, Groningen gas + Markerwaard-alternatief</t>
+        </is>
+      </c>
+      <c r="AK307" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL307" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM307" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>1.5.1.10.26</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Element 26 — Miljonair-migratie (Henley + box3)</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>Breuk-element 26 van 28</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Breuk-element 26 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Miljonair-migratie (Henley + box3).</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/miljonair-migratie.html</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr"/>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N308" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P308" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R308" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S308" t="n">
+        <v>26</v>
+      </c>
+      <c r="T308" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI308" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 26, Miljonair-migratie (Henley + box3)</t>
+        </is>
+      </c>
+      <c r="AK308" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL308" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM308" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>1.5.1.10.27</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Element 27 — EU werkloosheid EU-buren</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>Breuk-element 27 van 28</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Breuk-element 27 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: EU werkloosheid EU-buren.</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/eu-werkloosheid-buren.html</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr"/>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N309" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P309" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q309" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R309" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S309" t="n">
+        <v>27</v>
+      </c>
+      <c r="T309" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI309" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 27, EU werkloosheid EU-buren</t>
+        </is>
+      </c>
+      <c r="AK309" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL309" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM309" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>1.5.1.10.28</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Element 28 — Schiphol krimp (LVB 2026 + natuurvergunning)</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>Breuk-element 28 van 28</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Breuk-element 28 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Schiphol krimp (LVB 2026 + natuurvergunning).</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/schiphol-krimp.html</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr"/>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N310" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P310" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q310" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R310" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S310" t="n">
+        <v>28</v>
+      </c>
+      <c r="T310" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI310" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element 28, Schiphol krimp (LVB 2026 + natuurvergunning)</t>
+        </is>
+      </c>
+      <c r="AK310" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL310" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM310" t="inlineStr">
         <is>
           <t>nl</t>
         </is>

</xml_diff>

<commit_message>
publiceer: Nederland aug 2026 – aug 2028 — het complete beeld
- Xlsx: 29 rijen toegevoegd (hoofdpagina 1.5.1.10 + 28 elementen 1.5.1.10.1..28)
- 29 HTML-bestanden onder nl/nederland-kompleet/
- 30 assets onder assets/nederland-kompleet/ (hero + 29 grafieken)

De GitHub Action regenereert de 5 JSON-tabellen uit de xlsx.
Hoofdmenu-injectie in .ov-nav volgt in aparte commit conform MATRIX-REGELS §1B/§1C.
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR281"/>
+  <dimension ref="B2:AR310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -24998,6 +24998,2968 @@
         </is>
       </c>
       <c r="AM281" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>1.5.1</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Nederland aug 2026 – aug 2028: het complete beeld</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Systeembreuk en revolutie-kans — 28 breuk-elementen volledig uitgewerkt</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Compleet en volledig beeld van de systeembreuk en revolutie-kans Nederland aug 2026 – aug 2028. Alle 28 breuk-elementen met per-maand-dynamiek, brondocumentatie en revolutie-scenario's. Peildatum: 15 augustus 2026.</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/index.html</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>../assets/nederland-kompleet/H_nederland_kompleet.jpg</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N282" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P282" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q282" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S282" t="n">
+        <v>10</v>
+      </c>
+      <c r="T282" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI282" t="inlineStr">
+        <is>
+          <t>Nederland, systeembreuk, revolutie, BBP, werkloosheid, industrie, cascade, Rotterdam, Rijn, KVK, MKB, EBITDA, jachtwerven, demografie, zeespiegel, klimaat, AI, asiel, Groningen, Schiphol, kern-diagnose</t>
+        </is>
+      </c>
+      <c r="AK282" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL282" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM282" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>1.5.1.10.1</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Element 1 — Werkloosheid officieel versus reëel</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Breuk-element 1 van 28</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Breuk-element 1 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Werkloosheid officieel versus reëel.</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/werkloosheid-officieel-versus-reeel.html</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr"/>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N283" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P283" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q283" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R283" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S283" t="n">
+        <v>1</v>
+      </c>
+      <c r="T283" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI283" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Werkloosheid officieel versus reëel</t>
+        </is>
+      </c>
+      <c r="AK283" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL283" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM283" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>1.5.1.10.2</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Element 2 — Duitse industrie-cascade</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>Breuk-element 2 van 28</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Breuk-element 2 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Duitse industrie-cascade.</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/duitse-industrie-cascade.html</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr"/>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N284" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R284" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S284" t="n">
+        <v>2</v>
+      </c>
+      <c r="T284" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI284" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Duitse industrie-cascade</t>
+        </is>
+      </c>
+      <c r="AK284" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL284" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM284" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>1.5.1.10.3</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Element 3 — Nederlandse industrie-cascade</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Breuk-element 3 van 28</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Breuk-element 3 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Nederlandse industrie-cascade.</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/nederlandse-industrie-cascade.html</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr"/>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N285" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q285" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R285" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S285" t="n">
+        <v>3</v>
+      </c>
+      <c r="T285" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI285" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Nederlandse industrie-cascade</t>
+        </is>
+      </c>
+      <c r="AK285" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL285" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM285" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>1.5.1.10.4</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Element 4 — Multiplicator-effect banen</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Breuk-element 4 van 28</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Breuk-element 4 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Multiplicator-effect banen.</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/multiplicator-effect-banen.html</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr"/>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N286" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R286" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S286" t="n">
+        <v>4</v>
+      </c>
+      <c r="T286" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI286" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Multiplicator-effect banen</t>
+        </is>
+      </c>
+      <c r="AK286" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL286" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM286" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>1.5.1.10.5</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Element 5 — Rotterdam-doorvoer: permanent -30% + Rijn-laagwater</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Breuk-element 5 van 28</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Breuk-element 5 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Rotterdam-doorvoer: permanent -30% + Rijn-laagwater.</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/rotterdam-doorvoer.html</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr"/>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N287" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R287" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S287" t="n">
+        <v>5</v>
+      </c>
+      <c r="T287" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI287" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Rotterdam-doorvoer: permanent -30% + Rijn-laagwater</t>
+        </is>
+      </c>
+      <c r="AK287" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL287" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM287" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>1.5.1.10.6</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Element 6 — KVK stoppers-versnelling MKB</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Breuk-element 6 van 28</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Breuk-element 6 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: KVK stoppers-versnelling MKB.</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/kvk-stoppers-versnelling.html</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr"/>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N288" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R288" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S288" t="n">
+        <v>6</v>
+      </c>
+      <c r="T288" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI288" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, KVK stoppers-versnelling MKB</t>
+        </is>
+      </c>
+      <c r="AK288" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL288" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM288" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>1.5.1.10.7</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Element 7 — EBITDA-multiple collaps (opschmuck-mechaniek)</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Breuk-element 7 van 28</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Breuk-element 7 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: EBITDA-multiple collaps (opschmuck-mechaniek).</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/ebitda-multiple-collaps.html</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr"/>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N289" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R289" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S289" t="n">
+        <v>7</v>
+      </c>
+      <c r="T289" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI289" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, EBITDA-multiple collaps (opschmuck-mechaniek)</t>
+        </is>
+      </c>
+      <c r="AK289" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL289" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM289" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>1.5.1.10.8</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Element 8 — Middenstand exit-realisatie (5 op 6 intentie)</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Breuk-element 8 van 28</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Breuk-element 8 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Middenstand exit-realisatie (5 op 6 intentie).</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/middenstand-exit-realisatie.html</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr"/>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R290" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S290" t="n">
+        <v>8</v>
+      </c>
+      <c r="T290" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI290" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Middenstand exit-realisatie (5 op 6 intentie)</t>
+        </is>
+      </c>
+      <c r="AK290" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL290" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM290" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>1.5.1.10.9</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Element 9 — Jachtwerven-cascade (Lengers 28 juli 2026)</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Breuk-element 9 van 28</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Breuk-element 9 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Jachtwerven-cascade (Lengers 28 juli 2026).</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/jachtwerven-cascade.html</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr"/>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N291" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R291" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S291" t="n">
+        <v>9</v>
+      </c>
+      <c r="T291" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI291" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Jachtwerven-cascade (Lengers 28 juli 2026)</t>
+        </is>
+      </c>
+      <c r="AK291" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL291" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM291" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>1.5.1.10.10</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Element 10 — Balans-fictie MKB (Lengers case + EU-schaal)</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Breuk-element 10 van 28</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>Breuk-element 10 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Balans-fictie MKB (Lengers case + EU-schaal).</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/balans-fictie-mkb.html</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr"/>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N292" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R292" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S292" t="n">
+        <v>10</v>
+      </c>
+      <c r="T292" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI292" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Balans-fictie MKB (Lengers case + EU-schaal)</t>
+        </is>
+      </c>
+      <c r="AK292" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL292" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM292" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>1.5.1.10.11</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Element 11 — Consumentenvertrouwen</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Breuk-element 11 van 28</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>Breuk-element 11 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Consumentenvertrouwen.</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/consumentenvertrouwen.html</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr"/>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N293" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R293" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S293" t="n">
+        <v>11</v>
+      </c>
+      <c r="T293" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI293" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Consumentenvertrouwen</t>
+        </is>
+      </c>
+      <c r="AK293" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL293" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM293" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>1.5.1.10.12</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Element 12 — Premium-auto (BPM 3-fasen)</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Breuk-element 12 van 28</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>Breuk-element 12 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Premium-auto (BPM 3-fasen).</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/premium-auto-bpm.html</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr"/>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N294" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R294" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S294" t="n">
+        <v>12</v>
+      </c>
+      <c r="T294" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI294" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Premium-auto (BPM 3-fasen)</t>
+        </is>
+      </c>
+      <c r="AK294" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL294" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM294" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>1.5.1.10.13</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Element 13 — Superjachten (tweedeling)</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Breuk-element 13 van 28</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Breuk-element 13 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Superjachten (tweedeling).</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/superjachten-tweedeling.html</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr"/>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N295" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R295" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S295" t="n">
+        <v>13</v>
+      </c>
+      <c r="T295" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI295" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Superjachten (tweedeling)</t>
+        </is>
+      </c>
+      <c r="AK295" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL295" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM295" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>1.5.1.10.14</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Element 14 — EU fertiliteit 1,34 (Eurostat)</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Breuk-element 14 van 28</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Breuk-element 14 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: EU fertiliteit 1,34 (Eurostat).</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/eu-fertiliteit.html</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr"/>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N296" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R296" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S296" t="n">
+        <v>14</v>
+      </c>
+      <c r="T296" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI296" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, EU fertiliteit 1,34 (Eurostat)</t>
+        </is>
+      </c>
+      <c r="AK296" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL296" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM296" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>1.5.1.10.15</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Element 15 — NL TFR 1,42 (arbeidsaanbod 20 jaar out)</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>Breuk-element 15 van 28</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Breuk-element 15 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: NL TFR 1,42 (arbeidsaanbod 20 jaar out).</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/nl-tfr.html</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr"/>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N297" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R297" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S297" t="n">
+        <v>15</v>
+      </c>
+      <c r="T297" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI297" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, NL TFR 1,42 (arbeidsaanbod 20 jaar out)</t>
+        </is>
+      </c>
+      <c r="AK297" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL297" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM297" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>1.5.1.10.16</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Element 16 — EU-populatie 2100-projectie</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>Breuk-element 16 van 28</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Breuk-element 16 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: EU-populatie 2100-projectie.</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/eu-populatie-2100.html</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr"/>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N298" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R298" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S298" t="n">
+        <v>16</v>
+      </c>
+      <c r="T298" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI298" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, EU-populatie 2100-projectie</t>
+        </is>
+      </c>
+      <c r="AK298" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL298" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM298" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>1.5.1.10.17</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Element 17 — Zeespiegel + Deltaplan</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>Breuk-element 17 van 28</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Breuk-element 17 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Zeespiegel + Deltaplan.</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/zeespiegel-deltaplan.html</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr"/>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N299" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R299" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S299" t="n">
+        <v>17</v>
+      </c>
+      <c r="T299" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI299" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Zeespiegel + Deltaplan</t>
+        </is>
+      </c>
+      <c r="AK299" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL299" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM299" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>1.5.1.10.18</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Element 18 — RWS + ProRail achterstallig onderhoud</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>Breuk-element 18 van 28</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>Breuk-element 18 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: RWS + ProRail achterstallig onderhoud.</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/rws-prorail-onderhoud.html</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr"/>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N300" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q300" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R300" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S300" t="n">
+        <v>18</v>
+      </c>
+      <c r="T300" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI300" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, RWS + ProRail achterstallig onderhoud</t>
+        </is>
+      </c>
+      <c r="AK300" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL300" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM300" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>1.5.1.10.19</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Element 19 — EU bosbranden + klimaatschade</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>Breuk-element 19 van 28</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>Breuk-element 19 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: EU bosbranden + klimaatschade.</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/eu-bosbranden-klimaatschade.html</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr"/>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N301" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P301" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q301" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R301" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S301" t="n">
+        <v>19</v>
+      </c>
+      <c r="T301" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI301" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, EU bosbranden + klimaatschade</t>
+        </is>
+      </c>
+      <c r="AK301" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL301" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM301" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>1.5.1.10.20</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Element 20 — Rijn-waterstand (aug 2026 record)</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>Breuk-element 20 van 28</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Breuk-element 20 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Rijn-waterstand (aug 2026 record).</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/rijn-waterstand.html</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr"/>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N302" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q302" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R302" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S302" t="n">
+        <v>20</v>
+      </c>
+      <c r="T302" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI302" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Rijn-waterstand (aug 2026 record)</t>
+        </is>
+      </c>
+      <c r="AK302" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL302" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM302" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>1.5.1.10.21</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Element 21 — AI-disruptie hoger opgeleiden</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>Breuk-element 21 van 28</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Breuk-element 21 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: AI-disruptie hoger opgeleiden.</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/ai-disruptie.html</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr"/>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N303" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P303" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q303" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R303" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S303" t="n">
+        <v>21</v>
+      </c>
+      <c r="T303" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI303" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, AI-disruptie hoger opgeleiden</t>
+        </is>
+      </c>
+      <c r="AK303" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL303" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM303" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>1.5.1.10.22</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Element 22 — Asielkosten NL</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>Breuk-element 22 van 28</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>Breuk-element 22 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Asielkosten NL.</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/asielkosten-nl.html</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr"/>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N304" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P304" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q304" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R304" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S304" t="n">
+        <v>22</v>
+      </c>
+      <c r="T304" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI304" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Asielkosten NL</t>
+        </is>
+      </c>
+      <c r="AK304" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL304" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM304" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>1.5.1.10.23</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Element 23 — Kinderopvang bovenmatig gedeelte</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>Breuk-element 23 van 28</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Breuk-element 23 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Kinderopvang bovenmatig gedeelte.</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/kinderopvang-bovenmatig.html</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr"/>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N305" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P305" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q305" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R305" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S305" t="n">
+        <v>23</v>
+      </c>
+      <c r="T305" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI305" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Kinderopvang bovenmatig gedeelte</t>
+        </is>
+      </c>
+      <c r="AK305" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL305" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM305" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>1.5.1.10.24</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Element 24 — Vrachtauto elektrificatie (ZE-zone deadlines)</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Breuk-element 24 van 28</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>Breuk-element 24 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Vrachtauto elektrificatie (ZE-zone deadlines).</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/vrachtauto-elektrificatie.html</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr"/>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N306" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P306" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R306" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S306" t="n">
+        <v>24</v>
+      </c>
+      <c r="T306" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI306" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Vrachtauto elektrificatie (ZE-zone deadlines)</t>
+        </is>
+      </c>
+      <c r="AK306" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL306" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM306" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>1.5.1.10.25</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Element 25 — Groningen gas + Markerwaard-alternatief</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>Breuk-element 25 van 28</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>Breuk-element 25 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Groningen gas + Markerwaard-alternatief.</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/groningen-gas.html</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr"/>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N307" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P307" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R307" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S307" t="n">
+        <v>25</v>
+      </c>
+      <c r="T307" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI307" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Groningen gas + Markerwaard-alternatief</t>
+        </is>
+      </c>
+      <c r="AK307" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL307" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM307" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>1.5.1.10.26</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Element 26 — Miljonair-migratie (Henley + box3)</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>Breuk-element 26 van 28</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Breuk-element 26 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Miljonair-migratie (Henley + box3).</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/miljonair-migratie.html</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr"/>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N308" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P308" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R308" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S308" t="n">
+        <v>26</v>
+      </c>
+      <c r="T308" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI308" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Miljonair-migratie (Henley + box3)</t>
+        </is>
+      </c>
+      <c r="AK308" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL308" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM308" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>1.5.1.10.27</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Element 27 — EU werkloosheid EU-buren</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>Breuk-element 27 van 28</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Breuk-element 27 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: EU werkloosheid EU-buren.</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/eu-werkloosheid-buren.html</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr"/>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N309" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P309" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q309" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R309" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S309" t="n">
+        <v>27</v>
+      </c>
+      <c r="T309" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI309" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, EU werkloosheid EU-buren</t>
+        </is>
+      </c>
+      <c r="AK309" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL309" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM309" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>1.5.1.10.28</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>1.5.1.10</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Element 28 — Schiphol krimp (LVB 2026 + natuurvergunning)</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>Breuk-element 28 van 28</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Breuk-element 28 van 28 in de systeemanalyse Nederland aug 2026 – aug 2028: Schiphol krimp (LVB 2026 + natuurvergunning).</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>nederland-kompleet/schiphol-krimp.html</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr"/>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>standaard</t>
+        </is>
+      </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N310" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P310" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q310" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R310" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S310" t="n">
+        <v>28</v>
+      </c>
+      <c r="T310" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI310" t="inlineStr">
+        <is>
+          <t>Nederland, breuk-element, Schiphol krimp (LVB 2026 + natuurvergunning)</t>
+        </is>
+      </c>
+      <c r="AK310" s="3" t="n">
+        <v>46249</v>
+      </c>
+      <c r="AL310" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM310" t="inlineStr">
         <is>
           <t>nl</t>
         </is>

</xml_diff>

<commit_message>
xlsx(Knopen): 'Terug naar' invullen voor alle 269 artikelen zonder waarde
Conform MATRIX-REGELS §2.2/§3.4: elk artikel keert terug naar zijn eigen
taal-voorpagina. Voor NL = code 1.1.1 ("De voorpagina", url index.html).

- 269 artikelen aangepast (waren leeg)
- 4 artikelen ongewijzigd (waren al ingevuld)
- 35 niet-artikel rijen overgeslagen (ingang/onderwerp/talenring/taal)

Terug-knop wees eerder naar willekeurige plekken; nu consistent naar voorpagina.
GitHub Action regenereert 2_routes_nl.json (kolom terug_naar).
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -1680,6 +1680,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q15" t="inlineStr">
         <is>
           <t>self</t>
@@ -1855,6 +1860,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q17" t="inlineStr">
         <is>
           <t>self</t>
@@ -1950,6 +1960,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q18" t="inlineStr">
         <is>
           <t>self</t>
@@ -2048,6 +2063,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q19" t="inlineStr">
         <is>
           <t>self</t>
@@ -2146,6 +2166,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q20" t="inlineStr">
         <is>
           <t>self</t>
@@ -2321,6 +2346,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q22" t="inlineStr">
         <is>
           <t>self</t>
@@ -2421,6 +2451,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q23" t="inlineStr">
         <is>
           <t>self</t>
@@ -2509,6 +2544,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q24" t="inlineStr">
         <is>
           <t>self</t>
@@ -2592,6 +2632,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q25" t="inlineStr">
         <is>
           <t>self</t>
@@ -2682,6 +2727,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q26" t="inlineStr">
         <is>
           <t>self</t>
@@ -2852,6 +2902,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q28" t="inlineStr">
         <is>
           <t>self</t>
@@ -2937,6 +2992,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q29" t="inlineStr">
         <is>
           <t>self</t>
@@ -3022,6 +3082,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q30" t="inlineStr">
         <is>
           <t>self</t>
@@ -3107,6 +3172,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q31" t="inlineStr">
         <is>
           <t>self</t>
@@ -3192,6 +3262,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q32" t="inlineStr">
         <is>
           <t>self</t>
@@ -3282,6 +3357,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q33" t="inlineStr">
         <is>
           <t>self</t>
@@ -3467,6 +3547,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q35" t="inlineStr">
         <is>
           <t>self</t>
@@ -3565,6 +3650,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q36" t="inlineStr">
         <is>
           <t>self</t>
@@ -3658,6 +3748,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q37" t="inlineStr">
         <is>
           <t>self</t>
@@ -3753,6 +3848,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q38" t="inlineStr">
         <is>
           <t>self</t>
@@ -3838,6 +3938,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q39" t="inlineStr">
         <is>
           <t>self</t>
@@ -3921,6 +4026,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q40" t="inlineStr">
         <is>
           <t>self</t>
@@ -4009,6 +4119,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q41" t="inlineStr">
         <is>
           <t>self</t>
@@ -4172,6 +4287,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q43" t="inlineStr">
         <is>
           <t>self</t>
@@ -4262,6 +4382,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q44" t="inlineStr">
         <is>
           <t>self</t>
@@ -4360,6 +4485,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q45" t="inlineStr">
         <is>
           <t>self</t>
@@ -4453,6 +4583,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q46" t="inlineStr">
         <is>
           <t>self</t>
@@ -4541,6 +4676,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q47" t="inlineStr">
         <is>
           <t>self</t>
@@ -4641,6 +4781,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q48" t="inlineStr">
         <is>
           <t>self</t>
@@ -4731,6 +4876,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q49" t="inlineStr">
         <is>
           <t>self</t>
@@ -4826,6 +4976,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q50" t="inlineStr">
         <is>
           <t>self</t>
@@ -5004,6 +5159,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q52" t="inlineStr">
         <is>
           <t>self</t>
@@ -5102,6 +5262,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q53" t="inlineStr">
         <is>
           <t>self</t>
@@ -5190,6 +5355,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q54" t="inlineStr">
         <is>
           <t>self</t>
@@ -5280,6 +5450,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q55" t="inlineStr">
         <is>
           <t>self</t>
@@ -5370,6 +5545,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q56" t="inlineStr">
         <is>
           <t>self</t>
@@ -5460,6 +5640,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q57" t="inlineStr">
         <is>
           <t>self</t>
@@ -5630,6 +5815,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q59" t="inlineStr">
         <is>
           <t>self</t>
@@ -5720,6 +5910,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q60" t="inlineStr">
         <is>
           <t>self</t>
@@ -5810,6 +6005,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q61" t="inlineStr">
         <is>
           <t>self</t>
@@ -5900,6 +6100,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q62" t="inlineStr">
         <is>
           <t>self</t>
@@ -5990,6 +6195,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q63" t="inlineStr">
         <is>
           <t>self</t>
@@ -6080,6 +6290,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q64" t="inlineStr">
         <is>
           <t>self</t>
@@ -6170,6 +6385,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q65" t="inlineStr">
         <is>
           <t>self</t>
@@ -6255,6 +6475,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q66" t="inlineStr">
         <is>
           <t>self</t>
@@ -6340,6 +6565,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q67" t="inlineStr">
         <is>
           <t>self</t>
@@ -6440,6 +6670,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q68" t="inlineStr">
         <is>
           <t>self</t>
@@ -6605,6 +6840,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q70" t="inlineStr">
         <is>
           <t>self</t>
@@ -6685,6 +6925,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q71" t="inlineStr">
         <is>
           <t>self</t>
@@ -6765,6 +7010,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q72" t="inlineStr">
         <is>
           <t>self</t>
@@ -6845,6 +7095,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q73" t="inlineStr">
         <is>
           <t>self</t>
@@ -6925,6 +7180,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q74" t="inlineStr">
         <is>
           <t>self</t>
@@ -7085,6 +7345,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q76" t="inlineStr">
         <is>
           <t>self</t>
@@ -7165,6 +7430,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q77" t="inlineStr">
         <is>
           <t>self</t>
@@ -7245,6 +7515,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q78" t="inlineStr">
         <is>
           <t>self</t>
@@ -7325,6 +7600,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q79" t="inlineStr">
         <is>
           <t>self</t>
@@ -7495,6 +7775,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q81" t="inlineStr">
         <is>
           <t>self</t>
@@ -7593,6 +7878,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q82" t="inlineStr">
         <is>
           <t>self</t>
@@ -7691,6 +7981,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q83" t="inlineStr">
         <is>
           <t>self</t>
@@ -7866,6 +8161,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q85" t="inlineStr">
         <is>
           <t>self</t>
@@ -7954,6 +8254,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q86" t="inlineStr">
         <is>
           <t>self</t>
@@ -8059,6 +8364,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q87" t="inlineStr">
         <is>
           <t>self</t>
@@ -8147,6 +8457,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q88" t="inlineStr">
         <is>
           <t>self</t>
@@ -8227,6 +8542,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q89" t="inlineStr">
         <is>
           <t>self</t>
@@ -8307,6 +8627,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q90" t="inlineStr">
         <is>
           <t>self</t>
@@ -8472,6 +8797,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q92" t="inlineStr">
         <is>
           <t>self</t>
@@ -8562,6 +8892,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q93" t="inlineStr">
         <is>
           <t>self</t>
@@ -8652,6 +8987,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q94" t="inlineStr">
         <is>
           <t>self</t>
@@ -8742,6 +9082,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q95" t="inlineStr">
         <is>
           <t>self</t>
@@ -8910,6 +9255,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q97" t="inlineStr">
         <is>
           <t>self</t>
@@ -9005,6 +9355,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q98" t="inlineStr">
         <is>
           <t>self</t>
@@ -9093,6 +9448,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q99" t="inlineStr">
         <is>
           <t>self</t>
@@ -9268,6 +9628,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q101" t="inlineStr">
         <is>
           <t>self</t>
@@ -9348,6 +9713,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q102" t="inlineStr">
         <is>
           <t>self</t>
@@ -9428,6 +9798,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q103" t="inlineStr">
         <is>
           <t>self</t>
@@ -9508,6 +9883,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q104" t="inlineStr">
         <is>
           <t>self</t>
@@ -9588,6 +9968,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q105" t="inlineStr">
         <is>
           <t>self</t>
@@ -9753,6 +10138,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q107" t="inlineStr">
         <is>
           <t>self</t>
@@ -9836,6 +10226,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q108" t="inlineStr">
         <is>
           <t>self</t>
@@ -9926,6 +10321,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q109" t="inlineStr">
         <is>
           <t>self</t>
@@ -10026,6 +10426,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q110" t="inlineStr">
         <is>
           <t>self</t>
@@ -10114,6 +10519,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q111" t="inlineStr">
         <is>
           <t>self</t>
@@ -10197,6 +10607,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q112" t="inlineStr">
         <is>
           <t>self</t>
@@ -10282,6 +10697,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q113" t="inlineStr">
         <is>
           <t>self</t>
@@ -10372,6 +10792,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q114" t="inlineStr">
         <is>
           <t>self</t>
@@ -10542,6 +10967,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q116" t="inlineStr">
         <is>
           <t>self</t>
@@ -10642,6 +11072,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q117" t="inlineStr">
         <is>
           <t>self</t>
@@ -10747,6 +11182,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q118" t="inlineStr">
         <is>
           <t>self</t>
@@ -10847,6 +11287,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q119" t="inlineStr">
         <is>
           <t>self</t>
@@ -10945,6 +11390,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q120" t="inlineStr">
         <is>
           <t>self</t>
@@ -11033,6 +11483,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q121" t="inlineStr">
         <is>
           <t>self</t>
@@ -11113,6 +11568,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q122" t="inlineStr">
         <is>
           <t>self</t>
@@ -11193,6 +11653,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q123" t="inlineStr">
         <is>
           <t>self</t>
@@ -11273,6 +11738,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q124" t="inlineStr">
         <is>
           <t>self</t>
@@ -11438,6 +11908,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q126" t="inlineStr">
         <is>
           <t>self</t>
@@ -11543,6 +12018,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q127" t="inlineStr">
         <is>
           <t>self</t>
@@ -11631,6 +12111,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q128" t="inlineStr">
         <is>
           <t>self</t>
@@ -11726,6 +12211,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q129" t="inlineStr">
         <is>
           <t>self</t>
@@ -11809,6 +12299,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q130" t="inlineStr">
         <is>
           <t>self</t>
@@ -11892,6 +12387,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q131" t="inlineStr">
         <is>
           <t>self</t>
@@ -11975,6 +12475,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q132" t="inlineStr">
         <is>
           <t>self</t>
@@ -12060,6 +12565,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q133" t="inlineStr">
         <is>
           <t>self</t>
@@ -12148,6 +12658,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q134" t="inlineStr">
         <is>
           <t>self</t>
@@ -12241,6 +12756,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q135" t="inlineStr">
         <is>
           <t>self</t>
@@ -12339,6 +12859,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q136" t="inlineStr">
         <is>
           <t>self</t>
@@ -12427,6 +12952,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q137" t="inlineStr">
         <is>
           <t>self</t>
@@ -12507,6 +13037,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q138" t="inlineStr">
         <is>
           <t>self</t>
@@ -12587,6 +13122,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q139" t="inlineStr">
         <is>
           <t>self</t>
@@ -12747,6 +13287,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q141" t="inlineStr">
         <is>
           <t>self</t>
@@ -12827,6 +13372,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q142" t="inlineStr">
         <is>
           <t>self</t>
@@ -12912,6 +13462,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q143" t="inlineStr">
         <is>
           <t>self</t>
@@ -13007,6 +13562,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q144" t="inlineStr">
         <is>
           <t>self</t>
@@ -13087,6 +13647,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q145" t="inlineStr">
         <is>
           <t>self</t>
@@ -13167,6 +13732,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q146" t="inlineStr">
         <is>
           <t>self</t>
@@ -13252,6 +13822,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q147" t="inlineStr">
         <is>
           <t>self</t>
@@ -13347,6 +13922,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q148" t="inlineStr">
         <is>
           <t>self</t>
@@ -13427,6 +14007,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q149" t="inlineStr">
         <is>
           <t>self</t>
@@ -13507,6 +14092,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q150" t="inlineStr">
         <is>
           <t>self</t>
@@ -13587,6 +14177,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q151" t="inlineStr">
         <is>
           <t>self</t>
@@ -13667,6 +14262,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q152" t="inlineStr">
         <is>
           <t>self</t>
@@ -13747,6 +14347,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q153" t="inlineStr">
         <is>
           <t>self</t>
@@ -13827,6 +14432,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q154" t="inlineStr">
         <is>
           <t>self</t>
@@ -13907,6 +14517,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q155" t="inlineStr">
         <is>
           <t>self</t>
@@ -13987,6 +14602,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q156" t="inlineStr">
         <is>
           <t>self</t>
@@ -14067,6 +14687,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q157" t="inlineStr">
         <is>
           <t>self</t>
@@ -14147,6 +14772,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q158" t="inlineStr">
         <is>
           <t>self</t>
@@ -14227,6 +14857,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q159" t="inlineStr">
         <is>
           <t>self</t>
@@ -14312,6 +14947,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q160" t="inlineStr">
         <is>
           <t>self</t>
@@ -14412,6 +15052,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q161" t="inlineStr">
         <is>
           <t>self</t>
@@ -14512,6 +15157,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q162" t="inlineStr">
         <is>
           <t>self</t>
@@ -14607,6 +15257,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q163" t="inlineStr">
         <is>
           <t>self</t>
@@ -14767,6 +15422,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q165" t="inlineStr">
         <is>
           <t>self</t>
@@ -14847,6 +15507,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q166" t="inlineStr">
         <is>
           <t>self</t>
@@ -14932,6 +15597,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q167" t="inlineStr">
         <is>
           <t>self</t>
@@ -15017,6 +15687,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q168" t="inlineStr">
         <is>
           <t>self</t>
@@ -15102,6 +15777,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q169" t="inlineStr">
         <is>
           <t>self</t>
@@ -15187,6 +15867,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q170" t="inlineStr">
         <is>
           <t>self</t>
@@ -15272,6 +15957,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q171" t="inlineStr">
         <is>
           <t>self</t>
@@ -15357,6 +16047,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q172" t="inlineStr">
         <is>
           <t>self</t>
@@ -15442,6 +16137,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q173" t="inlineStr">
         <is>
           <t>self</t>
@@ -15527,6 +16227,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q174" t="inlineStr">
         <is>
           <t>self</t>
@@ -15612,6 +16317,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q175" t="inlineStr">
         <is>
           <t>self</t>
@@ -15697,6 +16407,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q176" t="inlineStr">
         <is>
           <t>self</t>
@@ -15782,6 +16497,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q177" t="inlineStr">
         <is>
           <t>self</t>
@@ -15867,6 +16587,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q178" t="inlineStr">
         <is>
           <t>self</t>
@@ -15952,6 +16677,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q179" t="inlineStr">
         <is>
           <t>self</t>
@@ -16042,6 +16772,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q180" t="inlineStr">
         <is>
           <t>self</t>
@@ -16132,6 +16867,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q181" t="inlineStr">
         <is>
           <t>self</t>
@@ -16222,6 +16962,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q182" t="inlineStr">
         <is>
           <t>self</t>
@@ -16322,6 +17067,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q183" t="inlineStr">
         <is>
           <t>self</t>
@@ -16402,6 +17152,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q184" t="inlineStr">
         <is>
           <t>self</t>
@@ -16487,6 +17242,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q185" t="inlineStr">
         <is>
           <t>self</t>
@@ -16570,6 +17330,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q186" t="inlineStr">
         <is>
           <t>self</t>
@@ -16650,6 +17415,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q187" t="inlineStr">
         <is>
           <t>self</t>
@@ -16810,6 +17580,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q189" t="inlineStr">
         <is>
           <t>self</t>
@@ -16895,6 +17670,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q190" t="inlineStr">
         <is>
           <t>self</t>
@@ -16985,6 +17765,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q191" t="inlineStr">
         <is>
           <t>self</t>
@@ -17075,6 +17860,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q192" t="inlineStr">
         <is>
           <t>self</t>
@@ -17165,6 +17955,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q193" t="inlineStr">
         <is>
           <t>self</t>
@@ -17255,6 +18050,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q194" t="inlineStr">
         <is>
           <t>self</t>
@@ -17345,6 +18145,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q195" t="inlineStr">
         <is>
           <t>self</t>
@@ -17435,6 +18240,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q196" t="inlineStr">
         <is>
           <t>self</t>
@@ -17525,6 +18335,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q197" t="inlineStr">
         <is>
           <t>self</t>
@@ -17615,6 +18430,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q198" t="inlineStr">
         <is>
           <t>self</t>
@@ -17705,6 +18525,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q199" t="inlineStr">
         <is>
           <t>self</t>
@@ -17790,6 +18615,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q200" t="inlineStr">
         <is>
           <t>self</t>
@@ -17955,6 +18785,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q202" t="inlineStr">
         <is>
           <t>self</t>
@@ -18045,6 +18880,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q203" t="inlineStr">
         <is>
           <t>self</t>
@@ -18135,6 +18975,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q204" t="inlineStr">
         <is>
           <t>self</t>
@@ -18225,6 +19070,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q205" t="inlineStr">
         <is>
           <t>self</t>
@@ -18315,6 +19165,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q206" t="inlineStr">
         <is>
           <t>self</t>
@@ -18400,6 +19255,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q207" t="inlineStr">
         <is>
           <t>self</t>
@@ -18480,6 +19340,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q208" t="inlineStr">
         <is>
           <t>self</t>
@@ -18560,6 +19425,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q209" t="inlineStr">
         <is>
           <t>self</t>
@@ -18730,6 +19600,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q211" t="inlineStr">
         <is>
           <t>self</t>
@@ -18820,6 +19695,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q212" t="inlineStr">
         <is>
           <t>self</t>
@@ -18900,6 +19780,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q213" t="inlineStr">
         <is>
           <t>self</t>
@@ -18980,6 +19865,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q214" t="inlineStr">
         <is>
           <t>self</t>
@@ -19060,6 +19950,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q215" t="inlineStr">
         <is>
           <t>self</t>
@@ -19150,6 +20045,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q216" t="inlineStr">
         <is>
           <t>self</t>
@@ -19245,6 +20145,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q217" t="inlineStr">
         <is>
           <t>self</t>
@@ -19343,6 +20248,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q218" t="inlineStr">
         <is>
           <t>self</t>
@@ -19436,6 +20346,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q219" t="inlineStr">
         <is>
           <t>self</t>
@@ -19536,6 +20451,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q220" t="inlineStr">
         <is>
           <t>self</t>
@@ -19619,6 +20539,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q221" t="inlineStr">
         <is>
           <t>self</t>
@@ -19704,6 +20629,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q222" t="inlineStr">
         <is>
           <t>self</t>
@@ -19794,6 +20724,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q223" t="inlineStr">
         <is>
           <t>self</t>
@@ -19884,6 +20819,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q224" t="inlineStr">
         <is>
           <t>self</t>
@@ -19974,6 +20914,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q225" t="inlineStr">
         <is>
           <t>self</t>
@@ -20064,6 +21009,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q226" t="inlineStr">
         <is>
           <t>self</t>
@@ -20154,6 +21104,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q227" t="inlineStr">
         <is>
           <t>self</t>
@@ -20244,6 +21199,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q228" t="inlineStr">
         <is>
           <t>self</t>
@@ -20334,6 +21294,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q229" t="inlineStr">
         <is>
           <t>self</t>
@@ -20424,6 +21389,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q230" t="inlineStr">
         <is>
           <t>self</t>
@@ -20514,6 +21484,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q231" t="inlineStr">
         <is>
           <t>self</t>
@@ -20594,6 +21569,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q232" t="inlineStr">
         <is>
           <t>self</t>
@@ -20684,6 +21664,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q233" t="inlineStr">
         <is>
           <t>self</t>
@@ -20782,6 +21767,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q234" t="inlineStr">
         <is>
           <t>self</t>
@@ -20880,6 +21870,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q235" t="inlineStr">
         <is>
           <t>self</t>
@@ -20973,6 +21968,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q236" t="inlineStr">
         <is>
           <t>self</t>
@@ -21063,6 +22063,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q237" t="inlineStr">
         <is>
           <t>self</t>
@@ -21163,6 +22168,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q238" t="inlineStr">
         <is>
           <t>self</t>
@@ -21263,6 +22273,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q239" t="inlineStr">
         <is>
           <t>self</t>
@@ -21363,6 +22378,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q240" t="inlineStr">
         <is>
           <t>self</t>
@@ -21463,6 +22483,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q241" t="inlineStr">
         <is>
           <t>self</t>
@@ -21568,6 +22593,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q242" t="inlineStr">
         <is>
           <t>self</t>
@@ -21666,6 +22696,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q243" t="inlineStr">
         <is>
           <t>self</t>
@@ -21761,6 +22796,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q244" t="inlineStr">
         <is>
           <t>self</t>
@@ -21861,6 +22901,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q245" t="inlineStr">
         <is>
           <t>self</t>
@@ -21961,6 +23006,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q246" t="inlineStr">
         <is>
           <t>self</t>
@@ -22051,6 +23101,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q247" t="inlineStr">
         <is>
           <t>self</t>
@@ -22141,6 +23196,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q248" t="inlineStr">
         <is>
           <t>self</t>
@@ -22229,6 +23289,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q249" t="inlineStr">
         <is>
           <t>self</t>
@@ -22314,6 +23379,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q250" t="inlineStr">
         <is>
           <t>self</t>
@@ -22397,6 +23467,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q251" t="inlineStr">
         <is>
           <t>self</t>
@@ -22477,6 +23552,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q252" t="inlineStr">
         <is>
           <t>self</t>
@@ -22557,6 +23637,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q253" t="inlineStr">
         <is>
           <t>self</t>
@@ -22637,6 +23722,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q254" t="inlineStr">
         <is>
           <t>self</t>
@@ -22717,6 +23807,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q255" t="inlineStr">
         <is>
           <t>self</t>
@@ -22797,6 +23892,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q256" t="inlineStr">
         <is>
           <t>self</t>
@@ -22882,6 +23982,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q257" t="inlineStr">
         <is>
           <t>self</t>
@@ -22967,6 +24072,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q258" t="inlineStr">
         <is>
           <t>self</t>
@@ -23052,6 +24162,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q259" t="inlineStr">
         <is>
           <t>self</t>
@@ -23132,6 +24247,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q260" t="inlineStr">
         <is>
           <t>self</t>
@@ -23212,6 +24332,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q261" t="inlineStr">
         <is>
           <t>self</t>
@@ -23287,6 +24412,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O262" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q262" t="inlineStr">
         <is>
           <t>self</t>
@@ -23367,6 +24497,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q263" t="inlineStr">
         <is>
           <t>self</t>
@@ -23442,6 +24577,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q264" t="inlineStr">
         <is>
           <t>self</t>
@@ -23517,6 +24657,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q265" t="inlineStr">
         <is>
           <t>self</t>
@@ -23597,6 +24742,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q266" t="inlineStr">
         <is>
           <t>self</t>
@@ -23677,6 +24827,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q267" t="inlineStr">
         <is>
           <t>self</t>
@@ -23757,6 +24912,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q268" t="inlineStr">
         <is>
           <t>self</t>
@@ -23832,6 +24992,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q269" t="inlineStr">
         <is>
           <t>self</t>
@@ -23912,6 +25077,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q270" t="inlineStr">
         <is>
           <t>self</t>
@@ -23997,6 +25167,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q271" t="inlineStr">
         <is>
           <t>self</t>
@@ -24087,6 +25262,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q272" t="inlineStr">
         <is>
           <t>self</t>
@@ -24182,6 +25362,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="R273" t="inlineStr">
         <is>
           <t>live</t>
@@ -24373,6 +25558,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="R275" t="inlineStr">
         <is>
           <t>live</t>
@@ -24647,6 +25837,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q278" t="inlineStr">
         <is>
           <t>self</t>
@@ -24750,6 +25945,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="Q279" t="inlineStr">
         <is>
           <t>self</t>
@@ -25069,6 +26269,11 @@
           <t>licht</t>
         </is>
       </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
+        </is>
+      </c>
       <c r="P282" t="inlineStr">
         <is>
           <t>auto</t>
@@ -25150,7 +26355,6 @@
           <t>nederland-kompleet/werkloosheid-officieel-versus-reeel.html</t>
         </is>
       </c>
-      <c r="J283" t="inlineStr"/>
       <c r="K283" t="inlineStr">
         <is>
           <t>center</t>
@@ -25169,6 +26373,11 @@
       <c r="N283" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P283" t="inlineStr">
@@ -25252,7 +26461,6 @@
           <t>nederland-kompleet/duitse-industrie-cascade.html</t>
         </is>
       </c>
-      <c r="J284" t="inlineStr"/>
       <c r="K284" t="inlineStr">
         <is>
           <t>center</t>
@@ -25271,6 +26479,11 @@
       <c r="N284" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P284" t="inlineStr">
@@ -25354,7 +26567,6 @@
           <t>nederland-kompleet/nederlandse-industrie-cascade.html</t>
         </is>
       </c>
-      <c r="J285" t="inlineStr"/>
       <c r="K285" t="inlineStr">
         <is>
           <t>center</t>
@@ -25373,6 +26585,11 @@
       <c r="N285" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P285" t="inlineStr">
@@ -25456,7 +26673,6 @@
           <t>nederland-kompleet/multiplicator-effect-banen.html</t>
         </is>
       </c>
-      <c r="J286" t="inlineStr"/>
       <c r="K286" t="inlineStr">
         <is>
           <t>center</t>
@@ -25475,6 +26691,11 @@
       <c r="N286" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P286" t="inlineStr">
@@ -25558,7 +26779,6 @@
           <t>nederland-kompleet/rotterdam-doorvoer.html</t>
         </is>
       </c>
-      <c r="J287" t="inlineStr"/>
       <c r="K287" t="inlineStr">
         <is>
           <t>center</t>
@@ -25577,6 +26797,11 @@
       <c r="N287" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P287" t="inlineStr">
@@ -25660,7 +26885,6 @@
           <t>nederland-kompleet/kvk-stoppers-versnelling.html</t>
         </is>
       </c>
-      <c r="J288" t="inlineStr"/>
       <c r="K288" t="inlineStr">
         <is>
           <t>center</t>
@@ -25679,6 +26903,11 @@
       <c r="N288" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P288" t="inlineStr">
@@ -25762,7 +26991,6 @@
           <t>nederland-kompleet/ebitda-multiple-collaps.html</t>
         </is>
       </c>
-      <c r="J289" t="inlineStr"/>
       <c r="K289" t="inlineStr">
         <is>
           <t>center</t>
@@ -25781,6 +27009,11 @@
       <c r="N289" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P289" t="inlineStr">
@@ -25864,7 +27097,6 @@
           <t>nederland-kompleet/middenstand-exit-realisatie.html</t>
         </is>
       </c>
-      <c r="J290" t="inlineStr"/>
       <c r="K290" t="inlineStr">
         <is>
           <t>center</t>
@@ -25883,6 +27115,11 @@
       <c r="N290" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P290" t="inlineStr">
@@ -25966,7 +27203,6 @@
           <t>nederland-kompleet/jachtwerven-cascade.html</t>
         </is>
       </c>
-      <c r="J291" t="inlineStr"/>
       <c r="K291" t="inlineStr">
         <is>
           <t>center</t>
@@ -25985,6 +27221,11 @@
       <c r="N291" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P291" t="inlineStr">
@@ -26068,7 +27309,6 @@
           <t>nederland-kompleet/balans-fictie-mkb.html</t>
         </is>
       </c>
-      <c r="J292" t="inlineStr"/>
       <c r="K292" t="inlineStr">
         <is>
           <t>center</t>
@@ -26087,6 +27327,11 @@
       <c r="N292" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P292" t="inlineStr">
@@ -26170,7 +27415,6 @@
           <t>nederland-kompleet/consumentenvertrouwen.html</t>
         </is>
       </c>
-      <c r="J293" t="inlineStr"/>
       <c r="K293" t="inlineStr">
         <is>
           <t>center</t>
@@ -26189,6 +27433,11 @@
       <c r="N293" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P293" t="inlineStr">
@@ -26272,7 +27521,6 @@
           <t>nederland-kompleet/premium-auto-bpm.html</t>
         </is>
       </c>
-      <c r="J294" t="inlineStr"/>
       <c r="K294" t="inlineStr">
         <is>
           <t>center</t>
@@ -26291,6 +27539,11 @@
       <c r="N294" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P294" t="inlineStr">
@@ -26374,7 +27627,6 @@
           <t>nederland-kompleet/superjachten-tweedeling.html</t>
         </is>
       </c>
-      <c r="J295" t="inlineStr"/>
       <c r="K295" t="inlineStr">
         <is>
           <t>center</t>
@@ -26393,6 +27645,11 @@
       <c r="N295" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P295" t="inlineStr">
@@ -26476,7 +27733,6 @@
           <t>nederland-kompleet/eu-fertiliteit.html</t>
         </is>
       </c>
-      <c r="J296" t="inlineStr"/>
       <c r="K296" t="inlineStr">
         <is>
           <t>center</t>
@@ -26495,6 +27751,11 @@
       <c r="N296" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P296" t="inlineStr">
@@ -26578,7 +27839,6 @@
           <t>nederland-kompleet/nl-tfr.html</t>
         </is>
       </c>
-      <c r="J297" t="inlineStr"/>
       <c r="K297" t="inlineStr">
         <is>
           <t>center</t>
@@ -26597,6 +27857,11 @@
       <c r="N297" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P297" t="inlineStr">
@@ -26680,7 +27945,6 @@
           <t>nederland-kompleet/eu-populatie-2100.html</t>
         </is>
       </c>
-      <c r="J298" t="inlineStr"/>
       <c r="K298" t="inlineStr">
         <is>
           <t>center</t>
@@ -26699,6 +27963,11 @@
       <c r="N298" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P298" t="inlineStr">
@@ -26782,7 +28051,6 @@
           <t>nederland-kompleet/zeespiegel-deltaplan.html</t>
         </is>
       </c>
-      <c r="J299" t="inlineStr"/>
       <c r="K299" t="inlineStr">
         <is>
           <t>center</t>
@@ -26801,6 +28069,11 @@
       <c r="N299" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P299" t="inlineStr">
@@ -26884,7 +28157,6 @@
           <t>nederland-kompleet/rws-prorail-onderhoud.html</t>
         </is>
       </c>
-      <c r="J300" t="inlineStr"/>
       <c r="K300" t="inlineStr">
         <is>
           <t>center</t>
@@ -26903,6 +28175,11 @@
       <c r="N300" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P300" t="inlineStr">
@@ -26986,7 +28263,6 @@
           <t>nederland-kompleet/eu-bosbranden-klimaatschade.html</t>
         </is>
       </c>
-      <c r="J301" t="inlineStr"/>
       <c r="K301" t="inlineStr">
         <is>
           <t>center</t>
@@ -27005,6 +28281,11 @@
       <c r="N301" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P301" t="inlineStr">
@@ -27088,7 +28369,6 @@
           <t>nederland-kompleet/rijn-waterstand.html</t>
         </is>
       </c>
-      <c r="J302" t="inlineStr"/>
       <c r="K302" t="inlineStr">
         <is>
           <t>center</t>
@@ -27107,6 +28387,11 @@
       <c r="N302" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P302" t="inlineStr">
@@ -27190,7 +28475,6 @@
           <t>nederland-kompleet/ai-disruptie.html</t>
         </is>
       </c>
-      <c r="J303" t="inlineStr"/>
       <c r="K303" t="inlineStr">
         <is>
           <t>center</t>
@@ -27209,6 +28493,11 @@
       <c r="N303" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P303" t="inlineStr">
@@ -27292,7 +28581,6 @@
           <t>nederland-kompleet/asielkosten-nl.html</t>
         </is>
       </c>
-      <c r="J304" t="inlineStr"/>
       <c r="K304" t="inlineStr">
         <is>
           <t>center</t>
@@ -27311,6 +28599,11 @@
       <c r="N304" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P304" t="inlineStr">
@@ -27394,7 +28687,6 @@
           <t>nederland-kompleet/kinderopvang-bovenmatig.html</t>
         </is>
       </c>
-      <c r="J305" t="inlineStr"/>
       <c r="K305" t="inlineStr">
         <is>
           <t>center</t>
@@ -27413,6 +28705,11 @@
       <c r="N305" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P305" t="inlineStr">
@@ -27496,7 +28793,6 @@
           <t>nederland-kompleet/vrachtauto-elektrificatie.html</t>
         </is>
       </c>
-      <c r="J306" t="inlineStr"/>
       <c r="K306" t="inlineStr">
         <is>
           <t>center</t>
@@ -27515,6 +28811,11 @@
       <c r="N306" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P306" t="inlineStr">
@@ -27598,7 +28899,6 @@
           <t>nederland-kompleet/groningen-gas.html</t>
         </is>
       </c>
-      <c r="J307" t="inlineStr"/>
       <c r="K307" t="inlineStr">
         <is>
           <t>center</t>
@@ -27617,6 +28917,11 @@
       <c r="N307" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P307" t="inlineStr">
@@ -27700,7 +29005,6 @@
           <t>nederland-kompleet/miljonair-migratie.html</t>
         </is>
       </c>
-      <c r="J308" t="inlineStr"/>
       <c r="K308" t="inlineStr">
         <is>
           <t>center</t>
@@ -27719,6 +29023,11 @@
       <c r="N308" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P308" t="inlineStr">
@@ -27802,7 +29111,6 @@
           <t>nederland-kompleet/eu-werkloosheid-buren.html</t>
         </is>
       </c>
-      <c r="J309" t="inlineStr"/>
       <c r="K309" t="inlineStr">
         <is>
           <t>center</t>
@@ -27821,6 +29129,11 @@
       <c r="N309" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P309" t="inlineStr">
@@ -27904,7 +29217,6 @@
           <t>nederland-kompleet/schiphol-krimp.html</t>
         </is>
       </c>
-      <c r="J310" t="inlineStr"/>
       <c r="K310" t="inlineStr">
         <is>
           <t>center</t>
@@ -27923,6 +29235,11 @@
       <c r="N310" t="inlineStr">
         <is>
           <t>licht</t>
+        </is>
+      </c>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="P310" t="inlineStr">

</xml_diff>

<commit_message>
xlsx: revert 'Terug naar' bulk-toevoegingen (commit 02db610c)
Verkeerde interpretatie van veld 'Terug naar'. Uit Kolommen-tabblad van vizier.xlsx:
   'terug_naar | Terug naar | Code; leeg = automatisch naar ouder'

Leeg BETEKENT dus 'automatisch naar de ouder'. Mijn commit 02db610c vulde alle
lege velden met '1.1.1' (voorpagina), wat de automatische ouder-terugval brak.

Deze commit haalt de 269 '1.1.1'-waardes weer weg. De 4 rijen die u zelf al had
ingevuld (1.3.2.11, 1.4.5.1.1, 1.1.1.21, 1.1.1.22) blijven ongewijzigd.
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -1680,11 +1680,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q15" t="inlineStr">
         <is>
           <t>self</t>
@@ -1860,11 +1855,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q17" t="inlineStr">
         <is>
           <t>self</t>
@@ -1960,11 +1950,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q18" t="inlineStr">
         <is>
           <t>self</t>
@@ -2063,11 +2048,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q19" t="inlineStr">
         <is>
           <t>self</t>
@@ -2166,11 +2146,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q20" t="inlineStr">
         <is>
           <t>self</t>
@@ -2346,11 +2321,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q22" t="inlineStr">
         <is>
           <t>self</t>
@@ -2451,11 +2421,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q23" t="inlineStr">
         <is>
           <t>self</t>
@@ -2544,11 +2509,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q24" t="inlineStr">
         <is>
           <t>self</t>
@@ -2632,11 +2592,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q25" t="inlineStr">
         <is>
           <t>self</t>
@@ -2727,11 +2682,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q26" t="inlineStr">
         <is>
           <t>self</t>
@@ -2902,11 +2852,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q28" t="inlineStr">
         <is>
           <t>self</t>
@@ -2992,11 +2937,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q29" t="inlineStr">
         <is>
           <t>self</t>
@@ -3082,11 +3022,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q30" t="inlineStr">
         <is>
           <t>self</t>
@@ -3172,11 +3107,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q31" t="inlineStr">
         <is>
           <t>self</t>
@@ -3262,11 +3192,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q32" t="inlineStr">
         <is>
           <t>self</t>
@@ -3357,11 +3282,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q33" t="inlineStr">
         <is>
           <t>self</t>
@@ -3547,11 +3467,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q35" t="inlineStr">
         <is>
           <t>self</t>
@@ -3650,11 +3565,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q36" t="inlineStr">
         <is>
           <t>self</t>
@@ -3748,11 +3658,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q37" t="inlineStr">
         <is>
           <t>self</t>
@@ -3848,11 +3753,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q38" t="inlineStr">
         <is>
           <t>self</t>
@@ -3938,11 +3838,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q39" t="inlineStr">
         <is>
           <t>self</t>
@@ -4026,11 +3921,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q40" t="inlineStr">
         <is>
           <t>self</t>
@@ -4119,11 +4009,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q41" t="inlineStr">
         <is>
           <t>self</t>
@@ -4287,11 +4172,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q43" t="inlineStr">
         <is>
           <t>self</t>
@@ -4382,11 +4262,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q44" t="inlineStr">
         <is>
           <t>self</t>
@@ -4485,11 +4360,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q45" t="inlineStr">
         <is>
           <t>self</t>
@@ -4583,11 +4453,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q46" t="inlineStr">
         <is>
           <t>self</t>
@@ -4676,11 +4541,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q47" t="inlineStr">
         <is>
           <t>self</t>
@@ -4781,11 +4641,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q48" t="inlineStr">
         <is>
           <t>self</t>
@@ -4876,11 +4731,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q49" t="inlineStr">
         <is>
           <t>self</t>
@@ -4976,11 +4826,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q50" t="inlineStr">
         <is>
           <t>self</t>
@@ -5159,11 +5004,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q52" t="inlineStr">
         <is>
           <t>self</t>
@@ -5262,11 +5102,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q53" t="inlineStr">
         <is>
           <t>self</t>
@@ -5355,11 +5190,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q54" t="inlineStr">
         <is>
           <t>self</t>
@@ -5450,11 +5280,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q55" t="inlineStr">
         <is>
           <t>self</t>
@@ -5545,11 +5370,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O56" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q56" t="inlineStr">
         <is>
           <t>self</t>
@@ -5640,11 +5460,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O57" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q57" t="inlineStr">
         <is>
           <t>self</t>
@@ -5815,11 +5630,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O59" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q59" t="inlineStr">
         <is>
           <t>self</t>
@@ -5910,11 +5720,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O60" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q60" t="inlineStr">
         <is>
           <t>self</t>
@@ -6005,11 +5810,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O61" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q61" t="inlineStr">
         <is>
           <t>self</t>
@@ -6100,11 +5900,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q62" t="inlineStr">
         <is>
           <t>self</t>
@@ -6195,11 +5990,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O63" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q63" t="inlineStr">
         <is>
           <t>self</t>
@@ -6290,11 +6080,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O64" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q64" t="inlineStr">
         <is>
           <t>self</t>
@@ -6385,11 +6170,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O65" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q65" t="inlineStr">
         <is>
           <t>self</t>
@@ -6475,11 +6255,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O66" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q66" t="inlineStr">
         <is>
           <t>self</t>
@@ -6565,11 +6340,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O67" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q67" t="inlineStr">
         <is>
           <t>self</t>
@@ -6670,11 +6440,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O68" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q68" t="inlineStr">
         <is>
           <t>self</t>
@@ -6840,11 +6605,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O70" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q70" t="inlineStr">
         <is>
           <t>self</t>
@@ -6925,11 +6685,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O71" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q71" t="inlineStr">
         <is>
           <t>self</t>
@@ -7010,11 +6765,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O72" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q72" t="inlineStr">
         <is>
           <t>self</t>
@@ -7095,11 +6845,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O73" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q73" t="inlineStr">
         <is>
           <t>self</t>
@@ -7180,11 +6925,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O74" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q74" t="inlineStr">
         <is>
           <t>self</t>
@@ -7345,11 +7085,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O76" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q76" t="inlineStr">
         <is>
           <t>self</t>
@@ -7430,11 +7165,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O77" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q77" t="inlineStr">
         <is>
           <t>self</t>
@@ -7515,11 +7245,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O78" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q78" t="inlineStr">
         <is>
           <t>self</t>
@@ -7600,11 +7325,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O79" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q79" t="inlineStr">
         <is>
           <t>self</t>
@@ -7775,11 +7495,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O81" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q81" t="inlineStr">
         <is>
           <t>self</t>
@@ -7878,11 +7593,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O82" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q82" t="inlineStr">
         <is>
           <t>self</t>
@@ -7981,11 +7691,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O83" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q83" t="inlineStr">
         <is>
           <t>self</t>
@@ -8161,11 +7866,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O85" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q85" t="inlineStr">
         <is>
           <t>self</t>
@@ -8254,11 +7954,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O86" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q86" t="inlineStr">
         <is>
           <t>self</t>
@@ -8364,11 +8059,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O87" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q87" t="inlineStr">
         <is>
           <t>self</t>
@@ -8457,11 +8147,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O88" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q88" t="inlineStr">
         <is>
           <t>self</t>
@@ -8542,11 +8227,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O89" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q89" t="inlineStr">
         <is>
           <t>self</t>
@@ -8627,11 +8307,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O90" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q90" t="inlineStr">
         <is>
           <t>self</t>
@@ -8797,11 +8472,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O92" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q92" t="inlineStr">
         <is>
           <t>self</t>
@@ -8892,11 +8562,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O93" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q93" t="inlineStr">
         <is>
           <t>self</t>
@@ -8987,11 +8652,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O94" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q94" t="inlineStr">
         <is>
           <t>self</t>
@@ -9082,11 +8742,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O95" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q95" t="inlineStr">
         <is>
           <t>self</t>
@@ -9255,11 +8910,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O97" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q97" t="inlineStr">
         <is>
           <t>self</t>
@@ -9355,11 +9005,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O98" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q98" t="inlineStr">
         <is>
           <t>self</t>
@@ -9448,11 +9093,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O99" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q99" t="inlineStr">
         <is>
           <t>self</t>
@@ -9628,11 +9268,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O101" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q101" t="inlineStr">
         <is>
           <t>self</t>
@@ -9713,11 +9348,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O102" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q102" t="inlineStr">
         <is>
           <t>self</t>
@@ -9798,11 +9428,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O103" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q103" t="inlineStr">
         <is>
           <t>self</t>
@@ -9883,11 +9508,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O104" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q104" t="inlineStr">
         <is>
           <t>self</t>
@@ -9968,11 +9588,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O105" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q105" t="inlineStr">
         <is>
           <t>self</t>
@@ -10138,11 +9753,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O107" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q107" t="inlineStr">
         <is>
           <t>self</t>
@@ -10226,11 +9836,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O108" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q108" t="inlineStr">
         <is>
           <t>self</t>
@@ -10321,11 +9926,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O109" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q109" t="inlineStr">
         <is>
           <t>self</t>
@@ -10426,11 +10026,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O110" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q110" t="inlineStr">
         <is>
           <t>self</t>
@@ -10519,11 +10114,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O111" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q111" t="inlineStr">
         <is>
           <t>self</t>
@@ -10607,11 +10197,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O112" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q112" t="inlineStr">
         <is>
           <t>self</t>
@@ -10697,11 +10282,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O113" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q113" t="inlineStr">
         <is>
           <t>self</t>
@@ -10792,11 +10372,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O114" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q114" t="inlineStr">
         <is>
           <t>self</t>
@@ -10967,11 +10542,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O116" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q116" t="inlineStr">
         <is>
           <t>self</t>
@@ -11072,11 +10642,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O117" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q117" t="inlineStr">
         <is>
           <t>self</t>
@@ -11182,11 +10747,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O118" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q118" t="inlineStr">
         <is>
           <t>self</t>
@@ -11287,11 +10847,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O119" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q119" t="inlineStr">
         <is>
           <t>self</t>
@@ -11390,11 +10945,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O120" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q120" t="inlineStr">
         <is>
           <t>self</t>
@@ -11483,11 +11033,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O121" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q121" t="inlineStr">
         <is>
           <t>self</t>
@@ -11568,11 +11113,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O122" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q122" t="inlineStr">
         <is>
           <t>self</t>
@@ -11653,11 +11193,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O123" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q123" t="inlineStr">
         <is>
           <t>self</t>
@@ -11738,11 +11273,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O124" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q124" t="inlineStr">
         <is>
           <t>self</t>
@@ -11908,11 +11438,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O126" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q126" t="inlineStr">
         <is>
           <t>self</t>
@@ -12018,11 +11543,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O127" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q127" t="inlineStr">
         <is>
           <t>self</t>
@@ -12111,11 +11631,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O128" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q128" t="inlineStr">
         <is>
           <t>self</t>
@@ -12211,11 +11726,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O129" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q129" t="inlineStr">
         <is>
           <t>self</t>
@@ -12299,11 +11809,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O130" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q130" t="inlineStr">
         <is>
           <t>self</t>
@@ -12387,11 +11892,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O131" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q131" t="inlineStr">
         <is>
           <t>self</t>
@@ -12475,11 +11975,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O132" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q132" t="inlineStr">
         <is>
           <t>self</t>
@@ -12565,11 +12060,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O133" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q133" t="inlineStr">
         <is>
           <t>self</t>
@@ -12658,11 +12148,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O134" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q134" t="inlineStr">
         <is>
           <t>self</t>
@@ -12756,11 +12241,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O135" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q135" t="inlineStr">
         <is>
           <t>self</t>
@@ -12859,11 +12339,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O136" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q136" t="inlineStr">
         <is>
           <t>self</t>
@@ -12952,11 +12427,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O137" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q137" t="inlineStr">
         <is>
           <t>self</t>
@@ -13037,11 +12507,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O138" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q138" t="inlineStr">
         <is>
           <t>self</t>
@@ -13122,11 +12587,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O139" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q139" t="inlineStr">
         <is>
           <t>self</t>
@@ -13287,11 +12747,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O141" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q141" t="inlineStr">
         <is>
           <t>self</t>
@@ -13372,11 +12827,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O142" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q142" t="inlineStr">
         <is>
           <t>self</t>
@@ -13462,11 +12912,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O143" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q143" t="inlineStr">
         <is>
           <t>self</t>
@@ -13562,11 +13007,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O144" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q144" t="inlineStr">
         <is>
           <t>self</t>
@@ -13647,11 +13087,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O145" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q145" t="inlineStr">
         <is>
           <t>self</t>
@@ -13732,11 +13167,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O146" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q146" t="inlineStr">
         <is>
           <t>self</t>
@@ -13822,11 +13252,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O147" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q147" t="inlineStr">
         <is>
           <t>self</t>
@@ -13922,11 +13347,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O148" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q148" t="inlineStr">
         <is>
           <t>self</t>
@@ -14007,11 +13427,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O149" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q149" t="inlineStr">
         <is>
           <t>self</t>
@@ -14092,11 +13507,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O150" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q150" t="inlineStr">
         <is>
           <t>self</t>
@@ -14177,11 +13587,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O151" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q151" t="inlineStr">
         <is>
           <t>self</t>
@@ -14262,11 +13667,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O152" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q152" t="inlineStr">
         <is>
           <t>self</t>
@@ -14347,11 +13747,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O153" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q153" t="inlineStr">
         <is>
           <t>self</t>
@@ -14432,11 +13827,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O154" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q154" t="inlineStr">
         <is>
           <t>self</t>
@@ -14517,11 +13907,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O155" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q155" t="inlineStr">
         <is>
           <t>self</t>
@@ -14602,11 +13987,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O156" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q156" t="inlineStr">
         <is>
           <t>self</t>
@@ -14687,11 +14067,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O157" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q157" t="inlineStr">
         <is>
           <t>self</t>
@@ -14772,11 +14147,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O158" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q158" t="inlineStr">
         <is>
           <t>self</t>
@@ -14857,11 +14227,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O159" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q159" t="inlineStr">
         <is>
           <t>self</t>
@@ -14947,11 +14312,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O160" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q160" t="inlineStr">
         <is>
           <t>self</t>
@@ -15052,11 +14412,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O161" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q161" t="inlineStr">
         <is>
           <t>self</t>
@@ -15157,11 +14512,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O162" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q162" t="inlineStr">
         <is>
           <t>self</t>
@@ -15257,11 +14607,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O163" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q163" t="inlineStr">
         <is>
           <t>self</t>
@@ -15422,11 +14767,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O165" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q165" t="inlineStr">
         <is>
           <t>self</t>
@@ -15507,11 +14847,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O166" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q166" t="inlineStr">
         <is>
           <t>self</t>
@@ -15597,11 +14932,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O167" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q167" t="inlineStr">
         <is>
           <t>self</t>
@@ -15687,11 +15017,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O168" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q168" t="inlineStr">
         <is>
           <t>self</t>
@@ -15777,11 +15102,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O169" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q169" t="inlineStr">
         <is>
           <t>self</t>
@@ -15867,11 +15187,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O170" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q170" t="inlineStr">
         <is>
           <t>self</t>
@@ -15957,11 +15272,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O171" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q171" t="inlineStr">
         <is>
           <t>self</t>
@@ -16047,11 +15357,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O172" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q172" t="inlineStr">
         <is>
           <t>self</t>
@@ -16137,11 +15442,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O173" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q173" t="inlineStr">
         <is>
           <t>self</t>
@@ -16227,11 +15527,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O174" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q174" t="inlineStr">
         <is>
           <t>self</t>
@@ -16317,11 +15612,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O175" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q175" t="inlineStr">
         <is>
           <t>self</t>
@@ -16407,11 +15697,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O176" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q176" t="inlineStr">
         <is>
           <t>self</t>
@@ -16497,11 +15782,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O177" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q177" t="inlineStr">
         <is>
           <t>self</t>
@@ -16587,11 +15867,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O178" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q178" t="inlineStr">
         <is>
           <t>self</t>
@@ -16677,11 +15952,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O179" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q179" t="inlineStr">
         <is>
           <t>self</t>
@@ -16772,11 +16042,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O180" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q180" t="inlineStr">
         <is>
           <t>self</t>
@@ -16867,11 +16132,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O181" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q181" t="inlineStr">
         <is>
           <t>self</t>
@@ -16962,11 +16222,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O182" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q182" t="inlineStr">
         <is>
           <t>self</t>
@@ -17067,11 +16322,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O183" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q183" t="inlineStr">
         <is>
           <t>self</t>
@@ -17152,11 +16402,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O184" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q184" t="inlineStr">
         <is>
           <t>self</t>
@@ -17242,11 +16487,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O185" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q185" t="inlineStr">
         <is>
           <t>self</t>
@@ -17330,11 +16570,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O186" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q186" t="inlineStr">
         <is>
           <t>self</t>
@@ -17415,11 +16650,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O187" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q187" t="inlineStr">
         <is>
           <t>self</t>
@@ -17580,11 +16810,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O189" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q189" t="inlineStr">
         <is>
           <t>self</t>
@@ -17670,11 +16895,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O190" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q190" t="inlineStr">
         <is>
           <t>self</t>
@@ -17765,11 +16985,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O191" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q191" t="inlineStr">
         <is>
           <t>self</t>
@@ -17860,11 +17075,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O192" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q192" t="inlineStr">
         <is>
           <t>self</t>
@@ -17955,11 +17165,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O193" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q193" t="inlineStr">
         <is>
           <t>self</t>
@@ -18050,11 +17255,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O194" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q194" t="inlineStr">
         <is>
           <t>self</t>
@@ -18145,11 +17345,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O195" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q195" t="inlineStr">
         <is>
           <t>self</t>
@@ -18240,11 +17435,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O196" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q196" t="inlineStr">
         <is>
           <t>self</t>
@@ -18335,11 +17525,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O197" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q197" t="inlineStr">
         <is>
           <t>self</t>
@@ -18430,11 +17615,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O198" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q198" t="inlineStr">
         <is>
           <t>self</t>
@@ -18525,11 +17705,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O199" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q199" t="inlineStr">
         <is>
           <t>self</t>
@@ -18615,11 +17790,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O200" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q200" t="inlineStr">
         <is>
           <t>self</t>
@@ -18785,11 +17955,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O202" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q202" t="inlineStr">
         <is>
           <t>self</t>
@@ -18880,11 +18045,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O203" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q203" t="inlineStr">
         <is>
           <t>self</t>
@@ -18975,11 +18135,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O204" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q204" t="inlineStr">
         <is>
           <t>self</t>
@@ -19070,11 +18225,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O205" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q205" t="inlineStr">
         <is>
           <t>self</t>
@@ -19165,11 +18315,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O206" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q206" t="inlineStr">
         <is>
           <t>self</t>
@@ -19255,11 +18400,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O207" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q207" t="inlineStr">
         <is>
           <t>self</t>
@@ -19340,11 +18480,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O208" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q208" t="inlineStr">
         <is>
           <t>self</t>
@@ -19425,11 +18560,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O209" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q209" t="inlineStr">
         <is>
           <t>self</t>
@@ -19600,11 +18730,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O211" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q211" t="inlineStr">
         <is>
           <t>self</t>
@@ -19695,11 +18820,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O212" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q212" t="inlineStr">
         <is>
           <t>self</t>
@@ -19780,11 +18900,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O213" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q213" t="inlineStr">
         <is>
           <t>self</t>
@@ -19865,11 +18980,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O214" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q214" t="inlineStr">
         <is>
           <t>self</t>
@@ -19950,11 +19060,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O215" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q215" t="inlineStr">
         <is>
           <t>self</t>
@@ -20045,11 +19150,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O216" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q216" t="inlineStr">
         <is>
           <t>self</t>
@@ -20145,11 +19245,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O217" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q217" t="inlineStr">
         <is>
           <t>self</t>
@@ -20248,11 +19343,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O218" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q218" t="inlineStr">
         <is>
           <t>self</t>
@@ -20346,11 +19436,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O219" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q219" t="inlineStr">
         <is>
           <t>self</t>
@@ -20451,11 +19536,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O220" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q220" t="inlineStr">
         <is>
           <t>self</t>
@@ -20539,11 +19619,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O221" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q221" t="inlineStr">
         <is>
           <t>self</t>
@@ -20629,11 +19704,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O222" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q222" t="inlineStr">
         <is>
           <t>self</t>
@@ -20724,11 +19794,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O223" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q223" t="inlineStr">
         <is>
           <t>self</t>
@@ -20819,11 +19884,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O224" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q224" t="inlineStr">
         <is>
           <t>self</t>
@@ -20914,11 +19974,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O225" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q225" t="inlineStr">
         <is>
           <t>self</t>
@@ -21009,11 +20064,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O226" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q226" t="inlineStr">
         <is>
           <t>self</t>
@@ -21104,11 +20154,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O227" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q227" t="inlineStr">
         <is>
           <t>self</t>
@@ -21199,11 +20244,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O228" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q228" t="inlineStr">
         <is>
           <t>self</t>
@@ -21294,11 +20334,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O229" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q229" t="inlineStr">
         <is>
           <t>self</t>
@@ -21389,11 +20424,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O230" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q230" t="inlineStr">
         <is>
           <t>self</t>
@@ -21484,11 +20514,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O231" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q231" t="inlineStr">
         <is>
           <t>self</t>
@@ -21569,11 +20594,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O232" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q232" t="inlineStr">
         <is>
           <t>self</t>
@@ -21664,11 +20684,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O233" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q233" t="inlineStr">
         <is>
           <t>self</t>
@@ -21767,11 +20782,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O234" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q234" t="inlineStr">
         <is>
           <t>self</t>
@@ -21870,11 +20880,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O235" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q235" t="inlineStr">
         <is>
           <t>self</t>
@@ -21968,11 +20973,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O236" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q236" t="inlineStr">
         <is>
           <t>self</t>
@@ -22063,11 +21063,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O237" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q237" t="inlineStr">
         <is>
           <t>self</t>
@@ -22168,11 +21163,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O238" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q238" t="inlineStr">
         <is>
           <t>self</t>
@@ -22273,11 +21263,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O239" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q239" t="inlineStr">
         <is>
           <t>self</t>
@@ -22378,11 +21363,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O240" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q240" t="inlineStr">
         <is>
           <t>self</t>
@@ -22483,11 +21463,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O241" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q241" t="inlineStr">
         <is>
           <t>self</t>
@@ -22593,11 +21568,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O242" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q242" t="inlineStr">
         <is>
           <t>self</t>
@@ -22696,11 +21666,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O243" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q243" t="inlineStr">
         <is>
           <t>self</t>
@@ -22796,11 +21761,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O244" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q244" t="inlineStr">
         <is>
           <t>self</t>
@@ -22901,11 +21861,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O245" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q245" t="inlineStr">
         <is>
           <t>self</t>
@@ -23006,11 +21961,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O246" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q246" t="inlineStr">
         <is>
           <t>self</t>
@@ -23101,11 +22051,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O247" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q247" t="inlineStr">
         <is>
           <t>self</t>
@@ -23196,11 +22141,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O248" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q248" t="inlineStr">
         <is>
           <t>self</t>
@@ -23289,11 +22229,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O249" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q249" t="inlineStr">
         <is>
           <t>self</t>
@@ -23379,11 +22314,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O250" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q250" t="inlineStr">
         <is>
           <t>self</t>
@@ -23467,11 +22397,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O251" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q251" t="inlineStr">
         <is>
           <t>self</t>
@@ -23552,11 +22477,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O252" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q252" t="inlineStr">
         <is>
           <t>self</t>
@@ -23637,11 +22557,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O253" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q253" t="inlineStr">
         <is>
           <t>self</t>
@@ -23722,11 +22637,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O254" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q254" t="inlineStr">
         <is>
           <t>self</t>
@@ -23807,11 +22717,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O255" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q255" t="inlineStr">
         <is>
           <t>self</t>
@@ -23892,11 +22797,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O256" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q256" t="inlineStr">
         <is>
           <t>self</t>
@@ -23982,11 +22882,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O257" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q257" t="inlineStr">
         <is>
           <t>self</t>
@@ -24072,11 +22967,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O258" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q258" t="inlineStr">
         <is>
           <t>self</t>
@@ -24162,11 +23052,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O259" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q259" t="inlineStr">
         <is>
           <t>self</t>
@@ -24247,11 +23132,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O260" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q260" t="inlineStr">
         <is>
           <t>self</t>
@@ -24332,11 +23212,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O261" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q261" t="inlineStr">
         <is>
           <t>self</t>
@@ -24412,11 +23287,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O262" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q262" t="inlineStr">
         <is>
           <t>self</t>
@@ -24497,11 +23367,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O263" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q263" t="inlineStr">
         <is>
           <t>self</t>
@@ -24577,11 +23442,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O264" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q264" t="inlineStr">
         <is>
           <t>self</t>
@@ -24657,11 +23517,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O265" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q265" t="inlineStr">
         <is>
           <t>self</t>
@@ -24742,11 +23597,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O266" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q266" t="inlineStr">
         <is>
           <t>self</t>
@@ -24827,11 +23677,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O267" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q267" t="inlineStr">
         <is>
           <t>self</t>
@@ -24912,11 +23757,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O268" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q268" t="inlineStr">
         <is>
           <t>self</t>
@@ -24992,11 +23832,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O269" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q269" t="inlineStr">
         <is>
           <t>self</t>
@@ -25077,11 +23912,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O270" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q270" t="inlineStr">
         <is>
           <t>self</t>
@@ -25167,11 +23997,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O271" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q271" t="inlineStr">
         <is>
           <t>self</t>
@@ -25262,11 +24087,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O272" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q272" t="inlineStr">
         <is>
           <t>self</t>
@@ -25362,11 +24182,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O273" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="R273" t="inlineStr">
         <is>
           <t>live</t>
@@ -25558,11 +24373,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O275" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="R275" t="inlineStr">
         <is>
           <t>live</t>
@@ -25837,11 +24647,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O278" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q278" t="inlineStr">
         <is>
           <t>self</t>
@@ -25945,11 +24750,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O279" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="Q279" t="inlineStr">
         <is>
           <t>self</t>
@@ -26269,11 +25069,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O282" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P282" t="inlineStr">
         <is>
           <t>auto</t>
@@ -26375,11 +25170,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O283" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P283" t="inlineStr">
         <is>
           <t>auto</t>
@@ -26481,11 +25271,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O284" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P284" t="inlineStr">
         <is>
           <t>auto</t>
@@ -26587,11 +25372,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O285" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P285" t="inlineStr">
         <is>
           <t>auto</t>
@@ -26693,11 +25473,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O286" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P286" t="inlineStr">
         <is>
           <t>auto</t>
@@ -26799,11 +25574,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O287" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P287" t="inlineStr">
         <is>
           <t>auto</t>
@@ -26905,11 +25675,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O288" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P288" t="inlineStr">
         <is>
           <t>auto</t>
@@ -27011,11 +25776,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O289" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P289" t="inlineStr">
         <is>
           <t>auto</t>
@@ -27117,11 +25877,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O290" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P290" t="inlineStr">
         <is>
           <t>auto</t>
@@ -27223,11 +25978,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O291" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P291" t="inlineStr">
         <is>
           <t>auto</t>
@@ -27329,11 +26079,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O292" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P292" t="inlineStr">
         <is>
           <t>auto</t>
@@ -27435,11 +26180,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O293" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P293" t="inlineStr">
         <is>
           <t>auto</t>
@@ -27541,11 +26281,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O294" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P294" t="inlineStr">
         <is>
           <t>auto</t>
@@ -27647,11 +26382,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O295" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P295" t="inlineStr">
         <is>
           <t>auto</t>
@@ -27753,11 +26483,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O296" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P296" t="inlineStr">
         <is>
           <t>auto</t>
@@ -27859,11 +26584,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O297" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P297" t="inlineStr">
         <is>
           <t>auto</t>
@@ -27965,11 +26685,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O298" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P298" t="inlineStr">
         <is>
           <t>auto</t>
@@ -28071,11 +26786,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O299" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P299" t="inlineStr">
         <is>
           <t>auto</t>
@@ -28177,11 +26887,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O300" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P300" t="inlineStr">
         <is>
           <t>auto</t>
@@ -28283,11 +26988,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O301" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P301" t="inlineStr">
         <is>
           <t>auto</t>
@@ -28389,11 +27089,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O302" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P302" t="inlineStr">
         <is>
           <t>auto</t>
@@ -28495,11 +27190,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O303" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P303" t="inlineStr">
         <is>
           <t>auto</t>
@@ -28601,11 +27291,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O304" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P304" t="inlineStr">
         <is>
           <t>auto</t>
@@ -28707,11 +27392,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O305" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P305" t="inlineStr">
         <is>
           <t>auto</t>
@@ -28813,11 +27493,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O306" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P306" t="inlineStr">
         <is>
           <t>auto</t>
@@ -28919,11 +27594,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O307" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P307" t="inlineStr">
         <is>
           <t>auto</t>
@@ -29025,11 +27695,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O308" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P308" t="inlineStr">
         <is>
           <t>auto</t>
@@ -29131,11 +27796,6 @@
           <t>licht</t>
         </is>
       </c>
-      <c r="O309" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
-        </is>
-      </c>
       <c r="P309" t="inlineStr">
         <is>
           <t>auto</t>
@@ -29235,11 +27895,6 @@
       <c r="N310" t="inlineStr">
         <is>
           <t>licht</t>
-        </is>
-      </c>
-      <c r="O310" t="inlineStr">
-        <is>
-          <t>1.1.1</t>
         </is>
       </c>
       <c r="P310" t="inlineStr">

</xml_diff>

<commit_message>
xlsx: taal-rootknoop Code 2 (Deutsch) hersteld
Rij overgenomen exact zoals in commit 3d41eb0a (24 juli 2026). 
Ontbrak in de xlsx sinds de foutieve "Nieuwe menustructuur"-commit van 25 juli.
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR310"/>
+  <dimension ref="B2:AR311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -27932,6 +27932,101 @@
         </is>
       </c>
       <c r="AM310" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>taal</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Deutsch</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>Das offene Visier</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>Nederlandse uitgave van Het Open Vizier — onderzoeksjournalistiek over governance, energie en economie.</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>center</t>
+        </is>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>geen</t>
+        </is>
+      </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="N311" t="inlineStr">
+        <is>
+          <t>licht</t>
+        </is>
+      </c>
+      <c r="P311" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="Q311" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="R311" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="T311" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI311" t="inlineStr">
+        <is>
+          <t>talen, nederlands</t>
+        </is>
+      </c>
+      <c r="AK311" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AL311" t="inlineStr">
+        <is>
+          <t>Jacobus van Merksteijn</t>
+        </is>
+      </c>
+      <c r="AM311" t="inlineStr">
         <is>
           <t>nl</t>
         </is>

</xml_diff>

<commit_message>
revert: verwijder overbodige rij "Code 2" (taal is al in eerste cijfer van code)
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR311"/>
+  <dimension ref="B2:AR310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -27932,101 +27932,6 @@
         </is>
       </c>
       <c r="AM310" t="inlineStr">
-        <is>
-          <t>nl</t>
-        </is>
-      </c>
-    </row>
-    <row r="311">
-      <c r="B311" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C311" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D311" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="E311" t="inlineStr">
-        <is>
-          <t>taal</t>
-        </is>
-      </c>
-      <c r="F311" t="inlineStr">
-        <is>
-          <t>Deutsch</t>
-        </is>
-      </c>
-      <c r="G311" t="inlineStr">
-        <is>
-          <t>Das offene Visier</t>
-        </is>
-      </c>
-      <c r="H311" t="inlineStr">
-        <is>
-          <t>Nederlandse uitgave van Het Open Vizier — onderzoeksjournalistiek over governance, energie en economie.</t>
-        </is>
-      </c>
-      <c r="K311" t="inlineStr">
-        <is>
-          <t>center</t>
-        </is>
-      </c>
-      <c r="L311" t="inlineStr">
-        <is>
-          <t>geen</t>
-        </is>
-      </c>
-      <c r="M311" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="N311" t="inlineStr">
-        <is>
-          <t>licht</t>
-        </is>
-      </c>
-      <c r="P311" t="inlineStr">
-        <is>
-          <t>auto</t>
-        </is>
-      </c>
-      <c r="Q311" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="R311" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="T311" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI311" t="inlineStr">
-        <is>
-          <t>talen, nederlands</t>
-        </is>
-      </c>
-      <c r="AK311" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="AL311" t="inlineStr">
-        <is>
-          <t>Jacobus van Merksteijn</t>
-        </is>
-      </c>
-      <c r="AM311" t="inlineStr">
         <is>
           <t>nl</t>
         </is>

</xml_diff>

<commit_message>
Xlsx v8: HTML-entities en site-suffixen uit menu-namen gestript
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -12932,7 +12932,7 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>Die KI als Chef — Das Offene Visier</t>
+          <t>Die KI als Chef</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -13418,7 +13418,7 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>Die KI als Chef — Das Offene Visier</t>
+          <t>Die KI als Chef</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -13656,7 +13656,7 @@
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>Der 7-Dim Film — Das offene Visier</t>
+          <t>Der 7-Dim Film</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -14815,7 +14815,7 @@
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>Das Märchen von Jacobus — Das Offene Visier</t>
+          <t>Das Märchen von Jacobus</t>
         </is>
       </c>
       <c r="I331" t="inlineStr">
@@ -15706,7 +15706,7 @@
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>Was stimmt nicht mit der Parteipolitik? — Das Offene Visier</t>
+          <t>Was stimmt nicht mit der Parteipolitik?</t>
         </is>
       </c>
       <c r="I353" t="inlineStr">
@@ -16627,7 +16627,7 @@
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>Ein Ferrari, der nach gemähtem Gras duftet — Das Offene Visier</t>
+          <t>Ein Ferrari, der nach gemähtem Gras duftet</t>
         </is>
       </c>
       <c r="I375" t="inlineStr">
@@ -17986,7 +17986,7 @@
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>Ausgabe Kind &amp;amp; Laufbahn</t>
+          <t>Ausgabe Kind &amp; Laufbahn</t>
         </is>
       </c>
       <c r="I408" t="inlineStr">
@@ -18353,7 +18353,7 @@
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>Nova Democratia — Das Offene Visier · Ausgabe 6 — Juni 2026</t>
+          <t>Nova Democratia</t>
         </is>
       </c>
       <c r="I417" t="inlineStr">
@@ -22736,7 +22736,7 @@
       </c>
       <c r="F523" t="inlineStr">
         <is>
-          <t>Was ich hinterlasse — Das Offene Visier</t>
+          <t>Was ich hinterlasse</t>
         </is>
       </c>
       <c r="I523" t="inlineStr">
@@ -23207,7 +23207,7 @@
       </c>
       <c r="F535" t="inlineStr">
         <is>
-          <t>Vortex-Hair™ Adaptive Dimple Golf Ball — Dossier · Das Offene Visier</t>
+          <t>Vortex-Hair™ Adaptive Dimple Golf Ball — Dossier</t>
         </is>
       </c>
       <c r="I535" t="inlineStr">
@@ -23326,7 +23326,7 @@
       </c>
       <c r="F538" t="inlineStr">
         <is>
-          <t>Vielen Dank — bitte bestätigen Sie Ihr Postfach — Das Offene Visier</t>
+          <t>Vielen Dank — bitte bestätigen Sie Ihr Postfach</t>
         </is>
       </c>
       <c r="I538" t="inlineStr">
@@ -23597,7 +23597,7 @@
       </c>
       <c r="F545" t="inlineStr">
         <is>
-          <t>Über diese Zeitung — Das Offene Visier</t>
+          <t>Über diese Zeitung</t>
         </is>
       </c>
       <c r="I545" t="inlineStr">
@@ -24293,7 +24293,7 @@
       </c>
       <c r="F563" t="inlineStr">
         <is>
-          <t>The AI as boss — The Open Vizier</t>
+          <t>The AI as boss</t>
         </is>
       </c>
       <c r="I563" t="inlineStr">
@@ -24779,7 +24779,7 @@
       </c>
       <c r="F575" t="inlineStr">
         <is>
-          <t>The AI as boss — The Open Vizier</t>
+          <t>The AI as boss</t>
         </is>
       </c>
       <c r="I575" t="inlineStr">
@@ -29347,7 +29347,7 @@
       </c>
       <c r="F686" t="inlineStr">
         <is>
-          <t>Child &amp;amp; Career edition</t>
+          <t>Child &amp; Career edition</t>
         </is>
       </c>
       <c r="I686" t="inlineStr">
@@ -30992,7 +30992,7 @@
       </c>
       <c r="F726" t="inlineStr">
         <is>
-          <t>They Are Killing Their Lifeline — The Open Vizier</t>
+          <t>They Are Killing Their Lifeline</t>
         </is>
       </c>
       <c r="I726" t="inlineStr">
@@ -32915,7 +32915,7 @@
       </c>
       <c r="F772" t="inlineStr">
         <is>
-          <t>The Dissidents — The Open Vizier · Edition 5 — July 2026</t>
+          <t>The Dissidents</t>
         </is>
       </c>
       <c r="I772" t="inlineStr">
@@ -35654,7 +35654,7 @@
       </c>
       <c r="F841" t="inlineStr">
         <is>
-          <t>ИИ как начальник — Открытое Забрало</t>
+          <t>ИИ как начальник</t>
         </is>
       </c>
       <c r="I841" t="inlineStr">
@@ -36135,7 +36135,7 @@
       </c>
       <c r="F853" t="inlineStr">
         <is>
-          <t>ИИ как начальник — Открытое Забрало</t>
+          <t>ИИ как начальник</t>
         </is>
       </c>
       <c r="I853" t="inlineStr">
@@ -36373,7 +36373,7 @@
       </c>
       <c r="F859" t="inlineStr">
         <is>
-          <t>Фильм 7-Dim — Открытое Забрало</t>
+          <t>Фильм 7-Dim</t>
         </is>
       </c>
       <c r="I859" t="inlineStr">
@@ -38413,7 +38413,7 @@
       </c>
       <c r="F909" t="inlineStr">
         <is>
-          <t>Что не так с партийной политикой? — Открытое забрало</t>
+          <t>Что не так с партийной политикой?</t>
         </is>
       </c>
       <c r="I909" t="inlineStr">
@@ -39309,7 +39309,7 @@
       </c>
       <c r="F931" t="inlineStr">
         <is>
-          <t>Ferrari, который пахнет скошенной травой — Открытое забрало</t>
+          <t>Ferrari, который пахнет скошенной травой</t>
         </is>
       </c>
       <c r="I931" t="inlineStr">
@@ -41025,7 +41025,7 @@
       </c>
       <c r="F973" t="inlineStr">
         <is>
-          <t>Nova Democratia — Открытое забрало · Выпуск 6 — Июнь 2026 г.</t>
+          <t>Nova Democratia</t>
         </is>
       </c>
       <c r="I973" t="inlineStr">
@@ -43648,7 +43648,7 @@
       </c>
       <c r="F1039" t="inlineStr">
         <is>
-          <t>Иммунная система, которая атакует здоровые клетки — Открытое забрало</t>
+          <t>Иммунная система, которая атакует здоровые клетки</t>
         </is>
       </c>
       <c r="I1039" t="inlineStr">
@@ -45283,7 +45283,7 @@
       </c>
       <c r="F1079" t="inlineStr">
         <is>
-          <t>То, что я оставляю — Открытое забрало</t>
+          <t>То, что я оставляю</t>
         </is>
       </c>
       <c r="I1079" t="inlineStr">
@@ -45749,7 +45749,7 @@
       </c>
       <c r="F1091" t="inlineStr">
         <is>
-          <t>Vortex-Hair™ Adaptive Dimple Golf Ball — Досье · Открытое забрало</t>
+          <t>Vortex-Hair™ Adaptive Dimple Golf Ball — Досье</t>
         </is>
       </c>
       <c r="I1091" t="inlineStr">
@@ -45868,7 +45868,7 @@
       </c>
       <c r="F1094" t="inlineStr">
         <is>
-          <t>Спасибо — проверьте Вашу почту — Открытое забрало</t>
+          <t>Спасибо — проверьте Вашу почту</t>
         </is>
       </c>
       <c r="I1094" t="inlineStr">
@@ -46139,7 +46139,7 @@
       </c>
       <c r="F1101" t="inlineStr">
         <is>
-          <t>Об этой газете — Открытое забрало</t>
+          <t>Об этой газете</t>
         </is>
       </c>
       <c r="I1101" t="inlineStr">
@@ -46182,7 +46182,7 @@
       </c>
       <c r="F1102" t="inlineStr">
         <is>
-          <t>Исследовать — Открытое забрало</t>
+          <t>Исследовать</t>
         </is>
       </c>
       <c r="I1102" t="inlineStr">
@@ -46835,7 +46835,7 @@
       </c>
       <c r="F1119" t="inlineStr">
         <is>
-          <t>L&amp;#x27;IA comme patron — La Visière Ouverte</t>
+          <t>L'IA comme patron</t>
         </is>
       </c>
       <c r="I1119" t="inlineStr">
@@ -47336,7 +47336,7 @@
       </c>
       <c r="F1131" t="inlineStr">
         <is>
-          <t>L&amp;#x27;IA comme patron — La Visière Ouverte</t>
+          <t>L'IA comme patron</t>
         </is>
       </c>
       <c r="I1131" t="inlineStr">
@@ -57756,7 +57756,7 @@
       </c>
       <c r="F1397" t="inlineStr">
         <is>
-          <t>La IA como jefe — La Visera Abierta</t>
+          <t>La IA como jefe</t>
         </is>
       </c>
       <c r="I1397" t="inlineStr">
@@ -58257,7 +58257,7 @@
       </c>
       <c r="F1409" t="inlineStr">
         <is>
-          <t>La IA como jefe — La Visera Abierta</t>
+          <t>La IA como jefe</t>
         </is>
       </c>
       <c r="I1409" t="inlineStr">
@@ -68877,7 +68877,7 @@
       </c>
       <c r="F1675" t="inlineStr">
         <is>
-          <t>L&amp;#x27;IA come capo — La Visiera Aperta</t>
+          <t>L'IA come capo</t>
         </is>
       </c>
       <c r="I1675" t="inlineStr">
@@ -69378,7 +69378,7 @@
       </c>
       <c r="F1687" t="inlineStr">
         <is>
-          <t>L&amp;#x27;IA come capo — La Visiera Aperta</t>
+          <t>L'IA come capo</t>
         </is>
       </c>
       <c r="I1687" t="inlineStr">
@@ -80013,7 +80013,7 @@
       </c>
       <c r="F1953" t="inlineStr">
         <is>
-          <t>A IA como chefe — A Viseira Aberta</t>
+          <t>A IA como chefe</t>
         </is>
       </c>
       <c r="I1953" t="inlineStr">
@@ -80514,7 +80514,7 @@
       </c>
       <c r="F1965" t="inlineStr">
         <is>
-          <t>A IA como chefe — A Viseira Aberta</t>
+          <t>A IA como chefe</t>
         </is>
       </c>
       <c r="I1965" t="inlineStr">

</xml_diff>

<commit_message>
Xlsx: nederland-kompleet-v3 toegevoegd onder Nederland (1.11.13) in alle 8 talen
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR2227"/>
+  <dimension ref="B2:AR2235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -91015,6 +91015,350 @@
         <v>1</v>
       </c>
     </row>
+    <row r="2228">
+      <c r="B2228" t="inlineStr">
+        <is>
+          <t>1.11.13</t>
+        </is>
+      </c>
+      <c r="C2228" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="D2228" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2228" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2228" t="inlineStr">
+        <is>
+          <t>Nederland aug 2026 – aug 2028: Systeembreuk in drie ordes</t>
+        </is>
+      </c>
+      <c r="I2228" t="inlineStr">
+        <is>
+          <t>nederland-kompleet-v3/</t>
+        </is>
+      </c>
+      <c r="R2228" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2228" t="n">
+        <v>13</v>
+      </c>
+      <c r="T2228" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2229">
+      <c r="B2229" t="inlineStr">
+        <is>
+          <t>2.11.13</t>
+        </is>
+      </c>
+      <c r="C2229" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="D2229" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2229" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2229" t="inlineStr">
+        <is>
+          <t>Niederlande Aug 2026 – Aug 2028: Systembruch in drei Ordnungen</t>
+        </is>
+      </c>
+      <c r="I2229" t="inlineStr">
+        <is>
+          <t>/nl/nederland-kompleet-v3/</t>
+        </is>
+      </c>
+      <c r="R2229" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2229" t="n">
+        <v>13</v>
+      </c>
+      <c r="T2229" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2230">
+      <c r="B2230" t="inlineStr">
+        <is>
+          <t>3.11.13</t>
+        </is>
+      </c>
+      <c r="C2230" t="inlineStr">
+        <is>
+          <t>3.11</t>
+        </is>
+      </c>
+      <c r="D2230" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2230" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2230" t="inlineStr">
+        <is>
+          <t>Netherlands Aug 2026 – Aug 2028: Systemic break in three orders</t>
+        </is>
+      </c>
+      <c r="I2230" t="inlineStr">
+        <is>
+          <t>/nl/nederland-kompleet-v3/</t>
+        </is>
+      </c>
+      <c r="R2230" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2230" t="n">
+        <v>13</v>
+      </c>
+      <c r="T2230" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2231">
+      <c r="B2231" t="inlineStr">
+        <is>
+          <t>4.11.13</t>
+        </is>
+      </c>
+      <c r="C2231" t="inlineStr">
+        <is>
+          <t>4.11</t>
+        </is>
+      </c>
+      <c r="D2231" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2231" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2231" t="inlineStr">
+        <is>
+          <t>Нидерланды авг 2026 – авг 2028: Системный разлом в трёх порядках</t>
+        </is>
+      </c>
+      <c r="I2231" t="inlineStr">
+        <is>
+          <t>/nl/nederland-kompleet-v3/</t>
+        </is>
+      </c>
+      <c r="R2231" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2231" t="n">
+        <v>13</v>
+      </c>
+      <c r="T2231" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2232">
+      <c r="B2232" t="inlineStr">
+        <is>
+          <t>5.11.13</t>
+        </is>
+      </c>
+      <c r="C2232" t="inlineStr">
+        <is>
+          <t>5.11</t>
+        </is>
+      </c>
+      <c r="D2232" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="E2232" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2232" t="inlineStr">
+        <is>
+          <t>Pays-Bas août 2026 – août 2028: Rupture systémique en trois ordres</t>
+        </is>
+      </c>
+      <c r="I2232" t="inlineStr">
+        <is>
+          <t>/nl/nederland-kompleet-v3/</t>
+        </is>
+      </c>
+      <c r="R2232" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2232" t="n">
+        <v>13</v>
+      </c>
+      <c r="T2232" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2233">
+      <c r="B2233" t="inlineStr">
+        <is>
+          <t>6.11.13</t>
+        </is>
+      </c>
+      <c r="C2233" t="inlineStr">
+        <is>
+          <t>6.11</t>
+        </is>
+      </c>
+      <c r="D2233" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="E2233" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2233" t="inlineStr">
+        <is>
+          <t>Países Bajos ago 2026 – ago 2028: Ruptura sistémica en tres órdenes</t>
+        </is>
+      </c>
+      <c r="I2233" t="inlineStr">
+        <is>
+          <t>/nl/nederland-kompleet-v3/</t>
+        </is>
+      </c>
+      <c r="R2233" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2233" t="n">
+        <v>13</v>
+      </c>
+      <c r="T2233" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2234">
+      <c r="B2234" t="inlineStr">
+        <is>
+          <t>7.11.13</t>
+        </is>
+      </c>
+      <c r="C2234" t="inlineStr">
+        <is>
+          <t>7.11</t>
+        </is>
+      </c>
+      <c r="D2234" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="E2234" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2234" t="inlineStr">
+        <is>
+          <t>Paesi Bassi ago 2026 – ago 2028: Rottura sistemica in tre ordini</t>
+        </is>
+      </c>
+      <c r="I2234" t="inlineStr">
+        <is>
+          <t>/nl/nederland-kompleet-v3/</t>
+        </is>
+      </c>
+      <c r="R2234" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2234" t="n">
+        <v>13</v>
+      </c>
+      <c r="T2234" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2235">
+      <c r="B2235" t="inlineStr">
+        <is>
+          <t>8.11.13</t>
+        </is>
+      </c>
+      <c r="C2235" t="inlineStr">
+        <is>
+          <t>8.11</t>
+        </is>
+      </c>
+      <c r="D2235" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="E2235" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2235" t="inlineStr">
+        <is>
+          <t>Países Baixos ago 2026 – ago 2028: Ruptura sistêmica em três ordens</t>
+        </is>
+      </c>
+      <c r="I2235" t="inlineStr">
+        <is>
+          <t>/nl/nederland-kompleet-v3/</t>
+        </is>
+      </c>
+      <c r="R2235" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2235" t="n">
+        <v>13</v>
+      </c>
+      <c r="T2235" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B2:AR65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Xlsx v10: Kosaris URLs + vertaalde titels voor DE/EN/RU/FR/ES/IT/PT
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -2963,7 +2963,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>kosaris-film/index.html</t>
+          <t>kosaris-film/</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -3001,12 +3001,12 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>De Kosaris — Het boek van de heilige Kosus</t>
+          <t>De Kosaris — Leesboek</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>leesboek/index.html</t>
+          <t>leesboek/</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -3044,12 +3044,12 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Het sprookje van Jacobus — een sprookje in zestien pagina's</t>
+          <t>Het sprookje van Jacobus</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>sprookjes/index.html</t>
+          <t>sprookjes/</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -3092,7 +3092,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>leesboek-boek-twee/index.html</t>
+          <t>leesboek-boek-twee/</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -3130,12 +3130,12 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Drie — Het boek van Anthea</t>
+          <t>De Kosaris — BOEK DRIE</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>leesboek-boek-drie/index.html</t>
+          <t>leesboek-boek-drie/</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -3173,12 +3173,12 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vier — Het boek van het hydrolysaat</t>
+          <t>De Kosaris — BOEK VIER</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>leesboek-boek-vier/index.html</t>
+          <t>leesboek-boek-vier/</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -3216,12 +3216,12 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vijf — Het boek van de partner</t>
+          <t>De Kosaris — BOEK VIJF</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>leesboek-boek-vijf/index.html</t>
+          <t>leesboek-boek-vijf/</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -14734,7 +14734,7 @@
       </c>
       <c r="I329" t="inlineStr">
         <is>
-          <t>kosaris-film/index.html</t>
+          <t>kosaris-film/</t>
         </is>
       </c>
       <c r="R329" t="inlineStr">
@@ -14789,7 +14789,7 @@
         <v>2</v>
       </c>
       <c r="T330" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="331">
@@ -14820,7 +14820,7 @@
       </c>
       <c r="I331" t="inlineStr">
         <is>
-          <t>maerchen/index.html</t>
+          <t>maerchen/</t>
         </is>
       </c>
       <c r="R331" t="inlineStr">
@@ -14858,7 +14858,12 @@
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Twee — Diakrisis</t>
+          <t>De Kosaris — Buch Zwei — Diakrisis</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>lesebuch-zwei/</t>
         </is>
       </c>
       <c r="R332" t="inlineStr">
@@ -14896,7 +14901,12 @@
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Drie — Het boek van Anthea</t>
+          <t>Der Kosaris — Buch Drei — Das Buch der Anthea</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>lesebuch-drei/</t>
         </is>
       </c>
       <c r="R333" t="inlineStr">
@@ -14934,7 +14944,12 @@
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vier — Het boek van het hydrolysaat</t>
+          <t>Der Kosaris — Buch Vier — Das Buch des Hydrolysats</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>lesebuch-vier/</t>
         </is>
       </c>
       <c r="R334" t="inlineStr">
@@ -14972,7 +14987,12 @@
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vijf — Het boek van de partner</t>
+          <t>Der Kosaris — Buch Fünf — Das Buch des Partners</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>lesebuch-fuenf/</t>
         </is>
       </c>
       <c r="R335" t="inlineStr">
@@ -15022,7 +15042,7 @@
         <v>8</v>
       </c>
       <c r="T336" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="337">
@@ -15060,7 +15080,7 @@
         <v>9</v>
       </c>
       <c r="T337" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="338">
@@ -26095,7 +26115,7 @@
       </c>
       <c r="I607" t="inlineStr">
         <is>
-          <t>kosaris-film/index.html</t>
+          <t>kosaris-film/</t>
         </is>
       </c>
       <c r="R607" t="inlineStr">
@@ -26150,7 +26170,7 @@
         <v>2</v>
       </c>
       <c r="T608" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="609">
@@ -26193,7 +26213,7 @@
         <v>3</v>
       </c>
       <c r="T609" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="610">
@@ -26219,7 +26239,12 @@
       </c>
       <c r="F610" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Twee — Diakrisis</t>
+          <t>De Kosaris — Book Two — Diakrisis</t>
+        </is>
+      </c>
+      <c r="I610" t="inlineStr">
+        <is>
+          <t>reading-book-two/</t>
         </is>
       </c>
       <c r="R610" t="inlineStr">
@@ -26257,7 +26282,12 @@
       </c>
       <c r="F611" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Drie — Het boek van Anthea</t>
+          <t>The Kosaris — Book Three — The Book of Anthea</t>
+        </is>
+      </c>
+      <c r="I611" t="inlineStr">
+        <is>
+          <t>reading-book-three/</t>
         </is>
       </c>
       <c r="R611" t="inlineStr">
@@ -26295,7 +26325,12 @@
       </c>
       <c r="F612" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vier — Het boek van het hydrolysaat</t>
+          <t>The Kosaris — Book Four — The Book of the Hydrolysate</t>
+        </is>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>reading-book-four/</t>
         </is>
       </c>
       <c r="R612" t="inlineStr">
@@ -26333,7 +26368,12 @@
       </c>
       <c r="F613" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vijf — Het boek van de partner</t>
+          <t>The Kosaris — Book Five — The Book of the Partner</t>
+        </is>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>reading-book-five/</t>
         </is>
       </c>
       <c r="R613" t="inlineStr">
@@ -26383,7 +26423,7 @@
         <v>8</v>
       </c>
       <c r="T614" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="615">
@@ -26421,7 +26461,7 @@
         <v>9</v>
       </c>
       <c r="T615" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="616">
@@ -37451,7 +37491,7 @@
       </c>
       <c r="I885" t="inlineStr">
         <is>
-          <t>kosaris-film/index.html</t>
+          <t>kosaris-film/</t>
         </is>
       </c>
       <c r="R885" t="inlineStr">
@@ -37506,7 +37546,7 @@
         <v>2</v>
       </c>
       <c r="T886" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="887">
@@ -37537,7 +37577,7 @@
       </c>
       <c r="I887" t="inlineStr">
         <is>
-          <t>skazki/index.html</t>
+          <t>skazki/</t>
         </is>
       </c>
       <c r="R887" t="inlineStr">
@@ -37575,7 +37615,12 @@
       </c>
       <c r="F888" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Twee — Diakrisis</t>
+          <t>Косарис — Книга вторая — Диакрисис</t>
+        </is>
+      </c>
+      <c r="I888" t="inlineStr">
+        <is>
+          <t>kniga-dva/</t>
         </is>
       </c>
       <c r="R888" t="inlineStr">
@@ -37613,7 +37658,12 @@
       </c>
       <c r="F889" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Drie — Het boek van Anthea</t>
+          <t>Косарис — Книга третья — Книга Антеи</t>
+        </is>
+      </c>
+      <c r="I889" t="inlineStr">
+        <is>
+          <t>kniga-tri/</t>
         </is>
       </c>
       <c r="R889" t="inlineStr">
@@ -37651,7 +37701,12 @@
       </c>
       <c r="F890" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vier — Het boek van het hydrolysaat</t>
+          <t>Косарис — Книга четвёртая — Книга гидролизата</t>
+        </is>
+      </c>
+      <c r="I890" t="inlineStr">
+        <is>
+          <t>kniga-chetyre/</t>
         </is>
       </c>
       <c r="R890" t="inlineStr">
@@ -37689,7 +37744,12 @@
       </c>
       <c r="F891" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vijf — Het boek van de partner</t>
+          <t>Косарис — Книга пятая — Книга партнёра</t>
+        </is>
+      </c>
+      <c r="I891" t="inlineStr">
+        <is>
+          <t>kniga-pyat/</t>
         </is>
       </c>
       <c r="R891" t="inlineStr">
@@ -37739,7 +37799,7 @@
         <v>8</v>
       </c>
       <c r="T892" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="893">
@@ -37777,7 +37837,7 @@
         <v>9</v>
       </c>
       <c r="T893" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="894">
@@ -48592,7 +48652,7 @@
       </c>
       <c r="I1163" t="inlineStr">
         <is>
-          <t>kosaris-film/index.html</t>
+          <t>kosaris-film/</t>
         </is>
       </c>
       <c r="R1163" t="inlineStr">
@@ -48647,7 +48707,7 @@
         <v>2</v>
       </c>
       <c r="T1164" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1165">
@@ -48678,7 +48738,7 @@
       </c>
       <c r="I1165" t="inlineStr">
         <is>
-          <t>contes/index.html</t>
+          <t>contes/</t>
         </is>
       </c>
       <c r="R1165" t="inlineStr">
@@ -48716,7 +48776,12 @@
       </c>
       <c r="F1166" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Twee — Diakrisis</t>
+          <t>De Kosaris — LIVRE DEUX — Diakrisis</t>
+        </is>
+      </c>
+      <c r="I1166" t="inlineStr">
+        <is>
+          <t>livre-deux/</t>
         </is>
       </c>
       <c r="R1166" t="inlineStr">
@@ -48754,7 +48819,12 @@
       </c>
       <c r="F1167" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Drie — Het boek van Anthea</t>
+          <t>Le Kosaris — Livre Trois — Le livre d'Anthea</t>
+        </is>
+      </c>
+      <c r="I1167" t="inlineStr">
+        <is>
+          <t>livre-trois/</t>
         </is>
       </c>
       <c r="R1167" t="inlineStr">
@@ -48792,7 +48862,12 @@
       </c>
       <c r="F1168" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vier — Het boek van het hydrolysaat</t>
+          <t>Le Kosaris — Livre Quatre — Le livre de l'hydrolysat</t>
+        </is>
+      </c>
+      <c r="I1168" t="inlineStr">
+        <is>
+          <t>livre-quatre/</t>
         </is>
       </c>
       <c r="R1168" t="inlineStr">
@@ -48830,7 +48905,12 @@
       </c>
       <c r="F1169" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vijf — Het boek van de partner</t>
+          <t>Le Kosaris — Livre Cinq — Le livre du partenaire</t>
+        </is>
+      </c>
+      <c r="I1169" t="inlineStr">
+        <is>
+          <t>livre-cinq/</t>
         </is>
       </c>
       <c r="R1169" t="inlineStr">
@@ -48880,7 +48960,7 @@
         <v>8</v>
       </c>
       <c r="T1170" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1171">
@@ -48918,7 +48998,7 @@
         <v>9</v>
       </c>
       <c r="T1171" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1172">
@@ -59528,7 +59608,7 @@
       </c>
       <c r="I1441" t="inlineStr">
         <is>
-          <t>kosaris-film/index.html</t>
+          <t>kosaris-film/</t>
         </is>
       </c>
       <c r="R1441" t="inlineStr">
@@ -59583,7 +59663,7 @@
         <v>2</v>
       </c>
       <c r="T1442" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1443">
@@ -59614,7 +59694,7 @@
       </c>
       <c r="I1443" t="inlineStr">
         <is>
-          <t>cuentos/index.html</t>
+          <t>cuentos/</t>
         </is>
       </c>
       <c r="R1443" t="inlineStr">
@@ -59652,7 +59732,12 @@
       </c>
       <c r="F1444" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Twee — Diakrisis</t>
+          <t>De Kosaris — Libro Dos — Diakrisis</t>
+        </is>
+      </c>
+      <c r="I1444" t="inlineStr">
+        <is>
+          <t>libro-dos/</t>
         </is>
       </c>
       <c r="R1444" t="inlineStr">
@@ -59690,7 +59775,12 @@
       </c>
       <c r="F1445" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Drie — Het boek van Anthea</t>
+          <t>El Kosaris — Libro Tres — El libro de Anthea</t>
+        </is>
+      </c>
+      <c r="I1445" t="inlineStr">
+        <is>
+          <t>libro-tres/</t>
         </is>
       </c>
       <c r="R1445" t="inlineStr">
@@ -59728,7 +59818,12 @@
       </c>
       <c r="F1446" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vier — Het boek van het hydrolysaat</t>
+          <t>El Kosaris — Libro Cuatro — El libro del hidrolizado</t>
+        </is>
+      </c>
+      <c r="I1446" t="inlineStr">
+        <is>
+          <t>libro-cuatro/</t>
         </is>
       </c>
       <c r="R1446" t="inlineStr">
@@ -59766,7 +59861,12 @@
       </c>
       <c r="F1447" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vijf — Het boek van de partner</t>
+          <t>El Kosaris — Libro Cinco — El libro del socio</t>
+        </is>
+      </c>
+      <c r="I1447" t="inlineStr">
+        <is>
+          <t>libro-cinco/</t>
         </is>
       </c>
       <c r="R1447" t="inlineStr">
@@ -59816,7 +59916,7 @@
         <v>8</v>
       </c>
       <c r="T1448" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1449">
@@ -59854,7 +59954,7 @@
         <v>9</v>
       </c>
       <c r="T1449" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1450">
@@ -70649,7 +70749,7 @@
       </c>
       <c r="I1719" t="inlineStr">
         <is>
-          <t>kosaris-film/index.html</t>
+          <t>kosaris-film/</t>
         </is>
       </c>
       <c r="R1719" t="inlineStr">
@@ -70704,7 +70804,7 @@
         <v>2</v>
       </c>
       <c r="T1720" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1721">
@@ -70747,7 +70847,7 @@
         <v>3</v>
       </c>
       <c r="T1721" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1722">
@@ -70773,7 +70873,12 @@
       </c>
       <c r="F1722" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Twee — Diakrisis</t>
+          <t>De Kosaris — Libro Due — Diakrisis</t>
+        </is>
+      </c>
+      <c r="I1722" t="inlineStr">
+        <is>
+          <t>libro-due/</t>
         </is>
       </c>
       <c r="R1722" t="inlineStr">
@@ -70811,7 +70916,12 @@
       </c>
       <c r="F1723" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Drie — Het boek van Anthea</t>
+          <t>Il Kosaris — Libro Tre — Il libro di Anthea</t>
+        </is>
+      </c>
+      <c r="I1723" t="inlineStr">
+        <is>
+          <t>libro-tre/</t>
         </is>
       </c>
       <c r="R1723" t="inlineStr">
@@ -70849,7 +70959,12 @@
       </c>
       <c r="F1724" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vier — Het boek van het hydrolysaat</t>
+          <t>Il Kosaris — Libro Quattro — Il libro dell'idrolizzato</t>
+        </is>
+      </c>
+      <c r="I1724" t="inlineStr">
+        <is>
+          <t>libro-quattro/</t>
         </is>
       </c>
       <c r="R1724" t="inlineStr">
@@ -70887,7 +71002,12 @@
       </c>
       <c r="F1725" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Vijf — Het boek van de partner</t>
+          <t>Il Kosaris — Libro Cinque — Il libro del partner</t>
+        </is>
+      </c>
+      <c r="I1725" t="inlineStr">
+        <is>
+          <t>libro-cinque/</t>
         </is>
       </c>
       <c r="R1725" t="inlineStr">
@@ -70937,7 +71057,7 @@
         <v>8</v>
       </c>
       <c r="T1726" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1727">
@@ -70975,7 +71095,7 @@
         <v>9</v>
       </c>
       <c r="T1727" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1728">
@@ -81785,7 +81905,7 @@
       </c>
       <c r="I1997" t="inlineStr">
         <is>
-          <t>kosaris-film/index.html</t>
+          <t>kosaris-film/</t>
         </is>
       </c>
       <c r="R1997" t="inlineStr">
@@ -81840,7 +81960,7 @@
         <v>2</v>
       </c>
       <c r="T1998" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1999">
@@ -81871,7 +81991,7 @@
       </c>
       <c r="I1999" t="inlineStr">
         <is>
-          <t>contos/index.html</t>
+          <t>contos/</t>
         </is>
       </c>
       <c r="R1999" t="inlineStr">
@@ -81921,7 +82041,7 @@
         <v>4</v>
       </c>
       <c r="T2000" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2001">
@@ -81959,7 +82079,7 @@
         <v>5</v>
       </c>
       <c r="T2001" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2002">
@@ -81997,7 +82117,7 @@
         <v>6</v>
       </c>
       <c r="T2002" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2003">
@@ -82035,7 +82155,7 @@
         <v>7</v>
       </c>
       <c r="T2003" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2004">
@@ -82073,7 +82193,7 @@
         <v>8</v>
       </c>
       <c r="T2004" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2005">
@@ -82111,7 +82231,7 @@
         <v>9</v>
       </c>
       <c r="T2005" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2006">

</xml_diff>

<commit_message>
Xlsx v11: Kosaris-films (Boek 2, Boek 3 opvoeding + delen) in NL/DE/EN/RU
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR2235"/>
+  <dimension ref="B2:AR2241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3259,7 +3259,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Twee — De Film</t>
+          <t>De Kosaris — Boek Twee — Diakrisis — Film</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Drie — De Opvoeding (Film)</t>
+          <t>De Kosaris — Boek Drie — De Opvoeding — Film</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -15030,7 +15030,12 @@
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Twee — De Film</t>
+          <t>Der Kosaris — Buch Zwei — Diakrisis — Film</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-twee-film.html</t>
         </is>
       </c>
       <c r="R336" t="inlineStr">
@@ -15042,7 +15047,7 @@
         <v>8</v>
       </c>
       <c r="T336" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="337">
@@ -15068,7 +15073,12 @@
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Drie — De Opvoeding (Film)</t>
+          <t>Der Kosaris — Buch Drei — Die Erziehung — Film</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-de-opvoeding.html</t>
         </is>
       </c>
       <c r="R337" t="inlineStr">
@@ -15080,7 +15090,7 @@
         <v>9</v>
       </c>
       <c r="T337" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="338">
@@ -26411,7 +26421,12 @@
       </c>
       <c r="F614" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Twee — De Film</t>
+          <t>The Kosaris — Book Two — Diakrisis — Film</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-twee-film.html</t>
         </is>
       </c>
       <c r="R614" t="inlineStr">
@@ -26423,7 +26438,7 @@
         <v>8</v>
       </c>
       <c r="T614" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="615">
@@ -26449,7 +26464,12 @@
       </c>
       <c r="F615" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Drie — De Opvoeding (Film)</t>
+          <t>The Kosaris — Book Three — Education — Film</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-de-opvoeding.html</t>
         </is>
       </c>
       <c r="R615" t="inlineStr">
@@ -26461,7 +26481,7 @@
         <v>9</v>
       </c>
       <c r="T615" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="616">
@@ -37787,7 +37807,12 @@
       </c>
       <c r="F892" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Twee — De Film</t>
+          <t>Косарис — Книга вторая — Диакрисис — Film</t>
+        </is>
+      </c>
+      <c r="I892" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-twee-film.html</t>
         </is>
       </c>
       <c r="R892" t="inlineStr">
@@ -37799,7 +37824,7 @@
         <v>8</v>
       </c>
       <c r="T892" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="893">
@@ -37825,7 +37850,12 @@
       </c>
       <c r="F893" t="inlineStr">
         <is>
-          <t>De Kosaris — Boek Drie — De Opvoeding (Film)</t>
+          <t>Косарис — Книга Третья — Воспитание — Фильм</t>
+        </is>
+      </c>
+      <c r="I893" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-de-opvoeding.html</t>
         </is>
       </c>
       <c r="R893" t="inlineStr">
@@ -37837,7 +37867,7 @@
         <v>9</v>
       </c>
       <c r="T893" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="894">
@@ -91476,6 +91506,264 @@
         <v>13</v>
       </c>
       <c r="T2235" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2236">
+      <c r="B2236" t="inlineStr">
+        <is>
+          <t>1.5.10</t>
+        </is>
+      </c>
+      <c r="C2236" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="D2236" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2236" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2236" t="inlineStr">
+        <is>
+          <t>De Kosaris — Boek Drie — De Opvoeding — Deel III</t>
+        </is>
+      </c>
+      <c r="I2236" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-deel-3-film.html</t>
+        </is>
+      </c>
+      <c r="R2236" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2236" t="n">
+        <v>10</v>
+      </c>
+      <c r="T2236" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2237">
+      <c r="B2237" t="inlineStr">
+        <is>
+          <t>2.5.10</t>
+        </is>
+      </c>
+      <c r="C2237" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="D2237" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2237" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2237" t="inlineStr">
+        <is>
+          <t>Der Kosaris — Buch Drei — Die Erziehung — Teil III</t>
+        </is>
+      </c>
+      <c r="I2237" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-deel-3-film.html</t>
+        </is>
+      </c>
+      <c r="R2237" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2237" t="n">
+        <v>10</v>
+      </c>
+      <c r="T2237" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2238">
+      <c r="B2238" t="inlineStr">
+        <is>
+          <t>3.5.10</t>
+        </is>
+      </c>
+      <c r="C2238" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="D2238" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2238" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2238" t="inlineStr">
+        <is>
+          <t>The Kosaris — Book Three — The Education — Part III</t>
+        </is>
+      </c>
+      <c r="I2238" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-deel-3-film.html</t>
+        </is>
+      </c>
+      <c r="R2238" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2238" t="n">
+        <v>10</v>
+      </c>
+      <c r="T2238" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2239">
+      <c r="B2239" t="inlineStr">
+        <is>
+          <t>4.5.10</t>
+        </is>
+      </c>
+      <c r="C2239" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="D2239" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2239" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2239" t="inlineStr">
+        <is>
+          <t>Косарис — Книга Третья — Воспитание — Часть III</t>
+        </is>
+      </c>
+      <c r="I2239" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-deel-3-film.html</t>
+        </is>
+      </c>
+      <c r="R2239" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2239" t="n">
+        <v>10</v>
+      </c>
+      <c r="T2239" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2240">
+      <c r="B2240" t="inlineStr">
+        <is>
+          <t>1.5.11</t>
+        </is>
+      </c>
+      <c r="C2240" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="D2240" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2240" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2240" t="inlineStr">
+        <is>
+          <t>De Kosaris — Boek Drie — De Opvoeding — Deel I</t>
+        </is>
+      </c>
+      <c r="I2240" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-deel-1-film.html</t>
+        </is>
+      </c>
+      <c r="R2240" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2240" t="n">
+        <v>11</v>
+      </c>
+      <c r="T2240" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2241">
+      <c r="B2241" t="inlineStr">
+        <is>
+          <t>1.5.12</t>
+        </is>
+      </c>
+      <c r="C2241" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="D2241" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2241" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2241" t="inlineStr">
+        <is>
+          <t>De Kosaris — Boek Drie — De Opvoeding — Deel II</t>
+        </is>
+      </c>
+      <c r="I2241" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-kosaris-boek-drie-deel-2-film.html</t>
+        </is>
+      </c>
+      <c r="R2241" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2241" t="n">
+        <v>12</v>
+      </c>
+      <c r="T2241" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Xlsx v12: klimaat-de-echte-analyse als 1.7.1, oude items +1 opgeschoven
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR2241"/>
+  <dimension ref="B2:AR2249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4089,7 +4089,7 @@
     <row r="78">
       <c r="B78" t="inlineStr">
         <is>
-          <t>1.7.1</t>
+          <t>1.7.2</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -4123,7 +4123,7 @@
         </is>
       </c>
       <c r="S78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T78" t="b">
         <v>1</v>
@@ -4132,7 +4132,7 @@
     <row r="79">
       <c r="B79" t="inlineStr">
         <is>
-          <t>1.7.2</t>
+          <t>1.7.3</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4166,7 +4166,7 @@
         </is>
       </c>
       <c r="S79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T79" t="b">
         <v>1</v>
@@ -4175,7 +4175,7 @@
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
-          <t>1.7.3</t>
+          <t>1.7.4</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="S80" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T80" t="b">
         <v>1</v>
@@ -4218,7 +4218,7 @@
     <row r="81">
       <c r="B81" t="inlineStr">
         <is>
-          <t>1.7.4</t>
+          <t>1.7.5</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -4252,7 +4252,7 @@
         </is>
       </c>
       <c r="S81" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T81" t="b">
         <v>1</v>
@@ -4261,7 +4261,7 @@
     <row r="82">
       <c r="B82" t="inlineStr">
         <is>
-          <t>1.7.5</t>
+          <t>1.7.6</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -4295,7 +4295,7 @@
         </is>
       </c>
       <c r="S82" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T82" t="b">
         <v>1</v>
@@ -4304,7 +4304,7 @@
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
-          <t>1.7.6</t>
+          <t>1.7.7</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4338,7 +4338,7 @@
         </is>
       </c>
       <c r="S83" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T83" t="b">
         <v>1</v>
@@ -4347,7 +4347,7 @@
     <row r="84">
       <c r="B84" t="inlineStr">
         <is>
-          <t>1.7.7</t>
+          <t>1.7.8</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4381,7 +4381,7 @@
         </is>
       </c>
       <c r="S84" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T84" t="b">
         <v>1</v>
@@ -4390,7 +4390,7 @@
     <row r="85">
       <c r="B85" t="inlineStr">
         <is>
-          <t>1.7.8</t>
+          <t>1.7.9</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4424,7 +4424,7 @@
         </is>
       </c>
       <c r="S85" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T85" t="b">
         <v>1</v>
@@ -4433,7 +4433,7 @@
     <row r="86">
       <c r="B86" t="inlineStr">
         <is>
-          <t>1.7.9</t>
+          <t>1.7.10</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4467,7 +4467,7 @@
         </is>
       </c>
       <c r="S86" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T86" t="b">
         <v>1</v>
@@ -4476,7 +4476,7 @@
     <row r="87">
       <c r="B87" t="inlineStr">
         <is>
-          <t>1.7.10</t>
+          <t>1.7.11</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4510,7 +4510,7 @@
         </is>
       </c>
       <c r="S87" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T87" t="b">
         <v>1</v>
@@ -4519,7 +4519,7 @@
     <row r="88">
       <c r="B88" t="inlineStr">
         <is>
-          <t>1.7.11</t>
+          <t>1.7.12</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4553,7 +4553,7 @@
         </is>
       </c>
       <c r="S88" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T88" t="b">
         <v>1</v>
@@ -4562,7 +4562,7 @@
     <row r="89">
       <c r="B89" t="inlineStr">
         <is>
-          <t>1.7.12</t>
+          <t>1.7.13</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4596,7 +4596,7 @@
         </is>
       </c>
       <c r="S89" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T89" t="b">
         <v>1</v>
@@ -4605,7 +4605,7 @@
     <row r="90">
       <c r="B90" t="inlineStr">
         <is>
-          <t>1.7.13</t>
+          <t>1.7.14</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -4639,7 +4639,7 @@
         </is>
       </c>
       <c r="S90" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T90" t="b">
         <v>1</v>
@@ -4648,7 +4648,7 @@
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t>1.7.14</t>
+          <t>1.7.15</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4682,7 +4682,7 @@
         </is>
       </c>
       <c r="S91" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T91" t="b">
         <v>1</v>
@@ -4691,7 +4691,7 @@
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
-          <t>1.7.15</t>
+          <t>1.7.16</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4725,7 +4725,7 @@
         </is>
       </c>
       <c r="S92" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T92" t="b">
         <v>1</v>
@@ -15840,7 +15840,7 @@
     <row r="356">
       <c r="B356" t="inlineStr">
         <is>
-          <t>2.7.1</t>
+          <t>2.7.2</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -15874,7 +15874,7 @@
         </is>
       </c>
       <c r="S356" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T356" t="b">
         <v>1</v>
@@ -15883,7 +15883,7 @@
     <row r="357">
       <c r="B357" t="inlineStr">
         <is>
-          <t>2.7.2</t>
+          <t>2.7.3</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -15917,7 +15917,7 @@
         </is>
       </c>
       <c r="S357" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T357" t="b">
         <v>1</v>
@@ -15926,7 +15926,7 @@
     <row r="358">
       <c r="B358" t="inlineStr">
         <is>
-          <t>2.7.3</t>
+          <t>2.7.4</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -15960,7 +15960,7 @@
         </is>
       </c>
       <c r="S358" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T358" t="b">
         <v>1</v>
@@ -15969,7 +15969,7 @@
     <row r="359">
       <c r="B359" t="inlineStr">
         <is>
-          <t>2.7.4</t>
+          <t>2.7.5</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -16003,7 +16003,7 @@
         </is>
       </c>
       <c r="S359" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T359" t="b">
         <v>1</v>
@@ -16012,7 +16012,7 @@
     <row r="360">
       <c r="B360" t="inlineStr">
         <is>
-          <t>2.7.5</t>
+          <t>2.7.6</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -16046,7 +16046,7 @@
         </is>
       </c>
       <c r="S360" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T360" t="b">
         <v>1</v>
@@ -16055,7 +16055,7 @@
     <row r="361">
       <c r="B361" t="inlineStr">
         <is>
-          <t>2.7.6</t>
+          <t>2.7.7</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -16089,7 +16089,7 @@
         </is>
       </c>
       <c r="S361" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T361" t="b">
         <v>1</v>
@@ -16098,7 +16098,7 @@
     <row r="362">
       <c r="B362" t="inlineStr">
         <is>
-          <t>2.7.7</t>
+          <t>2.7.8</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -16132,7 +16132,7 @@
         </is>
       </c>
       <c r="S362" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T362" t="b">
         <v>1</v>
@@ -16141,7 +16141,7 @@
     <row r="363">
       <c r="B363" t="inlineStr">
         <is>
-          <t>2.7.8</t>
+          <t>2.7.9</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -16170,7 +16170,7 @@
         </is>
       </c>
       <c r="S363" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T363" t="b">
         <v>1</v>
@@ -16179,7 +16179,7 @@
     <row r="364">
       <c r="B364" t="inlineStr">
         <is>
-          <t>2.7.9</t>
+          <t>2.7.10</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -16208,7 +16208,7 @@
         </is>
       </c>
       <c r="S364" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T364" t="b">
         <v>1</v>
@@ -16217,7 +16217,7 @@
     <row r="365">
       <c r="B365" t="inlineStr">
         <is>
-          <t>2.7.10</t>
+          <t>2.7.11</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -16251,7 +16251,7 @@
         </is>
       </c>
       <c r="S365" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T365" t="b">
         <v>1</v>
@@ -16260,7 +16260,7 @@
     <row r="366">
       <c r="B366" t="inlineStr">
         <is>
-          <t>2.7.11</t>
+          <t>2.7.12</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -16294,7 +16294,7 @@
         </is>
       </c>
       <c r="S366" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T366" t="b">
         <v>1</v>
@@ -16303,7 +16303,7 @@
     <row r="367">
       <c r="B367" t="inlineStr">
         <is>
-          <t>2.7.12</t>
+          <t>2.7.13</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -16337,7 +16337,7 @@
         </is>
       </c>
       <c r="S367" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T367" t="b">
         <v>1</v>
@@ -16346,7 +16346,7 @@
     <row r="368">
       <c r="B368" t="inlineStr">
         <is>
-          <t>2.7.13</t>
+          <t>2.7.14</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -16380,7 +16380,7 @@
         </is>
       </c>
       <c r="S368" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T368" t="b">
         <v>1</v>
@@ -16389,7 +16389,7 @@
     <row r="369">
       <c r="B369" t="inlineStr">
         <is>
-          <t>2.7.14</t>
+          <t>2.7.15</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -16418,7 +16418,7 @@
         </is>
       </c>
       <c r="S369" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T369" t="b">
         <v>1</v>
@@ -16427,7 +16427,7 @@
     <row r="370">
       <c r="B370" t="inlineStr">
         <is>
-          <t>2.7.15</t>
+          <t>2.7.16</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -16461,7 +16461,7 @@
         </is>
       </c>
       <c r="S370" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T370" t="b">
         <v>1</v>
@@ -27231,7 +27231,7 @@
     <row r="634">
       <c r="B634" t="inlineStr">
         <is>
-          <t>3.7.1</t>
+          <t>3.7.2</t>
         </is>
       </c>
       <c r="C634" t="inlineStr">
@@ -27265,7 +27265,7 @@
         </is>
       </c>
       <c r="S634" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T634" t="b">
         <v>1</v>
@@ -27274,7 +27274,7 @@
     <row r="635">
       <c r="B635" t="inlineStr">
         <is>
-          <t>3.7.2</t>
+          <t>3.7.3</t>
         </is>
       </c>
       <c r="C635" t="inlineStr">
@@ -27308,7 +27308,7 @@
         </is>
       </c>
       <c r="S635" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T635" t="b">
         <v>1</v>
@@ -27317,7 +27317,7 @@
     <row r="636">
       <c r="B636" t="inlineStr">
         <is>
-          <t>3.7.3</t>
+          <t>3.7.4</t>
         </is>
       </c>
       <c r="C636" t="inlineStr">
@@ -27351,7 +27351,7 @@
         </is>
       </c>
       <c r="S636" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T636" t="b">
         <v>1</v>
@@ -27360,7 +27360,7 @@
     <row r="637">
       <c r="B637" t="inlineStr">
         <is>
-          <t>3.7.4</t>
+          <t>3.7.5</t>
         </is>
       </c>
       <c r="C637" t="inlineStr">
@@ -27394,7 +27394,7 @@
         </is>
       </c>
       <c r="S637" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T637" t="b">
         <v>1</v>
@@ -27403,7 +27403,7 @@
     <row r="638">
       <c r="B638" t="inlineStr">
         <is>
-          <t>3.7.5</t>
+          <t>3.7.6</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
@@ -27437,7 +27437,7 @@
         </is>
       </c>
       <c r="S638" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T638" t="b">
         <v>1</v>
@@ -27446,7 +27446,7 @@
     <row r="639">
       <c r="B639" t="inlineStr">
         <is>
-          <t>3.7.6</t>
+          <t>3.7.7</t>
         </is>
       </c>
       <c r="C639" t="inlineStr">
@@ -27480,7 +27480,7 @@
         </is>
       </c>
       <c r="S639" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T639" t="b">
         <v>1</v>
@@ -27489,7 +27489,7 @@
     <row r="640">
       <c r="B640" t="inlineStr">
         <is>
-          <t>3.7.7</t>
+          <t>3.7.8</t>
         </is>
       </c>
       <c r="C640" t="inlineStr">
@@ -27523,7 +27523,7 @@
         </is>
       </c>
       <c r="S640" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T640" t="b">
         <v>1</v>
@@ -27532,7 +27532,7 @@
     <row r="641">
       <c r="B641" t="inlineStr">
         <is>
-          <t>3.7.8</t>
+          <t>3.7.9</t>
         </is>
       </c>
       <c r="C641" t="inlineStr">
@@ -27561,7 +27561,7 @@
         </is>
       </c>
       <c r="S641" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T641" t="b">
         <v>1</v>
@@ -27570,7 +27570,7 @@
     <row r="642">
       <c r="B642" t="inlineStr">
         <is>
-          <t>3.7.9</t>
+          <t>3.7.10</t>
         </is>
       </c>
       <c r="C642" t="inlineStr">
@@ -27599,7 +27599,7 @@
         </is>
       </c>
       <c r="S642" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T642" t="b">
         <v>1</v>
@@ -27608,7 +27608,7 @@
     <row r="643">
       <c r="B643" t="inlineStr">
         <is>
-          <t>3.7.10</t>
+          <t>3.7.11</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
@@ -27642,7 +27642,7 @@
         </is>
       </c>
       <c r="S643" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T643" t="b">
         <v>1</v>
@@ -27651,7 +27651,7 @@
     <row r="644">
       <c r="B644" t="inlineStr">
         <is>
-          <t>3.7.11</t>
+          <t>3.7.12</t>
         </is>
       </c>
       <c r="C644" t="inlineStr">
@@ -27685,7 +27685,7 @@
         </is>
       </c>
       <c r="S644" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T644" t="b">
         <v>1</v>
@@ -27694,7 +27694,7 @@
     <row r="645">
       <c r="B645" t="inlineStr">
         <is>
-          <t>3.7.12</t>
+          <t>3.7.13</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
@@ -27728,7 +27728,7 @@
         </is>
       </c>
       <c r="S645" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T645" t="b">
         <v>1</v>
@@ -27737,7 +27737,7 @@
     <row r="646">
       <c r="B646" t="inlineStr">
         <is>
-          <t>3.7.13</t>
+          <t>3.7.14</t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
@@ -27771,7 +27771,7 @@
         </is>
       </c>
       <c r="S646" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T646" t="b">
         <v>1</v>
@@ -27780,7 +27780,7 @@
     <row r="647">
       <c r="B647" t="inlineStr">
         <is>
-          <t>3.7.14</t>
+          <t>3.7.15</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
@@ -27809,7 +27809,7 @@
         </is>
       </c>
       <c r="S647" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T647" t="b">
         <v>1</v>
@@ -27818,7 +27818,7 @@
     <row r="648">
       <c r="B648" t="inlineStr">
         <is>
-          <t>3.7.15</t>
+          <t>3.7.16</t>
         </is>
       </c>
       <c r="C648" t="inlineStr">
@@ -27852,7 +27852,7 @@
         </is>
       </c>
       <c r="S648" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T648" t="b">
         <v>1</v>
@@ -38607,7 +38607,7 @@
     <row r="912">
       <c r="B912" t="inlineStr">
         <is>
-          <t>4.7.1</t>
+          <t>4.7.2</t>
         </is>
       </c>
       <c r="C912" t="inlineStr">
@@ -38641,7 +38641,7 @@
         </is>
       </c>
       <c r="S912" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T912" t="b">
         <v>1</v>
@@ -38650,7 +38650,7 @@
     <row r="913">
       <c r="B913" t="inlineStr">
         <is>
-          <t>4.7.2</t>
+          <t>4.7.3</t>
         </is>
       </c>
       <c r="C913" t="inlineStr">
@@ -38679,7 +38679,7 @@
         </is>
       </c>
       <c r="S913" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T913" t="b">
         <v>1</v>
@@ -38688,7 +38688,7 @@
     <row r="914">
       <c r="B914" t="inlineStr">
         <is>
-          <t>4.7.3</t>
+          <t>4.7.4</t>
         </is>
       </c>
       <c r="C914" t="inlineStr">
@@ -38717,7 +38717,7 @@
         </is>
       </c>
       <c r="S914" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T914" t="b">
         <v>1</v>
@@ -38726,7 +38726,7 @@
     <row r="915">
       <c r="B915" t="inlineStr">
         <is>
-          <t>4.7.4</t>
+          <t>4.7.5</t>
         </is>
       </c>
       <c r="C915" t="inlineStr">
@@ -38760,7 +38760,7 @@
         </is>
       </c>
       <c r="S915" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T915" t="b">
         <v>1</v>
@@ -38769,7 +38769,7 @@
     <row r="916">
       <c r="B916" t="inlineStr">
         <is>
-          <t>4.7.5</t>
+          <t>4.7.6</t>
         </is>
       </c>
       <c r="C916" t="inlineStr">
@@ -38803,7 +38803,7 @@
         </is>
       </c>
       <c r="S916" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T916" t="b">
         <v>1</v>
@@ -38812,7 +38812,7 @@
     <row r="917">
       <c r="B917" t="inlineStr">
         <is>
-          <t>4.7.6</t>
+          <t>4.7.7</t>
         </is>
       </c>
       <c r="C917" t="inlineStr">
@@ -38846,7 +38846,7 @@
         </is>
       </c>
       <c r="S917" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T917" t="b">
         <v>1</v>
@@ -38855,7 +38855,7 @@
     <row r="918">
       <c r="B918" t="inlineStr">
         <is>
-          <t>4.7.7</t>
+          <t>4.7.8</t>
         </is>
       </c>
       <c r="C918" t="inlineStr">
@@ -38889,7 +38889,7 @@
         </is>
       </c>
       <c r="S918" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T918" t="b">
         <v>1</v>
@@ -38898,7 +38898,7 @@
     <row r="919">
       <c r="B919" t="inlineStr">
         <is>
-          <t>4.7.8</t>
+          <t>4.7.9</t>
         </is>
       </c>
       <c r="C919" t="inlineStr">
@@ -38927,7 +38927,7 @@
         </is>
       </c>
       <c r="S919" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T919" t="b">
         <v>1</v>
@@ -38936,7 +38936,7 @@
     <row r="920">
       <c r="B920" t="inlineStr">
         <is>
-          <t>4.7.9</t>
+          <t>4.7.10</t>
         </is>
       </c>
       <c r="C920" t="inlineStr">
@@ -38965,7 +38965,7 @@
         </is>
       </c>
       <c r="S920" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T920" t="b">
         <v>1</v>
@@ -38974,7 +38974,7 @@
     <row r="921">
       <c r="B921" t="inlineStr">
         <is>
-          <t>4.7.10</t>
+          <t>4.7.11</t>
         </is>
       </c>
       <c r="C921" t="inlineStr">
@@ -39003,7 +39003,7 @@
         </is>
       </c>
       <c r="S921" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T921" t="b">
         <v>1</v>
@@ -39012,7 +39012,7 @@
     <row r="922">
       <c r="B922" t="inlineStr">
         <is>
-          <t>4.7.11</t>
+          <t>4.7.12</t>
         </is>
       </c>
       <c r="C922" t="inlineStr">
@@ -39046,7 +39046,7 @@
         </is>
       </c>
       <c r="S922" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T922" t="b">
         <v>1</v>
@@ -39055,7 +39055,7 @@
     <row r="923">
       <c r="B923" t="inlineStr">
         <is>
-          <t>4.7.12</t>
+          <t>4.7.13</t>
         </is>
       </c>
       <c r="C923" t="inlineStr">
@@ -39089,7 +39089,7 @@
         </is>
       </c>
       <c r="S923" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T923" t="b">
         <v>1</v>
@@ -39098,7 +39098,7 @@
     <row r="924">
       <c r="B924" t="inlineStr">
         <is>
-          <t>4.7.13</t>
+          <t>4.7.14</t>
         </is>
       </c>
       <c r="C924" t="inlineStr">
@@ -39132,7 +39132,7 @@
         </is>
       </c>
       <c r="S924" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T924" t="b">
         <v>1</v>
@@ -39141,7 +39141,7 @@
     <row r="925">
       <c r="B925" t="inlineStr">
         <is>
-          <t>4.7.14</t>
+          <t>4.7.15</t>
         </is>
       </c>
       <c r="C925" t="inlineStr">
@@ -39170,7 +39170,7 @@
         </is>
       </c>
       <c r="S925" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T925" t="b">
         <v>1</v>
@@ -39179,7 +39179,7 @@
     <row r="926">
       <c r="B926" t="inlineStr">
         <is>
-          <t>4.7.15</t>
+          <t>4.7.16</t>
         </is>
       </c>
       <c r="C926" t="inlineStr">
@@ -39213,7 +39213,7 @@
         </is>
       </c>
       <c r="S926" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T926" t="b">
         <v>1</v>
@@ -49743,7 +49743,7 @@
     <row r="1190">
       <c r="B1190" t="inlineStr">
         <is>
-          <t>5.7.1</t>
+          <t>5.7.2</t>
         </is>
       </c>
       <c r="C1190" t="inlineStr">
@@ -49777,7 +49777,7 @@
         </is>
       </c>
       <c r="S1190" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T1190" t="b">
         <v>1</v>
@@ -49786,7 +49786,7 @@
     <row r="1191">
       <c r="B1191" t="inlineStr">
         <is>
-          <t>5.7.2</t>
+          <t>5.7.3</t>
         </is>
       </c>
       <c r="C1191" t="inlineStr">
@@ -49815,7 +49815,7 @@
         </is>
       </c>
       <c r="S1191" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T1191" t="b">
         <v>1</v>
@@ -49824,7 +49824,7 @@
     <row r="1192">
       <c r="B1192" t="inlineStr">
         <is>
-          <t>5.7.3</t>
+          <t>5.7.4</t>
         </is>
       </c>
       <c r="C1192" t="inlineStr">
@@ -49853,7 +49853,7 @@
         </is>
       </c>
       <c r="S1192" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T1192" t="b">
         <v>1</v>
@@ -49862,7 +49862,7 @@
     <row r="1193">
       <c r="B1193" t="inlineStr">
         <is>
-          <t>5.7.4</t>
+          <t>5.7.5</t>
         </is>
       </c>
       <c r="C1193" t="inlineStr">
@@ -49891,7 +49891,7 @@
         </is>
       </c>
       <c r="S1193" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T1193" t="b">
         <v>1</v>
@@ -49900,7 +49900,7 @@
     <row r="1194">
       <c r="B1194" t="inlineStr">
         <is>
-          <t>5.7.5</t>
+          <t>5.7.6</t>
         </is>
       </c>
       <c r="C1194" t="inlineStr">
@@ -49929,7 +49929,7 @@
         </is>
       </c>
       <c r="S1194" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T1194" t="b">
         <v>1</v>
@@ -49938,7 +49938,7 @@
     <row r="1195">
       <c r="B1195" t="inlineStr">
         <is>
-          <t>5.7.6</t>
+          <t>5.7.7</t>
         </is>
       </c>
       <c r="C1195" t="inlineStr">
@@ -49967,7 +49967,7 @@
         </is>
       </c>
       <c r="S1195" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T1195" t="b">
         <v>1</v>
@@ -49976,7 +49976,7 @@
     <row r="1196">
       <c r="B1196" t="inlineStr">
         <is>
-          <t>5.7.7</t>
+          <t>5.7.8</t>
         </is>
       </c>
       <c r="C1196" t="inlineStr">
@@ -50010,7 +50010,7 @@
         </is>
       </c>
       <c r="S1196" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T1196" t="b">
         <v>1</v>
@@ -50019,7 +50019,7 @@
     <row r="1197">
       <c r="B1197" t="inlineStr">
         <is>
-          <t>5.7.8</t>
+          <t>5.7.9</t>
         </is>
       </c>
       <c r="C1197" t="inlineStr">
@@ -50048,7 +50048,7 @@
         </is>
       </c>
       <c r="S1197" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T1197" t="b">
         <v>1</v>
@@ -50057,7 +50057,7 @@
     <row r="1198">
       <c r="B1198" t="inlineStr">
         <is>
-          <t>5.7.9</t>
+          <t>5.7.10</t>
         </is>
       </c>
       <c r="C1198" t="inlineStr">
@@ -50086,7 +50086,7 @@
         </is>
       </c>
       <c r="S1198" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T1198" t="b">
         <v>1</v>
@@ -50095,7 +50095,7 @@
     <row r="1199">
       <c r="B1199" t="inlineStr">
         <is>
-          <t>5.7.10</t>
+          <t>5.7.11</t>
         </is>
       </c>
       <c r="C1199" t="inlineStr">
@@ -50124,7 +50124,7 @@
         </is>
       </c>
       <c r="S1199" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T1199" t="b">
         <v>1</v>
@@ -50133,7 +50133,7 @@
     <row r="1200">
       <c r="B1200" t="inlineStr">
         <is>
-          <t>5.7.11</t>
+          <t>5.7.12</t>
         </is>
       </c>
       <c r="C1200" t="inlineStr">
@@ -50162,7 +50162,7 @@
         </is>
       </c>
       <c r="S1200" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T1200" t="b">
         <v>1</v>
@@ -50171,7 +50171,7 @@
     <row r="1201">
       <c r="B1201" t="inlineStr">
         <is>
-          <t>5.7.12</t>
+          <t>5.7.13</t>
         </is>
       </c>
       <c r="C1201" t="inlineStr">
@@ -50200,7 +50200,7 @@
         </is>
       </c>
       <c r="S1201" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T1201" t="b">
         <v>1</v>
@@ -50209,7 +50209,7 @@
     <row r="1202">
       <c r="B1202" t="inlineStr">
         <is>
-          <t>5.7.13</t>
+          <t>5.7.14</t>
         </is>
       </c>
       <c r="C1202" t="inlineStr">
@@ -50238,7 +50238,7 @@
         </is>
       </c>
       <c r="S1202" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T1202" t="b">
         <v>1</v>
@@ -50247,7 +50247,7 @@
     <row r="1203">
       <c r="B1203" t="inlineStr">
         <is>
-          <t>5.7.14</t>
+          <t>5.7.15</t>
         </is>
       </c>
       <c r="C1203" t="inlineStr">
@@ -50281,7 +50281,7 @@
         </is>
       </c>
       <c r="S1203" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T1203" t="b">
         <v>1</v>
@@ -50290,7 +50290,7 @@
     <row r="1204">
       <c r="B1204" t="inlineStr">
         <is>
-          <t>5.7.15</t>
+          <t>5.7.16</t>
         </is>
       </c>
       <c r="C1204" t="inlineStr">
@@ -50319,7 +50319,7 @@
         </is>
       </c>
       <c r="S1204" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T1204" t="b">
         <v>1</v>
@@ -60724,7 +60724,7 @@
     <row r="1468">
       <c r="B1468" t="inlineStr">
         <is>
-          <t>6.7.1</t>
+          <t>6.7.2</t>
         </is>
       </c>
       <c r="C1468" t="inlineStr">
@@ -60758,7 +60758,7 @@
         </is>
       </c>
       <c r="S1468" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T1468" t="b">
         <v>1</v>
@@ -60767,7 +60767,7 @@
     <row r="1469">
       <c r="B1469" t="inlineStr">
         <is>
-          <t>6.7.2</t>
+          <t>6.7.3</t>
         </is>
       </c>
       <c r="C1469" t="inlineStr">
@@ -60801,7 +60801,7 @@
         </is>
       </c>
       <c r="S1469" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T1469" t="b">
         <v>1</v>
@@ -60810,7 +60810,7 @@
     <row r="1470">
       <c r="B1470" t="inlineStr">
         <is>
-          <t>6.7.3</t>
+          <t>6.7.4</t>
         </is>
       </c>
       <c r="C1470" t="inlineStr">
@@ -60844,7 +60844,7 @@
         </is>
       </c>
       <c r="S1470" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T1470" t="b">
         <v>1</v>
@@ -60853,7 +60853,7 @@
     <row r="1471">
       <c r="B1471" t="inlineStr">
         <is>
-          <t>6.7.4</t>
+          <t>6.7.5</t>
         </is>
       </c>
       <c r="C1471" t="inlineStr">
@@ -60887,7 +60887,7 @@
         </is>
       </c>
       <c r="S1471" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T1471" t="b">
         <v>1</v>
@@ -60896,7 +60896,7 @@
     <row r="1472">
       <c r="B1472" t="inlineStr">
         <is>
-          <t>6.7.5</t>
+          <t>6.7.6</t>
         </is>
       </c>
       <c r="C1472" t="inlineStr">
@@ -60925,7 +60925,7 @@
         </is>
       </c>
       <c r="S1472" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T1472" t="b">
         <v>1</v>
@@ -60934,7 +60934,7 @@
     <row r="1473">
       <c r="B1473" t="inlineStr">
         <is>
-          <t>6.7.6</t>
+          <t>6.7.7</t>
         </is>
       </c>
       <c r="C1473" t="inlineStr">
@@ -60968,7 +60968,7 @@
         </is>
       </c>
       <c r="S1473" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T1473" t="b">
         <v>1</v>
@@ -60977,7 +60977,7 @@
     <row r="1474">
       <c r="B1474" t="inlineStr">
         <is>
-          <t>6.7.7</t>
+          <t>6.7.8</t>
         </is>
       </c>
       <c r="C1474" t="inlineStr">
@@ -61011,7 +61011,7 @@
         </is>
       </c>
       <c r="S1474" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T1474" t="b">
         <v>1</v>
@@ -61020,7 +61020,7 @@
     <row r="1475">
       <c r="B1475" t="inlineStr">
         <is>
-          <t>6.7.8</t>
+          <t>6.7.9</t>
         </is>
       </c>
       <c r="C1475" t="inlineStr">
@@ -61049,7 +61049,7 @@
         </is>
       </c>
       <c r="S1475" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T1475" t="b">
         <v>1</v>
@@ -61058,7 +61058,7 @@
     <row r="1476">
       <c r="B1476" t="inlineStr">
         <is>
-          <t>6.7.9</t>
+          <t>6.7.10</t>
         </is>
       </c>
       <c r="C1476" t="inlineStr">
@@ -61087,7 +61087,7 @@
         </is>
       </c>
       <c r="S1476" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T1476" t="b">
         <v>1</v>
@@ -61096,7 +61096,7 @@
     <row r="1477">
       <c r="B1477" t="inlineStr">
         <is>
-          <t>6.7.10</t>
+          <t>6.7.11</t>
         </is>
       </c>
       <c r="C1477" t="inlineStr">
@@ -61125,7 +61125,7 @@
         </is>
       </c>
       <c r="S1477" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T1477" t="b">
         <v>1</v>
@@ -61134,7 +61134,7 @@
     <row r="1478">
       <c r="B1478" t="inlineStr">
         <is>
-          <t>6.7.11</t>
+          <t>6.7.12</t>
         </is>
       </c>
       <c r="C1478" t="inlineStr">
@@ -61168,7 +61168,7 @@
         </is>
       </c>
       <c r="S1478" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T1478" t="b">
         <v>1</v>
@@ -61177,7 +61177,7 @@
     <row r="1479">
       <c r="B1479" t="inlineStr">
         <is>
-          <t>6.7.12</t>
+          <t>6.7.13</t>
         </is>
       </c>
       <c r="C1479" t="inlineStr">
@@ -61211,7 +61211,7 @@
         </is>
       </c>
       <c r="S1479" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T1479" t="b">
         <v>1</v>
@@ -61220,7 +61220,7 @@
     <row r="1480">
       <c r="B1480" t="inlineStr">
         <is>
-          <t>6.7.13</t>
+          <t>6.7.14</t>
         </is>
       </c>
       <c r="C1480" t="inlineStr">
@@ -61254,7 +61254,7 @@
         </is>
       </c>
       <c r="S1480" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T1480" t="b">
         <v>1</v>
@@ -61263,7 +61263,7 @@
     <row r="1481">
       <c r="B1481" t="inlineStr">
         <is>
-          <t>6.7.14</t>
+          <t>6.7.15</t>
         </is>
       </c>
       <c r="C1481" t="inlineStr">
@@ -61297,7 +61297,7 @@
         </is>
       </c>
       <c r="S1481" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T1481" t="b">
         <v>1</v>
@@ -61306,7 +61306,7 @@
     <row r="1482">
       <c r="B1482" t="inlineStr">
         <is>
-          <t>6.7.15</t>
+          <t>6.7.16</t>
         </is>
       </c>
       <c r="C1482" t="inlineStr">
@@ -61340,7 +61340,7 @@
         </is>
       </c>
       <c r="S1482" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T1482" t="b">
         <v>1</v>
@@ -71875,7 +71875,7 @@
     <row r="1746">
       <c r="B1746" t="inlineStr">
         <is>
-          <t>7.7.1</t>
+          <t>7.7.2</t>
         </is>
       </c>
       <c r="C1746" t="inlineStr">
@@ -71909,7 +71909,7 @@
         </is>
       </c>
       <c r="S1746" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T1746" t="b">
         <v>1</v>
@@ -71918,7 +71918,7 @@
     <row r="1747">
       <c r="B1747" t="inlineStr">
         <is>
-          <t>7.7.2</t>
+          <t>7.7.3</t>
         </is>
       </c>
       <c r="C1747" t="inlineStr">
@@ -71952,7 +71952,7 @@
         </is>
       </c>
       <c r="S1747" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T1747" t="b">
         <v>1</v>
@@ -71961,7 +71961,7 @@
     <row r="1748">
       <c r="B1748" t="inlineStr">
         <is>
-          <t>7.7.3</t>
+          <t>7.7.4</t>
         </is>
       </c>
       <c r="C1748" t="inlineStr">
@@ -71995,7 +71995,7 @@
         </is>
       </c>
       <c r="S1748" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T1748" t="b">
         <v>1</v>
@@ -72004,7 +72004,7 @@
     <row r="1749">
       <c r="B1749" t="inlineStr">
         <is>
-          <t>7.7.4</t>
+          <t>7.7.5</t>
         </is>
       </c>
       <c r="C1749" t="inlineStr">
@@ -72038,7 +72038,7 @@
         </is>
       </c>
       <c r="S1749" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T1749" t="b">
         <v>1</v>
@@ -72047,7 +72047,7 @@
     <row r="1750">
       <c r="B1750" t="inlineStr">
         <is>
-          <t>7.7.5</t>
+          <t>7.7.6</t>
         </is>
       </c>
       <c r="C1750" t="inlineStr">
@@ -72076,7 +72076,7 @@
         </is>
       </c>
       <c r="S1750" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T1750" t="b">
         <v>1</v>
@@ -72085,7 +72085,7 @@
     <row r="1751">
       <c r="B1751" t="inlineStr">
         <is>
-          <t>7.7.6</t>
+          <t>7.7.7</t>
         </is>
       </c>
       <c r="C1751" t="inlineStr">
@@ -72119,7 +72119,7 @@
         </is>
       </c>
       <c r="S1751" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T1751" t="b">
         <v>1</v>
@@ -72128,7 +72128,7 @@
     <row r="1752">
       <c r="B1752" t="inlineStr">
         <is>
-          <t>7.7.7</t>
+          <t>7.7.8</t>
         </is>
       </c>
       <c r="C1752" t="inlineStr">
@@ -72162,7 +72162,7 @@
         </is>
       </c>
       <c r="S1752" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T1752" t="b">
         <v>1</v>
@@ -72171,7 +72171,7 @@
     <row r="1753">
       <c r="B1753" t="inlineStr">
         <is>
-          <t>7.7.8</t>
+          <t>7.7.9</t>
         </is>
       </c>
       <c r="C1753" t="inlineStr">
@@ -72200,7 +72200,7 @@
         </is>
       </c>
       <c r="S1753" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T1753" t="b">
         <v>1</v>
@@ -72209,7 +72209,7 @@
     <row r="1754">
       <c r="B1754" t="inlineStr">
         <is>
-          <t>7.7.9</t>
+          <t>7.7.10</t>
         </is>
       </c>
       <c r="C1754" t="inlineStr">
@@ -72238,7 +72238,7 @@
         </is>
       </c>
       <c r="S1754" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T1754" t="b">
         <v>1</v>
@@ -72247,7 +72247,7 @@
     <row r="1755">
       <c r="B1755" t="inlineStr">
         <is>
-          <t>7.7.10</t>
+          <t>7.7.11</t>
         </is>
       </c>
       <c r="C1755" t="inlineStr">
@@ -72276,7 +72276,7 @@
         </is>
       </c>
       <c r="S1755" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T1755" t="b">
         <v>1</v>
@@ -72285,7 +72285,7 @@
     <row r="1756">
       <c r="B1756" t="inlineStr">
         <is>
-          <t>7.7.11</t>
+          <t>7.7.12</t>
         </is>
       </c>
       <c r="C1756" t="inlineStr">
@@ -72319,7 +72319,7 @@
         </is>
       </c>
       <c r="S1756" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T1756" t="b">
         <v>1</v>
@@ -72328,7 +72328,7 @@
     <row r="1757">
       <c r="B1757" t="inlineStr">
         <is>
-          <t>7.7.12</t>
+          <t>7.7.13</t>
         </is>
       </c>
       <c r="C1757" t="inlineStr">
@@ -72362,7 +72362,7 @@
         </is>
       </c>
       <c r="S1757" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T1757" t="b">
         <v>1</v>
@@ -72371,7 +72371,7 @@
     <row r="1758">
       <c r="B1758" t="inlineStr">
         <is>
-          <t>7.7.13</t>
+          <t>7.7.14</t>
         </is>
       </c>
       <c r="C1758" t="inlineStr">
@@ -72405,7 +72405,7 @@
         </is>
       </c>
       <c r="S1758" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T1758" t="b">
         <v>1</v>
@@ -72414,7 +72414,7 @@
     <row r="1759">
       <c r="B1759" t="inlineStr">
         <is>
-          <t>7.7.14</t>
+          <t>7.7.15</t>
         </is>
       </c>
       <c r="C1759" t="inlineStr">
@@ -72448,7 +72448,7 @@
         </is>
       </c>
       <c r="S1759" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T1759" t="b">
         <v>1</v>
@@ -72457,7 +72457,7 @@
     <row r="1760">
       <c r="B1760" t="inlineStr">
         <is>
-          <t>7.7.15</t>
+          <t>7.7.16</t>
         </is>
       </c>
       <c r="C1760" t="inlineStr">
@@ -72491,7 +72491,7 @@
         </is>
       </c>
       <c r="S1760" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T1760" t="b">
         <v>1</v>
@@ -83011,7 +83011,7 @@
     <row r="2024">
       <c r="B2024" t="inlineStr">
         <is>
-          <t>8.7.1</t>
+          <t>8.7.2</t>
         </is>
       </c>
       <c r="C2024" t="inlineStr">
@@ -83045,7 +83045,7 @@
         </is>
       </c>
       <c r="S2024" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T2024" t="b">
         <v>1</v>
@@ -83054,7 +83054,7 @@
     <row r="2025">
       <c r="B2025" t="inlineStr">
         <is>
-          <t>8.7.2</t>
+          <t>8.7.3</t>
         </is>
       </c>
       <c r="C2025" t="inlineStr">
@@ -83088,7 +83088,7 @@
         </is>
       </c>
       <c r="S2025" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T2025" t="b">
         <v>1</v>
@@ -83097,7 +83097,7 @@
     <row r="2026">
       <c r="B2026" t="inlineStr">
         <is>
-          <t>8.7.3</t>
+          <t>8.7.4</t>
         </is>
       </c>
       <c r="C2026" t="inlineStr">
@@ -83131,7 +83131,7 @@
         </is>
       </c>
       <c r="S2026" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T2026" t="b">
         <v>1</v>
@@ -83140,7 +83140,7 @@
     <row r="2027">
       <c r="B2027" t="inlineStr">
         <is>
-          <t>8.7.4</t>
+          <t>8.7.5</t>
         </is>
       </c>
       <c r="C2027" t="inlineStr">
@@ -83174,7 +83174,7 @@
         </is>
       </c>
       <c r="S2027" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T2027" t="b">
         <v>1</v>
@@ -83183,7 +83183,7 @@
     <row r="2028">
       <c r="B2028" t="inlineStr">
         <is>
-          <t>8.7.5</t>
+          <t>8.7.6</t>
         </is>
       </c>
       <c r="C2028" t="inlineStr">
@@ -83212,7 +83212,7 @@
         </is>
       </c>
       <c r="S2028" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T2028" t="b">
         <v>1</v>
@@ -83221,7 +83221,7 @@
     <row r="2029">
       <c r="B2029" t="inlineStr">
         <is>
-          <t>8.7.6</t>
+          <t>8.7.7</t>
         </is>
       </c>
       <c r="C2029" t="inlineStr">
@@ -83255,7 +83255,7 @@
         </is>
       </c>
       <c r="S2029" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T2029" t="b">
         <v>1</v>
@@ -83264,7 +83264,7 @@
     <row r="2030">
       <c r="B2030" t="inlineStr">
         <is>
-          <t>8.7.7</t>
+          <t>8.7.8</t>
         </is>
       </c>
       <c r="C2030" t="inlineStr">
@@ -83298,7 +83298,7 @@
         </is>
       </c>
       <c r="S2030" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T2030" t="b">
         <v>1</v>
@@ -83307,7 +83307,7 @@
     <row r="2031">
       <c r="B2031" t="inlineStr">
         <is>
-          <t>8.7.8</t>
+          <t>8.7.9</t>
         </is>
       </c>
       <c r="C2031" t="inlineStr">
@@ -83336,7 +83336,7 @@
         </is>
       </c>
       <c r="S2031" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T2031" t="b">
         <v>1</v>
@@ -83345,7 +83345,7 @@
     <row r="2032">
       <c r="B2032" t="inlineStr">
         <is>
-          <t>8.7.9</t>
+          <t>8.7.10</t>
         </is>
       </c>
       <c r="C2032" t="inlineStr">
@@ -83374,7 +83374,7 @@
         </is>
       </c>
       <c r="S2032" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T2032" t="b">
         <v>1</v>
@@ -83383,7 +83383,7 @@
     <row r="2033">
       <c r="B2033" t="inlineStr">
         <is>
-          <t>8.7.10</t>
+          <t>8.7.11</t>
         </is>
       </c>
       <c r="C2033" t="inlineStr">
@@ -83412,7 +83412,7 @@
         </is>
       </c>
       <c r="S2033" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T2033" t="b">
         <v>1</v>
@@ -83421,7 +83421,7 @@
     <row r="2034">
       <c r="B2034" t="inlineStr">
         <is>
-          <t>8.7.11</t>
+          <t>8.7.12</t>
         </is>
       </c>
       <c r="C2034" t="inlineStr">
@@ -83455,7 +83455,7 @@
         </is>
       </c>
       <c r="S2034" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T2034" t="b">
         <v>1</v>
@@ -83464,7 +83464,7 @@
     <row r="2035">
       <c r="B2035" t="inlineStr">
         <is>
-          <t>8.7.12</t>
+          <t>8.7.13</t>
         </is>
       </c>
       <c r="C2035" t="inlineStr">
@@ -83498,7 +83498,7 @@
         </is>
       </c>
       <c r="S2035" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="T2035" t="b">
         <v>1</v>
@@ -83507,7 +83507,7 @@
     <row r="2036">
       <c r="B2036" t="inlineStr">
         <is>
-          <t>8.7.13</t>
+          <t>8.7.14</t>
         </is>
       </c>
       <c r="C2036" t="inlineStr">
@@ -83541,7 +83541,7 @@
         </is>
       </c>
       <c r="S2036" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T2036" t="b">
         <v>1</v>
@@ -83550,7 +83550,7 @@
     <row r="2037">
       <c r="B2037" t="inlineStr">
         <is>
-          <t>8.7.14</t>
+          <t>8.7.15</t>
         </is>
       </c>
       <c r="C2037" t="inlineStr">
@@ -83584,7 +83584,7 @@
         </is>
       </c>
       <c r="S2037" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="T2037" t="b">
         <v>1</v>
@@ -83593,7 +83593,7 @@
     <row r="2038">
       <c r="B2038" t="inlineStr">
         <is>
-          <t>8.7.15</t>
+          <t>8.7.16</t>
         </is>
       </c>
       <c r="C2038" t="inlineStr">
@@ -83627,7 +83627,7 @@
         </is>
       </c>
       <c r="S2038" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="T2038" t="b">
         <v>1</v>
@@ -91764,6 +91764,350 @@
         <v>12</v>
       </c>
       <c r="T2241" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2242">
+      <c r="B2242" t="inlineStr">
+        <is>
+          <t>1.7.1</t>
+        </is>
+      </c>
+      <c r="C2242" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="D2242" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2242" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2242" t="inlineStr">
+        <is>
+          <t>De echte klimaatanalyse</t>
+        </is>
+      </c>
+      <c r="I2242" t="inlineStr">
+        <is>
+          <t>wat-opkomt/klimaat-de-echte-analyse.html</t>
+        </is>
+      </c>
+      <c r="R2242" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2242" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2242" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2243">
+      <c r="B2243" t="inlineStr">
+        <is>
+          <t>2.7.1</t>
+        </is>
+      </c>
+      <c r="C2243" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="D2243" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2243" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2243" t="inlineStr">
+        <is>
+          <t>De echte klimaatanalyse</t>
+        </is>
+      </c>
+      <c r="I2243" t="inlineStr">
+        <is>
+          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+        </is>
+      </c>
+      <c r="R2243" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2243" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2243" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2244">
+      <c r="B2244" t="inlineStr">
+        <is>
+          <t>3.7.1</t>
+        </is>
+      </c>
+      <c r="C2244" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="D2244" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2244" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2244" t="inlineStr">
+        <is>
+          <t>De echte klimaatanalyse</t>
+        </is>
+      </c>
+      <c r="I2244" t="inlineStr">
+        <is>
+          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+        </is>
+      </c>
+      <c r="R2244" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2244" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2244" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2245">
+      <c r="B2245" t="inlineStr">
+        <is>
+          <t>4.7.1</t>
+        </is>
+      </c>
+      <c r="C2245" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="D2245" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2245" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2245" t="inlineStr">
+        <is>
+          <t>De echte klimaatanalyse</t>
+        </is>
+      </c>
+      <c r="I2245" t="inlineStr">
+        <is>
+          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+        </is>
+      </c>
+      <c r="R2245" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2245" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2245" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2246">
+      <c r="B2246" t="inlineStr">
+        <is>
+          <t>5.7.1</t>
+        </is>
+      </c>
+      <c r="C2246" t="inlineStr">
+        <is>
+          <t>5.7</t>
+        </is>
+      </c>
+      <c r="D2246" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="E2246" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2246" t="inlineStr">
+        <is>
+          <t>De echte klimaatanalyse</t>
+        </is>
+      </c>
+      <c r="I2246" t="inlineStr">
+        <is>
+          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+        </is>
+      </c>
+      <c r="R2246" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2246" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2246" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2247">
+      <c r="B2247" t="inlineStr">
+        <is>
+          <t>6.7.1</t>
+        </is>
+      </c>
+      <c r="C2247" t="inlineStr">
+        <is>
+          <t>6.7</t>
+        </is>
+      </c>
+      <c r="D2247" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="E2247" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2247" t="inlineStr">
+        <is>
+          <t>De echte klimaatanalyse</t>
+        </is>
+      </c>
+      <c r="I2247" t="inlineStr">
+        <is>
+          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+        </is>
+      </c>
+      <c r="R2247" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2247" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2247" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2248">
+      <c r="B2248" t="inlineStr">
+        <is>
+          <t>7.7.1</t>
+        </is>
+      </c>
+      <c r="C2248" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
+      </c>
+      <c r="D2248" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="E2248" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2248" t="inlineStr">
+        <is>
+          <t>De echte klimaatanalyse</t>
+        </is>
+      </c>
+      <c r="I2248" t="inlineStr">
+        <is>
+          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+        </is>
+      </c>
+      <c r="R2248" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2248" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2248" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2249">
+      <c r="B2249" t="inlineStr">
+        <is>
+          <t>8.7.1</t>
+        </is>
+      </c>
+      <c r="C2249" t="inlineStr">
+        <is>
+          <t>8.7</t>
+        </is>
+      </c>
+      <c r="D2249" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="E2249" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2249" t="inlineStr">
+        <is>
+          <t>De echte klimaatanalyse</t>
+        </is>
+      </c>
+      <c r="I2249" t="inlineStr">
+        <is>
+          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+        </is>
+      </c>
+      <c r="R2249" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2249" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2249" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Delen-dropdown via xlsx (1.18 per taal) + menu-loader herkent naam en zet data-ov-deel-trigger
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR2249"/>
+  <dimension ref="B2:AR2257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -92111,6 +92111,310 @@
         <v>1</v>
       </c>
     </row>
+    <row r="2250">
+      <c r="B2250" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="C2250" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2250" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2250" t="inlineStr">
+        <is>
+          <t>ingang</t>
+        </is>
+      </c>
+      <c r="F2250" t="inlineStr">
+        <is>
+          <t>Delen</t>
+        </is>
+      </c>
+      <c r="R2250" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2250" t="n">
+        <v>18</v>
+      </c>
+      <c r="T2250" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2251">
+      <c r="B2251" t="inlineStr">
+        <is>
+          <t>2.18</t>
+        </is>
+      </c>
+      <c r="C2251" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D2251" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2251" t="inlineStr">
+        <is>
+          <t>ingang</t>
+        </is>
+      </c>
+      <c r="F2251" t="inlineStr">
+        <is>
+          <t>Teilen</t>
+        </is>
+      </c>
+      <c r="R2251" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2251" t="n">
+        <v>18</v>
+      </c>
+      <c r="T2251" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2252">
+      <c r="B2252" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="C2252" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D2252" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2252" t="inlineStr">
+        <is>
+          <t>ingang</t>
+        </is>
+      </c>
+      <c r="F2252" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+      <c r="R2252" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2252" t="n">
+        <v>18</v>
+      </c>
+      <c r="T2252" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2253">
+      <c r="B2253" t="inlineStr">
+        <is>
+          <t>4.18</t>
+        </is>
+      </c>
+      <c r="C2253" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D2253" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2253" t="inlineStr">
+        <is>
+          <t>ingang</t>
+        </is>
+      </c>
+      <c r="F2253" t="inlineStr">
+        <is>
+          <t>Поделиться</t>
+        </is>
+      </c>
+      <c r="R2253" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2253" t="n">
+        <v>18</v>
+      </c>
+      <c r="T2253" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2254">
+      <c r="B2254" t="inlineStr">
+        <is>
+          <t>5.18</t>
+        </is>
+      </c>
+      <c r="C2254" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D2254" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="E2254" t="inlineStr">
+        <is>
+          <t>ingang</t>
+        </is>
+      </c>
+      <c r="F2254" t="inlineStr">
+        <is>
+          <t>Partager</t>
+        </is>
+      </c>
+      <c r="R2254" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2254" t="n">
+        <v>18</v>
+      </c>
+      <c r="T2254" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2255">
+      <c r="B2255" t="inlineStr">
+        <is>
+          <t>6.18</t>
+        </is>
+      </c>
+      <c r="C2255" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D2255" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="E2255" t="inlineStr">
+        <is>
+          <t>ingang</t>
+        </is>
+      </c>
+      <c r="F2255" t="inlineStr">
+        <is>
+          <t>Compartir</t>
+        </is>
+      </c>
+      <c r="R2255" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2255" t="n">
+        <v>18</v>
+      </c>
+      <c r="T2255" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2256">
+      <c r="B2256" t="inlineStr">
+        <is>
+          <t>7.18</t>
+        </is>
+      </c>
+      <c r="C2256" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D2256" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="E2256" t="inlineStr">
+        <is>
+          <t>ingang</t>
+        </is>
+      </c>
+      <c r="F2256" t="inlineStr">
+        <is>
+          <t>Condividi</t>
+        </is>
+      </c>
+      <c r="R2256" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2256" t="n">
+        <v>18</v>
+      </c>
+      <c r="T2256" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2257">
+      <c r="B2257" t="inlineStr">
+        <is>
+          <t>8.18</t>
+        </is>
+      </c>
+      <c r="C2257" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D2257" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="E2257" t="inlineStr">
+        <is>
+          <t>ingang</t>
+        </is>
+      </c>
+      <c r="F2257" t="inlineStr">
+        <is>
+          <t>Partilhar</t>
+        </is>
+      </c>
+      <c r="R2257" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2257" t="n">
+        <v>18</v>
+      </c>
+      <c r="T2257" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B2:AR65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Delen-dropdown: 7 acties in xlsx (1.18.1-7), taal-dupliceer verwijderd uit menu-loader
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR2257"/>
+  <dimension ref="B2:AR2313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -92415,6 +92415,2414 @@
         <v>1</v>
       </c>
     </row>
+    <row r="2258">
+      <c r="B2258" t="inlineStr">
+        <is>
+          <t>1.18.1</t>
+        </is>
+      </c>
+      <c r="C2258" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="D2258" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2258" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2258" t="inlineStr">
+        <is>
+          <t>Link kopiëren</t>
+        </is>
+      </c>
+      <c r="I2258" t="inlineStr">
+        <is>
+          <t>#action-copy</t>
+        </is>
+      </c>
+      <c r="R2258" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2258" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2258" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2259">
+      <c r="B2259" t="inlineStr">
+        <is>
+          <t>1.18.2</t>
+        </is>
+      </c>
+      <c r="C2259" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="D2259" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2259" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2259" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="I2259" t="inlineStr">
+        <is>
+          <t>#action-whatsapp</t>
+        </is>
+      </c>
+      <c r="R2259" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2259" t="n">
+        <v>2</v>
+      </c>
+      <c r="T2259" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2260">
+      <c r="B2260" t="inlineStr">
+        <is>
+          <t>1.18.3</t>
+        </is>
+      </c>
+      <c r="C2260" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="D2260" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2260" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2260" t="inlineStr">
+        <is>
+          <t>X (Twitter)</t>
+        </is>
+      </c>
+      <c r="I2260" t="inlineStr">
+        <is>
+          <t>#action-x</t>
+        </is>
+      </c>
+      <c r="R2260" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2260" t="n">
+        <v>3</v>
+      </c>
+      <c r="T2260" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2261">
+      <c r="B2261" t="inlineStr">
+        <is>
+          <t>1.18.4</t>
+        </is>
+      </c>
+      <c r="C2261" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="D2261" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2261" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2261" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="I2261" t="inlineStr">
+        <is>
+          <t>#action-linkedin</t>
+        </is>
+      </c>
+      <c r="R2261" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2261" t="n">
+        <v>4</v>
+      </c>
+      <c r="T2261" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2262">
+      <c r="B2262" t="inlineStr">
+        <is>
+          <t>1.18.5</t>
+        </is>
+      </c>
+      <c r="C2262" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="D2262" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2262" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2262" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="I2262" t="inlineStr">
+        <is>
+          <t>#action-facebook</t>
+        </is>
+      </c>
+      <c r="R2262" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2262" t="n">
+        <v>5</v>
+      </c>
+      <c r="T2262" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2263">
+      <c r="B2263" t="inlineStr">
+        <is>
+          <t>1.18.6</t>
+        </is>
+      </c>
+      <c r="C2263" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="D2263" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2263" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2263" t="inlineStr">
+        <is>
+          <t>Per e-mail</t>
+        </is>
+      </c>
+      <c r="I2263" t="inlineStr">
+        <is>
+          <t>#action-email</t>
+        </is>
+      </c>
+      <c r="R2263" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2263" t="n">
+        <v>6</v>
+      </c>
+      <c r="T2263" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2264">
+      <c r="B2264" t="inlineStr">
+        <is>
+          <t>1.18.7</t>
+        </is>
+      </c>
+      <c r="C2264" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="D2264" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2264" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2264" t="inlineStr">
+        <is>
+          <t>PDF downloaden</t>
+        </is>
+      </c>
+      <c r="I2264" t="inlineStr">
+        <is>
+          <t>#action-pdf</t>
+        </is>
+      </c>
+      <c r="R2264" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2264" t="n">
+        <v>7</v>
+      </c>
+      <c r="T2264" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2265">
+      <c r="B2265" t="inlineStr">
+        <is>
+          <t>2.18.1</t>
+        </is>
+      </c>
+      <c r="C2265" t="inlineStr">
+        <is>
+          <t>2.18</t>
+        </is>
+      </c>
+      <c r="D2265" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2265" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2265" t="inlineStr">
+        <is>
+          <t>Link kopieren</t>
+        </is>
+      </c>
+      <c r="I2265" t="inlineStr">
+        <is>
+          <t>#action-copy</t>
+        </is>
+      </c>
+      <c r="R2265" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2265" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2265" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2266">
+      <c r="B2266" t="inlineStr">
+        <is>
+          <t>2.18.2</t>
+        </is>
+      </c>
+      <c r="C2266" t="inlineStr">
+        <is>
+          <t>2.18</t>
+        </is>
+      </c>
+      <c r="D2266" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2266" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2266" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="I2266" t="inlineStr">
+        <is>
+          <t>#action-whatsapp</t>
+        </is>
+      </c>
+      <c r="R2266" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2266" t="n">
+        <v>2</v>
+      </c>
+      <c r="T2266" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2267">
+      <c r="B2267" t="inlineStr">
+        <is>
+          <t>2.18.3</t>
+        </is>
+      </c>
+      <c r="C2267" t="inlineStr">
+        <is>
+          <t>2.18</t>
+        </is>
+      </c>
+      <c r="D2267" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2267" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2267" t="inlineStr">
+        <is>
+          <t>X (Twitter)</t>
+        </is>
+      </c>
+      <c r="I2267" t="inlineStr">
+        <is>
+          <t>#action-x</t>
+        </is>
+      </c>
+      <c r="R2267" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2267" t="n">
+        <v>3</v>
+      </c>
+      <c r="T2267" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2268">
+      <c r="B2268" t="inlineStr">
+        <is>
+          <t>2.18.4</t>
+        </is>
+      </c>
+      <c r="C2268" t="inlineStr">
+        <is>
+          <t>2.18</t>
+        </is>
+      </c>
+      <c r="D2268" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2268" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2268" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="I2268" t="inlineStr">
+        <is>
+          <t>#action-linkedin</t>
+        </is>
+      </c>
+      <c r="R2268" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2268" t="n">
+        <v>4</v>
+      </c>
+      <c r="T2268" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2269">
+      <c r="B2269" t="inlineStr">
+        <is>
+          <t>2.18.5</t>
+        </is>
+      </c>
+      <c r="C2269" t="inlineStr">
+        <is>
+          <t>2.18</t>
+        </is>
+      </c>
+      <c r="D2269" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2269" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2269" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="I2269" t="inlineStr">
+        <is>
+          <t>#action-facebook</t>
+        </is>
+      </c>
+      <c r="R2269" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2269" t="n">
+        <v>5</v>
+      </c>
+      <c r="T2269" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2270">
+      <c r="B2270" t="inlineStr">
+        <is>
+          <t>2.18.6</t>
+        </is>
+      </c>
+      <c r="C2270" t="inlineStr">
+        <is>
+          <t>2.18</t>
+        </is>
+      </c>
+      <c r="D2270" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2270" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2270" t="inlineStr">
+        <is>
+          <t>Per E-Mail</t>
+        </is>
+      </c>
+      <c r="I2270" t="inlineStr">
+        <is>
+          <t>#action-email</t>
+        </is>
+      </c>
+      <c r="R2270" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2270" t="n">
+        <v>6</v>
+      </c>
+      <c r="T2270" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2271">
+      <c r="B2271" t="inlineStr">
+        <is>
+          <t>2.18.7</t>
+        </is>
+      </c>
+      <c r="C2271" t="inlineStr">
+        <is>
+          <t>2.18</t>
+        </is>
+      </c>
+      <c r="D2271" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2271" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2271" t="inlineStr">
+        <is>
+          <t>PDF herunterladen</t>
+        </is>
+      </c>
+      <c r="I2271" t="inlineStr">
+        <is>
+          <t>#action-pdf</t>
+        </is>
+      </c>
+      <c r="R2271" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2271" t="n">
+        <v>7</v>
+      </c>
+      <c r="T2271" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2272">
+      <c r="B2272" t="inlineStr">
+        <is>
+          <t>3.18.1</t>
+        </is>
+      </c>
+      <c r="C2272" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="D2272" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2272" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2272" t="inlineStr">
+        <is>
+          <t>Copy link</t>
+        </is>
+      </c>
+      <c r="I2272" t="inlineStr">
+        <is>
+          <t>#action-copy</t>
+        </is>
+      </c>
+      <c r="R2272" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2272" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2272" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2273">
+      <c r="B2273" t="inlineStr">
+        <is>
+          <t>3.18.2</t>
+        </is>
+      </c>
+      <c r="C2273" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="D2273" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2273" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2273" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="I2273" t="inlineStr">
+        <is>
+          <t>#action-whatsapp</t>
+        </is>
+      </c>
+      <c r="R2273" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2273" t="n">
+        <v>2</v>
+      </c>
+      <c r="T2273" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2274">
+      <c r="B2274" t="inlineStr">
+        <is>
+          <t>3.18.3</t>
+        </is>
+      </c>
+      <c r="C2274" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="D2274" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2274" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2274" t="inlineStr">
+        <is>
+          <t>X (Twitter)</t>
+        </is>
+      </c>
+      <c r="I2274" t="inlineStr">
+        <is>
+          <t>#action-x</t>
+        </is>
+      </c>
+      <c r="R2274" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2274" t="n">
+        <v>3</v>
+      </c>
+      <c r="T2274" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2275">
+      <c r="B2275" t="inlineStr">
+        <is>
+          <t>3.18.4</t>
+        </is>
+      </c>
+      <c r="C2275" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="D2275" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2275" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2275" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="I2275" t="inlineStr">
+        <is>
+          <t>#action-linkedin</t>
+        </is>
+      </c>
+      <c r="R2275" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2275" t="n">
+        <v>4</v>
+      </c>
+      <c r="T2275" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2276">
+      <c r="B2276" t="inlineStr">
+        <is>
+          <t>3.18.5</t>
+        </is>
+      </c>
+      <c r="C2276" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="D2276" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2276" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2276" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="I2276" t="inlineStr">
+        <is>
+          <t>#action-facebook</t>
+        </is>
+      </c>
+      <c r="R2276" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2276" t="n">
+        <v>5</v>
+      </c>
+      <c r="T2276" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2277">
+      <c r="B2277" t="inlineStr">
+        <is>
+          <t>3.18.6</t>
+        </is>
+      </c>
+      <c r="C2277" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="D2277" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2277" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2277" t="inlineStr">
+        <is>
+          <t>Send by email</t>
+        </is>
+      </c>
+      <c r="I2277" t="inlineStr">
+        <is>
+          <t>#action-email</t>
+        </is>
+      </c>
+      <c r="R2277" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2277" t="n">
+        <v>6</v>
+      </c>
+      <c r="T2277" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2278">
+      <c r="B2278" t="inlineStr">
+        <is>
+          <t>3.18.7</t>
+        </is>
+      </c>
+      <c r="C2278" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="D2278" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2278" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2278" t="inlineStr">
+        <is>
+          <t>Download PDF</t>
+        </is>
+      </c>
+      <c r="I2278" t="inlineStr">
+        <is>
+          <t>#action-pdf</t>
+        </is>
+      </c>
+      <c r="R2278" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2278" t="n">
+        <v>7</v>
+      </c>
+      <c r="T2278" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2279">
+      <c r="B2279" t="inlineStr">
+        <is>
+          <t>4.18.1</t>
+        </is>
+      </c>
+      <c r="C2279" t="inlineStr">
+        <is>
+          <t>4.18</t>
+        </is>
+      </c>
+      <c r="D2279" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2279" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2279" t="inlineStr">
+        <is>
+          <t>Скопировать ссылку</t>
+        </is>
+      </c>
+      <c r="I2279" t="inlineStr">
+        <is>
+          <t>#action-copy</t>
+        </is>
+      </c>
+      <c r="R2279" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2279" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2279" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2280">
+      <c r="B2280" t="inlineStr">
+        <is>
+          <t>4.18.2</t>
+        </is>
+      </c>
+      <c r="C2280" t="inlineStr">
+        <is>
+          <t>4.18</t>
+        </is>
+      </c>
+      <c r="D2280" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2280" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2280" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="I2280" t="inlineStr">
+        <is>
+          <t>#action-whatsapp</t>
+        </is>
+      </c>
+      <c r="R2280" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2280" t="n">
+        <v>2</v>
+      </c>
+      <c r="T2280" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2281">
+      <c r="B2281" t="inlineStr">
+        <is>
+          <t>4.18.3</t>
+        </is>
+      </c>
+      <c r="C2281" t="inlineStr">
+        <is>
+          <t>4.18</t>
+        </is>
+      </c>
+      <c r="D2281" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2281" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2281" t="inlineStr">
+        <is>
+          <t>X (Twitter)</t>
+        </is>
+      </c>
+      <c r="I2281" t="inlineStr">
+        <is>
+          <t>#action-x</t>
+        </is>
+      </c>
+      <c r="R2281" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2281" t="n">
+        <v>3</v>
+      </c>
+      <c r="T2281" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2282">
+      <c r="B2282" t="inlineStr">
+        <is>
+          <t>4.18.4</t>
+        </is>
+      </c>
+      <c r="C2282" t="inlineStr">
+        <is>
+          <t>4.18</t>
+        </is>
+      </c>
+      <c r="D2282" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2282" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2282" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="I2282" t="inlineStr">
+        <is>
+          <t>#action-linkedin</t>
+        </is>
+      </c>
+      <c r="R2282" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2282" t="n">
+        <v>4</v>
+      </c>
+      <c r="T2282" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2283">
+      <c r="B2283" t="inlineStr">
+        <is>
+          <t>4.18.5</t>
+        </is>
+      </c>
+      <c r="C2283" t="inlineStr">
+        <is>
+          <t>4.18</t>
+        </is>
+      </c>
+      <c r="D2283" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2283" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2283" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="I2283" t="inlineStr">
+        <is>
+          <t>#action-facebook</t>
+        </is>
+      </c>
+      <c r="R2283" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2283" t="n">
+        <v>5</v>
+      </c>
+      <c r="T2283" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2284">
+      <c r="B2284" t="inlineStr">
+        <is>
+          <t>4.18.6</t>
+        </is>
+      </c>
+      <c r="C2284" t="inlineStr">
+        <is>
+          <t>4.18</t>
+        </is>
+      </c>
+      <c r="D2284" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2284" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2284" t="inlineStr">
+        <is>
+          <t>По e-mail</t>
+        </is>
+      </c>
+      <c r="I2284" t="inlineStr">
+        <is>
+          <t>#action-email</t>
+        </is>
+      </c>
+      <c r="R2284" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2284" t="n">
+        <v>6</v>
+      </c>
+      <c r="T2284" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2285">
+      <c r="B2285" t="inlineStr">
+        <is>
+          <t>4.18.7</t>
+        </is>
+      </c>
+      <c r="C2285" t="inlineStr">
+        <is>
+          <t>4.18</t>
+        </is>
+      </c>
+      <c r="D2285" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2285" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2285" t="inlineStr">
+        <is>
+          <t>Скачать PDF</t>
+        </is>
+      </c>
+      <c r="I2285" t="inlineStr">
+        <is>
+          <t>#action-pdf</t>
+        </is>
+      </c>
+      <c r="R2285" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2285" t="n">
+        <v>7</v>
+      </c>
+      <c r="T2285" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2286">
+      <c r="B2286" t="inlineStr">
+        <is>
+          <t>5.18.1</t>
+        </is>
+      </c>
+      <c r="C2286" t="inlineStr">
+        <is>
+          <t>5.18</t>
+        </is>
+      </c>
+      <c r="D2286" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="E2286" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2286" t="inlineStr">
+        <is>
+          <t>Copier le lien</t>
+        </is>
+      </c>
+      <c r="I2286" t="inlineStr">
+        <is>
+          <t>#action-copy</t>
+        </is>
+      </c>
+      <c r="R2286" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2286" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2286" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2287">
+      <c r="B2287" t="inlineStr">
+        <is>
+          <t>5.18.2</t>
+        </is>
+      </c>
+      <c r="C2287" t="inlineStr">
+        <is>
+          <t>5.18</t>
+        </is>
+      </c>
+      <c r="D2287" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="E2287" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2287" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="I2287" t="inlineStr">
+        <is>
+          <t>#action-whatsapp</t>
+        </is>
+      </c>
+      <c r="R2287" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2287" t="n">
+        <v>2</v>
+      </c>
+      <c r="T2287" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2288">
+      <c r="B2288" t="inlineStr">
+        <is>
+          <t>5.18.3</t>
+        </is>
+      </c>
+      <c r="C2288" t="inlineStr">
+        <is>
+          <t>5.18</t>
+        </is>
+      </c>
+      <c r="D2288" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="E2288" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2288" t="inlineStr">
+        <is>
+          <t>X (Twitter)</t>
+        </is>
+      </c>
+      <c r="I2288" t="inlineStr">
+        <is>
+          <t>#action-x</t>
+        </is>
+      </c>
+      <c r="R2288" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2288" t="n">
+        <v>3</v>
+      </c>
+      <c r="T2288" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2289">
+      <c r="B2289" t="inlineStr">
+        <is>
+          <t>5.18.4</t>
+        </is>
+      </c>
+      <c r="C2289" t="inlineStr">
+        <is>
+          <t>5.18</t>
+        </is>
+      </c>
+      <c r="D2289" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="E2289" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2289" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="I2289" t="inlineStr">
+        <is>
+          <t>#action-linkedin</t>
+        </is>
+      </c>
+      <c r="R2289" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2289" t="n">
+        <v>4</v>
+      </c>
+      <c r="T2289" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2290">
+      <c r="B2290" t="inlineStr">
+        <is>
+          <t>5.18.5</t>
+        </is>
+      </c>
+      <c r="C2290" t="inlineStr">
+        <is>
+          <t>5.18</t>
+        </is>
+      </c>
+      <c r="D2290" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="E2290" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2290" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="I2290" t="inlineStr">
+        <is>
+          <t>#action-facebook</t>
+        </is>
+      </c>
+      <c r="R2290" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2290" t="n">
+        <v>5</v>
+      </c>
+      <c r="T2290" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2291">
+      <c r="B2291" t="inlineStr">
+        <is>
+          <t>5.18.6</t>
+        </is>
+      </c>
+      <c r="C2291" t="inlineStr">
+        <is>
+          <t>5.18</t>
+        </is>
+      </c>
+      <c r="D2291" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="E2291" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2291" t="inlineStr">
+        <is>
+          <t>Par e-mail</t>
+        </is>
+      </c>
+      <c r="I2291" t="inlineStr">
+        <is>
+          <t>#action-email</t>
+        </is>
+      </c>
+      <c r="R2291" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2291" t="n">
+        <v>6</v>
+      </c>
+      <c r="T2291" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2292">
+      <c r="B2292" t="inlineStr">
+        <is>
+          <t>5.18.7</t>
+        </is>
+      </c>
+      <c r="C2292" t="inlineStr">
+        <is>
+          <t>5.18</t>
+        </is>
+      </c>
+      <c r="D2292" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="E2292" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2292" t="inlineStr">
+        <is>
+          <t>Télécharger le PDF</t>
+        </is>
+      </c>
+      <c r="I2292" t="inlineStr">
+        <is>
+          <t>#action-pdf</t>
+        </is>
+      </c>
+      <c r="R2292" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2292" t="n">
+        <v>7</v>
+      </c>
+      <c r="T2292" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2293">
+      <c r="B2293" t="inlineStr">
+        <is>
+          <t>6.18.1</t>
+        </is>
+      </c>
+      <c r="C2293" t="inlineStr">
+        <is>
+          <t>6.18</t>
+        </is>
+      </c>
+      <c r="D2293" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="E2293" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2293" t="inlineStr">
+        <is>
+          <t>Copiar enlace</t>
+        </is>
+      </c>
+      <c r="I2293" t="inlineStr">
+        <is>
+          <t>#action-copy</t>
+        </is>
+      </c>
+      <c r="R2293" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2293" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2293" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2294">
+      <c r="B2294" t="inlineStr">
+        <is>
+          <t>6.18.2</t>
+        </is>
+      </c>
+      <c r="C2294" t="inlineStr">
+        <is>
+          <t>6.18</t>
+        </is>
+      </c>
+      <c r="D2294" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="E2294" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2294" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="I2294" t="inlineStr">
+        <is>
+          <t>#action-whatsapp</t>
+        </is>
+      </c>
+      <c r="R2294" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2294" t="n">
+        <v>2</v>
+      </c>
+      <c r="T2294" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2295">
+      <c r="B2295" t="inlineStr">
+        <is>
+          <t>6.18.3</t>
+        </is>
+      </c>
+      <c r="C2295" t="inlineStr">
+        <is>
+          <t>6.18</t>
+        </is>
+      </c>
+      <c r="D2295" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="E2295" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2295" t="inlineStr">
+        <is>
+          <t>X (Twitter)</t>
+        </is>
+      </c>
+      <c r="I2295" t="inlineStr">
+        <is>
+          <t>#action-x</t>
+        </is>
+      </c>
+      <c r="R2295" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2295" t="n">
+        <v>3</v>
+      </c>
+      <c r="T2295" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2296">
+      <c r="B2296" t="inlineStr">
+        <is>
+          <t>6.18.4</t>
+        </is>
+      </c>
+      <c r="C2296" t="inlineStr">
+        <is>
+          <t>6.18</t>
+        </is>
+      </c>
+      <c r="D2296" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="E2296" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2296" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="I2296" t="inlineStr">
+        <is>
+          <t>#action-linkedin</t>
+        </is>
+      </c>
+      <c r="R2296" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2296" t="n">
+        <v>4</v>
+      </c>
+      <c r="T2296" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2297">
+      <c r="B2297" t="inlineStr">
+        <is>
+          <t>6.18.5</t>
+        </is>
+      </c>
+      <c r="C2297" t="inlineStr">
+        <is>
+          <t>6.18</t>
+        </is>
+      </c>
+      <c r="D2297" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="E2297" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2297" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="I2297" t="inlineStr">
+        <is>
+          <t>#action-facebook</t>
+        </is>
+      </c>
+      <c r="R2297" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2297" t="n">
+        <v>5</v>
+      </c>
+      <c r="T2297" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2298">
+      <c r="B2298" t="inlineStr">
+        <is>
+          <t>6.18.6</t>
+        </is>
+      </c>
+      <c r="C2298" t="inlineStr">
+        <is>
+          <t>6.18</t>
+        </is>
+      </c>
+      <c r="D2298" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="E2298" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2298" t="inlineStr">
+        <is>
+          <t>Por correo</t>
+        </is>
+      </c>
+      <c r="I2298" t="inlineStr">
+        <is>
+          <t>#action-email</t>
+        </is>
+      </c>
+      <c r="R2298" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2298" t="n">
+        <v>6</v>
+      </c>
+      <c r="T2298" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2299">
+      <c r="B2299" t="inlineStr">
+        <is>
+          <t>6.18.7</t>
+        </is>
+      </c>
+      <c r="C2299" t="inlineStr">
+        <is>
+          <t>6.18</t>
+        </is>
+      </c>
+      <c r="D2299" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="E2299" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2299" t="inlineStr">
+        <is>
+          <t>Descargar PDF</t>
+        </is>
+      </c>
+      <c r="I2299" t="inlineStr">
+        <is>
+          <t>#action-pdf</t>
+        </is>
+      </c>
+      <c r="R2299" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2299" t="n">
+        <v>7</v>
+      </c>
+      <c r="T2299" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2300">
+      <c r="B2300" t="inlineStr">
+        <is>
+          <t>7.18.1</t>
+        </is>
+      </c>
+      <c r="C2300" t="inlineStr">
+        <is>
+          <t>7.18</t>
+        </is>
+      </c>
+      <c r="D2300" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="E2300" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2300" t="inlineStr">
+        <is>
+          <t>Copia link</t>
+        </is>
+      </c>
+      <c r="I2300" t="inlineStr">
+        <is>
+          <t>#action-copy</t>
+        </is>
+      </c>
+      <c r="R2300" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2300" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2300" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2301">
+      <c r="B2301" t="inlineStr">
+        <is>
+          <t>7.18.2</t>
+        </is>
+      </c>
+      <c r="C2301" t="inlineStr">
+        <is>
+          <t>7.18</t>
+        </is>
+      </c>
+      <c r="D2301" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="E2301" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2301" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="I2301" t="inlineStr">
+        <is>
+          <t>#action-whatsapp</t>
+        </is>
+      </c>
+      <c r="R2301" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2301" t="n">
+        <v>2</v>
+      </c>
+      <c r="T2301" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2302">
+      <c r="B2302" t="inlineStr">
+        <is>
+          <t>7.18.3</t>
+        </is>
+      </c>
+      <c r="C2302" t="inlineStr">
+        <is>
+          <t>7.18</t>
+        </is>
+      </c>
+      <c r="D2302" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="E2302" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2302" t="inlineStr">
+        <is>
+          <t>X (Twitter)</t>
+        </is>
+      </c>
+      <c r="I2302" t="inlineStr">
+        <is>
+          <t>#action-x</t>
+        </is>
+      </c>
+      <c r="R2302" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2302" t="n">
+        <v>3</v>
+      </c>
+      <c r="T2302" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2303">
+      <c r="B2303" t="inlineStr">
+        <is>
+          <t>7.18.4</t>
+        </is>
+      </c>
+      <c r="C2303" t="inlineStr">
+        <is>
+          <t>7.18</t>
+        </is>
+      </c>
+      <c r="D2303" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="E2303" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2303" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="I2303" t="inlineStr">
+        <is>
+          <t>#action-linkedin</t>
+        </is>
+      </c>
+      <c r="R2303" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2303" t="n">
+        <v>4</v>
+      </c>
+      <c r="T2303" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2304">
+      <c r="B2304" t="inlineStr">
+        <is>
+          <t>7.18.5</t>
+        </is>
+      </c>
+      <c r="C2304" t="inlineStr">
+        <is>
+          <t>7.18</t>
+        </is>
+      </c>
+      <c r="D2304" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="E2304" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2304" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="I2304" t="inlineStr">
+        <is>
+          <t>#action-facebook</t>
+        </is>
+      </c>
+      <c r="R2304" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2304" t="n">
+        <v>5</v>
+      </c>
+      <c r="T2304" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2305">
+      <c r="B2305" t="inlineStr">
+        <is>
+          <t>7.18.6</t>
+        </is>
+      </c>
+      <c r="C2305" t="inlineStr">
+        <is>
+          <t>7.18</t>
+        </is>
+      </c>
+      <c r="D2305" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="E2305" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2305" t="inlineStr">
+        <is>
+          <t>Per e-mail</t>
+        </is>
+      </c>
+      <c r="I2305" t="inlineStr">
+        <is>
+          <t>#action-email</t>
+        </is>
+      </c>
+      <c r="R2305" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2305" t="n">
+        <v>6</v>
+      </c>
+      <c r="T2305" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2306">
+      <c r="B2306" t="inlineStr">
+        <is>
+          <t>7.18.7</t>
+        </is>
+      </c>
+      <c r="C2306" t="inlineStr">
+        <is>
+          <t>7.18</t>
+        </is>
+      </c>
+      <c r="D2306" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="E2306" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2306" t="inlineStr">
+        <is>
+          <t>Scarica PDF</t>
+        </is>
+      </c>
+      <c r="I2306" t="inlineStr">
+        <is>
+          <t>#action-pdf</t>
+        </is>
+      </c>
+      <c r="R2306" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2306" t="n">
+        <v>7</v>
+      </c>
+      <c r="T2306" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2307">
+      <c r="B2307" t="inlineStr">
+        <is>
+          <t>8.18.1</t>
+        </is>
+      </c>
+      <c r="C2307" t="inlineStr">
+        <is>
+          <t>8.18</t>
+        </is>
+      </c>
+      <c r="D2307" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="E2307" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2307" t="inlineStr">
+        <is>
+          <t>Copiar ligação</t>
+        </is>
+      </c>
+      <c r="I2307" t="inlineStr">
+        <is>
+          <t>#action-copy</t>
+        </is>
+      </c>
+      <c r="R2307" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2307" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2307" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2308">
+      <c r="B2308" t="inlineStr">
+        <is>
+          <t>8.18.2</t>
+        </is>
+      </c>
+      <c r="C2308" t="inlineStr">
+        <is>
+          <t>8.18</t>
+        </is>
+      </c>
+      <c r="D2308" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="E2308" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2308" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="I2308" t="inlineStr">
+        <is>
+          <t>#action-whatsapp</t>
+        </is>
+      </c>
+      <c r="R2308" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2308" t="n">
+        <v>2</v>
+      </c>
+      <c r="T2308" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2309">
+      <c r="B2309" t="inlineStr">
+        <is>
+          <t>8.18.3</t>
+        </is>
+      </c>
+      <c r="C2309" t="inlineStr">
+        <is>
+          <t>8.18</t>
+        </is>
+      </c>
+      <c r="D2309" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="E2309" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2309" t="inlineStr">
+        <is>
+          <t>X (Twitter)</t>
+        </is>
+      </c>
+      <c r="I2309" t="inlineStr">
+        <is>
+          <t>#action-x</t>
+        </is>
+      </c>
+      <c r="R2309" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2309" t="n">
+        <v>3</v>
+      </c>
+      <c r="T2309" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2310">
+      <c r="B2310" t="inlineStr">
+        <is>
+          <t>8.18.4</t>
+        </is>
+      </c>
+      <c r="C2310" t="inlineStr">
+        <is>
+          <t>8.18</t>
+        </is>
+      </c>
+      <c r="D2310" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="E2310" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2310" t="inlineStr">
+        <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="I2310" t="inlineStr">
+        <is>
+          <t>#action-linkedin</t>
+        </is>
+      </c>
+      <c r="R2310" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2310" t="n">
+        <v>4</v>
+      </c>
+      <c r="T2310" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2311">
+      <c r="B2311" t="inlineStr">
+        <is>
+          <t>8.18.5</t>
+        </is>
+      </c>
+      <c r="C2311" t="inlineStr">
+        <is>
+          <t>8.18</t>
+        </is>
+      </c>
+      <c r="D2311" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="E2311" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2311" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="I2311" t="inlineStr">
+        <is>
+          <t>#action-facebook</t>
+        </is>
+      </c>
+      <c r="R2311" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2311" t="n">
+        <v>5</v>
+      </c>
+      <c r="T2311" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2312">
+      <c r="B2312" t="inlineStr">
+        <is>
+          <t>8.18.6</t>
+        </is>
+      </c>
+      <c r="C2312" t="inlineStr">
+        <is>
+          <t>8.18</t>
+        </is>
+      </c>
+      <c r="D2312" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="E2312" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2312" t="inlineStr">
+        <is>
+          <t>Por e-mail</t>
+        </is>
+      </c>
+      <c r="I2312" t="inlineStr">
+        <is>
+          <t>#action-email</t>
+        </is>
+      </c>
+      <c r="R2312" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2312" t="n">
+        <v>6</v>
+      </c>
+      <c r="T2312" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2313">
+      <c r="B2313" t="inlineStr">
+        <is>
+          <t>8.18.7</t>
+        </is>
+      </c>
+      <c r="C2313" t="inlineStr">
+        <is>
+          <t>8.18</t>
+        </is>
+      </c>
+      <c r="D2313" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="E2313" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2313" t="inlineStr">
+        <is>
+          <t>Descarregar PDF</t>
+        </is>
+      </c>
+      <c r="I2313" t="inlineStr">
+        <is>
+          <t>#action-pdf</t>
+        </is>
+      </c>
+      <c r="R2313" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2313" t="n">
+        <v>7</v>
+      </c>
+      <c r="T2313" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B2:AR65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Xlsx v15: .17 (Taal) gedeactiveerd — masthead heeft al taal-schakelaar
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -12456,7 +12456,7 @@
         <v>17</v>
       </c>
       <c r="T273" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="274">
@@ -12494,7 +12494,7 @@
         <v>1</v>
       </c>
       <c r="T274" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="275">
@@ -12537,7 +12537,7 @@
         <v>2</v>
       </c>
       <c r="T275" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="276">
@@ -12580,7 +12580,7 @@
         <v>3</v>
       </c>
       <c r="T276" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="277">
@@ -12623,7 +12623,7 @@
         <v>4</v>
       </c>
       <c r="T277" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="278">
@@ -12666,7 +12666,7 @@
         <v>5</v>
       </c>
       <c r="T278" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="279">
@@ -12709,7 +12709,7 @@
         <v>6</v>
       </c>
       <c r="T279" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="280">
@@ -12752,7 +12752,7 @@
         <v>7</v>
       </c>
       <c r="T280" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="281">
@@ -12795,7 +12795,7 @@
         <v>8</v>
       </c>
       <c r="T281" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="282">
@@ -23882,7 +23882,7 @@
         <v>17</v>
       </c>
       <c r="T551" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="552">
@@ -23920,7 +23920,7 @@
         <v>1</v>
       </c>
       <c r="T552" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="553">
@@ -23958,7 +23958,7 @@
         <v>2</v>
       </c>
       <c r="T553" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="554">
@@ -23996,7 +23996,7 @@
         <v>3</v>
       </c>
       <c r="T554" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="555">
@@ -24034,7 +24034,7 @@
         <v>4</v>
       </c>
       <c r="T555" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="556">
@@ -24072,7 +24072,7 @@
         <v>5</v>
       </c>
       <c r="T556" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="557">
@@ -24110,7 +24110,7 @@
         <v>6</v>
       </c>
       <c r="T557" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="558">
@@ -24148,7 +24148,7 @@
         <v>7</v>
       </c>
       <c r="T558" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="559">
@@ -24186,7 +24186,7 @@
         <v>8</v>
       </c>
       <c r="T559" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="560">
@@ -35273,7 +35273,7 @@
         <v>17</v>
       </c>
       <c r="T829" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="830">
@@ -35311,7 +35311,7 @@
         <v>1</v>
       </c>
       <c r="T830" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="831">
@@ -35349,7 +35349,7 @@
         <v>2</v>
       </c>
       <c r="T831" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="832">
@@ -35387,7 +35387,7 @@
         <v>3</v>
       </c>
       <c r="T832" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="833">
@@ -35425,7 +35425,7 @@
         <v>4</v>
       </c>
       <c r="T833" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="834">
@@ -35463,7 +35463,7 @@
         <v>5</v>
       </c>
       <c r="T834" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="835">
@@ -35501,7 +35501,7 @@
         <v>6</v>
       </c>
       <c r="T835" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="836">
@@ -35539,7 +35539,7 @@
         <v>7</v>
       </c>
       <c r="T836" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="837">
@@ -35577,7 +35577,7 @@
         <v>8</v>
       </c>
       <c r="T837" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="838">
@@ -46484,7 +46484,7 @@
         <v>17</v>
       </c>
       <c r="T1107" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1108">
@@ -46522,7 +46522,7 @@
         <v>1</v>
       </c>
       <c r="T1108" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1109">
@@ -46560,7 +46560,7 @@
         <v>2</v>
       </c>
       <c r="T1109" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1110">
@@ -46598,7 +46598,7 @@
         <v>3</v>
       </c>
       <c r="T1110" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1111">
@@ -46636,7 +46636,7 @@
         <v>4</v>
       </c>
       <c r="T1111" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1112">
@@ -46674,7 +46674,7 @@
         <v>5</v>
       </c>
       <c r="T1112" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1113">
@@ -46712,7 +46712,7 @@
         <v>6</v>
       </c>
       <c r="T1113" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1114">
@@ -46750,7 +46750,7 @@
         <v>7</v>
       </c>
       <c r="T1114" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1115">
@@ -46788,7 +46788,7 @@
         <v>8</v>
       </c>
       <c r="T1115" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1116">
@@ -57425,7 +57425,7 @@
         <v>17</v>
       </c>
       <c r="T1385" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1386">
@@ -57463,7 +57463,7 @@
         <v>1</v>
       </c>
       <c r="T1386" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1387">
@@ -57501,7 +57501,7 @@
         <v>2</v>
       </c>
       <c r="T1387" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1388">
@@ -57539,7 +57539,7 @@
         <v>3</v>
       </c>
       <c r="T1388" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1389">
@@ -57577,7 +57577,7 @@
         <v>4</v>
       </c>
       <c r="T1389" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1390">
@@ -57615,7 +57615,7 @@
         <v>5</v>
       </c>
       <c r="T1390" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1391">
@@ -57653,7 +57653,7 @@
         <v>6</v>
       </c>
       <c r="T1391" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1392">
@@ -57691,7 +57691,7 @@
         <v>7</v>
       </c>
       <c r="T1392" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1393">
@@ -57729,7 +57729,7 @@
         <v>8</v>
       </c>
       <c r="T1393" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1394">
@@ -68566,7 +68566,7 @@
         <v>17</v>
       </c>
       <c r="T1663" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1664">
@@ -68604,7 +68604,7 @@
         <v>1</v>
       </c>
       <c r="T1664" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1665">
@@ -68642,7 +68642,7 @@
         <v>2</v>
       </c>
       <c r="T1665" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1666">
@@ -68680,7 +68680,7 @@
         <v>3</v>
       </c>
       <c r="T1666" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1667">
@@ -68718,7 +68718,7 @@
         <v>4</v>
       </c>
       <c r="T1667" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1668">
@@ -68756,7 +68756,7 @@
         <v>5</v>
       </c>
       <c r="T1668" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1669">
@@ -68794,7 +68794,7 @@
         <v>6</v>
       </c>
       <c r="T1669" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1670">
@@ -68832,7 +68832,7 @@
         <v>7</v>
       </c>
       <c r="T1670" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1671">
@@ -68870,7 +68870,7 @@
         <v>8</v>
       </c>
       <c r="T1671" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1672">
@@ -79722,7 +79722,7 @@
         <v>17</v>
       </c>
       <c r="T1941" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1942">
@@ -79760,7 +79760,7 @@
         <v>1</v>
       </c>
       <c r="T1942" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1943">
@@ -79798,7 +79798,7 @@
         <v>2</v>
       </c>
       <c r="T1943" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1944">
@@ -79836,7 +79836,7 @@
         <v>3</v>
       </c>
       <c r="T1944" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1945">
@@ -79874,7 +79874,7 @@
         <v>4</v>
       </c>
       <c r="T1945" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1946">
@@ -79912,7 +79912,7 @@
         <v>5</v>
       </c>
       <c r="T1946" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1947">
@@ -79950,7 +79950,7 @@
         <v>6</v>
       </c>
       <c r="T1947" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1948">
@@ -79988,7 +79988,7 @@
         <v>7</v>
       </c>
       <c r="T1948" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1949">
@@ -80026,7 +80026,7 @@
         <v>8</v>
       </c>
       <c r="T1949" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1950">
@@ -90858,7 +90858,7 @@
         <v>17</v>
       </c>
       <c r="T2219" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2220">
@@ -90896,7 +90896,7 @@
         <v>1</v>
       </c>
       <c r="T2220" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2221">
@@ -90934,7 +90934,7 @@
         <v>2</v>
       </c>
       <c r="T2221" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2222">
@@ -90972,7 +90972,7 @@
         <v>3</v>
       </c>
       <c r="T2222" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2223">
@@ -91010,7 +91010,7 @@
         <v>4</v>
       </c>
       <c r="T2223" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2224">
@@ -91048,7 +91048,7 @@
         <v>5</v>
       </c>
       <c r="T2224" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2225">
@@ -91086,7 +91086,7 @@
         <v>6</v>
       </c>
       <c r="T2225" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2226">
@@ -91124,7 +91124,7 @@
         <v>7</v>
       </c>
       <c r="T2226" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2227">
@@ -91162,7 +91162,7 @@
         <v>8</v>
       </c>
       <c r="T2227" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2228">

</xml_diff>

<commit_message>
Delen: xlsx 1.18 = trigger, deel-menu.js autogenerate vult 7 items (originele werkwijze)
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -92455,7 +92455,7 @@
         <v>1</v>
       </c>
       <c r="T2258" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2259">
@@ -92498,7 +92498,7 @@
         <v>2</v>
       </c>
       <c r="T2259" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2260">
@@ -92541,7 +92541,7 @@
         <v>3</v>
       </c>
       <c r="T2260" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2261">
@@ -92584,7 +92584,7 @@
         <v>4</v>
       </c>
       <c r="T2261" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2262">
@@ -92627,7 +92627,7 @@
         <v>5</v>
       </c>
       <c r="T2262" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2263">
@@ -92670,7 +92670,7 @@
         <v>6</v>
       </c>
       <c r="T2263" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2264">
@@ -92713,7 +92713,7 @@
         <v>7</v>
       </c>
       <c r="T2264" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2265">
@@ -92756,7 +92756,7 @@
         <v>1</v>
       </c>
       <c r="T2265" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2266">
@@ -92799,7 +92799,7 @@
         <v>2</v>
       </c>
       <c r="T2266" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2267">
@@ -92842,7 +92842,7 @@
         <v>3</v>
       </c>
       <c r="T2267" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2268">
@@ -92885,7 +92885,7 @@
         <v>4</v>
       </c>
       <c r="T2268" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2269">
@@ -92928,7 +92928,7 @@
         <v>5</v>
       </c>
       <c r="T2269" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2270">
@@ -92971,7 +92971,7 @@
         <v>6</v>
       </c>
       <c r="T2270" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2271">
@@ -93014,7 +93014,7 @@
         <v>7</v>
       </c>
       <c r="T2271" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2272">
@@ -93057,7 +93057,7 @@
         <v>1</v>
       </c>
       <c r="T2272" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2273">
@@ -93100,7 +93100,7 @@
         <v>2</v>
       </c>
       <c r="T2273" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2274">
@@ -93143,7 +93143,7 @@
         <v>3</v>
       </c>
       <c r="T2274" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2275">
@@ -93186,7 +93186,7 @@
         <v>4</v>
       </c>
       <c r="T2275" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2276">
@@ -93229,7 +93229,7 @@
         <v>5</v>
       </c>
       <c r="T2276" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2277">
@@ -93272,7 +93272,7 @@
         <v>6</v>
       </c>
       <c r="T2277" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2278">
@@ -93315,7 +93315,7 @@
         <v>7</v>
       </c>
       <c r="T2278" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2279">
@@ -93358,7 +93358,7 @@
         <v>1</v>
       </c>
       <c r="T2279" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2280">
@@ -93401,7 +93401,7 @@
         <v>2</v>
       </c>
       <c r="T2280" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2281">
@@ -93444,7 +93444,7 @@
         <v>3</v>
       </c>
       <c r="T2281" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2282">
@@ -93487,7 +93487,7 @@
         <v>4</v>
       </c>
       <c r="T2282" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2283">
@@ -93530,7 +93530,7 @@
         <v>5</v>
       </c>
       <c r="T2283" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2284">
@@ -93573,7 +93573,7 @@
         <v>6</v>
       </c>
       <c r="T2284" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2285">
@@ -93616,7 +93616,7 @@
         <v>7</v>
       </c>
       <c r="T2285" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2286">
@@ -93659,7 +93659,7 @@
         <v>1</v>
       </c>
       <c r="T2286" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2287">
@@ -93702,7 +93702,7 @@
         <v>2</v>
       </c>
       <c r="T2287" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2288">
@@ -93745,7 +93745,7 @@
         <v>3</v>
       </c>
       <c r="T2288" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2289">
@@ -93788,7 +93788,7 @@
         <v>4</v>
       </c>
       <c r="T2289" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2290">
@@ -93831,7 +93831,7 @@
         <v>5</v>
       </c>
       <c r="T2290" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2291">
@@ -93874,7 +93874,7 @@
         <v>6</v>
       </c>
       <c r="T2291" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2292">
@@ -93917,7 +93917,7 @@
         <v>7</v>
       </c>
       <c r="T2292" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2293">
@@ -93960,7 +93960,7 @@
         <v>1</v>
       </c>
       <c r="T2293" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2294">
@@ -94003,7 +94003,7 @@
         <v>2</v>
       </c>
       <c r="T2294" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2295">
@@ -94046,7 +94046,7 @@
         <v>3</v>
       </c>
       <c r="T2295" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2296">
@@ -94089,7 +94089,7 @@
         <v>4</v>
       </c>
       <c r="T2296" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2297">
@@ -94132,7 +94132,7 @@
         <v>5</v>
       </c>
       <c r="T2297" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2298">
@@ -94175,7 +94175,7 @@
         <v>6</v>
       </c>
       <c r="T2298" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2299">
@@ -94218,7 +94218,7 @@
         <v>7</v>
       </c>
       <c r="T2299" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2300">
@@ -94261,7 +94261,7 @@
         <v>1</v>
       </c>
       <c r="T2300" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2301">
@@ -94304,7 +94304,7 @@
         <v>2</v>
       </c>
       <c r="T2301" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2302">
@@ -94347,7 +94347,7 @@
         <v>3</v>
       </c>
       <c r="T2302" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2303">
@@ -94390,7 +94390,7 @@
         <v>4</v>
       </c>
       <c r="T2303" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2304">
@@ -94433,7 +94433,7 @@
         <v>5</v>
       </c>
       <c r="T2304" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2305">
@@ -94476,7 +94476,7 @@
         <v>6</v>
       </c>
       <c r="T2305" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2306">
@@ -94519,7 +94519,7 @@
         <v>7</v>
       </c>
       <c r="T2306" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2307">
@@ -94562,7 +94562,7 @@
         <v>1</v>
       </c>
       <c r="T2307" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2308">
@@ -94605,7 +94605,7 @@
         <v>2</v>
       </c>
       <c r="T2308" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2309">
@@ -94648,7 +94648,7 @@
         <v>3</v>
       </c>
       <c r="T2309" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2310">
@@ -94691,7 +94691,7 @@
         <v>4</v>
       </c>
       <c r="T2310" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2311">
@@ -94734,7 +94734,7 @@
         <v>5</v>
       </c>
       <c r="T2311" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2312">
@@ -94777,7 +94777,7 @@
         <v>6</v>
       </c>
       <c r="T2312" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2313">
@@ -94820,7 +94820,7 @@
         <v>7</v>
       </c>
       <c r="T2313" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Delen: 100% uit xlsx via action:xxx URL-conventie (één bron, alle 8 talen)
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -92443,7 +92443,7 @@
       </c>
       <c r="I2258" t="inlineStr">
         <is>
-          <t>#action-copy</t>
+          <t>action:copy</t>
         </is>
       </c>
       <c r="R2258" t="inlineStr">
@@ -92455,7 +92455,7 @@
         <v>1</v>
       </c>
       <c r="T2258" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2259">
@@ -92486,7 +92486,7 @@
       </c>
       <c r="I2259" t="inlineStr">
         <is>
-          <t>#action-whatsapp</t>
+          <t>action:whatsapp</t>
         </is>
       </c>
       <c r="R2259" t="inlineStr">
@@ -92498,7 +92498,7 @@
         <v>2</v>
       </c>
       <c r="T2259" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2260">
@@ -92529,7 +92529,7 @@
       </c>
       <c r="I2260" t="inlineStr">
         <is>
-          <t>#action-x</t>
+          <t>action:x</t>
         </is>
       </c>
       <c r="R2260" t="inlineStr">
@@ -92541,7 +92541,7 @@
         <v>3</v>
       </c>
       <c r="T2260" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2261">
@@ -92572,7 +92572,7 @@
       </c>
       <c r="I2261" t="inlineStr">
         <is>
-          <t>#action-linkedin</t>
+          <t>action:linkedin</t>
         </is>
       </c>
       <c r="R2261" t="inlineStr">
@@ -92584,7 +92584,7 @@
         <v>4</v>
       </c>
       <c r="T2261" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2262">
@@ -92615,7 +92615,7 @@
       </c>
       <c r="I2262" t="inlineStr">
         <is>
-          <t>#action-facebook</t>
+          <t>action:facebook</t>
         </is>
       </c>
       <c r="R2262" t="inlineStr">
@@ -92627,7 +92627,7 @@
         <v>5</v>
       </c>
       <c r="T2262" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2263">
@@ -92658,7 +92658,7 @@
       </c>
       <c r="I2263" t="inlineStr">
         <is>
-          <t>#action-email</t>
+          <t>action:email</t>
         </is>
       </c>
       <c r="R2263" t="inlineStr">
@@ -92670,7 +92670,7 @@
         <v>6</v>
       </c>
       <c r="T2263" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2264">
@@ -92701,7 +92701,7 @@
       </c>
       <c r="I2264" t="inlineStr">
         <is>
-          <t>#action-pdf</t>
+          <t>action:pdf</t>
         </is>
       </c>
       <c r="R2264" t="inlineStr">
@@ -92713,7 +92713,7 @@
         <v>7</v>
       </c>
       <c r="T2264" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2265">
@@ -92744,7 +92744,7 @@
       </c>
       <c r="I2265" t="inlineStr">
         <is>
-          <t>#action-copy</t>
+          <t>action:copy</t>
         </is>
       </c>
       <c r="R2265" t="inlineStr">
@@ -92756,7 +92756,7 @@
         <v>1</v>
       </c>
       <c r="T2265" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2266">
@@ -92787,7 +92787,7 @@
       </c>
       <c r="I2266" t="inlineStr">
         <is>
-          <t>#action-whatsapp</t>
+          <t>action:whatsapp</t>
         </is>
       </c>
       <c r="R2266" t="inlineStr">
@@ -92799,7 +92799,7 @@
         <v>2</v>
       </c>
       <c r="T2266" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2267">
@@ -92830,7 +92830,7 @@
       </c>
       <c r="I2267" t="inlineStr">
         <is>
-          <t>#action-x</t>
+          <t>action:x</t>
         </is>
       </c>
       <c r="R2267" t="inlineStr">
@@ -92842,7 +92842,7 @@
         <v>3</v>
       </c>
       <c r="T2267" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2268">
@@ -92873,7 +92873,7 @@
       </c>
       <c r="I2268" t="inlineStr">
         <is>
-          <t>#action-linkedin</t>
+          <t>action:linkedin</t>
         </is>
       </c>
       <c r="R2268" t="inlineStr">
@@ -92885,7 +92885,7 @@
         <v>4</v>
       </c>
       <c r="T2268" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2269">
@@ -92916,7 +92916,7 @@
       </c>
       <c r="I2269" t="inlineStr">
         <is>
-          <t>#action-facebook</t>
+          <t>action:facebook</t>
         </is>
       </c>
       <c r="R2269" t="inlineStr">
@@ -92928,7 +92928,7 @@
         <v>5</v>
       </c>
       <c r="T2269" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2270">
@@ -92959,7 +92959,7 @@
       </c>
       <c r="I2270" t="inlineStr">
         <is>
-          <t>#action-email</t>
+          <t>action:email</t>
         </is>
       </c>
       <c r="R2270" t="inlineStr">
@@ -92971,7 +92971,7 @@
         <v>6</v>
       </c>
       <c r="T2270" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2271">
@@ -93002,7 +93002,7 @@
       </c>
       <c r="I2271" t="inlineStr">
         <is>
-          <t>#action-pdf</t>
+          <t>action:pdf</t>
         </is>
       </c>
       <c r="R2271" t="inlineStr">
@@ -93014,7 +93014,7 @@
         <v>7</v>
       </c>
       <c r="T2271" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2272">
@@ -93045,7 +93045,7 @@
       </c>
       <c r="I2272" t="inlineStr">
         <is>
-          <t>#action-copy</t>
+          <t>action:copy</t>
         </is>
       </c>
       <c r="R2272" t="inlineStr">
@@ -93057,7 +93057,7 @@
         <v>1</v>
       </c>
       <c r="T2272" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2273">
@@ -93088,7 +93088,7 @@
       </c>
       <c r="I2273" t="inlineStr">
         <is>
-          <t>#action-whatsapp</t>
+          <t>action:whatsapp</t>
         </is>
       </c>
       <c r="R2273" t="inlineStr">
@@ -93100,7 +93100,7 @@
         <v>2</v>
       </c>
       <c r="T2273" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2274">
@@ -93131,7 +93131,7 @@
       </c>
       <c r="I2274" t="inlineStr">
         <is>
-          <t>#action-x</t>
+          <t>action:x</t>
         </is>
       </c>
       <c r="R2274" t="inlineStr">
@@ -93143,7 +93143,7 @@
         <v>3</v>
       </c>
       <c r="T2274" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2275">
@@ -93174,7 +93174,7 @@
       </c>
       <c r="I2275" t="inlineStr">
         <is>
-          <t>#action-linkedin</t>
+          <t>action:linkedin</t>
         </is>
       </c>
       <c r="R2275" t="inlineStr">
@@ -93186,7 +93186,7 @@
         <v>4</v>
       </c>
       <c r="T2275" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2276">
@@ -93217,7 +93217,7 @@
       </c>
       <c r="I2276" t="inlineStr">
         <is>
-          <t>#action-facebook</t>
+          <t>action:facebook</t>
         </is>
       </c>
       <c r="R2276" t="inlineStr">
@@ -93229,7 +93229,7 @@
         <v>5</v>
       </c>
       <c r="T2276" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2277">
@@ -93260,7 +93260,7 @@
       </c>
       <c r="I2277" t="inlineStr">
         <is>
-          <t>#action-email</t>
+          <t>action:email</t>
         </is>
       </c>
       <c r="R2277" t="inlineStr">
@@ -93272,7 +93272,7 @@
         <v>6</v>
       </c>
       <c r="T2277" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2278">
@@ -93303,7 +93303,7 @@
       </c>
       <c r="I2278" t="inlineStr">
         <is>
-          <t>#action-pdf</t>
+          <t>action:pdf</t>
         </is>
       </c>
       <c r="R2278" t="inlineStr">
@@ -93315,7 +93315,7 @@
         <v>7</v>
       </c>
       <c r="T2278" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2279">
@@ -93346,7 +93346,7 @@
       </c>
       <c r="I2279" t="inlineStr">
         <is>
-          <t>#action-copy</t>
+          <t>action:copy</t>
         </is>
       </c>
       <c r="R2279" t="inlineStr">
@@ -93358,7 +93358,7 @@
         <v>1</v>
       </c>
       <c r="T2279" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2280">
@@ -93389,7 +93389,7 @@
       </c>
       <c r="I2280" t="inlineStr">
         <is>
-          <t>#action-whatsapp</t>
+          <t>action:whatsapp</t>
         </is>
       </c>
       <c r="R2280" t="inlineStr">
@@ -93401,7 +93401,7 @@
         <v>2</v>
       </c>
       <c r="T2280" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2281">
@@ -93432,7 +93432,7 @@
       </c>
       <c r="I2281" t="inlineStr">
         <is>
-          <t>#action-x</t>
+          <t>action:x</t>
         </is>
       </c>
       <c r="R2281" t="inlineStr">
@@ -93444,7 +93444,7 @@
         <v>3</v>
       </c>
       <c r="T2281" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2282">
@@ -93475,7 +93475,7 @@
       </c>
       <c r="I2282" t="inlineStr">
         <is>
-          <t>#action-linkedin</t>
+          <t>action:linkedin</t>
         </is>
       </c>
       <c r="R2282" t="inlineStr">
@@ -93487,7 +93487,7 @@
         <v>4</v>
       </c>
       <c r="T2282" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2283">
@@ -93518,7 +93518,7 @@
       </c>
       <c r="I2283" t="inlineStr">
         <is>
-          <t>#action-facebook</t>
+          <t>action:facebook</t>
         </is>
       </c>
       <c r="R2283" t="inlineStr">
@@ -93530,7 +93530,7 @@
         <v>5</v>
       </c>
       <c r="T2283" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2284">
@@ -93561,7 +93561,7 @@
       </c>
       <c r="I2284" t="inlineStr">
         <is>
-          <t>#action-email</t>
+          <t>action:email</t>
         </is>
       </c>
       <c r="R2284" t="inlineStr">
@@ -93573,7 +93573,7 @@
         <v>6</v>
       </c>
       <c r="T2284" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2285">
@@ -93604,7 +93604,7 @@
       </c>
       <c r="I2285" t="inlineStr">
         <is>
-          <t>#action-pdf</t>
+          <t>action:pdf</t>
         </is>
       </c>
       <c r="R2285" t="inlineStr">
@@ -93616,7 +93616,7 @@
         <v>7</v>
       </c>
       <c r="T2285" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2286">
@@ -93647,7 +93647,7 @@
       </c>
       <c r="I2286" t="inlineStr">
         <is>
-          <t>#action-copy</t>
+          <t>action:copy</t>
         </is>
       </c>
       <c r="R2286" t="inlineStr">
@@ -93659,7 +93659,7 @@
         <v>1</v>
       </c>
       <c r="T2286" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2287">
@@ -93690,7 +93690,7 @@
       </c>
       <c r="I2287" t="inlineStr">
         <is>
-          <t>#action-whatsapp</t>
+          <t>action:whatsapp</t>
         </is>
       </c>
       <c r="R2287" t="inlineStr">
@@ -93702,7 +93702,7 @@
         <v>2</v>
       </c>
       <c r="T2287" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2288">
@@ -93733,7 +93733,7 @@
       </c>
       <c r="I2288" t="inlineStr">
         <is>
-          <t>#action-x</t>
+          <t>action:x</t>
         </is>
       </c>
       <c r="R2288" t="inlineStr">
@@ -93745,7 +93745,7 @@
         <v>3</v>
       </c>
       <c r="T2288" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2289">
@@ -93776,7 +93776,7 @@
       </c>
       <c r="I2289" t="inlineStr">
         <is>
-          <t>#action-linkedin</t>
+          <t>action:linkedin</t>
         </is>
       </c>
       <c r="R2289" t="inlineStr">
@@ -93788,7 +93788,7 @@
         <v>4</v>
       </c>
       <c r="T2289" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2290">
@@ -93819,7 +93819,7 @@
       </c>
       <c r="I2290" t="inlineStr">
         <is>
-          <t>#action-facebook</t>
+          <t>action:facebook</t>
         </is>
       </c>
       <c r="R2290" t="inlineStr">
@@ -93831,7 +93831,7 @@
         <v>5</v>
       </c>
       <c r="T2290" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2291">
@@ -93862,7 +93862,7 @@
       </c>
       <c r="I2291" t="inlineStr">
         <is>
-          <t>#action-email</t>
+          <t>action:email</t>
         </is>
       </c>
       <c r="R2291" t="inlineStr">
@@ -93874,7 +93874,7 @@
         <v>6</v>
       </c>
       <c r="T2291" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2292">
@@ -93905,7 +93905,7 @@
       </c>
       <c r="I2292" t="inlineStr">
         <is>
-          <t>#action-pdf</t>
+          <t>action:pdf</t>
         </is>
       </c>
       <c r="R2292" t="inlineStr">
@@ -93917,7 +93917,7 @@
         <v>7</v>
       </c>
       <c r="T2292" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2293">
@@ -93948,7 +93948,7 @@
       </c>
       <c r="I2293" t="inlineStr">
         <is>
-          <t>#action-copy</t>
+          <t>action:copy</t>
         </is>
       </c>
       <c r="R2293" t="inlineStr">
@@ -93960,7 +93960,7 @@
         <v>1</v>
       </c>
       <c r="T2293" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2294">
@@ -93991,7 +93991,7 @@
       </c>
       <c r="I2294" t="inlineStr">
         <is>
-          <t>#action-whatsapp</t>
+          <t>action:whatsapp</t>
         </is>
       </c>
       <c r="R2294" t="inlineStr">
@@ -94003,7 +94003,7 @@
         <v>2</v>
       </c>
       <c r="T2294" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2295">
@@ -94034,7 +94034,7 @@
       </c>
       <c r="I2295" t="inlineStr">
         <is>
-          <t>#action-x</t>
+          <t>action:x</t>
         </is>
       </c>
       <c r="R2295" t="inlineStr">
@@ -94046,7 +94046,7 @@
         <v>3</v>
       </c>
       <c r="T2295" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2296">
@@ -94077,7 +94077,7 @@
       </c>
       <c r="I2296" t="inlineStr">
         <is>
-          <t>#action-linkedin</t>
+          <t>action:linkedin</t>
         </is>
       </c>
       <c r="R2296" t="inlineStr">
@@ -94089,7 +94089,7 @@
         <v>4</v>
       </c>
       <c r="T2296" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2297">
@@ -94120,7 +94120,7 @@
       </c>
       <c r="I2297" t="inlineStr">
         <is>
-          <t>#action-facebook</t>
+          <t>action:facebook</t>
         </is>
       </c>
       <c r="R2297" t="inlineStr">
@@ -94132,7 +94132,7 @@
         <v>5</v>
       </c>
       <c r="T2297" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2298">
@@ -94163,7 +94163,7 @@
       </c>
       <c r="I2298" t="inlineStr">
         <is>
-          <t>#action-email</t>
+          <t>action:email</t>
         </is>
       </c>
       <c r="R2298" t="inlineStr">
@@ -94175,7 +94175,7 @@
         <v>6</v>
       </c>
       <c r="T2298" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2299">
@@ -94206,7 +94206,7 @@
       </c>
       <c r="I2299" t="inlineStr">
         <is>
-          <t>#action-pdf</t>
+          <t>action:pdf</t>
         </is>
       </c>
       <c r="R2299" t="inlineStr">
@@ -94218,7 +94218,7 @@
         <v>7</v>
       </c>
       <c r="T2299" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2300">
@@ -94249,7 +94249,7 @@
       </c>
       <c r="I2300" t="inlineStr">
         <is>
-          <t>#action-copy</t>
+          <t>action:copy</t>
         </is>
       </c>
       <c r="R2300" t="inlineStr">
@@ -94261,7 +94261,7 @@
         <v>1</v>
       </c>
       <c r="T2300" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2301">
@@ -94292,7 +94292,7 @@
       </c>
       <c r="I2301" t="inlineStr">
         <is>
-          <t>#action-whatsapp</t>
+          <t>action:whatsapp</t>
         </is>
       </c>
       <c r="R2301" t="inlineStr">
@@ -94304,7 +94304,7 @@
         <v>2</v>
       </c>
       <c r="T2301" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2302">
@@ -94335,7 +94335,7 @@
       </c>
       <c r="I2302" t="inlineStr">
         <is>
-          <t>#action-x</t>
+          <t>action:x</t>
         </is>
       </c>
       <c r="R2302" t="inlineStr">
@@ -94347,7 +94347,7 @@
         <v>3</v>
       </c>
       <c r="T2302" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2303">
@@ -94378,7 +94378,7 @@
       </c>
       <c r="I2303" t="inlineStr">
         <is>
-          <t>#action-linkedin</t>
+          <t>action:linkedin</t>
         </is>
       </c>
       <c r="R2303" t="inlineStr">
@@ -94390,7 +94390,7 @@
         <v>4</v>
       </c>
       <c r="T2303" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2304">
@@ -94421,7 +94421,7 @@
       </c>
       <c r="I2304" t="inlineStr">
         <is>
-          <t>#action-facebook</t>
+          <t>action:facebook</t>
         </is>
       </c>
       <c r="R2304" t="inlineStr">
@@ -94433,7 +94433,7 @@
         <v>5</v>
       </c>
       <c r="T2304" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2305">
@@ -94464,7 +94464,7 @@
       </c>
       <c r="I2305" t="inlineStr">
         <is>
-          <t>#action-email</t>
+          <t>action:email</t>
         </is>
       </c>
       <c r="R2305" t="inlineStr">
@@ -94476,7 +94476,7 @@
         <v>6</v>
       </c>
       <c r="T2305" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2306">
@@ -94507,7 +94507,7 @@
       </c>
       <c r="I2306" t="inlineStr">
         <is>
-          <t>#action-pdf</t>
+          <t>action:pdf</t>
         </is>
       </c>
       <c r="R2306" t="inlineStr">
@@ -94519,7 +94519,7 @@
         <v>7</v>
       </c>
       <c r="T2306" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2307">
@@ -94550,7 +94550,7 @@
       </c>
       <c r="I2307" t="inlineStr">
         <is>
-          <t>#action-copy</t>
+          <t>action:copy</t>
         </is>
       </c>
       <c r="R2307" t="inlineStr">
@@ -94562,7 +94562,7 @@
         <v>1</v>
       </c>
       <c r="T2307" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2308">
@@ -94593,7 +94593,7 @@
       </c>
       <c r="I2308" t="inlineStr">
         <is>
-          <t>#action-whatsapp</t>
+          <t>action:whatsapp</t>
         </is>
       </c>
       <c r="R2308" t="inlineStr">
@@ -94605,7 +94605,7 @@
         <v>2</v>
       </c>
       <c r="T2308" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2309">
@@ -94636,7 +94636,7 @@
       </c>
       <c r="I2309" t="inlineStr">
         <is>
-          <t>#action-x</t>
+          <t>action:x</t>
         </is>
       </c>
       <c r="R2309" t="inlineStr">
@@ -94648,7 +94648,7 @@
         <v>3</v>
       </c>
       <c r="T2309" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2310">
@@ -94679,7 +94679,7 @@
       </c>
       <c r="I2310" t="inlineStr">
         <is>
-          <t>#action-linkedin</t>
+          <t>action:linkedin</t>
         </is>
       </c>
       <c r="R2310" t="inlineStr">
@@ -94691,7 +94691,7 @@
         <v>4</v>
       </c>
       <c r="T2310" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2311">
@@ -94722,7 +94722,7 @@
       </c>
       <c r="I2311" t="inlineStr">
         <is>
-          <t>#action-facebook</t>
+          <t>action:facebook</t>
         </is>
       </c>
       <c r="R2311" t="inlineStr">
@@ -94734,7 +94734,7 @@
         <v>5</v>
       </c>
       <c r="T2311" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2312">
@@ -94765,7 +94765,7 @@
       </c>
       <c r="I2312" t="inlineStr">
         <is>
-          <t>#action-email</t>
+          <t>action:email</t>
         </is>
       </c>
       <c r="R2312" t="inlineStr">
@@ -94777,7 +94777,7 @@
         <v>6</v>
       </c>
       <c r="T2312" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2313">
@@ -94808,7 +94808,7 @@
       </c>
       <c r="I2313" t="inlineStr">
         <is>
-          <t>#action-pdf</t>
+          <t>action:pdf</t>
         </is>
       </c>
       <c r="R2313" t="inlineStr">
@@ -94820,7 +94820,7 @@
         <v>7</v>
       </c>
       <c r="T2313" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EN-menu: 76 URLs ingevuld naar bestaande EN-vertalingen; 3.16.5 gedeactiveerd
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -24498,6 +24498,11 @@
           <t>GCS — krantbriefing</t>
         </is>
       </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>research/krantbriefing.html</t>
+        </is>
+      </c>
       <c r="R567" t="inlineStr">
         <is>
           <t>live</t>
@@ -24574,6 +24579,11 @@
           <t>GCS — volledig plan</t>
         </is>
       </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>research/gevoelsconnectiesysteem-volledig.html</t>
+        </is>
+      </c>
       <c r="R569" t="inlineStr">
         <is>
           <t>live</t>
@@ -24612,6 +24622,11 @@
           <t>Het gevoelsconnectiesysteem</t>
         </is>
       </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>research/gevoelsconnectiesysteem.html</t>
+        </is>
+      </c>
       <c r="R570" t="inlineStr">
         <is>
           <t>live</t>
@@ -24774,6 +24789,11 @@
           <t>Alles stroomt — de moeder van alle wetenschap</t>
         </is>
       </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>edition-1/fluid-dynamics.html</t>
+        </is>
+      </c>
       <c r="R574" t="inlineStr">
         <is>
           <t>live</t>
@@ -24898,6 +24918,11 @@
           <t>De Kosaris — Boek Twee — Diakrisis</t>
         </is>
       </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>reading-book-two/index.html</t>
+        </is>
+      </c>
       <c r="R577" t="inlineStr">
         <is>
           <t>live</t>
@@ -24936,6 +24961,11 @@
           <t>De Kosaris — Boek Drie — Het boek van Anthea</t>
         </is>
       </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>reading-book-three/index.html</t>
+        </is>
+      </c>
       <c r="R578" t="inlineStr">
         <is>
           <t>live</t>
@@ -24974,6 +25004,11 @@
           <t>De Kosaris — Boek Vier — Het boek van het hydrolysaat</t>
         </is>
       </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>reading-book-four/index.html</t>
+        </is>
+      </c>
       <c r="R579" t="inlineStr">
         <is>
           <t>live</t>
@@ -25012,6 +25047,11 @@
           <t>De Kosaris — Boek Vijf — Het boek van de partner</t>
         </is>
       </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>reading-book-five/index.html</t>
+        </is>
+      </c>
       <c r="R580" t="inlineStr">
         <is>
           <t>live</t>
@@ -25093,6 +25133,11 @@
           <t>Drie dimensies zijn te weinig</t>
         </is>
       </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>edition-1/dimensions.html</t>
+        </is>
+      </c>
       <c r="R582" t="inlineStr">
         <is>
           <t>live</t>
@@ -25174,6 +25219,11 @@
           <t>Hoe alles samenhangt</t>
         </is>
       </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>edition-1/synthesis.html</t>
+        </is>
+      </c>
       <c r="R584" t="inlineStr">
         <is>
           <t>live</t>
@@ -25298,6 +25348,11 @@
           <t>Zeven Dimensies</t>
         </is>
       </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>edition-2/seven-dimensions.html</t>
+        </is>
+      </c>
       <c r="R587" t="inlineStr">
         <is>
           <t>live</t>
@@ -25966,6 +26021,11 @@
           <t>Tien seconden</t>
         </is>
       </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>idee.html</t>
+        </is>
+      </c>
       <c r="R603" t="inlineStr">
         <is>
           <t>live</t>
@@ -26004,6 +26064,11 @@
           <t>Waarom ik ben zoals ik ben</t>
         </is>
       </c>
+      <c r="I604" t="inlineStr">
+        <is>
+          <t>edition-2/why-i-am-as-i-am.html</t>
+        </is>
+      </c>
       <c r="R604" t="inlineStr">
         <is>
           <t>live</t>
@@ -26844,6 +26909,11 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>stemgedrag.html</t>
+        </is>
+      </c>
       <c r="R624" t="inlineStr">
         <is>
           <t>live</t>
@@ -26968,6 +27038,11 @@
           <t>Het politieke landschap</t>
         </is>
       </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>what-surfaces/plundering-4-politieke-landschap.html</t>
+        </is>
+      </c>
       <c r="R627" t="inlineStr">
         <is>
           <t>live</t>
@@ -27092,6 +27167,11 @@
           <t>Trump als spiegel</t>
         </is>
       </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>what-surfaces/trump-als-spiegel.html</t>
+        </is>
+      </c>
       <c r="R630" t="inlineStr">
         <is>
           <t>live</t>
@@ -27555,6 +27635,11 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>nitrogen-edition/three-problems-one-answer.html</t>
+        </is>
+      </c>
       <c r="R641" t="inlineStr">
         <is>
           <t>live</t>
@@ -27593,6 +27678,11 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>climate-edition/index.html</t>
+        </is>
+      </c>
       <c r="R642" t="inlineStr">
         <is>
           <t>live</t>
@@ -27803,6 +27893,11 @@
           <t>Uw thermostaat is slimmer dan uw minister</t>
         </is>
       </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>edition-2/thermostat.html</t>
+        </is>
+      </c>
       <c r="R647" t="inlineStr">
         <is>
           <t>live</t>
@@ -28175,6 +28270,11 @@
           <t>De biomimetische krachtcentrale</t>
         </is>
       </c>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>edition-0/biomimetic-power-plant.html</t>
+        </is>
+      </c>
       <c r="R656" t="inlineStr">
         <is>
           <t>live</t>
@@ -28213,6 +28313,11 @@
           <t>De Brusselse Gevolgenkaart — BiCRS-versie</t>
         </is>
       </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>what-surfaces/brusselse-gevolgenkaart-bicrs.html</t>
+        </is>
+      </c>
       <c r="R657" t="inlineStr">
         <is>
           <t>live</t>
@@ -28294,6 +28399,11 @@
           <t>De op de natuur aangepaste analyse</t>
         </is>
       </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>what-surfaces/de-op-de-natuur-aangepaste-analyse.html</t>
+        </is>
+      </c>
       <c r="R659" t="inlineStr">
         <is>
           <t>live</t>
@@ -28375,6 +28485,11 @@
           <t>Editie Europa</t>
         </is>
       </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>edition-0/index.html</t>
+        </is>
+      </c>
       <c r="R661" t="inlineStr">
         <is>
           <t>live</t>
@@ -28413,6 +28528,11 @@
           <t>Mensen die mee bouwen</t>
         </is>
       </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>what-surfaces/mensen-die-mee-bouwen.html</t>
+        </is>
+      </c>
       <c r="R662" t="inlineStr">
         <is>
           <t>live</t>
@@ -28537,6 +28657,11 @@
           <t>Visie 2036</t>
         </is>
       </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>what-surfaces/carbon-alert-visie-2036.html</t>
+        </is>
+      </c>
       <c r="R665" t="inlineStr">
         <is>
           <t>live</t>
@@ -28575,6 +28700,11 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>edition-0/carbon-alert-europa.html</t>
+        </is>
+      </c>
       <c r="R666" t="inlineStr">
         <is>
           <t>live</t>
@@ -28780,6 +28910,11 @@
           <t>De actor is de regel</t>
         </is>
       </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>what-surfaces/de-actor-is-de-regel.html</t>
+        </is>
+      </c>
       <c r="R671" t="inlineStr">
         <is>
           <t>live</t>
@@ -29076,6 +29211,11 @@
           <t>De prijs van de bloei</t>
         </is>
       </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>edition-2/education-price-of-the-bloom.html</t>
+        </is>
+      </c>
       <c r="R678" t="inlineStr">
         <is>
           <t>live</t>
@@ -29372,6 +29512,11 @@
           <t>Editie 2</t>
         </is>
       </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>edition-2/index.html</t>
+        </is>
+      </c>
       <c r="R685" t="inlineStr">
         <is>
           <t>live</t>
@@ -29496,6 +29641,11 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>vote-impact-app/energie/index.html</t>
+        </is>
+      </c>
       <c r="R688" t="inlineStr">
         <is>
           <t>live</t>
@@ -29577,6 +29727,11 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>vote-impact-app/industrie/index.html</t>
+        </is>
+      </c>
       <c r="R690" t="inlineStr">
         <is>
           <t>live</t>
@@ -29615,6 +29770,11 @@
           <t>Kies een kant</t>
         </is>
       </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>edition-2/education-choose-a-side.html</t>
+        </is>
+      </c>
       <c r="R691" t="inlineStr">
         <is>
           <t>live</t>
@@ -29696,6 +29856,11 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/methode/index.html</t>
+        </is>
+      </c>
       <c r="R693" t="inlineStr">
         <is>
           <t>live</t>
@@ -29992,6 +30157,11 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/index.html</t>
+        </is>
+      </c>
       <c r="R700" t="inlineStr">
         <is>
           <t>live</t>
@@ -30030,6 +30200,11 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
+      <c r="I701" t="inlineStr">
+        <is>
+          <t>edition-4/artikel-00-redactie.html</t>
+        </is>
+      </c>
       <c r="R701" t="inlineStr">
         <is>
           <t>live</t>
@@ -30111,6 +30286,11 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
+      <c r="I703" t="inlineStr">
+        <is>
+          <t>vote-impact-app/scholing/index.html</t>
+        </is>
+      </c>
       <c r="R703" t="inlineStr">
         <is>
           <t>live</t>
@@ -30192,6 +30372,11 @@
           <t>Terug naar de werkbank, vooruit naar het denken</t>
         </is>
       </c>
+      <c r="I705" t="inlineStr">
+        <is>
+          <t>edition-2/education-back-to-the-workbench.html</t>
+        </is>
+      </c>
       <c r="R705" t="inlineStr">
         <is>
           <t>live</t>
@@ -30359,6 +30544,11 @@
           <t>Van leerfabriek naar leerwerkplaats</t>
         </is>
       </c>
+      <c r="I709" t="inlineStr">
+        <is>
+          <t>edition-1/education.html</t>
+        </is>
+      </c>
       <c r="R709" t="inlineStr">
         <is>
           <t>live</t>
@@ -30736,6 +30926,11 @@
           <t>De NEPK-Klimaatlogica: Zelfversterkende Systeemcrisis</t>
         </is>
       </c>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>edition-2/nepk-climate-logic.html</t>
+        </is>
+      </c>
       <c r="R718" t="inlineStr">
         <is>
           <t>live</t>
@@ -30936,6 +31131,11 @@
           <t>Nederland · Toekomst</t>
         </is>
       </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/netherlands/index.html</t>
+        </is>
+      </c>
       <c r="R723" t="inlineStr">
         <is>
           <t>live</t>
@@ -30974,6 +31174,11 @@
           <t>Stille Analyse</t>
         </is>
       </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>what-surfaces/gevolgenkaart-iii-stille-analyse.html</t>
+        </is>
+      </c>
       <c r="R724" t="inlineStr">
         <is>
           <t>live</t>
@@ -31260,6 +31465,11 @@
           <t>De Brusselse Gevolgenkaart — BiCRS-versie</t>
         </is>
       </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>what-surfaces/brusselse-gevolgenkaart-bicrs.html</t>
+        </is>
+      </c>
       <c r="R731" t="inlineStr">
         <is>
           <t>live</t>
@@ -31513,6 +31723,11 @@
           <t>Die Konsequenzkarte</t>
         </is>
       </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>what-surfaces/die-konsequenzkarte.html</t>
+        </is>
+      </c>
       <c r="R737" t="inlineStr">
         <is>
           <t>live</t>
@@ -31551,6 +31766,11 @@
           <t>Duitsland · Toekomst</t>
         </is>
       </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/duitsland/index.html</t>
+        </is>
+      </c>
       <c r="R738" t="inlineStr">
         <is>
           <t>live</t>
@@ -31718,6 +31938,11 @@
           <t>Europa · Toekomst</t>
         </is>
       </c>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/europa/index.html</t>
+        </is>
+      </c>
       <c r="R742" t="inlineStr">
         <is>
           <t>live</t>
@@ -32530,6 +32755,11 @@
           <t>Het immuunsysteem dat gezonde cellen aanvalt</t>
         </is>
       </c>
+      <c r="I761" t="inlineStr">
+        <is>
+          <t>what-surfaces/het-immuunsysteem-van-organisaties.html</t>
+        </is>
+      </c>
       <c r="R761" t="inlineStr">
         <is>
           <t>live</t>
@@ -32654,6 +32884,11 @@
           <t>Trump als spiegel</t>
         </is>
       </c>
+      <c r="I764" t="inlineStr">
+        <is>
+          <t>what-surfaces/trump-als-spiegel.html</t>
+        </is>
+      </c>
       <c r="R764" t="inlineStr">
         <is>
           <t>live</t>
@@ -32821,6 +33056,11 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
+      <c r="I768" t="inlineStr">
+        <is>
+          <t>edition-0/carbon-alert-europa.html</t>
+        </is>
+      </c>
       <c r="R768" t="inlineStr">
         <is>
           <t>live</t>
@@ -32859,6 +33099,11 @@
           <t>Zij doden hun levensaders</t>
         </is>
       </c>
+      <c r="I769" t="inlineStr">
+        <is>
+          <t>what-surfaces/zij-doden-hun-levensaders-brussel.html</t>
+        </is>
+      </c>
       <c r="R769" t="inlineStr">
         <is>
           <t>live</t>
@@ -33279,6 +33524,11 @@
           <t>Editie 1</t>
         </is>
       </c>
+      <c r="I779" t="inlineStr">
+        <is>
+          <t>edition-1/index.html</t>
+        </is>
+      </c>
       <c r="R779" t="inlineStr">
         <is>
           <t>live</t>
@@ -33317,6 +33567,11 @@
           <t>Editie 5 — portaal</t>
         </is>
       </c>
+      <c r="I780" t="inlineStr">
+        <is>
+          <t>edition-5/index.html</t>
+        </is>
+      </c>
       <c r="R780" t="inlineStr">
         <is>
           <t>live</t>
@@ -33355,6 +33610,11 @@
           <t>Een fusiereactor zonder magnetische kooi</t>
         </is>
       </c>
+      <c r="I781" t="inlineStr">
+        <is>
+          <t>edition-1/fusion.html</t>
+        </is>
+      </c>
       <c r="R781" t="inlineStr">
         <is>
           <t>live</t>
@@ -33393,6 +33653,11 @@
           <t>Veerkracht en Selectie</t>
         </is>
       </c>
+      <c r="I782" t="inlineStr">
+        <is>
+          <t>edition-2/resilience-and-selection.html</t>
+        </is>
+      </c>
       <c r="R782" t="inlineStr">
         <is>
           <t>live</t>
@@ -33431,6 +33696,11 @@
           <t>Wat er nu al ligt</t>
         </is>
       </c>
+      <c r="I783" t="inlineStr">
+        <is>
+          <t>edition-1/technical-solutions.html</t>
+        </is>
+      </c>
       <c r="R783" t="inlineStr">
         <is>
           <t>live</t>
@@ -33593,6 +33863,11 @@
           <t>Afloop</t>
         </is>
       </c>
+      <c r="I787" t="inlineStr">
+        <is>
+          <t>what-surfaces/plundering-3-afloop.html</t>
+        </is>
+      </c>
       <c r="R787" t="inlineStr">
         <is>
           <t>live</t>
@@ -33674,6 +33949,11 @@
           <t>De Grote Plundering</t>
         </is>
       </c>
+      <c r="I789" t="inlineStr">
+        <is>
+          <t>what-surfaces/de-grote-plundering.html</t>
+        </is>
+      </c>
       <c r="R789" t="inlineStr">
         <is>
           <t>live</t>
@@ -33712,6 +33992,11 @@
           <t>Diagnose</t>
         </is>
       </c>
+      <c r="I790" t="inlineStr">
+        <is>
+          <t>what-surfaces/plundering-1-diagnose.html</t>
+        </is>
+      </c>
       <c r="R790" t="inlineStr">
         <is>
           <t>live</t>
@@ -33922,6 +34207,11 @@
           <t>Het politieke landschap</t>
         </is>
       </c>
+      <c r="I795" t="inlineStr">
+        <is>
+          <t>what-surfaces/plundering-4-politieke-landschap.html</t>
+        </is>
+      </c>
       <c r="R795" t="inlineStr">
         <is>
           <t>live</t>
@@ -33960,6 +34250,11 @@
           <t>Mechaniek</t>
         </is>
       </c>
+      <c r="I796" t="inlineStr">
+        <is>
+          <t>what-surfaces/plundering-2-mechaniek.html</t>
+        </is>
+      </c>
       <c r="R796" t="inlineStr">
         <is>
           <t>live</t>
@@ -34079,6 +34374,11 @@
           <t>Van Belasten naar Aantrekken</t>
         </is>
       </c>
+      <c r="I799" t="inlineStr">
+        <is>
+          <t>edition-2/policy-advice-attract.html</t>
+        </is>
+      </c>
       <c r="R799" t="inlineStr">
         <is>
           <t>live</t>
@@ -34284,6 +34584,11 @@
           <t>Achter de Cijfers</t>
         </is>
       </c>
+      <c r="I804" t="inlineStr">
+        <is>
+          <t>research/index.html</t>
+        </is>
+      </c>
       <c r="R804" t="inlineStr">
         <is>
           <t>live</t>
@@ -34322,6 +34627,11 @@
           <t>Dossiers</t>
         </is>
       </c>
+      <c r="I805" t="inlineStr">
+        <is>
+          <t>dossiers/index.html</t>
+        </is>
+      </c>
       <c r="R805" t="inlineStr">
         <is>
           <t>live</t>
@@ -34360,6 +34670,11 @@
           <t>EU: BBP, Reële Lonen en de Overheidsmultiplicator</t>
         </is>
       </c>
+      <c r="I806" t="inlineStr">
+        <is>
+          <t>onderzoek/eu-multiplicator.html</t>
+        </is>
+      </c>
       <c r="R806" t="inlineStr">
         <is>
           <t>live</t>
@@ -34398,6 +34713,11 @@
           <t>GCS — krantbriefing</t>
         </is>
       </c>
+      <c r="I807" t="inlineStr">
+        <is>
+          <t>research/krantbriefing.html</t>
+        </is>
+      </c>
       <c r="R807" t="inlineStr">
         <is>
           <t>live</t>
@@ -34474,6 +34794,11 @@
           <t>GCS — volledig plan</t>
         </is>
       </c>
+      <c r="I809" t="inlineStr">
+        <is>
+          <t>research/gevoelsconnectiesysteem-volledig.html</t>
+        </is>
+      </c>
       <c r="R809" t="inlineStr">
         <is>
           <t>live</t>
@@ -34512,6 +34837,11 @@
           <t>Het gevoelsconnectiesysteem</t>
         </is>
       </c>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>research/gevoelsconnectiesysteem.html</t>
+        </is>
+      </c>
       <c r="R810" t="inlineStr">
         <is>
           <t>live</t>
@@ -34550,6 +34880,11 @@
           <t>Is Nederland op weg naar ontwikkelingslandstatus?</t>
         </is>
       </c>
+      <c r="I811" t="inlineStr">
+        <is>
+          <t>onderzoek/ontwikkelingslandstatus.html</t>
+        </is>
+      </c>
       <c r="R811" t="inlineStr">
         <is>
           <t>live</t>
@@ -34712,6 +35047,11 @@
           <t>Archief</t>
         </is>
       </c>
+      <c r="I815" t="inlineStr">
+        <is>
+          <t>archive.html</t>
+        </is>
+      </c>
       <c r="R815" t="inlineStr">
         <is>
           <t>live</t>
@@ -34793,6 +35133,11 @@
           <t>Colofon</t>
         </is>
       </c>
+      <c r="I817" t="inlineStr">
+        <is>
+          <t>colofon.html</t>
+        </is>
+      </c>
       <c r="R817" t="inlineStr">
         <is>
           <t>live</t>
@@ -34831,6 +35176,11 @@
           <t>Het Open Vizier verder dragen</t>
         </is>
       </c>
+      <c r="I818" t="inlineStr">
+        <is>
+          <t>delen.html</t>
+        </is>
+      </c>
       <c r="R818" t="inlineStr">
         <is>
           <t>live</t>
@@ -34878,7 +35228,7 @@
         <v>5</v>
       </c>
       <c r="T819" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="820">
@@ -34907,6 +35257,11 @@
           <t>Hoe u meedoet aan de discussie</t>
         </is>
       </c>
+      <c r="I820" t="inlineStr">
+        <is>
+          <t>edition-1/discussion.html</t>
+        </is>
+      </c>
       <c r="R820" t="inlineStr">
         <is>
           <t>live</t>
@@ -34945,6 +35300,11 @@
           <t>Navigatie</t>
         </is>
       </c>
+      <c r="I821" t="inlineStr">
+        <is>
+          <t>navigatie.html</t>
+        </is>
+      </c>
       <c r="R821" t="inlineStr">
         <is>
           <t>live</t>
@@ -34983,6 +35343,11 @@
           <t>Op de hoogte blijven</t>
         </is>
       </c>
+      <c r="I822" t="inlineStr">
+        <is>
+          <t>op-de-hoogte.html</t>
+        </is>
+      </c>
       <c r="R822" t="inlineStr">
         <is>
           <t>live</t>
@@ -35107,6 +35472,11 @@
           <t>Structuur — Beheer</t>
         </is>
       </c>
+      <c r="I825" t="inlineStr">
+        <is>
+          <t>structuur.html</t>
+        </is>
+      </c>
       <c r="R825" t="inlineStr">
         <is>
           <t>live</t>
@@ -35188,6 +35558,11 @@
           <t>Waarom deze krant?</t>
         </is>
       </c>
+      <c r="I827" t="inlineStr">
+        <is>
+          <t>edition-1/foreword.html</t>
+        </is>
+      </c>
       <c r="R827" t="inlineStr">
         <is>
           <t>live</t>
@@ -35224,6 +35599,11 @@
       <c r="F828" t="inlineStr">
         <is>
           <t>Wat opkomt</t>
+        </is>
+      </c>
+      <c r="I828" t="inlineStr">
+        <is>
+          <t>what-surfaces/index.html</t>
         </is>
       </c>
       <c r="R828" t="inlineStr">

</xml_diff>

<commit_message>
REVERT: xlsx + Kosaris boek3-deel1 videos terug naar staat 18 aug
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -24498,11 +24498,6 @@
           <t>GCS — krantbriefing</t>
         </is>
       </c>
-      <c r="I567" t="inlineStr">
-        <is>
-          <t>research/krantbriefing.html</t>
-        </is>
-      </c>
       <c r="R567" t="inlineStr">
         <is>
           <t>live</t>
@@ -24579,11 +24574,6 @@
           <t>GCS — volledig plan</t>
         </is>
       </c>
-      <c r="I569" t="inlineStr">
-        <is>
-          <t>research/gevoelsconnectiesysteem-volledig.html</t>
-        </is>
-      </c>
       <c r="R569" t="inlineStr">
         <is>
           <t>live</t>
@@ -24622,11 +24612,6 @@
           <t>Het gevoelsconnectiesysteem</t>
         </is>
       </c>
-      <c r="I570" t="inlineStr">
-        <is>
-          <t>research/gevoelsconnectiesysteem.html</t>
-        </is>
-      </c>
       <c r="R570" t="inlineStr">
         <is>
           <t>live</t>
@@ -24789,11 +24774,6 @@
           <t>Alles stroomt — de moeder van alle wetenschap</t>
         </is>
       </c>
-      <c r="I574" t="inlineStr">
-        <is>
-          <t>edition-1/fluid-dynamics.html</t>
-        </is>
-      </c>
       <c r="R574" t="inlineStr">
         <is>
           <t>live</t>
@@ -24918,11 +24898,6 @@
           <t>De Kosaris — Boek Twee — Diakrisis</t>
         </is>
       </c>
-      <c r="I577" t="inlineStr">
-        <is>
-          <t>reading-book-two/index.html</t>
-        </is>
-      </c>
       <c r="R577" t="inlineStr">
         <is>
           <t>live</t>
@@ -24961,11 +24936,6 @@
           <t>De Kosaris — Boek Drie — Het boek van Anthea</t>
         </is>
       </c>
-      <c r="I578" t="inlineStr">
-        <is>
-          <t>reading-book-three/index.html</t>
-        </is>
-      </c>
       <c r="R578" t="inlineStr">
         <is>
           <t>live</t>
@@ -25004,11 +24974,6 @@
           <t>De Kosaris — Boek Vier — Het boek van het hydrolysaat</t>
         </is>
       </c>
-      <c r="I579" t="inlineStr">
-        <is>
-          <t>reading-book-four/index.html</t>
-        </is>
-      </c>
       <c r="R579" t="inlineStr">
         <is>
           <t>live</t>
@@ -25047,11 +25012,6 @@
           <t>De Kosaris — Boek Vijf — Het boek van de partner</t>
         </is>
       </c>
-      <c r="I580" t="inlineStr">
-        <is>
-          <t>reading-book-five/index.html</t>
-        </is>
-      </c>
       <c r="R580" t="inlineStr">
         <is>
           <t>live</t>
@@ -25133,11 +25093,6 @@
           <t>Drie dimensies zijn te weinig</t>
         </is>
       </c>
-      <c r="I582" t="inlineStr">
-        <is>
-          <t>edition-1/dimensions.html</t>
-        </is>
-      </c>
       <c r="R582" t="inlineStr">
         <is>
           <t>live</t>
@@ -25219,11 +25174,6 @@
           <t>Hoe alles samenhangt</t>
         </is>
       </c>
-      <c r="I584" t="inlineStr">
-        <is>
-          <t>edition-1/synthesis.html</t>
-        </is>
-      </c>
       <c r="R584" t="inlineStr">
         <is>
           <t>live</t>
@@ -25348,11 +25298,6 @@
           <t>Zeven Dimensies</t>
         </is>
       </c>
-      <c r="I587" t="inlineStr">
-        <is>
-          <t>edition-2/seven-dimensions.html</t>
-        </is>
-      </c>
       <c r="R587" t="inlineStr">
         <is>
           <t>live</t>
@@ -26021,11 +25966,6 @@
           <t>Tien seconden</t>
         </is>
       </c>
-      <c r="I603" t="inlineStr">
-        <is>
-          <t>idee.html</t>
-        </is>
-      </c>
       <c r="R603" t="inlineStr">
         <is>
           <t>live</t>
@@ -26064,11 +26004,6 @@
           <t>Waarom ik ben zoals ik ben</t>
         </is>
       </c>
-      <c r="I604" t="inlineStr">
-        <is>
-          <t>edition-2/why-i-am-as-i-am.html</t>
-        </is>
-      </c>
       <c r="R604" t="inlineStr">
         <is>
           <t>live</t>
@@ -26909,11 +26844,6 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
-      <c r="I624" t="inlineStr">
-        <is>
-          <t>stemgedrag.html</t>
-        </is>
-      </c>
       <c r="R624" t="inlineStr">
         <is>
           <t>live</t>
@@ -27038,11 +26968,6 @@
           <t>Het politieke landschap</t>
         </is>
       </c>
-      <c r="I627" t="inlineStr">
-        <is>
-          <t>what-surfaces/plundering-4-politieke-landschap.html</t>
-        </is>
-      </c>
       <c r="R627" t="inlineStr">
         <is>
           <t>live</t>
@@ -27167,11 +27092,6 @@
           <t>Trump als spiegel</t>
         </is>
       </c>
-      <c r="I630" t="inlineStr">
-        <is>
-          <t>what-surfaces/trump-als-spiegel.html</t>
-        </is>
-      </c>
       <c r="R630" t="inlineStr">
         <is>
           <t>live</t>
@@ -27635,11 +27555,6 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
-      <c r="I641" t="inlineStr">
-        <is>
-          <t>nitrogen-edition/three-problems-one-answer.html</t>
-        </is>
-      </c>
       <c r="R641" t="inlineStr">
         <is>
           <t>live</t>
@@ -27678,11 +27593,6 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
-      <c r="I642" t="inlineStr">
-        <is>
-          <t>climate-edition/index.html</t>
-        </is>
-      </c>
       <c r="R642" t="inlineStr">
         <is>
           <t>live</t>
@@ -27893,11 +27803,6 @@
           <t>Uw thermostaat is slimmer dan uw minister</t>
         </is>
       </c>
-      <c r="I647" t="inlineStr">
-        <is>
-          <t>edition-2/thermostat.html</t>
-        </is>
-      </c>
       <c r="R647" t="inlineStr">
         <is>
           <t>live</t>
@@ -28270,11 +28175,6 @@
           <t>De biomimetische krachtcentrale</t>
         </is>
       </c>
-      <c r="I656" t="inlineStr">
-        <is>
-          <t>edition-0/biomimetic-power-plant.html</t>
-        </is>
-      </c>
       <c r="R656" t="inlineStr">
         <is>
           <t>live</t>
@@ -28313,11 +28213,6 @@
           <t>De Brusselse Gevolgenkaart — BiCRS-versie</t>
         </is>
       </c>
-      <c r="I657" t="inlineStr">
-        <is>
-          <t>what-surfaces/brusselse-gevolgenkaart-bicrs.html</t>
-        </is>
-      </c>
       <c r="R657" t="inlineStr">
         <is>
           <t>live</t>
@@ -28399,11 +28294,6 @@
           <t>De op de natuur aangepaste analyse</t>
         </is>
       </c>
-      <c r="I659" t="inlineStr">
-        <is>
-          <t>what-surfaces/de-op-de-natuur-aangepaste-analyse.html</t>
-        </is>
-      </c>
       <c r="R659" t="inlineStr">
         <is>
           <t>live</t>
@@ -28485,11 +28375,6 @@
           <t>Editie Europa</t>
         </is>
       </c>
-      <c r="I661" t="inlineStr">
-        <is>
-          <t>edition-0/index.html</t>
-        </is>
-      </c>
       <c r="R661" t="inlineStr">
         <is>
           <t>live</t>
@@ -28528,11 +28413,6 @@
           <t>Mensen die mee bouwen</t>
         </is>
       </c>
-      <c r="I662" t="inlineStr">
-        <is>
-          <t>what-surfaces/mensen-die-mee-bouwen.html</t>
-        </is>
-      </c>
       <c r="R662" t="inlineStr">
         <is>
           <t>live</t>
@@ -28657,11 +28537,6 @@
           <t>Visie 2036</t>
         </is>
       </c>
-      <c r="I665" t="inlineStr">
-        <is>
-          <t>what-surfaces/carbon-alert-visie-2036.html</t>
-        </is>
-      </c>
       <c r="R665" t="inlineStr">
         <is>
           <t>live</t>
@@ -28700,11 +28575,6 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
-      <c r="I666" t="inlineStr">
-        <is>
-          <t>edition-0/carbon-alert-europa.html</t>
-        </is>
-      </c>
       <c r="R666" t="inlineStr">
         <is>
           <t>live</t>
@@ -28910,11 +28780,6 @@
           <t>De actor is de regel</t>
         </is>
       </c>
-      <c r="I671" t="inlineStr">
-        <is>
-          <t>what-surfaces/de-actor-is-de-regel.html</t>
-        </is>
-      </c>
       <c r="R671" t="inlineStr">
         <is>
           <t>live</t>
@@ -29211,11 +29076,6 @@
           <t>De prijs van de bloei</t>
         </is>
       </c>
-      <c r="I678" t="inlineStr">
-        <is>
-          <t>edition-2/education-price-of-the-bloom.html</t>
-        </is>
-      </c>
       <c r="R678" t="inlineStr">
         <is>
           <t>live</t>
@@ -29512,11 +29372,6 @@
           <t>Editie 2</t>
         </is>
       </c>
-      <c r="I685" t="inlineStr">
-        <is>
-          <t>edition-2/index.html</t>
-        </is>
-      </c>
       <c r="R685" t="inlineStr">
         <is>
           <t>live</t>
@@ -29641,11 +29496,6 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
-      <c r="I688" t="inlineStr">
-        <is>
-          <t>vote-impact-app/energie/index.html</t>
-        </is>
-      </c>
       <c r="R688" t="inlineStr">
         <is>
           <t>live</t>
@@ -29727,11 +29577,6 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
-      <c r="I690" t="inlineStr">
-        <is>
-          <t>vote-impact-app/industrie/index.html</t>
-        </is>
-      </c>
       <c r="R690" t="inlineStr">
         <is>
           <t>live</t>
@@ -29770,11 +29615,6 @@
           <t>Kies een kant</t>
         </is>
       </c>
-      <c r="I691" t="inlineStr">
-        <is>
-          <t>edition-2/education-choose-a-side.html</t>
-        </is>
-      </c>
       <c r="R691" t="inlineStr">
         <is>
           <t>live</t>
@@ -29856,11 +29696,6 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
-      <c r="I693" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/methode/index.html</t>
-        </is>
-      </c>
       <c r="R693" t="inlineStr">
         <is>
           <t>live</t>
@@ -30157,11 +29992,6 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
-      <c r="I700" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/index.html</t>
-        </is>
-      </c>
       <c r="R700" t="inlineStr">
         <is>
           <t>live</t>
@@ -30200,11 +30030,6 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
-      <c r="I701" t="inlineStr">
-        <is>
-          <t>edition-4/artikel-00-redactie.html</t>
-        </is>
-      </c>
       <c r="R701" t="inlineStr">
         <is>
           <t>live</t>
@@ -30286,11 +30111,6 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
-      <c r="I703" t="inlineStr">
-        <is>
-          <t>vote-impact-app/scholing/index.html</t>
-        </is>
-      </c>
       <c r="R703" t="inlineStr">
         <is>
           <t>live</t>
@@ -30372,11 +30192,6 @@
           <t>Terug naar de werkbank, vooruit naar het denken</t>
         </is>
       </c>
-      <c r="I705" t="inlineStr">
-        <is>
-          <t>edition-2/education-back-to-the-workbench.html</t>
-        </is>
-      </c>
       <c r="R705" t="inlineStr">
         <is>
           <t>live</t>
@@ -30544,11 +30359,6 @@
           <t>Van leerfabriek naar leerwerkplaats</t>
         </is>
       </c>
-      <c r="I709" t="inlineStr">
-        <is>
-          <t>edition-1/education.html</t>
-        </is>
-      </c>
       <c r="R709" t="inlineStr">
         <is>
           <t>live</t>
@@ -30926,11 +30736,6 @@
           <t>De NEPK-Klimaatlogica: Zelfversterkende Systeemcrisis</t>
         </is>
       </c>
-      <c r="I718" t="inlineStr">
-        <is>
-          <t>edition-2/nepk-climate-logic.html</t>
-        </is>
-      </c>
       <c r="R718" t="inlineStr">
         <is>
           <t>live</t>
@@ -31131,11 +30936,6 @@
           <t>Nederland · Toekomst</t>
         </is>
       </c>
-      <c r="I723" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/netherlands/index.html</t>
-        </is>
-      </c>
       <c r="R723" t="inlineStr">
         <is>
           <t>live</t>
@@ -31174,11 +30974,6 @@
           <t>Stille Analyse</t>
         </is>
       </c>
-      <c r="I724" t="inlineStr">
-        <is>
-          <t>what-surfaces/gevolgenkaart-iii-stille-analyse.html</t>
-        </is>
-      </c>
       <c r="R724" t="inlineStr">
         <is>
           <t>live</t>
@@ -31465,11 +31260,6 @@
           <t>De Brusselse Gevolgenkaart — BiCRS-versie</t>
         </is>
       </c>
-      <c r="I731" t="inlineStr">
-        <is>
-          <t>what-surfaces/brusselse-gevolgenkaart-bicrs.html</t>
-        </is>
-      </c>
       <c r="R731" t="inlineStr">
         <is>
           <t>live</t>
@@ -31723,11 +31513,6 @@
           <t>Die Konsequenzkarte</t>
         </is>
       </c>
-      <c r="I737" t="inlineStr">
-        <is>
-          <t>what-surfaces/die-konsequenzkarte.html</t>
-        </is>
-      </c>
       <c r="R737" t="inlineStr">
         <is>
           <t>live</t>
@@ -31766,11 +31551,6 @@
           <t>Duitsland · Toekomst</t>
         </is>
       </c>
-      <c r="I738" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/duitsland/index.html</t>
-        </is>
-      </c>
       <c r="R738" t="inlineStr">
         <is>
           <t>live</t>
@@ -31938,11 +31718,6 @@
           <t>Europa · Toekomst</t>
         </is>
       </c>
-      <c r="I742" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/europa/index.html</t>
-        </is>
-      </c>
       <c r="R742" t="inlineStr">
         <is>
           <t>live</t>
@@ -32755,11 +32530,6 @@
           <t>Het immuunsysteem dat gezonde cellen aanvalt</t>
         </is>
       </c>
-      <c r="I761" t="inlineStr">
-        <is>
-          <t>what-surfaces/het-immuunsysteem-van-organisaties.html</t>
-        </is>
-      </c>
       <c r="R761" t="inlineStr">
         <is>
           <t>live</t>
@@ -32884,11 +32654,6 @@
           <t>Trump als spiegel</t>
         </is>
       </c>
-      <c r="I764" t="inlineStr">
-        <is>
-          <t>what-surfaces/trump-als-spiegel.html</t>
-        </is>
-      </c>
       <c r="R764" t="inlineStr">
         <is>
           <t>live</t>
@@ -33056,11 +32821,6 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
-      <c r="I768" t="inlineStr">
-        <is>
-          <t>edition-0/carbon-alert-europa.html</t>
-        </is>
-      </c>
       <c r="R768" t="inlineStr">
         <is>
           <t>live</t>
@@ -33099,11 +32859,6 @@
           <t>Zij doden hun levensaders</t>
         </is>
       </c>
-      <c r="I769" t="inlineStr">
-        <is>
-          <t>what-surfaces/zij-doden-hun-levensaders-brussel.html</t>
-        </is>
-      </c>
       <c r="R769" t="inlineStr">
         <is>
           <t>live</t>
@@ -33524,11 +33279,6 @@
           <t>Editie 1</t>
         </is>
       </c>
-      <c r="I779" t="inlineStr">
-        <is>
-          <t>edition-1/index.html</t>
-        </is>
-      </c>
       <c r="R779" t="inlineStr">
         <is>
           <t>live</t>
@@ -33567,11 +33317,6 @@
           <t>Editie 5 — portaal</t>
         </is>
       </c>
-      <c r="I780" t="inlineStr">
-        <is>
-          <t>edition-5/index.html</t>
-        </is>
-      </c>
       <c r="R780" t="inlineStr">
         <is>
           <t>live</t>
@@ -33610,11 +33355,6 @@
           <t>Een fusiereactor zonder magnetische kooi</t>
         </is>
       </c>
-      <c r="I781" t="inlineStr">
-        <is>
-          <t>edition-1/fusion.html</t>
-        </is>
-      </c>
       <c r="R781" t="inlineStr">
         <is>
           <t>live</t>
@@ -33653,11 +33393,6 @@
           <t>Veerkracht en Selectie</t>
         </is>
       </c>
-      <c r="I782" t="inlineStr">
-        <is>
-          <t>edition-2/resilience-and-selection.html</t>
-        </is>
-      </c>
       <c r="R782" t="inlineStr">
         <is>
           <t>live</t>
@@ -33696,11 +33431,6 @@
           <t>Wat er nu al ligt</t>
         </is>
       </c>
-      <c r="I783" t="inlineStr">
-        <is>
-          <t>edition-1/technical-solutions.html</t>
-        </is>
-      </c>
       <c r="R783" t="inlineStr">
         <is>
           <t>live</t>
@@ -33863,11 +33593,6 @@
           <t>Afloop</t>
         </is>
       </c>
-      <c r="I787" t="inlineStr">
-        <is>
-          <t>what-surfaces/plundering-3-afloop.html</t>
-        </is>
-      </c>
       <c r="R787" t="inlineStr">
         <is>
           <t>live</t>
@@ -33949,11 +33674,6 @@
           <t>De Grote Plundering</t>
         </is>
       </c>
-      <c r="I789" t="inlineStr">
-        <is>
-          <t>what-surfaces/de-grote-plundering.html</t>
-        </is>
-      </c>
       <c r="R789" t="inlineStr">
         <is>
           <t>live</t>
@@ -33992,11 +33712,6 @@
           <t>Diagnose</t>
         </is>
       </c>
-      <c r="I790" t="inlineStr">
-        <is>
-          <t>what-surfaces/plundering-1-diagnose.html</t>
-        </is>
-      </c>
       <c r="R790" t="inlineStr">
         <is>
           <t>live</t>
@@ -34207,11 +33922,6 @@
           <t>Het politieke landschap</t>
         </is>
       </c>
-      <c r="I795" t="inlineStr">
-        <is>
-          <t>what-surfaces/plundering-4-politieke-landschap.html</t>
-        </is>
-      </c>
       <c r="R795" t="inlineStr">
         <is>
           <t>live</t>
@@ -34250,11 +33960,6 @@
           <t>Mechaniek</t>
         </is>
       </c>
-      <c r="I796" t="inlineStr">
-        <is>
-          <t>what-surfaces/plundering-2-mechaniek.html</t>
-        </is>
-      </c>
       <c r="R796" t="inlineStr">
         <is>
           <t>live</t>
@@ -34374,11 +34079,6 @@
           <t>Van Belasten naar Aantrekken</t>
         </is>
       </c>
-      <c r="I799" t="inlineStr">
-        <is>
-          <t>edition-2/policy-advice-attract.html</t>
-        </is>
-      </c>
       <c r="R799" t="inlineStr">
         <is>
           <t>live</t>
@@ -34584,11 +34284,6 @@
           <t>Achter de Cijfers</t>
         </is>
       </c>
-      <c r="I804" t="inlineStr">
-        <is>
-          <t>research/index.html</t>
-        </is>
-      </c>
       <c r="R804" t="inlineStr">
         <is>
           <t>live</t>
@@ -34627,11 +34322,6 @@
           <t>Dossiers</t>
         </is>
       </c>
-      <c r="I805" t="inlineStr">
-        <is>
-          <t>dossiers/index.html</t>
-        </is>
-      </c>
       <c r="R805" t="inlineStr">
         <is>
           <t>live</t>
@@ -34670,11 +34360,6 @@
           <t>EU: BBP, Reële Lonen en de Overheidsmultiplicator</t>
         </is>
       </c>
-      <c r="I806" t="inlineStr">
-        <is>
-          <t>onderzoek/eu-multiplicator.html</t>
-        </is>
-      </c>
       <c r="R806" t="inlineStr">
         <is>
           <t>live</t>
@@ -34713,11 +34398,6 @@
           <t>GCS — krantbriefing</t>
         </is>
       </c>
-      <c r="I807" t="inlineStr">
-        <is>
-          <t>research/krantbriefing.html</t>
-        </is>
-      </c>
       <c r="R807" t="inlineStr">
         <is>
           <t>live</t>
@@ -34794,11 +34474,6 @@
           <t>GCS — volledig plan</t>
         </is>
       </c>
-      <c r="I809" t="inlineStr">
-        <is>
-          <t>research/gevoelsconnectiesysteem-volledig.html</t>
-        </is>
-      </c>
       <c r="R809" t="inlineStr">
         <is>
           <t>live</t>
@@ -34837,11 +34512,6 @@
           <t>Het gevoelsconnectiesysteem</t>
         </is>
       </c>
-      <c r="I810" t="inlineStr">
-        <is>
-          <t>research/gevoelsconnectiesysteem.html</t>
-        </is>
-      </c>
       <c r="R810" t="inlineStr">
         <is>
           <t>live</t>
@@ -34880,11 +34550,6 @@
           <t>Is Nederland op weg naar ontwikkelingslandstatus?</t>
         </is>
       </c>
-      <c r="I811" t="inlineStr">
-        <is>
-          <t>onderzoek/ontwikkelingslandstatus.html</t>
-        </is>
-      </c>
       <c r="R811" t="inlineStr">
         <is>
           <t>live</t>
@@ -35047,11 +34712,6 @@
           <t>Archief</t>
         </is>
       </c>
-      <c r="I815" t="inlineStr">
-        <is>
-          <t>archive.html</t>
-        </is>
-      </c>
       <c r="R815" t="inlineStr">
         <is>
           <t>live</t>
@@ -35133,11 +34793,6 @@
           <t>Colofon</t>
         </is>
       </c>
-      <c r="I817" t="inlineStr">
-        <is>
-          <t>colofon.html</t>
-        </is>
-      </c>
       <c r="R817" t="inlineStr">
         <is>
           <t>live</t>
@@ -35176,11 +34831,6 @@
           <t>Het Open Vizier verder dragen</t>
         </is>
       </c>
-      <c r="I818" t="inlineStr">
-        <is>
-          <t>delen.html</t>
-        </is>
-      </c>
       <c r="R818" t="inlineStr">
         <is>
           <t>live</t>
@@ -35228,7 +34878,7 @@
         <v>5</v>
       </c>
       <c r="T819" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="820">
@@ -35257,11 +34907,6 @@
           <t>Hoe u meedoet aan de discussie</t>
         </is>
       </c>
-      <c r="I820" t="inlineStr">
-        <is>
-          <t>edition-1/discussion.html</t>
-        </is>
-      </c>
       <c r="R820" t="inlineStr">
         <is>
           <t>live</t>
@@ -35300,11 +34945,6 @@
           <t>Navigatie</t>
         </is>
       </c>
-      <c r="I821" t="inlineStr">
-        <is>
-          <t>navigatie.html</t>
-        </is>
-      </c>
       <c r="R821" t="inlineStr">
         <is>
           <t>live</t>
@@ -35343,11 +34983,6 @@
           <t>Op de hoogte blijven</t>
         </is>
       </c>
-      <c r="I822" t="inlineStr">
-        <is>
-          <t>op-de-hoogte.html</t>
-        </is>
-      </c>
       <c r="R822" t="inlineStr">
         <is>
           <t>live</t>
@@ -35472,11 +35107,6 @@
           <t>Structuur — Beheer</t>
         </is>
       </c>
-      <c r="I825" t="inlineStr">
-        <is>
-          <t>structuur.html</t>
-        </is>
-      </c>
       <c r="R825" t="inlineStr">
         <is>
           <t>live</t>
@@ -35558,11 +35188,6 @@
           <t>Waarom deze krant?</t>
         </is>
       </c>
-      <c r="I827" t="inlineStr">
-        <is>
-          <t>edition-1/foreword.html</t>
-        </is>
-      </c>
       <c r="R827" t="inlineStr">
         <is>
           <t>live</t>
@@ -35599,11 +35224,6 @@
       <c r="F828" t="inlineStr">
         <is>
           <t>Wat opkomt</t>
-        </is>
-      </c>
-      <c r="I828" t="inlineStr">
-        <is>
-          <t>what-surfaces/index.html</t>
         </is>
       </c>
       <c r="R828" t="inlineStr">

</xml_diff>

<commit_message>
EN-menu: 29 URLs correct ingevuld op basis van geverifieerde bestanden
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -24498,6 +24498,11 @@
           <t>GCS — krantbriefing</t>
         </is>
       </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>research/krantbriefing.html</t>
+        </is>
+      </c>
       <c r="R567" t="inlineStr">
         <is>
           <t>live</t>
@@ -24574,6 +24579,11 @@
           <t>GCS — volledig plan</t>
         </is>
       </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>research/gevoelsconnectiesysteem-volledig.html</t>
+        </is>
+      </c>
       <c r="R569" t="inlineStr">
         <is>
           <t>live</t>
@@ -24612,6 +24622,11 @@
           <t>Het gevoelsconnectiesysteem</t>
         </is>
       </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>research/gevoelsconnectiesysteem.html</t>
+        </is>
+      </c>
       <c r="R570" t="inlineStr">
         <is>
           <t>live</t>
@@ -24898,6 +24913,11 @@
           <t>De Kosaris — Boek Twee — Diakrisis</t>
         </is>
       </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>reading-book-two/index.html</t>
+        </is>
+      </c>
       <c r="R577" t="inlineStr">
         <is>
           <t>live</t>
@@ -24936,6 +24956,11 @@
           <t>De Kosaris — Boek Drie — Het boek van Anthea</t>
         </is>
       </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>reading-book-three/index.html</t>
+        </is>
+      </c>
       <c r="R578" t="inlineStr">
         <is>
           <t>live</t>
@@ -24974,6 +24999,11 @@
           <t>De Kosaris — Boek Vier — Het boek van het hydrolysaat</t>
         </is>
       </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>reading-book-four/index.html</t>
+        </is>
+      </c>
       <c r="R579" t="inlineStr">
         <is>
           <t>live</t>
@@ -25012,6 +25042,11 @@
           <t>De Kosaris — Boek Vijf — Het boek van de partner</t>
         </is>
       </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>reading-book-five/index.html</t>
+        </is>
+      </c>
       <c r="R580" t="inlineStr">
         <is>
           <t>live</t>
@@ -25966,6 +26001,11 @@
           <t>Tien seconden</t>
         </is>
       </c>
+      <c r="I603" t="inlineStr">
+        <is>
+          <t>idee.html</t>
+        </is>
+      </c>
       <c r="R603" t="inlineStr">
         <is>
           <t>live</t>
@@ -26844,6 +26884,11 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>stemgedrag.html</t>
+        </is>
+      </c>
       <c r="R624" t="inlineStr">
         <is>
           <t>live</t>
@@ -26968,6 +27013,11 @@
           <t>Het politieke landschap</t>
         </is>
       </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>what-surfaces/plundering-4-politieke-landschap.html</t>
+        </is>
+      </c>
       <c r="R627" t="inlineStr">
         <is>
           <t>live</t>
@@ -27092,6 +27142,11 @@
           <t>Trump als spiegel</t>
         </is>
       </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>what-surfaces/trump-als-spiegel.html</t>
+        </is>
+      </c>
       <c r="R630" t="inlineStr">
         <is>
           <t>live</t>
@@ -27593,6 +27648,11 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>climate-edition/index.html</t>
+        </is>
+      </c>
       <c r="R642" t="inlineStr">
         <is>
           <t>live</t>
@@ -28213,6 +28273,11 @@
           <t>De Brusselse Gevolgenkaart — BiCRS-versie</t>
         </is>
       </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>what-surfaces/brusselse-gevolgenkaart-bicrs.html</t>
+        </is>
+      </c>
       <c r="R657" t="inlineStr">
         <is>
           <t>live</t>
@@ -28294,6 +28359,11 @@
           <t>De op de natuur aangepaste analyse</t>
         </is>
       </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>what-surfaces/de-op-de-natuur-aangepaste-analyse.html</t>
+        </is>
+      </c>
       <c r="R659" t="inlineStr">
         <is>
           <t>live</t>
@@ -28375,6 +28445,11 @@
           <t>Editie Europa</t>
         </is>
       </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>edition-0/index.html</t>
+        </is>
+      </c>
       <c r="R661" t="inlineStr">
         <is>
           <t>live</t>
@@ -28413,6 +28488,11 @@
           <t>Mensen die mee bouwen</t>
         </is>
       </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>what-surfaces/mensen-die-mee-bouwen.html</t>
+        </is>
+      </c>
       <c r="R662" t="inlineStr">
         <is>
           <t>live</t>
@@ -28537,6 +28617,11 @@
           <t>Visie 2036</t>
         </is>
       </c>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>what-surfaces/carbon-alert-visie-2036.html</t>
+        </is>
+      </c>
       <c r="R665" t="inlineStr">
         <is>
           <t>live</t>
@@ -28575,6 +28660,11 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>edition-0/carbon-alert-europa.html</t>
+        </is>
+      </c>
       <c r="R666" t="inlineStr">
         <is>
           <t>live</t>
@@ -28780,6 +28870,11 @@
           <t>De actor is de regel</t>
         </is>
       </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>what-surfaces/de-actor-is-de-regel.html</t>
+        </is>
+      </c>
       <c r="R671" t="inlineStr">
         <is>
           <t>live</t>
@@ -29372,6 +29467,11 @@
           <t>Editie 2</t>
         </is>
       </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>edition-2/index.html</t>
+        </is>
+      </c>
       <c r="R685" t="inlineStr">
         <is>
           <t>live</t>
@@ -29696,6 +29796,11 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/methode/index.html</t>
+        </is>
+      </c>
       <c r="R693" t="inlineStr">
         <is>
           <t>live</t>
@@ -29992,6 +30097,11 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
+      <c r="I700" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/index.html</t>
+        </is>
+      </c>
       <c r="R700" t="inlineStr">
         <is>
           <t>live</t>
@@ -30030,6 +30140,11 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
+      <c r="I701" t="inlineStr">
+        <is>
+          <t>edition-4/artikel-00-redactie.html</t>
+        </is>
+      </c>
       <c r="R701" t="inlineStr">
         <is>
           <t>live</t>
@@ -30936,6 +31051,11 @@
           <t>Nederland · Toekomst</t>
         </is>
       </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/nederland/index.html</t>
+        </is>
+      </c>
       <c r="R723" t="inlineStr">
         <is>
           <t>live</t>
@@ -30974,6 +31094,11 @@
           <t>Stille Analyse</t>
         </is>
       </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>what-surfaces/gevolgenkaart-iii-stille-analyse.html</t>
+        </is>
+      </c>
       <c r="R724" t="inlineStr">
         <is>
           <t>live</t>
@@ -31260,6 +31385,11 @@
           <t>De Brusselse Gevolgenkaart — BiCRS-versie</t>
         </is>
       </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>what-surfaces/brusselse-gevolgenkaart-bicrs.html</t>
+        </is>
+      </c>
       <c r="R731" t="inlineStr">
         <is>
           <t>live</t>
@@ -31513,6 +31643,11 @@
           <t>Die Konsequenzkarte</t>
         </is>
       </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>what-surfaces/die-konsequenzkarte.html</t>
+        </is>
+      </c>
       <c r="R737" t="inlineStr">
         <is>
           <t>live</t>
@@ -31551,6 +31686,11 @@
           <t>Duitsland · Toekomst</t>
         </is>
       </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/duitsland/index.html</t>
+        </is>
+      </c>
       <c r="R738" t="inlineStr">
         <is>
           <t>live</t>
@@ -31716,6 +31856,11 @@
       <c r="F742" t="inlineStr">
         <is>
           <t>Europa · Toekomst</t>
+        </is>
+      </c>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/europa/index.html</t>
         </is>
       </c>
       <c r="R742" t="inlineStr">

</xml_diff>

<commit_message>
DE-menu: 9 URLs correct ingevuld
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -13107,6 +13107,11 @@
           <t>GCS — krantbriefing</t>
         </is>
       </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>forschung/krantbriefing.html</t>
+        </is>
+      </c>
       <c r="R289" t="inlineStr">
         <is>
           <t>live</t>
@@ -13183,6 +13188,11 @@
           <t>GCS — volledig plan</t>
         </is>
       </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>forschung/gevoelsconnectiesysteem-volledig.html</t>
+        </is>
+      </c>
       <c r="R291" t="inlineStr">
         <is>
           <t>live</t>
@@ -13221,6 +13231,11 @@
           <t>Het gevoelsconnectiesysteem</t>
         </is>
       </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>forschung/gevoelsconnectiesysteem.html</t>
+        </is>
+      </c>
       <c r="R292" t="inlineStr">
         <is>
           <t>live</t>
@@ -14575,6 +14590,11 @@
           <t>Tien seconden</t>
         </is>
       </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>idee.html</t>
+        </is>
+      </c>
       <c r="R325" t="inlineStr">
         <is>
           <t>live</t>
@@ -15453,6 +15473,11 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>stemgedrag.html</t>
+        </is>
+      </c>
       <c r="R346" t="inlineStr">
         <is>
           <t>live</t>
@@ -16202,6 +16227,11 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>editie-klimaat/index.html</t>
+        </is>
+      </c>
       <c r="R364" t="inlineStr">
         <is>
           <t>live</t>
@@ -17184,6 +17214,11 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>ausgabe-0/carbon-alert-europa.html</t>
+        </is>
+      </c>
       <c r="R388" t="inlineStr">
         <is>
           <t>live</t>
@@ -17981,6 +18016,11 @@
           <t>Editie 2</t>
         </is>
       </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>ausgabe-2/index.html</t>
+        </is>
+      </c>
       <c r="R407" t="inlineStr">
         <is>
           <t>live</t>
@@ -18637,6 +18677,11 @@
       <c r="F423" t="inlineStr">
         <is>
           <t>Redactionele inleiding</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>ausgabe-4/artikel-00-redactie.html</t>
         </is>
       </c>
       <c r="R423" t="inlineStr">

</xml_diff>

<commit_message>
RU-menu: 17 URLs correct ingevuld
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -38415,6 +38415,11 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
+      <c r="I902" t="inlineStr">
+        <is>
+          <t>stemgedrag.html</t>
+        </is>
+      </c>
       <c r="R902" t="inlineStr">
         <is>
           <t>live</t>
@@ -39111,6 +39116,11 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
+      <c r="I919" t="inlineStr">
+        <is>
+          <t>editie-stikstof/drie-problemen-een-antwoord.html</t>
+        </is>
+      </c>
       <c r="R919" t="inlineStr">
         <is>
           <t>live</t>
@@ -39149,6 +39159,11 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
+      <c r="I920" t="inlineStr">
+        <is>
+          <t>editie-klimaat/index.html</t>
+        </is>
+      </c>
       <c r="R920" t="inlineStr">
         <is>
           <t>live</t>
@@ -39187,6 +39202,11 @@
           <t>Editie Stikstof</t>
         </is>
       </c>
+      <c r="I921" t="inlineStr">
+        <is>
+          <t>editie-stikstof/index.html</t>
+        </is>
+      </c>
       <c r="R921" t="inlineStr">
         <is>
           <t>live</t>
@@ -39473,6 +39493,11 @@
           <t>De Koolzaad-Multiplicator</t>
         </is>
       </c>
+      <c r="I928" t="inlineStr">
+        <is>
+          <t>editie-duitsland/raps-multiplicator-oost-duitsland.html</t>
+        </is>
+      </c>
       <c r="R928" t="inlineStr">
         <is>
           <t>live</t>
@@ -39554,6 +39579,11 @@
           <t>Editie Duitsland</t>
         </is>
       </c>
+      <c r="I930" t="inlineStr">
+        <is>
+          <t>editie-duitsland/index.html</t>
+        </is>
+      </c>
       <c r="R930" t="inlineStr">
         <is>
           <t>live</t>
@@ -40951,6 +40981,11 @@
           <t>Editie Kind &amp; Loopbaan</t>
         </is>
       </c>
+      <c r="I964" t="inlineStr">
+        <is>
+          <t>editie-kind-loopbaan/index.html</t>
+        </is>
+      </c>
       <c r="R964" t="inlineStr">
         <is>
           <t>live</t>
@@ -40989,6 +41024,11 @@
           <t>Editie Leiderschap</t>
         </is>
       </c>
+      <c r="I965" t="inlineStr">
+        <is>
+          <t>editie-leiderschap/index.html</t>
+        </is>
+      </c>
       <c r="R965" t="inlineStr">
         <is>
           <t>live</t>
@@ -41027,6 +41067,11 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
+      <c r="I966" t="inlineStr">
+        <is>
+          <t>toekomst/energie/index.html</t>
+        </is>
+      </c>
       <c r="R966" t="inlineStr">
         <is>
           <t>live</t>
@@ -41108,6 +41153,11 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
+      <c r="I968" t="inlineStr">
+        <is>
+          <t>toekomst/industrie/index.html</t>
+        </is>
+      </c>
       <c r="R968" t="inlineStr">
         <is>
           <t>live</t>
@@ -41227,6 +41277,11 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
+      <c r="I971" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/methode/index.html</t>
+        </is>
+      </c>
       <c r="R971" t="inlineStr">
         <is>
           <t>live</t>
@@ -41437,6 +41492,11 @@
           <t>Opvoeding · Toekomst</t>
         </is>
       </c>
+      <c r="I976" t="inlineStr">
+        <is>
+          <t>toekomst/opvoeding/index.html</t>
+        </is>
+      </c>
       <c r="R976" t="inlineStr">
         <is>
           <t>live</t>
@@ -41518,6 +41578,11 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
+      <c r="I978" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/index.html</t>
+        </is>
+      </c>
       <c r="R978" t="inlineStr">
         <is>
           <t>live</t>
@@ -41637,6 +41702,11 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
+      <c r="I981" t="inlineStr">
+        <is>
+          <t>toekomst/scholing/index.html</t>
+        </is>
+      </c>
       <c r="R981" t="inlineStr">
         <is>
           <t>live</t>
@@ -41675,6 +41745,11 @@
           <t>Soevereiniteit als cyclus</t>
         </is>
       </c>
+      <c r="I982" t="inlineStr">
+        <is>
+          <t>soevereiniteit-als-cyclus/index.html</t>
+        </is>
+      </c>
       <c r="R982" t="inlineStr">
         <is>
           <t>live</t>
@@ -41751,6 +41826,11 @@
           <t>Toekomst</t>
         </is>
       </c>
+      <c r="I984" t="inlineStr">
+        <is>
+          <t>toekomst/index.html</t>
+        </is>
+      </c>
       <c r="R984" t="inlineStr">
         <is>
           <t>live</t>
@@ -42121,6 +42201,11 @@
       <c r="F993" t="inlineStr">
         <is>
           <t>De eerste gemeente</t>
+        </is>
+      </c>
+      <c r="I993" t="inlineStr">
+        <is>
+          <t>de-eerste-gemeente/index.html</t>
         </is>
       </c>
       <c r="R993" t="inlineStr">

</xml_diff>

<commit_message>
FR-menu: 79 URLs ingevuld
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -47547,6 +47547,11 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
+      <c r="I1127" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-07-ai-onderwijs.html</t>
+        </is>
+      </c>
       <c r="R1127" t="inlineStr">
         <is>
           <t>live</t>
@@ -47666,6 +47671,11 @@
           <t>Alles stroomt — de moeder van alle wetenschap</t>
         </is>
       </c>
+      <c r="I1130" t="inlineStr">
+        <is>
+          <t>editie-1/stromingsleer.html</t>
+        </is>
+      </c>
       <c r="R1130" t="inlineStr">
         <is>
           <t>live</t>
@@ -47985,6 +47995,11 @@
           <t>Drie dimensies zijn te weinig</t>
         </is>
       </c>
+      <c r="I1138" t="inlineStr">
+        <is>
+          <t>editie-1/denkraam-7d.html</t>
+        </is>
+      </c>
       <c r="R1138" t="inlineStr">
         <is>
           <t>live</t>
@@ -48066,6 +48081,11 @@
           <t>Hoe alles samenhangt</t>
         </is>
       </c>
+      <c r="I1140" t="inlineStr">
+        <is>
+          <t>editie-1/samenhang.html</t>
+        </is>
+      </c>
       <c r="R1140" t="inlineStr">
         <is>
           <t>live</t>
@@ -48104,6 +48124,11 @@
           <t>Van de grot naar de zon</t>
         </is>
       </c>
+      <c r="I1141" t="inlineStr">
+        <is>
+          <t>wat-opkomt/van-de-grot-naar-de-zon.html</t>
+        </is>
+      </c>
       <c r="R1141" t="inlineStr">
         <is>
           <t>live</t>
@@ -48142,6 +48167,11 @@
           <t>Van quantumtheorie naar 7-dim</t>
         </is>
       </c>
+      <c r="I1142" t="inlineStr">
+        <is>
+          <t>wat-opkomt/van-quantum-naar-7d.html</t>
+        </is>
+      </c>
       <c r="R1142" t="inlineStr">
         <is>
           <t>live</t>
@@ -48299,6 +48329,11 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
+      <c r="I1146" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-04-bankier.html</t>
+        </is>
+      </c>
       <c r="R1146" t="inlineStr">
         <is>
           <t>live</t>
@@ -48337,6 +48372,11 @@
           <t>Communicatie tussen oergevoelens</t>
         </is>
       </c>
+      <c r="I1147" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-04-communicatie.html</t>
+        </is>
+      </c>
       <c r="R1147" t="inlineStr">
         <is>
           <t>live</t>
@@ -48375,6 +48415,11 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
+      <c r="I1148" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-02-ceo.html</t>
+        </is>
+      </c>
       <c r="R1148" t="inlineStr">
         <is>
           <t>live</t>
@@ -48413,6 +48458,11 @@
           <t>De drie hersenlagen</t>
         </is>
       </c>
+      <c r="I1149" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-03-drie-lagen.html</t>
+        </is>
+      </c>
       <c r="R1149" t="inlineStr">
         <is>
           <t>live</t>
@@ -48451,6 +48501,11 @@
           <t>De mens onder het ijs (Editie 3)</t>
         </is>
       </c>
+      <c r="I1150" t="inlineStr">
+        <is>
+          <t>editie-3/index.html</t>
+        </is>
+      </c>
       <c r="R1150" t="inlineStr">
         <is>
           <t>live</t>
@@ -48489,6 +48544,11 @@
           <t>De zeven dimensies</t>
         </is>
       </c>
+      <c r="I1151" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-02-zeven-dimensies.html</t>
+        </is>
+      </c>
       <c r="R1151" t="inlineStr">
         <is>
           <t>live</t>
@@ -48570,6 +48630,11 @@
           <t>Het oergevoel</t>
         </is>
       </c>
+      <c r="I1153" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-01-oergevoel.html</t>
+        </is>
+      </c>
       <c r="R1153" t="inlineStr">
         <is>
           <t>live</t>
@@ -48608,6 +48673,11 @@
           <t>Het oergevoel in de beroepspraktijk</t>
         </is>
       </c>
+      <c r="I1154" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-09-oergevoel-in-beroepspraktijk.html</t>
+        </is>
+      </c>
       <c r="R1154" t="inlineStr">
         <is>
           <t>live</t>
@@ -48646,6 +48716,11 @@
           <t>Mama ik heb honger</t>
         </is>
       </c>
+      <c r="I1155" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-06-mama.html</t>
+        </is>
+      </c>
       <c r="R1155" t="inlineStr">
         <is>
           <t>live</t>
@@ -48684,6 +48759,11 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
+      <c r="I1156" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-00-redactie.html</t>
+        </is>
+      </c>
       <c r="R1156" t="inlineStr">
         <is>
           <t>live</t>
@@ -48722,6 +48802,11 @@
           <t>Retrospectief</t>
         </is>
       </c>
+      <c r="I1157" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-08-retrospectief.html</t>
+        </is>
+      </c>
       <c r="R1157" t="inlineStr">
         <is>
           <t>live</t>
@@ -48760,6 +48845,11 @@
           <t>Ruimte voor het oergevoel</t>
         </is>
       </c>
+      <c r="I1158" t="inlineStr">
+        <is>
+          <t>wat-opkomt/manifest-ruimte-voor-het-oergevoel.html</t>
+        </is>
+      </c>
       <c r="R1158" t="inlineStr">
         <is>
           <t>live</t>
@@ -48798,6 +48888,11 @@
           <t>Tien seconden</t>
         </is>
       </c>
+      <c r="I1159" t="inlineStr">
+        <is>
+          <t>idee.html</t>
+        </is>
+      </c>
       <c r="R1159" t="inlineStr">
         <is>
           <t>live</t>
@@ -48879,6 +48974,11 @@
           <t>Wat we kinderen aandoen</t>
         </is>
       </c>
+      <c r="I1161" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-05-wat-we-doen.html</t>
+        </is>
+      </c>
       <c r="R1161" t="inlineStr">
         <is>
           <t>live</t>
@@ -49451,6 +49551,11 @@
           <t>De anti-immuunziekte van onze overheid slaat toe</t>
         </is>
       </c>
+      <c r="I1175" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-auto-immuunziekte-slaat-toe.html</t>
+        </is>
+      </c>
       <c r="R1175" t="inlineStr">
         <is>
           <t>live</t>
@@ -49532,6 +49637,11 @@
           <t>De matrix van de uittocht</t>
         </is>
       </c>
+      <c r="I1177" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-matrix-van-de-uittocht.html</t>
+        </is>
+      </c>
       <c r="R1177" t="inlineStr">
         <is>
           <t>live</t>
@@ -49656,6 +49766,11 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
+      <c r="I1180" t="inlineStr">
+        <is>
+          <t>stemgedrag.html</t>
+        </is>
+      </c>
       <c r="R1180" t="inlineStr">
         <is>
           <t>live</t>
@@ -49775,6 +49890,11 @@
           <t>Het politieke landschap</t>
         </is>
       </c>
+      <c r="I1183" t="inlineStr">
+        <is>
+          <t>wat-opkomt/plundering-4-politieke-landschap.html</t>
+        </is>
+      </c>
       <c r="R1183" t="inlineStr">
         <is>
           <t>live</t>
@@ -49813,6 +49933,11 @@
           <t>Moet Nederland ook volgen — laten wij onze industrie zakken?</t>
         </is>
       </c>
+      <c r="I1184" t="inlineStr">
+        <is>
+          <t>wat-opkomt/moet-nederland-ook-volgen.html</t>
+        </is>
+      </c>
       <c r="R1184" t="inlineStr">
         <is>
           <t>live</t>
@@ -49851,6 +49976,11 @@
           <t>Op de bok of op de bagagedrager</t>
         </is>
       </c>
+      <c r="I1185" t="inlineStr">
+        <is>
+          <t>wat-opkomt/aan-de-leiding-drie-blokken-zonder-subsidie.html</t>
+        </is>
+      </c>
       <c r="R1185" t="inlineStr">
         <is>
           <t>live</t>
@@ -49927,6 +50057,11 @@
           <t>Wat is er mis met partijpolitiek?</t>
         </is>
       </c>
+      <c r="I1187" t="inlineStr">
+        <is>
+          <t>editie-1/nova-democratia.html</t>
+        </is>
+      </c>
       <c r="R1187" t="inlineStr">
         <is>
           <t>live</t>
@@ -49965,6 +50100,11 @@
           <t>Ze weten het al. En ze doen het niet.</t>
         </is>
       </c>
+      <c r="I1188" t="inlineStr">
+        <is>
+          <t>wat-opkomt/ze-weten-het-al.html</t>
+        </is>
+      </c>
       <c r="R1188" t="inlineStr">
         <is>
           <t>live</t>
@@ -50084,6 +50224,11 @@
           <t>De anti-immuunziekte van onze overheid slaat toe</t>
         </is>
       </c>
+      <c r="I1191" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-auto-immuunziekte-slaat-toe.html</t>
+        </is>
+      </c>
       <c r="R1191" t="inlineStr">
         <is>
           <t>live</t>
@@ -50122,6 +50267,11 @@
           <t>De autoband is het nieuwe sigaret</t>
         </is>
       </c>
+      <c r="I1192" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-autoband-is-het-nieuwe-sigaret.html</t>
+        </is>
+      </c>
       <c r="R1192" t="inlineStr">
         <is>
           <t>live</t>
@@ -50160,6 +50310,11 @@
           <t>De boer én de natuur beide vooruit</t>
         </is>
       </c>
+      <c r="I1193" t="inlineStr">
+        <is>
+          <t>wat-opkomt/boer-en-natuur-beide-vooruit.html</t>
+        </is>
+      </c>
       <c r="R1193" t="inlineStr">
         <is>
           <t>live</t>
@@ -50198,6 +50353,11 @@
           <t>De methaan-misleiding</t>
         </is>
       </c>
+      <c r="I1194" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-04-methaan-misleiding.html</t>
+        </is>
+      </c>
       <c r="R1194" t="inlineStr">
         <is>
           <t>live</t>
@@ -50236,6 +50396,11 @@
           <t>De voedingslijn</t>
         </is>
       </c>
+      <c r="I1195" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-methodologie-van-de-aanpassing.html</t>
+        </is>
+      </c>
       <c r="R1195" t="inlineStr">
         <is>
           <t>live</t>
@@ -50317,6 +50482,11 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
+      <c r="I1197" t="inlineStr">
+        <is>
+          <t>editie-stikstof/drie-problemen-een-antwoord.html</t>
+        </is>
+      </c>
       <c r="R1197" t="inlineStr">
         <is>
           <t>live</t>
@@ -50355,6 +50525,11 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
+      <c r="I1198" t="inlineStr">
+        <is>
+          <t>editie-klimaat/index.html</t>
+        </is>
+      </c>
       <c r="R1198" t="inlineStr">
         <is>
           <t>live</t>
@@ -50393,6 +50568,11 @@
           <t>Editie Stikstof</t>
         </is>
       </c>
+      <c r="I1199" t="inlineStr">
+        <is>
+          <t>editie-stikstof/index.html</t>
+        </is>
+      </c>
       <c r="R1199" t="inlineStr">
         <is>
           <t>live</t>
@@ -50431,6 +50611,11 @@
           <t>Erfenisgolf — 240 miljard</t>
         </is>
       </c>
+      <c r="I1200" t="inlineStr">
+        <is>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
+        </is>
+      </c>
       <c r="R1200" t="inlineStr">
         <is>
           <t>live</t>
@@ -50507,6 +50692,11 @@
           <t>Laat de politici eerst naar de natuurschool</t>
         </is>
       </c>
+      <c r="I1202" t="inlineStr">
+        <is>
+          <t>wat-opkomt/naar-de-natuurschool.html</t>
+        </is>
+      </c>
       <c r="R1202" t="inlineStr">
         <is>
           <t>live</t>
@@ -50588,6 +50778,11 @@
           <t>Ze weten het al. En ze doen het niet.</t>
         </is>
       </c>
+      <c r="I1204" t="inlineStr">
+        <is>
+          <t>wat-opkomt/ze-weten-het-al.html</t>
+        </is>
+      </c>
       <c r="R1204" t="inlineStr">
         <is>
           <t>live</t>
@@ -50664,6 +50859,11 @@
           <t>De Koolzaad-Multiplicator</t>
         </is>
       </c>
+      <c r="I1206" t="inlineStr">
+        <is>
+          <t>editie-duitsland/raps-multiplicator-oost-duitsland.html</t>
+        </is>
+      </c>
       <c r="R1206" t="inlineStr">
         <is>
           <t>live</t>
@@ -50702,6 +50902,11 @@
           <t>De plant die verhuist</t>
         </is>
       </c>
+      <c r="I1207" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-05-plant-die-verhuist.html</t>
+        </is>
+      </c>
       <c r="R1207" t="inlineStr">
         <is>
           <t>live</t>
@@ -50740,6 +50945,11 @@
           <t>Editie Duitsland</t>
         </is>
       </c>
+      <c r="I1208" t="inlineStr">
+        <is>
+          <t>editie-duitsland/index.html</t>
+        </is>
+      </c>
       <c r="R1208" t="inlineStr">
         <is>
           <t>live</t>
@@ -50778,6 +50988,11 @@
           <t>Een Ferrari die naar gemaaid gras ruikt</t>
         </is>
       </c>
+      <c r="I1209" t="inlineStr">
+        <is>
+          <t>wat-opkomt/het-dagelijks-idee-ferrari-juncao.html</t>
+        </is>
+      </c>
       <c r="R1209" t="inlineStr">
         <is>
           <t>live</t>
@@ -50854,6 +51069,11 @@
           <t>Actievoerders bouwen continenten</t>
         </is>
       </c>
+      <c r="I1211" t="inlineStr">
+        <is>
+          <t>wat-opkomt/actievoerders-bouwen-continenten.html</t>
+        </is>
+      </c>
       <c r="R1211" t="inlineStr">
         <is>
           <t>live</t>
@@ -50892,6 +51112,11 @@
           <t>De biomimetische krachtcentrale</t>
         </is>
       </c>
+      <c r="I1212" t="inlineStr">
+        <is>
+          <t>editie-0/biomimetische-krachtcentrale.html</t>
+        </is>
+      </c>
       <c r="R1212" t="inlineStr">
         <is>
           <t>live</t>
@@ -50968,6 +51193,11 @@
           <t>De dertig cent die Europa omdraait</t>
         </is>
       </c>
+      <c r="I1214" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-dertig-cent-die-europa-omdraait.html</t>
+        </is>
+      </c>
       <c r="R1214" t="inlineStr">
         <is>
           <t>live</t>
@@ -51044,6 +51274,11 @@
           <t>De plastic-boete die een carbon-credit had moeten zijn</t>
         </is>
       </c>
+      <c r="I1216" t="inlineStr">
+        <is>
+          <t>wat-opkomt/plastic-boete-carbon-credit.html</t>
+        </is>
+      </c>
       <c r="R1216" t="inlineStr">
         <is>
           <t>live</t>
@@ -51082,6 +51317,11 @@
           <t>Editie Europa</t>
         </is>
       </c>
+      <c r="I1217" t="inlineStr">
+        <is>
+          <t>editie-0/index.html</t>
+        </is>
+      </c>
       <c r="R1217" t="inlineStr">
         <is>
           <t>live</t>
@@ -51120,6 +51360,11 @@
           <t>Mensen die mee bouwen</t>
         </is>
       </c>
+      <c r="I1218" t="inlineStr">
+        <is>
+          <t>wat-opkomt/mensen-die-mee-bouwen.html</t>
+        </is>
+      </c>
       <c r="R1218" t="inlineStr">
         <is>
           <t>live</t>
@@ -51158,6 +51403,11 @@
           <t>Op de bok of op de bagagedrager</t>
         </is>
       </c>
+      <c r="I1219" t="inlineStr">
+        <is>
+          <t>wat-opkomt/aan-de-leiding-drie-blokken-zonder-subsidie.html</t>
+        </is>
+      </c>
       <c r="R1219" t="inlineStr">
         <is>
           <t>live</t>
@@ -51239,6 +51489,11 @@
           <t>Visie 2036</t>
         </is>
       </c>
+      <c r="I1221" t="inlineStr">
+        <is>
+          <t>wat-opkomt/carbon-alert-visie-2036.html</t>
+        </is>
+      </c>
       <c r="R1221" t="inlineStr">
         <is>
           <t>live</t>
@@ -51277,6 +51532,11 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
+      <c r="I1222" t="inlineStr">
+        <is>
+          <t>editie-0/carbon-alert-europa.html</t>
+        </is>
+      </c>
       <c r="R1222" t="inlineStr">
         <is>
           <t>live</t>
@@ -51353,6 +51613,11 @@
           <t>Beslissen zonder uitzicht</t>
         </is>
       </c>
+      <c r="I1224" t="inlineStr">
+        <is>
+          <t>wat-opkomt/bbp-liegt.html</t>
+        </is>
+      </c>
       <c r="R1224" t="inlineStr">
         <is>
           <t>live</t>
@@ -51391,6 +51656,11 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
+      <c r="I1225" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-04-bankier.html</t>
+        </is>
+      </c>
       <c r="R1225" t="inlineStr">
         <is>
           <t>live</t>
@@ -51472,6 +51742,11 @@
           <t>De actor is de regel</t>
         </is>
       </c>
+      <c r="I1227" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-actor-is-de-regel.html</t>
+        </is>
+      </c>
       <c r="R1227" t="inlineStr">
         <is>
           <t>live</t>
@@ -51596,6 +51871,11 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
+      <c r="I1230" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-02-ceo.html</t>
+        </is>
+      </c>
       <c r="R1230" t="inlineStr">
         <is>
           <t>live</t>
@@ -51634,6 +51914,11 @@
           <t>De consultant bij het bijna-failliete bedrijf</t>
         </is>
       </c>
+      <c r="I1231" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-03-consultant.html</t>
+        </is>
+      </c>
       <c r="R1231" t="inlineStr">
         <is>
           <t>live</t>
@@ -51672,6 +51957,11 @@
           <t>De diepere vraag</t>
         </is>
       </c>
+      <c r="I1232" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-08-diepere-vraag.html</t>
+        </is>
+      </c>
       <c r="R1232" t="inlineStr">
         <is>
           <t>live</t>
@@ -51796,6 +52086,11 @@
           <t>De rechter zonder kompas</t>
         </is>
       </c>
+      <c r="I1235" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-07-rechter.html</t>
+        </is>
+      </c>
       <c r="R1235" t="inlineStr">
         <is>
           <t>live</t>
@@ -51834,6 +52129,11 @@
           <t>De toezichthouder die niets ziet</t>
         </is>
       </c>
+      <c r="I1236" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-06-toezichthouder.html</t>
+        </is>
+      </c>
       <c r="R1236" t="inlineStr">
         <is>
           <t>live</t>
@@ -51872,6 +52172,11 @@
           <t>De verzekeraar tegen het leven</t>
         </is>
       </c>
+      <c r="I1237" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-05-verzekeraar.html</t>
+        </is>
+      </c>
       <c r="R1237" t="inlineStr">
         <is>
           <t>live</t>
@@ -51910,6 +52215,11 @@
           <t>De wet van de papier-industrie</t>
         </is>
       </c>
+      <c r="I1238" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-01-wet-papier-industrie.html</t>
+        </is>
+      </c>
       <c r="R1238" t="inlineStr">
         <is>
           <t>live</t>
@@ -52072,6 +52382,11 @@
           <t>Editie Kind &amp; Loopbaan</t>
         </is>
       </c>
+      <c r="I1242" t="inlineStr">
+        <is>
+          <t>editie-kind-loopbaan/index.html</t>
+        </is>
+      </c>
       <c r="R1242" t="inlineStr">
         <is>
           <t>live</t>
@@ -52110,6 +52425,11 @@
           <t>Editie Leiderschap</t>
         </is>
       </c>
+      <c r="I1243" t="inlineStr">
+        <is>
+          <t>editie-leiderschap/index.html</t>
+        </is>
+      </c>
       <c r="R1243" t="inlineStr">
         <is>
           <t>live</t>
@@ -52148,6 +52468,11 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
+      <c r="I1244" t="inlineStr">
+        <is>
+          <t>toekomst/energie/index.html</t>
+        </is>
+      </c>
       <c r="R1244" t="inlineStr">
         <is>
           <t>live</t>
@@ -52186,6 +52511,11 @@
           <t>Hoe de papier-industrie macht kreeg over het echte werk</t>
         </is>
       </c>
+      <c r="I1245" t="inlineStr">
+        <is>
+          <t>editie-4/index.html</t>
+        </is>
+      </c>
       <c r="R1245" t="inlineStr">
         <is>
           <t>live</t>
@@ -52224,6 +52554,11 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
+      <c r="I1246" t="inlineStr">
+        <is>
+          <t>toekomst/industrie/index.html</t>
+        </is>
+      </c>
       <c r="R1246" t="inlineStr">
         <is>
           <t>live</t>
@@ -52348,6 +52683,11 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
+      <c r="I1249" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/methode/index.html</t>
+        </is>
+      </c>
       <c r="R1249" t="inlineStr">
         <is>
           <t>live</t>
@@ -52515,6 +52855,11 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
+      <c r="I1253" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-07-ai-onderwijs.html</t>
+        </is>
+      </c>
       <c r="R1253" t="inlineStr">
         <is>
           <t>live</t>
@@ -52553,6 +52898,11 @@
           <t>Opvoeding · Toekomst</t>
         </is>
       </c>
+      <c r="I1254" t="inlineStr">
+        <is>
+          <t>toekomst/opvoeding/index.html</t>
+        </is>
+      </c>
       <c r="R1254" t="inlineStr">
         <is>
           <t>live</t>
@@ -52634,6 +52984,11 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
+      <c r="I1256" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/index.html</t>
+        </is>
+      </c>
       <c r="R1256" t="inlineStr">
         <is>
           <t>live</t>
@@ -52672,6 +53027,11 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
+      <c r="I1257" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-00-redactie.html</t>
+        </is>
+      </c>
       <c r="R1257" t="inlineStr">
         <is>
           <t>live</t>
@@ -52710,6 +53070,11 @@
           <t>Retrospectief</t>
         </is>
       </c>
+      <c r="I1258" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-09-retrospectief.html</t>
+        </is>
+      </c>
       <c r="R1258" t="inlineStr">
         <is>
           <t>live</t>
@@ -52748,6 +53113,11 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
+      <c r="I1259" t="inlineStr">
+        <is>
+          <t>toekomst/scholing/index.html</t>
+        </is>
+      </c>
       <c r="R1259" t="inlineStr">
         <is>
           <t>live</t>
@@ -52786,6 +53156,11 @@
           <t>Soevereiniteit als cyclus</t>
         </is>
       </c>
+      <c r="I1260" t="inlineStr">
+        <is>
+          <t>soevereiniteit-als-cyclus/index.html</t>
+        </is>
+      </c>
       <c r="R1260" t="inlineStr">
         <is>
           <t>live</t>
@@ -52867,6 +53242,11 @@
           <t>Toekomst</t>
         </is>
       </c>
+      <c r="I1262" t="inlineStr">
+        <is>
+          <t>toekomst/index.html</t>
+        </is>
+      </c>
       <c r="R1262" t="inlineStr">
         <is>
           <t>live</t>
@@ -52991,6 +53371,11 @@
           <t>Van leerfabriek naar leerwerkplaats</t>
         </is>
       </c>
+      <c r="I1265" t="inlineStr">
+        <is>
+          <t>editie-1/onderwijs.html</t>
+        </is>
+      </c>
       <c r="R1265" t="inlineStr">
         <is>
           <t>live</t>
@@ -53239,6 +53624,11 @@
           <t>De eerste gemeente</t>
         </is>
       </c>
+      <c r="I1271" t="inlineStr">
+        <is>
+          <t>de-eerste-gemeente/index.html</t>
+        </is>
+      </c>
       <c r="R1271" t="inlineStr">
         <is>
           <t>live</t>
@@ -53275,6 +53665,11 @@
       <c r="F1272" t="inlineStr">
         <is>
           <t>De halve gemeente</t>
+        </is>
+      </c>
+      <c r="I1272" t="inlineStr">
+        <is>
+          <t>de-halve-gemeente/index.html</t>
         </is>
       </c>
       <c r="R1272" t="inlineStr">

</xml_diff>

<commit_message>
ES-menu: 65 URLs ingevuld
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -58883,6 +58883,11 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
+      <c r="I1405" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-07-ai-onderwijs.html</t>
+        </is>
+      </c>
       <c r="R1405" t="inlineStr">
         <is>
           <t>live</t>
@@ -59002,6 +59007,11 @@
           <t>Alles stroomt — de moeder van alle wetenschap</t>
         </is>
       </c>
+      <c r="I1408" t="inlineStr">
+        <is>
+          <t>editie-1/stromingsleer.html</t>
+        </is>
+      </c>
       <c r="R1408" t="inlineStr">
         <is>
           <t>live</t>
@@ -59321,6 +59331,11 @@
           <t>Drie dimensies zijn te weinig</t>
         </is>
       </c>
+      <c r="I1416" t="inlineStr">
+        <is>
+          <t>editie-1/denkraam-7d.html</t>
+        </is>
+      </c>
       <c r="R1416" t="inlineStr">
         <is>
           <t>live</t>
@@ -59402,6 +59417,11 @@
           <t>Hoe alles samenhangt</t>
         </is>
       </c>
+      <c r="I1418" t="inlineStr">
+        <is>
+          <t>editie-1/samenhang.html</t>
+        </is>
+      </c>
       <c r="R1418" t="inlineStr">
         <is>
           <t>live</t>
@@ -59645,6 +59665,11 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
+      <c r="I1424" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-04-bankier.html</t>
+        </is>
+      </c>
       <c r="R1424" t="inlineStr">
         <is>
           <t>live</t>
@@ -59683,6 +59708,11 @@
           <t>Communicatie tussen oergevoelens</t>
         </is>
       </c>
+      <c r="I1425" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-04-communicatie.html</t>
+        </is>
+      </c>
       <c r="R1425" t="inlineStr">
         <is>
           <t>live</t>
@@ -59721,6 +59751,11 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
+      <c r="I1426" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-02-ceo.html</t>
+        </is>
+      </c>
       <c r="R1426" t="inlineStr">
         <is>
           <t>live</t>
@@ -59759,6 +59794,11 @@
           <t>De drie hersenlagen</t>
         </is>
       </c>
+      <c r="I1427" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-03-drie-lagen.html</t>
+        </is>
+      </c>
       <c r="R1427" t="inlineStr">
         <is>
           <t>live</t>
@@ -59797,6 +59837,11 @@
           <t>De mens onder het ijs (Editie 3)</t>
         </is>
       </c>
+      <c r="I1428" t="inlineStr">
+        <is>
+          <t>editie-3/index.html</t>
+        </is>
+      </c>
       <c r="R1428" t="inlineStr">
         <is>
           <t>live</t>
@@ -59835,6 +59880,11 @@
           <t>De zeven dimensies</t>
         </is>
       </c>
+      <c r="I1429" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-02-zeven-dimensies.html</t>
+        </is>
+      </c>
       <c r="R1429" t="inlineStr">
         <is>
           <t>live</t>
@@ -59916,6 +59966,11 @@
           <t>Het oergevoel</t>
         </is>
       </c>
+      <c r="I1431" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-01-oergevoel.html</t>
+        </is>
+      </c>
       <c r="R1431" t="inlineStr">
         <is>
           <t>live</t>
@@ -59954,6 +60009,11 @@
           <t>Het oergevoel in de beroepspraktijk</t>
         </is>
       </c>
+      <c r="I1432" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-09-oergevoel-in-beroepspraktijk.html</t>
+        </is>
+      </c>
       <c r="R1432" t="inlineStr">
         <is>
           <t>live</t>
@@ -59992,6 +60052,11 @@
           <t>Mama ik heb honger</t>
         </is>
       </c>
+      <c r="I1433" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-06-mama.html</t>
+        </is>
+      </c>
       <c r="R1433" t="inlineStr">
         <is>
           <t>live</t>
@@ -60030,6 +60095,11 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
+      <c r="I1434" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-00-redactie.html</t>
+        </is>
+      </c>
       <c r="R1434" t="inlineStr">
         <is>
           <t>live</t>
@@ -60068,6 +60138,11 @@
           <t>Retrospectief</t>
         </is>
       </c>
+      <c r="I1435" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-08-retrospectief.html</t>
+        </is>
+      </c>
       <c r="R1435" t="inlineStr">
         <is>
           <t>live</t>
@@ -60149,6 +60224,11 @@
           <t>Tien seconden</t>
         </is>
       </c>
+      <c r="I1437" t="inlineStr">
+        <is>
+          <t>idee.html</t>
+        </is>
+      </c>
       <c r="R1437" t="inlineStr">
         <is>
           <t>live</t>
@@ -60230,6 +60310,11 @@
           <t>Wat we kinderen aandoen</t>
         </is>
       </c>
+      <c r="I1439" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-05-wat-we-doen.html</t>
+        </is>
+      </c>
       <c r="R1439" t="inlineStr">
         <is>
           <t>live</t>
@@ -61017,6 +61102,11 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
+      <c r="I1458" t="inlineStr">
+        <is>
+          <t>stemgedrag.html</t>
+        </is>
+      </c>
       <c r="R1458" t="inlineStr">
         <is>
           <t>live</t>
@@ -61298,6 +61388,11 @@
           <t>Wat is er mis met partijpolitiek?</t>
         </is>
       </c>
+      <c r="I1465" t="inlineStr">
+        <is>
+          <t>editie-1/nova-democratia.html</t>
+        </is>
+      </c>
       <c r="R1465" t="inlineStr">
         <is>
           <t>live</t>
@@ -61589,6 +61684,11 @@
           <t>De methaan-misleiding</t>
         </is>
       </c>
+      <c r="I1472" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-04-methaan-misleiding.html</t>
+        </is>
+      </c>
       <c r="R1472" t="inlineStr">
         <is>
           <t>live</t>
@@ -61713,6 +61813,11 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
+      <c r="I1475" t="inlineStr">
+        <is>
+          <t>editie-stikstof/drie-problemen-een-antwoord.html</t>
+        </is>
+      </c>
       <c r="R1475" t="inlineStr">
         <is>
           <t>live</t>
@@ -61751,6 +61856,11 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
+      <c r="I1476" t="inlineStr">
+        <is>
+          <t>editie-klimaat/index.html</t>
+        </is>
+      </c>
       <c r="R1476" t="inlineStr">
         <is>
           <t>live</t>
@@ -61789,6 +61899,11 @@
           <t>Editie Stikstof</t>
         </is>
       </c>
+      <c r="I1477" t="inlineStr">
+        <is>
+          <t>editie-stikstof/index.html</t>
+        </is>
+      </c>
       <c r="R1477" t="inlineStr">
         <is>
           <t>live</t>
@@ -62080,6 +62195,11 @@
           <t>De Koolzaad-Multiplicator</t>
         </is>
       </c>
+      <c r="I1484" t="inlineStr">
+        <is>
+          <t>editie-duitsland/raps-multiplicator-oost-duitsland.html</t>
+        </is>
+      </c>
       <c r="R1484" t="inlineStr">
         <is>
           <t>live</t>
@@ -62118,6 +62238,11 @@
           <t>De plant die verhuist</t>
         </is>
       </c>
+      <c r="I1485" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-05-plant-die-verhuist.html</t>
+        </is>
+      </c>
       <c r="R1485" t="inlineStr">
         <is>
           <t>live</t>
@@ -62156,6 +62281,11 @@
           <t>Editie Duitsland</t>
         </is>
       </c>
+      <c r="I1486" t="inlineStr">
+        <is>
+          <t>editie-duitsland/index.html</t>
+        </is>
+      </c>
       <c r="R1486" t="inlineStr">
         <is>
           <t>live</t>
@@ -62318,6 +62448,11 @@
           <t>De biomimetische krachtcentrale</t>
         </is>
       </c>
+      <c r="I1490" t="inlineStr">
+        <is>
+          <t>editie-0/biomimetische-krachtcentrale.html</t>
+        </is>
+      </c>
       <c r="R1490" t="inlineStr">
         <is>
           <t>live</t>
@@ -62518,6 +62653,11 @@
           <t>Editie Europa</t>
         </is>
       </c>
+      <c r="I1495" t="inlineStr">
+        <is>
+          <t>editie-0/index.html</t>
+        </is>
+      </c>
       <c r="R1495" t="inlineStr">
         <is>
           <t>live</t>
@@ -62718,6 +62858,11 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
+      <c r="I1500" t="inlineStr">
+        <is>
+          <t>editie-0/carbon-alert-europa.html</t>
+        </is>
+      </c>
       <c r="R1500" t="inlineStr">
         <is>
           <t>live</t>
@@ -62837,6 +62982,11 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
+      <c r="I1503" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-04-bankier.html</t>
+        </is>
+      </c>
       <c r="R1503" t="inlineStr">
         <is>
           <t>live</t>
@@ -63047,6 +63197,11 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
+      <c r="I1508" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-02-ceo.html</t>
+        </is>
+      </c>
       <c r="R1508" t="inlineStr">
         <is>
           <t>live</t>
@@ -63085,6 +63240,11 @@
           <t>De consultant bij het bijna-failliete bedrijf</t>
         </is>
       </c>
+      <c r="I1509" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-03-consultant.html</t>
+        </is>
+      </c>
       <c r="R1509" t="inlineStr">
         <is>
           <t>live</t>
@@ -63123,6 +63283,11 @@
           <t>De diepere vraag</t>
         </is>
       </c>
+      <c r="I1510" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-08-diepere-vraag.html</t>
+        </is>
+      </c>
       <c r="R1510" t="inlineStr">
         <is>
           <t>live</t>
@@ -63247,6 +63412,11 @@
           <t>De rechter zonder kompas</t>
         </is>
       </c>
+      <c r="I1513" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-07-rechter.html</t>
+        </is>
+      </c>
       <c r="R1513" t="inlineStr">
         <is>
           <t>live</t>
@@ -63285,6 +63455,11 @@
           <t>De toezichthouder die niets ziet</t>
         </is>
       </c>
+      <c r="I1514" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-06-toezichthouder.html</t>
+        </is>
+      </c>
       <c r="R1514" t="inlineStr">
         <is>
           <t>live</t>
@@ -63323,6 +63498,11 @@
           <t>De verzekeraar tegen het leven</t>
         </is>
       </c>
+      <c r="I1515" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-05-verzekeraar.html</t>
+        </is>
+      </c>
       <c r="R1515" t="inlineStr">
         <is>
           <t>live</t>
@@ -63361,6 +63541,11 @@
           <t>De wet van de papier-industrie</t>
         </is>
       </c>
+      <c r="I1516" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-01-wet-papier-industrie.html</t>
+        </is>
+      </c>
       <c r="R1516" t="inlineStr">
         <is>
           <t>live</t>
@@ -63523,6 +63708,11 @@
           <t>Editie Kind &amp; Loopbaan</t>
         </is>
       </c>
+      <c r="I1520" t="inlineStr">
+        <is>
+          <t>editie-kind-loopbaan/index.html</t>
+        </is>
+      </c>
       <c r="R1520" t="inlineStr">
         <is>
           <t>live</t>
@@ -63561,6 +63751,11 @@
           <t>Editie Leiderschap</t>
         </is>
       </c>
+      <c r="I1521" t="inlineStr">
+        <is>
+          <t>editie-leiderschap/index.html</t>
+        </is>
+      </c>
       <c r="R1521" t="inlineStr">
         <is>
           <t>live</t>
@@ -63599,6 +63794,11 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
+      <c r="I1522" t="inlineStr">
+        <is>
+          <t>toekomst/energie/index.html</t>
+        </is>
+      </c>
       <c r="R1522" t="inlineStr">
         <is>
           <t>live</t>
@@ -63637,6 +63837,11 @@
           <t>Hoe de papier-industrie macht kreeg over het echte werk</t>
         </is>
       </c>
+      <c r="I1523" t="inlineStr">
+        <is>
+          <t>editie-4/index.html</t>
+        </is>
+      </c>
       <c r="R1523" t="inlineStr">
         <is>
           <t>live</t>
@@ -63675,6 +63880,11 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
+      <c r="I1524" t="inlineStr">
+        <is>
+          <t>toekomst/industrie/index.html</t>
+        </is>
+      </c>
       <c r="R1524" t="inlineStr">
         <is>
           <t>live</t>
@@ -63799,6 +64009,11 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
+      <c r="I1527" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/methode/index.html</t>
+        </is>
+      </c>
       <c r="R1527" t="inlineStr">
         <is>
           <t>live</t>
@@ -63966,6 +64181,11 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
+      <c r="I1531" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-07-ai-onderwijs.html</t>
+        </is>
+      </c>
       <c r="R1531" t="inlineStr">
         <is>
           <t>live</t>
@@ -64004,6 +64224,11 @@
           <t>Opvoeding · Toekomst</t>
         </is>
       </c>
+      <c r="I1532" t="inlineStr">
+        <is>
+          <t>toekomst/opvoeding/index.html</t>
+        </is>
+      </c>
       <c r="R1532" t="inlineStr">
         <is>
           <t>live</t>
@@ -64085,6 +64310,11 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
+      <c r="I1534" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/index.html</t>
+        </is>
+      </c>
       <c r="R1534" t="inlineStr">
         <is>
           <t>live</t>
@@ -64123,6 +64353,11 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
+      <c r="I1535" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-00-redactie.html</t>
+        </is>
+      </c>
       <c r="R1535" t="inlineStr">
         <is>
           <t>live</t>
@@ -64161,6 +64396,11 @@
           <t>Retrospectief</t>
         </is>
       </c>
+      <c r="I1536" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-09-retrospectief.html</t>
+        </is>
+      </c>
       <c r="R1536" t="inlineStr">
         <is>
           <t>live</t>
@@ -64199,6 +64439,11 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
+      <c r="I1537" t="inlineStr">
+        <is>
+          <t>toekomst/scholing/index.html</t>
+        </is>
+      </c>
       <c r="R1537" t="inlineStr">
         <is>
           <t>live</t>
@@ -64237,6 +64482,11 @@
           <t>Soevereiniteit als cyclus</t>
         </is>
       </c>
+      <c r="I1538" t="inlineStr">
+        <is>
+          <t>soevereiniteit-als-cyclus/index.html</t>
+        </is>
+      </c>
       <c r="R1538" t="inlineStr">
         <is>
           <t>live</t>
@@ -64318,6 +64568,11 @@
           <t>Toekomst</t>
         </is>
       </c>
+      <c r="I1540" t="inlineStr">
+        <is>
+          <t>toekomst/index.html</t>
+        </is>
+      </c>
       <c r="R1540" t="inlineStr">
         <is>
           <t>live</t>
@@ -64442,6 +64697,11 @@
           <t>Van leerfabriek naar leerwerkplaats</t>
         </is>
       </c>
+      <c r="I1543" t="inlineStr">
+        <is>
+          <t>editie-1/onderwijs.html</t>
+        </is>
+      </c>
       <c r="R1543" t="inlineStr">
         <is>
           <t>live</t>
@@ -64690,6 +64950,11 @@
           <t>De eerste gemeente</t>
         </is>
       </c>
+      <c r="I1549" t="inlineStr">
+        <is>
+          <t>de-eerste-gemeente/index.html</t>
+        </is>
+      </c>
       <c r="R1549" t="inlineStr">
         <is>
           <t>live</t>
@@ -64728,6 +64993,11 @@
           <t>De halve gemeente</t>
         </is>
       </c>
+      <c r="I1550" t="inlineStr">
+        <is>
+          <t>de-halve-gemeente/index.html</t>
+        </is>
+      </c>
       <c r="R1550" t="inlineStr">
         <is>
           <t>live</t>
@@ -67313,6 +67583,11 @@
           <t>Een fusiereactor zonder magnetische kooi</t>
         </is>
       </c>
+      <c r="I1615" t="inlineStr">
+        <is>
+          <t>editie-1/kernfusie.html</t>
+        </is>
+      </c>
       <c r="R1615" t="inlineStr">
         <is>
           <t>live</t>
@@ -68609,6 +68884,11 @@
           <t>Vortex-Hair™ Adaptive Dimple Golf Ball — Dossier</t>
         </is>
       </c>
+      <c r="I1647" t="inlineStr">
+        <is>
+          <t>dossiers/vortex-hair.html</t>
+        </is>
+      </c>
       <c r="R1647" t="inlineStr">
         <is>
           <t>live</t>
@@ -68685,6 +68965,11 @@
           <t>Archief</t>
         </is>
       </c>
+      <c r="I1649" t="inlineStr">
+        <is>
+          <t>archief.html</t>
+        </is>
+      </c>
       <c r="R1649" t="inlineStr">
         <is>
           <t>live</t>
@@ -68723,6 +69008,11 @@
           <t>Bedankt — controleer uw inbox</t>
         </is>
       </c>
+      <c r="I1650" t="inlineStr">
+        <is>
+          <t>bedankt.html</t>
+        </is>
+      </c>
       <c r="R1650" t="inlineStr">
         <is>
           <t>live</t>
@@ -68799,6 +69089,11 @@
           <t>Het Open Vizier verder dragen</t>
         </is>
       </c>
+      <c r="I1652" t="inlineStr">
+        <is>
+          <t>delen.html</t>
+        </is>
+      </c>
       <c r="R1652" t="inlineStr">
         <is>
           <t>live</t>
@@ -68875,6 +69170,11 @@
           <t>Hoe u meedoet aan de discussie</t>
         </is>
       </c>
+      <c r="I1654" t="inlineStr">
+        <is>
+          <t>editie-1/discussie.html</t>
+        </is>
+      </c>
       <c r="R1654" t="inlineStr">
         <is>
           <t>live</t>
@@ -68913,6 +69213,11 @@
           <t>Navigatie</t>
         </is>
       </c>
+      <c r="I1655" t="inlineStr">
+        <is>
+          <t>navigatie.html</t>
+        </is>
+      </c>
       <c r="R1655" t="inlineStr">
         <is>
           <t>live</t>
@@ -68951,6 +69256,11 @@
           <t>Op de hoogte blijven</t>
         </is>
       </c>
+      <c r="I1656" t="inlineStr">
+        <is>
+          <t>op-de-hoogte.html</t>
+        </is>
+      </c>
       <c r="R1656" t="inlineStr">
         <is>
           <t>live</t>
@@ -68989,6 +69299,11 @@
           <t>Over deze krant</t>
         </is>
       </c>
+      <c r="I1657" t="inlineStr">
+        <is>
+          <t>over.html</t>
+        </is>
+      </c>
       <c r="R1657" t="inlineStr">
         <is>
           <t>live</t>
@@ -69070,6 +69385,11 @@
           <t>Structuur — Beheer</t>
         </is>
       </c>
+      <c r="I1659" t="inlineStr">
+        <is>
+          <t>structuur.html</t>
+        </is>
+      </c>
       <c r="R1659" t="inlineStr">
         <is>
           <t>live</t>
@@ -69149,6 +69469,11 @@
       <c r="F1661" t="inlineStr">
         <is>
           <t>Waarom deze krant?</t>
+        </is>
+      </c>
+      <c r="I1661" t="inlineStr">
+        <is>
+          <t>editie-1/voorwoord.html</t>
         </is>
       </c>
       <c r="R1661" t="inlineStr">

</xml_diff>

<commit_message>
IT-menu: 105 URLs ingevuld
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -70349,6 +70349,11 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
+      <c r="I1683" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-07-ai-onderwijs.html</t>
+        </is>
+      </c>
       <c r="R1683" t="inlineStr">
         <is>
           <t>live</t>
@@ -70468,6 +70473,11 @@
           <t>Alles stroomt — de moeder van alle wetenschap</t>
         </is>
       </c>
+      <c r="I1686" t="inlineStr">
+        <is>
+          <t>editie-1/stromingsleer.html</t>
+        </is>
+      </c>
       <c r="R1686" t="inlineStr">
         <is>
           <t>live</t>
@@ -70787,6 +70797,11 @@
           <t>Drie dimensies zijn te weinig</t>
         </is>
       </c>
+      <c r="I1694" t="inlineStr">
+        <is>
+          <t>editie-1/denkraam-7d.html</t>
+        </is>
+      </c>
       <c r="R1694" t="inlineStr">
         <is>
           <t>live</t>
@@ -70868,6 +70883,11 @@
           <t>Hoe alles samenhangt</t>
         </is>
       </c>
+      <c r="I1696" t="inlineStr">
+        <is>
+          <t>editie-1/samenhang.html</t>
+        </is>
+      </c>
       <c r="R1696" t="inlineStr">
         <is>
           <t>live</t>
@@ -71111,6 +71131,11 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
+      <c r="I1702" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-04-bankier.html</t>
+        </is>
+      </c>
       <c r="R1702" t="inlineStr">
         <is>
           <t>live</t>
@@ -71149,6 +71174,11 @@
           <t>Communicatie tussen oergevoelens</t>
         </is>
       </c>
+      <c r="I1703" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-04-communicatie.html</t>
+        </is>
+      </c>
       <c r="R1703" t="inlineStr">
         <is>
           <t>live</t>
@@ -71187,6 +71217,11 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
+      <c r="I1704" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-02-ceo.html</t>
+        </is>
+      </c>
       <c r="R1704" t="inlineStr">
         <is>
           <t>live</t>
@@ -71225,6 +71260,11 @@
           <t>De drie hersenlagen</t>
         </is>
       </c>
+      <c r="I1705" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-03-drie-lagen.html</t>
+        </is>
+      </c>
       <c r="R1705" t="inlineStr">
         <is>
           <t>live</t>
@@ -71263,6 +71303,11 @@
           <t>De mens onder het ijs (Editie 3)</t>
         </is>
       </c>
+      <c r="I1706" t="inlineStr">
+        <is>
+          <t>editie-3/index.html</t>
+        </is>
+      </c>
       <c r="R1706" t="inlineStr">
         <is>
           <t>live</t>
@@ -71301,6 +71346,11 @@
           <t>De zeven dimensies</t>
         </is>
       </c>
+      <c r="I1707" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-02-zeven-dimensies.html</t>
+        </is>
+      </c>
       <c r="R1707" t="inlineStr">
         <is>
           <t>live</t>
@@ -71382,6 +71432,11 @@
           <t>Het oergevoel</t>
         </is>
       </c>
+      <c r="I1709" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-01-oergevoel.html</t>
+        </is>
+      </c>
       <c r="R1709" t="inlineStr">
         <is>
           <t>live</t>
@@ -71420,6 +71475,11 @@
           <t>Het oergevoel in de beroepspraktijk</t>
         </is>
       </c>
+      <c r="I1710" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-09-oergevoel-in-beroepspraktijk.html</t>
+        </is>
+      </c>
       <c r="R1710" t="inlineStr">
         <is>
           <t>live</t>
@@ -71458,6 +71518,11 @@
           <t>Mama ik heb honger</t>
         </is>
       </c>
+      <c r="I1711" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-06-mama.html</t>
+        </is>
+      </c>
       <c r="R1711" t="inlineStr">
         <is>
           <t>live</t>
@@ -71496,6 +71561,11 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
+      <c r="I1712" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-00-redactie.html</t>
+        </is>
+      </c>
       <c r="R1712" t="inlineStr">
         <is>
           <t>live</t>
@@ -71534,6 +71604,11 @@
           <t>Retrospectief</t>
         </is>
       </c>
+      <c r="I1713" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-08-retrospectief.html</t>
+        </is>
+      </c>
       <c r="R1713" t="inlineStr">
         <is>
           <t>live</t>
@@ -71615,6 +71690,11 @@
           <t>Tien seconden</t>
         </is>
       </c>
+      <c r="I1715" t="inlineStr">
+        <is>
+          <t>idee.html</t>
+        </is>
+      </c>
       <c r="R1715" t="inlineStr">
         <is>
           <t>live</t>
@@ -71696,6 +71776,11 @@
           <t>Wat we kinderen aandoen</t>
         </is>
       </c>
+      <c r="I1717" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-05-wat-we-doen.html</t>
+        </is>
+      </c>
       <c r="R1717" t="inlineStr">
         <is>
           <t>live</t>
@@ -72488,6 +72573,11 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
+      <c r="I1736" t="inlineStr">
+        <is>
+          <t>stemgedrag.html</t>
+        </is>
+      </c>
       <c r="R1736" t="inlineStr">
         <is>
           <t>live</t>
@@ -72774,6 +72864,11 @@
           <t>Wat is er mis met partijpolitiek?</t>
         </is>
       </c>
+      <c r="I1743" t="inlineStr">
+        <is>
+          <t>editie-1/nova-democratia.html</t>
+        </is>
+      </c>
       <c r="R1743" t="inlineStr">
         <is>
           <t>live</t>
@@ -73065,6 +73160,11 @@
           <t>De methaan-misleiding</t>
         </is>
       </c>
+      <c r="I1750" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-04-methaan-misleiding.html</t>
+        </is>
+      </c>
       <c r="R1750" t="inlineStr">
         <is>
           <t>live</t>
@@ -73189,6 +73289,11 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
+      <c r="I1753" t="inlineStr">
+        <is>
+          <t>editie-stikstof/drie-problemen-een-antwoord.html</t>
+        </is>
+      </c>
       <c r="R1753" t="inlineStr">
         <is>
           <t>live</t>
@@ -73227,6 +73332,11 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
+      <c r="I1754" t="inlineStr">
+        <is>
+          <t>editie-klimaat/index.html</t>
+        </is>
+      </c>
       <c r="R1754" t="inlineStr">
         <is>
           <t>live</t>
@@ -73265,6 +73375,11 @@
           <t>Editie Stikstof</t>
         </is>
       </c>
+      <c r="I1755" t="inlineStr">
+        <is>
+          <t>editie-stikstof/index.html</t>
+        </is>
+      </c>
       <c r="R1755" t="inlineStr">
         <is>
           <t>live</t>
@@ -73556,6 +73671,11 @@
           <t>De Koolzaad-Multiplicator</t>
         </is>
       </c>
+      <c r="I1762" t="inlineStr">
+        <is>
+          <t>editie-duitsland/raps-multiplicator-oost-duitsland.html</t>
+        </is>
+      </c>
       <c r="R1762" t="inlineStr">
         <is>
           <t>live</t>
@@ -73594,6 +73714,11 @@
           <t>De plant die verhuist</t>
         </is>
       </c>
+      <c r="I1763" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-05-plant-die-verhuist.html</t>
+        </is>
+      </c>
       <c r="R1763" t="inlineStr">
         <is>
           <t>live</t>
@@ -73632,6 +73757,11 @@
           <t>Editie Duitsland</t>
         </is>
       </c>
+      <c r="I1764" t="inlineStr">
+        <is>
+          <t>editie-duitsland/index.html</t>
+        </is>
+      </c>
       <c r="R1764" t="inlineStr">
         <is>
           <t>live</t>
@@ -73794,6 +73924,11 @@
           <t>De biomimetische krachtcentrale</t>
         </is>
       </c>
+      <c r="I1768" t="inlineStr">
+        <is>
+          <t>editie-0/biomimetische-krachtcentrale.html</t>
+        </is>
+      </c>
       <c r="R1768" t="inlineStr">
         <is>
           <t>live</t>
@@ -73994,6 +74129,11 @@
           <t>Editie Europa</t>
         </is>
       </c>
+      <c r="I1773" t="inlineStr">
+        <is>
+          <t>editie-0/index.html</t>
+        </is>
+      </c>
       <c r="R1773" t="inlineStr">
         <is>
           <t>live</t>
@@ -74194,6 +74334,11 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
+      <c r="I1778" t="inlineStr">
+        <is>
+          <t>editie-0/carbon-alert-europa.html</t>
+        </is>
+      </c>
       <c r="R1778" t="inlineStr">
         <is>
           <t>live</t>
@@ -74313,6 +74458,11 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
+      <c r="I1781" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-04-bankier.html</t>
+        </is>
+      </c>
       <c r="R1781" t="inlineStr">
         <is>
           <t>live</t>
@@ -74523,6 +74673,11 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
+      <c r="I1786" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-02-ceo.html</t>
+        </is>
+      </c>
       <c r="R1786" t="inlineStr">
         <is>
           <t>live</t>
@@ -74561,6 +74716,11 @@
           <t>De consultant bij het bijna-failliete bedrijf</t>
         </is>
       </c>
+      <c r="I1787" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-03-consultant.html</t>
+        </is>
+      </c>
       <c r="R1787" t="inlineStr">
         <is>
           <t>live</t>
@@ -74599,6 +74759,11 @@
           <t>De diepere vraag</t>
         </is>
       </c>
+      <c r="I1788" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-08-diepere-vraag.html</t>
+        </is>
+      </c>
       <c r="R1788" t="inlineStr">
         <is>
           <t>live</t>
@@ -74723,6 +74888,11 @@
           <t>De rechter zonder kompas</t>
         </is>
       </c>
+      <c r="I1791" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-07-rechter.html</t>
+        </is>
+      </c>
       <c r="R1791" t="inlineStr">
         <is>
           <t>live</t>
@@ -74761,6 +74931,11 @@
           <t>De toezichthouder die niets ziet</t>
         </is>
       </c>
+      <c r="I1792" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-06-toezichthouder.html</t>
+        </is>
+      </c>
       <c r="R1792" t="inlineStr">
         <is>
           <t>live</t>
@@ -74799,6 +74974,11 @@
           <t>De verzekeraar tegen het leven</t>
         </is>
       </c>
+      <c r="I1793" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-05-verzekeraar.html</t>
+        </is>
+      </c>
       <c r="R1793" t="inlineStr">
         <is>
           <t>live</t>
@@ -74837,6 +75017,11 @@
           <t>De wet van de papier-industrie</t>
         </is>
       </c>
+      <c r="I1794" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-01-wet-papier-industrie.html</t>
+        </is>
+      </c>
       <c r="R1794" t="inlineStr">
         <is>
           <t>live</t>
@@ -74999,6 +75184,11 @@
           <t>Editie Kind &amp; Loopbaan</t>
         </is>
       </c>
+      <c r="I1798" t="inlineStr">
+        <is>
+          <t>editie-kind-loopbaan/index.html</t>
+        </is>
+      </c>
       <c r="R1798" t="inlineStr">
         <is>
           <t>live</t>
@@ -75037,6 +75227,11 @@
           <t>Editie Leiderschap</t>
         </is>
       </c>
+      <c r="I1799" t="inlineStr">
+        <is>
+          <t>editie-leiderschap/index.html</t>
+        </is>
+      </c>
       <c r="R1799" t="inlineStr">
         <is>
           <t>live</t>
@@ -75075,6 +75270,11 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
+      <c r="I1800" t="inlineStr">
+        <is>
+          <t>toekomst/energie/index.html</t>
+        </is>
+      </c>
       <c r="R1800" t="inlineStr">
         <is>
           <t>live</t>
@@ -75113,6 +75313,11 @@
           <t>Hoe de papier-industrie macht kreeg over het echte werk</t>
         </is>
       </c>
+      <c r="I1801" t="inlineStr">
+        <is>
+          <t>editie-4/index.html</t>
+        </is>
+      </c>
       <c r="R1801" t="inlineStr">
         <is>
           <t>live</t>
@@ -75151,6 +75356,11 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
+      <c r="I1802" t="inlineStr">
+        <is>
+          <t>toekomst/industrie/index.html</t>
+        </is>
+      </c>
       <c r="R1802" t="inlineStr">
         <is>
           <t>live</t>
@@ -75275,6 +75485,11 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
+      <c r="I1805" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/methode/index.html</t>
+        </is>
+      </c>
       <c r="R1805" t="inlineStr">
         <is>
           <t>live</t>
@@ -75442,6 +75657,11 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
+      <c r="I1809" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-07-ai-onderwijs.html</t>
+        </is>
+      </c>
       <c r="R1809" t="inlineStr">
         <is>
           <t>live</t>
@@ -75480,6 +75700,11 @@
           <t>Opvoeding · Toekomst</t>
         </is>
       </c>
+      <c r="I1810" t="inlineStr">
+        <is>
+          <t>toekomst/opvoeding/index.html</t>
+        </is>
+      </c>
       <c r="R1810" t="inlineStr">
         <is>
           <t>live</t>
@@ -75561,6 +75786,11 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
+      <c r="I1812" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/index.html</t>
+        </is>
+      </c>
       <c r="R1812" t="inlineStr">
         <is>
           <t>live</t>
@@ -75599,6 +75829,11 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
+      <c r="I1813" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-00-redactie.html</t>
+        </is>
+      </c>
       <c r="R1813" t="inlineStr">
         <is>
           <t>live</t>
@@ -75637,6 +75872,11 @@
           <t>Retrospectief</t>
         </is>
       </c>
+      <c r="I1814" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-09-retrospectief.html</t>
+        </is>
+      </c>
       <c r="R1814" t="inlineStr">
         <is>
           <t>live</t>
@@ -75675,6 +75915,11 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
+      <c r="I1815" t="inlineStr">
+        <is>
+          <t>toekomst/scholing/index.html</t>
+        </is>
+      </c>
       <c r="R1815" t="inlineStr">
         <is>
           <t>live</t>
@@ -75713,6 +75958,11 @@
           <t>Soevereiniteit als cyclus</t>
         </is>
       </c>
+      <c r="I1816" t="inlineStr">
+        <is>
+          <t>soevereiniteit-als-cyclus/index.html</t>
+        </is>
+      </c>
       <c r="R1816" t="inlineStr">
         <is>
           <t>live</t>
@@ -75794,6 +76044,11 @@
           <t>Toekomst</t>
         </is>
       </c>
+      <c r="I1818" t="inlineStr">
+        <is>
+          <t>toekomst/index.html</t>
+        </is>
+      </c>
       <c r="R1818" t="inlineStr">
         <is>
           <t>live</t>
@@ -75918,6 +76173,11 @@
           <t>Van leerfabriek naar leerwerkplaats</t>
         </is>
       </c>
+      <c r="I1821" t="inlineStr">
+        <is>
+          <t>editie-1/onderwijs.html</t>
+        </is>
+      </c>
       <c r="R1821" t="inlineStr">
         <is>
           <t>live</t>
@@ -76166,6 +76426,11 @@
           <t>De eerste gemeente</t>
         </is>
       </c>
+      <c r="I1827" t="inlineStr">
+        <is>
+          <t>de-eerste-gemeente/index.html</t>
+        </is>
+      </c>
       <c r="R1827" t="inlineStr">
         <is>
           <t>live</t>
@@ -76204,6 +76469,11 @@
           <t>De halve gemeente</t>
         </is>
       </c>
+      <c r="I1828" t="inlineStr">
+        <is>
+          <t>de-halve-gemeente/index.html</t>
+        </is>
+      </c>
       <c r="R1828" t="inlineStr">
         <is>
           <t>live</t>
@@ -76366,6 +76636,11 @@
           <t>Gevolgenkaart — Nederland</t>
         </is>
       </c>
+      <c r="I1832" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-nl/index.html</t>
+        </is>
+      </c>
       <c r="R1832" t="inlineStr">
         <is>
           <t>live</t>
@@ -76485,6 +76760,11 @@
           <t>Nederland · Toekomst</t>
         </is>
       </c>
+      <c r="I1835" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/nederland/index.html</t>
+        </is>
+      </c>
       <c r="R1835" t="inlineStr">
         <is>
           <t>live</t>
@@ -77110,6 +77390,11 @@
           <t>Duitsland · Toekomst</t>
         </is>
       </c>
+      <c r="I1850" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/duitsland/index.html</t>
+        </is>
+      </c>
       <c r="R1850" t="inlineStr">
         <is>
           <t>live</t>
@@ -77277,6 +77562,11 @@
           <t>Europa · Toekomst</t>
         </is>
       </c>
+      <c r="I1854" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/europa/index.html</t>
+        </is>
+      </c>
       <c r="R1854" t="inlineStr">
         <is>
           <t>live</t>
@@ -77315,6 +77605,11 @@
           <t>Gevolgenkaart EU-27</t>
         </is>
       </c>
+      <c r="I1855" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-eu/index.html</t>
+        </is>
+      </c>
       <c r="R1855" t="inlineStr">
         <is>
           <t>live</t>
@@ -77353,6 +77648,11 @@
           <t>Gevolgenkaart — Brazilië</t>
         </is>
       </c>
+      <c r="I1856" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-br/index.html</t>
+        </is>
+      </c>
       <c r="R1856" t="inlineStr">
         <is>
           <t>live</t>
@@ -77391,6 +77691,11 @@
           <t>Gevolgenkaart — China</t>
         </is>
       </c>
+      <c r="I1857" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-cn/index.html</t>
+        </is>
+      </c>
       <c r="R1857" t="inlineStr">
         <is>
           <t>live</t>
@@ -77429,6 +77734,11 @@
           <t>Gevolgenkaart — Cuba</t>
         </is>
       </c>
+      <c r="I1858" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-cu/index.html</t>
+        </is>
+      </c>
       <c r="R1858" t="inlineStr">
         <is>
           <t>live</t>
@@ -77467,6 +77777,11 @@
           <t>Gevolgenkaart — Duitsland</t>
         </is>
       </c>
+      <c r="I1859" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-de/index.html</t>
+        </is>
+      </c>
       <c r="R1859" t="inlineStr">
         <is>
           <t>live</t>
@@ -77505,6 +77820,11 @@
           <t>Gevolgenkaart — India</t>
         </is>
       </c>
+      <c r="I1860" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-in/index.html</t>
+        </is>
+      </c>
       <c r="R1860" t="inlineStr">
         <is>
           <t>live</t>
@@ -77543,6 +77863,11 @@
           <t>Gevolgenkaart — Iran</t>
         </is>
       </c>
+      <c r="I1861" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-ir/index.html</t>
+        </is>
+      </c>
       <c r="R1861" t="inlineStr">
         <is>
           <t>live</t>
@@ -77581,6 +77906,11 @@
           <t>Gevolgenkaart — Israël</t>
         </is>
       </c>
+      <c r="I1862" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-il/index.html</t>
+        </is>
+      </c>
       <c r="R1862" t="inlineStr">
         <is>
           <t>live</t>
@@ -77619,6 +77949,11 @@
           <t>Gevolgenkaart — Japan</t>
         </is>
       </c>
+      <c r="I1863" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-jp/index.html</t>
+        </is>
+      </c>
       <c r="R1863" t="inlineStr">
         <is>
           <t>live</t>
@@ -77657,6 +77992,11 @@
           <t>Gevolgenkaart — Spanje</t>
         </is>
       </c>
+      <c r="I1864" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-es/index.html</t>
+        </is>
+      </c>
       <c r="R1864" t="inlineStr">
         <is>
           <t>live</t>
@@ -77695,6 +78035,11 @@
           <t>Gevolgenkaart — Suriname</t>
         </is>
       </c>
+      <c r="I1865" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-sr/index.html</t>
+        </is>
+      </c>
       <c r="R1865" t="inlineStr">
         <is>
           <t>live</t>
@@ -77733,6 +78078,11 @@
           <t>Gevolgenkaart — Taiwan</t>
         </is>
       </c>
+      <c r="I1866" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-tw/index.html</t>
+        </is>
+      </c>
       <c r="R1866" t="inlineStr">
         <is>
           <t>live</t>
@@ -77771,6 +78121,11 @@
           <t>Gevolgenkaart — Verenigd Koninkrijk</t>
         </is>
       </c>
+      <c r="I1867" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-uk/index.html</t>
+        </is>
+      </c>
       <c r="R1867" t="inlineStr">
         <is>
           <t>live</t>
@@ -77809,6 +78164,11 @@
           <t>Gevolgenkaart — Verenigde Staten</t>
         </is>
       </c>
+      <c r="I1868" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-us/index.html</t>
+        </is>
+      </c>
       <c r="R1868" t="inlineStr">
         <is>
           <t>live</t>
@@ -77847,6 +78207,11 @@
           <t>Gevolgenkaart — Zuid-Afrika</t>
         </is>
       </c>
+      <c r="I1869" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-za/index.html</t>
+        </is>
+      </c>
       <c r="R1869" t="inlineStr">
         <is>
           <t>live</t>
@@ -77885,6 +78250,11 @@
           <t>Gevolgenkaart — Zuid-Korea</t>
         </is>
       </c>
+      <c r="I1870" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-kr/index.html</t>
+        </is>
+      </c>
       <c r="R1870" t="inlineStr">
         <is>
           <t>live</t>
@@ -77923,6 +78293,11 @@
           <t>Gevolgenkaart — Zweden</t>
         </is>
       </c>
+      <c r="I1871" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-se/index.html</t>
+        </is>
+      </c>
       <c r="R1871" t="inlineStr">
         <is>
           <t>live</t>
@@ -77961,6 +78336,11 @@
           <t>Gevolgenkaart — Zwitserland</t>
         </is>
       </c>
+      <c r="I1872" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-ch/index.html</t>
+        </is>
+      </c>
       <c r="R1872" t="inlineStr">
         <is>
           <t>live</t>
@@ -78295,6 +78675,11 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
+      <c r="I1880" t="inlineStr">
+        <is>
+          <t>editie-0/carbon-alert-europa.html</t>
+        </is>
+      </c>
       <c r="R1880" t="inlineStr">
         <is>
           <t>live</t>
@@ -78414,6 +78799,11 @@
           <t>Brief aan de lezer</t>
         </is>
       </c>
+      <c r="I1883" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-00-brief-aan-lezer.html</t>
+        </is>
+      </c>
       <c r="R1883" t="inlineStr">
         <is>
           <t>live</t>
@@ -78452,6 +78842,11 @@
           <t>De afwijkers</t>
         </is>
       </c>
+      <c r="I1884" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-07-afwijkers.html</t>
+        </is>
+      </c>
       <c r="R1884" t="inlineStr">
         <is>
           <t>live</t>
@@ -78490,6 +78885,11 @@
           <t>De eis aan de lezer</t>
         </is>
       </c>
+      <c r="I1885" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-08-eis-aan-lezer.html</t>
+        </is>
+      </c>
       <c r="R1885" t="inlineStr">
         <is>
           <t>live</t>
@@ -78528,6 +78928,11 @@
           <t>De methaan-misleiding</t>
         </is>
       </c>
+      <c r="I1886" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-04-methaan-misleiding.html</t>
+        </is>
+      </c>
       <c r="R1886" t="inlineStr">
         <is>
           <t>live</t>
@@ -78566,6 +78971,11 @@
           <t>De plant die verhuist</t>
         </is>
       </c>
+      <c r="I1887" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-05-plant-die-verhuist.html</t>
+        </is>
+      </c>
       <c r="R1887" t="inlineStr">
         <is>
           <t>live</t>
@@ -78604,6 +79014,11 @@
           <t>De succesformule die wij verleerd hebben</t>
         </is>
       </c>
+      <c r="I1888" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-02-succesformule.html</t>
+        </is>
+      </c>
       <c r="R1888" t="inlineStr">
         <is>
           <t>live</t>
@@ -78642,6 +79057,11 @@
           <t>De vergeten orde</t>
         </is>
       </c>
+      <c r="I1889" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-03-vergeten-orde.html</t>
+        </is>
+      </c>
       <c r="R1889" t="inlineStr">
         <is>
           <t>live</t>
@@ -78680,6 +79100,11 @@
           <t>De zeven van Bern</t>
         </is>
       </c>
+      <c r="I1890" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-06-zeven-van-bern.html</t>
+        </is>
+      </c>
       <c r="R1890" t="inlineStr">
         <is>
           <t>live</t>
@@ -78718,6 +79143,11 @@
           <t>Editie 1</t>
         </is>
       </c>
+      <c r="I1891" t="inlineStr">
+        <is>
+          <t>editie-1/index.html</t>
+        </is>
+      </c>
       <c r="R1891" t="inlineStr">
         <is>
           <t>live</t>
@@ -78756,6 +79186,11 @@
           <t>Editie 5 — portaal</t>
         </is>
       </c>
+      <c r="I1892" t="inlineStr">
+        <is>
+          <t>editie-5/index.html</t>
+        </is>
+      </c>
       <c r="R1892" t="inlineStr">
         <is>
           <t>live</t>
@@ -78794,6 +79229,11 @@
           <t>Een fusiereactor zonder magnetische kooi</t>
         </is>
       </c>
+      <c r="I1893" t="inlineStr">
+        <is>
+          <t>editie-1/kernfusie.html</t>
+        </is>
+      </c>
       <c r="R1893" t="inlineStr">
         <is>
           <t>live</t>
@@ -78875,6 +79315,11 @@
           <t>Wat er nu al ligt</t>
         </is>
       </c>
+      <c r="I1895" t="inlineStr">
+        <is>
+          <t>editie-1/technische-oplossingen.html</t>
+        </is>
+      </c>
       <c r="R1895" t="inlineStr">
         <is>
           <t>live</t>
@@ -78913,6 +79358,11 @@
           <t>七つ道具 — Zeven gereedschappen</t>
         </is>
       </c>
+      <c r="I1896" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-01-zeven-gereedschappen.html</t>
+        </is>
+      </c>
       <c r="R1896" t="inlineStr">
         <is>
           <t>live</t>
@@ -79647,6 +80097,11 @@
           <t>Wie zijn opbouwers wegjaagt</t>
         </is>
       </c>
+      <c r="I1914" t="inlineStr">
+        <is>
+          <t>opbouwers-wegjagen/index.html</t>
+        </is>
+      </c>
       <c r="R1914" t="inlineStr">
         <is>
           <t>live</t>
@@ -79723,6 +80178,11 @@
           <t>Achter de Cijfers</t>
         </is>
       </c>
+      <c r="I1916" t="inlineStr">
+        <is>
+          <t>onderzoek/index.html</t>
+        </is>
+      </c>
       <c r="R1916" t="inlineStr">
         <is>
           <t>live</t>
@@ -79761,6 +80221,11 @@
           <t>Dossiers</t>
         </is>
       </c>
+      <c r="I1917" t="inlineStr">
+        <is>
+          <t>dossiers/index.html</t>
+        </is>
+      </c>
       <c r="R1917" t="inlineStr">
         <is>
           <t>live</t>
@@ -79799,6 +80264,11 @@
           <t>EU: BBP, Reële Lonen en de Overheidsmultiplicator</t>
         </is>
       </c>
+      <c r="I1918" t="inlineStr">
+        <is>
+          <t>onderzoek/eu-multiplicator.html</t>
+        </is>
+      </c>
       <c r="R1918" t="inlineStr">
         <is>
           <t>live</t>
@@ -80009,6 +80479,11 @@
           <t>Is Nederland op weg naar ontwikkelingslandstatus?</t>
         </is>
       </c>
+      <c r="I1923" t="inlineStr">
+        <is>
+          <t>onderzoek/ontwikkelingslandstatus.html</t>
+        </is>
+      </c>
       <c r="R1923" t="inlineStr">
         <is>
           <t>live</t>
@@ -80090,6 +80565,11 @@
           <t>Vortex-Hair™ Adaptive Dimple Golf Ball — Dossier</t>
         </is>
       </c>
+      <c r="I1925" t="inlineStr">
+        <is>
+          <t>dossiers/vortex-hair.html</t>
+        </is>
+      </c>
       <c r="R1925" t="inlineStr">
         <is>
           <t>live</t>
@@ -80166,6 +80646,11 @@
           <t>Archief</t>
         </is>
       </c>
+      <c r="I1927" t="inlineStr">
+        <is>
+          <t>archief.html</t>
+        </is>
+      </c>
       <c r="R1927" t="inlineStr">
         <is>
           <t>live</t>
@@ -80204,6 +80689,11 @@
           <t>Bedankt — controleer uw inbox</t>
         </is>
       </c>
+      <c r="I1928" t="inlineStr">
+        <is>
+          <t>bedankt.html</t>
+        </is>
+      </c>
       <c r="R1928" t="inlineStr">
         <is>
           <t>live</t>
@@ -80280,6 +80770,11 @@
           <t>Het Open Vizier verder dragen</t>
         </is>
       </c>
+      <c r="I1930" t="inlineStr">
+        <is>
+          <t>delen.html</t>
+        </is>
+      </c>
       <c r="R1930" t="inlineStr">
         <is>
           <t>live</t>
@@ -80356,6 +80851,11 @@
           <t>Hoe u meedoet aan de discussie</t>
         </is>
       </c>
+      <c r="I1932" t="inlineStr">
+        <is>
+          <t>editie-1/discussie.html</t>
+        </is>
+      </c>
       <c r="R1932" t="inlineStr">
         <is>
           <t>live</t>
@@ -80394,6 +80894,11 @@
           <t>Navigatie</t>
         </is>
       </c>
+      <c r="I1933" t="inlineStr">
+        <is>
+          <t>navigatie.html</t>
+        </is>
+      </c>
       <c r="R1933" t="inlineStr">
         <is>
           <t>live</t>
@@ -80432,6 +80937,11 @@
           <t>Op de hoogte blijven</t>
         </is>
       </c>
+      <c r="I1934" t="inlineStr">
+        <is>
+          <t>op-de-hoogte.html</t>
+        </is>
+      </c>
       <c r="R1934" t="inlineStr">
         <is>
           <t>live</t>
@@ -80470,6 +80980,11 @@
           <t>Over deze krant</t>
         </is>
       </c>
+      <c r="I1935" t="inlineStr">
+        <is>
+          <t>over.html</t>
+        </is>
+      </c>
       <c r="R1935" t="inlineStr">
         <is>
           <t>live</t>
@@ -80551,6 +81066,11 @@
           <t>Structuur — Beheer</t>
         </is>
       </c>
+      <c r="I1937" t="inlineStr">
+        <is>
+          <t>structuur.html</t>
+        </is>
+      </c>
       <c r="R1937" t="inlineStr">
         <is>
           <t>live</t>
@@ -80630,6 +81150,11 @@
       <c r="F1939" t="inlineStr">
         <is>
           <t>Waarom deze krant?</t>
+        </is>
+      </c>
+      <c r="I1939" t="inlineStr">
+        <is>
+          <t>editie-1/voorwoord.html</t>
         </is>
       </c>
       <c r="R1939" t="inlineStr">

</xml_diff>

<commit_message>
PT-menu: 73 URLs ingevuld
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -82030,6 +82030,11 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
+      <c r="I1961" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-07-ai-onderwijs.html</t>
+        </is>
+      </c>
       <c r="R1961" t="inlineStr">
         <is>
           <t>live</t>
@@ -82149,6 +82154,11 @@
           <t>Alles stroomt — de moeder van alle wetenschap</t>
         </is>
       </c>
+      <c r="I1964" t="inlineStr">
+        <is>
+          <t>editie-1/stromingsleer.html</t>
+        </is>
+      </c>
       <c r="R1964" t="inlineStr">
         <is>
           <t>live</t>
@@ -82468,6 +82478,11 @@
           <t>Drie dimensies zijn te weinig</t>
         </is>
       </c>
+      <c r="I1972" t="inlineStr">
+        <is>
+          <t>editie-1/denkraam-7d.html</t>
+        </is>
+      </c>
       <c r="R1972" t="inlineStr">
         <is>
           <t>live</t>
@@ -82549,6 +82564,11 @@
           <t>Hoe alles samenhangt</t>
         </is>
       </c>
+      <c r="I1974" t="inlineStr">
+        <is>
+          <t>editie-1/samenhang.html</t>
+        </is>
+      </c>
       <c r="R1974" t="inlineStr">
         <is>
           <t>live</t>
@@ -82792,6 +82812,11 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
+      <c r="I1980" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-04-bankier.html</t>
+        </is>
+      </c>
       <c r="R1980" t="inlineStr">
         <is>
           <t>live</t>
@@ -82830,6 +82855,11 @@
           <t>Communicatie tussen oergevoelens</t>
         </is>
       </c>
+      <c r="I1981" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-04-communicatie.html</t>
+        </is>
+      </c>
       <c r="R1981" t="inlineStr">
         <is>
           <t>live</t>
@@ -82868,6 +82898,11 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
+      <c r="I1982" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-02-ceo.html</t>
+        </is>
+      </c>
       <c r="R1982" t="inlineStr">
         <is>
           <t>live</t>
@@ -82906,6 +82941,11 @@
           <t>De drie hersenlagen</t>
         </is>
       </c>
+      <c r="I1983" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-03-drie-lagen.html</t>
+        </is>
+      </c>
       <c r="R1983" t="inlineStr">
         <is>
           <t>live</t>
@@ -82944,6 +82984,11 @@
           <t>De mens onder het ijs (Editie 3)</t>
         </is>
       </c>
+      <c r="I1984" t="inlineStr">
+        <is>
+          <t>editie-3/index.html</t>
+        </is>
+      </c>
       <c r="R1984" t="inlineStr">
         <is>
           <t>live</t>
@@ -82982,6 +83027,11 @@
           <t>De zeven dimensies</t>
         </is>
       </c>
+      <c r="I1985" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-02-zeven-dimensies.html</t>
+        </is>
+      </c>
       <c r="R1985" t="inlineStr">
         <is>
           <t>live</t>
@@ -83063,6 +83113,11 @@
           <t>Het oergevoel</t>
         </is>
       </c>
+      <c r="I1987" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-01-oergevoel.html</t>
+        </is>
+      </c>
       <c r="R1987" t="inlineStr">
         <is>
           <t>live</t>
@@ -83101,6 +83156,11 @@
           <t>Het oergevoel in de beroepspraktijk</t>
         </is>
       </c>
+      <c r="I1988" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-09-oergevoel-in-beroepspraktijk.html</t>
+        </is>
+      </c>
       <c r="R1988" t="inlineStr">
         <is>
           <t>live</t>
@@ -83139,6 +83199,11 @@
           <t>Mama ik heb honger</t>
         </is>
       </c>
+      <c r="I1989" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-06-mama.html</t>
+        </is>
+      </c>
       <c r="R1989" t="inlineStr">
         <is>
           <t>live</t>
@@ -83177,6 +83242,11 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
+      <c r="I1990" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-00-redactie.html</t>
+        </is>
+      </c>
       <c r="R1990" t="inlineStr">
         <is>
           <t>live</t>
@@ -83215,6 +83285,11 @@
           <t>Retrospectief</t>
         </is>
       </c>
+      <c r="I1991" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-08-retrospectief.html</t>
+        </is>
+      </c>
       <c r="R1991" t="inlineStr">
         <is>
           <t>live</t>
@@ -83296,6 +83371,11 @@
           <t>Tien seconden</t>
         </is>
       </c>
+      <c r="I1993" t="inlineStr">
+        <is>
+          <t>idee.html</t>
+        </is>
+      </c>
       <c r="R1993" t="inlineStr">
         <is>
           <t>live</t>
@@ -83377,6 +83457,11 @@
           <t>Wat we kinderen aandoen</t>
         </is>
       </c>
+      <c r="I1995" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-05-wat-we-doen.html</t>
+        </is>
+      </c>
       <c r="R1995" t="inlineStr">
         <is>
           <t>live</t>
@@ -84149,6 +84234,11 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
+      <c r="I2014" t="inlineStr">
+        <is>
+          <t>stemgedrag.html</t>
+        </is>
+      </c>
       <c r="R2014" t="inlineStr">
         <is>
           <t>live</t>
@@ -84435,6 +84525,11 @@
           <t>Wat is er mis met partijpolitiek?</t>
         </is>
       </c>
+      <c r="I2021" t="inlineStr">
+        <is>
+          <t>editie-1/nova-democratia.html</t>
+        </is>
+      </c>
       <c r="R2021" t="inlineStr">
         <is>
           <t>live</t>
@@ -84726,6 +84821,11 @@
           <t>De methaan-misleiding</t>
         </is>
       </c>
+      <c r="I2028" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-04-methaan-misleiding.html</t>
+        </is>
+      </c>
       <c r="R2028" t="inlineStr">
         <is>
           <t>live</t>
@@ -84850,6 +84950,11 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
+      <c r="I2031" t="inlineStr">
+        <is>
+          <t>editie-stikstof/drie-problemen-een-antwoord.html</t>
+        </is>
+      </c>
       <c r="R2031" t="inlineStr">
         <is>
           <t>live</t>
@@ -84888,6 +84993,11 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
+      <c r="I2032" t="inlineStr">
+        <is>
+          <t>editie-klimaat/index.html</t>
+        </is>
+      </c>
       <c r="R2032" t="inlineStr">
         <is>
           <t>live</t>
@@ -84926,6 +85036,11 @@
           <t>Editie Stikstof</t>
         </is>
       </c>
+      <c r="I2033" t="inlineStr">
+        <is>
+          <t>editie-stikstof/index.html</t>
+        </is>
+      </c>
       <c r="R2033" t="inlineStr">
         <is>
           <t>live</t>
@@ -85217,6 +85332,11 @@
           <t>De Koolzaad-Multiplicator</t>
         </is>
       </c>
+      <c r="I2040" t="inlineStr">
+        <is>
+          <t>editie-duitsland/raps-multiplicator-oost-duitsland.html</t>
+        </is>
+      </c>
       <c r="R2040" t="inlineStr">
         <is>
           <t>live</t>
@@ -85255,6 +85375,11 @@
           <t>De plant die verhuist</t>
         </is>
       </c>
+      <c r="I2041" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-05-plant-die-verhuist.html</t>
+        </is>
+      </c>
       <c r="R2041" t="inlineStr">
         <is>
           <t>live</t>
@@ -85293,6 +85418,11 @@
           <t>Editie Duitsland</t>
         </is>
       </c>
+      <c r="I2042" t="inlineStr">
+        <is>
+          <t>editie-duitsland/index.html</t>
+        </is>
+      </c>
       <c r="R2042" t="inlineStr">
         <is>
           <t>live</t>
@@ -85455,6 +85585,11 @@
           <t>De biomimetische krachtcentrale</t>
         </is>
       </c>
+      <c r="I2046" t="inlineStr">
+        <is>
+          <t>editie-0/biomimetische-krachtcentrale.html</t>
+        </is>
+      </c>
       <c r="R2046" t="inlineStr">
         <is>
           <t>live</t>
@@ -85655,6 +85790,11 @@
           <t>Editie Europa</t>
         </is>
       </c>
+      <c r="I2051" t="inlineStr">
+        <is>
+          <t>editie-0/index.html</t>
+        </is>
+      </c>
       <c r="R2051" t="inlineStr">
         <is>
           <t>live</t>
@@ -85855,6 +85995,11 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
+      <c r="I2056" t="inlineStr">
+        <is>
+          <t>editie-0/carbon-alert-europa.html</t>
+        </is>
+      </c>
       <c r="R2056" t="inlineStr">
         <is>
           <t>live</t>
@@ -85974,6 +86119,11 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
+      <c r="I2059" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-04-bankier.html</t>
+        </is>
+      </c>
       <c r="R2059" t="inlineStr">
         <is>
           <t>live</t>
@@ -86184,6 +86334,11 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
+      <c r="I2064" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-02-ceo.html</t>
+        </is>
+      </c>
       <c r="R2064" t="inlineStr">
         <is>
           <t>live</t>
@@ -86222,6 +86377,11 @@
           <t>De consultant bij het bijna-failliete bedrijf</t>
         </is>
       </c>
+      <c r="I2065" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-03-consultant.html</t>
+        </is>
+      </c>
       <c r="R2065" t="inlineStr">
         <is>
           <t>live</t>
@@ -86260,6 +86420,11 @@
           <t>De diepere vraag</t>
         </is>
       </c>
+      <c r="I2066" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-08-diepere-vraag.html</t>
+        </is>
+      </c>
       <c r="R2066" t="inlineStr">
         <is>
           <t>live</t>
@@ -86384,6 +86549,11 @@
           <t>De rechter zonder kompas</t>
         </is>
       </c>
+      <c r="I2069" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-07-rechter.html</t>
+        </is>
+      </c>
       <c r="R2069" t="inlineStr">
         <is>
           <t>live</t>
@@ -86422,6 +86592,11 @@
           <t>De toezichthouder die niets ziet</t>
         </is>
       </c>
+      <c r="I2070" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-06-toezichthouder.html</t>
+        </is>
+      </c>
       <c r="R2070" t="inlineStr">
         <is>
           <t>live</t>
@@ -86460,6 +86635,11 @@
           <t>De verzekeraar tegen het leven</t>
         </is>
       </c>
+      <c r="I2071" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-05-verzekeraar.html</t>
+        </is>
+      </c>
       <c r="R2071" t="inlineStr">
         <is>
           <t>live</t>
@@ -86498,6 +86678,11 @@
           <t>De wet van de papier-industrie</t>
         </is>
       </c>
+      <c r="I2072" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-01-wet-papier-industrie.html</t>
+        </is>
+      </c>
       <c r="R2072" t="inlineStr">
         <is>
           <t>live</t>
@@ -86660,6 +86845,11 @@
           <t>Editie Kind &amp; Loopbaan</t>
         </is>
       </c>
+      <c r="I2076" t="inlineStr">
+        <is>
+          <t>editie-kind-loopbaan/index.html</t>
+        </is>
+      </c>
       <c r="R2076" t="inlineStr">
         <is>
           <t>live</t>
@@ -86698,6 +86888,11 @@
           <t>Editie Leiderschap</t>
         </is>
       </c>
+      <c r="I2077" t="inlineStr">
+        <is>
+          <t>editie-leiderschap/index.html</t>
+        </is>
+      </c>
       <c r="R2077" t="inlineStr">
         <is>
           <t>live</t>
@@ -86736,6 +86931,11 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
+      <c r="I2078" t="inlineStr">
+        <is>
+          <t>toekomst/energie/index.html</t>
+        </is>
+      </c>
       <c r="R2078" t="inlineStr">
         <is>
           <t>live</t>
@@ -86774,6 +86974,11 @@
           <t>Hoe de papier-industrie macht kreeg over het echte werk</t>
         </is>
       </c>
+      <c r="I2079" t="inlineStr">
+        <is>
+          <t>editie-4/index.html</t>
+        </is>
+      </c>
       <c r="R2079" t="inlineStr">
         <is>
           <t>live</t>
@@ -86812,6 +87017,11 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
+      <c r="I2080" t="inlineStr">
+        <is>
+          <t>toekomst/industrie/index.html</t>
+        </is>
+      </c>
       <c r="R2080" t="inlineStr">
         <is>
           <t>live</t>
@@ -86936,6 +87146,11 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
+      <c r="I2083" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/methode/index.html</t>
+        </is>
+      </c>
       <c r="R2083" t="inlineStr">
         <is>
           <t>live</t>
@@ -87103,6 +87318,11 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
+      <c r="I2087" t="inlineStr">
+        <is>
+          <t>editie-3/artikel-07-ai-onderwijs.html</t>
+        </is>
+      </c>
       <c r="R2087" t="inlineStr">
         <is>
           <t>live</t>
@@ -87141,6 +87361,11 @@
           <t>Opvoeding · Toekomst</t>
         </is>
       </c>
+      <c r="I2088" t="inlineStr">
+        <is>
+          <t>toekomst/opvoeding/index.html</t>
+        </is>
+      </c>
       <c r="R2088" t="inlineStr">
         <is>
           <t>live</t>
@@ -87222,6 +87447,11 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
+      <c r="I2090" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/index.html</t>
+        </is>
+      </c>
       <c r="R2090" t="inlineStr">
         <is>
           <t>live</t>
@@ -87260,6 +87490,11 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
+      <c r="I2091" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-00-redactie.html</t>
+        </is>
+      </c>
       <c r="R2091" t="inlineStr">
         <is>
           <t>live</t>
@@ -87298,6 +87533,11 @@
           <t>Retrospectief</t>
         </is>
       </c>
+      <c r="I2092" t="inlineStr">
+        <is>
+          <t>editie-4/artikel-09-retrospectief.html</t>
+        </is>
+      </c>
       <c r="R2092" t="inlineStr">
         <is>
           <t>live</t>
@@ -87336,6 +87576,11 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
+      <c r="I2093" t="inlineStr">
+        <is>
+          <t>toekomst/scholing/index.html</t>
+        </is>
+      </c>
       <c r="R2093" t="inlineStr">
         <is>
           <t>live</t>
@@ -87374,6 +87619,11 @@
           <t>Soevereiniteit als cyclus</t>
         </is>
       </c>
+      <c r="I2094" t="inlineStr">
+        <is>
+          <t>soevereiniteit-als-cyclus/index.html</t>
+        </is>
+      </c>
       <c r="R2094" t="inlineStr">
         <is>
           <t>live</t>
@@ -87455,6 +87705,11 @@
           <t>Toekomst</t>
         </is>
       </c>
+      <c r="I2096" t="inlineStr">
+        <is>
+          <t>toekomst/index.html</t>
+        </is>
+      </c>
       <c r="R2096" t="inlineStr">
         <is>
           <t>live</t>
@@ -87579,6 +87834,11 @@
           <t>Van leerfabriek naar leerwerkplaats</t>
         </is>
       </c>
+      <c r="I2099" t="inlineStr">
+        <is>
+          <t>editie-1/onderwijs.html</t>
+        </is>
+      </c>
       <c r="R2099" t="inlineStr">
         <is>
           <t>live</t>
@@ -87827,6 +88087,11 @@
           <t>De eerste gemeente</t>
         </is>
       </c>
+      <c r="I2105" t="inlineStr">
+        <is>
+          <t>de-eerste-gemeente/index.html</t>
+        </is>
+      </c>
       <c r="R2105" t="inlineStr">
         <is>
           <t>live</t>
@@ -87865,6 +88130,11 @@
           <t>De halve gemeente</t>
         </is>
       </c>
+      <c r="I2106" t="inlineStr">
+        <is>
+          <t>de-halve-gemeente/index.html</t>
+        </is>
+      </c>
       <c r="R2106" t="inlineStr">
         <is>
           <t>live</t>
@@ -88027,6 +88297,11 @@
           <t>Gevolgenkaart — Nederland</t>
         </is>
       </c>
+      <c r="I2110" t="inlineStr">
+        <is>
+          <t>gevolgenkaart-nl/index.html</t>
+        </is>
+      </c>
       <c r="R2110" t="inlineStr">
         <is>
           <t>live</t>
@@ -88146,6 +88421,11 @@
           <t>Nederland · Toekomst</t>
         </is>
       </c>
+      <c r="I2113" t="inlineStr">
+        <is>
+          <t>toekomst/overheden/nederland/index.html</t>
+        </is>
+      </c>
       <c r="R2113" t="inlineStr">
         <is>
           <t>live</t>
@@ -90536,6 +90816,11 @@
           <t>Wat er nu al ligt</t>
         </is>
       </c>
+      <c r="I2173" t="inlineStr">
+        <is>
+          <t>editie-1/technische-oplossingen.html</t>
+        </is>
+      </c>
       <c r="R2173" t="inlineStr">
         <is>
           <t>live</t>
@@ -90574,6 +90859,11 @@
           <t>七つ道具 — Zeven gereedschappen</t>
         </is>
       </c>
+      <c r="I2174" t="inlineStr">
+        <is>
+          <t>editie-5/artikel-01-zeven-gereedschappen.html</t>
+        </is>
+      </c>
       <c r="R2174" t="inlineStr">
         <is>
           <t>live</t>
@@ -91308,6 +91598,11 @@
           <t>Wie zijn opbouwers wegjaagt</t>
         </is>
       </c>
+      <c r="I2192" t="inlineStr">
+        <is>
+          <t>opbouwers-wegjagen/index.html</t>
+        </is>
+      </c>
       <c r="R2192" t="inlineStr">
         <is>
           <t>live</t>
@@ -91384,6 +91679,11 @@
           <t>Achter de Cijfers</t>
         </is>
       </c>
+      <c r="I2194" t="inlineStr">
+        <is>
+          <t>onderzoek/index.html</t>
+        </is>
+      </c>
       <c r="R2194" t="inlineStr">
         <is>
           <t>live</t>
@@ -91422,6 +91722,11 @@
           <t>Dossiers</t>
         </is>
       </c>
+      <c r="I2195" t="inlineStr">
+        <is>
+          <t>dossiers/index.html</t>
+        </is>
+      </c>
       <c r="R2195" t="inlineStr">
         <is>
           <t>live</t>
@@ -91460,6 +91765,11 @@
           <t>EU: BBP, Reële Lonen en de Overheidsmultiplicator</t>
         </is>
       </c>
+      <c r="I2196" t="inlineStr">
+        <is>
+          <t>onderzoek/eu-multiplicator.html</t>
+        </is>
+      </c>
       <c r="R2196" t="inlineStr">
         <is>
           <t>live</t>
@@ -91670,6 +91980,11 @@
           <t>Is Nederland op weg naar ontwikkelingslandstatus?</t>
         </is>
       </c>
+      <c r="I2201" t="inlineStr">
+        <is>
+          <t>onderzoek/ontwikkelingslandstatus.html</t>
+        </is>
+      </c>
       <c r="R2201" t="inlineStr">
         <is>
           <t>live</t>
@@ -91751,6 +92066,11 @@
           <t>Vortex-Hair™ Adaptive Dimple Golf Ball — Dossier</t>
         </is>
       </c>
+      <c r="I2203" t="inlineStr">
+        <is>
+          <t>dossiers/vortex-hair.html</t>
+        </is>
+      </c>
       <c r="R2203" t="inlineStr">
         <is>
           <t>live</t>
@@ -91827,6 +92147,11 @@
           <t>Archief</t>
         </is>
       </c>
+      <c r="I2205" t="inlineStr">
+        <is>
+          <t>archief.html</t>
+        </is>
+      </c>
       <c r="R2205" t="inlineStr">
         <is>
           <t>live</t>
@@ -91865,6 +92190,11 @@
           <t>Bedankt — controleer uw inbox</t>
         </is>
       </c>
+      <c r="I2206" t="inlineStr">
+        <is>
+          <t>bedankt.html</t>
+        </is>
+      </c>
       <c r="R2206" t="inlineStr">
         <is>
           <t>live</t>
@@ -91941,6 +92271,11 @@
           <t>Het Open Vizier verder dragen</t>
         </is>
       </c>
+      <c r="I2208" t="inlineStr">
+        <is>
+          <t>delen.html</t>
+        </is>
+      </c>
       <c r="R2208" t="inlineStr">
         <is>
           <t>live</t>
@@ -92017,6 +92352,11 @@
           <t>Hoe u meedoet aan de discussie</t>
         </is>
       </c>
+      <c r="I2210" t="inlineStr">
+        <is>
+          <t>editie-1/discussie.html</t>
+        </is>
+      </c>
       <c r="R2210" t="inlineStr">
         <is>
           <t>live</t>
@@ -92055,6 +92395,11 @@
           <t>Navigatie</t>
         </is>
       </c>
+      <c r="I2211" t="inlineStr">
+        <is>
+          <t>navigatie.html</t>
+        </is>
+      </c>
       <c r="R2211" t="inlineStr">
         <is>
           <t>live</t>
@@ -92093,6 +92438,11 @@
           <t>Op de hoogte blijven</t>
         </is>
       </c>
+      <c r="I2212" t="inlineStr">
+        <is>
+          <t>op-de-hoogte.html</t>
+        </is>
+      </c>
       <c r="R2212" t="inlineStr">
         <is>
           <t>live</t>
@@ -92131,6 +92481,11 @@
           <t>Over deze krant</t>
         </is>
       </c>
+      <c r="I2213" t="inlineStr">
+        <is>
+          <t>over.html</t>
+        </is>
+      </c>
       <c r="R2213" t="inlineStr">
         <is>
           <t>live</t>
@@ -92212,6 +92567,11 @@
           <t>Structuur — Beheer</t>
         </is>
       </c>
+      <c r="I2215" t="inlineStr">
+        <is>
+          <t>structuur.html</t>
+        </is>
+      </c>
       <c r="R2215" t="inlineStr">
         <is>
           <t>live</t>
@@ -92291,6 +92651,11 @@
       <c r="F2217" t="inlineStr">
         <is>
           <t>Waarom deze krant?</t>
+        </is>
+      </c>
+      <c r="I2217" t="inlineStr">
+        <is>
+          <t>editie-1/voorwoord.html</t>
         </is>
       </c>
       <c r="R2217" t="inlineStr">

</xml_diff>

<commit_message>
REVERT: xlsx terug naar staat vóór bulk-taal-updates (EN,DE,RU,FR,ES,IT,PT)
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -13107,11 +13107,6 @@
           <t>GCS — krantbriefing</t>
         </is>
       </c>
-      <c r="I289" t="inlineStr">
-        <is>
-          <t>forschung/krantbriefing.html</t>
-        </is>
-      </c>
       <c r="R289" t="inlineStr">
         <is>
           <t>live</t>
@@ -13188,11 +13183,6 @@
           <t>GCS — volledig plan</t>
         </is>
       </c>
-      <c r="I291" t="inlineStr">
-        <is>
-          <t>forschung/gevoelsconnectiesysteem-volledig.html</t>
-        </is>
-      </c>
       <c r="R291" t="inlineStr">
         <is>
           <t>live</t>
@@ -13231,11 +13221,6 @@
           <t>Het gevoelsconnectiesysteem</t>
         </is>
       </c>
-      <c r="I292" t="inlineStr">
-        <is>
-          <t>forschung/gevoelsconnectiesysteem.html</t>
-        </is>
-      </c>
       <c r="R292" t="inlineStr">
         <is>
           <t>live</t>
@@ -14590,11 +14575,6 @@
           <t>Tien seconden</t>
         </is>
       </c>
-      <c r="I325" t="inlineStr">
-        <is>
-          <t>idee.html</t>
-        </is>
-      </c>
       <c r="R325" t="inlineStr">
         <is>
           <t>live</t>
@@ -15473,11 +15453,6 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
-      <c r="I346" t="inlineStr">
-        <is>
-          <t>stemgedrag.html</t>
-        </is>
-      </c>
       <c r="R346" t="inlineStr">
         <is>
           <t>live</t>
@@ -16227,11 +16202,6 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
-      <c r="I364" t="inlineStr">
-        <is>
-          <t>editie-klimaat/index.html</t>
-        </is>
-      </c>
       <c r="R364" t="inlineStr">
         <is>
           <t>live</t>
@@ -17214,11 +17184,6 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
-      <c r="I388" t="inlineStr">
-        <is>
-          <t>ausgabe-0/carbon-alert-europa.html</t>
-        </is>
-      </c>
       <c r="R388" t="inlineStr">
         <is>
           <t>live</t>
@@ -18016,11 +17981,6 @@
           <t>Editie 2</t>
         </is>
       </c>
-      <c r="I407" t="inlineStr">
-        <is>
-          <t>ausgabe-2/index.html</t>
-        </is>
-      </c>
       <c r="R407" t="inlineStr">
         <is>
           <t>live</t>
@@ -18679,11 +18639,6 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
-      <c r="I423" t="inlineStr">
-        <is>
-          <t>ausgabe-4/artikel-00-redactie.html</t>
-        </is>
-      </c>
       <c r="R423" t="inlineStr">
         <is>
           <t>live</t>
@@ -24543,11 +24498,6 @@
           <t>GCS — krantbriefing</t>
         </is>
       </c>
-      <c r="I567" t="inlineStr">
-        <is>
-          <t>research/krantbriefing.html</t>
-        </is>
-      </c>
       <c r="R567" t="inlineStr">
         <is>
           <t>live</t>
@@ -24624,11 +24574,6 @@
           <t>GCS — volledig plan</t>
         </is>
       </c>
-      <c r="I569" t="inlineStr">
-        <is>
-          <t>research/gevoelsconnectiesysteem-volledig.html</t>
-        </is>
-      </c>
       <c r="R569" t="inlineStr">
         <is>
           <t>live</t>
@@ -24667,11 +24612,6 @@
           <t>Het gevoelsconnectiesysteem</t>
         </is>
       </c>
-      <c r="I570" t="inlineStr">
-        <is>
-          <t>research/gevoelsconnectiesysteem.html</t>
-        </is>
-      </c>
       <c r="R570" t="inlineStr">
         <is>
           <t>live</t>
@@ -24958,11 +24898,6 @@
           <t>De Kosaris — Boek Twee — Diakrisis</t>
         </is>
       </c>
-      <c r="I577" t="inlineStr">
-        <is>
-          <t>reading-book-two/index.html</t>
-        </is>
-      </c>
       <c r="R577" t="inlineStr">
         <is>
           <t>live</t>
@@ -25001,11 +24936,6 @@
           <t>De Kosaris — Boek Drie — Het boek van Anthea</t>
         </is>
       </c>
-      <c r="I578" t="inlineStr">
-        <is>
-          <t>reading-book-three/index.html</t>
-        </is>
-      </c>
       <c r="R578" t="inlineStr">
         <is>
           <t>live</t>
@@ -25044,11 +24974,6 @@
           <t>De Kosaris — Boek Vier — Het boek van het hydrolysaat</t>
         </is>
       </c>
-      <c r="I579" t="inlineStr">
-        <is>
-          <t>reading-book-four/index.html</t>
-        </is>
-      </c>
       <c r="R579" t="inlineStr">
         <is>
           <t>live</t>
@@ -25087,11 +25012,6 @@
           <t>De Kosaris — Boek Vijf — Het boek van de partner</t>
         </is>
       </c>
-      <c r="I580" t="inlineStr">
-        <is>
-          <t>reading-book-five/index.html</t>
-        </is>
-      </c>
       <c r="R580" t="inlineStr">
         <is>
           <t>live</t>
@@ -26046,11 +25966,6 @@
           <t>Tien seconden</t>
         </is>
       </c>
-      <c r="I603" t="inlineStr">
-        <is>
-          <t>idee.html</t>
-        </is>
-      </c>
       <c r="R603" t="inlineStr">
         <is>
           <t>live</t>
@@ -26929,11 +26844,6 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
-      <c r="I624" t="inlineStr">
-        <is>
-          <t>stemgedrag.html</t>
-        </is>
-      </c>
       <c r="R624" t="inlineStr">
         <is>
           <t>live</t>
@@ -27058,11 +26968,6 @@
           <t>Het politieke landschap</t>
         </is>
       </c>
-      <c r="I627" t="inlineStr">
-        <is>
-          <t>what-surfaces/plundering-4-politieke-landschap.html</t>
-        </is>
-      </c>
       <c r="R627" t="inlineStr">
         <is>
           <t>live</t>
@@ -27187,11 +27092,6 @@
           <t>Trump als spiegel</t>
         </is>
       </c>
-      <c r="I630" t="inlineStr">
-        <is>
-          <t>what-surfaces/trump-als-spiegel.html</t>
-        </is>
-      </c>
       <c r="R630" t="inlineStr">
         <is>
           <t>live</t>
@@ -27693,11 +27593,6 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
-      <c r="I642" t="inlineStr">
-        <is>
-          <t>climate-edition/index.html</t>
-        </is>
-      </c>
       <c r="R642" t="inlineStr">
         <is>
           <t>live</t>
@@ -28318,11 +28213,6 @@
           <t>De Brusselse Gevolgenkaart — BiCRS-versie</t>
         </is>
       </c>
-      <c r="I657" t="inlineStr">
-        <is>
-          <t>what-surfaces/brusselse-gevolgenkaart-bicrs.html</t>
-        </is>
-      </c>
       <c r="R657" t="inlineStr">
         <is>
           <t>live</t>
@@ -28404,11 +28294,6 @@
           <t>De op de natuur aangepaste analyse</t>
         </is>
       </c>
-      <c r="I659" t="inlineStr">
-        <is>
-          <t>what-surfaces/de-op-de-natuur-aangepaste-analyse.html</t>
-        </is>
-      </c>
       <c r="R659" t="inlineStr">
         <is>
           <t>live</t>
@@ -28490,11 +28375,6 @@
           <t>Editie Europa</t>
         </is>
       </c>
-      <c r="I661" t="inlineStr">
-        <is>
-          <t>edition-0/index.html</t>
-        </is>
-      </c>
       <c r="R661" t="inlineStr">
         <is>
           <t>live</t>
@@ -28533,11 +28413,6 @@
           <t>Mensen die mee bouwen</t>
         </is>
       </c>
-      <c r="I662" t="inlineStr">
-        <is>
-          <t>what-surfaces/mensen-die-mee-bouwen.html</t>
-        </is>
-      </c>
       <c r="R662" t="inlineStr">
         <is>
           <t>live</t>
@@ -28662,11 +28537,6 @@
           <t>Visie 2036</t>
         </is>
       </c>
-      <c r="I665" t="inlineStr">
-        <is>
-          <t>what-surfaces/carbon-alert-visie-2036.html</t>
-        </is>
-      </c>
       <c r="R665" t="inlineStr">
         <is>
           <t>live</t>
@@ -28705,11 +28575,6 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
-      <c r="I666" t="inlineStr">
-        <is>
-          <t>edition-0/carbon-alert-europa.html</t>
-        </is>
-      </c>
       <c r="R666" t="inlineStr">
         <is>
           <t>live</t>
@@ -28915,11 +28780,6 @@
           <t>De actor is de regel</t>
         </is>
       </c>
-      <c r="I671" t="inlineStr">
-        <is>
-          <t>what-surfaces/de-actor-is-de-regel.html</t>
-        </is>
-      </c>
       <c r="R671" t="inlineStr">
         <is>
           <t>live</t>
@@ -29512,11 +29372,6 @@
           <t>Editie 2</t>
         </is>
       </c>
-      <c r="I685" t="inlineStr">
-        <is>
-          <t>edition-2/index.html</t>
-        </is>
-      </c>
       <c r="R685" t="inlineStr">
         <is>
           <t>live</t>
@@ -29841,11 +29696,6 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
-      <c r="I693" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/methode/index.html</t>
-        </is>
-      </c>
       <c r="R693" t="inlineStr">
         <is>
           <t>live</t>
@@ -30142,11 +29992,6 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
-      <c r="I700" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/index.html</t>
-        </is>
-      </c>
       <c r="R700" t="inlineStr">
         <is>
           <t>live</t>
@@ -30185,11 +30030,6 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
-      <c r="I701" t="inlineStr">
-        <is>
-          <t>edition-4/artikel-00-redactie.html</t>
-        </is>
-      </c>
       <c r="R701" t="inlineStr">
         <is>
           <t>live</t>
@@ -31096,11 +30936,6 @@
           <t>Nederland · Toekomst</t>
         </is>
       </c>
-      <c r="I723" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/nederland/index.html</t>
-        </is>
-      </c>
       <c r="R723" t="inlineStr">
         <is>
           <t>live</t>
@@ -31139,11 +30974,6 @@
           <t>Stille Analyse</t>
         </is>
       </c>
-      <c r="I724" t="inlineStr">
-        <is>
-          <t>what-surfaces/gevolgenkaart-iii-stille-analyse.html</t>
-        </is>
-      </c>
       <c r="R724" t="inlineStr">
         <is>
           <t>live</t>
@@ -31430,11 +31260,6 @@
           <t>De Brusselse Gevolgenkaart — BiCRS-versie</t>
         </is>
       </c>
-      <c r="I731" t="inlineStr">
-        <is>
-          <t>what-surfaces/brusselse-gevolgenkaart-bicrs.html</t>
-        </is>
-      </c>
       <c r="R731" t="inlineStr">
         <is>
           <t>live</t>
@@ -31688,11 +31513,6 @@
           <t>Die Konsequenzkarte</t>
         </is>
       </c>
-      <c r="I737" t="inlineStr">
-        <is>
-          <t>what-surfaces/die-konsequenzkarte.html</t>
-        </is>
-      </c>
       <c r="R737" t="inlineStr">
         <is>
           <t>live</t>
@@ -31731,11 +31551,6 @@
           <t>Duitsland · Toekomst</t>
         </is>
       </c>
-      <c r="I738" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/duitsland/index.html</t>
-        </is>
-      </c>
       <c r="R738" t="inlineStr">
         <is>
           <t>live</t>
@@ -31903,11 +31718,6 @@
           <t>Europa · Toekomst</t>
         </is>
       </c>
-      <c r="I742" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/europa/index.html</t>
-        </is>
-      </c>
       <c r="R742" t="inlineStr">
         <is>
           <t>live</t>
@@ -38415,11 +38225,6 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
-      <c r="I902" t="inlineStr">
-        <is>
-          <t>stemgedrag.html</t>
-        </is>
-      </c>
       <c r="R902" t="inlineStr">
         <is>
           <t>live</t>
@@ -39116,11 +38921,6 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
-      <c r="I919" t="inlineStr">
-        <is>
-          <t>editie-stikstof/drie-problemen-een-antwoord.html</t>
-        </is>
-      </c>
       <c r="R919" t="inlineStr">
         <is>
           <t>live</t>
@@ -39159,11 +38959,6 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
-      <c r="I920" t="inlineStr">
-        <is>
-          <t>editie-klimaat/index.html</t>
-        </is>
-      </c>
       <c r="R920" t="inlineStr">
         <is>
           <t>live</t>
@@ -39202,11 +38997,6 @@
           <t>Editie Stikstof</t>
         </is>
       </c>
-      <c r="I921" t="inlineStr">
-        <is>
-          <t>editie-stikstof/index.html</t>
-        </is>
-      </c>
       <c r="R921" t="inlineStr">
         <is>
           <t>live</t>
@@ -39493,11 +39283,6 @@
           <t>De Koolzaad-Multiplicator</t>
         </is>
       </c>
-      <c r="I928" t="inlineStr">
-        <is>
-          <t>editie-duitsland/raps-multiplicator-oost-duitsland.html</t>
-        </is>
-      </c>
       <c r="R928" t="inlineStr">
         <is>
           <t>live</t>
@@ -39579,11 +39364,6 @@
           <t>Editie Duitsland</t>
         </is>
       </c>
-      <c r="I930" t="inlineStr">
-        <is>
-          <t>editie-duitsland/index.html</t>
-        </is>
-      </c>
       <c r="R930" t="inlineStr">
         <is>
           <t>live</t>
@@ -40981,11 +40761,6 @@
           <t>Editie Kind &amp; Loopbaan</t>
         </is>
       </c>
-      <c r="I964" t="inlineStr">
-        <is>
-          <t>editie-kind-loopbaan/index.html</t>
-        </is>
-      </c>
       <c r="R964" t="inlineStr">
         <is>
           <t>live</t>
@@ -41024,11 +40799,6 @@
           <t>Editie Leiderschap</t>
         </is>
       </c>
-      <c r="I965" t="inlineStr">
-        <is>
-          <t>editie-leiderschap/index.html</t>
-        </is>
-      </c>
       <c r="R965" t="inlineStr">
         <is>
           <t>live</t>
@@ -41067,11 +40837,6 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
-      <c r="I966" t="inlineStr">
-        <is>
-          <t>toekomst/energie/index.html</t>
-        </is>
-      </c>
       <c r="R966" t="inlineStr">
         <is>
           <t>live</t>
@@ -41153,11 +40918,6 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
-      <c r="I968" t="inlineStr">
-        <is>
-          <t>toekomst/industrie/index.html</t>
-        </is>
-      </c>
       <c r="R968" t="inlineStr">
         <is>
           <t>live</t>
@@ -41277,11 +41037,6 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
-      <c r="I971" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/methode/index.html</t>
-        </is>
-      </c>
       <c r="R971" t="inlineStr">
         <is>
           <t>live</t>
@@ -41492,11 +41247,6 @@
           <t>Opvoeding · Toekomst</t>
         </is>
       </c>
-      <c r="I976" t="inlineStr">
-        <is>
-          <t>toekomst/opvoeding/index.html</t>
-        </is>
-      </c>
       <c r="R976" t="inlineStr">
         <is>
           <t>live</t>
@@ -41578,11 +41328,6 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
-      <c r="I978" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/index.html</t>
-        </is>
-      </c>
       <c r="R978" t="inlineStr">
         <is>
           <t>live</t>
@@ -41702,11 +41447,6 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
-      <c r="I981" t="inlineStr">
-        <is>
-          <t>toekomst/scholing/index.html</t>
-        </is>
-      </c>
       <c r="R981" t="inlineStr">
         <is>
           <t>live</t>
@@ -41745,11 +41485,6 @@
           <t>Soevereiniteit als cyclus</t>
         </is>
       </c>
-      <c r="I982" t="inlineStr">
-        <is>
-          <t>soevereiniteit-als-cyclus/index.html</t>
-        </is>
-      </c>
       <c r="R982" t="inlineStr">
         <is>
           <t>live</t>
@@ -41826,11 +41561,6 @@
           <t>Toekomst</t>
         </is>
       </c>
-      <c r="I984" t="inlineStr">
-        <is>
-          <t>toekomst/index.html</t>
-        </is>
-      </c>
       <c r="R984" t="inlineStr">
         <is>
           <t>live</t>
@@ -42203,11 +41933,6 @@
           <t>De eerste gemeente</t>
         </is>
       </c>
-      <c r="I993" t="inlineStr">
-        <is>
-          <t>de-eerste-gemeente/index.html</t>
-        </is>
-      </c>
       <c r="R993" t="inlineStr">
         <is>
           <t>live</t>
@@ -47547,11 +47272,6 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
-      <c r="I1127" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-07-ai-onderwijs.html</t>
-        </is>
-      </c>
       <c r="R1127" t="inlineStr">
         <is>
           <t>live</t>
@@ -47671,11 +47391,6 @@
           <t>Alles stroomt — de moeder van alle wetenschap</t>
         </is>
       </c>
-      <c r="I1130" t="inlineStr">
-        <is>
-          <t>editie-1/stromingsleer.html</t>
-        </is>
-      </c>
       <c r="R1130" t="inlineStr">
         <is>
           <t>live</t>
@@ -47995,11 +47710,6 @@
           <t>Drie dimensies zijn te weinig</t>
         </is>
       </c>
-      <c r="I1138" t="inlineStr">
-        <is>
-          <t>editie-1/denkraam-7d.html</t>
-        </is>
-      </c>
       <c r="R1138" t="inlineStr">
         <is>
           <t>live</t>
@@ -48081,11 +47791,6 @@
           <t>Hoe alles samenhangt</t>
         </is>
       </c>
-      <c r="I1140" t="inlineStr">
-        <is>
-          <t>editie-1/samenhang.html</t>
-        </is>
-      </c>
       <c r="R1140" t="inlineStr">
         <is>
           <t>live</t>
@@ -48124,11 +47829,6 @@
           <t>Van de grot naar de zon</t>
         </is>
       </c>
-      <c r="I1141" t="inlineStr">
-        <is>
-          <t>wat-opkomt/van-de-grot-naar-de-zon.html</t>
-        </is>
-      </c>
       <c r="R1141" t="inlineStr">
         <is>
           <t>live</t>
@@ -48167,11 +47867,6 @@
           <t>Van quantumtheorie naar 7-dim</t>
         </is>
       </c>
-      <c r="I1142" t="inlineStr">
-        <is>
-          <t>wat-opkomt/van-quantum-naar-7d.html</t>
-        </is>
-      </c>
       <c r="R1142" t="inlineStr">
         <is>
           <t>live</t>
@@ -48329,11 +48024,6 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
-      <c r="I1146" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-04-bankier.html</t>
-        </is>
-      </c>
       <c r="R1146" t="inlineStr">
         <is>
           <t>live</t>
@@ -48372,11 +48062,6 @@
           <t>Communicatie tussen oergevoelens</t>
         </is>
       </c>
-      <c r="I1147" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-04-communicatie.html</t>
-        </is>
-      </c>
       <c r="R1147" t="inlineStr">
         <is>
           <t>live</t>
@@ -48415,11 +48100,6 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
-      <c r="I1148" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-02-ceo.html</t>
-        </is>
-      </c>
       <c r="R1148" t="inlineStr">
         <is>
           <t>live</t>
@@ -48458,11 +48138,6 @@
           <t>De drie hersenlagen</t>
         </is>
       </c>
-      <c r="I1149" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-03-drie-lagen.html</t>
-        </is>
-      </c>
       <c r="R1149" t="inlineStr">
         <is>
           <t>live</t>
@@ -48501,11 +48176,6 @@
           <t>De mens onder het ijs (Editie 3)</t>
         </is>
       </c>
-      <c r="I1150" t="inlineStr">
-        <is>
-          <t>editie-3/index.html</t>
-        </is>
-      </c>
       <c r="R1150" t="inlineStr">
         <is>
           <t>live</t>
@@ -48544,11 +48214,6 @@
           <t>De zeven dimensies</t>
         </is>
       </c>
-      <c r="I1151" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-02-zeven-dimensies.html</t>
-        </is>
-      </c>
       <c r="R1151" t="inlineStr">
         <is>
           <t>live</t>
@@ -48630,11 +48295,6 @@
           <t>Het oergevoel</t>
         </is>
       </c>
-      <c r="I1153" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-01-oergevoel.html</t>
-        </is>
-      </c>
       <c r="R1153" t="inlineStr">
         <is>
           <t>live</t>
@@ -48673,11 +48333,6 @@
           <t>Het oergevoel in de beroepspraktijk</t>
         </is>
       </c>
-      <c r="I1154" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-09-oergevoel-in-beroepspraktijk.html</t>
-        </is>
-      </c>
       <c r="R1154" t="inlineStr">
         <is>
           <t>live</t>
@@ -48716,11 +48371,6 @@
           <t>Mama ik heb honger</t>
         </is>
       </c>
-      <c r="I1155" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-06-mama.html</t>
-        </is>
-      </c>
       <c r="R1155" t="inlineStr">
         <is>
           <t>live</t>
@@ -48759,11 +48409,6 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
-      <c r="I1156" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-00-redactie.html</t>
-        </is>
-      </c>
       <c r="R1156" t="inlineStr">
         <is>
           <t>live</t>
@@ -48802,11 +48447,6 @@
           <t>Retrospectief</t>
         </is>
       </c>
-      <c r="I1157" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-08-retrospectief.html</t>
-        </is>
-      </c>
       <c r="R1157" t="inlineStr">
         <is>
           <t>live</t>
@@ -48845,11 +48485,6 @@
           <t>Ruimte voor het oergevoel</t>
         </is>
       </c>
-      <c r="I1158" t="inlineStr">
-        <is>
-          <t>wat-opkomt/manifest-ruimte-voor-het-oergevoel.html</t>
-        </is>
-      </c>
       <c r="R1158" t="inlineStr">
         <is>
           <t>live</t>
@@ -48888,11 +48523,6 @@
           <t>Tien seconden</t>
         </is>
       </c>
-      <c r="I1159" t="inlineStr">
-        <is>
-          <t>idee.html</t>
-        </is>
-      </c>
       <c r="R1159" t="inlineStr">
         <is>
           <t>live</t>
@@ -48974,11 +48604,6 @@
           <t>Wat we kinderen aandoen</t>
         </is>
       </c>
-      <c r="I1161" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-05-wat-we-doen.html</t>
-        </is>
-      </c>
       <c r="R1161" t="inlineStr">
         <is>
           <t>live</t>
@@ -49551,11 +49176,6 @@
           <t>De anti-immuunziekte van onze overheid slaat toe</t>
         </is>
       </c>
-      <c r="I1175" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-auto-immuunziekte-slaat-toe.html</t>
-        </is>
-      </c>
       <c r="R1175" t="inlineStr">
         <is>
           <t>live</t>
@@ -49637,11 +49257,6 @@
           <t>De matrix van de uittocht</t>
         </is>
       </c>
-      <c r="I1177" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-matrix-van-de-uittocht.html</t>
-        </is>
-      </c>
       <c r="R1177" t="inlineStr">
         <is>
           <t>live</t>
@@ -49766,11 +49381,6 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
-      <c r="I1180" t="inlineStr">
-        <is>
-          <t>stemgedrag.html</t>
-        </is>
-      </c>
       <c r="R1180" t="inlineStr">
         <is>
           <t>live</t>
@@ -49890,11 +49500,6 @@
           <t>Het politieke landschap</t>
         </is>
       </c>
-      <c r="I1183" t="inlineStr">
-        <is>
-          <t>wat-opkomt/plundering-4-politieke-landschap.html</t>
-        </is>
-      </c>
       <c r="R1183" t="inlineStr">
         <is>
           <t>live</t>
@@ -49933,11 +49538,6 @@
           <t>Moet Nederland ook volgen — laten wij onze industrie zakken?</t>
         </is>
       </c>
-      <c r="I1184" t="inlineStr">
-        <is>
-          <t>wat-opkomt/moet-nederland-ook-volgen.html</t>
-        </is>
-      </c>
       <c r="R1184" t="inlineStr">
         <is>
           <t>live</t>
@@ -49976,11 +49576,6 @@
           <t>Op de bok of op de bagagedrager</t>
         </is>
       </c>
-      <c r="I1185" t="inlineStr">
-        <is>
-          <t>wat-opkomt/aan-de-leiding-drie-blokken-zonder-subsidie.html</t>
-        </is>
-      </c>
       <c r="R1185" t="inlineStr">
         <is>
           <t>live</t>
@@ -50057,11 +49652,6 @@
           <t>Wat is er mis met partijpolitiek?</t>
         </is>
       </c>
-      <c r="I1187" t="inlineStr">
-        <is>
-          <t>editie-1/nova-democratia.html</t>
-        </is>
-      </c>
       <c r="R1187" t="inlineStr">
         <is>
           <t>live</t>
@@ -50100,11 +49690,6 @@
           <t>Ze weten het al. En ze doen het niet.</t>
         </is>
       </c>
-      <c r="I1188" t="inlineStr">
-        <is>
-          <t>wat-opkomt/ze-weten-het-al.html</t>
-        </is>
-      </c>
       <c r="R1188" t="inlineStr">
         <is>
           <t>live</t>
@@ -50224,11 +49809,6 @@
           <t>De anti-immuunziekte van onze overheid slaat toe</t>
         </is>
       </c>
-      <c r="I1191" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-auto-immuunziekte-slaat-toe.html</t>
-        </is>
-      </c>
       <c r="R1191" t="inlineStr">
         <is>
           <t>live</t>
@@ -50267,11 +49847,6 @@
           <t>De autoband is het nieuwe sigaret</t>
         </is>
       </c>
-      <c r="I1192" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-autoband-is-het-nieuwe-sigaret.html</t>
-        </is>
-      </c>
       <c r="R1192" t="inlineStr">
         <is>
           <t>live</t>
@@ -50310,11 +49885,6 @@
           <t>De boer én de natuur beide vooruit</t>
         </is>
       </c>
-      <c r="I1193" t="inlineStr">
-        <is>
-          <t>wat-opkomt/boer-en-natuur-beide-vooruit.html</t>
-        </is>
-      </c>
       <c r="R1193" t="inlineStr">
         <is>
           <t>live</t>
@@ -50353,11 +49923,6 @@
           <t>De methaan-misleiding</t>
         </is>
       </c>
-      <c r="I1194" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-04-methaan-misleiding.html</t>
-        </is>
-      </c>
       <c r="R1194" t="inlineStr">
         <is>
           <t>live</t>
@@ -50396,11 +49961,6 @@
           <t>De voedingslijn</t>
         </is>
       </c>
-      <c r="I1195" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-methodologie-van-de-aanpassing.html</t>
-        </is>
-      </c>
       <c r="R1195" t="inlineStr">
         <is>
           <t>live</t>
@@ -50482,11 +50042,6 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
-      <c r="I1197" t="inlineStr">
-        <is>
-          <t>editie-stikstof/drie-problemen-een-antwoord.html</t>
-        </is>
-      </c>
       <c r="R1197" t="inlineStr">
         <is>
           <t>live</t>
@@ -50525,11 +50080,6 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
-      <c r="I1198" t="inlineStr">
-        <is>
-          <t>editie-klimaat/index.html</t>
-        </is>
-      </c>
       <c r="R1198" t="inlineStr">
         <is>
           <t>live</t>
@@ -50568,11 +50118,6 @@
           <t>Editie Stikstof</t>
         </is>
       </c>
-      <c r="I1199" t="inlineStr">
-        <is>
-          <t>editie-stikstof/index.html</t>
-        </is>
-      </c>
       <c r="R1199" t="inlineStr">
         <is>
           <t>live</t>
@@ -50611,11 +50156,6 @@
           <t>Erfenisgolf — 240 miljard</t>
         </is>
       </c>
-      <c r="I1200" t="inlineStr">
-        <is>
-          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
-        </is>
-      </c>
       <c r="R1200" t="inlineStr">
         <is>
           <t>live</t>
@@ -50692,11 +50232,6 @@
           <t>Laat de politici eerst naar de natuurschool</t>
         </is>
       </c>
-      <c r="I1202" t="inlineStr">
-        <is>
-          <t>wat-opkomt/naar-de-natuurschool.html</t>
-        </is>
-      </c>
       <c r="R1202" t="inlineStr">
         <is>
           <t>live</t>
@@ -50778,11 +50313,6 @@
           <t>Ze weten het al. En ze doen het niet.</t>
         </is>
       </c>
-      <c r="I1204" t="inlineStr">
-        <is>
-          <t>wat-opkomt/ze-weten-het-al.html</t>
-        </is>
-      </c>
       <c r="R1204" t="inlineStr">
         <is>
           <t>live</t>
@@ -50859,11 +50389,6 @@
           <t>De Koolzaad-Multiplicator</t>
         </is>
       </c>
-      <c r="I1206" t="inlineStr">
-        <is>
-          <t>editie-duitsland/raps-multiplicator-oost-duitsland.html</t>
-        </is>
-      </c>
       <c r="R1206" t="inlineStr">
         <is>
           <t>live</t>
@@ -50902,11 +50427,6 @@
           <t>De plant die verhuist</t>
         </is>
       </c>
-      <c r="I1207" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-05-plant-die-verhuist.html</t>
-        </is>
-      </c>
       <c r="R1207" t="inlineStr">
         <is>
           <t>live</t>
@@ -50945,11 +50465,6 @@
           <t>Editie Duitsland</t>
         </is>
       </c>
-      <c r="I1208" t="inlineStr">
-        <is>
-          <t>editie-duitsland/index.html</t>
-        </is>
-      </c>
       <c r="R1208" t="inlineStr">
         <is>
           <t>live</t>
@@ -50988,11 +50503,6 @@
           <t>Een Ferrari die naar gemaaid gras ruikt</t>
         </is>
       </c>
-      <c r="I1209" t="inlineStr">
-        <is>
-          <t>wat-opkomt/het-dagelijks-idee-ferrari-juncao.html</t>
-        </is>
-      </c>
       <c r="R1209" t="inlineStr">
         <is>
           <t>live</t>
@@ -51069,11 +50579,6 @@
           <t>Actievoerders bouwen continenten</t>
         </is>
       </c>
-      <c r="I1211" t="inlineStr">
-        <is>
-          <t>wat-opkomt/actievoerders-bouwen-continenten.html</t>
-        </is>
-      </c>
       <c r="R1211" t="inlineStr">
         <is>
           <t>live</t>
@@ -51112,11 +50617,6 @@
           <t>De biomimetische krachtcentrale</t>
         </is>
       </c>
-      <c r="I1212" t="inlineStr">
-        <is>
-          <t>editie-0/biomimetische-krachtcentrale.html</t>
-        </is>
-      </c>
       <c r="R1212" t="inlineStr">
         <is>
           <t>live</t>
@@ -51193,11 +50693,6 @@
           <t>De dertig cent die Europa omdraait</t>
         </is>
       </c>
-      <c r="I1214" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-dertig-cent-die-europa-omdraait.html</t>
-        </is>
-      </c>
       <c r="R1214" t="inlineStr">
         <is>
           <t>live</t>
@@ -51274,11 +50769,6 @@
           <t>De plastic-boete die een carbon-credit had moeten zijn</t>
         </is>
       </c>
-      <c r="I1216" t="inlineStr">
-        <is>
-          <t>wat-opkomt/plastic-boete-carbon-credit.html</t>
-        </is>
-      </c>
       <c r="R1216" t="inlineStr">
         <is>
           <t>live</t>
@@ -51317,11 +50807,6 @@
           <t>Editie Europa</t>
         </is>
       </c>
-      <c r="I1217" t="inlineStr">
-        <is>
-          <t>editie-0/index.html</t>
-        </is>
-      </c>
       <c r="R1217" t="inlineStr">
         <is>
           <t>live</t>
@@ -51360,11 +50845,6 @@
           <t>Mensen die mee bouwen</t>
         </is>
       </c>
-      <c r="I1218" t="inlineStr">
-        <is>
-          <t>wat-opkomt/mensen-die-mee-bouwen.html</t>
-        </is>
-      </c>
       <c r="R1218" t="inlineStr">
         <is>
           <t>live</t>
@@ -51403,11 +50883,6 @@
           <t>Op de bok of op de bagagedrager</t>
         </is>
       </c>
-      <c r="I1219" t="inlineStr">
-        <is>
-          <t>wat-opkomt/aan-de-leiding-drie-blokken-zonder-subsidie.html</t>
-        </is>
-      </c>
       <c r="R1219" t="inlineStr">
         <is>
           <t>live</t>
@@ -51489,11 +50964,6 @@
           <t>Visie 2036</t>
         </is>
       </c>
-      <c r="I1221" t="inlineStr">
-        <is>
-          <t>wat-opkomt/carbon-alert-visie-2036.html</t>
-        </is>
-      </c>
       <c r="R1221" t="inlineStr">
         <is>
           <t>live</t>
@@ -51532,11 +51002,6 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
-      <c r="I1222" t="inlineStr">
-        <is>
-          <t>editie-0/carbon-alert-europa.html</t>
-        </is>
-      </c>
       <c r="R1222" t="inlineStr">
         <is>
           <t>live</t>
@@ -51613,11 +51078,6 @@
           <t>Beslissen zonder uitzicht</t>
         </is>
       </c>
-      <c r="I1224" t="inlineStr">
-        <is>
-          <t>wat-opkomt/bbp-liegt.html</t>
-        </is>
-      </c>
       <c r="R1224" t="inlineStr">
         <is>
           <t>live</t>
@@ -51656,11 +51116,6 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
-      <c r="I1225" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-04-bankier.html</t>
-        </is>
-      </c>
       <c r="R1225" t="inlineStr">
         <is>
           <t>live</t>
@@ -51742,11 +51197,6 @@
           <t>De actor is de regel</t>
         </is>
       </c>
-      <c r="I1227" t="inlineStr">
-        <is>
-          <t>wat-opkomt/de-actor-is-de-regel.html</t>
-        </is>
-      </c>
       <c r="R1227" t="inlineStr">
         <is>
           <t>live</t>
@@ -51871,11 +51321,6 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
-      <c r="I1230" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-02-ceo.html</t>
-        </is>
-      </c>
       <c r="R1230" t="inlineStr">
         <is>
           <t>live</t>
@@ -51914,11 +51359,6 @@
           <t>De consultant bij het bijna-failliete bedrijf</t>
         </is>
       </c>
-      <c r="I1231" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-03-consultant.html</t>
-        </is>
-      </c>
       <c r="R1231" t="inlineStr">
         <is>
           <t>live</t>
@@ -51957,11 +51397,6 @@
           <t>De diepere vraag</t>
         </is>
       </c>
-      <c r="I1232" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-08-diepere-vraag.html</t>
-        </is>
-      </c>
       <c r="R1232" t="inlineStr">
         <is>
           <t>live</t>
@@ -52086,11 +51521,6 @@
           <t>De rechter zonder kompas</t>
         </is>
       </c>
-      <c r="I1235" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-07-rechter.html</t>
-        </is>
-      </c>
       <c r="R1235" t="inlineStr">
         <is>
           <t>live</t>
@@ -52129,11 +51559,6 @@
           <t>De toezichthouder die niets ziet</t>
         </is>
       </c>
-      <c r="I1236" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-06-toezichthouder.html</t>
-        </is>
-      </c>
       <c r="R1236" t="inlineStr">
         <is>
           <t>live</t>
@@ -52172,11 +51597,6 @@
           <t>De verzekeraar tegen het leven</t>
         </is>
       </c>
-      <c r="I1237" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-05-verzekeraar.html</t>
-        </is>
-      </c>
       <c r="R1237" t="inlineStr">
         <is>
           <t>live</t>
@@ -52215,11 +51635,6 @@
           <t>De wet van de papier-industrie</t>
         </is>
       </c>
-      <c r="I1238" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-01-wet-papier-industrie.html</t>
-        </is>
-      </c>
       <c r="R1238" t="inlineStr">
         <is>
           <t>live</t>
@@ -52382,11 +51797,6 @@
           <t>Editie Kind &amp; Loopbaan</t>
         </is>
       </c>
-      <c r="I1242" t="inlineStr">
-        <is>
-          <t>editie-kind-loopbaan/index.html</t>
-        </is>
-      </c>
       <c r="R1242" t="inlineStr">
         <is>
           <t>live</t>
@@ -52425,11 +51835,6 @@
           <t>Editie Leiderschap</t>
         </is>
       </c>
-      <c r="I1243" t="inlineStr">
-        <is>
-          <t>editie-leiderschap/index.html</t>
-        </is>
-      </c>
       <c r="R1243" t="inlineStr">
         <is>
           <t>live</t>
@@ -52468,11 +51873,6 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
-      <c r="I1244" t="inlineStr">
-        <is>
-          <t>toekomst/energie/index.html</t>
-        </is>
-      </c>
       <c r="R1244" t="inlineStr">
         <is>
           <t>live</t>
@@ -52511,11 +51911,6 @@
           <t>Hoe de papier-industrie macht kreeg over het echte werk</t>
         </is>
       </c>
-      <c r="I1245" t="inlineStr">
-        <is>
-          <t>editie-4/index.html</t>
-        </is>
-      </c>
       <c r="R1245" t="inlineStr">
         <is>
           <t>live</t>
@@ -52554,11 +51949,6 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
-      <c r="I1246" t="inlineStr">
-        <is>
-          <t>toekomst/industrie/index.html</t>
-        </is>
-      </c>
       <c r="R1246" t="inlineStr">
         <is>
           <t>live</t>
@@ -52683,11 +52073,6 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
-      <c r="I1249" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/methode/index.html</t>
-        </is>
-      </c>
       <c r="R1249" t="inlineStr">
         <is>
           <t>live</t>
@@ -52855,11 +52240,6 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
-      <c r="I1253" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-07-ai-onderwijs.html</t>
-        </is>
-      </c>
       <c r="R1253" t="inlineStr">
         <is>
           <t>live</t>
@@ -52898,11 +52278,6 @@
           <t>Opvoeding · Toekomst</t>
         </is>
       </c>
-      <c r="I1254" t="inlineStr">
-        <is>
-          <t>toekomst/opvoeding/index.html</t>
-        </is>
-      </c>
       <c r="R1254" t="inlineStr">
         <is>
           <t>live</t>
@@ -52984,11 +52359,6 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
-      <c r="I1256" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/index.html</t>
-        </is>
-      </c>
       <c r="R1256" t="inlineStr">
         <is>
           <t>live</t>
@@ -53027,11 +52397,6 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
-      <c r="I1257" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-00-redactie.html</t>
-        </is>
-      </c>
       <c r="R1257" t="inlineStr">
         <is>
           <t>live</t>
@@ -53070,11 +52435,6 @@
           <t>Retrospectief</t>
         </is>
       </c>
-      <c r="I1258" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-09-retrospectief.html</t>
-        </is>
-      </c>
       <c r="R1258" t="inlineStr">
         <is>
           <t>live</t>
@@ -53113,11 +52473,6 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
-      <c r="I1259" t="inlineStr">
-        <is>
-          <t>toekomst/scholing/index.html</t>
-        </is>
-      </c>
       <c r="R1259" t="inlineStr">
         <is>
           <t>live</t>
@@ -53156,11 +52511,6 @@
           <t>Soevereiniteit als cyclus</t>
         </is>
       </c>
-      <c r="I1260" t="inlineStr">
-        <is>
-          <t>soevereiniteit-als-cyclus/index.html</t>
-        </is>
-      </c>
       <c r="R1260" t="inlineStr">
         <is>
           <t>live</t>
@@ -53242,11 +52592,6 @@
           <t>Toekomst</t>
         </is>
       </c>
-      <c r="I1262" t="inlineStr">
-        <is>
-          <t>toekomst/index.html</t>
-        </is>
-      </c>
       <c r="R1262" t="inlineStr">
         <is>
           <t>live</t>
@@ -53371,11 +52716,6 @@
           <t>Van leerfabriek naar leerwerkplaats</t>
         </is>
       </c>
-      <c r="I1265" t="inlineStr">
-        <is>
-          <t>editie-1/onderwijs.html</t>
-        </is>
-      </c>
       <c r="R1265" t="inlineStr">
         <is>
           <t>live</t>
@@ -53624,11 +52964,6 @@
           <t>De eerste gemeente</t>
         </is>
       </c>
-      <c r="I1271" t="inlineStr">
-        <is>
-          <t>de-eerste-gemeente/index.html</t>
-        </is>
-      </c>
       <c r="R1271" t="inlineStr">
         <is>
           <t>live</t>
@@ -53667,11 +53002,6 @@
           <t>De halve gemeente</t>
         </is>
       </c>
-      <c r="I1272" t="inlineStr">
-        <is>
-          <t>de-halve-gemeente/index.html</t>
-        </is>
-      </c>
       <c r="R1272" t="inlineStr">
         <is>
           <t>live</t>
@@ -58883,11 +58213,6 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
-      <c r="I1405" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-07-ai-onderwijs.html</t>
-        </is>
-      </c>
       <c r="R1405" t="inlineStr">
         <is>
           <t>live</t>
@@ -59007,11 +58332,6 @@
           <t>Alles stroomt — de moeder van alle wetenschap</t>
         </is>
       </c>
-      <c r="I1408" t="inlineStr">
-        <is>
-          <t>editie-1/stromingsleer.html</t>
-        </is>
-      </c>
       <c r="R1408" t="inlineStr">
         <is>
           <t>live</t>
@@ -59331,11 +58651,6 @@
           <t>Drie dimensies zijn te weinig</t>
         </is>
       </c>
-      <c r="I1416" t="inlineStr">
-        <is>
-          <t>editie-1/denkraam-7d.html</t>
-        </is>
-      </c>
       <c r="R1416" t="inlineStr">
         <is>
           <t>live</t>
@@ -59417,11 +58732,6 @@
           <t>Hoe alles samenhangt</t>
         </is>
       </c>
-      <c r="I1418" t="inlineStr">
-        <is>
-          <t>editie-1/samenhang.html</t>
-        </is>
-      </c>
       <c r="R1418" t="inlineStr">
         <is>
           <t>live</t>
@@ -59665,11 +58975,6 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
-      <c r="I1424" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-04-bankier.html</t>
-        </is>
-      </c>
       <c r="R1424" t="inlineStr">
         <is>
           <t>live</t>
@@ -59708,11 +59013,6 @@
           <t>Communicatie tussen oergevoelens</t>
         </is>
       </c>
-      <c r="I1425" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-04-communicatie.html</t>
-        </is>
-      </c>
       <c r="R1425" t="inlineStr">
         <is>
           <t>live</t>
@@ -59751,11 +59051,6 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
-      <c r="I1426" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-02-ceo.html</t>
-        </is>
-      </c>
       <c r="R1426" t="inlineStr">
         <is>
           <t>live</t>
@@ -59794,11 +59089,6 @@
           <t>De drie hersenlagen</t>
         </is>
       </c>
-      <c r="I1427" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-03-drie-lagen.html</t>
-        </is>
-      </c>
       <c r="R1427" t="inlineStr">
         <is>
           <t>live</t>
@@ -59837,11 +59127,6 @@
           <t>De mens onder het ijs (Editie 3)</t>
         </is>
       </c>
-      <c r="I1428" t="inlineStr">
-        <is>
-          <t>editie-3/index.html</t>
-        </is>
-      </c>
       <c r="R1428" t="inlineStr">
         <is>
           <t>live</t>
@@ -59880,11 +59165,6 @@
           <t>De zeven dimensies</t>
         </is>
       </c>
-      <c r="I1429" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-02-zeven-dimensies.html</t>
-        </is>
-      </c>
       <c r="R1429" t="inlineStr">
         <is>
           <t>live</t>
@@ -59966,11 +59246,6 @@
           <t>Het oergevoel</t>
         </is>
       </c>
-      <c r="I1431" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-01-oergevoel.html</t>
-        </is>
-      </c>
       <c r="R1431" t="inlineStr">
         <is>
           <t>live</t>
@@ -60009,11 +59284,6 @@
           <t>Het oergevoel in de beroepspraktijk</t>
         </is>
       </c>
-      <c r="I1432" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-09-oergevoel-in-beroepspraktijk.html</t>
-        </is>
-      </c>
       <c r="R1432" t="inlineStr">
         <is>
           <t>live</t>
@@ -60052,11 +59322,6 @@
           <t>Mama ik heb honger</t>
         </is>
       </c>
-      <c r="I1433" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-06-mama.html</t>
-        </is>
-      </c>
       <c r="R1433" t="inlineStr">
         <is>
           <t>live</t>
@@ -60095,11 +59360,6 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
-      <c r="I1434" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-00-redactie.html</t>
-        </is>
-      </c>
       <c r="R1434" t="inlineStr">
         <is>
           <t>live</t>
@@ -60138,11 +59398,6 @@
           <t>Retrospectief</t>
         </is>
       </c>
-      <c r="I1435" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-08-retrospectief.html</t>
-        </is>
-      </c>
       <c r="R1435" t="inlineStr">
         <is>
           <t>live</t>
@@ -60224,11 +59479,6 @@
           <t>Tien seconden</t>
         </is>
       </c>
-      <c r="I1437" t="inlineStr">
-        <is>
-          <t>idee.html</t>
-        </is>
-      </c>
       <c r="R1437" t="inlineStr">
         <is>
           <t>live</t>
@@ -60310,11 +59560,6 @@
           <t>Wat we kinderen aandoen</t>
         </is>
       </c>
-      <c r="I1439" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-05-wat-we-doen.html</t>
-        </is>
-      </c>
       <c r="R1439" t="inlineStr">
         <is>
           <t>live</t>
@@ -61102,11 +60347,6 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
-      <c r="I1458" t="inlineStr">
-        <is>
-          <t>stemgedrag.html</t>
-        </is>
-      </c>
       <c r="R1458" t="inlineStr">
         <is>
           <t>live</t>
@@ -61388,11 +60628,6 @@
           <t>Wat is er mis met partijpolitiek?</t>
         </is>
       </c>
-      <c r="I1465" t="inlineStr">
-        <is>
-          <t>editie-1/nova-democratia.html</t>
-        </is>
-      </c>
       <c r="R1465" t="inlineStr">
         <is>
           <t>live</t>
@@ -61684,11 +60919,6 @@
           <t>De methaan-misleiding</t>
         </is>
       </c>
-      <c r="I1472" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-04-methaan-misleiding.html</t>
-        </is>
-      </c>
       <c r="R1472" t="inlineStr">
         <is>
           <t>live</t>
@@ -61813,11 +61043,6 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
-      <c r="I1475" t="inlineStr">
-        <is>
-          <t>editie-stikstof/drie-problemen-een-antwoord.html</t>
-        </is>
-      </c>
       <c r="R1475" t="inlineStr">
         <is>
           <t>live</t>
@@ -61856,11 +61081,6 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
-      <c r="I1476" t="inlineStr">
-        <is>
-          <t>editie-klimaat/index.html</t>
-        </is>
-      </c>
       <c r="R1476" t="inlineStr">
         <is>
           <t>live</t>
@@ -61899,11 +61119,6 @@
           <t>Editie Stikstof</t>
         </is>
       </c>
-      <c r="I1477" t="inlineStr">
-        <is>
-          <t>editie-stikstof/index.html</t>
-        </is>
-      </c>
       <c r="R1477" t="inlineStr">
         <is>
           <t>live</t>
@@ -62195,11 +61410,6 @@
           <t>De Koolzaad-Multiplicator</t>
         </is>
       </c>
-      <c r="I1484" t="inlineStr">
-        <is>
-          <t>editie-duitsland/raps-multiplicator-oost-duitsland.html</t>
-        </is>
-      </c>
       <c r="R1484" t="inlineStr">
         <is>
           <t>live</t>
@@ -62238,11 +61448,6 @@
           <t>De plant die verhuist</t>
         </is>
       </c>
-      <c r="I1485" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-05-plant-die-verhuist.html</t>
-        </is>
-      </c>
       <c r="R1485" t="inlineStr">
         <is>
           <t>live</t>
@@ -62281,11 +61486,6 @@
           <t>Editie Duitsland</t>
         </is>
       </c>
-      <c r="I1486" t="inlineStr">
-        <is>
-          <t>editie-duitsland/index.html</t>
-        </is>
-      </c>
       <c r="R1486" t="inlineStr">
         <is>
           <t>live</t>
@@ -62448,11 +61648,6 @@
           <t>De biomimetische krachtcentrale</t>
         </is>
       </c>
-      <c r="I1490" t="inlineStr">
-        <is>
-          <t>editie-0/biomimetische-krachtcentrale.html</t>
-        </is>
-      </c>
       <c r="R1490" t="inlineStr">
         <is>
           <t>live</t>
@@ -62653,11 +61848,6 @@
           <t>Editie Europa</t>
         </is>
       </c>
-      <c r="I1495" t="inlineStr">
-        <is>
-          <t>editie-0/index.html</t>
-        </is>
-      </c>
       <c r="R1495" t="inlineStr">
         <is>
           <t>live</t>
@@ -62858,11 +62048,6 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
-      <c r="I1500" t="inlineStr">
-        <is>
-          <t>editie-0/carbon-alert-europa.html</t>
-        </is>
-      </c>
       <c r="R1500" t="inlineStr">
         <is>
           <t>live</t>
@@ -62982,11 +62167,6 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
-      <c r="I1503" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-04-bankier.html</t>
-        </is>
-      </c>
       <c r="R1503" t="inlineStr">
         <is>
           <t>live</t>
@@ -63197,11 +62377,6 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
-      <c r="I1508" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-02-ceo.html</t>
-        </is>
-      </c>
       <c r="R1508" t="inlineStr">
         <is>
           <t>live</t>
@@ -63240,11 +62415,6 @@
           <t>De consultant bij het bijna-failliete bedrijf</t>
         </is>
       </c>
-      <c r="I1509" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-03-consultant.html</t>
-        </is>
-      </c>
       <c r="R1509" t="inlineStr">
         <is>
           <t>live</t>
@@ -63283,11 +62453,6 @@
           <t>De diepere vraag</t>
         </is>
       </c>
-      <c r="I1510" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-08-diepere-vraag.html</t>
-        </is>
-      </c>
       <c r="R1510" t="inlineStr">
         <is>
           <t>live</t>
@@ -63412,11 +62577,6 @@
           <t>De rechter zonder kompas</t>
         </is>
       </c>
-      <c r="I1513" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-07-rechter.html</t>
-        </is>
-      </c>
       <c r="R1513" t="inlineStr">
         <is>
           <t>live</t>
@@ -63455,11 +62615,6 @@
           <t>De toezichthouder die niets ziet</t>
         </is>
       </c>
-      <c r="I1514" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-06-toezichthouder.html</t>
-        </is>
-      </c>
       <c r="R1514" t="inlineStr">
         <is>
           <t>live</t>
@@ -63498,11 +62653,6 @@
           <t>De verzekeraar tegen het leven</t>
         </is>
       </c>
-      <c r="I1515" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-05-verzekeraar.html</t>
-        </is>
-      </c>
       <c r="R1515" t="inlineStr">
         <is>
           <t>live</t>
@@ -63541,11 +62691,6 @@
           <t>De wet van de papier-industrie</t>
         </is>
       </c>
-      <c r="I1516" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-01-wet-papier-industrie.html</t>
-        </is>
-      </c>
       <c r="R1516" t="inlineStr">
         <is>
           <t>live</t>
@@ -63708,11 +62853,6 @@
           <t>Editie Kind &amp; Loopbaan</t>
         </is>
       </c>
-      <c r="I1520" t="inlineStr">
-        <is>
-          <t>editie-kind-loopbaan/index.html</t>
-        </is>
-      </c>
       <c r="R1520" t="inlineStr">
         <is>
           <t>live</t>
@@ -63751,11 +62891,6 @@
           <t>Editie Leiderschap</t>
         </is>
       </c>
-      <c r="I1521" t="inlineStr">
-        <is>
-          <t>editie-leiderschap/index.html</t>
-        </is>
-      </c>
       <c r="R1521" t="inlineStr">
         <is>
           <t>live</t>
@@ -63794,11 +62929,6 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
-      <c r="I1522" t="inlineStr">
-        <is>
-          <t>toekomst/energie/index.html</t>
-        </is>
-      </c>
       <c r="R1522" t="inlineStr">
         <is>
           <t>live</t>
@@ -63837,11 +62967,6 @@
           <t>Hoe de papier-industrie macht kreeg over het echte werk</t>
         </is>
       </c>
-      <c r="I1523" t="inlineStr">
-        <is>
-          <t>editie-4/index.html</t>
-        </is>
-      </c>
       <c r="R1523" t="inlineStr">
         <is>
           <t>live</t>
@@ -63880,11 +63005,6 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
-      <c r="I1524" t="inlineStr">
-        <is>
-          <t>toekomst/industrie/index.html</t>
-        </is>
-      </c>
       <c r="R1524" t="inlineStr">
         <is>
           <t>live</t>
@@ -64009,11 +63129,6 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
-      <c r="I1527" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/methode/index.html</t>
-        </is>
-      </c>
       <c r="R1527" t="inlineStr">
         <is>
           <t>live</t>
@@ -64181,11 +63296,6 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
-      <c r="I1531" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-07-ai-onderwijs.html</t>
-        </is>
-      </c>
       <c r="R1531" t="inlineStr">
         <is>
           <t>live</t>
@@ -64224,11 +63334,6 @@
           <t>Opvoeding · Toekomst</t>
         </is>
       </c>
-      <c r="I1532" t="inlineStr">
-        <is>
-          <t>toekomst/opvoeding/index.html</t>
-        </is>
-      </c>
       <c r="R1532" t="inlineStr">
         <is>
           <t>live</t>
@@ -64310,11 +63415,6 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
-      <c r="I1534" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/index.html</t>
-        </is>
-      </c>
       <c r="R1534" t="inlineStr">
         <is>
           <t>live</t>
@@ -64353,11 +63453,6 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
-      <c r="I1535" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-00-redactie.html</t>
-        </is>
-      </c>
       <c r="R1535" t="inlineStr">
         <is>
           <t>live</t>
@@ -64396,11 +63491,6 @@
           <t>Retrospectief</t>
         </is>
       </c>
-      <c r="I1536" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-09-retrospectief.html</t>
-        </is>
-      </c>
       <c r="R1536" t="inlineStr">
         <is>
           <t>live</t>
@@ -64439,11 +63529,6 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
-      <c r="I1537" t="inlineStr">
-        <is>
-          <t>toekomst/scholing/index.html</t>
-        </is>
-      </c>
       <c r="R1537" t="inlineStr">
         <is>
           <t>live</t>
@@ -64482,11 +63567,6 @@
           <t>Soevereiniteit als cyclus</t>
         </is>
       </c>
-      <c r="I1538" t="inlineStr">
-        <is>
-          <t>soevereiniteit-als-cyclus/index.html</t>
-        </is>
-      </c>
       <c r="R1538" t="inlineStr">
         <is>
           <t>live</t>
@@ -64568,11 +63648,6 @@
           <t>Toekomst</t>
         </is>
       </c>
-      <c r="I1540" t="inlineStr">
-        <is>
-          <t>toekomst/index.html</t>
-        </is>
-      </c>
       <c r="R1540" t="inlineStr">
         <is>
           <t>live</t>
@@ -64697,11 +63772,6 @@
           <t>Van leerfabriek naar leerwerkplaats</t>
         </is>
       </c>
-      <c r="I1543" t="inlineStr">
-        <is>
-          <t>editie-1/onderwijs.html</t>
-        </is>
-      </c>
       <c r="R1543" t="inlineStr">
         <is>
           <t>live</t>
@@ -64950,11 +64020,6 @@
           <t>De eerste gemeente</t>
         </is>
       </c>
-      <c r="I1549" t="inlineStr">
-        <is>
-          <t>de-eerste-gemeente/index.html</t>
-        </is>
-      </c>
       <c r="R1549" t="inlineStr">
         <is>
           <t>live</t>
@@ -64993,11 +64058,6 @@
           <t>De halve gemeente</t>
         </is>
       </c>
-      <c r="I1550" t="inlineStr">
-        <is>
-          <t>de-halve-gemeente/index.html</t>
-        </is>
-      </c>
       <c r="R1550" t="inlineStr">
         <is>
           <t>live</t>
@@ -67583,11 +66643,6 @@
           <t>Een fusiereactor zonder magnetische kooi</t>
         </is>
       </c>
-      <c r="I1615" t="inlineStr">
-        <is>
-          <t>editie-1/kernfusie.html</t>
-        </is>
-      </c>
       <c r="R1615" t="inlineStr">
         <is>
           <t>live</t>
@@ -68884,11 +67939,6 @@
           <t>Vortex-Hair™ Adaptive Dimple Golf Ball — Dossier</t>
         </is>
       </c>
-      <c r="I1647" t="inlineStr">
-        <is>
-          <t>dossiers/vortex-hair.html</t>
-        </is>
-      </c>
       <c r="R1647" t="inlineStr">
         <is>
           <t>live</t>
@@ -68965,11 +68015,6 @@
           <t>Archief</t>
         </is>
       </c>
-      <c r="I1649" t="inlineStr">
-        <is>
-          <t>archief.html</t>
-        </is>
-      </c>
       <c r="R1649" t="inlineStr">
         <is>
           <t>live</t>
@@ -69008,11 +68053,6 @@
           <t>Bedankt — controleer uw inbox</t>
         </is>
       </c>
-      <c r="I1650" t="inlineStr">
-        <is>
-          <t>bedankt.html</t>
-        </is>
-      </c>
       <c r="R1650" t="inlineStr">
         <is>
           <t>live</t>
@@ -69089,11 +68129,6 @@
           <t>Het Open Vizier verder dragen</t>
         </is>
       </c>
-      <c r="I1652" t="inlineStr">
-        <is>
-          <t>delen.html</t>
-        </is>
-      </c>
       <c r="R1652" t="inlineStr">
         <is>
           <t>live</t>
@@ -69170,11 +68205,6 @@
           <t>Hoe u meedoet aan de discussie</t>
         </is>
       </c>
-      <c r="I1654" t="inlineStr">
-        <is>
-          <t>editie-1/discussie.html</t>
-        </is>
-      </c>
       <c r="R1654" t="inlineStr">
         <is>
           <t>live</t>
@@ -69213,11 +68243,6 @@
           <t>Navigatie</t>
         </is>
       </c>
-      <c r="I1655" t="inlineStr">
-        <is>
-          <t>navigatie.html</t>
-        </is>
-      </c>
       <c r="R1655" t="inlineStr">
         <is>
           <t>live</t>
@@ -69256,11 +68281,6 @@
           <t>Op de hoogte blijven</t>
         </is>
       </c>
-      <c r="I1656" t="inlineStr">
-        <is>
-          <t>op-de-hoogte.html</t>
-        </is>
-      </c>
       <c r="R1656" t="inlineStr">
         <is>
           <t>live</t>
@@ -69299,11 +68319,6 @@
           <t>Over deze krant</t>
         </is>
       </c>
-      <c r="I1657" t="inlineStr">
-        <is>
-          <t>over.html</t>
-        </is>
-      </c>
       <c r="R1657" t="inlineStr">
         <is>
           <t>live</t>
@@ -69385,11 +68400,6 @@
           <t>Structuur — Beheer</t>
         </is>
       </c>
-      <c r="I1659" t="inlineStr">
-        <is>
-          <t>structuur.html</t>
-        </is>
-      </c>
       <c r="R1659" t="inlineStr">
         <is>
           <t>live</t>
@@ -69471,11 +68481,6 @@
           <t>Waarom deze krant?</t>
         </is>
       </c>
-      <c r="I1661" t="inlineStr">
-        <is>
-          <t>editie-1/voorwoord.html</t>
-        </is>
-      </c>
       <c r="R1661" t="inlineStr">
         <is>
           <t>live</t>
@@ -70349,11 +69354,6 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
-      <c r="I1683" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-07-ai-onderwijs.html</t>
-        </is>
-      </c>
       <c r="R1683" t="inlineStr">
         <is>
           <t>live</t>
@@ -70473,11 +69473,6 @@
           <t>Alles stroomt — de moeder van alle wetenschap</t>
         </is>
       </c>
-      <c r="I1686" t="inlineStr">
-        <is>
-          <t>editie-1/stromingsleer.html</t>
-        </is>
-      </c>
       <c r="R1686" t="inlineStr">
         <is>
           <t>live</t>
@@ -70797,11 +69792,6 @@
           <t>Drie dimensies zijn te weinig</t>
         </is>
       </c>
-      <c r="I1694" t="inlineStr">
-        <is>
-          <t>editie-1/denkraam-7d.html</t>
-        </is>
-      </c>
       <c r="R1694" t="inlineStr">
         <is>
           <t>live</t>
@@ -70883,11 +69873,6 @@
           <t>Hoe alles samenhangt</t>
         </is>
       </c>
-      <c r="I1696" t="inlineStr">
-        <is>
-          <t>editie-1/samenhang.html</t>
-        </is>
-      </c>
       <c r="R1696" t="inlineStr">
         <is>
           <t>live</t>
@@ -71131,11 +70116,6 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
-      <c r="I1702" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-04-bankier.html</t>
-        </is>
-      </c>
       <c r="R1702" t="inlineStr">
         <is>
           <t>live</t>
@@ -71174,11 +70154,6 @@
           <t>Communicatie tussen oergevoelens</t>
         </is>
       </c>
-      <c r="I1703" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-04-communicatie.html</t>
-        </is>
-      </c>
       <c r="R1703" t="inlineStr">
         <is>
           <t>live</t>
@@ -71217,11 +70192,6 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
-      <c r="I1704" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-02-ceo.html</t>
-        </is>
-      </c>
       <c r="R1704" t="inlineStr">
         <is>
           <t>live</t>
@@ -71260,11 +70230,6 @@
           <t>De drie hersenlagen</t>
         </is>
       </c>
-      <c r="I1705" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-03-drie-lagen.html</t>
-        </is>
-      </c>
       <c r="R1705" t="inlineStr">
         <is>
           <t>live</t>
@@ -71303,11 +70268,6 @@
           <t>De mens onder het ijs (Editie 3)</t>
         </is>
       </c>
-      <c r="I1706" t="inlineStr">
-        <is>
-          <t>editie-3/index.html</t>
-        </is>
-      </c>
       <c r="R1706" t="inlineStr">
         <is>
           <t>live</t>
@@ -71346,11 +70306,6 @@
           <t>De zeven dimensies</t>
         </is>
       </c>
-      <c r="I1707" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-02-zeven-dimensies.html</t>
-        </is>
-      </c>
       <c r="R1707" t="inlineStr">
         <is>
           <t>live</t>
@@ -71432,11 +70387,6 @@
           <t>Het oergevoel</t>
         </is>
       </c>
-      <c r="I1709" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-01-oergevoel.html</t>
-        </is>
-      </c>
       <c r="R1709" t="inlineStr">
         <is>
           <t>live</t>
@@ -71475,11 +70425,6 @@
           <t>Het oergevoel in de beroepspraktijk</t>
         </is>
       </c>
-      <c r="I1710" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-09-oergevoel-in-beroepspraktijk.html</t>
-        </is>
-      </c>
       <c r="R1710" t="inlineStr">
         <is>
           <t>live</t>
@@ -71518,11 +70463,6 @@
           <t>Mama ik heb honger</t>
         </is>
       </c>
-      <c r="I1711" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-06-mama.html</t>
-        </is>
-      </c>
       <c r="R1711" t="inlineStr">
         <is>
           <t>live</t>
@@ -71561,11 +70501,6 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
-      <c r="I1712" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-00-redactie.html</t>
-        </is>
-      </c>
       <c r="R1712" t="inlineStr">
         <is>
           <t>live</t>
@@ -71604,11 +70539,6 @@
           <t>Retrospectief</t>
         </is>
       </c>
-      <c r="I1713" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-08-retrospectief.html</t>
-        </is>
-      </c>
       <c r="R1713" t="inlineStr">
         <is>
           <t>live</t>
@@ -71690,11 +70620,6 @@
           <t>Tien seconden</t>
         </is>
       </c>
-      <c r="I1715" t="inlineStr">
-        <is>
-          <t>idee.html</t>
-        </is>
-      </c>
       <c r="R1715" t="inlineStr">
         <is>
           <t>live</t>
@@ -71776,11 +70701,6 @@
           <t>Wat we kinderen aandoen</t>
         </is>
       </c>
-      <c r="I1717" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-05-wat-we-doen.html</t>
-        </is>
-      </c>
       <c r="R1717" t="inlineStr">
         <is>
           <t>live</t>
@@ -72573,11 +71493,6 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
-      <c r="I1736" t="inlineStr">
-        <is>
-          <t>stemgedrag.html</t>
-        </is>
-      </c>
       <c r="R1736" t="inlineStr">
         <is>
           <t>live</t>
@@ -72864,11 +71779,6 @@
           <t>Wat is er mis met partijpolitiek?</t>
         </is>
       </c>
-      <c r="I1743" t="inlineStr">
-        <is>
-          <t>editie-1/nova-democratia.html</t>
-        </is>
-      </c>
       <c r="R1743" t="inlineStr">
         <is>
           <t>live</t>
@@ -73160,11 +72070,6 @@
           <t>De methaan-misleiding</t>
         </is>
       </c>
-      <c r="I1750" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-04-methaan-misleiding.html</t>
-        </is>
-      </c>
       <c r="R1750" t="inlineStr">
         <is>
           <t>live</t>
@@ -73289,11 +72194,6 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
-      <c r="I1753" t="inlineStr">
-        <is>
-          <t>editie-stikstof/drie-problemen-een-antwoord.html</t>
-        </is>
-      </c>
       <c r="R1753" t="inlineStr">
         <is>
           <t>live</t>
@@ -73332,11 +72232,6 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
-      <c r="I1754" t="inlineStr">
-        <is>
-          <t>editie-klimaat/index.html</t>
-        </is>
-      </c>
       <c r="R1754" t="inlineStr">
         <is>
           <t>live</t>
@@ -73375,11 +72270,6 @@
           <t>Editie Stikstof</t>
         </is>
       </c>
-      <c r="I1755" t="inlineStr">
-        <is>
-          <t>editie-stikstof/index.html</t>
-        </is>
-      </c>
       <c r="R1755" t="inlineStr">
         <is>
           <t>live</t>
@@ -73671,11 +72561,6 @@
           <t>De Koolzaad-Multiplicator</t>
         </is>
       </c>
-      <c r="I1762" t="inlineStr">
-        <is>
-          <t>editie-duitsland/raps-multiplicator-oost-duitsland.html</t>
-        </is>
-      </c>
       <c r="R1762" t="inlineStr">
         <is>
           <t>live</t>
@@ -73714,11 +72599,6 @@
           <t>De plant die verhuist</t>
         </is>
       </c>
-      <c r="I1763" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-05-plant-die-verhuist.html</t>
-        </is>
-      </c>
       <c r="R1763" t="inlineStr">
         <is>
           <t>live</t>
@@ -73757,11 +72637,6 @@
           <t>Editie Duitsland</t>
         </is>
       </c>
-      <c r="I1764" t="inlineStr">
-        <is>
-          <t>editie-duitsland/index.html</t>
-        </is>
-      </c>
       <c r="R1764" t="inlineStr">
         <is>
           <t>live</t>
@@ -73924,11 +72799,6 @@
           <t>De biomimetische krachtcentrale</t>
         </is>
       </c>
-      <c r="I1768" t="inlineStr">
-        <is>
-          <t>editie-0/biomimetische-krachtcentrale.html</t>
-        </is>
-      </c>
       <c r="R1768" t="inlineStr">
         <is>
           <t>live</t>
@@ -74129,11 +72999,6 @@
           <t>Editie Europa</t>
         </is>
       </c>
-      <c r="I1773" t="inlineStr">
-        <is>
-          <t>editie-0/index.html</t>
-        </is>
-      </c>
       <c r="R1773" t="inlineStr">
         <is>
           <t>live</t>
@@ -74334,11 +73199,6 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
-      <c r="I1778" t="inlineStr">
-        <is>
-          <t>editie-0/carbon-alert-europa.html</t>
-        </is>
-      </c>
       <c r="R1778" t="inlineStr">
         <is>
           <t>live</t>
@@ -74458,11 +73318,6 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
-      <c r="I1781" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-04-bankier.html</t>
-        </is>
-      </c>
       <c r="R1781" t="inlineStr">
         <is>
           <t>live</t>
@@ -74673,11 +73528,6 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
-      <c r="I1786" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-02-ceo.html</t>
-        </is>
-      </c>
       <c r="R1786" t="inlineStr">
         <is>
           <t>live</t>
@@ -74716,11 +73566,6 @@
           <t>De consultant bij het bijna-failliete bedrijf</t>
         </is>
       </c>
-      <c r="I1787" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-03-consultant.html</t>
-        </is>
-      </c>
       <c r="R1787" t="inlineStr">
         <is>
           <t>live</t>
@@ -74759,11 +73604,6 @@
           <t>De diepere vraag</t>
         </is>
       </c>
-      <c r="I1788" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-08-diepere-vraag.html</t>
-        </is>
-      </c>
       <c r="R1788" t="inlineStr">
         <is>
           <t>live</t>
@@ -74888,11 +73728,6 @@
           <t>De rechter zonder kompas</t>
         </is>
       </c>
-      <c r="I1791" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-07-rechter.html</t>
-        </is>
-      </c>
       <c r="R1791" t="inlineStr">
         <is>
           <t>live</t>
@@ -74931,11 +73766,6 @@
           <t>De toezichthouder die niets ziet</t>
         </is>
       </c>
-      <c r="I1792" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-06-toezichthouder.html</t>
-        </is>
-      </c>
       <c r="R1792" t="inlineStr">
         <is>
           <t>live</t>
@@ -74974,11 +73804,6 @@
           <t>De verzekeraar tegen het leven</t>
         </is>
       </c>
-      <c r="I1793" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-05-verzekeraar.html</t>
-        </is>
-      </c>
       <c r="R1793" t="inlineStr">
         <is>
           <t>live</t>
@@ -75017,11 +73842,6 @@
           <t>De wet van de papier-industrie</t>
         </is>
       </c>
-      <c r="I1794" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-01-wet-papier-industrie.html</t>
-        </is>
-      </c>
       <c r="R1794" t="inlineStr">
         <is>
           <t>live</t>
@@ -75184,11 +74004,6 @@
           <t>Editie Kind &amp; Loopbaan</t>
         </is>
       </c>
-      <c r="I1798" t="inlineStr">
-        <is>
-          <t>editie-kind-loopbaan/index.html</t>
-        </is>
-      </c>
       <c r="R1798" t="inlineStr">
         <is>
           <t>live</t>
@@ -75227,11 +74042,6 @@
           <t>Editie Leiderschap</t>
         </is>
       </c>
-      <c r="I1799" t="inlineStr">
-        <is>
-          <t>editie-leiderschap/index.html</t>
-        </is>
-      </c>
       <c r="R1799" t="inlineStr">
         <is>
           <t>live</t>
@@ -75270,11 +74080,6 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
-      <c r="I1800" t="inlineStr">
-        <is>
-          <t>toekomst/energie/index.html</t>
-        </is>
-      </c>
       <c r="R1800" t="inlineStr">
         <is>
           <t>live</t>
@@ -75313,11 +74118,6 @@
           <t>Hoe de papier-industrie macht kreeg over het echte werk</t>
         </is>
       </c>
-      <c r="I1801" t="inlineStr">
-        <is>
-          <t>editie-4/index.html</t>
-        </is>
-      </c>
       <c r="R1801" t="inlineStr">
         <is>
           <t>live</t>
@@ -75356,11 +74156,6 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
-      <c r="I1802" t="inlineStr">
-        <is>
-          <t>toekomst/industrie/index.html</t>
-        </is>
-      </c>
       <c r="R1802" t="inlineStr">
         <is>
           <t>live</t>
@@ -75485,11 +74280,6 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
-      <c r="I1805" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/methode/index.html</t>
-        </is>
-      </c>
       <c r="R1805" t="inlineStr">
         <is>
           <t>live</t>
@@ -75657,11 +74447,6 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
-      <c r="I1809" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-07-ai-onderwijs.html</t>
-        </is>
-      </c>
       <c r="R1809" t="inlineStr">
         <is>
           <t>live</t>
@@ -75700,11 +74485,6 @@
           <t>Opvoeding · Toekomst</t>
         </is>
       </c>
-      <c r="I1810" t="inlineStr">
-        <is>
-          <t>toekomst/opvoeding/index.html</t>
-        </is>
-      </c>
       <c r="R1810" t="inlineStr">
         <is>
           <t>live</t>
@@ -75786,11 +74566,6 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
-      <c r="I1812" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/index.html</t>
-        </is>
-      </c>
       <c r="R1812" t="inlineStr">
         <is>
           <t>live</t>
@@ -75829,11 +74604,6 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
-      <c r="I1813" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-00-redactie.html</t>
-        </is>
-      </c>
       <c r="R1813" t="inlineStr">
         <is>
           <t>live</t>
@@ -75872,11 +74642,6 @@
           <t>Retrospectief</t>
         </is>
       </c>
-      <c r="I1814" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-09-retrospectief.html</t>
-        </is>
-      </c>
       <c r="R1814" t="inlineStr">
         <is>
           <t>live</t>
@@ -75915,11 +74680,6 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
-      <c r="I1815" t="inlineStr">
-        <is>
-          <t>toekomst/scholing/index.html</t>
-        </is>
-      </c>
       <c r="R1815" t="inlineStr">
         <is>
           <t>live</t>
@@ -75958,11 +74718,6 @@
           <t>Soevereiniteit als cyclus</t>
         </is>
       </c>
-      <c r="I1816" t="inlineStr">
-        <is>
-          <t>soevereiniteit-als-cyclus/index.html</t>
-        </is>
-      </c>
       <c r="R1816" t="inlineStr">
         <is>
           <t>live</t>
@@ -76044,11 +74799,6 @@
           <t>Toekomst</t>
         </is>
       </c>
-      <c r="I1818" t="inlineStr">
-        <is>
-          <t>toekomst/index.html</t>
-        </is>
-      </c>
       <c r="R1818" t="inlineStr">
         <is>
           <t>live</t>
@@ -76173,11 +74923,6 @@
           <t>Van leerfabriek naar leerwerkplaats</t>
         </is>
       </c>
-      <c r="I1821" t="inlineStr">
-        <is>
-          <t>editie-1/onderwijs.html</t>
-        </is>
-      </c>
       <c r="R1821" t="inlineStr">
         <is>
           <t>live</t>
@@ -76426,11 +75171,6 @@
           <t>De eerste gemeente</t>
         </is>
       </c>
-      <c r="I1827" t="inlineStr">
-        <is>
-          <t>de-eerste-gemeente/index.html</t>
-        </is>
-      </c>
       <c r="R1827" t="inlineStr">
         <is>
           <t>live</t>
@@ -76469,11 +75209,6 @@
           <t>De halve gemeente</t>
         </is>
       </c>
-      <c r="I1828" t="inlineStr">
-        <is>
-          <t>de-halve-gemeente/index.html</t>
-        </is>
-      </c>
       <c r="R1828" t="inlineStr">
         <is>
           <t>live</t>
@@ -76636,11 +75371,6 @@
           <t>Gevolgenkaart — Nederland</t>
         </is>
       </c>
-      <c r="I1832" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-nl/index.html</t>
-        </is>
-      </c>
       <c r="R1832" t="inlineStr">
         <is>
           <t>live</t>
@@ -76760,11 +75490,6 @@
           <t>Nederland · Toekomst</t>
         </is>
       </c>
-      <c r="I1835" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/nederland/index.html</t>
-        </is>
-      </c>
       <c r="R1835" t="inlineStr">
         <is>
           <t>live</t>
@@ -77390,11 +76115,6 @@
           <t>Duitsland · Toekomst</t>
         </is>
       </c>
-      <c r="I1850" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/duitsland/index.html</t>
-        </is>
-      </c>
       <c r="R1850" t="inlineStr">
         <is>
           <t>live</t>
@@ -77562,11 +76282,6 @@
           <t>Europa · Toekomst</t>
         </is>
       </c>
-      <c r="I1854" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/europa/index.html</t>
-        </is>
-      </c>
       <c r="R1854" t="inlineStr">
         <is>
           <t>live</t>
@@ -77605,11 +76320,6 @@
           <t>Gevolgenkaart EU-27</t>
         </is>
       </c>
-      <c r="I1855" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-eu/index.html</t>
-        </is>
-      </c>
       <c r="R1855" t="inlineStr">
         <is>
           <t>live</t>
@@ -77648,11 +76358,6 @@
           <t>Gevolgenkaart — Brazilië</t>
         </is>
       </c>
-      <c r="I1856" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-br/index.html</t>
-        </is>
-      </c>
       <c r="R1856" t="inlineStr">
         <is>
           <t>live</t>
@@ -77691,11 +76396,6 @@
           <t>Gevolgenkaart — China</t>
         </is>
       </c>
-      <c r="I1857" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-cn/index.html</t>
-        </is>
-      </c>
       <c r="R1857" t="inlineStr">
         <is>
           <t>live</t>
@@ -77734,11 +76434,6 @@
           <t>Gevolgenkaart — Cuba</t>
         </is>
       </c>
-      <c r="I1858" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-cu/index.html</t>
-        </is>
-      </c>
       <c r="R1858" t="inlineStr">
         <is>
           <t>live</t>
@@ -77777,11 +76472,6 @@
           <t>Gevolgenkaart — Duitsland</t>
         </is>
       </c>
-      <c r="I1859" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-de/index.html</t>
-        </is>
-      </c>
       <c r="R1859" t="inlineStr">
         <is>
           <t>live</t>
@@ -77820,11 +76510,6 @@
           <t>Gevolgenkaart — India</t>
         </is>
       </c>
-      <c r="I1860" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-in/index.html</t>
-        </is>
-      </c>
       <c r="R1860" t="inlineStr">
         <is>
           <t>live</t>
@@ -77863,11 +76548,6 @@
           <t>Gevolgenkaart — Iran</t>
         </is>
       </c>
-      <c r="I1861" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-ir/index.html</t>
-        </is>
-      </c>
       <c r="R1861" t="inlineStr">
         <is>
           <t>live</t>
@@ -77906,11 +76586,6 @@
           <t>Gevolgenkaart — Israël</t>
         </is>
       </c>
-      <c r="I1862" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-il/index.html</t>
-        </is>
-      </c>
       <c r="R1862" t="inlineStr">
         <is>
           <t>live</t>
@@ -77949,11 +76624,6 @@
           <t>Gevolgenkaart — Japan</t>
         </is>
       </c>
-      <c r="I1863" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-jp/index.html</t>
-        </is>
-      </c>
       <c r="R1863" t="inlineStr">
         <is>
           <t>live</t>
@@ -77992,11 +76662,6 @@
           <t>Gevolgenkaart — Spanje</t>
         </is>
       </c>
-      <c r="I1864" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-es/index.html</t>
-        </is>
-      </c>
       <c r="R1864" t="inlineStr">
         <is>
           <t>live</t>
@@ -78035,11 +76700,6 @@
           <t>Gevolgenkaart — Suriname</t>
         </is>
       </c>
-      <c r="I1865" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-sr/index.html</t>
-        </is>
-      </c>
       <c r="R1865" t="inlineStr">
         <is>
           <t>live</t>
@@ -78078,11 +76738,6 @@
           <t>Gevolgenkaart — Taiwan</t>
         </is>
       </c>
-      <c r="I1866" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-tw/index.html</t>
-        </is>
-      </c>
       <c r="R1866" t="inlineStr">
         <is>
           <t>live</t>
@@ -78121,11 +76776,6 @@
           <t>Gevolgenkaart — Verenigd Koninkrijk</t>
         </is>
       </c>
-      <c r="I1867" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-uk/index.html</t>
-        </is>
-      </c>
       <c r="R1867" t="inlineStr">
         <is>
           <t>live</t>
@@ -78164,11 +76814,6 @@
           <t>Gevolgenkaart — Verenigde Staten</t>
         </is>
       </c>
-      <c r="I1868" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-us/index.html</t>
-        </is>
-      </c>
       <c r="R1868" t="inlineStr">
         <is>
           <t>live</t>
@@ -78207,11 +76852,6 @@
           <t>Gevolgenkaart — Zuid-Afrika</t>
         </is>
       </c>
-      <c r="I1869" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-za/index.html</t>
-        </is>
-      </c>
       <c r="R1869" t="inlineStr">
         <is>
           <t>live</t>
@@ -78250,11 +76890,6 @@
           <t>Gevolgenkaart — Zuid-Korea</t>
         </is>
       </c>
-      <c r="I1870" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-kr/index.html</t>
-        </is>
-      </c>
       <c r="R1870" t="inlineStr">
         <is>
           <t>live</t>
@@ -78293,11 +76928,6 @@
           <t>Gevolgenkaart — Zweden</t>
         </is>
       </c>
-      <c r="I1871" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-se/index.html</t>
-        </is>
-      </c>
       <c r="R1871" t="inlineStr">
         <is>
           <t>live</t>
@@ -78336,11 +76966,6 @@
           <t>Gevolgenkaart — Zwitserland</t>
         </is>
       </c>
-      <c r="I1872" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-ch/index.html</t>
-        </is>
-      </c>
       <c r="R1872" t="inlineStr">
         <is>
           <t>live</t>
@@ -78675,11 +77300,6 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
-      <c r="I1880" t="inlineStr">
-        <is>
-          <t>editie-0/carbon-alert-europa.html</t>
-        </is>
-      </c>
       <c r="R1880" t="inlineStr">
         <is>
           <t>live</t>
@@ -78799,11 +77419,6 @@
           <t>Brief aan de lezer</t>
         </is>
       </c>
-      <c r="I1883" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-00-brief-aan-lezer.html</t>
-        </is>
-      </c>
       <c r="R1883" t="inlineStr">
         <is>
           <t>live</t>
@@ -78842,11 +77457,6 @@
           <t>De afwijkers</t>
         </is>
       </c>
-      <c r="I1884" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-07-afwijkers.html</t>
-        </is>
-      </c>
       <c r="R1884" t="inlineStr">
         <is>
           <t>live</t>
@@ -78885,11 +77495,6 @@
           <t>De eis aan de lezer</t>
         </is>
       </c>
-      <c r="I1885" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-08-eis-aan-lezer.html</t>
-        </is>
-      </c>
       <c r="R1885" t="inlineStr">
         <is>
           <t>live</t>
@@ -78928,11 +77533,6 @@
           <t>De methaan-misleiding</t>
         </is>
       </c>
-      <c r="I1886" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-04-methaan-misleiding.html</t>
-        </is>
-      </c>
       <c r="R1886" t="inlineStr">
         <is>
           <t>live</t>
@@ -78971,11 +77571,6 @@
           <t>De plant die verhuist</t>
         </is>
       </c>
-      <c r="I1887" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-05-plant-die-verhuist.html</t>
-        </is>
-      </c>
       <c r="R1887" t="inlineStr">
         <is>
           <t>live</t>
@@ -79014,11 +77609,6 @@
           <t>De succesformule die wij verleerd hebben</t>
         </is>
       </c>
-      <c r="I1888" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-02-succesformule.html</t>
-        </is>
-      </c>
       <c r="R1888" t="inlineStr">
         <is>
           <t>live</t>
@@ -79057,11 +77647,6 @@
           <t>De vergeten orde</t>
         </is>
       </c>
-      <c r="I1889" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-03-vergeten-orde.html</t>
-        </is>
-      </c>
       <c r="R1889" t="inlineStr">
         <is>
           <t>live</t>
@@ -79100,11 +77685,6 @@
           <t>De zeven van Bern</t>
         </is>
       </c>
-      <c r="I1890" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-06-zeven-van-bern.html</t>
-        </is>
-      </c>
       <c r="R1890" t="inlineStr">
         <is>
           <t>live</t>
@@ -79143,11 +77723,6 @@
           <t>Editie 1</t>
         </is>
       </c>
-      <c r="I1891" t="inlineStr">
-        <is>
-          <t>editie-1/index.html</t>
-        </is>
-      </c>
       <c r="R1891" t="inlineStr">
         <is>
           <t>live</t>
@@ -79186,11 +77761,6 @@
           <t>Editie 5 — portaal</t>
         </is>
       </c>
-      <c r="I1892" t="inlineStr">
-        <is>
-          <t>editie-5/index.html</t>
-        </is>
-      </c>
       <c r="R1892" t="inlineStr">
         <is>
           <t>live</t>
@@ -79229,11 +77799,6 @@
           <t>Een fusiereactor zonder magnetische kooi</t>
         </is>
       </c>
-      <c r="I1893" t="inlineStr">
-        <is>
-          <t>editie-1/kernfusie.html</t>
-        </is>
-      </c>
       <c r="R1893" t="inlineStr">
         <is>
           <t>live</t>
@@ -79315,11 +77880,6 @@
           <t>Wat er nu al ligt</t>
         </is>
       </c>
-      <c r="I1895" t="inlineStr">
-        <is>
-          <t>editie-1/technische-oplossingen.html</t>
-        </is>
-      </c>
       <c r="R1895" t="inlineStr">
         <is>
           <t>live</t>
@@ -79358,11 +77918,6 @@
           <t>七つ道具 — Zeven gereedschappen</t>
         </is>
       </c>
-      <c r="I1896" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-01-zeven-gereedschappen.html</t>
-        </is>
-      </c>
       <c r="R1896" t="inlineStr">
         <is>
           <t>live</t>
@@ -80097,11 +78652,6 @@
           <t>Wie zijn opbouwers wegjaagt</t>
         </is>
       </c>
-      <c r="I1914" t="inlineStr">
-        <is>
-          <t>opbouwers-wegjagen/index.html</t>
-        </is>
-      </c>
       <c r="R1914" t="inlineStr">
         <is>
           <t>live</t>
@@ -80178,11 +78728,6 @@
           <t>Achter de Cijfers</t>
         </is>
       </c>
-      <c r="I1916" t="inlineStr">
-        <is>
-          <t>onderzoek/index.html</t>
-        </is>
-      </c>
       <c r="R1916" t="inlineStr">
         <is>
           <t>live</t>
@@ -80221,11 +78766,6 @@
           <t>Dossiers</t>
         </is>
       </c>
-      <c r="I1917" t="inlineStr">
-        <is>
-          <t>dossiers/index.html</t>
-        </is>
-      </c>
       <c r="R1917" t="inlineStr">
         <is>
           <t>live</t>
@@ -80264,11 +78804,6 @@
           <t>EU: BBP, Reële Lonen en de Overheidsmultiplicator</t>
         </is>
       </c>
-      <c r="I1918" t="inlineStr">
-        <is>
-          <t>onderzoek/eu-multiplicator.html</t>
-        </is>
-      </c>
       <c r="R1918" t="inlineStr">
         <is>
           <t>live</t>
@@ -80479,11 +79014,6 @@
           <t>Is Nederland op weg naar ontwikkelingslandstatus?</t>
         </is>
       </c>
-      <c r="I1923" t="inlineStr">
-        <is>
-          <t>onderzoek/ontwikkelingslandstatus.html</t>
-        </is>
-      </c>
       <c r="R1923" t="inlineStr">
         <is>
           <t>live</t>
@@ -80565,11 +79095,6 @@
           <t>Vortex-Hair™ Adaptive Dimple Golf Ball — Dossier</t>
         </is>
       </c>
-      <c r="I1925" t="inlineStr">
-        <is>
-          <t>dossiers/vortex-hair.html</t>
-        </is>
-      </c>
       <c r="R1925" t="inlineStr">
         <is>
           <t>live</t>
@@ -80646,11 +79171,6 @@
           <t>Archief</t>
         </is>
       </c>
-      <c r="I1927" t="inlineStr">
-        <is>
-          <t>archief.html</t>
-        </is>
-      </c>
       <c r="R1927" t="inlineStr">
         <is>
           <t>live</t>
@@ -80689,11 +79209,6 @@
           <t>Bedankt — controleer uw inbox</t>
         </is>
       </c>
-      <c r="I1928" t="inlineStr">
-        <is>
-          <t>bedankt.html</t>
-        </is>
-      </c>
       <c r="R1928" t="inlineStr">
         <is>
           <t>live</t>
@@ -80770,11 +79285,6 @@
           <t>Het Open Vizier verder dragen</t>
         </is>
       </c>
-      <c r="I1930" t="inlineStr">
-        <is>
-          <t>delen.html</t>
-        </is>
-      </c>
       <c r="R1930" t="inlineStr">
         <is>
           <t>live</t>
@@ -80851,11 +79361,6 @@
           <t>Hoe u meedoet aan de discussie</t>
         </is>
       </c>
-      <c r="I1932" t="inlineStr">
-        <is>
-          <t>editie-1/discussie.html</t>
-        </is>
-      </c>
       <c r="R1932" t="inlineStr">
         <is>
           <t>live</t>
@@ -80894,11 +79399,6 @@
           <t>Navigatie</t>
         </is>
       </c>
-      <c r="I1933" t="inlineStr">
-        <is>
-          <t>navigatie.html</t>
-        </is>
-      </c>
       <c r="R1933" t="inlineStr">
         <is>
           <t>live</t>
@@ -80937,11 +79437,6 @@
           <t>Op de hoogte blijven</t>
         </is>
       </c>
-      <c r="I1934" t="inlineStr">
-        <is>
-          <t>op-de-hoogte.html</t>
-        </is>
-      </c>
       <c r="R1934" t="inlineStr">
         <is>
           <t>live</t>
@@ -80980,11 +79475,6 @@
           <t>Over deze krant</t>
         </is>
       </c>
-      <c r="I1935" t="inlineStr">
-        <is>
-          <t>over.html</t>
-        </is>
-      </c>
       <c r="R1935" t="inlineStr">
         <is>
           <t>live</t>
@@ -81066,11 +79556,6 @@
           <t>Structuur — Beheer</t>
         </is>
       </c>
-      <c r="I1937" t="inlineStr">
-        <is>
-          <t>structuur.html</t>
-        </is>
-      </c>
       <c r="R1937" t="inlineStr">
         <is>
           <t>live</t>
@@ -81152,11 +79637,6 @@
           <t>Waarom deze krant?</t>
         </is>
       </c>
-      <c r="I1939" t="inlineStr">
-        <is>
-          <t>editie-1/voorwoord.html</t>
-        </is>
-      </c>
       <c r="R1939" t="inlineStr">
         <is>
           <t>live</t>
@@ -82030,11 +80510,6 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
-      <c r="I1961" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-07-ai-onderwijs.html</t>
-        </is>
-      </c>
       <c r="R1961" t="inlineStr">
         <is>
           <t>live</t>
@@ -82154,11 +80629,6 @@
           <t>Alles stroomt — de moeder van alle wetenschap</t>
         </is>
       </c>
-      <c r="I1964" t="inlineStr">
-        <is>
-          <t>editie-1/stromingsleer.html</t>
-        </is>
-      </c>
       <c r="R1964" t="inlineStr">
         <is>
           <t>live</t>
@@ -82478,11 +80948,6 @@
           <t>Drie dimensies zijn te weinig</t>
         </is>
       </c>
-      <c r="I1972" t="inlineStr">
-        <is>
-          <t>editie-1/denkraam-7d.html</t>
-        </is>
-      </c>
       <c r="R1972" t="inlineStr">
         <is>
           <t>live</t>
@@ -82564,11 +81029,6 @@
           <t>Hoe alles samenhangt</t>
         </is>
       </c>
-      <c r="I1974" t="inlineStr">
-        <is>
-          <t>editie-1/samenhang.html</t>
-        </is>
-      </c>
       <c r="R1974" t="inlineStr">
         <is>
           <t>live</t>
@@ -82812,11 +81272,6 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
-      <c r="I1980" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-04-bankier.html</t>
-        </is>
-      </c>
       <c r="R1980" t="inlineStr">
         <is>
           <t>live</t>
@@ -82855,11 +81310,6 @@
           <t>Communicatie tussen oergevoelens</t>
         </is>
       </c>
-      <c r="I1981" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-04-communicatie.html</t>
-        </is>
-      </c>
       <c r="R1981" t="inlineStr">
         <is>
           <t>live</t>
@@ -82898,11 +81348,6 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
-      <c r="I1982" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-02-ceo.html</t>
-        </is>
-      </c>
       <c r="R1982" t="inlineStr">
         <is>
           <t>live</t>
@@ -82941,11 +81386,6 @@
           <t>De drie hersenlagen</t>
         </is>
       </c>
-      <c r="I1983" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-03-drie-lagen.html</t>
-        </is>
-      </c>
       <c r="R1983" t="inlineStr">
         <is>
           <t>live</t>
@@ -82984,11 +81424,6 @@
           <t>De mens onder het ijs (Editie 3)</t>
         </is>
       </c>
-      <c r="I1984" t="inlineStr">
-        <is>
-          <t>editie-3/index.html</t>
-        </is>
-      </c>
       <c r="R1984" t="inlineStr">
         <is>
           <t>live</t>
@@ -83027,11 +81462,6 @@
           <t>De zeven dimensies</t>
         </is>
       </c>
-      <c r="I1985" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-02-zeven-dimensies.html</t>
-        </is>
-      </c>
       <c r="R1985" t="inlineStr">
         <is>
           <t>live</t>
@@ -83113,11 +81543,6 @@
           <t>Het oergevoel</t>
         </is>
       </c>
-      <c r="I1987" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-01-oergevoel.html</t>
-        </is>
-      </c>
       <c r="R1987" t="inlineStr">
         <is>
           <t>live</t>
@@ -83156,11 +81581,6 @@
           <t>Het oergevoel in de beroepspraktijk</t>
         </is>
       </c>
-      <c r="I1988" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-09-oergevoel-in-beroepspraktijk.html</t>
-        </is>
-      </c>
       <c r="R1988" t="inlineStr">
         <is>
           <t>live</t>
@@ -83199,11 +81619,6 @@
           <t>Mama ik heb honger</t>
         </is>
       </c>
-      <c r="I1989" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-06-mama.html</t>
-        </is>
-      </c>
       <c r="R1989" t="inlineStr">
         <is>
           <t>live</t>
@@ -83242,11 +81657,6 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
-      <c r="I1990" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-00-redactie.html</t>
-        </is>
-      </c>
       <c r="R1990" t="inlineStr">
         <is>
           <t>live</t>
@@ -83285,11 +81695,6 @@
           <t>Retrospectief</t>
         </is>
       </c>
-      <c r="I1991" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-08-retrospectief.html</t>
-        </is>
-      </c>
       <c r="R1991" t="inlineStr">
         <is>
           <t>live</t>
@@ -83371,11 +81776,6 @@
           <t>Tien seconden</t>
         </is>
       </c>
-      <c r="I1993" t="inlineStr">
-        <is>
-          <t>idee.html</t>
-        </is>
-      </c>
       <c r="R1993" t="inlineStr">
         <is>
           <t>live</t>
@@ -83457,11 +81857,6 @@
           <t>Wat we kinderen aandoen</t>
         </is>
       </c>
-      <c r="I1995" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-05-wat-we-doen.html</t>
-        </is>
-      </c>
       <c r="R1995" t="inlineStr">
         <is>
           <t>live</t>
@@ -84234,11 +82629,6 @@
           <t>Een matrixen-bestand als spiegel van de politiek</t>
         </is>
       </c>
-      <c r="I2014" t="inlineStr">
-        <is>
-          <t>stemgedrag.html</t>
-        </is>
-      </c>
       <c r="R2014" t="inlineStr">
         <is>
           <t>live</t>
@@ -84525,11 +82915,6 @@
           <t>Wat is er mis met partijpolitiek?</t>
         </is>
       </c>
-      <c r="I2021" t="inlineStr">
-        <is>
-          <t>editie-1/nova-democratia.html</t>
-        </is>
-      </c>
       <c r="R2021" t="inlineStr">
         <is>
           <t>live</t>
@@ -84821,11 +83206,6 @@
           <t>De methaan-misleiding</t>
         </is>
       </c>
-      <c r="I2028" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-04-methaan-misleiding.html</t>
-        </is>
-      </c>
       <c r="R2028" t="inlineStr">
         <is>
           <t>live</t>
@@ -84950,11 +83330,6 @@
           <t>Drie problemen, één antwoord</t>
         </is>
       </c>
-      <c r="I2031" t="inlineStr">
-        <is>
-          <t>editie-stikstof/drie-problemen-een-antwoord.html</t>
-        </is>
-      </c>
       <c r="R2031" t="inlineStr">
         <is>
           <t>live</t>
@@ -84993,11 +83368,6 @@
           <t>Editie Klimaat</t>
         </is>
       </c>
-      <c r="I2032" t="inlineStr">
-        <is>
-          <t>editie-klimaat/index.html</t>
-        </is>
-      </c>
       <c r="R2032" t="inlineStr">
         <is>
           <t>live</t>
@@ -85036,11 +83406,6 @@
           <t>Editie Stikstof</t>
         </is>
       </c>
-      <c r="I2033" t="inlineStr">
-        <is>
-          <t>editie-stikstof/index.html</t>
-        </is>
-      </c>
       <c r="R2033" t="inlineStr">
         <is>
           <t>live</t>
@@ -85332,11 +83697,6 @@
           <t>De Koolzaad-Multiplicator</t>
         </is>
       </c>
-      <c r="I2040" t="inlineStr">
-        <is>
-          <t>editie-duitsland/raps-multiplicator-oost-duitsland.html</t>
-        </is>
-      </c>
       <c r="R2040" t="inlineStr">
         <is>
           <t>live</t>
@@ -85375,11 +83735,6 @@
           <t>De plant die verhuist</t>
         </is>
       </c>
-      <c r="I2041" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-05-plant-die-verhuist.html</t>
-        </is>
-      </c>
       <c r="R2041" t="inlineStr">
         <is>
           <t>live</t>
@@ -85418,11 +83773,6 @@
           <t>Editie Duitsland</t>
         </is>
       </c>
-      <c r="I2042" t="inlineStr">
-        <is>
-          <t>editie-duitsland/index.html</t>
-        </is>
-      </c>
       <c r="R2042" t="inlineStr">
         <is>
           <t>live</t>
@@ -85585,11 +83935,6 @@
           <t>De biomimetische krachtcentrale</t>
         </is>
       </c>
-      <c r="I2046" t="inlineStr">
-        <is>
-          <t>editie-0/biomimetische-krachtcentrale.html</t>
-        </is>
-      </c>
       <c r="R2046" t="inlineStr">
         <is>
           <t>live</t>
@@ -85790,11 +84135,6 @@
           <t>Editie Europa</t>
         </is>
       </c>
-      <c r="I2051" t="inlineStr">
-        <is>
-          <t>editie-0/index.html</t>
-        </is>
-      </c>
       <c r="R2051" t="inlineStr">
         <is>
           <t>live</t>
@@ -85995,11 +84335,6 @@
           <t>Wat Brussel werkelijk krijgt</t>
         </is>
       </c>
-      <c r="I2056" t="inlineStr">
-        <is>
-          <t>editie-0/carbon-alert-europa.html</t>
-        </is>
-      </c>
       <c r="R2056" t="inlineStr">
         <is>
           <t>live</t>
@@ -86119,11 +84454,6 @@
           <t>Bij banken het oergevoel verloren</t>
         </is>
       </c>
-      <c r="I2059" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-04-bankier.html</t>
-        </is>
-      </c>
       <c r="R2059" t="inlineStr">
         <is>
           <t>live</t>
@@ -86334,11 +84664,6 @@
           <t>De CEO en het oergevoel</t>
         </is>
       </c>
-      <c r="I2064" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-02-ceo.html</t>
-        </is>
-      </c>
       <c r="R2064" t="inlineStr">
         <is>
           <t>live</t>
@@ -86377,11 +84702,6 @@
           <t>De consultant bij het bijna-failliete bedrijf</t>
         </is>
       </c>
-      <c r="I2065" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-03-consultant.html</t>
-        </is>
-      </c>
       <c r="R2065" t="inlineStr">
         <is>
           <t>live</t>
@@ -86420,11 +84740,6 @@
           <t>De diepere vraag</t>
         </is>
       </c>
-      <c r="I2066" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-08-diepere-vraag.html</t>
-        </is>
-      </c>
       <c r="R2066" t="inlineStr">
         <is>
           <t>live</t>
@@ -86549,11 +84864,6 @@
           <t>De rechter zonder kompas</t>
         </is>
       </c>
-      <c r="I2069" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-07-rechter.html</t>
-        </is>
-      </c>
       <c r="R2069" t="inlineStr">
         <is>
           <t>live</t>
@@ -86592,11 +84902,6 @@
           <t>De toezichthouder die niets ziet</t>
         </is>
       </c>
-      <c r="I2070" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-06-toezichthouder.html</t>
-        </is>
-      </c>
       <c r="R2070" t="inlineStr">
         <is>
           <t>live</t>
@@ -86635,11 +84940,6 @@
           <t>De verzekeraar tegen het leven</t>
         </is>
       </c>
-      <c r="I2071" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-05-verzekeraar.html</t>
-        </is>
-      </c>
       <c r="R2071" t="inlineStr">
         <is>
           <t>live</t>
@@ -86678,11 +84978,6 @@
           <t>De wet van de papier-industrie</t>
         </is>
       </c>
-      <c r="I2072" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-01-wet-papier-industrie.html</t>
-        </is>
-      </c>
       <c r="R2072" t="inlineStr">
         <is>
           <t>live</t>
@@ -86845,11 +85140,6 @@
           <t>Editie Kind &amp; Loopbaan</t>
         </is>
       </c>
-      <c r="I2076" t="inlineStr">
-        <is>
-          <t>editie-kind-loopbaan/index.html</t>
-        </is>
-      </c>
       <c r="R2076" t="inlineStr">
         <is>
           <t>live</t>
@@ -86888,11 +85178,6 @@
           <t>Editie Leiderschap</t>
         </is>
       </c>
-      <c r="I2077" t="inlineStr">
-        <is>
-          <t>editie-leiderschap/index.html</t>
-        </is>
-      </c>
       <c r="R2077" t="inlineStr">
         <is>
           <t>live</t>
@@ -86931,11 +85216,6 @@
           <t>Energie · Toekomst</t>
         </is>
       </c>
-      <c r="I2078" t="inlineStr">
-        <is>
-          <t>toekomst/energie/index.html</t>
-        </is>
-      </c>
       <c r="R2078" t="inlineStr">
         <is>
           <t>live</t>
@@ -86974,11 +85254,6 @@
           <t>Hoe de papier-industrie macht kreeg over het echte werk</t>
         </is>
       </c>
-      <c r="I2079" t="inlineStr">
-        <is>
-          <t>editie-4/index.html</t>
-        </is>
-      </c>
       <c r="R2079" t="inlineStr">
         <is>
           <t>live</t>
@@ -87017,11 +85292,6 @@
           <t>Industrie · Toekomst</t>
         </is>
       </c>
-      <c r="I2080" t="inlineStr">
-        <is>
-          <t>toekomst/industrie/index.html</t>
-        </is>
-      </c>
       <c r="R2080" t="inlineStr">
         <is>
           <t>live</t>
@@ -87146,11 +85416,6 @@
           <t>Methode · Toekomst</t>
         </is>
       </c>
-      <c r="I2083" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/methode/index.html</t>
-        </is>
-      </c>
       <c r="R2083" t="inlineStr">
         <is>
           <t>live</t>
@@ -87318,11 +85583,6 @@
           <t>Onderwijs in het AI-tijdperk</t>
         </is>
       </c>
-      <c r="I2087" t="inlineStr">
-        <is>
-          <t>editie-3/artikel-07-ai-onderwijs.html</t>
-        </is>
-      </c>
       <c r="R2087" t="inlineStr">
         <is>
           <t>live</t>
@@ -87361,11 +85621,6 @@
           <t>Opvoeding · Toekomst</t>
         </is>
       </c>
-      <c r="I2088" t="inlineStr">
-        <is>
-          <t>toekomst/opvoeding/index.html</t>
-        </is>
-      </c>
       <c r="R2088" t="inlineStr">
         <is>
           <t>live</t>
@@ -87447,11 +85702,6 @@
           <t>Overheden · Toekomst</t>
         </is>
       </c>
-      <c r="I2090" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/index.html</t>
-        </is>
-      </c>
       <c r="R2090" t="inlineStr">
         <is>
           <t>live</t>
@@ -87490,11 +85740,6 @@
           <t>Redactionele inleiding</t>
         </is>
       </c>
-      <c r="I2091" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-00-redactie.html</t>
-        </is>
-      </c>
       <c r="R2091" t="inlineStr">
         <is>
           <t>live</t>
@@ -87533,11 +85778,6 @@
           <t>Retrospectief</t>
         </is>
       </c>
-      <c r="I2092" t="inlineStr">
-        <is>
-          <t>editie-4/artikel-09-retrospectief.html</t>
-        </is>
-      </c>
       <c r="R2092" t="inlineStr">
         <is>
           <t>live</t>
@@ -87576,11 +85816,6 @@
           <t>Scholing · Toekomst</t>
         </is>
       </c>
-      <c r="I2093" t="inlineStr">
-        <is>
-          <t>toekomst/scholing/index.html</t>
-        </is>
-      </c>
       <c r="R2093" t="inlineStr">
         <is>
           <t>live</t>
@@ -87619,11 +85854,6 @@
           <t>Soevereiniteit als cyclus</t>
         </is>
       </c>
-      <c r="I2094" t="inlineStr">
-        <is>
-          <t>soevereiniteit-als-cyclus/index.html</t>
-        </is>
-      </c>
       <c r="R2094" t="inlineStr">
         <is>
           <t>live</t>
@@ -87705,11 +85935,6 @@
           <t>Toekomst</t>
         </is>
       </c>
-      <c r="I2096" t="inlineStr">
-        <is>
-          <t>toekomst/index.html</t>
-        </is>
-      </c>
       <c r="R2096" t="inlineStr">
         <is>
           <t>live</t>
@@ -87834,11 +86059,6 @@
           <t>Van leerfabriek naar leerwerkplaats</t>
         </is>
       </c>
-      <c r="I2099" t="inlineStr">
-        <is>
-          <t>editie-1/onderwijs.html</t>
-        </is>
-      </c>
       <c r="R2099" t="inlineStr">
         <is>
           <t>live</t>
@@ -88087,11 +86307,6 @@
           <t>De eerste gemeente</t>
         </is>
       </c>
-      <c r="I2105" t="inlineStr">
-        <is>
-          <t>de-eerste-gemeente/index.html</t>
-        </is>
-      </c>
       <c r="R2105" t="inlineStr">
         <is>
           <t>live</t>
@@ -88130,11 +86345,6 @@
           <t>De halve gemeente</t>
         </is>
       </c>
-      <c r="I2106" t="inlineStr">
-        <is>
-          <t>de-halve-gemeente/index.html</t>
-        </is>
-      </c>
       <c r="R2106" t="inlineStr">
         <is>
           <t>live</t>
@@ -88297,11 +86507,6 @@
           <t>Gevolgenkaart — Nederland</t>
         </is>
       </c>
-      <c r="I2110" t="inlineStr">
-        <is>
-          <t>gevolgenkaart-nl/index.html</t>
-        </is>
-      </c>
       <c r="R2110" t="inlineStr">
         <is>
           <t>live</t>
@@ -88421,11 +86626,6 @@
           <t>Nederland · Toekomst</t>
         </is>
       </c>
-      <c r="I2113" t="inlineStr">
-        <is>
-          <t>toekomst/overheden/nederland/index.html</t>
-        </is>
-      </c>
       <c r="R2113" t="inlineStr">
         <is>
           <t>live</t>
@@ -90816,11 +89016,6 @@
           <t>Wat er nu al ligt</t>
         </is>
       </c>
-      <c r="I2173" t="inlineStr">
-        <is>
-          <t>editie-1/technische-oplossingen.html</t>
-        </is>
-      </c>
       <c r="R2173" t="inlineStr">
         <is>
           <t>live</t>
@@ -90859,11 +89054,6 @@
           <t>七つ道具 — Zeven gereedschappen</t>
         </is>
       </c>
-      <c r="I2174" t="inlineStr">
-        <is>
-          <t>editie-5/artikel-01-zeven-gereedschappen.html</t>
-        </is>
-      </c>
       <c r="R2174" t="inlineStr">
         <is>
           <t>live</t>
@@ -91598,11 +89788,6 @@
           <t>Wie zijn opbouwers wegjaagt</t>
         </is>
       </c>
-      <c r="I2192" t="inlineStr">
-        <is>
-          <t>opbouwers-wegjagen/index.html</t>
-        </is>
-      </c>
       <c r="R2192" t="inlineStr">
         <is>
           <t>live</t>
@@ -91679,11 +89864,6 @@
           <t>Achter de Cijfers</t>
         </is>
       </c>
-      <c r="I2194" t="inlineStr">
-        <is>
-          <t>onderzoek/index.html</t>
-        </is>
-      </c>
       <c r="R2194" t="inlineStr">
         <is>
           <t>live</t>
@@ -91722,11 +89902,6 @@
           <t>Dossiers</t>
         </is>
       </c>
-      <c r="I2195" t="inlineStr">
-        <is>
-          <t>dossiers/index.html</t>
-        </is>
-      </c>
       <c r="R2195" t="inlineStr">
         <is>
           <t>live</t>
@@ -91765,11 +89940,6 @@
           <t>EU: BBP, Reële Lonen en de Overheidsmultiplicator</t>
         </is>
       </c>
-      <c r="I2196" t="inlineStr">
-        <is>
-          <t>onderzoek/eu-multiplicator.html</t>
-        </is>
-      </c>
       <c r="R2196" t="inlineStr">
         <is>
           <t>live</t>
@@ -91980,11 +90150,6 @@
           <t>Is Nederland op weg naar ontwikkelingslandstatus?</t>
         </is>
       </c>
-      <c r="I2201" t="inlineStr">
-        <is>
-          <t>onderzoek/ontwikkelingslandstatus.html</t>
-        </is>
-      </c>
       <c r="R2201" t="inlineStr">
         <is>
           <t>live</t>
@@ -92066,11 +90231,6 @@
           <t>Vortex-Hair™ Adaptive Dimple Golf Ball — Dossier</t>
         </is>
       </c>
-      <c r="I2203" t="inlineStr">
-        <is>
-          <t>dossiers/vortex-hair.html</t>
-        </is>
-      </c>
       <c r="R2203" t="inlineStr">
         <is>
           <t>live</t>
@@ -92147,11 +90307,6 @@
           <t>Archief</t>
         </is>
       </c>
-      <c r="I2205" t="inlineStr">
-        <is>
-          <t>archief.html</t>
-        </is>
-      </c>
       <c r="R2205" t="inlineStr">
         <is>
           <t>live</t>
@@ -92190,11 +90345,6 @@
           <t>Bedankt — controleer uw inbox</t>
         </is>
       </c>
-      <c r="I2206" t="inlineStr">
-        <is>
-          <t>bedankt.html</t>
-        </is>
-      </c>
       <c r="R2206" t="inlineStr">
         <is>
           <t>live</t>
@@ -92271,11 +90421,6 @@
           <t>Het Open Vizier verder dragen</t>
         </is>
       </c>
-      <c r="I2208" t="inlineStr">
-        <is>
-          <t>delen.html</t>
-        </is>
-      </c>
       <c r="R2208" t="inlineStr">
         <is>
           <t>live</t>
@@ -92352,11 +90497,6 @@
           <t>Hoe u meedoet aan de discussie</t>
         </is>
       </c>
-      <c r="I2210" t="inlineStr">
-        <is>
-          <t>editie-1/discussie.html</t>
-        </is>
-      </c>
       <c r="R2210" t="inlineStr">
         <is>
           <t>live</t>
@@ -92395,11 +90535,6 @@
           <t>Navigatie</t>
         </is>
       </c>
-      <c r="I2211" t="inlineStr">
-        <is>
-          <t>navigatie.html</t>
-        </is>
-      </c>
       <c r="R2211" t="inlineStr">
         <is>
           <t>live</t>
@@ -92438,11 +90573,6 @@
           <t>Op de hoogte blijven</t>
         </is>
       </c>
-      <c r="I2212" t="inlineStr">
-        <is>
-          <t>op-de-hoogte.html</t>
-        </is>
-      </c>
       <c r="R2212" t="inlineStr">
         <is>
           <t>live</t>
@@ -92481,11 +90611,6 @@
           <t>Over deze krant</t>
         </is>
       </c>
-      <c r="I2213" t="inlineStr">
-        <is>
-          <t>over.html</t>
-        </is>
-      </c>
       <c r="R2213" t="inlineStr">
         <is>
           <t>live</t>
@@ -92567,11 +90692,6 @@
           <t>Structuur — Beheer</t>
         </is>
       </c>
-      <c r="I2215" t="inlineStr">
-        <is>
-          <t>structuur.html</t>
-        </is>
-      </c>
       <c r="R2215" t="inlineStr">
         <is>
           <t>live</t>
@@ -92651,11 +90771,6 @@
       <c r="F2217" t="inlineStr">
         <is>
           <t>Waarom deze krant?</t>
-        </is>
-      </c>
-      <c r="I2217" t="inlineStr">
-        <is>
-          <t>editie-1/voorwoord.html</t>
         </is>
       </c>
       <c r="R2217" t="inlineStr">

</xml_diff>

<commit_message>
Publish: Juncao-artikel "De overheid koos de duurste weg" + hero + banner + menu (X.7.17 alle 8 talen)
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR2313"/>
+  <dimension ref="A2:AR2321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -94823,6 +94823,350 @@
         <v>1</v>
       </c>
     </row>
+    <row r="2314">
+      <c r="B2314" t="inlineStr">
+        <is>
+          <t>1.7.17</t>
+        </is>
+      </c>
+      <c r="C2314" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="D2314" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2314" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2314" t="inlineStr">
+        <is>
+          <t>De overheid koos de duurste weg — en gaat er nog steeds op door</t>
+        </is>
+      </c>
+      <c r="I2314" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-overheid-koos-de-duurste-weg.html</t>
+        </is>
+      </c>
+      <c r="R2314" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2314" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2314" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2315">
+      <c r="B2315" t="inlineStr">
+        <is>
+          <t>2.7.17</t>
+        </is>
+      </c>
+      <c r="C2315" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="D2315" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2315" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2315" t="inlineStr">
+        <is>
+          <t>Die Regierung wählte den teuersten Weg — und macht damit weiter</t>
+        </is>
+      </c>
+      <c r="I2315" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-overheid-koos-de-duurste-weg.html</t>
+        </is>
+      </c>
+      <c r="R2315" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2315" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2315" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2316">
+      <c r="B2316" t="inlineStr">
+        <is>
+          <t>3.7.17</t>
+        </is>
+      </c>
+      <c r="C2316" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="D2316" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2316" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2316" t="inlineStr">
+        <is>
+          <t>The government chose the most expensive path — and keeps going</t>
+        </is>
+      </c>
+      <c r="I2316" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-overheid-koos-de-duurste-weg.html</t>
+        </is>
+      </c>
+      <c r="R2316" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2316" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2316" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2317">
+      <c r="B2317" t="inlineStr">
+        <is>
+          <t>4.7.17</t>
+        </is>
+      </c>
+      <c r="C2317" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="D2317" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2317" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2317" t="inlineStr">
+        <is>
+          <t>Правительство выбрало самый дорогой путь — и продолжает по нему идти</t>
+        </is>
+      </c>
+      <c r="I2317" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-overheid-koos-de-duurste-weg.html</t>
+        </is>
+      </c>
+      <c r="R2317" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2317" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2317" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2318">
+      <c r="B2318" t="inlineStr">
+        <is>
+          <t>5.7.17</t>
+        </is>
+      </c>
+      <c r="C2318" t="inlineStr">
+        <is>
+          <t>5.7</t>
+        </is>
+      </c>
+      <c r="D2318" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="E2318" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2318" t="inlineStr">
+        <is>
+          <t>Le gouvernement a choisi la voie la plus coûteuse — et il continue</t>
+        </is>
+      </c>
+      <c r="I2318" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-overheid-koos-de-duurste-weg.html</t>
+        </is>
+      </c>
+      <c r="R2318" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2318" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2318" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2319">
+      <c r="B2319" t="inlineStr">
+        <is>
+          <t>6.7.17</t>
+        </is>
+      </c>
+      <c r="C2319" t="inlineStr">
+        <is>
+          <t>6.7</t>
+        </is>
+      </c>
+      <c r="D2319" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="E2319" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2319" t="inlineStr">
+        <is>
+          <t>El gobierno eligió el camino más caro — y sigue por él</t>
+        </is>
+      </c>
+      <c r="I2319" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-overheid-koos-de-duurste-weg.html</t>
+        </is>
+      </c>
+      <c r="R2319" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2319" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2319" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2320">
+      <c r="B2320" t="inlineStr">
+        <is>
+          <t>7.7.17</t>
+        </is>
+      </c>
+      <c r="C2320" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
+      </c>
+      <c r="D2320" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="E2320" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2320" t="inlineStr">
+        <is>
+          <t>Il governo ha scelto la via più costosa — e continua a percorrerla</t>
+        </is>
+      </c>
+      <c r="I2320" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-overheid-koos-de-duurste-weg.html</t>
+        </is>
+      </c>
+      <c r="R2320" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2320" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2320" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2321">
+      <c r="B2321" t="inlineStr">
+        <is>
+          <t>8.7.17</t>
+        </is>
+      </c>
+      <c r="C2321" t="inlineStr">
+        <is>
+          <t>8.7</t>
+        </is>
+      </c>
+      <c r="D2321" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="E2321" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2321" t="inlineStr">
+        <is>
+          <t>O governo escolheu o caminho mais caro — e continua nele</t>
+        </is>
+      </c>
+      <c r="I2321" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-overheid-koos-de-duurste-weg.html</t>
+        </is>
+      </c>
+      <c r="R2321" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2321" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2321" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B2:AR65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Publish De Plantroute (v7 vol-LCA): artikel + hero + banner + menu X.7.18 alle 8 talen
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR2321"/>
+  <dimension ref="A2:AR2329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -95167,6 +95167,350 @@
         <v>1</v>
       </c>
     </row>
+    <row r="2322">
+      <c r="B2322" t="inlineStr">
+        <is>
+          <t>1.7.18</t>
+        </is>
+      </c>
+      <c r="C2322" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="D2322" t="inlineStr">
+        <is>
+          <t>nl</t>
+        </is>
+      </c>
+      <c r="E2322" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2322" t="inlineStr">
+        <is>
+          <t>De Plantroute — de enige route die werkt</t>
+        </is>
+      </c>
+      <c r="I2322" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-plantroute.html</t>
+        </is>
+      </c>
+      <c r="R2322" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2322" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2322" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2323">
+      <c r="B2323" t="inlineStr">
+        <is>
+          <t>2.7.18</t>
+        </is>
+      </c>
+      <c r="C2323" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="D2323" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2323" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2323" t="inlineStr">
+        <is>
+          <t>Die Pflanzenroute — die einzige Route, die funktioniert</t>
+        </is>
+      </c>
+      <c r="I2323" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-plantroute.html</t>
+        </is>
+      </c>
+      <c r="R2323" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2323" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2323" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2324">
+      <c r="B2324" t="inlineStr">
+        <is>
+          <t>3.7.18</t>
+        </is>
+      </c>
+      <c r="C2324" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="D2324" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2324" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2324" t="inlineStr">
+        <is>
+          <t>The Plant Route — the only route that works</t>
+        </is>
+      </c>
+      <c r="I2324" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-plantroute.html</t>
+        </is>
+      </c>
+      <c r="R2324" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2324" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2324" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2325">
+      <c r="B2325" t="inlineStr">
+        <is>
+          <t>4.7.18</t>
+        </is>
+      </c>
+      <c r="C2325" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="D2325" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2325" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2325" t="inlineStr">
+        <is>
+          <t>Растительный путь — единственный путь, который работает</t>
+        </is>
+      </c>
+      <c r="I2325" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-plantroute.html</t>
+        </is>
+      </c>
+      <c r="R2325" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2325" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2325" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2326">
+      <c r="B2326" t="inlineStr">
+        <is>
+          <t>5.7.18</t>
+        </is>
+      </c>
+      <c r="C2326" t="inlineStr">
+        <is>
+          <t>5.7</t>
+        </is>
+      </c>
+      <c r="D2326" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="E2326" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2326" t="inlineStr">
+        <is>
+          <t>La Voie Végétale — la seule voie qui fonctionne</t>
+        </is>
+      </c>
+      <c r="I2326" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-plantroute.html</t>
+        </is>
+      </c>
+      <c r="R2326" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2326" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2326" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2327">
+      <c r="B2327" t="inlineStr">
+        <is>
+          <t>6.7.18</t>
+        </is>
+      </c>
+      <c r="C2327" t="inlineStr">
+        <is>
+          <t>6.7</t>
+        </is>
+      </c>
+      <c r="D2327" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="E2327" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2327" t="inlineStr">
+        <is>
+          <t>La Vía Vegetal — la única vía que funciona</t>
+        </is>
+      </c>
+      <c r="I2327" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-plantroute.html</t>
+        </is>
+      </c>
+      <c r="R2327" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2327" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2327" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2328">
+      <c r="B2328" t="inlineStr">
+        <is>
+          <t>7.7.18</t>
+        </is>
+      </c>
+      <c r="C2328" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
+      </c>
+      <c r="D2328" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="E2328" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2328" t="inlineStr">
+        <is>
+          <t>La Via Vegetale — l'unica via che funziona</t>
+        </is>
+      </c>
+      <c r="I2328" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-plantroute.html</t>
+        </is>
+      </c>
+      <c r="R2328" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2328" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2328" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2329">
+      <c r="B2329" t="inlineStr">
+        <is>
+          <t>8.7.18</t>
+        </is>
+      </c>
+      <c r="C2329" t="inlineStr">
+        <is>
+          <t>8.7</t>
+        </is>
+      </c>
+      <c r="D2329" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="E2329" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2329" t="inlineStr">
+        <is>
+          <t>A Via Vegetal — a única via que funciona</t>
+        </is>
+      </c>
+      <c r="I2329" t="inlineStr">
+        <is>
+          <t>wat-opkomt/de-plantroute.html</t>
+        </is>
+      </c>
+      <c r="R2329" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2329" t="n">
+        <v>16</v>
+      </c>
+      <c r="T2329" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B2:AR65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Xlsx: URLs voor 6 nieuw-vertaalde artikelen in taal-menu ingevuld waar leeg
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AR2329"/>
+  <dimension ref="B2:AR2329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -14537,6 +14537,11 @@
           <t>Ruimte voor het oergevoel</t>
         </is>
       </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>wat-opkomt/manifest-ruimte-voor-het-oergevoel.html</t>
+        </is>
+      </c>
       <c r="R324" t="inlineStr">
         <is>
           <t>live</t>
@@ -25928,6 +25933,11 @@
           <t>Ruimte voor het oergevoel</t>
         </is>
       </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>wat-opkomt/manifest-ruimte-voor-het-oergevoel.html</t>
+        </is>
+      </c>
       <c r="R602" t="inlineStr">
         <is>
           <t>live</t>
@@ -37314,6 +37324,11 @@
           <t>Ruimte voor het oergevoel</t>
         </is>
       </c>
+      <c r="I880" t="inlineStr">
+        <is>
+          <t>wat-opkomt/manifest-ruimte-voor-het-oergevoel.html</t>
+        </is>
+      </c>
       <c r="R880" t="inlineStr">
         <is>
           <t>live</t>
@@ -48485,6 +48500,11 @@
           <t>Ruimte voor het oergevoel</t>
         </is>
       </c>
+      <c r="I1158" t="inlineStr">
+        <is>
+          <t>wat-opkomt/manifest-ruimte-voor-het-oergevoel.html</t>
+        </is>
+      </c>
       <c r="R1158" t="inlineStr">
         <is>
           <t>live</t>
@@ -50194,6 +50214,11 @@
           <t>Het klimaatdividend</t>
         </is>
       </c>
+      <c r="I1201" t="inlineStr">
+        <is>
+          <t>wat-opkomt/klimaatdividend.html</t>
+        </is>
+      </c>
       <c r="R1201" t="inlineStr">
         <is>
           <t>live</t>
@@ -56044,6 +56069,11 @@
       <c r="F1350" t="inlineStr">
         <is>
           <t>Het klimaatdividend</t>
+        </is>
+      </c>
+      <c r="I1350" t="inlineStr">
+        <is>
+          <t>wat-opkomt/klimaatdividend.html</t>
         </is>
       </c>
       <c r="R1350" t="inlineStr">

</xml_diff>

<commit_message>
Xlsx: 29 taal-URLs uitgelijnd op werkelijk aanwezige HTML-bestanden
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -16333,7 +16333,7 @@
       </c>
       <c r="I367" t="inlineStr">
         <is>
-          <t>was-aufkommt/klimadividende.html</t>
+          <t>wat-opkomt/klimaatdividend.html</t>
         </is>
       </c>
       <c r="R367" t="inlineStr">
@@ -21184,7 +21184,7 @@
       </c>
       <c r="I484" t="inlineStr">
         <is>
-          <t>was-aufkommt/mappa-tal-konsegwenzi.html</t>
+          <t>wat-opkomt/mappa-tal-konsegwenzi.html</t>
         </is>
       </c>
       <c r="R484" t="inlineStr">
@@ -22495,7 +22495,7 @@
       </c>
       <c r="I516" t="inlineStr">
         <is>
-          <t>was-aufkommt/klimadividende.html</t>
+          <t>wat-opkomt/klimaatdividend.html</t>
         </is>
       </c>
       <c r="R516" t="inlineStr">
@@ -27729,7 +27729,7 @@
       </c>
       <c r="I645" t="inlineStr">
         <is>
-          <t>what-surfaces/climate-dividend.html</t>
+          <t>wat-opkomt/klimaatdividend.html</t>
         </is>
       </c>
       <c r="R645" t="inlineStr">
@@ -32580,7 +32580,7 @@
       </c>
       <c r="I762" t="inlineStr">
         <is>
-          <t>what-surfaces/mappa-tal-konsegwenzi.html</t>
+          <t>wat-opkomt/mappa-tal-konsegwenzi.html</t>
         </is>
       </c>
       <c r="R762" t="inlineStr">
@@ -33891,7 +33891,7 @@
       </c>
       <c r="I794" t="inlineStr">
         <is>
-          <t>what-surfaces/climate-dividend.html</t>
+          <t>wat-opkomt/klimaatdividend.html</t>
         </is>
       </c>
       <c r="R794" t="inlineStr">
@@ -39095,7 +39095,7 @@
       </c>
       <c r="I923" t="inlineStr">
         <is>
-          <t>chto-vsplyvaet/klimaatdividend.html</t>
+          <t>wat-opkomt/klimaatdividend.html</t>
         </is>
       </c>
       <c r="R923" t="inlineStr">
@@ -43801,7 +43801,7 @@
       </c>
       <c r="I1040" t="inlineStr">
         <is>
-          <t>chto-vsplyvaet/mappa-tal-konsegwenzi.html</t>
+          <t>wat-opkomt/mappa-tal-konsegwenzi.html</t>
         </is>
       </c>
       <c r="R1040" t="inlineStr">
@@ -45112,7 +45112,7 @@
       </c>
       <c r="I1072" t="inlineStr">
         <is>
-          <t>chto-vsplyvaet/klimaatdividend.html</t>
+          <t>wat-opkomt/klimaatdividend.html</t>
         </is>
       </c>
       <c r="R1072" t="inlineStr">
@@ -54812,7 +54812,7 @@
       </c>
       <c r="I1318" t="inlineStr">
         <is>
-          <t>ce-qui-emerge/mappa-tal-konsegwenzi.html</t>
+          <t>wat-opkomt/mappa-tal-konsegwenzi.html</t>
         </is>
       </c>
       <c r="R1318" t="inlineStr">
@@ -59468,7 +59468,7 @@
       </c>
       <c r="I1436" t="inlineStr">
         <is>
-          <t>lo-que-emerge/manifest-ruimte-voor-het-oergevoel.html</t>
+          <t>wat-opkomt/manifest-ruimte-voor-het-oergevoel.html</t>
         </is>
       </c>
       <c r="R1436" t="inlineStr">
@@ -61232,7 +61232,7 @@
       </c>
       <c r="I1479" t="inlineStr">
         <is>
-          <t>lo-que-emerge/klimaatdividend.html</t>
+          <t>wat-opkomt/klimaatdividend.html</t>
         </is>
       </c>
       <c r="R1479" t="inlineStr">
@@ -65923,7 +65923,7 @@
       </c>
       <c r="I1596" t="inlineStr">
         <is>
-          <t>lo-que-emerge/mappa-tal-konsegwenzi.html</t>
+          <t>wat-opkomt/mappa-tal-konsegwenzi.html</t>
         </is>
       </c>
       <c r="R1596" t="inlineStr">
@@ -67199,7 +67199,7 @@
       </c>
       <c r="I1628" t="inlineStr">
         <is>
-          <t>lo-que-emerge/klimaatdividend.html</t>
+          <t>wat-opkomt/klimaatdividend.html</t>
         </is>
       </c>
       <c r="R1628" t="inlineStr">
@@ -70609,7 +70609,7 @@
       </c>
       <c r="I1714" t="inlineStr">
         <is>
-          <t>cio-che-emerge/manifest-ruimte-voor-het-oergevoel.html</t>
+          <t>wat-opkomt/manifest-ruimte-voor-het-oergevoel.html</t>
         </is>
       </c>
       <c r="R1714" t="inlineStr">
@@ -72383,7 +72383,7 @@
       </c>
       <c r="I1757" t="inlineStr">
         <is>
-          <t>cio-che-emerge/klimaatdividend.html</t>
+          <t>wat-opkomt/klimaatdividend.html</t>
         </is>
       </c>
       <c r="R1757" t="inlineStr">
@@ -77079,7 +77079,7 @@
       </c>
       <c r="I1874" t="inlineStr">
         <is>
-          <t>cio-che-emerge/mappa-tal-konsegwenzi.html</t>
+          <t>wat-opkomt/mappa-tal-konsegwenzi.html</t>
         </is>
       </c>
       <c r="R1874" t="inlineStr">
@@ -78355,7 +78355,7 @@
       </c>
       <c r="I1906" t="inlineStr">
         <is>
-          <t>cio-che-emerge/klimaatdividend.html</t>
+          <t>wat-opkomt/klimaatdividend.html</t>
         </is>
       </c>
       <c r="R1906" t="inlineStr">
@@ -81765,7 +81765,7 @@
       </c>
       <c r="I1992" t="inlineStr">
         <is>
-          <t>o-que-emerge/manifest-ruimte-voor-het-oergevoel.html</t>
+          <t>wat-opkomt/manifest-ruimte-voor-het-oergevoel.html</t>
         </is>
       </c>
       <c r="R1992" t="inlineStr">
@@ -83519,7 +83519,7 @@
       </c>
       <c r="I2035" t="inlineStr">
         <is>
-          <t>o-que-emerge/klimaatdividend.html</t>
+          <t>wat-opkomt/klimaatdividend.html</t>
         </is>
       </c>
       <c r="R2035" t="inlineStr">
@@ -88215,7 +88215,7 @@
       </c>
       <c r="I2152" t="inlineStr">
         <is>
-          <t>o-que-emerge/mappa-tal-konsegwenzi.html</t>
+          <t>wat-opkomt/mappa-tal-konsegwenzi.html</t>
         </is>
       </c>
       <c r="R2152" t="inlineStr">
@@ -89491,7 +89491,7 @@
       </c>
       <c r="I2184" t="inlineStr">
         <is>
-          <t>o-que-emerge/klimaatdividend.html</t>
+          <t>wat-opkomt/klimaatdividend.html</t>
         </is>
       </c>
       <c r="R2184" t="inlineStr">
@@ -91868,7 +91868,7 @@
       </c>
       <c r="I2243" t="inlineStr">
         <is>
-          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+          <t>wat-opkomt/klimaat-de-echte-analyse.html</t>
         </is>
       </c>
       <c r="R2243" t="inlineStr">
@@ -91911,7 +91911,7 @@
       </c>
       <c r="I2244" t="inlineStr">
         <is>
-          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+          <t>wat-opkomt/klimaat-de-echte-analyse.html</t>
         </is>
       </c>
       <c r="R2244" t="inlineStr">
@@ -91954,7 +91954,7 @@
       </c>
       <c r="I2245" t="inlineStr">
         <is>
-          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+          <t>wat-opkomt/klimaat-de-echte-analyse.html</t>
         </is>
       </c>
       <c r="R2245" t="inlineStr">
@@ -91997,7 +91997,7 @@
       </c>
       <c r="I2246" t="inlineStr">
         <is>
-          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+          <t>wat-opkomt/klimaat-de-echte-analyse.html</t>
         </is>
       </c>
       <c r="R2246" t="inlineStr">
@@ -92040,7 +92040,7 @@
       </c>
       <c r="I2247" t="inlineStr">
         <is>
-          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+          <t>wat-opkomt/klimaat-de-echte-analyse.html</t>
         </is>
       </c>
       <c r="R2247" t="inlineStr">
@@ -92083,7 +92083,7 @@
       </c>
       <c r="I2248" t="inlineStr">
         <is>
-          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+          <t>wat-opkomt/klimaat-de-echte-analyse.html</t>
         </is>
       </c>
       <c r="R2248" t="inlineStr">
@@ -92126,7 +92126,7 @@
       </c>
       <c r="I2249" t="inlineStr">
         <is>
-          <t>/nl/wat-opkomt/klimaat-de-echte-analyse.html</t>
+          <t>wat-opkomt/klimaat-de-echte-analyse.html</t>
         </is>
       </c>
       <c r="R2249" t="inlineStr">

</xml_diff>

<commit_message>
Xlsx: 56 taal-URLs top 10 recent artikelen op wat-opkomt/<slug>.html gezet
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -13066,7 +13066,7 @@
       </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>was-aufkommt/erst-das-reptil.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R288" t="inlineStr">
@@ -14281,7 +14281,7 @@
       </c>
       <c r="I318" t="inlineStr">
         <is>
-          <t>was-aufkommt/erst-das-reptil.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R318" t="inlineStr">
@@ -15541,7 +15541,7 @@
       </c>
       <c r="I348" t="inlineStr">
         <is>
-          <t>was-aufkommt/frankreich-revolutionaerer-moment.html</t>
+          <t>wat-opkomt/frankrijk-revolutionair-moment.html</t>
         </is>
       </c>
       <c r="R348" t="inlineStr">
@@ -16290,7 +16290,7 @@
       </c>
       <c r="I366" t="inlineStr">
         <is>
-          <t>was-aufkommt/erbschaftswelle-240-milliarden.html</t>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
         </is>
       </c>
       <c r="R366" t="inlineStr">
@@ -20248,7 +20248,7 @@
       </c>
       <c r="I462" t="inlineStr">
         <is>
-          <t>was-aufkommt/die-natur-angepasste-analyse.html</t>
+          <t>wat-opkomt/europa-hoeft-geen-schadekaart-te-zijn.html</t>
         </is>
       </c>
       <c r="R462" t="inlineStr">
@@ -20291,7 +20291,7 @@
       </c>
       <c r="I463" t="inlineStr">
         <is>
-          <t>was-aufkommt/europa-erneut.html</t>
+          <t>wat-opkomt/europa-opnieuw.html</t>
         </is>
       </c>
       <c r="R463" t="inlineStr">
@@ -22452,7 +22452,7 @@
       </c>
       <c r="I515" t="inlineStr">
         <is>
-          <t>was-aufkommt/erbschaftswelle-240-milliarden.html</t>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
         </is>
       </c>
       <c r="R515" t="inlineStr">
@@ -22733,7 +22733,7 @@
       </c>
       <c r="I522" t="inlineStr">
         <is>
-          <t>was-aufkommt/loch-im-boden.html</t>
+          <t>wat-opkomt/gat-in-de-grond.html</t>
         </is>
       </c>
       <c r="R522" t="inlineStr">
@@ -24462,7 +24462,7 @@
       </c>
       <c r="I566" t="inlineStr">
         <is>
-          <t>what-surfaces/first-the-reptile.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R566" t="inlineStr">
@@ -25677,7 +25677,7 @@
       </c>
       <c r="I596" t="inlineStr">
         <is>
-          <t>what-surfaces/first-the-reptile.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R596" t="inlineStr">
@@ -26937,7 +26937,7 @@
       </c>
       <c r="I626" t="inlineStr">
         <is>
-          <t>what-surfaces/france-revolutionary-moment.html</t>
+          <t>wat-opkomt/frankrijk-revolutionair-moment.html</t>
         </is>
       </c>
       <c r="R626" t="inlineStr">
@@ -27686,7 +27686,7 @@
       </c>
       <c r="I644" t="inlineStr">
         <is>
-          <t>what-surfaces/inheritance-wave-240-billion.html</t>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
         </is>
       </c>
       <c r="R644" t="inlineStr">
@@ -31644,7 +31644,7 @@
       </c>
       <c r="I740" t="inlineStr">
         <is>
-          <t>what-surfaces/europe-need-not-be-a-damage-map.html</t>
+          <t>wat-opkomt/europa-hoeft-geen-schadekaart-te-zijn.html</t>
         </is>
       </c>
       <c r="R740" t="inlineStr">
@@ -31687,7 +31687,7 @@
       </c>
       <c r="I741" t="inlineStr">
         <is>
-          <t>what-surfaces/europe-anew.html</t>
+          <t>wat-opkomt/europa-opnieuw.html</t>
         </is>
       </c>
       <c r="R741" t="inlineStr">
@@ -33848,7 +33848,7 @@
       </c>
       <c r="I793" t="inlineStr">
         <is>
-          <t>what-surfaces/inheritance-wave-240-billion.html</t>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
         </is>
       </c>
       <c r="R793" t="inlineStr">
@@ -34129,7 +34129,7 @@
       </c>
       <c r="I800" t="inlineStr">
         <is>
-          <t>what-surfaces/hole-in-the-ground.html</t>
+          <t>wat-opkomt/gat-in-de-grond.html</t>
         </is>
       </c>
       <c r="R800" t="inlineStr">
@@ -35858,7 +35858,7 @@
       </c>
       <c r="I844" t="inlineStr">
         <is>
-          <t>chto-vsplyvaet/snachala-reptiliya.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R844" t="inlineStr">
@@ -37068,7 +37068,7 @@
       </c>
       <c r="I874" t="inlineStr">
         <is>
-          <t>chto-vsplyvaet/snachala-reptiliya.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R874" t="inlineStr">
@@ -38321,6 +38321,11 @@
           <t>Frankrijk — revolutionair moment</t>
         </is>
       </c>
+      <c r="I904" t="inlineStr">
+        <is>
+          <t>wat-opkomt/frankrijk-revolutionair-moment.html</t>
+        </is>
+      </c>
       <c r="R904" t="inlineStr">
         <is>
           <t>live</t>
@@ -39052,7 +39057,7 @@
       </c>
       <c r="I922" t="inlineStr">
         <is>
-          <t>chto-vsplyvaet/erfenisgolf-240-miljard.html</t>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
         </is>
       </c>
       <c r="R922" t="inlineStr">
@@ -42950,7 +42955,7 @@
       </c>
       <c r="I1018" t="inlineStr">
         <is>
-          <t>chto-vsplyvaet/europa-hoeft-geen-schadekaart-te-zijn.html</t>
+          <t>wat-opkomt/europa-hoeft-geen-schadekaart-te-zijn.html</t>
         </is>
       </c>
       <c r="R1018" t="inlineStr">
@@ -42993,7 +42998,7 @@
       </c>
       <c r="I1019" t="inlineStr">
         <is>
-          <t>chto-vsplyvaet/europa-opnieuw.html</t>
+          <t>wat-opkomt/europa-opnieuw.html</t>
         </is>
       </c>
       <c r="R1019" t="inlineStr">
@@ -45069,7 +45074,7 @@
       </c>
       <c r="I1071" t="inlineStr">
         <is>
-          <t>chto-vsplyvaet/erfenisgolf-240-miljard.html</t>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
         </is>
       </c>
       <c r="R1071" t="inlineStr">
@@ -45350,7 +45355,7 @@
       </c>
       <c r="I1078" t="inlineStr">
         <is>
-          <t>chto-vsplyvaet/gat-in-de-grond.html</t>
+          <t>wat-opkomt/gat-in-de-grond.html</t>
         </is>
       </c>
       <c r="R1078" t="inlineStr">
@@ -47074,7 +47079,7 @@
       </c>
       <c r="I1122" t="inlineStr">
         <is>
-          <t>ce-qui-emerge/d-abord-le-reptile.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R1122" t="inlineStr">
@@ -48269,7 +48274,7 @@
       </c>
       <c r="I1152" t="inlineStr">
         <is>
-          <t>ce-qui-emerge/d-abord-le-reptile.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R1152" t="inlineStr">
@@ -49482,6 +49487,11 @@
           <t>Frankrijk — revolutionair moment</t>
         </is>
       </c>
+      <c r="I1182" t="inlineStr">
+        <is>
+          <t>wat-opkomt/frankrijk-revolutionair-moment.html</t>
+        </is>
+      </c>
       <c r="R1182" t="inlineStr">
         <is>
           <t>live</t>
@@ -50176,6 +50186,11 @@
           <t>Erfenisgolf — 240 miljard</t>
         </is>
       </c>
+      <c r="I1200" t="inlineStr">
+        <is>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
+        </is>
+      </c>
       <c r="R1200" t="inlineStr">
         <is>
           <t>live</t>
@@ -53966,7 +53981,7 @@
       </c>
       <c r="I1296" t="inlineStr">
         <is>
-          <t>ce-qui-emerge/gevolgenkaart-iii-stille-analyse.html</t>
+          <t>wat-opkomt/europa-hoeft-geen-schadekaart-te-zijn.html</t>
         </is>
       </c>
       <c r="R1296" t="inlineStr">
@@ -54007,6 +54022,11 @@
           <t>Europa opnieuw</t>
         </is>
       </c>
+      <c r="I1297" t="inlineStr">
+        <is>
+          <t>wat-opkomt/europa-opnieuw.html</t>
+        </is>
+      </c>
       <c r="R1297" t="inlineStr">
         <is>
           <t>live</t>
@@ -56033,6 +56053,11 @@
           <t>Erfenisgolf — 240 miljard</t>
         </is>
       </c>
+      <c r="I1349" t="inlineStr">
+        <is>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
+        </is>
+      </c>
       <c r="R1349" t="inlineStr">
         <is>
           <t>live</t>
@@ -56309,6 +56334,11 @@
           <t>Vierhonderdvijftig miljoen voor een gat in de grond</t>
         </is>
       </c>
+      <c r="I1356" t="inlineStr">
+        <is>
+          <t>wat-opkomt/gat-in-de-grond.html</t>
+        </is>
+      </c>
       <c r="R1356" t="inlineStr">
         <is>
           <t>live</t>
@@ -58030,7 +58060,7 @@
       </c>
       <c r="I1400" t="inlineStr">
         <is>
-          <t>lo-que-emerge/primero-el-reptil.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R1400" t="inlineStr">
@@ -59235,7 +59265,7 @@
       </c>
       <c r="I1430" t="inlineStr">
         <is>
-          <t>lo-que-emerge/primero-el-reptil.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R1430" t="inlineStr">
@@ -60458,6 +60488,11 @@
           <t>Frankrijk — revolutionair moment</t>
         </is>
       </c>
+      <c r="I1460" t="inlineStr">
+        <is>
+          <t>wat-opkomt/frankrijk-revolutionair-moment.html</t>
+        </is>
+      </c>
       <c r="R1460" t="inlineStr">
         <is>
           <t>live</t>
@@ -61189,7 +61224,7 @@
       </c>
       <c r="I1478" t="inlineStr">
         <is>
-          <t>lo-que-emerge/erfenisgolf-240-miljard.html</t>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
         </is>
       </c>
       <c r="R1478" t="inlineStr">
@@ -65072,7 +65107,7 @@
       </c>
       <c r="I1574" t="inlineStr">
         <is>
-          <t>lo-que-emerge/europa-hoeft-geen-schadekaart-te-zijn.html</t>
+          <t>wat-opkomt/europa-hoeft-geen-schadekaart-te-zijn.html</t>
         </is>
       </c>
       <c r="R1574" t="inlineStr">
@@ -65115,7 +65150,7 @@
       </c>
       <c r="I1575" t="inlineStr">
         <is>
-          <t>lo-que-emerge/europa-opnieuw.html</t>
+          <t>wat-opkomt/europa-opnieuw.html</t>
         </is>
       </c>
       <c r="R1575" t="inlineStr">
@@ -67156,7 +67191,7 @@
       </c>
       <c r="I1627" t="inlineStr">
         <is>
-          <t>lo-que-emerge/erfenisgolf-240-miljard.html</t>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
         </is>
       </c>
       <c r="R1627" t="inlineStr">
@@ -67442,7 +67477,7 @@
       </c>
       <c r="I1634" t="inlineStr">
         <is>
-          <t>lo-que-emerge/gat-in-de-grond.html</t>
+          <t>wat-opkomt/gat-in-de-grond.html</t>
         </is>
       </c>
       <c r="R1634" t="inlineStr">
@@ -69171,7 +69206,7 @@
       </c>
       <c r="I1678" t="inlineStr">
         <is>
-          <t>cio-che-emerge/prima-il-rettile.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R1678" t="inlineStr">
@@ -70376,7 +70411,7 @@
       </c>
       <c r="I1708" t="inlineStr">
         <is>
-          <t>cio-che-emerge/prima-il-rettile.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R1708" t="inlineStr">
@@ -71606,7 +71641,7 @@
       </c>
       <c r="I1738" t="inlineStr">
         <is>
-          <t>cio-che-emerge/frankrijk-revolutionair-moment.html</t>
+          <t>wat-opkomt/frankrijk-revolutionair-moment.html</t>
         </is>
       </c>
       <c r="R1738" t="inlineStr">
@@ -72340,7 +72375,7 @@
       </c>
       <c r="I1756" t="inlineStr">
         <is>
-          <t>cio-che-emerge/erfenisgolf-240-miljard.html</t>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
         </is>
       </c>
       <c r="R1756" t="inlineStr">
@@ -76228,7 +76263,7 @@
       </c>
       <c r="I1852" t="inlineStr">
         <is>
-          <t>cio-che-emerge/europa-hoeft-geen-schadekaart-te-zijn.html</t>
+          <t>wat-opkomt/europa-hoeft-geen-schadekaart-te-zijn.html</t>
         </is>
       </c>
       <c r="R1852" t="inlineStr">
@@ -76271,7 +76306,7 @@
       </c>
       <c r="I1853" t="inlineStr">
         <is>
-          <t>cio-che-emerge/europa-opnieuw.html</t>
+          <t>wat-opkomt/europa-opnieuw.html</t>
         </is>
       </c>
       <c r="R1853" t="inlineStr">
@@ -78312,7 +78347,7 @@
       </c>
       <c r="I1905" t="inlineStr">
         <is>
-          <t>cio-che-emerge/erfenisgolf-240-miljard.html</t>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
         </is>
       </c>
       <c r="R1905" t="inlineStr">
@@ -78598,7 +78633,7 @@
       </c>
       <c r="I1912" t="inlineStr">
         <is>
-          <t>cio-che-emerge/gat-in-de-grond.html</t>
+          <t>wat-opkomt/gat-in-de-grond.html</t>
         </is>
       </c>
       <c r="R1912" t="inlineStr">
@@ -80327,7 +80362,7 @@
       </c>
       <c r="I1956" t="inlineStr">
         <is>
-          <t>o-que-emerge/primeiro-o-reptil.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R1956" t="inlineStr">
@@ -81532,7 +81567,7 @@
       </c>
       <c r="I1986" t="inlineStr">
         <is>
-          <t>o-que-emerge/primeiro-o-reptil.html</t>
+          <t>wat-opkomt/eerst-het-reptiel.html</t>
         </is>
       </c>
       <c r="R1986" t="inlineStr">
@@ -82742,7 +82777,7 @@
       </c>
       <c r="I2016" t="inlineStr">
         <is>
-          <t>o-que-emerge/frankrijk-revolutionair-moment.html</t>
+          <t>wat-opkomt/frankrijk-revolutionair-moment.html</t>
         </is>
       </c>
       <c r="R2016" t="inlineStr">
@@ -83476,7 +83511,7 @@
       </c>
       <c r="I2034" t="inlineStr">
         <is>
-          <t>o-que-emerge/erfenisgolf-240-miljard.html</t>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
         </is>
       </c>
       <c r="R2034" t="inlineStr">
@@ -87364,7 +87399,7 @@
       </c>
       <c r="I2130" t="inlineStr">
         <is>
-          <t>o-que-emerge/europa-hoeft-geen-schadekaart-te-zijn.html</t>
+          <t>wat-opkomt/europa-hoeft-geen-schadekaart-te-zijn.html</t>
         </is>
       </c>
       <c r="R2130" t="inlineStr">
@@ -87407,7 +87442,7 @@
       </c>
       <c r="I2131" t="inlineStr">
         <is>
-          <t>o-que-emerge/europa-opnieuw.html</t>
+          <t>wat-opkomt/europa-opnieuw.html</t>
         </is>
       </c>
       <c r="R2131" t="inlineStr">
@@ -89448,7 +89483,7 @@
       </c>
       <c r="I2183" t="inlineStr">
         <is>
-          <t>o-que-emerge/erfenisgolf-240-miljard.html</t>
+          <t>wat-opkomt/erfenisgolf-240-miljard.html</t>
         </is>
       </c>
       <c r="R2183" t="inlineStr">
@@ -89734,7 +89769,7 @@
       </c>
       <c r="I2190" t="inlineStr">
         <is>
-          <t>o-que-emerge/gat-in-de-grond.html</t>
+          <t>wat-opkomt/gat-in-de-grond.html</t>
         </is>
       </c>
       <c r="R2190" t="inlineStr">

</xml_diff>

<commit_message>
Xlsx: fix duplicate Volgorde voor artikelen X.7.17 en X.7.18 (waren 16)
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -95850,7 +95850,7 @@
         </is>
       </c>
       <c r="S2314" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T2314" t="b">
         <v>1</v>
@@ -95893,7 +95893,7 @@
         </is>
       </c>
       <c r="S2315" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T2315" t="b">
         <v>1</v>
@@ -95936,7 +95936,7 @@
         </is>
       </c>
       <c r="S2316" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T2316" t="b">
         <v>1</v>
@@ -95979,7 +95979,7 @@
         </is>
       </c>
       <c r="S2317" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T2317" t="b">
         <v>1</v>
@@ -96022,7 +96022,7 @@
         </is>
       </c>
       <c r="S2318" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T2318" t="b">
         <v>1</v>
@@ -96065,7 +96065,7 @@
         </is>
       </c>
       <c r="S2319" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T2319" t="b">
         <v>1</v>
@@ -96108,7 +96108,7 @@
         </is>
       </c>
       <c r="S2320" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T2320" t="b">
         <v>1</v>
@@ -96151,7 +96151,7 @@
         </is>
       </c>
       <c r="S2321" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T2321" t="b">
         <v>1</v>
@@ -96194,7 +96194,7 @@
         </is>
       </c>
       <c r="S2322" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="T2322" t="b">
         <v>1</v>
@@ -96237,7 +96237,7 @@
         </is>
       </c>
       <c r="S2323" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="T2323" t="b">
         <v>1</v>
@@ -96280,7 +96280,7 @@
         </is>
       </c>
       <c r="S2324" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="T2324" t="b">
         <v>1</v>
@@ -96323,7 +96323,7 @@
         </is>
       </c>
       <c r="S2325" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="T2325" t="b">
         <v>1</v>
@@ -96366,7 +96366,7 @@
         </is>
       </c>
       <c r="S2326" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="T2326" t="b">
         <v>1</v>
@@ -96409,7 +96409,7 @@
         </is>
       </c>
       <c r="S2327" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="T2327" t="b">
         <v>1</v>
@@ -96452,7 +96452,7 @@
         </is>
       </c>
       <c r="S2328" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="T2328" t="b">
         <v>1</v>
@@ -96495,7 +96495,7 @@
         </is>
       </c>
       <c r="S2329" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="T2329" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
xlsx: 7 rijen toegevoegd voor gedachte-in-de-kluis (EN/DE/FR/ES/IT/PT/RU)
</commit_message>
<xml_diff>
--- a/nl/_data/vizier.xlsx
+++ b/nl/_data/vizier.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AR2329"/>
+  <dimension ref="A2:AR2336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -96501,6 +96501,412 @@
         <v>1</v>
       </c>
     </row>
+    <row r="2330">
+      <c r="B2330" t="inlineStr">
+        <is>
+          <t>3.7.1</t>
+        </is>
+      </c>
+      <c r="C2330" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="D2330" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="E2330" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2330" t="inlineStr">
+        <is>
+          <t>The thought in the vault</t>
+        </is>
+      </c>
+      <c r="G2330" t="inlineStr">
+        <is>
+          <t>European innovation cannot but withdraw — in defence, in order to survive</t>
+        </is>
+      </c>
+      <c r="H2330" t="inlineStr">
+        <is>
+          <t>European innovation cannot but withdraw — in defence, in order to survive</t>
+        </is>
+      </c>
+      <c r="I2330" t="inlineStr">
+        <is>
+          <t>wat-opkomt/gedachte-in-de-kluis.html</t>
+        </is>
+      </c>
+      <c r="R2330" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2330" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2330" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO2330" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2331">
+      <c r="B2331" t="inlineStr">
+        <is>
+          <t>2.7.1</t>
+        </is>
+      </c>
+      <c r="C2331" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="D2331" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="E2331" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2331" t="inlineStr">
+        <is>
+          <t>Der Gedanke im Tresor</t>
+        </is>
+      </c>
+      <c r="G2331" t="inlineStr">
+        <is>
+          <t>Europäische Innovation kann nicht anders als sich zurückziehen — zur Verteidigung, um zu überleben</t>
+        </is>
+      </c>
+      <c r="H2331" t="inlineStr">
+        <is>
+          <t>Europäische Innovation kann nicht anders als sich zurückziehen — zur Verteidigung, um zu überleben</t>
+        </is>
+      </c>
+      <c r="I2331" t="inlineStr">
+        <is>
+          <t>wat-opkomt/gedachte-in-de-kluis.html</t>
+        </is>
+      </c>
+      <c r="R2331" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2331" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2331" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO2331" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2332">
+      <c r="B2332" t="inlineStr">
+        <is>
+          <t>5.7.1</t>
+        </is>
+      </c>
+      <c r="C2332" t="inlineStr">
+        <is>
+          <t>5.7</t>
+        </is>
+      </c>
+      <c r="D2332" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="E2332" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2332" t="inlineStr">
+        <is>
+          <t>La pensée dans le coffre</t>
+        </is>
+      </c>
+      <c r="G2332" t="inlineStr">
+        <is>
+          <t>L'innovation européenne ne peut que se retirer — en défense, pour survivre</t>
+        </is>
+      </c>
+      <c r="H2332" t="inlineStr">
+        <is>
+          <t>L'innovation européenne ne peut que se retirer — en défense, pour survivre</t>
+        </is>
+      </c>
+      <c r="I2332" t="inlineStr">
+        <is>
+          <t>wat-opkomt/gedachte-in-de-kluis.html</t>
+        </is>
+      </c>
+      <c r="R2332" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2332" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2332" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO2332" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2333">
+      <c r="B2333" t="inlineStr">
+        <is>
+          <t>6.7.1</t>
+        </is>
+      </c>
+      <c r="C2333" t="inlineStr">
+        <is>
+          <t>6.7</t>
+        </is>
+      </c>
+      <c r="D2333" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="E2333" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2333" t="inlineStr">
+        <is>
+          <t>El pensamiento en la caja fuerte</t>
+        </is>
+      </c>
+      <c r="G2333" t="inlineStr">
+        <is>
+          <t>La innovación europea no puede sino retirarse — en defensa, para sobrevivir</t>
+        </is>
+      </c>
+      <c r="H2333" t="inlineStr">
+        <is>
+          <t>La innovación europea no puede sino retirarse — en defensa, para sobrevivir</t>
+        </is>
+      </c>
+      <c r="I2333" t="inlineStr">
+        <is>
+          <t>wat-opkomt/gedachte-in-de-kluis.html</t>
+        </is>
+      </c>
+      <c r="R2333" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2333" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2333" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO2333" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2334">
+      <c r="B2334" t="inlineStr">
+        <is>
+          <t>7.7.1</t>
+        </is>
+      </c>
+      <c r="C2334" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
+      </c>
+      <c r="D2334" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="E2334" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2334" t="inlineStr">
+        <is>
+          <t>Il pensiero nella cassaforte</t>
+        </is>
+      </c>
+      <c r="G2334" t="inlineStr">
+        <is>
+          <t>L'innovazione europea non può che ritirarsi — in difesa, per sopravvivere</t>
+        </is>
+      </c>
+      <c r="H2334" t="inlineStr">
+        <is>
+          <t>L'innovazione europea non può che ritirarsi — in difesa, per sopravvivere</t>
+        </is>
+      </c>
+      <c r="I2334" t="inlineStr">
+        <is>
+          <t>wat-opkomt/gedachte-in-de-kluis.html</t>
+        </is>
+      </c>
+      <c r="R2334" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2334" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2334" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO2334" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2335">
+      <c r="B2335" t="inlineStr">
+        <is>
+          <t>8.7.1</t>
+        </is>
+      </c>
+      <c r="C2335" t="inlineStr">
+        <is>
+          <t>8.7</t>
+        </is>
+      </c>
+      <c r="D2335" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+      <c r="E2335" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2335" t="inlineStr">
+        <is>
+          <t>O pensamento no cofre</t>
+        </is>
+      </c>
+      <c r="G2335" t="inlineStr">
+        <is>
+          <t>A inovação europeia não pode senão retirar-se — em defesa, para sobreviver</t>
+        </is>
+      </c>
+      <c r="H2335" t="inlineStr">
+        <is>
+          <t>A inovação europeia não pode senão retirar-se — em defesa, para sobreviver</t>
+        </is>
+      </c>
+      <c r="I2335" t="inlineStr">
+        <is>
+          <t>wat-opkomt/gedachte-in-de-kluis.html</t>
+        </is>
+      </c>
+      <c r="R2335" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2335" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2335" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO2335" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="2336">
+      <c r="B2336" t="inlineStr">
+        <is>
+          <t>4.7.1</t>
+        </is>
+      </c>
+      <c r="C2336" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="D2336" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E2336" t="inlineStr">
+        <is>
+          <t>artikel</t>
+        </is>
+      </c>
+      <c r="F2336" t="inlineStr">
+        <is>
+          <t>Мысль в сейфе</t>
+        </is>
+      </c>
+      <c r="G2336" t="inlineStr">
+        <is>
+          <t>Европейская инновация не может не отступить — в оборону, чтобы выжить</t>
+        </is>
+      </c>
+      <c r="H2336" t="inlineStr">
+        <is>
+          <t>Европейская инновация не может не отступить — в оборону, чтобы выжить</t>
+        </is>
+      </c>
+      <c r="I2336" t="inlineStr">
+        <is>
+          <t>wat-opkomt/gedachte-in-de-kluis.html</t>
+        </is>
+      </c>
+      <c r="R2336" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="S2336" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2336" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO2336" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="B2:AR65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>